<commit_message>
auto: 2026-09-13 06:57 자동 백업
</commit_message>
<xml_diff>
--- a/trend/stock_trend_history.xlsx
+++ b/trend/stock_trend_history.xlsx
@@ -694,7 +694,7 @@
     <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-09-12 06:54</t>
+          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-09-13 06:54</t>
         </is>
       </c>
     </row>
@@ -787,21 +787,21 @@
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-09-12) 상위: 반도체  점수 56.0점</t>
+          <t>⚡ 최신(2026-09-13) 상위: 반도체  점수 48.0점</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-09-12) 상위: 삼성전자  점수 24.0점</t>
+          <t>⚡ 최신(2026-09-13) 상위: 인공지능  점수 18.0점</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-09-12) 상위: 바이오  점수 21.0점</t>
+          <t>⚡ 최신(2026-09-13) 상위: 삼성전자  점수 15.0점</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="15" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B14" s="15" t="n">
@@ -928,10 +928,10 @@
         </is>
       </c>
       <c r="D14" s="15" t="n">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="E14" s="15" t="n">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="F14" s="15" t="n">
         <v>0</v>
@@ -947,7 +947,7 @@
       </c>
       <c r="J14" s="17" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 한국경제 헤드라인 언급 / 네이버뉴스 기사 언급</t>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K14" s="17" t="inlineStr">
@@ -959,7 +959,7 @@
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="15" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B15" s="15" t="n">
@@ -967,14 +967,14 @@
       </c>
       <c r="C15" s="16" t="inlineStr">
         <is>
-          <t>삼성전자</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="D15" s="15" t="n">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="E15" s="15" t="n">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="F15" s="15" t="n">
         <v>0</v>
@@ -982,15 +982,15 @@
       <c r="G15" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H15" s="18" t="n">
-        <v>-3.53</v>
-      </c>
-      <c r="I15" s="19" t="n">
-        <v>1.57</v>
+      <c r="H15" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I15" s="15" t="n">
+        <v/>
       </c>
       <c r="J15" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 기사 언급</t>
+          <t>매일경제 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K15" s="17" t="inlineStr">
@@ -1002,7 +1002,7 @@
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="15" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B16" s="15" t="n">
@@ -1010,14 +1010,14 @@
       </c>
       <c r="C16" s="16" t="inlineStr">
         <is>
-          <t>바이오</t>
+          <t>삼성전자</t>
         </is>
       </c>
       <c r="D16" s="15" t="n">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="E16" s="15" t="n">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="F16" s="15" t="n">
         <v>0</v>
@@ -1025,27 +1025,25 @@
       <c r="G16" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H16" s="15" t="n">
+      <c r="H16" s="18" t="n">
+        <v>-3.53</v>
+      </c>
+      <c r="I16" s="19" t="n">
+        <v>1.57</v>
+      </c>
+      <c r="J16" s="17" t="inlineStr">
+        <is>
+          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K16" s="17" t="n">
         <v/>
-      </c>
-      <c r="I16" s="15" t="n">
-        <v/>
-      </c>
-      <c r="J16" s="17" t="inlineStr">
-        <is>
-          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K16" s="17" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B17" s="15" t="n">
@@ -1053,14 +1051,14 @@
       </c>
       <c r="C17" s="16" t="inlineStr">
         <is>
-          <t>KB금융</t>
+          <t>바이오</t>
         </is>
       </c>
       <c r="D17" s="15" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E17" s="15" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F17" s="15" t="n">
         <v>0</v>
@@ -1068,25 +1066,27 @@
       <c r="G17" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H17" s="19" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="I17" s="19" t="n">
-        <v>3.43</v>
+      <c r="H17" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I17" s="15" t="n">
+        <v/>
       </c>
       <c r="J17" s="17" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K17" s="17" t="n">
-        <v/>
+          <t>매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K17" s="17" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B18" s="15" t="n">
@@ -1094,14 +1094,14 @@
       </c>
       <c r="C18" s="16" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>KB금융</t>
         </is>
       </c>
       <c r="D18" s="15" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E18" s="15" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F18" s="15" t="n">
         <v>0</v>
@@ -1109,27 +1109,25 @@
       <c r="G18" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H18" s="15" t="n">
+      <c r="H18" s="19" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="I18" s="19" t="n">
+        <v>3.43</v>
+      </c>
+      <c r="J18" s="17" t="inlineStr">
+        <is>
+          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K18" s="17" t="n">
         <v/>
-      </c>
-      <c r="I18" s="15" t="n">
-        <v/>
-      </c>
-      <c r="J18" s="17" t="inlineStr">
-        <is>
-          <t>매일경제 기사 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급</t>
-        </is>
-      </c>
-      <c r="K18" s="17" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B19" s="15" t="n">
@@ -1137,14 +1135,14 @@
       </c>
       <c r="C19" s="16" t="inlineStr">
         <is>
-          <t>인공지능</t>
+          <t>LG</t>
         </is>
       </c>
       <c r="D19" s="15" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="E19" s="15" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="F19" s="15" t="n">
         <v>0</v>
@@ -1152,27 +1150,25 @@
       <c r="G19" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H19" s="15" t="n">
+      <c r="H19" s="18" t="n">
+        <v>-4.66</v>
+      </c>
+      <c r="I19" s="18" t="n">
+        <v>-7.1</v>
+      </c>
+      <c r="J19" s="17" t="inlineStr">
+        <is>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K19" s="17" t="n">
         <v/>
-      </c>
-      <c r="I19" s="15" t="n">
-        <v/>
-      </c>
-      <c r="J19" s="17" t="inlineStr">
-        <is>
-          <t>네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K19" s="17" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B20" s="15" t="n">
@@ -1180,14 +1176,14 @@
       </c>
       <c r="C20" s="16" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>비에이치아이</t>
         </is>
       </c>
       <c r="D20" s="15" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E20" s="15" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F20" s="15" t="n">
         <v>0</v>
@@ -1195,25 +1191,27 @@
       <c r="G20" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H20" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I20" s="15" t="n">
-        <v/>
+      <c r="H20" s="19" t="n">
+        <v>2.24</v>
+      </c>
+      <c r="I20" s="19" t="n">
+        <v>14</v>
       </c>
       <c r="J20" s="17" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K20" s="17" t="n">
-        <v/>
+          <t>중요공시 1건 / 네이버뉴스 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K20" s="17" t="inlineStr">
+        <is>
+          <t>네이버, 공시</t>
+        </is>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="15" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B21" s="15" t="n">
@@ -1221,7 +1219,7 @@
       </c>
       <c r="C21" s="16" t="inlineStr">
         <is>
-          <t>원전</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="D21" s="15" t="n">
@@ -1244,17 +1242,19 @@
       </c>
       <c r="J21" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K21" s="17" t="n">
-        <v/>
+          <t>매일경제 기사 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
+        </is>
+      </c>
+      <c r="K21" s="17" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="20" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B22" s="20" t="n">
@@ -1285,19 +1285,19 @@
       </c>
       <c r="J22" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +782% / 중요공시 6건</t>
+          <t>네이버 검색 당일 +1153% / 중요공시 6건</t>
         </is>
       </c>
       <c r="K22" s="23" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="20" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B23" s="20" t="n">
@@ -1305,42 +1305,40 @@
       </c>
       <c r="C23" s="21" t="inlineStr">
         <is>
-          <t>대우건설</t>
+          <t>대한항공</t>
         </is>
       </c>
       <c r="D23" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E23" s="20" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F23" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G23" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H23" s="22" t="n">
-        <v>0.71</v>
-      </c>
-      <c r="I23" s="22" t="n">
-        <v>18.04</v>
+      <c r="H23" s="24" t="n">
+        <v>-2.03</v>
+      </c>
+      <c r="I23" s="24" t="n">
+        <v>-4.14</v>
       </c>
       <c r="J23" s="23" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 3일 +100% / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K23" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K23" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="20" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B24" s="20" t="n">
@@ -1348,7 +1346,7 @@
       </c>
       <c r="C24" s="21" t="inlineStr">
         <is>
-          <t>대한항공</t>
+          <t>SG</t>
         </is>
       </c>
       <c r="D24" s="20" t="n">
@@ -1364,14 +1362,14 @@
         <v>0</v>
       </c>
       <c r="H24" s="24" t="n">
-        <v>-2.03</v>
-      </c>
-      <c r="I24" s="24" t="n">
-        <v>-4.14</v>
+        <v>-5.34</v>
+      </c>
+      <c r="I24" s="22" t="n">
+        <v>6.45</v>
       </c>
       <c r="J24" s="23" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+          <t>한국경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K24" s="23" t="n">
@@ -1381,7 +1379,7 @@
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="20" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B25" s="20" t="n">
@@ -1389,40 +1387,42 @@
       </c>
       <c r="C25" s="21" t="inlineStr">
         <is>
-          <t>SG</t>
+          <t>넥사다이내믹스</t>
         </is>
       </c>
       <c r="D25" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E25" s="20" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F25" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G25" s="20" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H25" s="24" t="n">
-        <v>-5.34</v>
+        <v>-3.61</v>
       </c>
       <c r="I25" s="22" t="n">
-        <v>6.45</v>
+        <v>7.65</v>
       </c>
       <c r="J25" s="23" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K25" s="23" t="n">
-        <v/>
+          <t>중요공시 5건 / 중요공시 7일 +400%</t>
+        </is>
+      </c>
+      <c r="K25" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="20" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B26" s="20" t="n">
@@ -1430,30 +1430,30 @@
       </c>
       <c r="C26" s="21" t="inlineStr">
         <is>
-          <t>넥사다이내믹스</t>
+          <t>루멘스</t>
         </is>
       </c>
       <c r="D26" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E26" s="20" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F26" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G26" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="H26" s="24" t="n">
-        <v>-3.61</v>
-      </c>
-      <c r="I26" s="22" t="n">
-        <v>7.65</v>
+        <v>0</v>
+      </c>
+      <c r="H26" s="22" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="I26" s="24" t="n">
+        <v>-5.58</v>
       </c>
       <c r="J26" s="23" t="inlineStr">
         <is>
-          <t>중요공시 5건 / 중요공시 7일 +400%</t>
+          <t>중요공시 5건 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K26" s="23" t="inlineStr">
@@ -1465,7 +1465,7 @@
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="20" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B27" s="20" t="n">
@@ -1473,30 +1473,30 @@
       </c>
       <c r="C27" s="21" t="inlineStr">
         <is>
-          <t>루멘스</t>
+          <t>본느</t>
         </is>
       </c>
       <c r="D27" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E27" s="20" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F27" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G27" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H27" s="22" t="n">
-        <v>0.39</v>
+        <v>3</v>
+      </c>
+      <c r="H27" s="24" t="n">
+        <v>-11.52</v>
       </c>
       <c r="I27" s="24" t="n">
-        <v>-5.58</v>
+        <v>-7.67</v>
       </c>
       <c r="J27" s="23" t="inlineStr">
         <is>
-          <t>중요공시 5건 / 매일경제 헤드라인 언급</t>
+          <t>중요공시 3건 / 중요공시 7일 +50%</t>
         </is>
       </c>
       <c r="K27" s="23" t="inlineStr">
@@ -1508,7 +1508,7 @@
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="20" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B28" s="20" t="n">
@@ -1516,42 +1516,40 @@
       </c>
       <c r="C28" s="21" t="inlineStr">
         <is>
-          <t>본느</t>
+          <t>방산</t>
         </is>
       </c>
       <c r="D28" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E28" s="20" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F28" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G28" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="H28" s="24" t="n">
-        <v>-11.52</v>
-      </c>
-      <c r="I28" s="24" t="n">
-        <v>-7.67</v>
+        <v>0</v>
+      </c>
+      <c r="H28" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I28" s="20" t="n">
+        <v/>
       </c>
       <c r="J28" s="23" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 7일 +50%</t>
-        </is>
-      </c>
-      <c r="K28" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>매일경제 기사 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K28" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="20" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B29" s="20" t="n">
@@ -1559,7 +1557,7 @@
       </c>
       <c r="C29" s="21" t="inlineStr">
         <is>
-          <t>LG</t>
+          <t>비에이치</t>
         </is>
       </c>
       <c r="D29" s="20" t="n">
@@ -1575,24 +1573,26 @@
         <v>0</v>
       </c>
       <c r="H29" s="24" t="n">
-        <v>-4.66</v>
+        <v>-1.25</v>
       </c>
       <c r="I29" s="24" t="n">
-        <v>-7.1</v>
+        <v>-12.95</v>
       </c>
       <c r="J29" s="23" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K29" s="23" t="n">
-        <v/>
+          <t>네이버뉴스 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K29" s="23" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="20" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B30" s="20" t="n">
@@ -1600,7 +1600,7 @@
       </c>
       <c r="C30" s="21" t="inlineStr">
         <is>
-          <t>SK하이닉스</t>
+          <t>대우건설</t>
         </is>
       </c>
       <c r="D30" s="20" t="n">
@@ -1615,27 +1615,27 @@
       <c r="G30" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H30" s="24" t="n">
-        <v>-2.21</v>
+      <c r="H30" s="22" t="n">
+        <v>0.71</v>
       </c>
       <c r="I30" s="22" t="n">
-        <v>10.02</v>
+        <v>18.04</v>
       </c>
       <c r="J30" s="23" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
+          <t>중요공시 2건 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K30" s="23" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="20" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B31" s="20" t="n">
@@ -1643,14 +1643,14 @@
       </c>
       <c r="C31" s="21" t="inlineStr">
         <is>
-          <t>코스나인</t>
+          <t>원전</t>
         </is>
       </c>
       <c r="D31" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E31" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F31" s="20" t="n">
         <v>0</v>
@@ -1658,27 +1658,25 @@
       <c r="G31" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H31" s="24" t="n">
-        <v>-23.08</v>
-      </c>
-      <c r="I31" s="24" t="n">
-        <v>-97.92</v>
+      <c r="H31" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I31" s="20" t="n">
+        <v/>
       </c>
       <c r="J31" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +750% / 중요공시 2건</t>
-        </is>
-      </c>
-      <c r="K31" s="23" t="inlineStr">
-        <is>
-          <t>공시, 네이버</t>
-        </is>
+          <t>매일경제 기사 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K31" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="20" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B32" s="20" t="n">
@@ -1686,7 +1684,7 @@
       </c>
       <c r="C32" s="21" t="inlineStr">
         <is>
-          <t>코다코</t>
+          <t>코스나인</t>
         </is>
       </c>
       <c r="D32" s="20" t="n">
@@ -1701,27 +1699,27 @@
       <c r="G32" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H32" s="22" t="n">
-        <v>10.24</v>
+      <c r="H32" s="24" t="n">
+        <v>-23.08</v>
       </c>
       <c r="I32" s="24" t="n">
-        <v>-99.45</v>
+        <v>-97.92</v>
       </c>
       <c r="J32" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +646% / 중요공시 2건</t>
+          <t>네이버 검색 당일 +1174% / 중요공시 2건</t>
         </is>
       </c>
       <c r="K32" s="23" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="20" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B33" s="20" t="n">
@@ -1729,7 +1727,7 @@
       </c>
       <c r="C33" s="21" t="inlineStr">
         <is>
-          <t>헝셩그룹</t>
+          <t>코다코</t>
         </is>
       </c>
       <c r="D33" s="20" t="n">
@@ -1745,26 +1743,26 @@
         <v>0</v>
       </c>
       <c r="H33" s="22" t="n">
-        <v>14.63</v>
-      </c>
-      <c r="I33" s="22" t="n">
-        <v>5.94</v>
+        <v>10.24</v>
+      </c>
+      <c r="I33" s="24" t="n">
+        <v>-99.45</v>
       </c>
       <c r="J33" s="23" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
+          <t>네이버 검색 당일 +994% / 중요공시 2건</t>
         </is>
       </c>
       <c r="K33" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="20" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B34" s="20" t="n">
@@ -1772,42 +1770,42 @@
       </c>
       <c r="C34" s="21" t="inlineStr">
         <is>
-          <t>셀트리온</t>
+          <t>한국석유</t>
         </is>
       </c>
       <c r="D34" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E34" s="20" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F34" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G34" s="20" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H34" s="24" t="n">
-        <v>-1.44</v>
-      </c>
-      <c r="I34" s="24" t="n">
-        <v>-5.26</v>
+        <v>-3.22</v>
+      </c>
+      <c r="I34" s="22" t="n">
+        <v>8.83</v>
       </c>
       <c r="J34" s="23" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 7일 +100%</t>
+          <t>네이버 검색 당일 +122% / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K34" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="20" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B35" s="20" t="n">
@@ -1815,7 +1813,7 @@
       </c>
       <c r="C35" s="21" t="inlineStr">
         <is>
-          <t>샘표</t>
+          <t>수성웹툰</t>
         </is>
       </c>
       <c r="D35" s="20" t="n">
@@ -1830,27 +1828,27 @@
       <c r="G35" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H35" s="22" t="n">
-        <v>3.23</v>
-      </c>
-      <c r="I35" s="22" t="n">
-        <v>33.72</v>
+      <c r="H35" s="24" t="n">
+        <v>-25.47</v>
+      </c>
+      <c r="I35" s="24" t="n">
+        <v>-49.62</v>
       </c>
       <c r="J35" s="23" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 한국경제 헤드라인 언급</t>
+          <t>네이버 검색 당일 +121% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K35" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="20" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B36" s="20" t="n">
@@ -1858,7 +1856,7 @@
       </c>
       <c r="C36" s="21" t="inlineStr">
         <is>
-          <t>아티스트스튜디오</t>
+          <t>흥아해운</t>
         </is>
       </c>
       <c r="D36" s="20" t="n">
@@ -1874,26 +1872,24 @@
         <v>0</v>
       </c>
       <c r="H36" s="24" t="n">
-        <v>-13.9</v>
-      </c>
-      <c r="I36" s="24" t="n">
-        <v>-8.789999999999999</v>
+        <v>-1.21</v>
+      </c>
+      <c r="I36" s="22" t="n">
+        <v>8.93</v>
       </c>
       <c r="J36" s="23" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K36" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K36" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="20" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B37" s="20" t="n">
@@ -1901,7 +1897,7 @@
       </c>
       <c r="C37" s="21" t="inlineStr">
         <is>
-          <t>비에이치아이</t>
+          <t>삼성E&amp;A</t>
         </is>
       </c>
       <c r="D37" s="20" t="n">
@@ -1917,10 +1913,10 @@
         <v>0</v>
       </c>
       <c r="H37" s="22" t="n">
-        <v>2.24</v>
+        <v>1.19</v>
       </c>
       <c r="I37" s="22" t="n">
-        <v>14</v>
+        <v>11.23</v>
       </c>
       <c r="J37" s="23" t="inlineStr">
         <is>
@@ -1936,7 +1932,7 @@
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="20" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B38" s="20" t="n">
@@ -1944,7 +1940,7 @@
       </c>
       <c r="C38" s="21" t="inlineStr">
         <is>
-          <t>바이오비쥬</t>
+          <t>대한광통신</t>
         </is>
       </c>
       <c r="D38" s="20" t="n">
@@ -1959,27 +1955,27 @@
       <c r="G38" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H38" s="22" t="n">
-        <v>7.28</v>
+      <c r="H38" s="24" t="n">
+        <v>-4</v>
       </c>
       <c r="I38" s="22" t="n">
-        <v>5.46</v>
+        <v>8.76</v>
       </c>
       <c r="J38" s="23" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
+          <t>네이버뉴스 헤드라인 언급</t>
         </is>
       </c>
       <c r="K38" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="20" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B39" s="20" t="n">
@@ -1987,7 +1983,7 @@
       </c>
       <c r="C39" s="21" t="inlineStr">
         <is>
-          <t>넥써쓰</t>
+          <t>헝셩그룹</t>
         </is>
       </c>
       <c r="D39" s="20" t="n">
@@ -2003,10 +1999,10 @@
         <v>0</v>
       </c>
       <c r="H39" s="22" t="n">
-        <v>2.08</v>
+        <v>14.63</v>
       </c>
       <c r="I39" s="22" t="n">
-        <v>5.99</v>
+        <v>5.94</v>
       </c>
       <c r="J39" s="23" t="inlineStr">
         <is>
@@ -2022,7 +2018,7 @@
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="20" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B40" s="20" t="n">
@@ -2030,40 +2026,42 @@
       </c>
       <c r="C40" s="21" t="inlineStr">
         <is>
-          <t>로보티즈</t>
+          <t>금호건설</t>
         </is>
       </c>
       <c r="D40" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E40" s="20" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F40" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G40" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H40" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="I40" s="22" t="n">
-        <v>6.24</v>
+        <v>3</v>
+      </c>
+      <c r="H40" s="24" t="n">
+        <v>-2.19</v>
+      </c>
+      <c r="I40" s="24" t="n">
+        <v>-8.58</v>
       </c>
       <c r="J40" s="23" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K40" s="23" t="n">
-        <v/>
+          <t>중요공시 2건 / 중요공시 7일 +100%</t>
+        </is>
+      </c>
+      <c r="K40" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="20" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B41" s="20" t="n">
@@ -2071,384 +2069,378 @@
       </c>
       <c r="C41" s="21" t="inlineStr">
         <is>
+          <t>셀트리온</t>
+        </is>
+      </c>
+      <c r="D41" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="E41" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="F41" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G41" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="H41" s="24" t="n">
+        <v>-1.44</v>
+      </c>
+      <c r="I41" s="24" t="n">
+        <v>-5.26</v>
+      </c>
+      <c r="J41" s="23" t="inlineStr">
+        <is>
+          <t>중요공시 2건 / 중요공시 7일 +100%</t>
+        </is>
+      </c>
+      <c r="K41" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="18" customHeight="1">
+      <c r="A42" s="20" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B42" s="20" t="n">
+        <v>29</v>
+      </c>
+      <c r="C42" s="21" t="inlineStr">
+        <is>
+          <t>샘표</t>
+        </is>
+      </c>
+      <c r="D42" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="E42" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F42" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G42" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H42" s="22" t="n">
+        <v>3.23</v>
+      </c>
+      <c r="I42" s="22" t="n">
+        <v>33.72</v>
+      </c>
+      <c r="J42" s="23" t="inlineStr">
+        <is>
+          <t>중요공시 1건 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K42" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="18" customHeight="1">
+      <c r="A43" s="20" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B43" s="20" t="n">
+        <v>30</v>
+      </c>
+      <c r="C43" s="21" t="inlineStr">
+        <is>
+          <t>아티스트스튜디오</t>
+        </is>
+      </c>
+      <c r="D43" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="E43" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F43" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G43" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H43" s="24" t="n">
+        <v>-13.9</v>
+      </c>
+      <c r="I43" s="24" t="n">
+        <v>-8.789999999999999</v>
+      </c>
+      <c r="J43" s="23" t="inlineStr">
+        <is>
+          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K43" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="18" customHeight="1">
+      <c r="A44" s="20" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B44" s="20" t="n">
+        <v>31</v>
+      </c>
+      <c r="C44" s="21" t="inlineStr">
+        <is>
+          <t>바이오비쥬</t>
+        </is>
+      </c>
+      <c r="D44" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="E44" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F44" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G44" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H44" s="22" t="n">
+        <v>7.28</v>
+      </c>
+      <c r="I44" s="22" t="n">
+        <v>5.46</v>
+      </c>
+      <c r="J44" s="23" t="inlineStr">
+        <is>
+          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K44" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="18" customHeight="1">
+      <c r="A45" s="20" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B45" s="20" t="n">
+        <v>32</v>
+      </c>
+      <c r="C45" s="21" t="inlineStr">
+        <is>
+          <t>넥써쓰</t>
+        </is>
+      </c>
+      <c r="D45" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="E45" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F45" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H45" s="22" t="n">
+        <v>2.08</v>
+      </c>
+      <c r="I45" s="22" t="n">
+        <v>5.99</v>
+      </c>
+      <c r="J45" s="23" t="inlineStr">
+        <is>
+          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K45" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="18" customHeight="1">
+      <c r="A46" s="20" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B46" s="20" t="n">
+        <v>33</v>
+      </c>
+      <c r="C46" s="21" t="inlineStr">
+        <is>
+          <t>로봇</t>
+        </is>
+      </c>
+      <c r="D46" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="E46" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F46" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G46" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H46" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I46" s="20" t="n">
+        <v/>
+      </c>
+      <c r="J46" s="23" t="inlineStr">
+        <is>
+          <t>매일경제 기사 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K46" s="23" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="47" ht="18" customHeight="1">
+      <c r="A47" s="20" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B47" s="20" t="n">
+        <v>34</v>
+      </c>
+      <c r="C47" s="21" t="inlineStr">
+        <is>
+          <t>로보티즈</t>
+        </is>
+      </c>
+      <c r="D47" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="E47" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F47" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H47" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="I47" s="22" t="n">
+        <v>6.24</v>
+      </c>
+      <c r="J47" s="23" t="inlineStr">
+        <is>
+          <t>매일경제 기사 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K47" s="23" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="48" ht="18" customHeight="1">
+      <c r="A48" s="20" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B48" s="20" t="n">
+        <v>35</v>
+      </c>
+      <c r="C48" s="21" t="inlineStr">
+        <is>
           <t>전기차</t>
         </is>
       </c>
-      <c r="D41" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E41" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F41" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G41" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H41" s="20" t="n">
+      <c r="D48" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="E48" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F48" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G48" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H48" s="20" t="n">
         <v/>
       </c>
-      <c r="I41" s="20" t="n">
+      <c r="I48" s="20" t="n">
         <v/>
       </c>
-      <c r="J41" s="23" t="inlineStr">
+      <c r="J48" s="23" t="inlineStr">
         <is>
           <t>매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
-      <c r="K41" s="23" t="n">
+      <c r="K48" s="23" t="n">
         <v/>
       </c>
     </row>
-    <row r="42" ht="18" customHeight="1">
-      <c r="A42" s="25" t="inlineStr">
-        <is>
-          <t>2026-09-12</t>
-        </is>
-      </c>
-      <c r="B42" s="25" t="n">
-        <v>29</v>
-      </c>
-      <c r="C42" s="26" t="inlineStr">
-        <is>
-          <t>삼미금속</t>
-        </is>
-      </c>
-      <c r="D42" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="E42" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="F42" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="G42" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H42" s="27" t="n">
-        <v>-2.69</v>
-      </c>
-      <c r="I42" s="28" t="n">
-        <v>47.19</v>
-      </c>
-      <c r="J42" s="29" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +888%</t>
-        </is>
-      </c>
-      <c r="K42" s="29" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="18" customHeight="1">
-      <c r="A43" s="25" t="inlineStr">
-        <is>
-          <t>2026-09-12</t>
-        </is>
-      </c>
-      <c r="B43" s="25" t="n">
-        <v>30</v>
-      </c>
-      <c r="C43" s="26" t="inlineStr">
-        <is>
-          <t>액스비스</t>
-        </is>
-      </c>
-      <c r="D43" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="E43" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="F43" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="G43" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H43" s="28" t="n">
-        <v>11.97</v>
-      </c>
-      <c r="I43" s="28" t="n">
-        <v>57.45</v>
-      </c>
-      <c r="J43" s="29" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +449%</t>
-        </is>
-      </c>
-      <c r="K43" s="29" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="18" customHeight="1">
-      <c r="A44" s="25" t="inlineStr">
-        <is>
-          <t>2026-09-12</t>
-        </is>
-      </c>
-      <c r="B44" s="25" t="n">
-        <v>31</v>
-      </c>
-      <c r="C44" s="26" t="inlineStr">
-        <is>
-          <t>카프로</t>
-        </is>
-      </c>
-      <c r="D44" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="E44" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="F44" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="G44" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H44" s="27" t="n">
-        <v>-16.67</v>
-      </c>
-      <c r="I44" s="27" t="n">
-        <v>-96.72</v>
-      </c>
-      <c r="J44" s="29" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +404%</t>
-        </is>
-      </c>
-      <c r="K44" s="29" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="18" customHeight="1">
-      <c r="A45" s="25" t="inlineStr">
-        <is>
-          <t>2026-09-12</t>
-        </is>
-      </c>
-      <c r="B45" s="25" t="n">
-        <v>32</v>
-      </c>
-      <c r="C45" s="26" t="inlineStr">
-        <is>
-          <t>엔에이치스팩34호</t>
-        </is>
-      </c>
-      <c r="D45" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="E45" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="F45" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="G45" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H45" s="27" t="n">
-        <v>-6.94</v>
-      </c>
-      <c r="I45" s="27" t="n">
-        <v>-6.94</v>
-      </c>
-      <c r="J45" s="29" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +398%</t>
-        </is>
-      </c>
-      <c r="K45" s="29" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="18" customHeight="1">
-      <c r="A46" s="25" t="inlineStr">
-        <is>
-          <t>2026-09-12</t>
-        </is>
-      </c>
-      <c r="B46" s="25" t="n">
-        <v>33</v>
-      </c>
-      <c r="C46" s="26" t="inlineStr">
-        <is>
-          <t>샘표식품</t>
-        </is>
-      </c>
-      <c r="D46" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="E46" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="F46" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="G46" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H46" s="27" t="n">
-        <v>-14.76</v>
-      </c>
-      <c r="I46" s="28" t="n">
-        <v>10.78</v>
-      </c>
-      <c r="J46" s="29" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +342%</t>
-        </is>
-      </c>
-      <c r="K46" s="29" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="18" customHeight="1">
-      <c r="A47" s="25" t="inlineStr">
-        <is>
-          <t>2026-09-12</t>
-        </is>
-      </c>
-      <c r="B47" s="25" t="n">
-        <v>34</v>
-      </c>
-      <c r="C47" s="26" t="inlineStr">
-        <is>
-          <t>서전기전</t>
-        </is>
-      </c>
-      <c r="D47" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="E47" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="F47" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="G47" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H47" s="27" t="n">
-        <v>-3.51</v>
-      </c>
-      <c r="I47" s="28" t="n">
-        <v>24.43</v>
-      </c>
-      <c r="J47" s="29" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +330%</t>
-        </is>
-      </c>
-      <c r="K47" s="29" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="18" customHeight="1">
-      <c r="A48" s="25" t="inlineStr">
-        <is>
-          <t>2026-09-12</t>
-        </is>
-      </c>
-      <c r="B48" s="25" t="n">
-        <v>35</v>
-      </c>
-      <c r="C48" s="26" t="inlineStr">
-        <is>
-          <t>머큐리</t>
-        </is>
-      </c>
-      <c r="D48" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="E48" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="F48" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="G48" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H48" s="27" t="n">
-        <v>-4.43</v>
-      </c>
-      <c r="I48" s="28" t="n">
-        <v>39.71</v>
-      </c>
-      <c r="J48" s="29" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +279%</t>
-        </is>
-      </c>
-      <c r="K48" s="29" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
-      </c>
-    </row>
     <row r="49" ht="18" customHeight="1">
-      <c r="A49" s="25" t="inlineStr">
-        <is>
-          <t>2026-09-12</t>
-        </is>
-      </c>
-      <c r="B49" s="25" t="n">
+      <c r="A49" s="20" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B49" s="20" t="n">
         <v>36</v>
       </c>
-      <c r="C49" s="26" t="inlineStr">
-        <is>
-          <t>오르비텍</t>
-        </is>
-      </c>
-      <c r="D49" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="E49" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="F49" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="G49" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H49" s="27" t="n">
-        <v>-3.34</v>
-      </c>
-      <c r="I49" s="28" t="n">
-        <v>40.35</v>
-      </c>
-      <c r="J49" s="29" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +243%</t>
-        </is>
-      </c>
-      <c r="K49" s="29" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+      <c r="C49" s="21" t="inlineStr">
+        <is>
+          <t>혜인</t>
+        </is>
+      </c>
+      <c r="D49" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="E49" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F49" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G49" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H49" s="22" t="n">
+        <v>3.85</v>
+      </c>
+      <c r="I49" s="24" t="n">
+        <v>-11.27</v>
+      </c>
+      <c r="J49" s="23" t="inlineStr">
+        <is>
+          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K49" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B50" s="25" t="n">
@@ -2456,7 +2448,7 @@
       </c>
       <c r="C50" s="26" t="inlineStr">
         <is>
-          <t>한빛레이저</t>
+          <t>삼미금속</t>
         </is>
       </c>
       <c r="D50" s="25" t="n">
@@ -2471,15 +2463,15 @@
       <c r="G50" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H50" s="28" t="n">
-        <v>2.83</v>
+      <c r="H50" s="27" t="n">
+        <v>-2.69</v>
       </c>
       <c r="I50" s="28" t="n">
-        <v>36.01</v>
+        <v>47.19</v>
       </c>
       <c r="J50" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +216%</t>
+          <t>네이버 검색 당일 +1054%</t>
         </is>
       </c>
       <c r="K50" s="29" t="inlineStr">
@@ -2491,7 +2483,7 @@
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B51" s="25" t="n">
@@ -2499,7 +2491,7 @@
       </c>
       <c r="C51" s="26" t="inlineStr">
         <is>
-          <t>빛과전자</t>
+          <t>액스비스</t>
         </is>
       </c>
       <c r="D51" s="25" t="n">
@@ -2514,15 +2506,15 @@
       <c r="G51" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H51" s="27" t="n">
-        <v>-1.4</v>
+      <c r="H51" s="28" t="n">
+        <v>11.97</v>
       </c>
       <c r="I51" s="28" t="n">
-        <v>42.54</v>
+        <v>57.45</v>
       </c>
       <c r="J51" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +157%</t>
+          <t>네이버 검색 당일 +735%</t>
         </is>
       </c>
       <c r="K51" s="29" t="inlineStr">
@@ -2534,7 +2526,7 @@
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B52" s="25" t="n">
@@ -2542,7 +2534,7 @@
       </c>
       <c r="C52" s="26" t="inlineStr">
         <is>
-          <t>에스투더블유</t>
+          <t>샘표식품</t>
         </is>
       </c>
       <c r="D52" s="25" t="n">
@@ -2557,15 +2549,15 @@
       <c r="G52" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H52" s="28" t="n">
-        <v>26.38</v>
+      <c r="H52" s="27" t="n">
+        <v>-14.76</v>
       </c>
       <c r="I52" s="28" t="n">
-        <v>52.78</v>
+        <v>10.78</v>
       </c>
       <c r="J52" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +143%</t>
+          <t>네이버 검색 당일 +663%</t>
         </is>
       </c>
       <c r="K52" s="29" t="inlineStr">
@@ -2577,7 +2569,7 @@
     <row r="53" ht="18" customHeight="1">
       <c r="A53" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B53" s="25" t="n">
@@ -2585,7 +2577,7 @@
       </c>
       <c r="C53" s="26" t="inlineStr">
         <is>
-          <t>스트라드비젼</t>
+          <t>엔에이치스팩34호</t>
         </is>
       </c>
       <c r="D53" s="25" t="n">
@@ -2601,14 +2593,14 @@
         <v>0</v>
       </c>
       <c r="H53" s="27" t="n">
-        <v>-0.39</v>
-      </c>
-      <c r="I53" s="28" t="n">
-        <v>35.05</v>
+        <v>-6.94</v>
+      </c>
+      <c r="I53" s="27" t="n">
+        <v>-6.94</v>
       </c>
       <c r="J53" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +111%</t>
+          <t>네이버 검색 당일 +486%</t>
         </is>
       </c>
       <c r="K53" s="29" t="inlineStr">
@@ -2620,7 +2612,7 @@
     <row r="54" ht="18" customHeight="1">
       <c r="A54" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B54" s="25" t="n">
@@ -2628,7 +2620,7 @@
       </c>
       <c r="C54" s="26" t="inlineStr">
         <is>
-          <t>원풍물산</t>
+          <t>카프로</t>
         </is>
       </c>
       <c r="D54" s="25" t="n">
@@ -2644,26 +2636,26 @@
         <v>0</v>
       </c>
       <c r="H54" s="27" t="n">
-        <v>-1.47</v>
+        <v>-16.67</v>
       </c>
       <c r="I54" s="27" t="n">
-        <v>-68.62</v>
+        <v>-96.72</v>
       </c>
       <c r="J54" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +74% / 중요공시 1건</t>
+          <t>네이버 검색 당일 +470%</t>
         </is>
       </c>
       <c r="K54" s="29" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="55" ht="18" customHeight="1">
       <c r="A55" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B55" s="25" t="n">
@@ -2671,7 +2663,7 @@
       </c>
       <c r="C55" s="26" t="inlineStr">
         <is>
-          <t>수성웹툰</t>
+          <t>에스투더블유</t>
         </is>
       </c>
       <c r="D55" s="25" t="n">
@@ -2686,27 +2678,27 @@
       <c r="G55" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H55" s="27" t="n">
-        <v>-25.47</v>
-      </c>
-      <c r="I55" s="27" t="n">
-        <v>-49.62</v>
+      <c r="H55" s="28" t="n">
+        <v>26.38</v>
+      </c>
+      <c r="I55" s="28" t="n">
+        <v>52.78</v>
       </c>
       <c r="J55" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +68% / 중요공시 1건</t>
+          <t>네이버 검색 당일 +403%</t>
         </is>
       </c>
       <c r="K55" s="29" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="56" ht="18" customHeight="1">
       <c r="A56" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B56" s="25" t="n">
@@ -2714,7 +2706,7 @@
       </c>
       <c r="C56" s="26" t="inlineStr">
         <is>
-          <t>엑스게이트</t>
+          <t>서전기전</t>
         </is>
       </c>
       <c r="D56" s="25" t="n">
@@ -2729,15 +2721,15 @@
       <c r="G56" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H56" s="28" t="n">
-        <v>29.94</v>
+      <c r="H56" s="27" t="n">
+        <v>-3.51</v>
       </c>
       <c r="I56" s="28" t="n">
-        <v>40.51</v>
+        <v>24.43</v>
       </c>
       <c r="J56" s="29" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급</t>
+          <t>네이버 검색 당일 +398%</t>
         </is>
       </c>
       <c r="K56" s="29" t="inlineStr">
@@ -2749,7 +2741,7 @@
     <row r="57" ht="18" customHeight="1">
       <c r="A57" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B57" s="25" t="n">
@@ -2757,7 +2749,7 @@
       </c>
       <c r="C57" s="26" t="inlineStr">
         <is>
-          <t>두산에너빌리티</t>
+          <t>머큐리</t>
         </is>
       </c>
       <c r="D57" s="25" t="n">
@@ -2772,25 +2764,27 @@
       <c r="G57" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H57" s="28" t="n">
-        <v>1</v>
+      <c r="H57" s="27" t="n">
+        <v>-4.43</v>
       </c>
       <c r="I57" s="28" t="n">
-        <v>14.65</v>
+        <v>39.71</v>
       </c>
       <c r="J57" s="29" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K57" s="29" t="n">
-        <v/>
+          <t>네이버 검색 당일 +359%</t>
+        </is>
+      </c>
+      <c r="K57" s="29" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="58" ht="18" customHeight="1">
       <c r="A58" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B58" s="25" t="n">
@@ -2798,7 +2792,7 @@
       </c>
       <c r="C58" s="26" t="inlineStr">
         <is>
-          <t>삼성E&amp;A</t>
+          <t>오르비텍</t>
         </is>
       </c>
       <c r="D58" s="25" t="n">
@@ -2813,27 +2807,27 @@
       <c r="G58" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H58" s="28" t="n">
-        <v>1.19</v>
+      <c r="H58" s="27" t="n">
+        <v>-3.34</v>
       </c>
       <c r="I58" s="28" t="n">
-        <v>11.23</v>
+        <v>40.35</v>
       </c>
       <c r="J58" s="29" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 한국경제 헤드라인 언급</t>
+          <t>네이버 검색 당일 +296%</t>
         </is>
       </c>
       <c r="K58" s="29" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="59" ht="18" customHeight="1">
       <c r="A59" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B59" s="25" t="n">
@@ -2841,7 +2835,7 @@
       </c>
       <c r="C59" s="26" t="inlineStr">
         <is>
-          <t>흥아해운</t>
+          <t>한빛레이저</t>
         </is>
       </c>
       <c r="D59" s="25" t="n">
@@ -2856,25 +2850,27 @@
       <c r="G59" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H59" s="27" t="n">
-        <v>-1.21</v>
+      <c r="H59" s="28" t="n">
+        <v>2.83</v>
       </c>
       <c r="I59" s="28" t="n">
-        <v>8.93</v>
+        <v>36.01</v>
       </c>
       <c r="J59" s="29" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K59" s="29" t="n">
-        <v/>
+          <t>네이버 검색 당일 +273%</t>
+        </is>
+      </c>
+      <c r="K59" s="29" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="60" ht="18" customHeight="1">
       <c r="A60" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B60" s="25" t="n">
@@ -2882,7 +2878,7 @@
       </c>
       <c r="C60" s="26" t="inlineStr">
         <is>
-          <t>삼성전자우</t>
+          <t>빛과전자</t>
         </is>
       </c>
       <c r="D60" s="25" t="n">
@@ -2898,24 +2894,26 @@
         <v>0</v>
       </c>
       <c r="H60" s="27" t="n">
-        <v>-4.78</v>
+        <v>-1.4</v>
       </c>
       <c r="I60" s="28" t="n">
-        <v>0.89</v>
+        <v>42.54</v>
       </c>
       <c r="J60" s="29" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K60" s="29" t="n">
-        <v/>
+          <t>네이버 검색 당일 +204%</t>
+        </is>
+      </c>
+      <c r="K60" s="29" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="61" ht="18" customHeight="1">
       <c r="A61" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B61" s="25" t="n">
@@ -2923,7 +2921,7 @@
       </c>
       <c r="C61" s="26" t="inlineStr">
         <is>
-          <t>엠젠솔루션</t>
+          <t>원익피앤이</t>
         </is>
       </c>
       <c r="D61" s="25" t="n">
@@ -2938,27 +2936,27 @@
       <c r="G61" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H61" s="27" t="n">
-        <v>-8.75</v>
+      <c r="H61" s="28" t="n">
+        <v>6.62</v>
       </c>
       <c r="I61" s="28" t="n">
-        <v>15.63</v>
+        <v>41</v>
       </c>
       <c r="J61" s="29" t="inlineStr">
         <is>
-          <t>중요공시 5건</t>
+          <t>네이버 검색 당일 +200%</t>
         </is>
       </c>
       <c r="K61" s="29" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="62" ht="18" customHeight="1">
       <c r="A62" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B62" s="25" t="n">
@@ -2966,7 +2964,7 @@
       </c>
       <c r="C62" s="26" t="inlineStr">
         <is>
-          <t>모아데이타</t>
+          <t>엑스게이트</t>
         </is>
       </c>
       <c r="D62" s="25" t="n">
@@ -2981,27 +2979,27 @@
       <c r="G62" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H62" s="27" t="n">
-        <v>-3.4</v>
-      </c>
-      <c r="I62" s="27" t="n">
-        <v>-7.79</v>
+      <c r="H62" s="28" t="n">
+        <v>29.94</v>
+      </c>
+      <c r="I62" s="28" t="n">
+        <v>40.51</v>
       </c>
       <c r="J62" s="29" t="inlineStr">
         <is>
-          <t>중요공시 4건</t>
+          <t>네이버 검색 당일 +198%</t>
         </is>
       </c>
       <c r="K62" s="29" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="63" ht="18" customHeight="1">
       <c r="A63" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B63" s="25" t="n">
@@ -3009,35 +3007,35 @@
       </c>
       <c r="C63" s="26" t="inlineStr">
         <is>
-          <t>CG인바이츠</t>
+          <t>케이에스피</t>
         </is>
       </c>
       <c r="D63" s="25" t="n">
         <v>3</v>
       </c>
       <c r="E63" s="25" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F63" s="25" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G63" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H63" s="27" t="n">
-        <v>-4.7</v>
+      <c r="H63" s="28" t="n">
+        <v>6.57</v>
       </c>
       <c r="I63" s="28" t="n">
-        <v>7.32</v>
+        <v>29.35</v>
       </c>
       <c r="J63" s="29" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 3일 +100%</t>
+          <t>네이버 검색 당일 +183%</t>
         </is>
       </c>
       <c r="K63" s="29" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
@@ -3134,22 +3132,22 @@
         <v>1</v>
       </c>
       <c r="C3" s="25" t="n">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="D3" s="25" t="n">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="E3" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F3" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G3" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="H3" s="25" t="n"/>
@@ -3158,37 +3156,33 @@
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="26" t="inlineStr">
         <is>
-          <t>삼성전자</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="B4" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C4" s="25" t="n">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="D4" s="25" t="n">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="E4" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F4" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G4" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
-        </is>
-      </c>
-      <c r="H4" s="27" t="n">
-        <v>-3.53</v>
-      </c>
-      <c r="I4" s="28" t="n">
-        <v>1.57</v>
-      </c>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="H4" s="25" t="n"/>
+      <c r="I4" s="25" t="n"/>
     </row>
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="26" t="inlineStr">
@@ -3200,22 +3194,22 @@
         <v>1</v>
       </c>
       <c r="C5" s="25" t="n">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="D5" s="25" t="n">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="E5" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F5" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G5" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="H5" s="25" t="n"/>
@@ -3224,135 +3218,147 @@
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="26" t="inlineStr">
         <is>
-          <t>KB금융</t>
+          <t>삼성전자</t>
         </is>
       </c>
       <c r="B6" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="25" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D6" s="25" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E6" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F6" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G6" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
-        </is>
-      </c>
-      <c r="H6" s="28" t="n">
-        <v>2.6</v>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="H6" s="27" t="n">
+        <v>-3.53</v>
       </c>
       <c r="I6" s="28" t="n">
-        <v>3.43</v>
+        <v>1.57</v>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="26" t="inlineStr">
         <is>
-          <t>인공지능</t>
+          <t>KB금융</t>
         </is>
       </c>
       <c r="B7" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="25" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D7" s="25" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E7" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F7" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G7" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
-        </is>
-      </c>
-      <c r="H7" s="25" t="n"/>
-      <c r="I7" s="25" t="n"/>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="H7" s="28" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="I7" s="28" t="n">
+        <v>3.43</v>
+      </c>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="26" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>LG</t>
         </is>
       </c>
       <c r="B8" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="25" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D8" s="25" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="E8" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F8" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G8" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
-        </is>
-      </c>
-      <c r="H8" s="25" t="n"/>
-      <c r="I8" s="25" t="n"/>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="H8" s="27" t="n">
+        <v>-4.66</v>
+      </c>
+      <c r="I8" s="27" t="n">
+        <v>-7.1</v>
+      </c>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="26" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>비에이치아이</t>
         </is>
       </c>
       <c r="B9" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D9" s="25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E9" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F9" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G9" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
-        </is>
-      </c>
-      <c r="H9" s="25" t="n"/>
-      <c r="I9" s="25" t="n"/>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="H9" s="28" t="n">
+        <v>2.24</v>
+      </c>
+      <c r="I9" s="28" t="n">
+        <v>14</v>
+      </c>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="26" t="inlineStr">
         <is>
-          <t>원전</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="B10" s="25" t="n">
@@ -3369,12 +3375,12 @@
       </c>
       <c r="F10" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G10" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="H10" s="25" t="n"/>
@@ -3383,7 +3389,7 @@
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="26" t="inlineStr">
         <is>
-          <t>LG</t>
+          <t>SG</t>
         </is>
       </c>
       <c r="B11" s="25" t="n">
@@ -3400,25 +3406,25 @@
       </c>
       <c r="F11" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G11" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="H11" s="27" t="n">
-        <v>-4.66</v>
-      </c>
-      <c r="I11" s="27" t="n">
-        <v>-7.1</v>
+        <v>-5.34</v>
+      </c>
+      <c r="I11" s="28" t="n">
+        <v>6.45</v>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="26" t="inlineStr">
         <is>
-          <t>SG</t>
+          <t>넥사다이내믹스</t>
         </is>
       </c>
       <c r="B12" s="25" t="n">
@@ -3435,25 +3441,25 @@
       </c>
       <c r="F12" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G12" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="H12" s="27" t="n">
-        <v>-5.34</v>
+        <v>-3.61</v>
       </c>
       <c r="I12" s="28" t="n">
-        <v>6.45</v>
+        <v>7.65</v>
       </c>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>넥사다이내믹스</t>
+          <t>대한항공</t>
         </is>
       </c>
       <c r="B13" s="25" t="n">
@@ -3470,25 +3476,25 @@
       </c>
       <c r="F13" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G13" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="H13" s="27" t="n">
-        <v>-3.61</v>
-      </c>
-      <c r="I13" s="28" t="n">
-        <v>7.65</v>
+        <v>-2.03</v>
+      </c>
+      <c r="I13" s="27" t="n">
+        <v>-4.14</v>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>대우건설</t>
+          <t>더코디</t>
         </is>
       </c>
       <c r="B14" s="25" t="n">
@@ -3505,25 +3511,25 @@
       </c>
       <c r="F14" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G14" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
-        </is>
-      </c>
-      <c r="H14" s="28" t="n">
-        <v>0.71</v>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="H14" s="25" t="n">
+        <v>0</v>
       </c>
       <c r="I14" s="28" t="n">
-        <v>18.04</v>
+        <v>185.01</v>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>대한항공</t>
+          <t>루멘스</t>
         </is>
       </c>
       <c r="B15" s="25" t="n">
@@ -3540,25 +3546,25 @@
       </c>
       <c r="F15" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G15" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
-        </is>
-      </c>
-      <c r="H15" s="27" t="n">
-        <v>-2.03</v>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="H15" s="28" t="n">
+        <v>0.39</v>
       </c>
       <c r="I15" s="27" t="n">
-        <v>-4.14</v>
+        <v>-5.58</v>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>더코디</t>
+          <t>방산</t>
         </is>
       </c>
       <c r="B16" s="25" t="n">
@@ -3575,25 +3581,21 @@
       </c>
       <c r="F16" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G16" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
-        </is>
-      </c>
-      <c r="H16" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="I16" s="28" t="n">
-        <v>185.01</v>
-      </c>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="H16" s="25" t="n"/>
+      <c r="I16" s="25" t="n"/>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>루멘스</t>
+          <t>본느</t>
         </is>
       </c>
       <c r="B17" s="25" t="n">
@@ -3610,25 +3612,25 @@
       </c>
       <c r="F17" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G17" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
-        </is>
-      </c>
-      <c r="H17" s="28" t="n">
-        <v>0.39</v>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="H17" s="27" t="n">
+        <v>-11.52</v>
       </c>
       <c r="I17" s="27" t="n">
-        <v>-5.58</v>
+        <v>-7.67</v>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="26" t="inlineStr">
         <is>
-          <t>본느</t>
+          <t>비에이치</t>
         </is>
       </c>
       <c r="B18" s="25" t="n">
@@ -3645,25 +3647,25 @@
       </c>
       <c r="F18" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G18" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="H18" s="27" t="n">
-        <v>-11.52</v>
+        <v>-1.25</v>
       </c>
       <c r="I18" s="27" t="n">
-        <v>-7.67</v>
+        <v>-12.95</v>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>SK하이닉스</t>
+          <t>대우건설</t>
         </is>
       </c>
       <c r="B19" s="25" t="n">
@@ -3680,60 +3682,56 @@
       </c>
       <c r="F19" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G19" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
-        </is>
-      </c>
-      <c r="H19" s="27" t="n">
-        <v>-2.21</v>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="H19" s="28" t="n">
+        <v>0.71</v>
       </c>
       <c r="I19" s="28" t="n">
-        <v>10.02</v>
+        <v>18.04</v>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="26" t="inlineStr">
         <is>
-          <t>넥써쓰</t>
+          <t>원전</t>
         </is>
       </c>
       <c r="B20" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C20" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D20" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E20" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F20" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G20" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
-        </is>
-      </c>
-      <c r="H20" s="28" t="n">
-        <v>2.08</v>
-      </c>
-      <c r="I20" s="28" t="n">
-        <v>5.99</v>
-      </c>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="H20" s="25" t="n"/>
+      <c r="I20" s="25" t="n"/>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="26" t="inlineStr">
         <is>
-          <t>로보티즈</t>
+          <t>금호건설</t>
         </is>
       </c>
       <c r="B21" s="25" t="n">
@@ -3750,25 +3748,25 @@
       </c>
       <c r="F21" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G21" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
-        </is>
-      </c>
-      <c r="H21" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="I21" s="28" t="n">
-        <v>6.24</v>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="H21" s="27" t="n">
+        <v>-2.19</v>
+      </c>
+      <c r="I21" s="27" t="n">
+        <v>-8.58</v>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="26" t="inlineStr">
         <is>
-          <t>바이오비쥬</t>
+          <t>넥써쓰</t>
         </is>
       </c>
       <c r="B22" s="25" t="n">
@@ -3785,25 +3783,25 @@
       </c>
       <c r="F22" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G22" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="H22" s="28" t="n">
-        <v>7.28</v>
+        <v>2.08</v>
       </c>
       <c r="I22" s="28" t="n">
-        <v>5.46</v>
+        <v>5.99</v>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="26" t="inlineStr">
         <is>
-          <t>비에이치아이</t>
+          <t>대한광통신</t>
         </is>
       </c>
       <c r="B23" s="25" t="n">
@@ -3820,25 +3818,25 @@
       </c>
       <c r="F23" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G23" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
-        </is>
-      </c>
-      <c r="H23" s="28" t="n">
-        <v>2.24</v>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="H23" s="27" t="n">
+        <v>-4</v>
       </c>
       <c r="I23" s="28" t="n">
-        <v>14</v>
+        <v>8.76</v>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="26" t="inlineStr">
         <is>
-          <t>샘표</t>
+          <t>로보티즈</t>
         </is>
       </c>
       <c r="B24" s="25" t="n">
@@ -3855,25 +3853,25 @@
       </c>
       <c r="F24" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G24" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
-        </is>
-      </c>
-      <c r="H24" s="28" t="n">
-        <v>3.23</v>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="H24" s="25" t="n">
+        <v>0</v>
       </c>
       <c r="I24" s="28" t="n">
-        <v>33.72</v>
+        <v>6.24</v>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="26" t="inlineStr">
         <is>
-          <t>셀트리온</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="B25" s="25" t="n">
@@ -3890,25 +3888,21 @@
       </c>
       <c r="F25" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G25" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
-        </is>
-      </c>
-      <c r="H25" s="27" t="n">
-        <v>-1.44</v>
-      </c>
-      <c r="I25" s="27" t="n">
-        <v>-5.26</v>
-      </c>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="H25" s="25" t="n"/>
+      <c r="I25" s="25" t="n"/>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="26" t="inlineStr">
         <is>
-          <t>아티스트스튜디오</t>
+          <t>바이오비쥬</t>
         </is>
       </c>
       <c r="B26" s="25" t="n">
@@ -3925,25 +3919,25 @@
       </c>
       <c r="F26" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G26" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
-        </is>
-      </c>
-      <c r="H26" s="27" t="n">
-        <v>-13.9</v>
-      </c>
-      <c r="I26" s="27" t="n">
-        <v>-8.789999999999999</v>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="H26" s="28" t="n">
+        <v>7.28</v>
+      </c>
+      <c r="I26" s="28" t="n">
+        <v>5.46</v>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="26" t="inlineStr">
         <is>
-          <t>전기차</t>
+          <t>삼성E&amp;A</t>
         </is>
       </c>
       <c r="B27" s="25" t="n">
@@ -3960,21 +3954,25 @@
       </c>
       <c r="F27" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G27" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
-        </is>
-      </c>
-      <c r="H27" s="25" t="n"/>
-      <c r="I27" s="25" t="n"/>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="H27" s="28" t="n">
+        <v>1.19</v>
+      </c>
+      <c r="I27" s="28" t="n">
+        <v>11.23</v>
+      </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="26" t="inlineStr">
         <is>
-          <t>코다코</t>
+          <t>샘표</t>
         </is>
       </c>
       <c r="B28" s="25" t="n">
@@ -3991,25 +3989,25 @@
       </c>
       <c r="F28" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G28" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="H28" s="28" t="n">
-        <v>10.24</v>
-      </c>
-      <c r="I28" s="27" t="n">
-        <v>-99.45</v>
+        <v>3.23</v>
+      </c>
+      <c r="I28" s="28" t="n">
+        <v>33.72</v>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="26" t="inlineStr">
         <is>
-          <t>코스나인</t>
+          <t>셀트리온</t>
         </is>
       </c>
       <c r="B29" s="25" t="n">
@@ -4026,25 +4024,25 @@
       </c>
       <c r="F29" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G29" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="H29" s="27" t="n">
-        <v>-23.08</v>
+        <v>-1.44</v>
       </c>
       <c r="I29" s="27" t="n">
-        <v>-97.92</v>
+        <v>-5.26</v>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="26" t="inlineStr">
         <is>
-          <t>헝셩그룹</t>
+          <t>수성웹툰</t>
         </is>
       </c>
       <c r="B30" s="25" t="n">
@@ -4061,305 +4059,301 @@
       </c>
       <c r="F30" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G30" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
-        </is>
-      </c>
-      <c r="H30" s="28" t="n">
-        <v>14.63</v>
-      </c>
-      <c r="I30" s="28" t="n">
-        <v>5.94</v>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="H30" s="27" t="n">
+        <v>-25.47</v>
+      </c>
+      <c r="I30" s="27" t="n">
+        <v>-49.62</v>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="26" t="inlineStr">
         <is>
-          <t>CG인바이츠</t>
+          <t>아티스트스튜디오</t>
         </is>
       </c>
       <c r="B31" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C31" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D31" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E31" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F31" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G31" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="H31" s="27" t="n">
-        <v>-4.7</v>
-      </c>
-      <c r="I31" s="28" t="n">
-        <v>7.32</v>
+        <v>-13.9</v>
+      </c>
+      <c r="I31" s="27" t="n">
+        <v>-8.789999999999999</v>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="26" t="inlineStr">
         <is>
-          <t>두산에너빌리티</t>
+          <t>전기차</t>
         </is>
       </c>
       <c r="B32" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C32" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D32" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E32" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F32" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G32" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
-        </is>
-      </c>
-      <c r="H32" s="28" t="n">
-        <v>1</v>
-      </c>
-      <c r="I32" s="28" t="n">
-        <v>14.65</v>
-      </c>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="H32" s="25" t="n"/>
+      <c r="I32" s="25" t="n"/>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="26" t="inlineStr">
         <is>
-          <t>머큐리</t>
+          <t>코다코</t>
         </is>
       </c>
       <c r="B33" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C33" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D33" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E33" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F33" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G33" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
-        </is>
-      </c>
-      <c r="H33" s="27" t="n">
-        <v>-4.43</v>
-      </c>
-      <c r="I33" s="28" t="n">
-        <v>39.71</v>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="H33" s="28" t="n">
+        <v>10.24</v>
+      </c>
+      <c r="I33" s="27" t="n">
+        <v>-99.45</v>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="26" t="inlineStr">
         <is>
-          <t>모아데이타</t>
+          <t>코스나인</t>
         </is>
       </c>
       <c r="B34" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C34" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D34" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E34" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F34" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G34" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="H34" s="27" t="n">
-        <v>-3.4</v>
+        <v>-23.08</v>
       </c>
       <c r="I34" s="27" t="n">
-        <v>-7.79</v>
+        <v>-97.92</v>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="26" t="inlineStr">
         <is>
-          <t>빛과전자</t>
+          <t>한국석유</t>
         </is>
       </c>
       <c r="B35" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C35" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D35" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E35" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F35" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G35" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="H35" s="27" t="n">
-        <v>-1.4</v>
+        <v>-3.22</v>
       </c>
       <c r="I35" s="28" t="n">
-        <v>42.54</v>
+        <v>8.83</v>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="26" t="inlineStr">
         <is>
-          <t>삼미금속</t>
+          <t>헝셩그룹</t>
         </is>
       </c>
       <c r="B36" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C36" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D36" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E36" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F36" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G36" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
-        </is>
-      </c>
-      <c r="H36" s="27" t="n">
-        <v>-2.69</v>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="H36" s="28" t="n">
+        <v>14.63</v>
       </c>
       <c r="I36" s="28" t="n">
-        <v>47.19</v>
+        <v>5.94</v>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="26" t="inlineStr">
         <is>
-          <t>삼성E&amp;A</t>
+          <t>혜인</t>
         </is>
       </c>
       <c r="B37" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C37" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D37" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E37" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F37" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G37" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="H37" s="28" t="n">
-        <v>1.19</v>
-      </c>
-      <c r="I37" s="28" t="n">
-        <v>11.23</v>
+        <v>3.85</v>
+      </c>
+      <c r="I37" s="27" t="n">
+        <v>-11.27</v>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="26" t="inlineStr">
         <is>
-          <t>삼성전자우</t>
+          <t>흥아해운</t>
         </is>
       </c>
       <c r="B38" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C38" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D38" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E38" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F38" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G38" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="H38" s="27" t="n">
-        <v>-4.78</v>
+        <v>-1.21</v>
       </c>
       <c r="I38" s="28" t="n">
-        <v>0.89</v>
+        <v>8.93</v>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="26" t="inlineStr">
         <is>
-          <t>샘표식품</t>
+          <t>머큐리</t>
         </is>
       </c>
       <c r="B39" s="25" t="n">
@@ -4376,25 +4370,25 @@
       </c>
       <c r="F39" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G39" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="H39" s="27" t="n">
-        <v>-14.76</v>
+        <v>-4.43</v>
       </c>
       <c r="I39" s="28" t="n">
-        <v>10.78</v>
+        <v>39.71</v>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="26" t="inlineStr">
         <is>
-          <t>서전기전</t>
+          <t>빛과전자</t>
         </is>
       </c>
       <c r="B40" s="25" t="n">
@@ -4411,25 +4405,25 @@
       </c>
       <c r="F40" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G40" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="H40" s="27" t="n">
-        <v>-3.51</v>
+        <v>-1.4</v>
       </c>
       <c r="I40" s="28" t="n">
-        <v>24.43</v>
+        <v>42.54</v>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="26" t="inlineStr">
         <is>
-          <t>수성웹툰</t>
+          <t>삼미금속</t>
         </is>
       </c>
       <c r="B41" s="25" t="n">
@@ -4446,25 +4440,25 @@
       </c>
       <c r="F41" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G41" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="H41" s="27" t="n">
-        <v>-25.47</v>
-      </c>
-      <c r="I41" s="27" t="n">
-        <v>-49.62</v>
+        <v>-2.69</v>
+      </c>
+      <c r="I41" s="28" t="n">
+        <v>47.19</v>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="26" t="inlineStr">
         <is>
-          <t>스트라드비젼</t>
+          <t>샘표식품</t>
         </is>
       </c>
       <c r="B42" s="25" t="n">
@@ -4481,25 +4475,25 @@
       </c>
       <c r="F42" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G42" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="H42" s="27" t="n">
-        <v>-0.39</v>
+        <v>-14.76</v>
       </c>
       <c r="I42" s="28" t="n">
-        <v>35.05</v>
+        <v>10.78</v>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="26" t="inlineStr">
         <is>
-          <t>액스비스</t>
+          <t>서전기전</t>
         </is>
       </c>
       <c r="B43" s="25" t="n">
@@ -4516,25 +4510,25 @@
       </c>
       <c r="F43" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G43" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
-        </is>
-      </c>
-      <c r="H43" s="28" t="n">
-        <v>11.97</v>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="H43" s="27" t="n">
+        <v>-3.51</v>
       </c>
       <c r="I43" s="28" t="n">
-        <v>57.45</v>
+        <v>24.43</v>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="26" t="inlineStr">
         <is>
-          <t>에스투더블유</t>
+          <t>액스비스</t>
         </is>
       </c>
       <c r="B44" s="25" t="n">
@@ -4551,25 +4545,25 @@
       </c>
       <c r="F44" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G44" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="H44" s="28" t="n">
-        <v>26.38</v>
+        <v>11.97</v>
       </c>
       <c r="I44" s="28" t="n">
-        <v>52.78</v>
+        <v>57.45</v>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="26" t="inlineStr">
         <is>
-          <t>엑스게이트</t>
+          <t>에스투더블유</t>
         </is>
       </c>
       <c r="B45" s="25" t="n">
@@ -4586,25 +4580,25 @@
       </c>
       <c r="F45" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G45" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="H45" s="28" t="n">
-        <v>29.94</v>
+        <v>26.38</v>
       </c>
       <c r="I45" s="28" t="n">
-        <v>40.51</v>
+        <v>52.78</v>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="26" t="inlineStr">
         <is>
-          <t>엔에이치스팩34호</t>
+          <t>엑스게이트</t>
         </is>
       </c>
       <c r="B46" s="25" t="n">
@@ -4621,25 +4615,25 @@
       </c>
       <c r="F46" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G46" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
-        </is>
-      </c>
-      <c r="H46" s="27" t="n">
-        <v>-6.94</v>
-      </c>
-      <c r="I46" s="27" t="n">
-        <v>-6.94</v>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="H46" s="28" t="n">
+        <v>29.94</v>
+      </c>
+      <c r="I46" s="28" t="n">
+        <v>40.51</v>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="26" t="inlineStr">
         <is>
-          <t>엠젠솔루션</t>
+          <t>엔에이치스팩34호</t>
         </is>
       </c>
       <c r="B47" s="25" t="n">
@@ -4656,19 +4650,19 @@
       </c>
       <c r="F47" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G47" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="H47" s="27" t="n">
-        <v>-8.75</v>
-      </c>
-      <c r="I47" s="28" t="n">
-        <v>15.63</v>
+        <v>-6.94</v>
+      </c>
+      <c r="I47" s="27" t="n">
+        <v>-6.94</v>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
@@ -4691,12 +4685,12 @@
       </c>
       <c r="F48" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G48" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="H48" s="27" t="n">
@@ -4709,7 +4703,7 @@
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="26" t="inlineStr">
         <is>
-          <t>원풍물산</t>
+          <t>원익피앤이</t>
         </is>
       </c>
       <c r="B49" s="25" t="n">
@@ -4726,19 +4720,19 @@
       </c>
       <c r="F49" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G49" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
-        </is>
-      </c>
-      <c r="H49" s="27" t="n">
-        <v>-1.47</v>
-      </c>
-      <c r="I49" s="27" t="n">
-        <v>-68.62</v>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="H49" s="28" t="n">
+        <v>6.62</v>
+      </c>
+      <c r="I49" s="28" t="n">
+        <v>41</v>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
@@ -4761,12 +4755,12 @@
       </c>
       <c r="F50" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G50" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="H50" s="27" t="n">
@@ -4779,7 +4773,7 @@
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="26" t="inlineStr">
         <is>
-          <t>한빛레이저</t>
+          <t>케이에스피</t>
         </is>
       </c>
       <c r="B51" s="25" t="n">
@@ -4796,25 +4790,25 @@
       </c>
       <c r="F51" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G51" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="H51" s="28" t="n">
-        <v>2.83</v>
+        <v>6.57</v>
       </c>
       <c r="I51" s="28" t="n">
-        <v>36.01</v>
+        <v>29.35</v>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="26" t="inlineStr">
         <is>
-          <t>흥아해운</t>
+          <t>한빛레이저</t>
         </is>
       </c>
       <c r="B52" s="25" t="n">
@@ -4831,19 +4825,19 @@
       </c>
       <c r="F52" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G52" s="25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
-        </is>
-      </c>
-      <c r="H52" s="27" t="n">
-        <v>-1.21</v>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="H52" s="28" t="n">
+        <v>2.83</v>
       </c>
       <c r="I52" s="28" t="n">
-        <v>8.93</v>
+        <v>36.01</v>
       </c>
     </row>
   </sheetData>
@@ -4927,19 +4921,19 @@
         <v>1</v>
       </c>
       <c r="C3" s="36" t="n">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="D3" s="36" t="n">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="E3" s="36" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="F3" s="37" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G3" s="37" t="inlineStr">
@@ -4958,19 +4952,19 @@
         <v>1</v>
       </c>
       <c r="C4" s="36" t="n">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="D4" s="36" t="n">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="E4" s="36" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="F4" s="37" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G4" s="37" t="inlineStr">
@@ -4996,12 +4990,12 @@
       </c>
       <c r="E5" s="36" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="F5" s="37" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G5" s="37" t="inlineStr">
@@ -5013,26 +5007,26 @@
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="35" t="inlineStr">
         <is>
-          <t>원전</t>
+          <t>방산</t>
         </is>
       </c>
       <c r="B6" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="36" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D6" s="36" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E6" s="36" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="F6" s="37" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G6" s="37" t="inlineStr">
@@ -5044,26 +5038,26 @@
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="35" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>원전</t>
         </is>
       </c>
       <c r="B7" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="36" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D7" s="36" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E7" s="36" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="F7" s="37" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G7" s="37" t="inlineStr">
@@ -5075,26 +5069,26 @@
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="35" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="B8" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="36" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="D8" s="36" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="E8" s="36" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="F8" s="37" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G8" s="37" t="inlineStr">
@@ -5106,65 +5100,69 @@
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="35" t="inlineStr">
         <is>
+          <t>제약</t>
+        </is>
+      </c>
+      <c r="B9" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" s="36" t="n">
+        <v>7</v>
+      </c>
+      <c r="D9" s="36" t="n">
+        <v>7</v>
+      </c>
+      <c r="E9" s="36" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="F9" s="37" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="G9" s="37" t="inlineStr">
+        <is>
+          <t>⚡ 관심</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="35" t="inlineStr">
+        <is>
           <t>인공지능</t>
         </is>
       </c>
-      <c r="B9" s="36" t="n">
-        <v>1</v>
-      </c>
-      <c r="C9" s="36" t="n">
-        <v>13</v>
-      </c>
-      <c r="D9" s="36" t="n">
-        <v>13</v>
-      </c>
-      <c r="E9" s="36" t="inlineStr">
-        <is>
-          <t>2026-09-12</t>
-        </is>
-      </c>
-      <c r="F9" s="37" t="inlineStr">
-        <is>
-          <t>2026-09-12</t>
-        </is>
-      </c>
-      <c r="G9" s="37" t="inlineStr">
+      <c r="B10" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" s="36" t="n">
+        <v>18</v>
+      </c>
+      <c r="D10" s="36" t="n">
+        <v>18</v>
+      </c>
+      <c r="E10" s="36" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="F10" s="37" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="G10" s="37" t="inlineStr">
         <is>
           <t>⚡ 관심</t>
         </is>
       </c>
-    </row>
-    <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="26" t="inlineStr">
-        <is>
-          <t>이차전지</t>
-        </is>
-      </c>
-      <c r="B10" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="C10" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="D10" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="E10" s="25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F10" s="29" t="inlineStr">
-        <is>
-          <t>감지 없음</t>
-        </is>
-      </c>
-      <c r="G10" s="29" t="inlineStr"/>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="26" t="inlineStr">
         <is>
-          <t>AI반도체</t>
+          <t>이차전지</t>
         </is>
       </c>
       <c r="B11" s="25" t="n">
@@ -5191,7 +5189,7 @@
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="26" t="inlineStr">
         <is>
-          <t>방산</t>
+          <t>AI반도체</t>
         </is>
       </c>
       <c r="B12" s="25" t="n">

</xml_diff>

<commit_message>
auto: 2026-09-14 07:08 자동 백업
</commit_message>
<xml_diff>
--- a/trend/stock_trend_history.xlsx
+++ b/trend/stock_trend_history.xlsx
@@ -694,7 +694,7 @@
     <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-09-13 06:54</t>
+          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-09-14 06:54</t>
         </is>
       </c>
     </row>
@@ -708,7 +708,7 @@
       </c>
       <c r="E3" s="3" t="n"/>
       <c r="G3" s="5" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="H3" s="3" t="n"/>
       <c r="J3" s="6" t="n">
@@ -787,21 +787,21 @@
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-09-13) 상위: 반도체  점수 48.0점</t>
+          <t>⚡ 최신(2026-09-14) 상위: 반도체  점수 52.0점</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-09-13) 상위: 인공지능  점수 18.0점</t>
+          <t>⚡ 최신(2026-09-14) 상위: 인공지능  점수 21.0점</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-09-13) 상위: 삼성전자  점수 15.0점</t>
+          <t>⚡ 최신(2026-09-14) 상위: 바이오  점수 18.0점</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="15" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B14" s="15" t="n">
@@ -928,10 +928,10 @@
         </is>
       </c>
       <c r="D14" s="15" t="n">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="E14" s="15" t="n">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="F14" s="15" t="n">
         <v>0</v>
@@ -947,7 +947,7 @@
       </c>
       <c r="J14" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
+          <t>매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K14" s="17" t="inlineStr">
@@ -959,7 +959,7 @@
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="15" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B15" s="15" t="n">
@@ -971,10 +971,10 @@
         </is>
       </c>
       <c r="D15" s="15" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E15" s="15" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="F15" s="15" t="n">
         <v>0</v>
@@ -990,7 +990,7 @@
       </c>
       <c r="J15" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+          <t>매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K15" s="17" t="inlineStr">
@@ -1002,7 +1002,7 @@
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="15" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B16" s="15" t="n">
@@ -1010,14 +1010,14 @@
       </c>
       <c r="C16" s="16" t="inlineStr">
         <is>
-          <t>삼성전자</t>
+          <t>바이오</t>
         </is>
       </c>
       <c r="D16" s="15" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="E16" s="15" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="F16" s="15" t="n">
         <v>0</v>
@@ -1025,25 +1025,27 @@
       <c r="G16" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H16" s="18" t="n">
-        <v>-3.53</v>
-      </c>
-      <c r="I16" s="19" t="n">
-        <v>1.57</v>
+      <c r="H16" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I16" s="15" t="n">
+        <v/>
       </c>
       <c r="J16" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K16" s="17" t="n">
-        <v/>
+          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 한국경제 헤드라인 언급 / 네이버뉴스 기사 언급</t>
+        </is>
+      </c>
+      <c r="K16" s="17" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B17" s="15" t="n">
@@ -1051,14 +1053,14 @@
       </c>
       <c r="C17" s="16" t="inlineStr">
         <is>
-          <t>바이오</t>
+          <t>삼성전자</t>
         </is>
       </c>
       <c r="D17" s="15" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="E17" s="15" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F17" s="15" t="n">
         <v>0</v>
@@ -1066,27 +1068,25 @@
       <c r="G17" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H17" s="15" t="n">
+      <c r="H17" s="18" t="n">
+        <v>-3.53</v>
+      </c>
+      <c r="I17" s="19" t="n">
+        <v>1.57</v>
+      </c>
+      <c r="J17" s="17" t="inlineStr">
+        <is>
+          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K17" s="17" t="n">
         <v/>
-      </c>
-      <c r="I17" s="15" t="n">
-        <v/>
-      </c>
-      <c r="J17" s="17" t="inlineStr">
-        <is>
-          <t>매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K17" s="17" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B18" s="15" t="n">
@@ -1094,14 +1094,14 @@
       </c>
       <c r="C18" s="16" t="inlineStr">
         <is>
-          <t>KB금융</t>
+          <t>LG</t>
         </is>
       </c>
       <c r="D18" s="15" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E18" s="15" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="F18" s="15" t="n">
         <v>0</v>
@@ -1109,25 +1109,27 @@
       <c r="G18" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H18" s="19" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="I18" s="19" t="n">
-        <v>3.43</v>
+      <c r="H18" s="18" t="n">
+        <v>-4.66</v>
+      </c>
+      <c r="I18" s="18" t="n">
+        <v>-7.1</v>
       </c>
       <c r="J18" s="17" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K18" s="17" t="n">
-        <v/>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K18" s="17" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B19" s="15" t="n">
@@ -1135,14 +1137,14 @@
       </c>
       <c r="C19" s="16" t="inlineStr">
         <is>
-          <t>LG</t>
+          <t>KB금융</t>
         </is>
       </c>
       <c r="D19" s="15" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E19" s="15" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="F19" s="15" t="n">
         <v>0</v>
@@ -1150,15 +1152,15 @@
       <c r="G19" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H19" s="18" t="n">
-        <v>-4.66</v>
-      </c>
-      <c r="I19" s="18" t="n">
-        <v>-7.1</v>
+      <c r="H19" s="19" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="I19" s="19" t="n">
+        <v>3.43</v>
       </c>
       <c r="J19" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K19" s="17" t="n">
@@ -1168,7 +1170,7 @@
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B20" s="15" t="n">
@@ -1176,14 +1178,14 @@
       </c>
       <c r="C20" s="16" t="inlineStr">
         <is>
-          <t>비에이치아이</t>
+          <t>원전</t>
         </is>
       </c>
       <c r="D20" s="15" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="E20" s="15" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="F20" s="15" t="n">
         <v>0</v>
@@ -1191,27 +1193,27 @@
       <c r="G20" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H20" s="19" t="n">
-        <v>2.24</v>
-      </c>
-      <c r="I20" s="19" t="n">
-        <v>14</v>
+      <c r="H20" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I20" s="15" t="n">
+        <v/>
       </c>
       <c r="J20" s="17" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 네이버뉴스 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K20" s="17" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="15" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B21" s="15" t="n">
@@ -1223,10 +1225,10 @@
         </is>
       </c>
       <c r="D21" s="15" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="E21" s="15" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="F21" s="15" t="n">
         <v>0</v>
@@ -1242,7 +1244,7 @@
       </c>
       <c r="J21" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 매일경제 기사 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K21" s="17" t="inlineStr">
@@ -1252,134 +1254,136 @@
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
-      <c r="A22" s="20" t="inlineStr">
-        <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="B22" s="20" t="n">
+      <c r="A22" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B22" s="15" t="n">
         <v>9</v>
       </c>
-      <c r="C22" s="21" t="inlineStr">
-        <is>
-          <t>더코디</t>
-        </is>
-      </c>
-      <c r="D22" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="E22" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="F22" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G22" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H22" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="I22" s="22" t="n">
-        <v>185.01</v>
-      </c>
-      <c r="J22" s="23" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +1153% / 중요공시 6건</t>
-        </is>
-      </c>
-      <c r="K22" s="23" t="inlineStr">
+      <c r="C22" s="16" t="inlineStr">
+        <is>
+          <t>삼성전자우</t>
+        </is>
+      </c>
+      <c r="D22" s="15" t="n">
+        <v>9</v>
+      </c>
+      <c r="E22" s="15" t="n">
+        <v>9</v>
+      </c>
+      <c r="F22" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" s="18" t="n">
+        <v>-4.78</v>
+      </c>
+      <c r="I22" s="19" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="J22" s="17" t="inlineStr">
+        <is>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K22" s="17" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="23" ht="18" customHeight="1">
+      <c r="A23" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B23" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="C23" s="16" t="inlineStr">
+        <is>
+          <t>셀트리온</t>
+        </is>
+      </c>
+      <c r="D23" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="E23" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="F23" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="H23" s="18" t="n">
+        <v>-1.44</v>
+      </c>
+      <c r="I23" s="18" t="n">
+        <v>-5.26</v>
+      </c>
+      <c r="J23" s="17" t="inlineStr">
+        <is>
+          <t>중요공시 2건 / 중요공시 7일 +100% / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급</t>
+        </is>
+      </c>
+      <c r="K23" s="17" t="inlineStr">
         <is>
           <t>네이버, 공시</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="20" t="inlineStr">
-        <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="B23" s="20" t="n">
-        <v>10</v>
-      </c>
-      <c r="C23" s="21" t="inlineStr">
-        <is>
-          <t>대한항공</t>
-        </is>
-      </c>
-      <c r="D23" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="E23" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="F23" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G23" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H23" s="24" t="n">
-        <v>-2.03</v>
-      </c>
-      <c r="I23" s="24" t="n">
-        <v>-4.14</v>
-      </c>
-      <c r="J23" s="23" t="inlineStr">
-        <is>
-          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K23" s="23" t="n">
-        <v/>
-      </c>
-    </row>
     <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="20" t="inlineStr">
-        <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="B24" s="20" t="n">
+      <c r="A24" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B24" s="15" t="n">
         <v>11</v>
       </c>
-      <c r="C24" s="21" t="inlineStr">
-        <is>
-          <t>SG</t>
-        </is>
-      </c>
-      <c r="D24" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="E24" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="F24" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G24" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H24" s="24" t="n">
-        <v>-5.34</v>
-      </c>
-      <c r="I24" s="22" t="n">
-        <v>6.45</v>
-      </c>
-      <c r="J24" s="23" t="inlineStr">
-        <is>
-          <t>한국경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K24" s="23" t="n">
-        <v/>
+      <c r="C24" s="16" t="inlineStr">
+        <is>
+          <t>DB</t>
+        </is>
+      </c>
+      <c r="D24" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="E24" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="F24" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" s="18" t="n">
+        <v>-0.06</v>
+      </c>
+      <c r="I24" s="19" t="n">
+        <v>9.42</v>
+      </c>
+      <c r="J24" s="17" t="inlineStr">
+        <is>
+          <t>Google 급상승 검색어 등장 (US) / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K24" s="17" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="20" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B25" s="20" t="n">
@@ -1387,42 +1391,42 @@
       </c>
       <c r="C25" s="21" t="inlineStr">
         <is>
-          <t>넥사다이내믹스</t>
+          <t>더코디</t>
         </is>
       </c>
       <c r="D25" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E25" s="20" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F25" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G25" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="H25" s="24" t="n">
-        <v>-3.61</v>
+        <v>0</v>
+      </c>
+      <c r="H25" s="20" t="n">
+        <v>0</v>
       </c>
       <c r="I25" s="22" t="n">
-        <v>7.65</v>
+        <v>185.01</v>
       </c>
       <c r="J25" s="23" t="inlineStr">
         <is>
-          <t>중요공시 5건 / 중요공시 7일 +400%</t>
+          <t>네이버 검색 당일 +1211% / 중요공시 6건</t>
         </is>
       </c>
       <c r="K25" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="20" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B26" s="20" t="n">
@@ -1430,7 +1434,7 @@
       </c>
       <c r="C26" s="21" t="inlineStr">
         <is>
-          <t>루멘스</t>
+          <t>에스투더블유</t>
         </is>
       </c>
       <c r="D26" s="20" t="n">
@@ -1446,26 +1450,26 @@
         <v>0</v>
       </c>
       <c r="H26" s="22" t="n">
-        <v>0.39</v>
-      </c>
-      <c r="I26" s="24" t="n">
-        <v>-5.58</v>
+        <v>26.38</v>
+      </c>
+      <c r="I26" s="22" t="n">
+        <v>52.78</v>
       </c>
       <c r="J26" s="23" t="inlineStr">
         <is>
-          <t>중요공시 5건 / 매일경제 헤드라인 언급</t>
+          <t>네이버 검색 당일 +451% / 네이버뉴스 헤드라인 언급</t>
         </is>
       </c>
       <c r="K26" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="20" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B27" s="20" t="n">
@@ -1473,42 +1477,40 @@
       </c>
       <c r="C27" s="21" t="inlineStr">
         <is>
-          <t>본느</t>
+          <t>LG디스플레이</t>
         </is>
       </c>
       <c r="D27" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E27" s="20" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F27" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G27" s="20" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H27" s="24" t="n">
-        <v>-11.52</v>
+        <v>-0.78</v>
       </c>
       <c r="I27" s="24" t="n">
-        <v>-7.67</v>
+        <v>-2.52</v>
       </c>
       <c r="J27" s="23" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 7일 +50%</t>
-        </is>
-      </c>
-      <c r="K27" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K27" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="20" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B28" s="20" t="n">
@@ -1516,7 +1518,7 @@
       </c>
       <c r="C28" s="21" t="inlineStr">
         <is>
-          <t>방산</t>
+          <t>루멘스</t>
         </is>
       </c>
       <c r="D28" s="20" t="n">
@@ -1531,25 +1533,27 @@
       <c r="G28" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H28" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I28" s="20" t="n">
-        <v/>
+      <c r="H28" s="22" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="I28" s="24" t="n">
+        <v>-5.58</v>
       </c>
       <c r="J28" s="23" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K28" s="23" t="n">
-        <v/>
+          <t>중요공시 5건 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K28" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="20" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B29" s="20" t="n">
@@ -1557,7 +1561,7 @@
       </c>
       <c r="C29" s="21" t="inlineStr">
         <is>
-          <t>비에이치</t>
+          <t>삼성전기</t>
         </is>
       </c>
       <c r="D29" s="20" t="n">
@@ -1572,27 +1576,25 @@
       <c r="G29" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H29" s="24" t="n">
-        <v>-1.25</v>
+      <c r="H29" s="20" t="n">
+        <v>0</v>
       </c>
       <c r="I29" s="24" t="n">
-        <v>-12.95</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="J29" s="23" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K29" s="23" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+          <t>매일경제 기사 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K29" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="20" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B30" s="20" t="n">
@@ -1600,7 +1602,7 @@
       </c>
       <c r="C30" s="21" t="inlineStr">
         <is>
-          <t>대우건설</t>
+          <t>방산</t>
         </is>
       </c>
       <c r="D30" s="20" t="n">
@@ -1615,27 +1617,25 @@
       <c r="G30" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H30" s="22" t="n">
-        <v>0.71</v>
-      </c>
-      <c r="I30" s="22" t="n">
-        <v>18.04</v>
+      <c r="H30" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I30" s="20" t="n">
+        <v/>
       </c>
       <c r="J30" s="23" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K30" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K30" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="20" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B31" s="20" t="n">
@@ -1643,14 +1643,14 @@
       </c>
       <c r="C31" s="21" t="inlineStr">
         <is>
-          <t>원전</t>
+          <t>코스나인</t>
         </is>
       </c>
       <c r="D31" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E31" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F31" s="20" t="n">
         <v>0</v>
@@ -1658,25 +1658,27 @@
       <c r="G31" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H31" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I31" s="20" t="n">
-        <v/>
+      <c r="H31" s="24" t="n">
+        <v>-23.08</v>
+      </c>
+      <c r="I31" s="24" t="n">
+        <v>-97.92</v>
       </c>
       <c r="J31" s="23" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K31" s="23" t="n">
-        <v/>
+          <t>네이버 검색 당일 +1239% / 중요공시 2건</t>
+        </is>
+      </c>
+      <c r="K31" s="23" t="inlineStr">
+        <is>
+          <t>네이버, 공시</t>
+        </is>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="20" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B32" s="20" t="n">
@@ -1684,7 +1686,7 @@
       </c>
       <c r="C32" s="21" t="inlineStr">
         <is>
-          <t>코스나인</t>
+          <t>코다코</t>
         </is>
       </c>
       <c r="D32" s="20" t="n">
@@ -1699,15 +1701,15 @@
       <c r="G32" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H32" s="24" t="n">
-        <v>-23.08</v>
+      <c r="H32" s="22" t="n">
+        <v>10.24</v>
       </c>
       <c r="I32" s="24" t="n">
-        <v>-97.92</v>
+        <v>-99.45</v>
       </c>
       <c r="J32" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +1174% / 중요공시 2건</t>
+          <t>네이버 검색 당일 +1086% / 중요공시 2건</t>
         </is>
       </c>
       <c r="K32" s="23" t="inlineStr">
@@ -1719,7 +1721,7 @@
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="20" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B33" s="20" t="n">
@@ -1727,7 +1729,7 @@
       </c>
       <c r="C33" s="21" t="inlineStr">
         <is>
-          <t>코다코</t>
+          <t>한국석유</t>
         </is>
       </c>
       <c r="D33" s="20" t="n">
@@ -1742,27 +1744,27 @@
       <c r="G33" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H33" s="22" t="n">
-        <v>10.24</v>
-      </c>
-      <c r="I33" s="24" t="n">
-        <v>-99.45</v>
+      <c r="H33" s="24" t="n">
+        <v>-3.22</v>
+      </c>
+      <c r="I33" s="22" t="n">
+        <v>8.83</v>
       </c>
       <c r="J33" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +994% / 중요공시 2건</t>
+          <t>네이버 검색 당일 +132% / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K33" s="23" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="20" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B34" s="20" t="n">
@@ -1770,7 +1772,7 @@
       </c>
       <c r="C34" s="21" t="inlineStr">
         <is>
-          <t>한국석유</t>
+          <t>수성웹툰</t>
         </is>
       </c>
       <c r="D34" s="20" t="n">
@@ -1786,26 +1788,26 @@
         <v>0</v>
       </c>
       <c r="H34" s="24" t="n">
-        <v>-3.22</v>
-      </c>
-      <c r="I34" s="22" t="n">
-        <v>8.83</v>
+        <v>-25.47</v>
+      </c>
+      <c r="I34" s="24" t="n">
+        <v>-49.62</v>
       </c>
       <c r="J34" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +122% / 매일경제 기사 언급</t>
+          <t>네이버 검색 당일 +132% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K34" s="23" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="20" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B35" s="20" t="n">
@@ -1813,7 +1815,7 @@
       </c>
       <c r="C35" s="21" t="inlineStr">
         <is>
-          <t>수성웹툰</t>
+          <t>원풍물산</t>
         </is>
       </c>
       <c r="D35" s="20" t="n">
@@ -1829,14 +1831,14 @@
         <v>0</v>
       </c>
       <c r="H35" s="24" t="n">
-        <v>-25.47</v>
+        <v>-1.47</v>
       </c>
       <c r="I35" s="24" t="n">
-        <v>-49.62</v>
+        <v>-68.62</v>
       </c>
       <c r="J35" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +121% / 중요공시 1건</t>
+          <t>네이버 검색 당일 +101% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K35" s="23" t="inlineStr">
@@ -1848,7 +1850,7 @@
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="20" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B36" s="20" t="n">
@@ -1856,40 +1858,42 @@
       </c>
       <c r="C36" s="21" t="inlineStr">
         <is>
-          <t>흥아해운</t>
+          <t>에넥스</t>
         </is>
       </c>
       <c r="D36" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E36" s="20" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F36" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G36" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H36" s="24" t="n">
-        <v>-1.21</v>
+        <v>3</v>
+      </c>
+      <c r="H36" s="22" t="n">
+        <v>10.85</v>
       </c>
       <c r="I36" s="22" t="n">
-        <v>8.93</v>
+        <v>14.32</v>
       </c>
       <c r="J36" s="23" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K36" s="23" t="n">
-        <v/>
+          <t>중요공시 2건 / 중요공시 7일 +100%</t>
+        </is>
+      </c>
+      <c r="K36" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="20" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B37" s="20" t="n">
@@ -1897,7 +1901,7 @@
       </c>
       <c r="C37" s="21" t="inlineStr">
         <is>
-          <t>삼성E&amp;A</t>
+          <t>삼성바이오로직스</t>
         </is>
       </c>
       <c r="D37" s="20" t="n">
@@ -1912,27 +1916,27 @@
       <c r="G37" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H37" s="22" t="n">
-        <v>1.19</v>
-      </c>
-      <c r="I37" s="22" t="n">
-        <v>11.23</v>
+      <c r="H37" s="24" t="n">
+        <v>-0.5600000000000001</v>
+      </c>
+      <c r="I37" s="24" t="n">
+        <v>-2.21</v>
       </c>
       <c r="J37" s="23" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 한국경제 헤드라인 언급</t>
+          <t>중요공시 2건 / 네이버뉴스 헤드라인 언급</t>
         </is>
       </c>
       <c r="K37" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="20" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B38" s="20" t="n">
@@ -1940,7 +1944,7 @@
       </c>
       <c r="C38" s="21" t="inlineStr">
         <is>
-          <t>대한광통신</t>
+          <t>아티스트스튜디오</t>
         </is>
       </c>
       <c r="D38" s="20" t="n">
@@ -1956,26 +1960,26 @@
         <v>0</v>
       </c>
       <c r="H38" s="24" t="n">
-        <v>-4</v>
-      </c>
-      <c r="I38" s="22" t="n">
-        <v>8.76</v>
+        <v>-13.9</v>
+      </c>
+      <c r="I38" s="24" t="n">
+        <v>-8.789999999999999</v>
       </c>
       <c r="J38" s="23" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급</t>
+          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K38" s="23" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="20" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B39" s="20" t="n">
@@ -1983,7 +1987,7 @@
       </c>
       <c r="C39" s="21" t="inlineStr">
         <is>
-          <t>헝셩그룹</t>
+          <t>KT</t>
         </is>
       </c>
       <c r="D39" s="20" t="n">
@@ -1999,26 +2003,24 @@
         <v>0</v>
       </c>
       <c r="H39" s="22" t="n">
-        <v>14.63</v>
-      </c>
-      <c r="I39" s="22" t="n">
-        <v>5.94</v>
+        <v>1.35</v>
+      </c>
+      <c r="I39" s="24" t="n">
+        <v>-2.95</v>
       </c>
       <c r="J39" s="23" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K39" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>매일경제 기사 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K39" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="20" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B40" s="20" t="n">
@@ -2026,421 +2028,427 @@
       </c>
       <c r="C40" s="21" t="inlineStr">
         <is>
-          <t>금호건설</t>
+          <t>현대차</t>
         </is>
       </c>
       <c r="D40" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E40" s="20" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F40" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G40" s="20" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H40" s="24" t="n">
-        <v>-2.19</v>
+        <v>-1.67</v>
       </c>
       <c r="I40" s="24" t="n">
-        <v>-8.58</v>
+        <v>-0.26</v>
       </c>
       <c r="J40" s="23" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 7일 +100%</t>
-        </is>
-      </c>
-      <c r="K40" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K40" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
-      <c r="A41" s="20" t="inlineStr">
-        <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="B41" s="20" t="n">
+      <c r="A41" s="25" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B41" s="25" t="n">
         <v>28</v>
       </c>
-      <c r="C41" s="21" t="inlineStr">
-        <is>
-          <t>셀트리온</t>
-        </is>
-      </c>
-      <c r="D41" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E41" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="F41" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G41" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="H41" s="24" t="n">
-        <v>-1.44</v>
-      </c>
-      <c r="I41" s="24" t="n">
-        <v>-5.26</v>
-      </c>
-      <c r="J41" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 2건 / 중요공시 7일 +100%</t>
-        </is>
-      </c>
-      <c r="K41" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
+      <c r="C41" s="26" t="inlineStr">
+        <is>
+          <t>삼미금속</t>
+        </is>
+      </c>
+      <c r="D41" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E41" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F41" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G41" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H41" s="27" t="n">
+        <v>-2.69</v>
+      </c>
+      <c r="I41" s="28" t="n">
+        <v>47.19</v>
+      </c>
+      <c r="J41" s="29" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +1091%</t>
+        </is>
+      </c>
+      <c r="K41" s="29" t="inlineStr">
+        <is>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
-      <c r="A42" s="20" t="inlineStr">
-        <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="B42" s="20" t="n">
+      <c r="A42" s="25" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B42" s="25" t="n">
         <v>29</v>
       </c>
-      <c r="C42" s="21" t="inlineStr">
-        <is>
-          <t>샘표</t>
-        </is>
-      </c>
-      <c r="D42" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E42" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F42" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G42" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H42" s="22" t="n">
-        <v>3.23</v>
-      </c>
-      <c r="I42" s="22" t="n">
-        <v>33.72</v>
-      </c>
-      <c r="J42" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 1건 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K42" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
+      <c r="C42" s="26" t="inlineStr">
+        <is>
+          <t>액스비스</t>
+        </is>
+      </c>
+      <c r="D42" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E42" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F42" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G42" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H42" s="28" t="n">
+        <v>11.97</v>
+      </c>
+      <c r="I42" s="28" t="n">
+        <v>57.45</v>
+      </c>
+      <c r="J42" s="29" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +784%</t>
+        </is>
+      </c>
+      <c r="K42" s="29" t="inlineStr">
+        <is>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
-      <c r="A43" s="20" t="inlineStr">
-        <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="B43" s="20" t="n">
+      <c r="A43" s="25" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B43" s="25" t="n">
         <v>30</v>
       </c>
-      <c r="C43" s="21" t="inlineStr">
-        <is>
-          <t>아티스트스튜디오</t>
-        </is>
-      </c>
-      <c r="D43" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E43" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F43" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G43" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H43" s="24" t="n">
-        <v>-13.9</v>
-      </c>
-      <c r="I43" s="24" t="n">
-        <v>-8.789999999999999</v>
-      </c>
-      <c r="J43" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K43" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
+      <c r="C43" s="26" t="inlineStr">
+        <is>
+          <t>샘표식품</t>
+        </is>
+      </c>
+      <c r="D43" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E43" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F43" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G43" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H43" s="27" t="n">
+        <v>-14.76</v>
+      </c>
+      <c r="I43" s="28" t="n">
+        <v>10.78</v>
+      </c>
+      <c r="J43" s="29" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +713%</t>
+        </is>
+      </c>
+      <c r="K43" s="29" t="inlineStr">
+        <is>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
-      <c r="A44" s="20" t="inlineStr">
-        <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="B44" s="20" t="n">
+      <c r="A44" s="25" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B44" s="25" t="n">
         <v>31</v>
       </c>
-      <c r="C44" s="21" t="inlineStr">
-        <is>
-          <t>바이오비쥬</t>
-        </is>
-      </c>
-      <c r="D44" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E44" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F44" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G44" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H44" s="22" t="n">
-        <v>7.28</v>
-      </c>
-      <c r="I44" s="22" t="n">
-        <v>5.46</v>
-      </c>
-      <c r="J44" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K44" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
+      <c r="C44" s="26" t="inlineStr">
+        <is>
+          <t>엔에이치스팩34호</t>
+        </is>
+      </c>
+      <c r="D44" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E44" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F44" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G44" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H44" s="27" t="n">
+        <v>-6.94</v>
+      </c>
+      <c r="I44" s="27" t="n">
+        <v>-6.94</v>
+      </c>
+      <c r="J44" s="29" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +496%</t>
+        </is>
+      </c>
+      <c r="K44" s="29" t="inlineStr">
+        <is>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
-      <c r="A45" s="20" t="inlineStr">
-        <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="B45" s="20" t="n">
+      <c r="A45" s="25" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B45" s="25" t="n">
         <v>32</v>
       </c>
-      <c r="C45" s="21" t="inlineStr">
-        <is>
-          <t>넥써쓰</t>
-        </is>
-      </c>
-      <c r="D45" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E45" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F45" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G45" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H45" s="22" t="n">
-        <v>2.08</v>
-      </c>
-      <c r="I45" s="22" t="n">
-        <v>5.99</v>
-      </c>
-      <c r="J45" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K45" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
+      <c r="C45" s="26" t="inlineStr">
+        <is>
+          <t>카프로</t>
+        </is>
+      </c>
+      <c r="D45" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E45" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F45" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H45" s="27" t="n">
+        <v>-16.67</v>
+      </c>
+      <c r="I45" s="27" t="n">
+        <v>-96.72</v>
+      </c>
+      <c r="J45" s="29" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +487%</t>
+        </is>
+      </c>
+      <c r="K45" s="29" t="inlineStr">
+        <is>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
-      <c r="A46" s="20" t="inlineStr">
-        <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="B46" s="20" t="n">
+      <c r="A46" s="25" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B46" s="25" t="n">
         <v>33</v>
       </c>
-      <c r="C46" s="21" t="inlineStr">
-        <is>
-          <t>로봇</t>
-        </is>
-      </c>
-      <c r="D46" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E46" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F46" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G46" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H46" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I46" s="20" t="n">
-        <v/>
-      </c>
-      <c r="J46" s="23" t="inlineStr">
-        <is>
-          <t>매일경제 기사 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K46" s="23" t="n">
-        <v/>
+      <c r="C46" s="26" t="inlineStr">
+        <is>
+          <t>서전기전</t>
+        </is>
+      </c>
+      <c r="D46" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E46" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F46" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G46" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H46" s="27" t="n">
+        <v>-3.51</v>
+      </c>
+      <c r="I46" s="28" t="n">
+        <v>24.43</v>
+      </c>
+      <c r="J46" s="29" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +410%</t>
+        </is>
+      </c>
+      <c r="K46" s="29" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
-      <c r="A47" s="20" t="inlineStr">
-        <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="B47" s="20" t="n">
+      <c r="A47" s="25" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B47" s="25" t="n">
         <v>34</v>
       </c>
-      <c r="C47" s="21" t="inlineStr">
-        <is>
-          <t>로보티즈</t>
-        </is>
-      </c>
-      <c r="D47" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E47" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F47" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G47" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H47" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="I47" s="22" t="n">
-        <v>6.24</v>
-      </c>
-      <c r="J47" s="23" t="inlineStr">
-        <is>
-          <t>매일경제 기사 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K47" s="23" t="n">
-        <v/>
+      <c r="C47" s="26" t="inlineStr">
+        <is>
+          <t>머큐리</t>
+        </is>
+      </c>
+      <c r="D47" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E47" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F47" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H47" s="27" t="n">
+        <v>-4.43</v>
+      </c>
+      <c r="I47" s="28" t="n">
+        <v>39.71</v>
+      </c>
+      <c r="J47" s="29" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +380%</t>
+        </is>
+      </c>
+      <c r="K47" s="29" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
-      <c r="A48" s="20" t="inlineStr">
-        <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="B48" s="20" t="n">
+      <c r="A48" s="25" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B48" s="25" t="n">
         <v>35</v>
       </c>
-      <c r="C48" s="21" t="inlineStr">
-        <is>
-          <t>전기차</t>
-        </is>
-      </c>
-      <c r="D48" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E48" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F48" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G48" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H48" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I48" s="20" t="n">
-        <v/>
-      </c>
-      <c r="J48" s="23" t="inlineStr">
-        <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K48" s="23" t="n">
-        <v/>
+      <c r="C48" s="26" t="inlineStr">
+        <is>
+          <t>오르비텍</t>
+        </is>
+      </c>
+      <c r="D48" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E48" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F48" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G48" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H48" s="27" t="n">
+        <v>-3.34</v>
+      </c>
+      <c r="I48" s="28" t="n">
+        <v>40.35</v>
+      </c>
+      <c r="J48" s="29" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +307%</t>
+        </is>
+      </c>
+      <c r="K48" s="29" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
-      <c r="A49" s="20" t="inlineStr">
-        <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="B49" s="20" t="n">
+      <c r="A49" s="25" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B49" s="25" t="n">
         <v>36</v>
       </c>
-      <c r="C49" s="21" t="inlineStr">
-        <is>
-          <t>혜인</t>
-        </is>
-      </c>
-      <c r="D49" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E49" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F49" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G49" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H49" s="22" t="n">
-        <v>3.85</v>
-      </c>
-      <c r="I49" s="24" t="n">
-        <v>-11.27</v>
-      </c>
-      <c r="J49" s="23" t="inlineStr">
-        <is>
-          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K49" s="23" t="n">
-        <v/>
+      <c r="C49" s="26" t="inlineStr">
+        <is>
+          <t>한빛레이저</t>
+        </is>
+      </c>
+      <c r="D49" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E49" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F49" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G49" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H49" s="28" t="n">
+        <v>2.83</v>
+      </c>
+      <c r="I49" s="28" t="n">
+        <v>36.01</v>
+      </c>
+      <c r="J49" s="29" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +282%</t>
+        </is>
+      </c>
+      <c r="K49" s="29" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B50" s="25" t="n">
@@ -2448,7 +2456,7 @@
       </c>
       <c r="C50" s="26" t="inlineStr">
         <is>
-          <t>삼미금속</t>
+          <t>엑스게이트</t>
         </is>
       </c>
       <c r="D50" s="25" t="n">
@@ -2463,15 +2471,15 @@
       <c r="G50" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H50" s="27" t="n">
-        <v>-2.69</v>
+      <c r="H50" s="28" t="n">
+        <v>29.94</v>
       </c>
       <c r="I50" s="28" t="n">
-        <v>47.19</v>
+        <v>40.51</v>
       </c>
       <c r="J50" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +1054%</t>
+          <t>네이버 검색 당일 +236%</t>
         </is>
       </c>
       <c r="K50" s="29" t="inlineStr">
@@ -2483,7 +2491,7 @@
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B51" s="25" t="n">
@@ -2491,7 +2499,7 @@
       </c>
       <c r="C51" s="26" t="inlineStr">
         <is>
-          <t>액스비스</t>
+          <t>원익피앤이</t>
         </is>
       </c>
       <c r="D51" s="25" t="n">
@@ -2507,14 +2515,14 @@
         <v>0</v>
       </c>
       <c r="H51" s="28" t="n">
-        <v>11.97</v>
+        <v>6.62</v>
       </c>
       <c r="I51" s="28" t="n">
-        <v>57.45</v>
+        <v>41</v>
       </c>
       <c r="J51" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +735%</t>
+          <t>네이버 검색 당일 +220%</t>
         </is>
       </c>
       <c r="K51" s="29" t="inlineStr">
@@ -2526,7 +2534,7 @@
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B52" s="25" t="n">
@@ -2534,7 +2542,7 @@
       </c>
       <c r="C52" s="26" t="inlineStr">
         <is>
-          <t>샘표식품</t>
+          <t>빛과전자</t>
         </is>
       </c>
       <c r="D52" s="25" t="n">
@@ -2550,14 +2558,14 @@
         <v>0</v>
       </c>
       <c r="H52" s="27" t="n">
-        <v>-14.76</v>
+        <v>-1.4</v>
       </c>
       <c r="I52" s="28" t="n">
-        <v>10.78</v>
+        <v>42.54</v>
       </c>
       <c r="J52" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +663%</t>
+          <t>네이버 검색 당일 +211%</t>
         </is>
       </c>
       <c r="K52" s="29" t="inlineStr">
@@ -2569,7 +2577,7 @@
     <row r="53" ht="18" customHeight="1">
       <c r="A53" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B53" s="25" t="n">
@@ -2577,7 +2585,7 @@
       </c>
       <c r="C53" s="26" t="inlineStr">
         <is>
-          <t>엔에이치스팩34호</t>
+          <t>케이에스피</t>
         </is>
       </c>
       <c r="D53" s="25" t="n">
@@ -2592,15 +2600,15 @@
       <c r="G53" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H53" s="27" t="n">
-        <v>-6.94</v>
-      </c>
-      <c r="I53" s="27" t="n">
-        <v>-6.94</v>
+      <c r="H53" s="28" t="n">
+        <v>6.57</v>
+      </c>
+      <c r="I53" s="28" t="n">
+        <v>29.35</v>
       </c>
       <c r="J53" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +486%</t>
+          <t>네이버 검색 당일 +198%</t>
         </is>
       </c>
       <c r="K53" s="29" t="inlineStr">
@@ -2612,7 +2620,7 @@
     <row r="54" ht="18" customHeight="1">
       <c r="A54" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B54" s="25" t="n">
@@ -2620,7 +2628,7 @@
       </c>
       <c r="C54" s="26" t="inlineStr">
         <is>
-          <t>카프로</t>
+          <t>샌즈랩</t>
         </is>
       </c>
       <c r="D54" s="25" t="n">
@@ -2635,15 +2643,15 @@
       <c r="G54" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H54" s="27" t="n">
-        <v>-16.67</v>
-      </c>
-      <c r="I54" s="27" t="n">
-        <v>-96.72</v>
+      <c r="H54" s="28" t="n">
+        <v>29.8</v>
+      </c>
+      <c r="I54" s="28" t="n">
+        <v>31.03</v>
       </c>
       <c r="J54" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +470%</t>
+          <t>네이버 검색 당일 +193%</t>
         </is>
       </c>
       <c r="K54" s="29" t="inlineStr">
@@ -2655,7 +2663,7 @@
     <row r="55" ht="18" customHeight="1">
       <c r="A55" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B55" s="25" t="n">
@@ -2663,7 +2671,7 @@
       </c>
       <c r="C55" s="26" t="inlineStr">
         <is>
-          <t>에스투더블유</t>
+          <t>피아이이</t>
         </is>
       </c>
       <c r="D55" s="25" t="n">
@@ -2679,14 +2687,14 @@
         <v>0</v>
       </c>
       <c r="H55" s="28" t="n">
-        <v>26.38</v>
+        <v>7.61</v>
       </c>
       <c r="I55" s="28" t="n">
-        <v>52.78</v>
+        <v>37.84</v>
       </c>
       <c r="J55" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +403%</t>
+          <t>네이버 검색 당일 +178%</t>
         </is>
       </c>
       <c r="K55" s="29" t="inlineStr">
@@ -2698,7 +2706,7 @@
     <row r="56" ht="18" customHeight="1">
       <c r="A56" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B56" s="25" t="n">
@@ -2706,7 +2714,7 @@
       </c>
       <c r="C56" s="26" t="inlineStr">
         <is>
-          <t>서전기전</t>
+          <t>스트라드비젼</t>
         </is>
       </c>
       <c r="D56" s="25" t="n">
@@ -2722,14 +2730,14 @@
         <v>0</v>
       </c>
       <c r="H56" s="27" t="n">
-        <v>-3.51</v>
+        <v>-0.39</v>
       </c>
       <c r="I56" s="28" t="n">
-        <v>24.43</v>
+        <v>35.05</v>
       </c>
       <c r="J56" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +398%</t>
+          <t>네이버 검색 당일 +168%</t>
         </is>
       </c>
       <c r="K56" s="29" t="inlineStr">
@@ -2741,7 +2749,7 @@
     <row r="57" ht="18" customHeight="1">
       <c r="A57" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B57" s="25" t="n">
@@ -2749,7 +2757,7 @@
       </c>
       <c r="C57" s="26" t="inlineStr">
         <is>
-          <t>머큐리</t>
+          <t>금강철강</t>
         </is>
       </c>
       <c r="D57" s="25" t="n">
@@ -2764,15 +2772,15 @@
       <c r="G57" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H57" s="27" t="n">
-        <v>-4.43</v>
+      <c r="H57" s="28" t="n">
+        <v>2.34</v>
       </c>
       <c r="I57" s="28" t="n">
-        <v>39.71</v>
+        <v>30.51</v>
       </c>
       <c r="J57" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +359%</t>
+          <t>네이버 검색 당일 +165%</t>
         </is>
       </c>
       <c r="K57" s="29" t="inlineStr">
@@ -2784,7 +2792,7 @@
     <row r="58" ht="18" customHeight="1">
       <c r="A58" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B58" s="25" t="n">
@@ -2792,7 +2800,7 @@
       </c>
       <c r="C58" s="26" t="inlineStr">
         <is>
-          <t>오르비텍</t>
+          <t>우리로</t>
         </is>
       </c>
       <c r="D58" s="25" t="n">
@@ -2807,15 +2815,15 @@
       <c r="G58" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H58" s="27" t="n">
-        <v>-3.34</v>
+      <c r="H58" s="28" t="n">
+        <v>7.31</v>
       </c>
       <c r="I58" s="28" t="n">
-        <v>40.35</v>
+        <v>48.55</v>
       </c>
       <c r="J58" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +296%</t>
+          <t>네이버 검색 당일 +161%</t>
         </is>
       </c>
       <c r="K58" s="29" t="inlineStr">
@@ -2827,7 +2835,7 @@
     <row r="59" ht="18" customHeight="1">
       <c r="A59" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B59" s="25" t="n">
@@ -2835,7 +2843,7 @@
       </c>
       <c r="C59" s="26" t="inlineStr">
         <is>
-          <t>한빛레이저</t>
+          <t>우리넷</t>
         </is>
       </c>
       <c r="D59" s="25" t="n">
@@ -2851,14 +2859,14 @@
         <v>0</v>
       </c>
       <c r="H59" s="28" t="n">
-        <v>2.83</v>
+        <v>3.49</v>
       </c>
       <c r="I59" s="28" t="n">
-        <v>36.01</v>
+        <v>15.6</v>
       </c>
       <c r="J59" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +273%</t>
+          <t>네이버 검색 당일 +158%</t>
         </is>
       </c>
       <c r="K59" s="29" t="inlineStr">
@@ -2870,7 +2878,7 @@
     <row r="60" ht="18" customHeight="1">
       <c r="A60" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B60" s="25" t="n">
@@ -2878,7 +2886,7 @@
       </c>
       <c r="C60" s="26" t="inlineStr">
         <is>
-          <t>빛과전자</t>
+          <t>아모텍</t>
         </is>
       </c>
       <c r="D60" s="25" t="n">
@@ -2893,15 +2901,15 @@
       <c r="G60" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H60" s="27" t="n">
-        <v>-1.4</v>
+      <c r="H60" s="28" t="n">
+        <v>29.98</v>
       </c>
       <c r="I60" s="28" t="n">
-        <v>42.54</v>
+        <v>34.01</v>
       </c>
       <c r="J60" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +204%</t>
+          <t>네이버 검색 당일 +140%</t>
         </is>
       </c>
       <c r="K60" s="29" t="inlineStr">
@@ -2913,7 +2921,7 @@
     <row r="61" ht="18" customHeight="1">
       <c r="A61" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B61" s="25" t="n">
@@ -2921,7 +2929,7 @@
       </c>
       <c r="C61" s="26" t="inlineStr">
         <is>
-          <t>원익피앤이</t>
+          <t>드림시큐리티</t>
         </is>
       </c>
       <c r="D61" s="25" t="n">
@@ -2937,14 +2945,14 @@
         <v>0</v>
       </c>
       <c r="H61" s="28" t="n">
-        <v>6.62</v>
+        <v>23.29</v>
       </c>
       <c r="I61" s="28" t="n">
-        <v>41</v>
+        <v>29.38</v>
       </c>
       <c r="J61" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +200%</t>
+          <t>네이버 검색 당일 +124%</t>
         </is>
       </c>
       <c r="K61" s="29" t="inlineStr">
@@ -2956,7 +2964,7 @@
     <row r="62" ht="18" customHeight="1">
       <c r="A62" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B62" s="25" t="n">
@@ -2964,7 +2972,7 @@
       </c>
       <c r="C62" s="26" t="inlineStr">
         <is>
-          <t>엑스게이트</t>
+          <t>넥스틸</t>
         </is>
       </c>
       <c r="D62" s="25" t="n">
@@ -2980,14 +2988,14 @@
         <v>0</v>
       </c>
       <c r="H62" s="28" t="n">
-        <v>29.94</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="I62" s="28" t="n">
-        <v>40.51</v>
+        <v>10.7</v>
       </c>
       <c r="J62" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +198%</t>
+          <t>네이버 검색 당일 +118%</t>
         </is>
       </c>
       <c r="K62" s="29" t="inlineStr">
@@ -2999,7 +3007,7 @@
     <row r="63" ht="18" customHeight="1">
       <c r="A63" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B63" s="25" t="n">
@@ -3007,7 +3015,7 @@
       </c>
       <c r="C63" s="26" t="inlineStr">
         <is>
-          <t>케이에스피</t>
+          <t>우리기술</t>
         </is>
       </c>
       <c r="D63" s="25" t="n">
@@ -3022,15 +3030,15 @@
       <c r="G63" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H63" s="28" t="n">
-        <v>6.57</v>
+      <c r="H63" s="27" t="n">
+        <v>-3.77</v>
       </c>
       <c r="I63" s="28" t="n">
-        <v>29.35</v>
+        <v>32.17</v>
       </c>
       <c r="J63" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +183%</t>
+          <t>네이버 검색 당일 +115%</t>
         </is>
       </c>
       <c r="K63" s="29" t="inlineStr">
@@ -3132,22 +3140,22 @@
         <v>1</v>
       </c>
       <c r="C3" s="25" t="n">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="D3" s="25" t="n">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="E3" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F3" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G3" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="H3" s="25" t="n"/>
@@ -3163,22 +3171,22 @@
         <v>1</v>
       </c>
       <c r="C4" s="25" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="D4" s="25" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E4" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F4" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G4" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="H4" s="25" t="n"/>
@@ -3194,22 +3202,22 @@
         <v>1</v>
       </c>
       <c r="C5" s="25" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="D5" s="25" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="E5" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F5" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G5" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="H5" s="25" t="n"/>
@@ -3218,142 +3226,138 @@
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="26" t="inlineStr">
         <is>
-          <t>삼성전자</t>
+          <t>LG</t>
         </is>
       </c>
       <c r="B6" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="25" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D6" s="25" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="E6" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F6" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G6" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="H6" s="27" t="n">
-        <v>-3.53</v>
-      </c>
-      <c r="I6" s="28" t="n">
-        <v>1.57</v>
+        <v>-4.66</v>
+      </c>
+      <c r="I6" s="27" t="n">
+        <v>-7.1</v>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="26" t="inlineStr">
         <is>
-          <t>KB금융</t>
+          <t>삼성전자</t>
         </is>
       </c>
       <c r="B7" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="25" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D7" s="25" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E7" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F7" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G7" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="H7" s="28" t="n">
-        <v>2.6</v>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="H7" s="27" t="n">
+        <v>-3.53</v>
       </c>
       <c r="I7" s="28" t="n">
-        <v>3.43</v>
+        <v>1.57</v>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="26" t="inlineStr">
         <is>
-          <t>LG</t>
+          <t>KB금융</t>
         </is>
       </c>
       <c r="B8" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="25" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="D8" s="25" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E8" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F8" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G8" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="H8" s="27" t="n">
-        <v>-4.66</v>
-      </c>
-      <c r="I8" s="27" t="n">
-        <v>-7.1</v>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="H8" s="28" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="I8" s="28" t="n">
+        <v>3.43</v>
       </c>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="26" t="inlineStr">
         <is>
-          <t>비에이치아이</t>
+          <t>원전</t>
         </is>
       </c>
       <c r="B9" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="25" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="D9" s="25" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="E9" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F9" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G9" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="H9" s="28" t="n">
-        <v>2.24</v>
-      </c>
-      <c r="I9" s="28" t="n">
-        <v>14</v>
-      </c>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="H9" s="25" t="n"/>
+      <c r="I9" s="25" t="n"/>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="26" t="inlineStr">
@@ -3365,22 +3369,22 @@
         <v>1</v>
       </c>
       <c r="C10" s="25" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="D10" s="25" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="E10" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F10" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G10" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="H10" s="25" t="n"/>
@@ -3389,112 +3393,112 @@
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="26" t="inlineStr">
         <is>
-          <t>SG</t>
+          <t>삼성전자우</t>
         </is>
       </c>
       <c r="B11" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="25" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D11" s="25" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E11" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F11" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G11" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="H11" s="27" t="n">
-        <v>-5.34</v>
+        <v>-4.78</v>
       </c>
       <c r="I11" s="28" t="n">
-        <v>6.45</v>
+        <v>0.89</v>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="26" t="inlineStr">
         <is>
-          <t>넥사다이내믹스</t>
+          <t>DB</t>
         </is>
       </c>
       <c r="B12" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C12" s="25" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D12" s="25" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E12" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F12" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G12" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="H12" s="27" t="n">
-        <v>-3.61</v>
+        <v>-0.06</v>
       </c>
       <c r="I12" s="28" t="n">
-        <v>7.65</v>
+        <v>9.42</v>
       </c>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>대한항공</t>
+          <t>셀트리온</t>
         </is>
       </c>
       <c r="B13" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C13" s="25" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D13" s="25" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E13" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F13" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G13" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="H13" s="27" t="n">
-        <v>-2.03</v>
+        <v>-1.44</v>
       </c>
       <c r="I13" s="27" t="n">
-        <v>-4.14</v>
+        <v>-5.26</v>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>더코디</t>
+          <t>LG디스플레이</t>
         </is>
       </c>
       <c r="B14" s="25" t="n">
@@ -3511,25 +3515,25 @@
       </c>
       <c r="F14" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G14" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="H14" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="I14" s="28" t="n">
-        <v>185.01</v>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="H14" s="27" t="n">
+        <v>-0.78</v>
+      </c>
+      <c r="I14" s="27" t="n">
+        <v>-2.52</v>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>루멘스</t>
+          <t>더코디</t>
         </is>
       </c>
       <c r="B15" s="25" t="n">
@@ -3546,25 +3550,25 @@
       </c>
       <c r="F15" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G15" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="H15" s="28" t="n">
-        <v>0.39</v>
-      </c>
-      <c r="I15" s="27" t="n">
-        <v>-5.58</v>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="H15" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="28" t="n">
+        <v>185.01</v>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>방산</t>
+          <t>루멘스</t>
         </is>
       </c>
       <c r="B16" s="25" t="n">
@@ -3581,21 +3585,25 @@
       </c>
       <c r="F16" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G16" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="H16" s="25" t="n"/>
-      <c r="I16" s="25" t="n"/>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="H16" s="28" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="I16" s="27" t="n">
+        <v>-5.58</v>
+      </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>본느</t>
+          <t>삼성전기</t>
         </is>
       </c>
       <c r="B17" s="25" t="n">
@@ -3612,25 +3620,25 @@
       </c>
       <c r="F17" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G17" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="H17" s="27" t="n">
-        <v>-11.52</v>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="H17" s="25" t="n">
+        <v>0</v>
       </c>
       <c r="I17" s="27" t="n">
-        <v>-7.67</v>
+        <v>-0.07000000000000001</v>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="26" t="inlineStr">
         <is>
-          <t>비에이치</t>
+          <t>에스투더블유</t>
         </is>
       </c>
       <c r="B18" s="25" t="n">
@@ -3647,25 +3655,25 @@
       </c>
       <c r="F18" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G18" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="H18" s="27" t="n">
-        <v>-1.25</v>
-      </c>
-      <c r="I18" s="27" t="n">
-        <v>-12.95</v>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="H18" s="28" t="n">
+        <v>26.38</v>
+      </c>
+      <c r="I18" s="28" t="n">
+        <v>52.78</v>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>대우건설</t>
+          <t>방산</t>
         </is>
       </c>
       <c r="B19" s="25" t="n">
@@ -3682,56 +3690,56 @@
       </c>
       <c r="F19" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G19" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="H19" s="28" t="n">
-        <v>0.71</v>
-      </c>
-      <c r="I19" s="28" t="n">
-        <v>18.04</v>
-      </c>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="H19" s="25" t="n"/>
+      <c r="I19" s="25" t="n"/>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="26" t="inlineStr">
         <is>
-          <t>원전</t>
+          <t>KT</t>
         </is>
       </c>
       <c r="B20" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C20" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D20" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E20" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F20" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G20" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="H20" s="25" t="n"/>
-      <c r="I20" s="25" t="n"/>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="H20" s="28" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="I20" s="27" t="n">
+        <v>-2.95</v>
+      </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="26" t="inlineStr">
         <is>
-          <t>금호건설</t>
+          <t>삼성바이오로직스</t>
         </is>
       </c>
       <c r="B21" s="25" t="n">
@@ -3748,25 +3756,25 @@
       </c>
       <c r="F21" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G21" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="H21" s="27" t="n">
-        <v>-2.19</v>
+        <v>-0.5600000000000001</v>
       </c>
       <c r="I21" s="27" t="n">
-        <v>-8.58</v>
+        <v>-2.21</v>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="26" t="inlineStr">
         <is>
-          <t>넥써쓰</t>
+          <t>수성웹툰</t>
         </is>
       </c>
       <c r="B22" s="25" t="n">
@@ -3783,25 +3791,25 @@
       </c>
       <c r="F22" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G22" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="H22" s="28" t="n">
-        <v>2.08</v>
-      </c>
-      <c r="I22" s="28" t="n">
-        <v>5.99</v>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="H22" s="27" t="n">
+        <v>-25.47</v>
+      </c>
+      <c r="I22" s="27" t="n">
+        <v>-49.62</v>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="26" t="inlineStr">
         <is>
-          <t>대한광통신</t>
+          <t>아티스트스튜디오</t>
         </is>
       </c>
       <c r="B23" s="25" t="n">
@@ -3818,25 +3826,25 @@
       </c>
       <c r="F23" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G23" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="H23" s="27" t="n">
-        <v>-4</v>
-      </c>
-      <c r="I23" s="28" t="n">
-        <v>8.76</v>
+        <v>-13.9</v>
+      </c>
+      <c r="I23" s="27" t="n">
+        <v>-8.789999999999999</v>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="26" t="inlineStr">
         <is>
-          <t>로보티즈</t>
+          <t>에넥스</t>
         </is>
       </c>
       <c r="B24" s="25" t="n">
@@ -3853,25 +3861,25 @@
       </c>
       <c r="F24" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G24" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="H24" s="25" t="n">
-        <v>0</v>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="H24" s="28" t="n">
+        <v>10.85</v>
       </c>
       <c r="I24" s="28" t="n">
-        <v>6.24</v>
+        <v>14.32</v>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="26" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>원풍물산</t>
         </is>
       </c>
       <c r="B25" s="25" t="n">
@@ -3888,21 +3896,25 @@
       </c>
       <c r="F25" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G25" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="H25" s="25" t="n"/>
-      <c r="I25" s="25" t="n"/>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="H25" s="27" t="n">
+        <v>-1.47</v>
+      </c>
+      <c r="I25" s="27" t="n">
+        <v>-68.62</v>
+      </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="26" t="inlineStr">
         <is>
-          <t>바이오비쥬</t>
+          <t>코다코</t>
         </is>
       </c>
       <c r="B26" s="25" t="n">
@@ -3919,25 +3931,25 @@
       </c>
       <c r="F26" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G26" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="H26" s="28" t="n">
-        <v>7.28</v>
-      </c>
-      <c r="I26" s="28" t="n">
-        <v>5.46</v>
+        <v>10.24</v>
+      </c>
+      <c r="I26" s="27" t="n">
+        <v>-99.45</v>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="26" t="inlineStr">
         <is>
-          <t>삼성E&amp;A</t>
+          <t>코스나인</t>
         </is>
       </c>
       <c r="B27" s="25" t="n">
@@ -3954,25 +3966,25 @@
       </c>
       <c r="F27" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G27" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="H27" s="28" t="n">
-        <v>1.19</v>
-      </c>
-      <c r="I27" s="28" t="n">
-        <v>11.23</v>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="H27" s="27" t="n">
+        <v>-23.08</v>
+      </c>
+      <c r="I27" s="27" t="n">
+        <v>-97.92</v>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="26" t="inlineStr">
         <is>
-          <t>샘표</t>
+          <t>한국석유</t>
         </is>
       </c>
       <c r="B28" s="25" t="n">
@@ -3989,25 +4001,25 @@
       </c>
       <c r="F28" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G28" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="H28" s="28" t="n">
-        <v>3.23</v>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="H28" s="27" t="n">
+        <v>-3.22</v>
       </c>
       <c r="I28" s="28" t="n">
-        <v>33.72</v>
+        <v>8.83</v>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="26" t="inlineStr">
         <is>
-          <t>셀트리온</t>
+          <t>현대차</t>
         </is>
       </c>
       <c r="B29" s="25" t="n">
@@ -4024,336 +4036,340 @@
       </c>
       <c r="F29" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G29" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="H29" s="27" t="n">
-        <v>-1.44</v>
+        <v>-1.67</v>
       </c>
       <c r="I29" s="27" t="n">
-        <v>-5.26</v>
+        <v>-0.26</v>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="26" t="inlineStr">
         <is>
-          <t>수성웹툰</t>
+          <t>금강철강</t>
         </is>
       </c>
       <c r="B30" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C30" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D30" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E30" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F30" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G30" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="H30" s="27" t="n">
-        <v>-25.47</v>
-      </c>
-      <c r="I30" s="27" t="n">
-        <v>-49.62</v>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="H30" s="28" t="n">
+        <v>2.34</v>
+      </c>
+      <c r="I30" s="28" t="n">
+        <v>30.51</v>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="26" t="inlineStr">
         <is>
-          <t>아티스트스튜디오</t>
+          <t>넥스틸</t>
         </is>
       </c>
       <c r="B31" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C31" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D31" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E31" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F31" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G31" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="H31" s="27" t="n">
-        <v>-13.9</v>
-      </c>
-      <c r="I31" s="27" t="n">
-        <v>-8.789999999999999</v>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="H31" s="28" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="I31" s="28" t="n">
+        <v>10.7</v>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="26" t="inlineStr">
         <is>
-          <t>전기차</t>
+          <t>드림시큐리티</t>
         </is>
       </c>
       <c r="B32" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C32" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D32" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E32" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F32" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G32" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="H32" s="25" t="n"/>
-      <c r="I32" s="25" t="n"/>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="H32" s="28" t="n">
+        <v>23.29</v>
+      </c>
+      <c r="I32" s="28" t="n">
+        <v>29.38</v>
+      </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="26" t="inlineStr">
         <is>
-          <t>코다코</t>
+          <t>머큐리</t>
         </is>
       </c>
       <c r="B33" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C33" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D33" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E33" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F33" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G33" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="H33" s="28" t="n">
-        <v>10.24</v>
-      </c>
-      <c r="I33" s="27" t="n">
-        <v>-99.45</v>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="H33" s="27" t="n">
+        <v>-4.43</v>
+      </c>
+      <c r="I33" s="28" t="n">
+        <v>39.71</v>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="26" t="inlineStr">
         <is>
-          <t>코스나인</t>
+          <t>빛과전자</t>
         </is>
       </c>
       <c r="B34" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C34" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D34" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E34" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F34" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G34" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="H34" s="27" t="n">
-        <v>-23.08</v>
-      </c>
-      <c r="I34" s="27" t="n">
-        <v>-97.92</v>
+        <v>-1.4</v>
+      </c>
+      <c r="I34" s="28" t="n">
+        <v>42.54</v>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="26" t="inlineStr">
         <is>
-          <t>한국석유</t>
+          <t>삼미금속</t>
         </is>
       </c>
       <c r="B35" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C35" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D35" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E35" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F35" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G35" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="H35" s="27" t="n">
-        <v>-3.22</v>
+        <v>-2.69</v>
       </c>
       <c r="I35" s="28" t="n">
-        <v>8.83</v>
+        <v>47.19</v>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="26" t="inlineStr">
         <is>
-          <t>헝셩그룹</t>
+          <t>샌즈랩</t>
         </is>
       </c>
       <c r="B36" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C36" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D36" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E36" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F36" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G36" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="H36" s="28" t="n">
-        <v>14.63</v>
+        <v>29.8</v>
       </c>
       <c r="I36" s="28" t="n">
-        <v>5.94</v>
+        <v>31.03</v>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="26" t="inlineStr">
         <is>
-          <t>혜인</t>
+          <t>샘표식품</t>
         </is>
       </c>
       <c r="B37" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C37" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D37" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E37" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F37" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G37" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="H37" s="28" t="n">
-        <v>3.85</v>
-      </c>
-      <c r="I37" s="27" t="n">
-        <v>-11.27</v>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="H37" s="27" t="n">
+        <v>-14.76</v>
+      </c>
+      <c r="I37" s="28" t="n">
+        <v>10.78</v>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="26" t="inlineStr">
         <is>
-          <t>흥아해운</t>
+          <t>서전기전</t>
         </is>
       </c>
       <c r="B38" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C38" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D38" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E38" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F38" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G38" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="H38" s="27" t="n">
-        <v>-1.21</v>
+        <v>-3.51</v>
       </c>
       <c r="I38" s="28" t="n">
-        <v>8.93</v>
+        <v>24.43</v>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="26" t="inlineStr">
         <is>
-          <t>머큐리</t>
+          <t>스트라드비젼</t>
         </is>
       </c>
       <c r="B39" s="25" t="n">
@@ -4370,25 +4386,25 @@
       </c>
       <c r="F39" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G39" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="H39" s="27" t="n">
-        <v>-4.43</v>
+        <v>-0.39</v>
       </c>
       <c r="I39" s="28" t="n">
-        <v>39.71</v>
+        <v>35.05</v>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="26" t="inlineStr">
         <is>
-          <t>빛과전자</t>
+          <t>아모텍</t>
         </is>
       </c>
       <c r="B40" s="25" t="n">
@@ -4405,25 +4421,25 @@
       </c>
       <c r="F40" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G40" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="H40" s="27" t="n">
-        <v>-1.4</v>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="H40" s="28" t="n">
+        <v>29.98</v>
       </c>
       <c r="I40" s="28" t="n">
-        <v>42.54</v>
+        <v>34.01</v>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="26" t="inlineStr">
         <is>
-          <t>삼미금속</t>
+          <t>액스비스</t>
         </is>
       </c>
       <c r="B41" s="25" t="n">
@@ -4440,25 +4456,25 @@
       </c>
       <c r="F41" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G41" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="H41" s="27" t="n">
-        <v>-2.69</v>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="H41" s="28" t="n">
+        <v>11.97</v>
       </c>
       <c r="I41" s="28" t="n">
-        <v>47.19</v>
+        <v>57.45</v>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="26" t="inlineStr">
         <is>
-          <t>샘표식품</t>
+          <t>엑스게이트</t>
         </is>
       </c>
       <c r="B42" s="25" t="n">
@@ -4475,25 +4491,25 @@
       </c>
       <c r="F42" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G42" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="H42" s="27" t="n">
-        <v>-14.76</v>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="H42" s="28" t="n">
+        <v>29.94</v>
       </c>
       <c r="I42" s="28" t="n">
-        <v>10.78</v>
+        <v>40.51</v>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="26" t="inlineStr">
         <is>
-          <t>서전기전</t>
+          <t>엔에이치스팩34호</t>
         </is>
       </c>
       <c r="B43" s="25" t="n">
@@ -4510,25 +4526,25 @@
       </c>
       <c r="F43" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G43" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="H43" s="27" t="n">
-        <v>-3.51</v>
-      </c>
-      <c r="I43" s="28" t="n">
-        <v>24.43</v>
+        <v>-6.94</v>
+      </c>
+      <c r="I43" s="27" t="n">
+        <v>-6.94</v>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="26" t="inlineStr">
         <is>
-          <t>액스비스</t>
+          <t>오르비텍</t>
         </is>
       </c>
       <c r="B44" s="25" t="n">
@@ -4545,25 +4561,25 @@
       </c>
       <c r="F44" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G44" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="H44" s="28" t="n">
-        <v>11.97</v>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="H44" s="27" t="n">
+        <v>-3.34</v>
       </c>
       <c r="I44" s="28" t="n">
-        <v>57.45</v>
+        <v>40.35</v>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="26" t="inlineStr">
         <is>
-          <t>에스투더블유</t>
+          <t>우리기술</t>
         </is>
       </c>
       <c r="B45" s="25" t="n">
@@ -4580,25 +4596,25 @@
       </c>
       <c r="F45" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G45" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="H45" s="28" t="n">
-        <v>26.38</v>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="H45" s="27" t="n">
+        <v>-3.77</v>
       </c>
       <c r="I45" s="28" t="n">
-        <v>52.78</v>
+        <v>32.17</v>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="26" t="inlineStr">
         <is>
-          <t>엑스게이트</t>
+          <t>우리넷</t>
         </is>
       </c>
       <c r="B46" s="25" t="n">
@@ -4615,25 +4631,25 @@
       </c>
       <c r="F46" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G46" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="H46" s="28" t="n">
-        <v>29.94</v>
+        <v>3.49</v>
       </c>
       <c r="I46" s="28" t="n">
-        <v>40.51</v>
+        <v>15.6</v>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="26" t="inlineStr">
         <is>
-          <t>엔에이치스팩34호</t>
+          <t>우리로</t>
         </is>
       </c>
       <c r="B47" s="25" t="n">
@@ -4650,25 +4666,25 @@
       </c>
       <c r="F47" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G47" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="H47" s="27" t="n">
-        <v>-6.94</v>
-      </c>
-      <c r="I47" s="27" t="n">
-        <v>-6.94</v>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="H47" s="28" t="n">
+        <v>7.31</v>
+      </c>
+      <c r="I47" s="28" t="n">
+        <v>48.55</v>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="26" t="inlineStr">
         <is>
-          <t>오르비텍</t>
+          <t>원익피앤이</t>
         </is>
       </c>
       <c r="B48" s="25" t="n">
@@ -4685,25 +4701,25 @@
       </c>
       <c r="F48" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G48" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="H48" s="27" t="n">
-        <v>-3.34</v>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="H48" s="28" t="n">
+        <v>6.62</v>
       </c>
       <c r="I48" s="28" t="n">
-        <v>40.35</v>
+        <v>41</v>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="26" t="inlineStr">
         <is>
-          <t>원익피앤이</t>
+          <t>카프로</t>
         </is>
       </c>
       <c r="B49" s="25" t="n">
@@ -4720,25 +4736,25 @@
       </c>
       <c r="F49" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G49" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="H49" s="28" t="n">
-        <v>6.62</v>
-      </c>
-      <c r="I49" s="28" t="n">
-        <v>41</v>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="H49" s="27" t="n">
+        <v>-16.67</v>
+      </c>
+      <c r="I49" s="27" t="n">
+        <v>-96.72</v>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="26" t="inlineStr">
         <is>
-          <t>카프로</t>
+          <t>케이에스피</t>
         </is>
       </c>
       <c r="B50" s="25" t="n">
@@ -4755,25 +4771,25 @@
       </c>
       <c r="F50" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G50" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="H50" s="27" t="n">
-        <v>-16.67</v>
-      </c>
-      <c r="I50" s="27" t="n">
-        <v>-96.72</v>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="H50" s="28" t="n">
+        <v>6.57</v>
+      </c>
+      <c r="I50" s="28" t="n">
+        <v>29.35</v>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="26" t="inlineStr">
         <is>
-          <t>케이에스피</t>
+          <t>피아이이</t>
         </is>
       </c>
       <c r="B51" s="25" t="n">
@@ -4790,19 +4806,19 @@
       </c>
       <c r="F51" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G51" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="H51" s="28" t="n">
-        <v>6.57</v>
+        <v>7.61</v>
       </c>
       <c r="I51" s="28" t="n">
-        <v>29.35</v>
+        <v>37.84</v>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
@@ -4825,12 +4841,12 @@
       </c>
       <c r="F52" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G52" s="25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="H52" s="28" t="n">
@@ -4921,19 +4937,19 @@
         <v>1</v>
       </c>
       <c r="C3" s="36" t="n">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="D3" s="36" t="n">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="E3" s="36" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="F3" s="37" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G3" s="37" t="inlineStr">
@@ -4952,19 +4968,19 @@
         <v>1</v>
       </c>
       <c r="C4" s="36" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="D4" s="36" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="E4" s="36" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="F4" s="37" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G4" s="37" t="inlineStr">
@@ -4976,26 +4992,26 @@
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="35" t="inlineStr">
         <is>
-          <t>전기차</t>
+          <t>방산</t>
         </is>
       </c>
       <c r="B5" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="36" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D5" s="36" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E5" s="36" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="F5" s="37" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G5" s="37" t="inlineStr">
@@ -5007,26 +5023,26 @@
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="35" t="inlineStr">
         <is>
-          <t>방산</t>
+          <t>원전</t>
         </is>
       </c>
       <c r="B6" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="36" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="D6" s="36" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="E6" s="36" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="F6" s="37" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G6" s="37" t="inlineStr">
@@ -5038,26 +5054,26 @@
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="35" t="inlineStr">
         <is>
-          <t>원전</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="B7" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="36" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="D7" s="36" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="E7" s="36" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="F7" s="37" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G7" s="37" t="inlineStr">
@@ -5069,26 +5085,26 @@
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="35" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="B8" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="36" t="n">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="D8" s="36" t="n">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="E8" s="36" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="F8" s="37" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G8" s="37" t="inlineStr">
@@ -5098,71 +5114,63 @@
       </c>
     </row>
     <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="35" t="inlineStr">
-        <is>
-          <t>제약</t>
-        </is>
-      </c>
-      <c r="B9" s="36" t="n">
-        <v>1</v>
-      </c>
-      <c r="C9" s="36" t="n">
-        <v>7</v>
-      </c>
-      <c r="D9" s="36" t="n">
-        <v>7</v>
-      </c>
-      <c r="E9" s="36" t="inlineStr">
-        <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="F9" s="37" t="inlineStr">
-        <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="G9" s="37" t="inlineStr">
-        <is>
-          <t>⚡ 관심</t>
-        </is>
-      </c>
+      <c r="A9" s="26" t="inlineStr">
+        <is>
+          <t>이차전지</t>
+        </is>
+      </c>
+      <c r="B9" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F9" s="29" t="inlineStr">
+        <is>
+          <t>감지 없음</t>
+        </is>
+      </c>
+      <c r="G9" s="29" t="inlineStr"/>
     </row>
     <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="35" t="inlineStr">
-        <is>
-          <t>인공지능</t>
-        </is>
-      </c>
-      <c r="B10" s="36" t="n">
-        <v>1</v>
-      </c>
-      <c r="C10" s="36" t="n">
-        <v>18</v>
-      </c>
-      <c r="D10" s="36" t="n">
-        <v>18</v>
-      </c>
-      <c r="E10" s="36" t="inlineStr">
-        <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="F10" s="37" t="inlineStr">
-        <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="G10" s="37" t="inlineStr">
-        <is>
-          <t>⚡ 관심</t>
-        </is>
-      </c>
+      <c r="A10" s="26" t="inlineStr">
+        <is>
+          <t>AI반도체</t>
+        </is>
+      </c>
+      <c r="B10" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F10" s="29" t="inlineStr">
+        <is>
+          <t>감지 없음</t>
+        </is>
+      </c>
+      <c r="G10" s="29" t="inlineStr"/>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="26" t="inlineStr">
         <is>
-          <t>이차전지</t>
+          <t>전기차</t>
         </is>
       </c>
       <c r="B11" s="25" t="n">
@@ -5189,7 +5197,7 @@
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="26" t="inlineStr">
         <is>
-          <t>AI반도체</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="B12" s="25" t="n">

</xml_diff>

<commit_message>
auto: 2026-09-15 07:17 자동 백업
</commit_message>
<xml_diff>
--- a/trend/stock_trend_history.xlsx
+++ b/trend/stock_trend_history.xlsx
@@ -258,13 +258,13 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -694,7 +694,7 @@
     <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-09-14 06:54</t>
+          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-09-15 06:54</t>
         </is>
       </c>
     </row>
@@ -708,7 +708,7 @@
       </c>
       <c r="E3" s="3" t="n"/>
       <c r="G3" s="5" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="H3" s="3" t="n"/>
       <c r="J3" s="6" t="n">
@@ -787,21 +787,21 @@
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-09-14) 상위: 반도체  점수 52.0점</t>
+          <t>⚡ 최신(2026-09-15) 상위: 반도체  점수 57.0점</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-09-14) 상위: 인공지능  점수 21.0점</t>
+          <t>⚡ 최신(2026-09-15) 상위: 삼성전자  점수 19.0점</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-09-14) 상위: 바이오  점수 18.0점</t>
+          <t>⚡ 최신(2026-09-15) 상위: 로봇  점수 18.0점</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="15" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B14" s="15" t="n">
@@ -928,10 +928,10 @@
         </is>
       </c>
       <c r="D14" s="15" t="n">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="E14" s="15" t="n">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="F14" s="15" t="n">
         <v>0</v>
@@ -947,7 +947,7 @@
       </c>
       <c r="J14" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 헤드라인 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K14" s="17" t="inlineStr">
@@ -959,7 +959,7 @@
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="15" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B15" s="15" t="n">
@@ -967,14 +967,14 @@
       </c>
       <c r="C15" s="16" t="inlineStr">
         <is>
-          <t>인공지능</t>
+          <t>삼성전자</t>
         </is>
       </c>
       <c r="D15" s="15" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E15" s="15" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="F15" s="15" t="n">
         <v>0</v>
@@ -982,15 +982,15 @@
       <c r="G15" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H15" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I15" s="15" t="n">
-        <v/>
+      <c r="H15" s="18" t="n">
+        <v>-4.24</v>
+      </c>
+      <c r="I15" s="18" t="n">
+        <v>-7.96</v>
       </c>
       <c r="J15" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+          <t>네이버뉴스 기사 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K15" s="17" t="inlineStr">
@@ -1002,7 +1002,7 @@
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="15" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B16" s="15" t="n">
@@ -1010,7 +1010,7 @@
       </c>
       <c r="C16" s="16" t="inlineStr">
         <is>
-          <t>바이오</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="D16" s="15" t="n">
@@ -1033,19 +1033,17 @@
       </c>
       <c r="J16" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 한국경제 헤드라인 언급 / 네이버뉴스 기사 언급</t>
-        </is>
-      </c>
-      <c r="K16" s="17" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K16" s="17" t="n">
+        <v/>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B17" s="15" t="n">
@@ -1053,7 +1051,7 @@
       </c>
       <c r="C17" s="16" t="inlineStr">
         <is>
-          <t>삼성전자</t>
+          <t>LG</t>
         </is>
       </c>
       <c r="D17" s="15" t="n">
@@ -1069,24 +1067,26 @@
         <v>0</v>
       </c>
       <c r="H17" s="18" t="n">
-        <v>-3.53</v>
-      </c>
-      <c r="I17" s="19" t="n">
-        <v>1.57</v>
+        <v>-0.89</v>
+      </c>
+      <c r="I17" s="18" t="n">
+        <v>-10.44</v>
       </c>
       <c r="J17" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K17" s="17" t="n">
-        <v/>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 기사 언급</t>
+        </is>
+      </c>
+      <c r="K17" s="17" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B18" s="15" t="n">
@@ -1094,14 +1094,14 @@
       </c>
       <c r="C18" s="16" t="inlineStr">
         <is>
-          <t>LG</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="D18" s="15" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="E18" s="15" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F18" s="15" t="n">
         <v>0</v>
@@ -1109,15 +1109,15 @@
       <c r="G18" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H18" s="18" t="n">
-        <v>-4.66</v>
-      </c>
-      <c r="I18" s="18" t="n">
-        <v>-7.1</v>
+      <c r="H18" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I18" s="15" t="n">
+        <v/>
       </c>
       <c r="J18" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+          <t>네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K18" s="17" t="inlineStr">
@@ -1129,7 +1129,7 @@
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B19" s="15" t="n">
@@ -1141,10 +1141,10 @@
         </is>
       </c>
       <c r="D19" s="15" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E19" s="15" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F19" s="15" t="n">
         <v>0</v>
@@ -1153,14 +1153,14 @@
         <v>0</v>
       </c>
       <c r="H19" s="19" t="n">
-        <v>2.6</v>
+        <v>1.85</v>
       </c>
       <c r="I19" s="19" t="n">
-        <v>3.43</v>
+        <v>3.01</v>
       </c>
       <c r="J19" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K19" s="17" t="n">
@@ -1170,7 +1170,7 @@
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B20" s="15" t="n">
@@ -1178,14 +1178,14 @@
       </c>
       <c r="C20" s="16" t="inlineStr">
         <is>
-          <t>원전</t>
+          <t>바이오</t>
         </is>
       </c>
       <c r="D20" s="15" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E20" s="15" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="F20" s="15" t="n">
         <v>0</v>
@@ -1201,7 +1201,7 @@
       </c>
       <c r="J20" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 헤드라인 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K20" s="17" t="inlineStr">
@@ -1213,7 +1213,7 @@
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="15" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B21" s="15" t="n">
@@ -1221,42 +1221,42 @@
       </c>
       <c r="C21" s="16" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>KS인더스트리</t>
         </is>
       </c>
       <c r="D21" s="15" t="n">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="E21" s="15" t="n">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="F21" s="15" t="n">
         <v>0</v>
       </c>
       <c r="G21" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H21" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I21" s="15" t="n">
-        <v/>
+        <v>3</v>
+      </c>
+      <c r="H21" s="19" t="n">
+        <v>29.97</v>
+      </c>
+      <c r="I21" s="19" t="n">
+        <v>48.4</v>
       </c>
       <c r="J21" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 매일경제 기사 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
+          <t>중요공시 3건 / 중요공시 7일 +200% / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K21" s="17" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="15" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B22" s="15" t="n">
@@ -1264,14 +1264,14 @@
       </c>
       <c r="C22" s="16" t="inlineStr">
         <is>
-          <t>삼성전자우</t>
+          <t>SK하이닉스</t>
         </is>
       </c>
       <c r="D22" s="15" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E22" s="15" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F22" s="15" t="n">
         <v>0</v>
@@ -1280,24 +1280,26 @@
         <v>0</v>
       </c>
       <c r="H22" s="18" t="n">
-        <v>-4.78</v>
-      </c>
-      <c r="I22" s="19" t="n">
-        <v>0.89</v>
+        <v>-7.12</v>
+      </c>
+      <c r="I22" s="18" t="n">
+        <v>-5.61</v>
       </c>
       <c r="J22" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K22" s="17" t="n">
-        <v/>
+          <t>네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K22" s="17" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="15" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B23" s="15" t="n">
@@ -1305,42 +1307,42 @@
       </c>
       <c r="C23" s="16" t="inlineStr">
         <is>
-          <t>셀트리온</t>
+          <t>현대건설</t>
         </is>
       </c>
       <c r="D23" s="15" t="n">
         <v>8</v>
       </c>
       <c r="E23" s="15" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F23" s="15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G23" s="15" t="n">
         <v>3</v>
       </c>
       <c r="H23" s="18" t="n">
-        <v>-1.44</v>
+        <v>-6.97</v>
       </c>
       <c r="I23" s="18" t="n">
-        <v>-5.26</v>
+        <v>-1.1</v>
       </c>
       <c r="J23" s="17" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 7일 +100% / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급</t>
+          <t>중요공시 3건 / 중요공시 3일 +200% / 중요공시 7일 +200%</t>
         </is>
       </c>
       <c r="K23" s="17" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="15" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B24" s="15" t="n">
@@ -1348,7 +1350,7 @@
       </c>
       <c r="C24" s="16" t="inlineStr">
         <is>
-          <t>DB</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="D24" s="15" t="n">
@@ -1363,113 +1365,113 @@
       <c r="G24" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H24" s="18" t="n">
-        <v>-0.06</v>
-      </c>
-      <c r="I24" s="19" t="n">
-        <v>9.42</v>
+      <c r="H24" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I24" s="15" t="n">
+        <v/>
       </c>
       <c r="J24" s="17" t="inlineStr">
         <is>
-          <t>Google 급상승 검색어 등장 (US) / 매일경제 헤드라인 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K24" s="17" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
-      <c r="A25" s="20" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="B25" s="20" t="n">
+      <c r="A25" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B25" s="15" t="n">
         <v>12</v>
       </c>
-      <c r="C25" s="21" t="inlineStr">
-        <is>
-          <t>더코디</t>
-        </is>
-      </c>
-      <c r="D25" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="E25" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="F25" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G25" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H25" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="I25" s="22" t="n">
-        <v>185.01</v>
-      </c>
-      <c r="J25" s="23" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +1211% / 중요공시 6건</t>
-        </is>
-      </c>
-      <c r="K25" s="23" t="inlineStr">
+      <c r="C25" s="16" t="inlineStr">
+        <is>
+          <t>우리로</t>
+        </is>
+      </c>
+      <c r="D25" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="E25" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="F25" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" s="18" t="n">
+        <v>-0.97</v>
+      </c>
+      <c r="I25" s="19" t="n">
+        <v>46.65</v>
+      </c>
+      <c r="J25" s="17" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +172% / 중요공시 1건 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K25" s="17" t="inlineStr">
         <is>
           <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
-      <c r="A26" s="20" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="B26" s="20" t="n">
+      <c r="A26" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B26" s="15" t="n">
         <v>13</v>
       </c>
-      <c r="C26" s="21" t="inlineStr">
-        <is>
-          <t>에스투더블유</t>
-        </is>
-      </c>
-      <c r="D26" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="E26" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="F26" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G26" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H26" s="22" t="n">
-        <v>26.38</v>
-      </c>
-      <c r="I26" s="22" t="n">
-        <v>52.78</v>
-      </c>
-      <c r="J26" s="23" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +451% / 네이버뉴스 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K26" s="23" t="inlineStr">
-        <is>
-          <t>네이버</t>
+      <c r="C26" s="16" t="inlineStr">
+        <is>
+          <t>코나아이</t>
+        </is>
+      </c>
+      <c r="D26" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="E26" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="F26" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" s="19" t="n">
+        <v>7</v>
+      </c>
+      <c r="I26" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="J26" s="17" t="inlineStr">
+        <is>
+          <t>중요공시 2건 / 네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K26" s="17" t="inlineStr">
+        <is>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="20" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B27" s="20" t="n">
@@ -1477,7 +1479,7 @@
       </c>
       <c r="C27" s="21" t="inlineStr">
         <is>
-          <t>LG디스플레이</t>
+          <t>현대차</t>
         </is>
       </c>
       <c r="D27" s="20" t="n">
@@ -1492,15 +1494,15 @@
       <c r="G27" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H27" s="24" t="n">
-        <v>-0.78</v>
-      </c>
-      <c r="I27" s="24" t="n">
-        <v>-2.52</v>
+      <c r="H27" s="22" t="n">
+        <v>-3.92</v>
+      </c>
+      <c r="I27" s="22" t="n">
+        <v>-6.49</v>
       </c>
       <c r="J27" s="23" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>매일경제 기사 언급 / 매일경제 기사 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K27" s="23" t="n">
@@ -1510,7 +1512,7 @@
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="20" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B28" s="20" t="n">
@@ -1518,7 +1520,7 @@
       </c>
       <c r="C28" s="21" t="inlineStr">
         <is>
-          <t>루멘스</t>
+          <t>방산</t>
         </is>
       </c>
       <c r="D28" s="20" t="n">
@@ -1533,27 +1535,25 @@
       <c r="G28" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H28" s="22" t="n">
-        <v>0.39</v>
-      </c>
-      <c r="I28" s="24" t="n">
-        <v>-5.58</v>
+      <c r="H28" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I28" s="20" t="n">
+        <v/>
       </c>
       <c r="J28" s="23" t="inlineStr">
         <is>
-          <t>중요공시 5건 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K28" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K28" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="20" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B29" s="20" t="n">
@@ -1561,7 +1561,7 @@
       </c>
       <c r="C29" s="21" t="inlineStr">
         <is>
-          <t>삼성전기</t>
+          <t>고영</t>
         </is>
       </c>
       <c r="D29" s="20" t="n">
@@ -1576,15 +1576,15 @@
       <c r="G29" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H29" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="I29" s="24" t="n">
-        <v>-0.07000000000000001</v>
+      <c r="H29" s="22" t="n">
+        <v>-3.62</v>
+      </c>
+      <c r="I29" s="22" t="n">
+        <v>-5.16</v>
       </c>
       <c r="J29" s="23" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K29" s="23" t="n">
@@ -1594,7 +1594,7 @@
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="20" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B30" s="20" t="n">
@@ -1602,40 +1602,42 @@
       </c>
       <c r="C30" s="21" t="inlineStr">
         <is>
-          <t>방산</t>
+          <t>넥사다이내믹스</t>
         </is>
       </c>
       <c r="D30" s="20" t="n">
         <v>5</v>
       </c>
       <c r="E30" s="20" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F30" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G30" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H30" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I30" s="20" t="n">
-        <v/>
+      <c r="H30" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="I30" s="22" t="n">
+        <v>-5.65</v>
       </c>
       <c r="J30" s="23" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K30" s="23" t="n">
-        <v/>
+          <t>중요공시 5건 / 중요공시 3일 +67%</t>
+        </is>
+      </c>
+      <c r="K30" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="20" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B31" s="20" t="n">
@@ -1643,42 +1645,42 @@
       </c>
       <c r="C31" s="21" t="inlineStr">
         <is>
-          <t>코스나인</t>
+          <t>삼성바이오로직스</t>
         </is>
       </c>
       <c r="D31" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E31" s="20" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F31" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G31" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H31" s="24" t="n">
-        <v>-23.08</v>
-      </c>
-      <c r="I31" s="24" t="n">
-        <v>-97.92</v>
+        <v>3</v>
+      </c>
+      <c r="H31" s="22" t="n">
+        <v>-0.92</v>
+      </c>
+      <c r="I31" s="22" t="n">
+        <v>-4.37</v>
       </c>
       <c r="J31" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +1239% / 중요공시 2건</t>
+          <t>중요공시 2건 / 중요공시 7일 +100% / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K31" s="23" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="20" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B32" s="20" t="n">
@@ -1686,14 +1688,14 @@
       </c>
       <c r="C32" s="21" t="inlineStr">
         <is>
-          <t>코다코</t>
+          <t>GS</t>
         </is>
       </c>
       <c r="D32" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E32" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F32" s="20" t="n">
         <v>0</v>
@@ -1702,26 +1704,26 @@
         <v>0</v>
       </c>
       <c r="H32" s="22" t="n">
-        <v>10.24</v>
-      </c>
-      <c r="I32" s="24" t="n">
-        <v>-99.45</v>
+        <v>-3.87</v>
+      </c>
+      <c r="I32" s="22" t="n">
+        <v>-8.92</v>
       </c>
       <c r="J32" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +1086% / 중요공시 2건</t>
+          <t>Google 급상승 검색어 등장 (US)</t>
         </is>
       </c>
       <c r="K32" s="23" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>Google</t>
         </is>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="20" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B33" s="20" t="n">
@@ -1729,14 +1731,14 @@
       </c>
       <c r="C33" s="21" t="inlineStr">
         <is>
-          <t>한국석유</t>
+          <t>조선</t>
         </is>
       </c>
       <c r="D33" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E33" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F33" s="20" t="n">
         <v>0</v>
@@ -1744,27 +1746,25 @@
       <c r="G33" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H33" s="24" t="n">
-        <v>-3.22</v>
-      </c>
-      <c r="I33" s="22" t="n">
-        <v>8.83</v>
+      <c r="H33" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I33" s="20" t="n">
+        <v/>
       </c>
       <c r="J33" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +132% / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K33" s="23" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K33" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="20" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B34" s="20" t="n">
@@ -1772,14 +1772,14 @@
       </c>
       <c r="C34" s="21" t="inlineStr">
         <is>
-          <t>수성웹툰</t>
+          <t>LG전자</t>
         </is>
       </c>
       <c r="D34" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E34" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F34" s="20" t="n">
         <v>0</v>
@@ -1787,27 +1787,27 @@
       <c r="G34" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H34" s="24" t="n">
-        <v>-25.47</v>
-      </c>
-      <c r="I34" s="24" t="n">
-        <v>-49.62</v>
+      <c r="H34" s="22" t="n">
+        <v>-2.31</v>
+      </c>
+      <c r="I34" s="22" t="n">
+        <v>-8.93</v>
       </c>
       <c r="J34" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +132% / 중요공시 1건</t>
+          <t>매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K34" s="23" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="20" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B35" s="20" t="n">
@@ -1815,7 +1815,7 @@
       </c>
       <c r="C35" s="21" t="inlineStr">
         <is>
-          <t>원풍물산</t>
+          <t>코스나인</t>
         </is>
       </c>
       <c r="D35" s="20" t="n">
@@ -1830,15 +1830,15 @@
       <c r="G35" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H35" s="24" t="n">
-        <v>-1.47</v>
-      </c>
-      <c r="I35" s="24" t="n">
-        <v>-68.62</v>
+      <c r="H35" s="22" t="n">
+        <v>-30</v>
+      </c>
+      <c r="I35" s="22" t="n">
+        <v>-98.54000000000001</v>
       </c>
       <c r="J35" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +101% / 중요공시 1건</t>
+          <t>네이버 검색 당일 +1295% / 중요공시 2건</t>
         </is>
       </c>
       <c r="K35" s="23" t="inlineStr">
@@ -1850,7 +1850,7 @@
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="20" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B36" s="20" t="n">
@@ -1858,42 +1858,42 @@
       </c>
       <c r="C36" s="21" t="inlineStr">
         <is>
-          <t>에넥스</t>
+          <t>코다코</t>
         </is>
       </c>
       <c r="D36" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E36" s="20" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F36" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G36" s="20" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H36" s="22" t="n">
-        <v>10.85</v>
+        <v>-33.63</v>
       </c>
       <c r="I36" s="22" t="n">
-        <v>14.32</v>
+        <v>-99.64</v>
       </c>
       <c r="J36" s="23" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 7일 +100%</t>
+          <t>네이버 검색 당일 +1164% / 중요공시 2건</t>
         </is>
       </c>
       <c r="K36" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="20" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B37" s="20" t="n">
@@ -1901,7 +1901,7 @@
       </c>
       <c r="C37" s="21" t="inlineStr">
         <is>
-          <t>삼성바이오로직스</t>
+          <t>수성웹툰</t>
         </is>
       </c>
       <c r="D37" s="20" t="n">
@@ -1916,15 +1916,15 @@
       <c r="G37" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H37" s="24" t="n">
-        <v>-0.5600000000000001</v>
-      </c>
-      <c r="I37" s="24" t="n">
-        <v>-2.21</v>
+      <c r="H37" s="22" t="n">
+        <v>-14.07</v>
+      </c>
+      <c r="I37" s="22" t="n">
+        <v>-66.67</v>
       </c>
       <c r="J37" s="23" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 네이버뉴스 헤드라인 언급</t>
+          <t>네이버 검색 당일 +139% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K37" s="23" t="inlineStr">
@@ -1936,7 +1936,7 @@
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="20" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B38" s="20" t="n">
@@ -1944,7 +1944,7 @@
       </c>
       <c r="C38" s="21" t="inlineStr">
         <is>
-          <t>아티스트스튜디오</t>
+          <t>원풍물산</t>
         </is>
       </c>
       <c r="D38" s="20" t="n">
@@ -1959,27 +1959,27 @@
       <c r="G38" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H38" s="24" t="n">
-        <v>-13.9</v>
-      </c>
-      <c r="I38" s="24" t="n">
-        <v>-8.789999999999999</v>
+      <c r="H38" s="22" t="n">
+        <v>-26.12</v>
+      </c>
+      <c r="I38" s="22" t="n">
+        <v>-66.89</v>
       </c>
       <c r="J38" s="23" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
+          <t>네이버 검색 당일 +106% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K38" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="20" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B39" s="20" t="n">
@@ -1987,7 +1987,7 @@
       </c>
       <c r="C39" s="21" t="inlineStr">
         <is>
-          <t>KT</t>
+          <t>삼성중공업</t>
         </is>
       </c>
       <c r="D39" s="20" t="n">
@@ -2002,25 +2002,27 @@
       <c r="G39" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H39" s="22" t="n">
-        <v>1.35</v>
+      <c r="H39" s="24" t="n">
+        <v>3.27</v>
       </c>
       <c r="I39" s="24" t="n">
-        <v>-2.95</v>
+        <v>3.27</v>
       </c>
       <c r="J39" s="23" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K39" s="23" t="n">
-        <v/>
+          <t>중요공시 2건 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K39" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="20" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B40" s="20" t="n">
@@ -2028,7 +2030,7 @@
       </c>
       <c r="C40" s="21" t="inlineStr">
         <is>
-          <t>현대차</t>
+          <t>인피니트헬스케어</t>
         </is>
       </c>
       <c r="D40" s="20" t="n">
@@ -2044,153 +2046,151 @@
         <v>0</v>
       </c>
       <c r="H40" s="24" t="n">
-        <v>-1.67</v>
+        <v>30</v>
       </c>
       <c r="I40" s="24" t="n">
-        <v>-0.26</v>
+        <v>24.29</v>
       </c>
       <c r="J40" s="23" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K40" s="23" t="n">
+          <t>중요공시 1건 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K40" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="18" customHeight="1">
+      <c r="A41" s="20" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B41" s="20" t="n">
+        <v>28</v>
+      </c>
+      <c r="C41" s="21" t="inlineStr">
+        <is>
+          <t>전기차</t>
+        </is>
+      </c>
+      <c r="D41" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="E41" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F41" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G41" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H41" s="20" t="n">
         <v/>
       </c>
-    </row>
-    <row r="41" ht="18" customHeight="1">
-      <c r="A41" s="25" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="B41" s="25" t="n">
-        <v>28</v>
-      </c>
-      <c r="C41" s="26" t="inlineStr">
-        <is>
-          <t>삼미금속</t>
-        </is>
-      </c>
-      <c r="D41" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="E41" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="F41" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="G41" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H41" s="27" t="n">
-        <v>-2.69</v>
-      </c>
-      <c r="I41" s="28" t="n">
-        <v>47.19</v>
-      </c>
-      <c r="J41" s="29" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +1091%</t>
-        </is>
-      </c>
-      <c r="K41" s="29" t="inlineStr">
+      <c r="I41" s="20" t="n">
+        <v/>
+      </c>
+      <c r="J41" s="23" t="inlineStr">
+        <is>
+          <t>네이버뉴스 기사 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K41" s="23" t="inlineStr">
         <is>
           <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
-      <c r="A42" s="25" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="B42" s="25" t="n">
+      <c r="A42" s="20" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B42" s="20" t="n">
         <v>29</v>
       </c>
-      <c r="C42" s="26" t="inlineStr">
-        <is>
-          <t>액스비스</t>
-        </is>
-      </c>
-      <c r="D42" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="E42" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="F42" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="G42" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H42" s="28" t="n">
-        <v>11.97</v>
-      </c>
-      <c r="I42" s="28" t="n">
-        <v>57.45</v>
-      </c>
-      <c r="J42" s="29" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +784%</t>
-        </is>
-      </c>
-      <c r="K42" s="29" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+      <c r="C42" s="21" t="inlineStr">
+        <is>
+          <t>원전</t>
+        </is>
+      </c>
+      <c r="D42" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="E42" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F42" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G42" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H42" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I42" s="20" t="n">
+        <v/>
+      </c>
+      <c r="J42" s="23" t="inlineStr">
+        <is>
+          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K42" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
-      <c r="A43" s="25" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="B43" s="25" t="n">
+      <c r="A43" s="20" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B43" s="20" t="n">
         <v>30</v>
       </c>
-      <c r="C43" s="26" t="inlineStr">
-        <is>
-          <t>샘표식품</t>
-        </is>
-      </c>
-      <c r="D43" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="E43" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="F43" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="G43" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H43" s="27" t="n">
-        <v>-14.76</v>
-      </c>
-      <c r="I43" s="28" t="n">
-        <v>10.78</v>
-      </c>
-      <c r="J43" s="29" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +713%</t>
-        </is>
-      </c>
-      <c r="K43" s="29" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+      <c r="C43" s="21" t="inlineStr">
+        <is>
+          <t>아모레퍼시픽</t>
+        </is>
+      </c>
+      <c r="D43" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="E43" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F43" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G43" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H43" s="24" t="n">
+        <v>2.78</v>
+      </c>
+      <c r="I43" s="24" t="n">
+        <v>2.56</v>
+      </c>
+      <c r="J43" s="23" t="inlineStr">
+        <is>
+          <t>한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K43" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B44" s="25" t="n">
@@ -2198,7 +2198,7 @@
       </c>
       <c r="C44" s="26" t="inlineStr">
         <is>
-          <t>엔에이치스팩34호</t>
+          <t>삼미금속</t>
         </is>
       </c>
       <c r="D44" s="25" t="n">
@@ -2214,14 +2214,14 @@
         <v>0</v>
       </c>
       <c r="H44" s="27" t="n">
-        <v>-6.94</v>
-      </c>
-      <c r="I44" s="27" t="n">
-        <v>-6.94</v>
+        <v>-8.220000000000001</v>
+      </c>
+      <c r="I44" s="28" t="n">
+        <v>10.59</v>
       </c>
       <c r="J44" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +496%</t>
+          <t>네이버 검색 당일 +1128%</t>
         </is>
       </c>
       <c r="K44" s="29" t="inlineStr">
@@ -2233,7 +2233,7 @@
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B45" s="25" t="n">
@@ -2241,7 +2241,7 @@
       </c>
       <c r="C45" s="26" t="inlineStr">
         <is>
-          <t>카프로</t>
+          <t>액스비스</t>
         </is>
       </c>
       <c r="D45" s="25" t="n">
@@ -2257,14 +2257,14 @@
         <v>0</v>
       </c>
       <c r="H45" s="27" t="n">
-        <v>-16.67</v>
-      </c>
-      <c r="I45" s="27" t="n">
-        <v>-96.72</v>
+        <v>-3.59</v>
+      </c>
+      <c r="I45" s="28" t="n">
+        <v>47.72</v>
       </c>
       <c r="J45" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +487%</t>
+          <t>네이버 검색 당일 +831%</t>
         </is>
       </c>
       <c r="K45" s="29" t="inlineStr">
@@ -2276,7 +2276,7 @@
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B46" s="25" t="n">
@@ -2284,7 +2284,7 @@
       </c>
       <c r="C46" s="26" t="inlineStr">
         <is>
-          <t>서전기전</t>
+          <t>엔에이치스팩34호</t>
         </is>
       </c>
       <c r="D46" s="25" t="n">
@@ -2299,15 +2299,15 @@
       <c r="G46" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H46" s="27" t="n">
-        <v>-3.51</v>
-      </c>
-      <c r="I46" s="28" t="n">
-        <v>24.43</v>
+      <c r="H46" s="28" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="I46" s="27" t="n">
+        <v>-6.8</v>
       </c>
       <c r="J46" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +410%</t>
+          <t>네이버 검색 당일 +503%</t>
         </is>
       </c>
       <c r="K46" s="29" t="inlineStr">
@@ -2319,7 +2319,7 @@
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B47" s="25" t="n">
@@ -2327,7 +2327,7 @@
       </c>
       <c r="C47" s="26" t="inlineStr">
         <is>
-          <t>머큐리</t>
+          <t>카프로</t>
         </is>
       </c>
       <c r="D47" s="25" t="n">
@@ -2343,14 +2343,14 @@
         <v>0</v>
       </c>
       <c r="H47" s="27" t="n">
-        <v>-4.43</v>
-      </c>
-      <c r="I47" s="28" t="n">
-        <v>39.71</v>
+        <v>-40.83</v>
+      </c>
+      <c r="I47" s="27" t="n">
+        <v>-98.06</v>
       </c>
       <c r="J47" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +380%</t>
+          <t>네이버 검색 당일 +500%</t>
         </is>
       </c>
       <c r="K47" s="29" t="inlineStr">
@@ -2362,7 +2362,7 @@
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B48" s="25" t="n">
@@ -2370,7 +2370,7 @@
       </c>
       <c r="C48" s="26" t="inlineStr">
         <is>
-          <t>오르비텍</t>
+          <t>에스투더블유</t>
         </is>
       </c>
       <c r="D48" s="25" t="n">
@@ -2385,15 +2385,15 @@
       <c r="G48" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H48" s="27" t="n">
-        <v>-3.34</v>
+      <c r="H48" s="28" t="n">
+        <v>7.95</v>
       </c>
       <c r="I48" s="28" t="n">
-        <v>40.35</v>
+        <v>66.98</v>
       </c>
       <c r="J48" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +307%</t>
+          <t>네이버 검색 당일 +490%</t>
         </is>
       </c>
       <c r="K48" s="29" t="inlineStr">
@@ -2405,7 +2405,7 @@
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B49" s="25" t="n">
@@ -2413,7 +2413,7 @@
       </c>
       <c r="C49" s="26" t="inlineStr">
         <is>
-          <t>한빛레이저</t>
+          <t>머큐리</t>
         </is>
       </c>
       <c r="D49" s="25" t="n">
@@ -2429,14 +2429,14 @@
         <v>0</v>
       </c>
       <c r="H49" s="28" t="n">
-        <v>2.83</v>
+        <v>0.11</v>
       </c>
       <c r="I49" s="28" t="n">
-        <v>36.01</v>
+        <v>41.31</v>
       </c>
       <c r="J49" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +282%</t>
+          <t>네이버 검색 당일 +397%</t>
         </is>
       </c>
       <c r="K49" s="29" t="inlineStr">
@@ -2448,7 +2448,7 @@
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B50" s="25" t="n">
@@ -2472,14 +2472,14 @@
         <v>0</v>
       </c>
       <c r="H50" s="28" t="n">
-        <v>29.94</v>
+        <v>6.97</v>
       </c>
       <c r="I50" s="28" t="n">
-        <v>40.51</v>
+        <v>51.63</v>
       </c>
       <c r="J50" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +236%</t>
+          <t>네이버 검색 당일 +275%</t>
         </is>
       </c>
       <c r="K50" s="29" t="inlineStr">
@@ -2491,7 +2491,7 @@
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B51" s="25" t="n">
@@ -2499,7 +2499,7 @@
       </c>
       <c r="C51" s="26" t="inlineStr">
         <is>
-          <t>원익피앤이</t>
+          <t>샌즈랩</t>
         </is>
       </c>
       <c r="D51" s="25" t="n">
@@ -2515,14 +2515,14 @@
         <v>0</v>
       </c>
       <c r="H51" s="28" t="n">
-        <v>6.62</v>
+        <v>29.95</v>
       </c>
       <c r="I51" s="28" t="n">
-        <v>41</v>
+        <v>70.48</v>
       </c>
       <c r="J51" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +220%</t>
+          <t>네이버 검색 당일 +246%</t>
         </is>
       </c>
       <c r="K51" s="29" t="inlineStr">
@@ -2534,7 +2534,7 @@
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B52" s="25" t="n">
@@ -2542,7 +2542,7 @@
       </c>
       <c r="C52" s="26" t="inlineStr">
         <is>
-          <t>빛과전자</t>
+          <t>에스엠벡셀</t>
         </is>
       </c>
       <c r="D52" s="25" t="n">
@@ -2558,14 +2558,14 @@
         <v>0</v>
       </c>
       <c r="H52" s="27" t="n">
-        <v>-1.4</v>
+        <v>-8.199999999999999</v>
       </c>
       <c r="I52" s="28" t="n">
-        <v>42.54</v>
+        <v>38.56</v>
       </c>
       <c r="J52" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +211%</t>
+          <t>네이버 검색 당일 +244%</t>
         </is>
       </c>
       <c r="K52" s="29" t="inlineStr">
@@ -2577,7 +2577,7 @@
     <row r="53" ht="18" customHeight="1">
       <c r="A53" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B53" s="25" t="n">
@@ -2585,7 +2585,7 @@
       </c>
       <c r="C53" s="26" t="inlineStr">
         <is>
-          <t>케이에스피</t>
+          <t>빛과전자</t>
         </is>
       </c>
       <c r="D53" s="25" t="n">
@@ -2601,14 +2601,14 @@
         <v>0</v>
       </c>
       <c r="H53" s="28" t="n">
-        <v>6.57</v>
+        <v>12.53</v>
       </c>
       <c r="I53" s="28" t="n">
-        <v>29.35</v>
+        <v>55.54</v>
       </c>
       <c r="J53" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +198%</t>
+          <t>네이버 검색 당일 +218%</t>
         </is>
       </c>
       <c r="K53" s="29" t="inlineStr">
@@ -2620,7 +2620,7 @@
     <row r="54" ht="18" customHeight="1">
       <c r="A54" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B54" s="25" t="n">
@@ -2628,7 +2628,7 @@
       </c>
       <c r="C54" s="26" t="inlineStr">
         <is>
-          <t>샌즈랩</t>
+          <t>금강철강</t>
         </is>
       </c>
       <c r="D54" s="25" t="n">
@@ -2644,14 +2644,14 @@
         <v>0</v>
       </c>
       <c r="H54" s="28" t="n">
-        <v>29.8</v>
+        <v>0.13</v>
       </c>
       <c r="I54" s="28" t="n">
-        <v>31.03</v>
+        <v>22.93</v>
       </c>
       <c r="J54" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +193%</t>
+          <t>네이버 검색 당일 +173%</t>
         </is>
       </c>
       <c r="K54" s="29" t="inlineStr">
@@ -2663,7 +2663,7 @@
     <row r="55" ht="18" customHeight="1">
       <c r="A55" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B55" s="25" t="n">
@@ -2671,7 +2671,7 @@
       </c>
       <c r="C55" s="26" t="inlineStr">
         <is>
-          <t>피아이이</t>
+          <t>우리넷</t>
         </is>
       </c>
       <c r="D55" s="25" t="n">
@@ -2687,14 +2687,14 @@
         <v>0</v>
       </c>
       <c r="H55" s="28" t="n">
-        <v>7.61</v>
+        <v>7.71</v>
       </c>
       <c r="I55" s="28" t="n">
-        <v>37.84</v>
+        <v>24.69</v>
       </c>
       <c r="J55" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +178%</t>
+          <t>네이버 검색 당일 +171%</t>
         </is>
       </c>
       <c r="K55" s="29" t="inlineStr">
@@ -2706,7 +2706,7 @@
     <row r="56" ht="18" customHeight="1">
       <c r="A56" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B56" s="25" t="n">
@@ -2714,7 +2714,7 @@
       </c>
       <c r="C56" s="26" t="inlineStr">
         <is>
-          <t>스트라드비젼</t>
+          <t>아모텍</t>
         </is>
       </c>
       <c r="D56" s="25" t="n">
@@ -2729,15 +2729,15 @@
       <c r="G56" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H56" s="27" t="n">
-        <v>-0.39</v>
+      <c r="H56" s="28" t="n">
+        <v>4.43</v>
       </c>
       <c r="I56" s="28" t="n">
-        <v>35.05</v>
+        <v>41.07</v>
       </c>
       <c r="J56" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +168%</t>
+          <t>네이버 검색 당일 +167%</t>
         </is>
       </c>
       <c r="K56" s="29" t="inlineStr">
@@ -2749,7 +2749,7 @@
     <row r="57" ht="18" customHeight="1">
       <c r="A57" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B57" s="25" t="n">
@@ -2757,7 +2757,7 @@
       </c>
       <c r="C57" s="26" t="inlineStr">
         <is>
-          <t>금강철강</t>
+          <t>드림시큐리티</t>
         </is>
       </c>
       <c r="D57" s="25" t="n">
@@ -2773,14 +2773,14 @@
         <v>0</v>
       </c>
       <c r="H57" s="28" t="n">
-        <v>2.34</v>
+        <v>5.53</v>
       </c>
       <c r="I57" s="28" t="n">
-        <v>30.51</v>
+        <v>37.22</v>
       </c>
       <c r="J57" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +165%</t>
+          <t>네이버 검색 당일 +147%</t>
         </is>
       </c>
       <c r="K57" s="29" t="inlineStr">
@@ -2792,7 +2792,7 @@
     <row r="58" ht="18" customHeight="1">
       <c r="A58" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B58" s="25" t="n">
@@ -2800,7 +2800,7 @@
       </c>
       <c r="C58" s="26" t="inlineStr">
         <is>
-          <t>우리로</t>
+          <t>넥스틸</t>
         </is>
       </c>
       <c r="D58" s="25" t="n">
@@ -2816,14 +2816,14 @@
         <v>0</v>
       </c>
       <c r="H58" s="28" t="n">
-        <v>7.31</v>
+        <v>1.53</v>
       </c>
       <c r="I58" s="28" t="n">
-        <v>48.55</v>
+        <v>10.27</v>
       </c>
       <c r="J58" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +161%</t>
+          <t>네이버 검색 당일 +131%</t>
         </is>
       </c>
       <c r="K58" s="29" t="inlineStr">
@@ -2835,7 +2835,7 @@
     <row r="59" ht="18" customHeight="1">
       <c r="A59" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B59" s="25" t="n">
@@ -2843,7 +2843,7 @@
       </c>
       <c r="C59" s="26" t="inlineStr">
         <is>
-          <t>우리넷</t>
+          <t>메가터치</t>
         </is>
       </c>
       <c r="D59" s="25" t="n">
@@ -2858,15 +2858,15 @@
       <c r="G59" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H59" s="28" t="n">
-        <v>3.49</v>
+      <c r="H59" s="27" t="n">
+        <v>-1.19</v>
       </c>
       <c r="I59" s="28" t="n">
-        <v>15.6</v>
+        <v>17.49</v>
       </c>
       <c r="J59" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +158%</t>
+          <t>네이버 검색 당일 +125%</t>
         </is>
       </c>
       <c r="K59" s="29" t="inlineStr">
@@ -2878,7 +2878,7 @@
     <row r="60" ht="18" customHeight="1">
       <c r="A60" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B60" s="25" t="n">
@@ -2886,7 +2886,7 @@
       </c>
       <c r="C60" s="26" t="inlineStr">
         <is>
-          <t>아모텍</t>
+          <t>우리기술</t>
         </is>
       </c>
       <c r="D60" s="25" t="n">
@@ -2901,15 +2901,15 @@
       <c r="G60" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H60" s="28" t="n">
-        <v>29.98</v>
+      <c r="H60" s="27" t="n">
+        <v>-2.35</v>
       </c>
       <c r="I60" s="28" t="n">
-        <v>34.01</v>
+        <v>25.64</v>
       </c>
       <c r="J60" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +140%</t>
+          <t>네이버 검색 당일 +119%</t>
         </is>
       </c>
       <c r="K60" s="29" t="inlineStr">
@@ -2921,7 +2921,7 @@
     <row r="61" ht="18" customHeight="1">
       <c r="A61" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B61" s="25" t="n">
@@ -2929,7 +2929,7 @@
       </c>
       <c r="C61" s="26" t="inlineStr">
         <is>
-          <t>드림시큐리티</t>
+          <t>빛샘전자</t>
         </is>
       </c>
       <c r="D61" s="25" t="n">
@@ -2945,14 +2945,14 @@
         <v>0</v>
       </c>
       <c r="H61" s="28" t="n">
-        <v>23.29</v>
+        <v>30</v>
       </c>
       <c r="I61" s="28" t="n">
-        <v>29.38</v>
+        <v>38.4</v>
       </c>
       <c r="J61" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +124%</t>
+          <t>네이버 검색 당일 +117%</t>
         </is>
       </c>
       <c r="K61" s="29" t="inlineStr">
@@ -2964,7 +2964,7 @@
     <row r="62" ht="18" customHeight="1">
       <c r="A62" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B62" s="25" t="n">
@@ -2972,7 +2972,7 @@
       </c>
       <c r="C62" s="26" t="inlineStr">
         <is>
-          <t>넥스틸</t>
+          <t>흥구석유</t>
         </is>
       </c>
       <c r="D62" s="25" t="n">
@@ -2988,14 +2988,14 @@
         <v>0</v>
       </c>
       <c r="H62" s="28" t="n">
-        <v>0.07000000000000001</v>
+        <v>4.38</v>
       </c>
       <c r="I62" s="28" t="n">
-        <v>10.7</v>
+        <v>35.8</v>
       </c>
       <c r="J62" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +118%</t>
+          <t>네이버 검색 당일 +115%</t>
         </is>
       </c>
       <c r="K62" s="29" t="inlineStr">
@@ -3007,7 +3007,7 @@
     <row r="63" ht="18" customHeight="1">
       <c r="A63" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B63" s="25" t="n">
@@ -3015,7 +3015,7 @@
       </c>
       <c r="C63" s="26" t="inlineStr">
         <is>
-          <t>우리기술</t>
+          <t>모니터랩</t>
         </is>
       </c>
       <c r="D63" s="25" t="n">
@@ -3030,15 +3030,15 @@
       <c r="G63" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H63" s="27" t="n">
-        <v>-3.77</v>
+      <c r="H63" s="28" t="n">
+        <v>5.53</v>
       </c>
       <c r="I63" s="28" t="n">
-        <v>32.17</v>
+        <v>17.05</v>
       </c>
       <c r="J63" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +115%</t>
+          <t>네이버 검색 당일 +108%</t>
         </is>
       </c>
       <c r="K63" s="29" t="inlineStr">
@@ -3140,22 +3140,22 @@
         <v>1</v>
       </c>
       <c r="C3" s="25" t="n">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="D3" s="25" t="n">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="E3" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F3" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G3" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="H3" s="25" t="n"/>
@@ -3164,38 +3164,42 @@
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="26" t="inlineStr">
         <is>
-          <t>인공지능</t>
+          <t>삼성전자</t>
         </is>
       </c>
       <c r="B4" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C4" s="25" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D4" s="25" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E4" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F4" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G4" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="H4" s="25" t="n"/>
-      <c r="I4" s="25" t="n"/>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="H4" s="27" t="n">
+        <v>-4.24</v>
+      </c>
+      <c r="I4" s="27" t="n">
+        <v>-7.96</v>
+      </c>
     </row>
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="26" t="inlineStr">
         <is>
-          <t>바이오</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="B5" s="25" t="n">
@@ -3212,12 +3216,12 @@
       </c>
       <c r="F5" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G5" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="H5" s="25" t="n"/>
@@ -3243,117 +3247,113 @@
       </c>
       <c r="F6" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G6" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="H6" s="27" t="n">
-        <v>-4.66</v>
+        <v>-0.89</v>
       </c>
       <c r="I6" s="27" t="n">
-        <v>-7.1</v>
+        <v>-10.44</v>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="26" t="inlineStr">
         <is>
-          <t>삼성전자</t>
+          <t>KB금융</t>
         </is>
       </c>
       <c r="B7" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="25" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D7" s="25" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="E7" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F7" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G7" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="H7" s="27" t="n">
-        <v>-3.53</v>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="H7" s="28" t="n">
+        <v>1.85</v>
       </c>
       <c r="I7" s="28" t="n">
-        <v>1.57</v>
+        <v>3.01</v>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="26" t="inlineStr">
         <is>
-          <t>KB금융</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="B8" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="25" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D8" s="25" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E8" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F8" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G8" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="H8" s="28" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="I8" s="28" t="n">
-        <v>3.43</v>
-      </c>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="H8" s="25" t="n"/>
+      <c r="I8" s="25" t="n"/>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="26" t="inlineStr">
         <is>
-          <t>원전</t>
+          <t>바이오</t>
         </is>
       </c>
       <c r="B9" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="25" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D9" s="25" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E9" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F9" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G9" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="H9" s="25" t="n"/>
@@ -3362,73 +3362,77 @@
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="26" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>KS인더스트리</t>
         </is>
       </c>
       <c r="B10" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C10" s="25" t="n">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="D10" s="25" t="n">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="E10" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F10" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G10" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="H10" s="25" t="n"/>
-      <c r="I10" s="25" t="n"/>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="H10" s="28" t="n">
+        <v>29.97</v>
+      </c>
+      <c r="I10" s="28" t="n">
+        <v>48.4</v>
+      </c>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="26" t="inlineStr">
         <is>
-          <t>삼성전자우</t>
+          <t>SK하이닉스</t>
         </is>
       </c>
       <c r="B11" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="25" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D11" s="25" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E11" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F11" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G11" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="H11" s="27" t="n">
-        <v>-4.78</v>
-      </c>
-      <c r="I11" s="28" t="n">
-        <v>0.89</v>
+        <v>-7.12</v>
+      </c>
+      <c r="I11" s="27" t="n">
+        <v>-5.61</v>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="26" t="inlineStr">
         <is>
-          <t>DB</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="B12" s="25" t="n">
@@ -3445,25 +3449,21 @@
       </c>
       <c r="F12" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G12" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="H12" s="27" t="n">
-        <v>-0.06</v>
-      </c>
-      <c r="I12" s="28" t="n">
-        <v>9.42</v>
-      </c>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="H12" s="25" t="n"/>
+      <c r="I12" s="25" t="n"/>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>셀트리온</t>
+          <t>현대건설</t>
         </is>
       </c>
       <c r="B13" s="25" t="n">
@@ -3480,95 +3480,95 @@
       </c>
       <c r="F13" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G13" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="H13" s="27" t="n">
-        <v>-1.44</v>
+        <v>-6.97</v>
       </c>
       <c r="I13" s="27" t="n">
-        <v>-5.26</v>
+        <v>-1.1</v>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>LG디스플레이</t>
+          <t>우리로</t>
         </is>
       </c>
       <c r="B14" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C14" s="25" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D14" s="25" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E14" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F14" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G14" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="H14" s="27" t="n">
-        <v>-0.78</v>
-      </c>
-      <c r="I14" s="27" t="n">
-        <v>-2.52</v>
+        <v>-0.97</v>
+      </c>
+      <c r="I14" s="28" t="n">
+        <v>46.65</v>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>더코디</t>
+          <t>코나아이</t>
         </is>
       </c>
       <c r="B15" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C15" s="25" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D15" s="25" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E15" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F15" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G15" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="H15" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="I15" s="28" t="n">
-        <v>185.01</v>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="H15" s="28" t="n">
+        <v>7</v>
+      </c>
+      <c r="I15" s="25" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>루멘스</t>
+          <t>고영</t>
         </is>
       </c>
       <c r="B16" s="25" t="n">
@@ -3585,25 +3585,25 @@
       </c>
       <c r="F16" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G16" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="H16" s="28" t="n">
-        <v>0.39</v>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="H16" s="27" t="n">
+        <v>-3.62</v>
       </c>
       <c r="I16" s="27" t="n">
-        <v>-5.58</v>
+        <v>-5.16</v>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>삼성전기</t>
+          <t>방산</t>
         </is>
       </c>
       <c r="B17" s="25" t="n">
@@ -3620,25 +3620,21 @@
       </c>
       <c r="F17" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G17" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="H17" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="I17" s="27" t="n">
-        <v>-0.07000000000000001</v>
-      </c>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="H17" s="25" t="n"/>
+      <c r="I17" s="25" t="n"/>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="26" t="inlineStr">
         <is>
-          <t>에스투더블유</t>
+          <t>현대차</t>
         </is>
       </c>
       <c r="B18" s="25" t="n">
@@ -3655,25 +3651,25 @@
       </c>
       <c r="F18" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G18" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="H18" s="28" t="n">
-        <v>26.38</v>
-      </c>
-      <c r="I18" s="28" t="n">
-        <v>52.78</v>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="H18" s="27" t="n">
+        <v>-3.92</v>
+      </c>
+      <c r="I18" s="27" t="n">
+        <v>-6.49</v>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>방산</t>
+          <t>GS</t>
         </is>
       </c>
       <c r="B19" s="25" t="n">
@@ -3690,161 +3686,161 @@
       </c>
       <c r="F19" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G19" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="H19" s="25" t="n"/>
-      <c r="I19" s="25" t="n"/>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="H19" s="27" t="n">
+        <v>-3.87</v>
+      </c>
+      <c r="I19" s="27" t="n">
+        <v>-8.92</v>
+      </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="26" t="inlineStr">
         <is>
-          <t>KT</t>
+          <t>LG전자</t>
         </is>
       </c>
       <c r="B20" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C20" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D20" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E20" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F20" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G20" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="H20" s="28" t="n">
-        <v>1.35</v>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="H20" s="27" t="n">
+        <v>-2.31</v>
       </c>
       <c r="I20" s="27" t="n">
-        <v>-2.95</v>
+        <v>-8.93</v>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="26" t="inlineStr">
         <is>
-          <t>삼성바이오로직스</t>
+          <t>넥사다이내믹스</t>
         </is>
       </c>
       <c r="B21" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C21" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D21" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E21" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F21" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G21" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="H21" s="27" t="n">
-        <v>-0.5600000000000001</v>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="H21" s="28" t="n">
+        <v>2</v>
       </c>
       <c r="I21" s="27" t="n">
-        <v>-2.21</v>
+        <v>-5.65</v>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="26" t="inlineStr">
         <is>
-          <t>수성웹툰</t>
+          <t>삼성바이오로직스</t>
         </is>
       </c>
       <c r="B22" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C22" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D22" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E22" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F22" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G22" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="H22" s="27" t="n">
-        <v>-25.47</v>
+        <v>-0.92</v>
       </c>
       <c r="I22" s="27" t="n">
-        <v>-49.62</v>
+        <v>-4.37</v>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="26" t="inlineStr">
         <is>
-          <t>아티스트스튜디오</t>
+          <t>조선</t>
         </is>
       </c>
       <c r="B23" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C23" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D23" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E23" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F23" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G23" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="H23" s="27" t="n">
-        <v>-13.9</v>
-      </c>
-      <c r="I23" s="27" t="n">
-        <v>-8.789999999999999</v>
-      </c>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="H23" s="25" t="n"/>
+      <c r="I23" s="25" t="n"/>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="26" t="inlineStr">
         <is>
-          <t>에넥스</t>
+          <t>삼성중공업</t>
         </is>
       </c>
       <c r="B24" s="25" t="n">
@@ -3861,25 +3857,25 @@
       </c>
       <c r="F24" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G24" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="H24" s="28" t="n">
-        <v>10.85</v>
+        <v>3.27</v>
       </c>
       <c r="I24" s="28" t="n">
-        <v>14.32</v>
+        <v>3.27</v>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="26" t="inlineStr">
         <is>
-          <t>원풍물산</t>
+          <t>수성웹툰</t>
         </is>
       </c>
       <c r="B25" s="25" t="n">
@@ -3896,25 +3892,25 @@
       </c>
       <c r="F25" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G25" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="H25" s="27" t="n">
-        <v>-1.47</v>
+        <v>-14.07</v>
       </c>
       <c r="I25" s="27" t="n">
-        <v>-68.62</v>
+        <v>-66.67</v>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="26" t="inlineStr">
         <is>
-          <t>코다코</t>
+          <t>아모레퍼시픽</t>
         </is>
       </c>
       <c r="B26" s="25" t="n">
@@ -3931,25 +3927,25 @@
       </c>
       <c r="F26" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G26" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="H26" s="28" t="n">
-        <v>10.24</v>
-      </c>
-      <c r="I26" s="27" t="n">
-        <v>-99.45</v>
+        <v>2.78</v>
+      </c>
+      <c r="I26" s="28" t="n">
+        <v>2.56</v>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="26" t="inlineStr">
         <is>
-          <t>코스나인</t>
+          <t>원전</t>
         </is>
       </c>
       <c r="B27" s="25" t="n">
@@ -3966,25 +3962,21 @@
       </c>
       <c r="F27" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G27" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="H27" s="27" t="n">
-        <v>-23.08</v>
-      </c>
-      <c r="I27" s="27" t="n">
-        <v>-97.92</v>
-      </c>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="H27" s="25" t="n"/>
+      <c r="I27" s="25" t="n"/>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="26" t="inlineStr">
         <is>
-          <t>한국석유</t>
+          <t>원풍물산</t>
         </is>
       </c>
       <c r="B28" s="25" t="n">
@@ -4001,25 +3993,25 @@
       </c>
       <c r="F28" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G28" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="H28" s="27" t="n">
-        <v>-3.22</v>
-      </c>
-      <c r="I28" s="28" t="n">
-        <v>8.83</v>
+        <v>-26.12</v>
+      </c>
+      <c r="I28" s="27" t="n">
+        <v>-66.89</v>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="26" t="inlineStr">
         <is>
-          <t>현대차</t>
+          <t>인피니트헬스케어</t>
         </is>
       </c>
       <c r="B29" s="25" t="n">
@@ -4036,130 +4028,126 @@
       </c>
       <c r="F29" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G29" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="H29" s="27" t="n">
-        <v>-1.67</v>
-      </c>
-      <c r="I29" s="27" t="n">
-        <v>-0.26</v>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="H29" s="28" t="n">
+        <v>30</v>
+      </c>
+      <c r="I29" s="28" t="n">
+        <v>24.29</v>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="26" t="inlineStr">
         <is>
-          <t>금강철강</t>
+          <t>전기차</t>
         </is>
       </c>
       <c r="B30" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C30" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D30" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E30" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F30" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G30" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="H30" s="28" t="n">
-        <v>2.34</v>
-      </c>
-      <c r="I30" s="28" t="n">
-        <v>30.51</v>
-      </c>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="H30" s="25" t="n"/>
+      <c r="I30" s="25" t="n"/>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="26" t="inlineStr">
         <is>
-          <t>넥스틸</t>
+          <t>코다코</t>
         </is>
       </c>
       <c r="B31" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C31" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D31" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E31" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F31" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G31" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="H31" s="28" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="I31" s="28" t="n">
-        <v>10.7</v>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="H31" s="27" t="n">
+        <v>-33.63</v>
+      </c>
+      <c r="I31" s="27" t="n">
+        <v>-99.64</v>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="26" t="inlineStr">
         <is>
-          <t>드림시큐리티</t>
+          <t>코스나인</t>
         </is>
       </c>
       <c r="B32" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C32" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D32" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E32" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F32" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G32" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="H32" s="28" t="n">
-        <v>23.29</v>
-      </c>
-      <c r="I32" s="28" t="n">
-        <v>29.38</v>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="H32" s="27" t="n">
+        <v>-30</v>
+      </c>
+      <c r="I32" s="27" t="n">
+        <v>-98.54000000000001</v>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="26" t="inlineStr">
         <is>
-          <t>머큐리</t>
+          <t>금강철강</t>
         </is>
       </c>
       <c r="B33" s="25" t="n">
@@ -4176,25 +4164,25 @@
       </c>
       <c r="F33" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G33" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="H33" s="27" t="n">
-        <v>-4.43</v>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="H33" s="28" t="n">
+        <v>0.13</v>
       </c>
       <c r="I33" s="28" t="n">
-        <v>39.71</v>
+        <v>22.93</v>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="26" t="inlineStr">
         <is>
-          <t>빛과전자</t>
+          <t>넥스틸</t>
         </is>
       </c>
       <c r="B34" s="25" t="n">
@@ -4211,25 +4199,25 @@
       </c>
       <c r="F34" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G34" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="H34" s="27" t="n">
-        <v>-1.4</v>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="H34" s="28" t="n">
+        <v>1.53</v>
       </c>
       <c r="I34" s="28" t="n">
-        <v>42.54</v>
+        <v>10.27</v>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="26" t="inlineStr">
         <is>
-          <t>삼미금속</t>
+          <t>드림시큐리티</t>
         </is>
       </c>
       <c r="B35" s="25" t="n">
@@ -4246,25 +4234,25 @@
       </c>
       <c r="F35" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G35" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="H35" s="27" t="n">
-        <v>-2.69</v>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="H35" s="28" t="n">
+        <v>5.53</v>
       </c>
       <c r="I35" s="28" t="n">
-        <v>47.19</v>
+        <v>37.22</v>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="26" t="inlineStr">
         <is>
-          <t>샌즈랩</t>
+          <t>머큐리</t>
         </is>
       </c>
       <c r="B36" s="25" t="n">
@@ -4281,25 +4269,25 @@
       </c>
       <c r="F36" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G36" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="H36" s="28" t="n">
-        <v>29.8</v>
+        <v>0.11</v>
       </c>
       <c r="I36" s="28" t="n">
-        <v>31.03</v>
+        <v>41.31</v>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="26" t="inlineStr">
         <is>
-          <t>샘표식품</t>
+          <t>메가터치</t>
         </is>
       </c>
       <c r="B37" s="25" t="n">
@@ -4316,25 +4304,25 @@
       </c>
       <c r="F37" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G37" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="H37" s="27" t="n">
-        <v>-14.76</v>
+        <v>-1.19</v>
       </c>
       <c r="I37" s="28" t="n">
-        <v>10.78</v>
+        <v>17.49</v>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="26" t="inlineStr">
         <is>
-          <t>서전기전</t>
+          <t>모니터랩</t>
         </is>
       </c>
       <c r="B38" s="25" t="n">
@@ -4351,25 +4339,25 @@
       </c>
       <c r="F38" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G38" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="H38" s="27" t="n">
-        <v>-3.51</v>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="H38" s="28" t="n">
+        <v>5.53</v>
       </c>
       <c r="I38" s="28" t="n">
-        <v>24.43</v>
+        <v>17.05</v>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="26" t="inlineStr">
         <is>
-          <t>스트라드비젼</t>
+          <t>빛과전자</t>
         </is>
       </c>
       <c r="B39" s="25" t="n">
@@ -4386,25 +4374,25 @@
       </c>
       <c r="F39" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G39" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="H39" s="27" t="n">
-        <v>-0.39</v>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="H39" s="28" t="n">
+        <v>12.53</v>
       </c>
       <c r="I39" s="28" t="n">
-        <v>35.05</v>
+        <v>55.54</v>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="26" t="inlineStr">
         <is>
-          <t>아모텍</t>
+          <t>빛샘전자</t>
         </is>
       </c>
       <c r="B40" s="25" t="n">
@@ -4421,25 +4409,25 @@
       </c>
       <c r="F40" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G40" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="H40" s="28" t="n">
-        <v>29.98</v>
+        <v>30</v>
       </c>
       <c r="I40" s="28" t="n">
-        <v>34.01</v>
+        <v>38.4</v>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="26" t="inlineStr">
         <is>
-          <t>액스비스</t>
+          <t>삼미금속</t>
         </is>
       </c>
       <c r="B41" s="25" t="n">
@@ -4456,25 +4444,25 @@
       </c>
       <c r="F41" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G41" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="H41" s="28" t="n">
-        <v>11.97</v>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="H41" s="27" t="n">
+        <v>-8.220000000000001</v>
       </c>
       <c r="I41" s="28" t="n">
-        <v>57.45</v>
+        <v>10.59</v>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="26" t="inlineStr">
         <is>
-          <t>엑스게이트</t>
+          <t>샌즈랩</t>
         </is>
       </c>
       <c r="B42" s="25" t="n">
@@ -4491,25 +4479,25 @@
       </c>
       <c r="F42" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G42" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="H42" s="28" t="n">
-        <v>29.94</v>
+        <v>29.95</v>
       </c>
       <c r="I42" s="28" t="n">
-        <v>40.51</v>
+        <v>70.48</v>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="26" t="inlineStr">
         <is>
-          <t>엔에이치스팩34호</t>
+          <t>아모텍</t>
         </is>
       </c>
       <c r="B43" s="25" t="n">
@@ -4526,25 +4514,25 @@
       </c>
       <c r="F43" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G43" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="H43" s="27" t="n">
-        <v>-6.94</v>
-      </c>
-      <c r="I43" s="27" t="n">
-        <v>-6.94</v>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="H43" s="28" t="n">
+        <v>4.43</v>
+      </c>
+      <c r="I43" s="28" t="n">
+        <v>41.07</v>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="26" t="inlineStr">
         <is>
-          <t>오르비텍</t>
+          <t>액스비스</t>
         </is>
       </c>
       <c r="B44" s="25" t="n">
@@ -4561,25 +4549,25 @@
       </c>
       <c r="F44" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G44" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="H44" s="27" t="n">
-        <v>-3.34</v>
+        <v>-3.59</v>
       </c>
       <c r="I44" s="28" t="n">
-        <v>40.35</v>
+        <v>47.72</v>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="26" t="inlineStr">
         <is>
-          <t>우리기술</t>
+          <t>에스엠벡셀</t>
         </is>
       </c>
       <c r="B45" s="25" t="n">
@@ -4596,25 +4584,25 @@
       </c>
       <c r="F45" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G45" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="H45" s="27" t="n">
-        <v>-3.77</v>
+        <v>-8.199999999999999</v>
       </c>
       <c r="I45" s="28" t="n">
-        <v>32.17</v>
+        <v>38.56</v>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="26" t="inlineStr">
         <is>
-          <t>우리넷</t>
+          <t>에스투더블유</t>
         </is>
       </c>
       <c r="B46" s="25" t="n">
@@ -4631,25 +4619,25 @@
       </c>
       <c r="F46" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G46" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="H46" s="28" t="n">
-        <v>3.49</v>
+        <v>7.95</v>
       </c>
       <c r="I46" s="28" t="n">
-        <v>15.6</v>
+        <v>66.98</v>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="26" t="inlineStr">
         <is>
-          <t>우리로</t>
+          <t>엑스게이트</t>
         </is>
       </c>
       <c r="B47" s="25" t="n">
@@ -4666,25 +4654,25 @@
       </c>
       <c r="F47" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G47" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="H47" s="28" t="n">
-        <v>7.31</v>
+        <v>6.97</v>
       </c>
       <c r="I47" s="28" t="n">
-        <v>48.55</v>
+        <v>51.63</v>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="26" t="inlineStr">
         <is>
-          <t>원익피앤이</t>
+          <t>엔에이치스팩34호</t>
         </is>
       </c>
       <c r="B48" s="25" t="n">
@@ -4701,25 +4689,25 @@
       </c>
       <c r="F48" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G48" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="H48" s="28" t="n">
-        <v>6.62</v>
-      </c>
-      <c r="I48" s="28" t="n">
-        <v>41</v>
+        <v>0.16</v>
+      </c>
+      <c r="I48" s="27" t="n">
+        <v>-6.8</v>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="26" t="inlineStr">
         <is>
-          <t>카프로</t>
+          <t>우리기술</t>
         </is>
       </c>
       <c r="B49" s="25" t="n">
@@ -4736,25 +4724,25 @@
       </c>
       <c r="F49" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G49" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="H49" s="27" t="n">
-        <v>-16.67</v>
-      </c>
-      <c r="I49" s="27" t="n">
-        <v>-96.72</v>
+        <v>-2.35</v>
+      </c>
+      <c r="I49" s="28" t="n">
+        <v>25.64</v>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="26" t="inlineStr">
         <is>
-          <t>케이에스피</t>
+          <t>우리넷</t>
         </is>
       </c>
       <c r="B50" s="25" t="n">
@@ -4771,25 +4759,25 @@
       </c>
       <c r="F50" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G50" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="H50" s="28" t="n">
-        <v>6.57</v>
+        <v>7.71</v>
       </c>
       <c r="I50" s="28" t="n">
-        <v>29.35</v>
+        <v>24.69</v>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="26" t="inlineStr">
         <is>
-          <t>피아이이</t>
+          <t>카프로</t>
         </is>
       </c>
       <c r="B51" s="25" t="n">
@@ -4806,25 +4794,25 @@
       </c>
       <c r="F51" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G51" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="H51" s="28" t="n">
-        <v>7.61</v>
-      </c>
-      <c r="I51" s="28" t="n">
-        <v>37.84</v>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="H51" s="27" t="n">
+        <v>-40.83</v>
+      </c>
+      <c r="I51" s="27" t="n">
+        <v>-98.06</v>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="26" t="inlineStr">
         <is>
-          <t>한빛레이저</t>
+          <t>흥구석유</t>
         </is>
       </c>
       <c r="B52" s="25" t="n">
@@ -4841,19 +4829,19 @@
       </c>
       <c r="F52" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G52" s="25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="H52" s="28" t="n">
-        <v>2.83</v>
+        <v>4.38</v>
       </c>
       <c r="I52" s="28" t="n">
-        <v>36.01</v>
+        <v>35.8</v>
       </c>
     </row>
   </sheetData>
@@ -4937,19 +4925,19 @@
         <v>1</v>
       </c>
       <c r="C3" s="36" t="n">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="D3" s="36" t="n">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="E3" s="36" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="F3" s="37" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G3" s="37" t="inlineStr">
@@ -4968,19 +4956,19 @@
         <v>1</v>
       </c>
       <c r="C4" s="36" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="D4" s="36" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="E4" s="36" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="F4" s="37" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G4" s="37" t="inlineStr">
@@ -4992,26 +4980,26 @@
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="35" t="inlineStr">
         <is>
-          <t>방산</t>
+          <t>전기차</t>
         </is>
       </c>
       <c r="B5" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="36" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D5" s="36" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E5" s="36" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="F5" s="37" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G5" s="37" t="inlineStr">
@@ -5023,26 +5011,26 @@
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="35" t="inlineStr">
         <is>
-          <t>원전</t>
+          <t>방산</t>
         </is>
       </c>
       <c r="B6" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="36" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="D6" s="36" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="E6" s="36" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="F6" s="37" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G6" s="37" t="inlineStr">
@@ -5054,26 +5042,26 @@
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="35" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>원전</t>
         </is>
       </c>
       <c r="B7" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="36" t="n">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="D7" s="36" t="n">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="E7" s="36" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="F7" s="37" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G7" s="37" t="inlineStr">
@@ -5085,119 +5073,131 @@
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="35" t="inlineStr">
         <is>
+          <t>로봇</t>
+        </is>
+      </c>
+      <c r="B8" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" s="36" t="n">
+        <v>18</v>
+      </c>
+      <c r="D8" s="36" t="n">
+        <v>18</v>
+      </c>
+      <c r="E8" s="36" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="F8" s="37" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="G8" s="37" t="inlineStr">
+        <is>
+          <t>⚡ 관심</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="35" t="inlineStr">
+        <is>
+          <t>조선</t>
+        </is>
+      </c>
+      <c r="B9" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" s="36" t="n">
+        <v>5</v>
+      </c>
+      <c r="D9" s="36" t="n">
+        <v>5</v>
+      </c>
+      <c r="E9" s="36" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="F9" s="37" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="G9" s="37" t="inlineStr">
+        <is>
+          <t>⚡ 관심</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="35" t="inlineStr">
+        <is>
+          <t>제약</t>
+        </is>
+      </c>
+      <c r="B10" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" s="36" t="n">
+        <v>8</v>
+      </c>
+      <c r="D10" s="36" t="n">
+        <v>8</v>
+      </c>
+      <c r="E10" s="36" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="F10" s="37" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="G10" s="37" t="inlineStr">
+        <is>
+          <t>⚡ 관심</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="35" t="inlineStr">
+        <is>
           <t>인공지능</t>
         </is>
       </c>
-      <c r="B8" s="36" t="n">
-        <v>1</v>
-      </c>
-      <c r="C8" s="36" t="n">
-        <v>21</v>
-      </c>
-      <c r="D8" s="36" t="n">
-        <v>21</v>
-      </c>
-      <c r="E8" s="36" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="F8" s="37" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="G8" s="37" t="inlineStr">
+      <c r="B11" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" s="36" t="n">
+        <v>15</v>
+      </c>
+      <c r="D11" s="36" t="n">
+        <v>15</v>
+      </c>
+      <c r="E11" s="36" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="F11" s="37" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="G11" s="37" t="inlineStr">
         <is>
           <t>⚡ 관심</t>
         </is>
       </c>
-    </row>
-    <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="26" t="inlineStr">
-        <is>
-          <t>이차전지</t>
-        </is>
-      </c>
-      <c r="B9" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="C9" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="D9" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="E9" s="25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F9" s="29" t="inlineStr">
-        <is>
-          <t>감지 없음</t>
-        </is>
-      </c>
-      <c r="G9" s="29" t="inlineStr"/>
-    </row>
-    <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="26" t="inlineStr">
-        <is>
-          <t>AI반도체</t>
-        </is>
-      </c>
-      <c r="B10" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="C10" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="D10" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="E10" s="25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F10" s="29" t="inlineStr">
-        <is>
-          <t>감지 없음</t>
-        </is>
-      </c>
-      <c r="G10" s="29" t="inlineStr"/>
-    </row>
-    <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="26" t="inlineStr">
-        <is>
-          <t>전기차</t>
-        </is>
-      </c>
-      <c r="B11" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="C11" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="D11" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" s="25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F11" s="29" t="inlineStr">
-        <is>
-          <t>감지 없음</t>
-        </is>
-      </c>
-      <c r="G11" s="29" t="inlineStr"/>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="26" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>이차전지</t>
         </is>
       </c>
       <c r="B12" s="25" t="n">
@@ -5224,7 +5224,7 @@
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>수소</t>
+          <t>AI반도체</t>
         </is>
       </c>
       <c r="B13" s="25" t="n">
@@ -5251,7 +5251,7 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>태양광</t>
+          <t>수소</t>
         </is>
       </c>
       <c r="B14" s="25" t="n">
@@ -5278,7 +5278,7 @@
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>게임</t>
+          <t>태양광</t>
         </is>
       </c>
       <c r="B15" s="25" t="n">
@@ -5305,7 +5305,7 @@
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>엔터</t>
+          <t>게임</t>
         </is>
       </c>
       <c r="B16" s="25" t="n">
@@ -5332,7 +5332,7 @@
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>핀테크</t>
+          <t>엔터</t>
         </is>
       </c>
       <c r="B17" s="25" t="n">
@@ -5359,7 +5359,7 @@
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="26" t="inlineStr">
         <is>
-          <t>클라우드</t>
+          <t>핀테크</t>
         </is>
       </c>
       <c r="B18" s="25" t="n">
@@ -5386,7 +5386,7 @@
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>조선</t>
+          <t>클라우드</t>
         </is>
       </c>
       <c r="B19" s="25" t="n">

</xml_diff>

<commit_message>
auto: 2026-09-19 07:14 자동 백업
</commit_message>
<xml_diff>
--- a/trend/stock_trend_history.xlsx
+++ b/trend/stock_trend_history.xlsx
@@ -258,11 +258,11 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -694,7 +694,7 @@
     <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-09-18 06:54</t>
+          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-09-19 06:54</t>
         </is>
       </c>
     </row>
@@ -787,21 +787,21 @@
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-09-18) 상위: 반도체  점수 46.0점</t>
+          <t>⚡ 최신(2026-09-19) 상위: 반도체  점수 50.0점</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-09-18) 상위: 인공지능  점수 17.0점</t>
+          <t>⚡ 최신(2026-09-19) 상위: 바이오  점수 20.0점</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-09-18) 상위: SK하이닉스  점수 16.0점</t>
+          <t>⚡ 최신(2026-09-19) 상위: 삼성전자  점수 19.0점</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="15" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B14" s="15" t="n">
@@ -928,10 +928,10 @@
         </is>
       </c>
       <c r="D14" s="15" t="n">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="E14" s="15" t="n">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="F14" s="15" t="n">
         <v>0</v>
@@ -947,7 +947,7 @@
       </c>
       <c r="J14" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급</t>
         </is>
       </c>
       <c r="K14" s="17" t="inlineStr">
@@ -959,7 +959,7 @@
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="15" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B15" s="15" t="n">
@@ -967,14 +967,14 @@
       </c>
       <c r="C15" s="16" t="inlineStr">
         <is>
-          <t>인공지능</t>
+          <t>바이오</t>
         </is>
       </c>
       <c r="D15" s="15" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E15" s="15" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="F15" s="15" t="n">
         <v>0</v>
@@ -990,7 +990,7 @@
       </c>
       <c r="J15" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+          <t>매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K15" s="17" t="inlineStr">
@@ -1002,7 +1002,7 @@
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="15" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B16" s="15" t="n">
@@ -1010,14 +1010,14 @@
       </c>
       <c r="C16" s="16" t="inlineStr">
         <is>
-          <t>SK하이닉스</t>
+          <t>삼성전자</t>
         </is>
       </c>
       <c r="D16" s="15" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="E16" s="15" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="F16" s="15" t="n">
         <v>0</v>
@@ -1026,26 +1026,24 @@
         <v>0</v>
       </c>
       <c r="H16" s="18" t="n">
-        <v>0.51</v>
-      </c>
-      <c r="I16" s="19" t="n">
-        <v>-4.7</v>
+        <v>1.56</v>
+      </c>
+      <c r="I16" s="18" t="n">
+        <v>0.19</v>
       </c>
       <c r="J16" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K16" s="17" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K16" s="17" t="n">
+        <v/>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B17" s="15" t="n">
@@ -1053,14 +1051,14 @@
       </c>
       <c r="C17" s="16" t="inlineStr">
         <is>
-          <t>삼성전자</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="D17" s="15" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E17" s="15" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F17" s="15" t="n">
         <v>0</v>
@@ -1068,25 +1066,27 @@
       <c r="G17" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H17" s="18" t="n">
-        <v>0.99</v>
-      </c>
-      <c r="I17" s="19" t="n">
-        <v>-4.83</v>
+      <c r="H17" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I17" s="15" t="n">
+        <v/>
       </c>
       <c r="J17" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K17" s="17" t="n">
-        <v/>
+          <t>네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
+        </is>
+      </c>
+      <c r="K17" s="17" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B18" s="15" t="n">
@@ -1094,14 +1094,14 @@
       </c>
       <c r="C18" s="16" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>SK하이닉스</t>
         </is>
       </c>
       <c r="D18" s="15" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="E18" s="15" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F18" s="15" t="n">
         <v>0</v>
@@ -1109,25 +1109,27 @@
       <c r="G18" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H18" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I18" s="15" t="n">
-        <v/>
+      <c r="H18" s="18" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="I18" s="18" t="n">
+        <v>2.04</v>
       </c>
       <c r="J18" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K18" s="17" t="n">
-        <v/>
+          <t>매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K18" s="17" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B19" s="15" t="n">
@@ -1135,14 +1137,14 @@
       </c>
       <c r="C19" s="16" t="inlineStr">
         <is>
-          <t>원전</t>
+          <t>삼성전기</t>
         </is>
       </c>
       <c r="D19" s="15" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E19" s="15" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F19" s="15" t="n">
         <v>0</v>
@@ -1150,15 +1152,15 @@
       <c r="G19" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H19" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I19" s="15" t="n">
-        <v/>
+      <c r="H19" s="18" t="n">
+        <v>2.74</v>
+      </c>
+      <c r="I19" s="19" t="n">
+        <v>-0.86</v>
       </c>
       <c r="J19" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K19" s="17" t="n">
@@ -1168,7 +1170,7 @@
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B20" s="15" t="n">
@@ -1176,14 +1178,14 @@
       </c>
       <c r="C20" s="16" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>LG</t>
         </is>
       </c>
       <c r="D20" s="15" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E20" s="15" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F20" s="15" t="n">
         <v>0</v>
@@ -1191,15 +1193,15 @@
       <c r="G20" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H20" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I20" s="15" t="n">
-        <v/>
+      <c r="H20" s="19" t="n">
+        <v>-0.62</v>
+      </c>
+      <c r="I20" s="19" t="n">
+        <v>-0.36</v>
       </c>
       <c r="J20" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K20" s="17" t="n">
@@ -1209,7 +1211,7 @@
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="15" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B21" s="15" t="n">
@@ -1217,14 +1219,14 @@
       </c>
       <c r="C21" s="16" t="inlineStr">
         <is>
-          <t>방산</t>
+          <t>한화시스템</t>
         </is>
       </c>
       <c r="D21" s="15" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E21" s="15" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F21" s="15" t="n">
         <v>0</v>
@@ -1232,25 +1234,27 @@
       <c r="G21" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H21" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I21" s="15" t="n">
-        <v/>
+      <c r="H21" s="18" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="I21" s="18" t="n">
+        <v>12.69</v>
       </c>
       <c r="J21" s="17" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K21" s="17" t="n">
-        <v/>
+          <t>중요공시 1건 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K21" s="17" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="15" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B22" s="15" t="n">
@@ -1258,42 +1262,42 @@
       </c>
       <c r="C22" s="16" t="inlineStr">
         <is>
-          <t>비투엔</t>
+          <t>미투온</t>
         </is>
       </c>
       <c r="D22" s="15" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E22" s="15" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F22" s="15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G22" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H22" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="I22" s="19" t="n">
-        <v>-8.470000000000001</v>
+      <c r="H22" s="19" t="n">
+        <v>-8.24</v>
+      </c>
+      <c r="I22" s="18" t="n">
+        <v>52.37</v>
       </c>
       <c r="J22" s="17" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 3일 +200% / 한국경제 헤드라인 언급</t>
+          <t>네이버 검색 당일 +952% / 중요공시 2건 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K22" s="17" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="15" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B23" s="15" t="n">
@@ -1301,42 +1305,42 @@
       </c>
       <c r="C23" s="16" t="inlineStr">
         <is>
-          <t>KS인더스트리</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="D23" s="15" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E23" s="15" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="F23" s="15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G23" s="15" t="n">
-        <v>3</v>
-      </c>
-      <c r="H23" s="19" t="n">
-        <v>-3.39</v>
-      </c>
-      <c r="I23" s="18" t="n">
-        <v>39.51</v>
+        <v>0</v>
+      </c>
+      <c r="H23" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I23" s="15" t="n">
+        <v/>
       </c>
       <c r="J23" s="17" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 3일 +50% / 중요공시 7일 +200%</t>
+          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K23" s="17" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="15" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B24" s="15" t="n">
@@ -1344,14 +1348,14 @@
       </c>
       <c r="C24" s="16" t="inlineStr">
         <is>
-          <t>철강</t>
+          <t>스테이블코인</t>
         </is>
       </c>
       <c r="D24" s="15" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E24" s="15" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F24" s="15" t="n">
         <v>0</v>
@@ -1367,19 +1371,17 @@
       </c>
       <c r="J24" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K24" s="17" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K24" s="17" t="n">
+        <v/>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="15" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B25" s="15" t="n">
@@ -1387,14 +1389,14 @@
       </c>
       <c r="C25" s="16" t="inlineStr">
         <is>
-          <t>카카오</t>
+          <t>게임</t>
         </is>
       </c>
       <c r="D25" s="15" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E25" s="15" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F25" s="15" t="n">
         <v>0</v>
@@ -1402,27 +1404,25 @@
       <c r="G25" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H25" s="18" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="I25" s="19" t="n">
-        <v>-3.15</v>
+      <c r="H25" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I25" s="15" t="n">
+        <v/>
       </c>
       <c r="J25" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K25" s="17" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+          <t>한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K25" s="17" t="n">
+        <v/>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="15" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B26" s="15" t="n">
@@ -1430,7 +1430,7 @@
       </c>
       <c r="C26" s="16" t="inlineStr">
         <is>
-          <t>미투온</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="D26" s="15" t="n">
@@ -1445,27 +1445,27 @@
       <c r="G26" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H26" s="18" t="n">
-        <v>18.49</v>
-      </c>
-      <c r="I26" s="18" t="n">
-        <v>67.90000000000001</v>
+      <c r="H26" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I26" s="15" t="n">
+        <v/>
       </c>
       <c r="J26" s="17" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +484% / 중요공시 2건 / 매일경제 헤드라인 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K26" s="17" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="20" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B27" s="20" t="n">
@@ -1473,7 +1473,7 @@
       </c>
       <c r="C27" s="21" t="inlineStr">
         <is>
-          <t>대모</t>
+          <t>전기차</t>
         </is>
       </c>
       <c r="D27" s="20" t="n">
@@ -1488,25 +1488,27 @@
       <c r="G27" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H27" s="22" t="n">
-        <v>5.24</v>
-      </c>
-      <c r="I27" s="22" t="n">
-        <v>0.48</v>
-      </c>
-      <c r="J27" s="23" t="inlineStr">
-        <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K27" s="23" t="n">
+      <c r="H27" s="20" t="n">
         <v/>
+      </c>
+      <c r="I27" s="20" t="n">
+        <v/>
+      </c>
+      <c r="J27" s="22" t="inlineStr">
+        <is>
+          <t>네이버뉴스 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K27" s="22" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="20" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B28" s="20" t="n">
@@ -1514,42 +1516,42 @@
       </c>
       <c r="C28" s="21" t="inlineStr">
         <is>
-          <t>현대건설</t>
+          <t>태양광</t>
         </is>
       </c>
       <c r="D28" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E28" s="20" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F28" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G28" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H28" s="22" t="n">
-        <v>2.02</v>
-      </c>
-      <c r="I28" s="24" t="n">
-        <v>-3.58</v>
-      </c>
-      <c r="J28" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 2건 / 중요공시 3일 +100% / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K28" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
+      <c r="H28" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I28" s="20" t="n">
+        <v/>
+      </c>
+      <c r="J28" s="22" t="inlineStr">
+        <is>
+          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K28" s="22" t="inlineStr">
+        <is>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="20" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B29" s="20" t="n">
@@ -1557,33 +1559,33 @@
       </c>
       <c r="C29" s="21" t="inlineStr">
         <is>
-          <t>한화시스템</t>
+          <t>GS건설</t>
         </is>
       </c>
       <c r="D29" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E29" s="20" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F29" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G29" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H29" s="22" t="n">
-        <v>15.53</v>
-      </c>
-      <c r="I29" s="22" t="n">
-        <v>9.94</v>
-      </c>
-      <c r="J29" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 1건 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K29" s="23" t="inlineStr">
+      <c r="H29" s="23" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="I29" s="24" t="n">
+        <v>-3.38</v>
+      </c>
+      <c r="J29" s="22" t="inlineStr">
+        <is>
+          <t>중요공시 3건 / 중요공시 3일 +50%</t>
+        </is>
+      </c>
+      <c r="K29" s="22" t="inlineStr">
         <is>
           <t>공시</t>
         </is>
@@ -1592,7 +1594,7 @@
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="20" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B30" s="20" t="n">
@@ -1600,40 +1602,42 @@
       </c>
       <c r="C30" s="21" t="inlineStr">
         <is>
-          <t>현대모비스</t>
+          <t>프리티</t>
         </is>
       </c>
       <c r="D30" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E30" s="20" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F30" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G30" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H30" s="20" t="n">
-        <v>0</v>
+      <c r="H30" s="24" t="n">
+        <v>-29.91</v>
       </c>
       <c r="I30" s="24" t="n">
-        <v>-7.7</v>
-      </c>
-      <c r="J30" s="23" t="inlineStr">
-        <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K30" s="23" t="n">
-        <v/>
+        <v>-35.77</v>
+      </c>
+      <c r="J30" s="22" t="inlineStr">
+        <is>
+          <t>중요공시 3건 / 중요공시 3일 +200%</t>
+        </is>
+      </c>
+      <c r="K30" s="22" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="20" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B31" s="20" t="n">
@@ -1641,14 +1645,14 @@
       </c>
       <c r="C31" s="21" t="inlineStr">
         <is>
-          <t>제일기획</t>
+          <t>조선</t>
         </is>
       </c>
       <c r="D31" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E31" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F31" s="20" t="n">
         <v>0</v>
@@ -1656,25 +1660,27 @@
       <c r="G31" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H31" s="24" t="n">
-        <v>-0.57</v>
-      </c>
-      <c r="I31" s="24" t="n">
-        <v>-7.26</v>
-      </c>
-      <c r="J31" s="23" t="inlineStr">
-        <is>
-          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K31" s="23" t="n">
+      <c r="H31" s="20" t="n">
         <v/>
+      </c>
+      <c r="I31" s="20" t="n">
+        <v/>
+      </c>
+      <c r="J31" s="22" t="inlineStr">
+        <is>
+          <t>Google 급상승 검색어 등장 (KR)</t>
+        </is>
+      </c>
+      <c r="K31" s="22" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="20" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B32" s="20" t="n">
@@ -1682,14 +1688,14 @@
       </c>
       <c r="C32" s="21" t="inlineStr">
         <is>
-          <t>조선</t>
+          <t>현대차</t>
         </is>
       </c>
       <c r="D32" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E32" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F32" s="20" t="n">
         <v>0</v>
@@ -1697,27 +1703,25 @@
       <c r="G32" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H32" s="20" t="n">
+      <c r="H32" s="23" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="I32" s="24" t="n">
+        <v>-4.18</v>
+      </c>
+      <c r="J32" s="22" t="inlineStr">
+        <is>
+          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K32" s="22" t="n">
         <v/>
-      </c>
-      <c r="I32" s="20" t="n">
-        <v/>
-      </c>
-      <c r="J32" s="23" t="inlineStr">
-        <is>
-          <t>매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K32" s="23" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="20" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B33" s="20" t="n">
@@ -1725,14 +1729,14 @@
       </c>
       <c r="C33" s="21" t="inlineStr">
         <is>
-          <t>바이오</t>
+          <t>뷰티스킨</t>
         </is>
       </c>
       <c r="D33" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E33" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F33" s="20" t="n">
         <v>0</v>
@@ -1740,27 +1744,27 @@
       <c r="G33" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H33" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I33" s="20" t="n">
-        <v/>
-      </c>
-      <c r="J33" s="23" t="inlineStr">
-        <is>
-          <t>매일경제 기사 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K33" s="23" t="inlineStr">
-        <is>
-          <t>네이버</t>
+      <c r="H33" s="23" t="n">
+        <v>9.699999999999999</v>
+      </c>
+      <c r="I33" s="23" t="n">
+        <v>28.54</v>
+      </c>
+      <c r="J33" s="22" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +173% / 중요공시 1건</t>
+        </is>
+      </c>
+      <c r="K33" s="22" t="inlineStr">
+        <is>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="20" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B34" s="20" t="n">
@@ -1768,14 +1772,14 @@
       </c>
       <c r="C34" s="21" t="inlineStr">
         <is>
-          <t>KT</t>
+          <t>비츠로테크</t>
         </is>
       </c>
       <c r="D34" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E34" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F34" s="20" t="n">
         <v>0</v>
@@ -1783,25 +1787,27 @@
       <c r="G34" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H34" s="22" t="n">
-        <v>1.13</v>
-      </c>
-      <c r="I34" s="22" t="n">
-        <v>3.08</v>
-      </c>
-      <c r="J34" s="23" t="inlineStr">
-        <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K34" s="23" t="n">
-        <v/>
+      <c r="H34" s="23" t="n">
+        <v>1.66</v>
+      </c>
+      <c r="I34" s="23" t="n">
+        <v>33.07</v>
+      </c>
+      <c r="J34" s="22" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +108% / 중요공시 1건</t>
+        </is>
+      </c>
+      <c r="K34" s="22" t="inlineStr">
+        <is>
+          <t>공시, 네이버</t>
+        </is>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="20" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B35" s="20" t="n">
@@ -1809,7 +1815,7 @@
       </c>
       <c r="C35" s="21" t="inlineStr">
         <is>
-          <t>이뮨온시아</t>
+          <t>대한항공</t>
         </is>
       </c>
       <c r="D35" s="20" t="n">
@@ -1824,27 +1830,25 @@
       <c r="G35" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H35" s="22" t="n">
-        <v>2.34</v>
-      </c>
-      <c r="I35" s="22" t="n">
-        <v>23.2</v>
-      </c>
-      <c r="J35" s="23" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +261% / 중요공시 2건</t>
-        </is>
-      </c>
-      <c r="K35" s="23" t="inlineStr">
-        <is>
-          <t>네이버, 공시</t>
-        </is>
+      <c r="H35" s="24" t="n">
+        <v>-1.35</v>
+      </c>
+      <c r="I35" s="23" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="J35" s="22" t="inlineStr">
+        <is>
+          <t>한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K35" s="22" t="n">
+        <v/>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="20" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B36" s="20" t="n">
@@ -1852,7 +1856,7 @@
       </c>
       <c r="C36" s="21" t="inlineStr">
         <is>
-          <t>한국첨단소재</t>
+          <t>한섬</t>
         </is>
       </c>
       <c r="D36" s="20" t="n">
@@ -1867,27 +1871,27 @@
       <c r="G36" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H36" s="24" t="n">
-        <v>-8.470000000000001</v>
-      </c>
-      <c r="I36" s="22" t="n">
-        <v>61.76</v>
-      </c>
-      <c r="J36" s="23" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +190% / 중요공시 1건</t>
-        </is>
-      </c>
-      <c r="K36" s="23" t="inlineStr">
-        <is>
-          <t>네이버, 공시</t>
+      <c r="H36" s="23" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="I36" s="23" t="n">
+        <v>15.81</v>
+      </c>
+      <c r="J36" s="22" t="inlineStr">
+        <is>
+          <t>중요공시 1건 / 네이버뉴스 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K36" s="22" t="inlineStr">
+        <is>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="20" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B37" s="20" t="n">
@@ -1895,7 +1899,7 @@
       </c>
       <c r="C37" s="21" t="inlineStr">
         <is>
-          <t>LG디스플레이</t>
+          <t>LS마린솔루션</t>
         </is>
       </c>
       <c r="D37" s="20" t="n">
@@ -1910,25 +1914,27 @@
       <c r="G37" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H37" s="24" t="n">
-        <v>-0.82</v>
-      </c>
-      <c r="I37" s="24" t="n">
-        <v>-5.91</v>
-      </c>
-      <c r="J37" s="23" t="inlineStr">
-        <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K37" s="23" t="n">
-        <v/>
+      <c r="H37" s="23" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="I37" s="23" t="n">
+        <v>4.18</v>
+      </c>
+      <c r="J37" s="22" t="inlineStr">
+        <is>
+          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K37" s="22" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="20" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B38" s="20" t="n">
@@ -1936,85 +1942,83 @@
       </c>
       <c r="C38" s="21" t="inlineStr">
         <is>
-          <t>시선AI</t>
+          <t>철강</t>
         </is>
       </c>
       <c r="D38" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E38" s="20" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F38" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G38" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="H38" s="24" t="n">
-        <v>-2.27</v>
-      </c>
-      <c r="I38" s="22" t="n">
-        <v>5.01</v>
-      </c>
-      <c r="J38" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 2건 / 중요공시 7일 +100%</t>
-        </is>
-      </c>
-      <c r="K38" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+        <v>0</v>
+      </c>
+      <c r="H38" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I38" s="20" t="n">
+        <v/>
+      </c>
+      <c r="J38" s="22" t="inlineStr">
+        <is>
+          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K38" s="22" t="n">
+        <v/>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
-      <c r="A39" s="20" t="inlineStr">
-        <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="B39" s="20" t="n">
+      <c r="A39" s="25" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B39" s="25" t="n">
         <v>26</v>
       </c>
-      <c r="C39" s="21" t="inlineStr">
-        <is>
-          <t>에이피알</t>
-        </is>
-      </c>
-      <c r="D39" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E39" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F39" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G39" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H39" s="22" t="n">
-        <v>1.28</v>
-      </c>
-      <c r="I39" s="24" t="n">
-        <v>-1.66</v>
-      </c>
-      <c r="J39" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 1건 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K39" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
+      <c r="C39" s="26" t="inlineStr">
+        <is>
+          <t>아이티센피엔에스</t>
+        </is>
+      </c>
+      <c r="D39" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E39" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F39" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G39" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H39" s="27" t="n">
+        <v>-3.01</v>
+      </c>
+      <c r="I39" s="28" t="n">
+        <v>66.41</v>
+      </c>
+      <c r="J39" s="29" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +700%</t>
+        </is>
+      </c>
+      <c r="K39" s="29" t="inlineStr">
+        <is>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B40" s="25" t="n">
@@ -2022,7 +2026,7 @@
       </c>
       <c r="C40" s="26" t="inlineStr">
         <is>
-          <t>아이티센피엔에스</t>
+          <t>빛샘전자</t>
         </is>
       </c>
       <c r="D40" s="25" t="n">
@@ -2037,15 +2041,15 @@
       <c r="G40" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H40" s="27" t="n">
-        <v>-4.6</v>
+      <c r="H40" s="28" t="n">
+        <v>3.86</v>
       </c>
       <c r="I40" s="28" t="n">
-        <v>74.28</v>
+        <v>57.08</v>
       </c>
       <c r="J40" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +316%</t>
+          <t>네이버 검색 당일 +366%</t>
         </is>
       </c>
       <c r="K40" s="29" t="inlineStr">
@@ -2057,7 +2061,7 @@
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B41" s="25" t="n">
@@ -2065,7 +2069,7 @@
       </c>
       <c r="C41" s="26" t="inlineStr">
         <is>
-          <t>동국산업</t>
+          <t>큐라티스</t>
         </is>
       </c>
       <c r="D41" s="25" t="n">
@@ -2080,15 +2084,15 @@
       <c r="G41" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H41" s="28" t="n">
-        <v>4.87</v>
+      <c r="H41" s="27" t="n">
+        <v>-5.09</v>
       </c>
       <c r="I41" s="28" t="n">
-        <v>40.24</v>
+        <v>58.13</v>
       </c>
       <c r="J41" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +310%</t>
+          <t>네이버 검색 당일 +261%</t>
         </is>
       </c>
       <c r="K41" s="29" t="inlineStr">
@@ -2100,7 +2104,7 @@
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B42" s="25" t="n">
@@ -2108,7 +2112,7 @@
       </c>
       <c r="C42" s="26" t="inlineStr">
         <is>
-          <t>빛샘전자</t>
+          <t>한켐</t>
         </is>
       </c>
       <c r="D42" s="25" t="n">
@@ -2124,14 +2128,14 @@
         <v>0</v>
       </c>
       <c r="H42" s="27" t="n">
-        <v>-3.24</v>
+        <v>-5.41</v>
       </c>
       <c r="I42" s="28" t="n">
-        <v>47.26</v>
+        <v>37.38</v>
       </c>
       <c r="J42" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +245%</t>
+          <t>네이버 검색 당일 +259%</t>
         </is>
       </c>
       <c r="K42" s="29" t="inlineStr">
@@ -2143,7 +2147,7 @@
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B43" s="25" t="n">
@@ -2167,14 +2171,14 @@
         <v>0</v>
       </c>
       <c r="H43" s="27" t="n">
-        <v>-3.81</v>
+        <v>-3.27</v>
       </c>
       <c r="I43" s="28" t="n">
-        <v>25.49</v>
+        <v>16.48</v>
       </c>
       <c r="J43" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +191%</t>
+          <t>네이버 검색 당일 +245%</t>
         </is>
       </c>
       <c r="K43" s="29" t="inlineStr">
@@ -2186,7 +2190,7 @@
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B44" s="25" t="n">
@@ -2194,7 +2198,7 @@
       </c>
       <c r="C44" s="26" t="inlineStr">
         <is>
-          <t>한컴위드</t>
+          <t>한국첨단소재</t>
         </is>
       </c>
       <c r="D44" s="25" t="n">
@@ -2210,14 +2214,14 @@
         <v>0</v>
       </c>
       <c r="H44" s="27" t="n">
-        <v>-3.77</v>
+        <v>-2.92</v>
       </c>
       <c r="I44" s="28" t="n">
-        <v>37.47</v>
+        <v>50.25</v>
       </c>
       <c r="J44" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +156%</t>
+          <t>네이버 검색 당일 +244%</t>
         </is>
       </c>
       <c r="K44" s="29" t="inlineStr">
@@ -2229,7 +2233,7 @@
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B45" s="25" t="n">
@@ -2237,7 +2241,7 @@
       </c>
       <c r="C45" s="26" t="inlineStr">
         <is>
-          <t>뷰티스킨</t>
+          <t>한컴위드</t>
         </is>
       </c>
       <c r="D45" s="25" t="n">
@@ -2253,26 +2257,26 @@
         <v>0</v>
       </c>
       <c r="H45" s="27" t="n">
-        <v>-8.66</v>
+        <v>-3.33</v>
       </c>
       <c r="I45" s="28" t="n">
-        <v>23.34</v>
+        <v>25.13</v>
       </c>
       <c r="J45" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +74% / 중요공시 1건</t>
+          <t>네이버 검색 당일 +219%</t>
         </is>
       </c>
       <c r="K45" s="29" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B46" s="25" t="n">
@@ -2280,7 +2284,7 @@
       </c>
       <c r="C46" s="26" t="inlineStr">
         <is>
-          <t>아티스트컴퍼니</t>
+          <t>진양화학</t>
         </is>
       </c>
       <c r="D46" s="25" t="n">
@@ -2296,26 +2300,26 @@
         <v>0</v>
       </c>
       <c r="H46" s="27" t="n">
-        <v>-12.57</v>
+        <v>-6.03</v>
       </c>
       <c r="I46" s="28" t="n">
-        <v>13.04</v>
+        <v>22.47</v>
       </c>
       <c r="J46" s="29" t="inlineStr">
         <is>
-          <t>중요공시 3건</t>
+          <t>네이버 검색 당일 +132%</t>
         </is>
       </c>
       <c r="K46" s="29" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B47" s="25" t="n">
@@ -2323,7 +2327,7 @@
       </c>
       <c r="C47" s="26" t="inlineStr">
         <is>
-          <t>센서뷰</t>
+          <t>티엠씨</t>
         </is>
       </c>
       <c r="D47" s="25" t="n">
@@ -2339,24 +2343,26 @@
         <v>0</v>
       </c>
       <c r="H47" s="28" t="n">
-        <v>23.98</v>
+        <v>7.8</v>
       </c>
       <c r="I47" s="28" t="n">
-        <v>45.38</v>
+        <v>37.22</v>
       </c>
       <c r="J47" s="29" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K47" s="29" t="n">
-        <v/>
+          <t>네이버 검색 당일 +126%</t>
+        </is>
+      </c>
+      <c r="K47" s="29" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B48" s="25" t="n">
@@ -2364,42 +2370,42 @@
       </c>
       <c r="C48" s="26" t="inlineStr">
         <is>
-          <t>삼성중공업</t>
+          <t>광전자</t>
         </is>
       </c>
       <c r="D48" s="25" t="n">
         <v>3</v>
       </c>
       <c r="E48" s="25" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F48" s="25" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G48" s="25" t="n">
         <v>0</v>
       </c>
       <c r="H48" s="28" t="n">
-        <v>5.9</v>
+        <v>3.53</v>
       </c>
       <c r="I48" s="28" t="n">
-        <v>0.9399999999999999</v>
+        <v>33.67</v>
       </c>
       <c r="J48" s="29" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 3일 +100%</t>
+          <t>네이버 검색 당일 +118%</t>
         </is>
       </c>
       <c r="K48" s="29" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B49" s="25" t="n">
@@ -2407,7 +2413,7 @@
       </c>
       <c r="C49" s="26" t="inlineStr">
         <is>
-          <t>대한항공</t>
+          <t>한컴라이프케어</t>
         </is>
       </c>
       <c r="D49" s="25" t="n">
@@ -2423,24 +2429,26 @@
         <v>0</v>
       </c>
       <c r="H49" s="28" t="n">
-        <v>1.03</v>
-      </c>
-      <c r="I49" s="25" t="n">
-        <v>0</v>
+        <v>4.85</v>
+      </c>
+      <c r="I49" s="28" t="n">
+        <v>20.23</v>
       </c>
       <c r="J49" s="29" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K49" s="29" t="n">
-        <v/>
+          <t>네이버 검색 당일 +116%</t>
+        </is>
+      </c>
+      <c r="K49" s="29" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B50" s="25" t="n">
@@ -2448,42 +2456,42 @@
       </c>
       <c r="C50" s="26" t="inlineStr">
         <is>
-          <t>스피어</t>
+          <t>진영</t>
         </is>
       </c>
       <c r="D50" s="25" t="n">
         <v>3</v>
       </c>
       <c r="E50" s="25" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F50" s="25" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G50" s="25" t="n">
         <v>0</v>
       </c>
       <c r="H50" s="28" t="n">
-        <v>18.43</v>
+        <v>8.460000000000001</v>
       </c>
       <c r="I50" s="28" t="n">
-        <v>17.85</v>
+        <v>11.76</v>
       </c>
       <c r="J50" s="29" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 3일 +100%</t>
+          <t>네이버 검색 당일 +57% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K50" s="29" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B51" s="25" t="n">
@@ -2491,7 +2499,7 @@
       </c>
       <c r="C51" s="26" t="inlineStr">
         <is>
-          <t>현대약품</t>
+          <t>스피어</t>
         </is>
       </c>
       <c r="D51" s="25" t="n">
@@ -2507,24 +2515,26 @@
         <v>0</v>
       </c>
       <c r="H51" s="28" t="n">
-        <v>3.45</v>
+        <v>1.45</v>
       </c>
       <c r="I51" s="28" t="n">
-        <v>7.47</v>
+        <v>21.95</v>
       </c>
       <c r="J51" s="29" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K51" s="29" t="n">
-        <v/>
+          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K51" s="29" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B52" s="25" t="n">
@@ -2532,7 +2542,7 @@
       </c>
       <c r="C52" s="26" t="inlineStr">
         <is>
-          <t>한화엔진</t>
+          <t>대한광통신</t>
         </is>
       </c>
       <c r="D52" s="25" t="n">
@@ -2548,24 +2558,26 @@
         <v>0</v>
       </c>
       <c r="H52" s="28" t="n">
-        <v>11.85</v>
+        <v>13.23</v>
       </c>
       <c r="I52" s="28" t="n">
-        <v>11.27</v>
+        <v>30.04</v>
       </c>
       <c r="J52" s="29" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K52" s="29" t="n">
-        <v/>
+          <t>네이버뉴스 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K52" s="29" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="53" ht="18" customHeight="1">
       <c r="A53" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B53" s="25" t="n">
@@ -2573,7 +2585,7 @@
       </c>
       <c r="C53" s="26" t="inlineStr">
         <is>
-          <t>하나마이크론</t>
+          <t>삼성중공업</t>
         </is>
       </c>
       <c r="D53" s="25" t="n">
@@ -2588,25 +2600,27 @@
       <c r="G53" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H53" s="28" t="n">
-        <v>6.75</v>
-      </c>
-      <c r="I53" s="28" t="n">
-        <v>5.42</v>
+      <c r="H53" s="27" t="n">
+        <v>-2.32</v>
+      </c>
+      <c r="I53" s="27" t="n">
+        <v>-1.64</v>
       </c>
       <c r="J53" s="29" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K53" s="29" t="n">
-        <v/>
+          <t>중요공시 1건 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K53" s="29" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="54" ht="18" customHeight="1">
       <c r="A54" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B54" s="25" t="n">
@@ -2614,7 +2628,7 @@
       </c>
       <c r="C54" s="26" t="inlineStr">
         <is>
-          <t>더코디</t>
+          <t>삼성전자우</t>
         </is>
       </c>
       <c r="D54" s="25" t="n">
@@ -2630,26 +2644,24 @@
         <v>0</v>
       </c>
       <c r="H54" s="28" t="n">
-        <v>5.38</v>
-      </c>
-      <c r="I54" s="27" t="n">
-        <v>-20.83</v>
+        <v>0.41</v>
+      </c>
+      <c r="I54" s="28" t="n">
+        <v>1.86</v>
       </c>
       <c r="J54" s="29" t="inlineStr">
         <is>
-          <t>중요공시 7건</t>
-        </is>
-      </c>
-      <c r="K54" s="29" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K54" s="29" t="n">
+        <v/>
       </c>
     </row>
     <row r="55" ht="18" customHeight="1">
       <c r="A55" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B55" s="25" t="n">
@@ -2657,7 +2669,7 @@
       </c>
       <c r="C55" s="26" t="inlineStr">
         <is>
-          <t>모티브링크</t>
+          <t>엔에프씨</t>
         </is>
       </c>
       <c r="D55" s="25" t="n">
@@ -2673,26 +2685,24 @@
         <v>0</v>
       </c>
       <c r="H55" s="28" t="n">
-        <v>5.93</v>
+        <v>28.91</v>
       </c>
       <c r="I55" s="28" t="n">
-        <v>6.19</v>
+        <v>16.2</v>
       </c>
       <c r="J55" s="29" t="inlineStr">
         <is>
-          <t>중요공시 3건</t>
-        </is>
-      </c>
-      <c r="K55" s="29" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K55" s="29" t="n">
+        <v/>
       </c>
     </row>
     <row r="56" ht="18" customHeight="1">
       <c r="A56" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B56" s="25" t="n">
@@ -2700,7 +2710,7 @@
       </c>
       <c r="C56" s="26" t="inlineStr">
         <is>
-          <t>한전산업</t>
+          <t>현대약품</t>
         </is>
       </c>
       <c r="D56" s="25" t="n">
@@ -2715,27 +2725,25 @@
       <c r="G56" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H56" s="28" t="n">
-        <v>2.29</v>
-      </c>
-      <c r="I56" s="27" t="n">
-        <v>-1.74</v>
+      <c r="H56" s="27" t="n">
+        <v>-4.76</v>
+      </c>
+      <c r="I56" s="28" t="n">
+        <v>1.83</v>
       </c>
       <c r="J56" s="29" t="inlineStr">
         <is>
-          <t>중요공시 3건</t>
-        </is>
-      </c>
-      <c r="K56" s="29" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K56" s="29" t="n">
+        <v/>
       </c>
     </row>
     <row r="57" ht="18" customHeight="1">
       <c r="A57" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B57" s="25" t="n">
@@ -2743,7 +2751,7 @@
       </c>
       <c r="C57" s="26" t="inlineStr">
         <is>
-          <t>넥사다이내믹스</t>
+          <t>대한전선</t>
         </is>
       </c>
       <c r="D57" s="25" t="n">
@@ -2759,26 +2767,26 @@
         <v>0</v>
       </c>
       <c r="H57" s="28" t="n">
-        <v>1.81</v>
-      </c>
-      <c r="I57" s="27" t="n">
-        <v>-5.53</v>
+        <v>10.28</v>
+      </c>
+      <c r="I57" s="28" t="n">
+        <v>7.29</v>
       </c>
       <c r="J57" s="29" t="inlineStr">
         <is>
-          <t>중요공시 3건</t>
+          <t>네이버뉴스 헤드라인 언급</t>
         </is>
       </c>
       <c r="K57" s="29" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="58" ht="18" customHeight="1">
       <c r="A58" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B58" s="25" t="n">
@@ -2786,7 +2794,7 @@
       </c>
       <c r="C58" s="26" t="inlineStr">
         <is>
-          <t>삼성E&amp;A</t>
+          <t>더코디</t>
         </is>
       </c>
       <c r="D58" s="25" t="n">
@@ -2801,15 +2809,15 @@
       <c r="G58" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H58" s="28" t="n">
-        <v>2.39</v>
-      </c>
-      <c r="I58" s="28" t="n">
-        <v>1.98</v>
+      <c r="H58" s="27" t="n">
+        <v>-29.89</v>
+      </c>
+      <c r="I58" s="27" t="n">
+        <v>-44.49</v>
       </c>
       <c r="J58" s="29" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 한국경제 헤드라인 언급</t>
+          <t>중요공시 10건</t>
         </is>
       </c>
       <c r="K58" s="29" t="inlineStr">
@@ -2821,7 +2829,7 @@
     <row r="59" ht="18" customHeight="1">
       <c r="A59" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B59" s="25" t="n">
@@ -2829,7 +2837,7 @@
       </c>
       <c r="C59" s="26" t="inlineStr">
         <is>
-          <t>전기차</t>
+          <t>파이온엑스</t>
         </is>
       </c>
       <c r="D59" s="25" t="n">
@@ -2844,27 +2852,27 @@
       <c r="G59" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H59" s="25" t="n">
-        <v/>
-      </c>
-      <c r="I59" s="25" t="n">
-        <v/>
+      <c r="H59" s="27" t="n">
+        <v>-22.35</v>
+      </c>
+      <c r="I59" s="27" t="n">
+        <v>-33.73</v>
       </c>
       <c r="J59" s="29" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급</t>
+          <t>중요공시 4건</t>
         </is>
       </c>
       <c r="K59" s="29" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="60" ht="18" customHeight="1">
       <c r="A60" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B60" s="25" t="n">
@@ -2872,7 +2880,7 @@
       </c>
       <c r="C60" s="26" t="inlineStr">
         <is>
-          <t>SG</t>
+          <t>아티스트컴퍼니</t>
         </is>
       </c>
       <c r="D60" s="25" t="n">
@@ -2887,25 +2895,27 @@
       <c r="G60" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H60" s="28" t="n">
-        <v>2.33</v>
-      </c>
-      <c r="I60" s="27" t="n">
-        <v>-10.45</v>
+      <c r="H60" s="27" t="n">
+        <v>-3.18</v>
+      </c>
+      <c r="I60" s="28" t="n">
+        <v>11.13</v>
       </c>
       <c r="J60" s="29" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K60" s="29" t="n">
-        <v/>
+          <t>중요공시 3건</t>
+        </is>
+      </c>
+      <c r="K60" s="29" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="61" ht="18" customHeight="1">
       <c r="A61" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B61" s="25" t="n">
@@ -2913,7 +2923,7 @@
       </c>
       <c r="C61" s="26" t="inlineStr">
         <is>
-          <t>카카오뱅크</t>
+          <t>한전산업</t>
         </is>
       </c>
       <c r="D61" s="25" t="n">
@@ -2928,25 +2938,27 @@
       <c r="G61" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H61" s="27" t="n">
-        <v>-0.48</v>
+      <c r="H61" s="28" t="n">
+        <v>0.31</v>
       </c>
       <c r="I61" s="27" t="n">
-        <v>-2.34</v>
+        <v>-4.05</v>
       </c>
       <c r="J61" s="29" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K61" s="29" t="n">
-        <v/>
+          <t>중요공시 3건</t>
+        </is>
+      </c>
+      <c r="K61" s="29" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="62" ht="18" customHeight="1">
       <c r="A62" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B62" s="25" t="n">
@@ -2954,40 +2966,42 @@
       </c>
       <c r="C62" s="26" t="inlineStr">
         <is>
-          <t>RFHIC</t>
+          <t>두산퓨얼셀</t>
         </is>
       </c>
       <c r="D62" s="25" t="n">
         <v>3</v>
       </c>
       <c r="E62" s="25" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F62" s="25" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G62" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H62" s="28" t="n">
-        <v>3.65</v>
+      <c r="H62" s="27" t="n">
+        <v>-1.57</v>
       </c>
       <c r="I62" s="28" t="n">
-        <v>5.06</v>
+        <v>2.87</v>
       </c>
       <c r="J62" s="29" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K62" s="29" t="n">
-        <v/>
+          <t>중요공시 2건 / 중요공시 3일 +100%</t>
+        </is>
+      </c>
+      <c r="K62" s="29" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="63" ht="18" customHeight="1">
       <c r="A63" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B63" s="25" t="n">
@@ -2995,7 +3009,7 @@
       </c>
       <c r="C63" s="26" t="inlineStr">
         <is>
-          <t>비츠로셀</t>
+          <t>한화솔루션</t>
         </is>
       </c>
       <c r="D63" s="25" t="n">
@@ -3010,19 +3024,21 @@
       <c r="G63" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H63" s="28" t="n">
-        <v>5</v>
-      </c>
-      <c r="I63" s="28" t="n">
-        <v>3.89</v>
+      <c r="H63" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="I63" s="27" t="n">
+        <v>-3.86</v>
       </c>
       <c r="J63" s="29" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K63" s="29" t="n">
-        <v/>
+          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K63" s="29" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -3118,22 +3134,22 @@
         <v>1</v>
       </c>
       <c r="C3" s="25" t="n">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="D3" s="25" t="n">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="E3" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F3" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="G3" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="H3" s="25" t="n"/>
@@ -3142,29 +3158,29 @@
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="26" t="inlineStr">
         <is>
-          <t>인공지능</t>
+          <t>바이오</t>
         </is>
       </c>
       <c r="B4" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C4" s="25" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D4" s="25" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E4" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F4" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="G4" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="H4" s="25" t="n"/>
@@ -3173,337 +3189,341 @@
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="26" t="inlineStr">
         <is>
-          <t>SK하이닉스</t>
+          <t>삼성전자</t>
         </is>
       </c>
       <c r="B5" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="25" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="D5" s="25" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="E5" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F5" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="G5" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="H5" s="28" t="n">
-        <v>0.51</v>
-      </c>
-      <c r="I5" s="27" t="n">
-        <v>-4.7</v>
+        <v>1.56</v>
+      </c>
+      <c r="I5" s="28" t="n">
+        <v>0.19</v>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="26" t="inlineStr">
         <is>
-          <t>삼성전자</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="B6" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="25" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="D6" s="25" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E6" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F6" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="G6" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="H6" s="28" t="n">
-        <v>0.99</v>
-      </c>
-      <c r="I6" s="27" t="n">
-        <v>-4.83</v>
-      </c>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="H6" s="25" t="n"/>
+      <c r="I6" s="25" t="n"/>
     </row>
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="26" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>SK하이닉스</t>
         </is>
       </c>
       <c r="B7" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="25" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D7" s="25" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="E7" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F7" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="G7" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="H7" s="25" t="n"/>
-      <c r="I7" s="25" t="n"/>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="H7" s="28" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="I7" s="28" t="n">
+        <v>2.04</v>
+      </c>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="26" t="inlineStr">
         <is>
-          <t>원전</t>
+          <t>삼성전기</t>
         </is>
       </c>
       <c r="B8" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="25" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D8" s="25" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E8" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F8" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="G8" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="H8" s="25" t="n"/>
-      <c r="I8" s="25" t="n"/>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="H8" s="28" t="n">
+        <v>2.74</v>
+      </c>
+      <c r="I8" s="27" t="n">
+        <v>-0.86</v>
+      </c>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="26" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>LG</t>
         </is>
       </c>
       <c r="B9" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="25" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D9" s="25" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E9" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F9" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="G9" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="H9" s="25" t="n"/>
-      <c r="I9" s="25" t="n"/>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="H9" s="27" t="n">
+        <v>-0.62</v>
+      </c>
+      <c r="I9" s="27" t="n">
+        <v>-0.36</v>
+      </c>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="26" t="inlineStr">
         <is>
-          <t>방산</t>
+          <t>한화시스템</t>
         </is>
       </c>
       <c r="B10" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C10" s="25" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D10" s="25" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E10" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F10" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="G10" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="H10" s="25" t="n"/>
-      <c r="I10" s="25" t="n"/>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="H10" s="28" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="I10" s="28" t="n">
+        <v>12.69</v>
+      </c>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="26" t="inlineStr">
         <is>
-          <t>KS인더스트리</t>
+          <t>게임</t>
         </is>
       </c>
       <c r="B11" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D11" s="25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E11" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F11" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="G11" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="H11" s="27" t="n">
-        <v>-3.39</v>
-      </c>
-      <c r="I11" s="28" t="n">
-        <v>39.51</v>
-      </c>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="H11" s="25" t="n"/>
+      <c r="I11" s="25" t="n"/>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="26" t="inlineStr">
         <is>
-          <t>비투엔</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="B12" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C12" s="25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D12" s="25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E12" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F12" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="G12" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="H12" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="I12" s="27" t="n">
-        <v>-8.470000000000001</v>
-      </c>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="H12" s="25" t="n"/>
+      <c r="I12" s="25" t="n"/>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>철강</t>
+          <t>미투온</t>
         </is>
       </c>
       <c r="B13" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C13" s="25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D13" s="25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E13" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F13" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="G13" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="H13" s="25" t="n"/>
-      <c r="I13" s="25" t="n"/>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="H13" s="27" t="n">
+        <v>-8.24</v>
+      </c>
+      <c r="I13" s="28" t="n">
+        <v>52.37</v>
+      </c>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>카카오</t>
+          <t>스테이블코인</t>
         </is>
       </c>
       <c r="B14" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C14" s="25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D14" s="25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E14" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F14" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="G14" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="H14" s="28" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="I14" s="27" t="n">
-        <v>-3.15</v>
-      </c>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="H14" s="25" t="n"/>
+      <c r="I14" s="25" t="n"/>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>미투온</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="B15" s="25" t="n">
@@ -3520,25 +3540,21 @@
       </c>
       <c r="F15" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="G15" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="H15" s="28" t="n">
-        <v>18.49</v>
-      </c>
-      <c r="I15" s="28" t="n">
-        <v>67.90000000000001</v>
-      </c>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="H15" s="25" t="n"/>
+      <c r="I15" s="25" t="n"/>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>대모</t>
+          <t>전기차</t>
         </is>
       </c>
       <c r="B16" s="25" t="n">
@@ -3555,25 +3571,21 @@
       </c>
       <c r="F16" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="G16" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="H16" s="28" t="n">
-        <v>5.24</v>
-      </c>
-      <c r="I16" s="28" t="n">
-        <v>0.48</v>
-      </c>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="H16" s="25" t="n"/>
+      <c r="I16" s="25" t="n"/>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>제일기획</t>
+          <t>태양광</t>
         </is>
       </c>
       <c r="B17" s="25" t="n">
@@ -3590,227 +3602,227 @@
       </c>
       <c r="F17" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="G17" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="H17" s="27" t="n">
-        <v>-0.57</v>
-      </c>
-      <c r="I17" s="27" t="n">
-        <v>-7.26</v>
-      </c>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="H17" s="25" t="n"/>
+      <c r="I17" s="25" t="n"/>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="26" t="inlineStr">
         <is>
-          <t>조선</t>
+          <t>GS건설</t>
         </is>
       </c>
       <c r="B18" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C18" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D18" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E18" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F18" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="G18" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="H18" s="25" t="n"/>
-      <c r="I18" s="25" t="n"/>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="H18" s="28" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="I18" s="27" t="n">
+        <v>-3.38</v>
+      </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>한화시스템</t>
+          <t>조선</t>
         </is>
       </c>
       <c r="B19" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C19" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D19" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E19" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F19" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="G19" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="H19" s="28" t="n">
-        <v>15.53</v>
-      </c>
-      <c r="I19" s="28" t="n">
-        <v>9.94</v>
-      </c>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="H19" s="25" t="n"/>
+      <c r="I19" s="25" t="n"/>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="26" t="inlineStr">
         <is>
-          <t>현대건설</t>
+          <t>프리티</t>
         </is>
       </c>
       <c r="B20" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C20" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D20" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E20" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F20" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="G20" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="H20" s="28" t="n">
-        <v>2.02</v>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="H20" s="27" t="n">
+        <v>-29.91</v>
       </c>
       <c r="I20" s="27" t="n">
-        <v>-3.58</v>
+        <v>-35.77</v>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="26" t="inlineStr">
         <is>
-          <t>현대모비스</t>
+          <t>현대차</t>
         </is>
       </c>
       <c r="B21" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C21" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D21" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E21" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F21" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="G21" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="H21" s="25" t="n">
-        <v>0</v>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="H21" s="28" t="n">
+        <v>0.55</v>
       </c>
       <c r="I21" s="27" t="n">
-        <v>-7.7</v>
+        <v>-4.18</v>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="26" t="inlineStr">
         <is>
-          <t>KT</t>
+          <t>LS마린솔루션</t>
         </is>
       </c>
       <c r="B22" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C22" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D22" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E22" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F22" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="G22" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="H22" s="28" t="n">
-        <v>1.13</v>
+        <v>3.7</v>
       </c>
       <c r="I22" s="28" t="n">
-        <v>3.08</v>
+        <v>4.18</v>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="26" t="inlineStr">
         <is>
-          <t>바이오</t>
+          <t>대한항공</t>
         </is>
       </c>
       <c r="B23" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C23" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D23" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E23" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F23" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="G23" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="H23" s="25" t="n"/>
-      <c r="I23" s="25" t="n"/>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="H23" s="27" t="n">
+        <v>-1.35</v>
+      </c>
+      <c r="I23" s="28" t="n">
+        <v>0.6899999999999999</v>
+      </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="26" t="inlineStr">
         <is>
-          <t>LG디스플레이</t>
+          <t>뷰티스킨</t>
         </is>
       </c>
       <c r="B24" s="25" t="n">
@@ -3827,25 +3839,25 @@
       </c>
       <c r="F24" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="G24" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="H24" s="27" t="n">
-        <v>-0.82</v>
-      </c>
-      <c r="I24" s="27" t="n">
-        <v>-5.91</v>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="H24" s="28" t="n">
+        <v>9.699999999999999</v>
+      </c>
+      <c r="I24" s="28" t="n">
+        <v>28.54</v>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="26" t="inlineStr">
         <is>
-          <t>시선AI</t>
+          <t>비츠로테크</t>
         </is>
       </c>
       <c r="B25" s="25" t="n">
@@ -3862,25 +3874,25 @@
       </c>
       <c r="F25" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="G25" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="H25" s="27" t="n">
-        <v>-2.27</v>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="H25" s="28" t="n">
+        <v>1.66</v>
       </c>
       <c r="I25" s="28" t="n">
-        <v>5.01</v>
+        <v>33.07</v>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="26" t="inlineStr">
         <is>
-          <t>에이피알</t>
+          <t>철강</t>
         </is>
       </c>
       <c r="B26" s="25" t="n">
@@ -3897,25 +3909,21 @@
       </c>
       <c r="F26" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="G26" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="H26" s="28" t="n">
-        <v>1.28</v>
-      </c>
-      <c r="I26" s="27" t="n">
-        <v>-1.66</v>
-      </c>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="H26" s="25" t="n"/>
+      <c r="I26" s="25" t="n"/>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="26" t="inlineStr">
         <is>
-          <t>이뮨온시아</t>
+          <t>한섬</t>
         </is>
       </c>
       <c r="B27" s="25" t="n">
@@ -3932,60 +3940,60 @@
       </c>
       <c r="F27" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="G27" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="H27" s="28" t="n">
-        <v>2.34</v>
+        <v>10.4</v>
       </c>
       <c r="I27" s="28" t="n">
-        <v>23.2</v>
+        <v>15.81</v>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="26" t="inlineStr">
         <is>
-          <t>한국첨단소재</t>
+          <t>광전자</t>
         </is>
       </c>
       <c r="B28" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C28" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D28" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E28" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F28" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="G28" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="H28" s="27" t="n">
-        <v>-8.470000000000001</v>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="H28" s="28" t="n">
+        <v>3.53</v>
       </c>
       <c r="I28" s="28" t="n">
-        <v>61.76</v>
+        <v>33.67</v>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="26" t="inlineStr">
         <is>
-          <t>RFHIC</t>
+          <t>대한광통신</t>
         </is>
       </c>
       <c r="B29" s="25" t="n">
@@ -4002,25 +4010,25 @@
       </c>
       <c r="F29" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="G29" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="H29" s="28" t="n">
-        <v>3.65</v>
+        <v>13.23</v>
       </c>
       <c r="I29" s="28" t="n">
-        <v>5.06</v>
+        <v>30.04</v>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="26" t="inlineStr">
         <is>
-          <t>SG</t>
+          <t>대한전선</t>
         </is>
       </c>
       <c r="B30" s="25" t="n">
@@ -4037,25 +4045,25 @@
       </c>
       <c r="F30" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="G30" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="H30" s="28" t="n">
-        <v>2.33</v>
-      </c>
-      <c r="I30" s="27" t="n">
-        <v>-10.45</v>
+        <v>10.28</v>
+      </c>
+      <c r="I30" s="28" t="n">
+        <v>7.29</v>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="26" t="inlineStr">
         <is>
-          <t>넥사다이내믹스</t>
+          <t>더코디</t>
         </is>
       </c>
       <c r="B31" s="25" t="n">
@@ -4072,25 +4080,25 @@
       </c>
       <c r="F31" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="G31" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="H31" s="28" t="n">
-        <v>1.81</v>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="H31" s="27" t="n">
+        <v>-29.89</v>
       </c>
       <c r="I31" s="27" t="n">
-        <v>-5.53</v>
+        <v>-44.49</v>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="26" t="inlineStr">
         <is>
-          <t>대한항공</t>
+          <t>두산퓨얼셀</t>
         </is>
       </c>
       <c r="B32" s="25" t="n">
@@ -4107,25 +4115,25 @@
       </c>
       <c r="F32" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="G32" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="H32" s="28" t="n">
-        <v>1.03</v>
-      </c>
-      <c r="I32" s="25" t="n">
-        <v>0</v>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="H32" s="27" t="n">
+        <v>-1.57</v>
+      </c>
+      <c r="I32" s="28" t="n">
+        <v>2.87</v>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="26" t="inlineStr">
         <is>
-          <t>더코디</t>
+          <t>빛샘전자</t>
         </is>
       </c>
       <c r="B33" s="25" t="n">
@@ -4142,25 +4150,25 @@
       </c>
       <c r="F33" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="G33" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="H33" s="28" t="n">
-        <v>5.38</v>
-      </c>
-      <c r="I33" s="27" t="n">
-        <v>-20.83</v>
+        <v>3.86</v>
+      </c>
+      <c r="I33" s="28" t="n">
+        <v>57.08</v>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="26" t="inlineStr">
         <is>
-          <t>동국산업</t>
+          <t>삼성전자우</t>
         </is>
       </c>
       <c r="B34" s="25" t="n">
@@ -4177,25 +4185,25 @@
       </c>
       <c r="F34" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="G34" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="H34" s="28" t="n">
-        <v>4.87</v>
+        <v>0.41</v>
       </c>
       <c r="I34" s="28" t="n">
-        <v>40.24</v>
+        <v>1.86</v>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="26" t="inlineStr">
         <is>
-          <t>모티브링크</t>
+          <t>삼성중공업</t>
         </is>
       </c>
       <c r="B35" s="25" t="n">
@@ -4212,25 +4220,25 @@
       </c>
       <c r="F35" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="G35" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="H35" s="28" t="n">
-        <v>5.93</v>
-      </c>
-      <c r="I35" s="28" t="n">
-        <v>6.19</v>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="H35" s="27" t="n">
+        <v>-2.32</v>
+      </c>
+      <c r="I35" s="27" t="n">
+        <v>-1.64</v>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="26" t="inlineStr">
         <is>
-          <t>뷰티스킨</t>
+          <t>스피어</t>
         </is>
       </c>
       <c r="B36" s="25" t="n">
@@ -4247,25 +4255,25 @@
       </c>
       <c r="F36" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="G36" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="H36" s="27" t="n">
-        <v>-8.66</v>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="H36" s="28" t="n">
+        <v>1.45</v>
       </c>
       <c r="I36" s="28" t="n">
-        <v>23.34</v>
+        <v>21.95</v>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="26" t="inlineStr">
         <is>
-          <t>비츠로셀</t>
+          <t>아이티센피엔에스</t>
         </is>
       </c>
       <c r="B37" s="25" t="n">
@@ -4282,25 +4290,25 @@
       </c>
       <c r="F37" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="G37" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="H37" s="28" t="n">
-        <v>5</v>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="H37" s="27" t="n">
+        <v>-3.01</v>
       </c>
       <c r="I37" s="28" t="n">
-        <v>3.89</v>
+        <v>66.41</v>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="26" t="inlineStr">
         <is>
-          <t>빛샘전자</t>
+          <t>아톤</t>
         </is>
       </c>
       <c r="B38" s="25" t="n">
@@ -4317,25 +4325,25 @@
       </c>
       <c r="F38" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="G38" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="H38" s="27" t="n">
-        <v>-3.24</v>
+        <v>-3.27</v>
       </c>
       <c r="I38" s="28" t="n">
-        <v>47.26</v>
+        <v>16.48</v>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="26" t="inlineStr">
         <is>
-          <t>삼성E&amp;A</t>
+          <t>아티스트컴퍼니</t>
         </is>
       </c>
       <c r="B39" s="25" t="n">
@@ -4352,25 +4360,25 @@
       </c>
       <c r="F39" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="G39" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="H39" s="28" t="n">
-        <v>2.39</v>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="H39" s="27" t="n">
+        <v>-3.18</v>
       </c>
       <c r="I39" s="28" t="n">
-        <v>1.98</v>
+        <v>11.13</v>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="26" t="inlineStr">
         <is>
-          <t>삼성중공업</t>
+          <t>엔에프씨</t>
         </is>
       </c>
       <c r="B40" s="25" t="n">
@@ -4387,25 +4395,25 @@
       </c>
       <c r="F40" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="G40" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="H40" s="28" t="n">
-        <v>5.9</v>
+        <v>28.91</v>
       </c>
       <c r="I40" s="28" t="n">
-        <v>0.9399999999999999</v>
+        <v>16.2</v>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="26" t="inlineStr">
         <is>
-          <t>센서뷰</t>
+          <t>진양화학</t>
         </is>
       </c>
       <c r="B41" s="25" t="n">
@@ -4422,25 +4430,25 @@
       </c>
       <c r="F41" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="G41" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="H41" s="28" t="n">
-        <v>23.98</v>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="H41" s="27" t="n">
+        <v>-6.03</v>
       </c>
       <c r="I41" s="28" t="n">
-        <v>45.38</v>
+        <v>22.47</v>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="26" t="inlineStr">
         <is>
-          <t>스피어</t>
+          <t>진영</t>
         </is>
       </c>
       <c r="B42" s="25" t="n">
@@ -4457,25 +4465,25 @@
       </c>
       <c r="F42" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="G42" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="H42" s="28" t="n">
-        <v>18.43</v>
+        <v>8.460000000000001</v>
       </c>
       <c r="I42" s="28" t="n">
-        <v>17.85</v>
+        <v>11.76</v>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="26" t="inlineStr">
         <is>
-          <t>아이티센피엔에스</t>
+          <t>큐라티스</t>
         </is>
       </c>
       <c r="B43" s="25" t="n">
@@ -4492,25 +4500,25 @@
       </c>
       <c r="F43" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="G43" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="H43" s="27" t="n">
-        <v>-4.6</v>
+        <v>-5.09</v>
       </c>
       <c r="I43" s="28" t="n">
-        <v>74.28</v>
+        <v>58.13</v>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="26" t="inlineStr">
         <is>
-          <t>아톤</t>
+          <t>티엠씨</t>
         </is>
       </c>
       <c r="B44" s="25" t="n">
@@ -4527,25 +4535,25 @@
       </c>
       <c r="F44" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="G44" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="H44" s="27" t="n">
-        <v>-3.81</v>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="H44" s="28" t="n">
+        <v>7.8</v>
       </c>
       <c r="I44" s="28" t="n">
-        <v>25.49</v>
+        <v>37.22</v>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="26" t="inlineStr">
         <is>
-          <t>아티스트컴퍼니</t>
+          <t>파이온엑스</t>
         </is>
       </c>
       <c r="B45" s="25" t="n">
@@ -4562,25 +4570,25 @@
       </c>
       <c r="F45" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="G45" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="H45" s="27" t="n">
-        <v>-12.57</v>
-      </c>
-      <c r="I45" s="28" t="n">
-        <v>13.04</v>
+        <v>-22.35</v>
+      </c>
+      <c r="I45" s="27" t="n">
+        <v>-33.73</v>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="26" t="inlineStr">
         <is>
-          <t>전기차</t>
+          <t>한국첨단소재</t>
         </is>
       </c>
       <c r="B46" s="25" t="n">
@@ -4597,21 +4605,25 @@
       </c>
       <c r="F46" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="G46" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="H46" s="25" t="n"/>
-      <c r="I46" s="25" t="n"/>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="H46" s="27" t="n">
+        <v>-2.92</v>
+      </c>
+      <c r="I46" s="28" t="n">
+        <v>50.25</v>
+      </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="26" t="inlineStr">
         <is>
-          <t>카카오뱅크</t>
+          <t>한전산업</t>
         </is>
       </c>
       <c r="B47" s="25" t="n">
@@ -4628,25 +4640,25 @@
       </c>
       <c r="F47" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="G47" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="H47" s="27" t="n">
-        <v>-0.48</v>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="H47" s="28" t="n">
+        <v>0.31</v>
       </c>
       <c r="I47" s="27" t="n">
-        <v>-2.34</v>
+        <v>-4.05</v>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="26" t="inlineStr">
         <is>
-          <t>하나마이크론</t>
+          <t>한컴라이프케어</t>
         </is>
       </c>
       <c r="B48" s="25" t="n">
@@ -4663,25 +4675,25 @@
       </c>
       <c r="F48" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="G48" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="H48" s="28" t="n">
-        <v>6.75</v>
+        <v>4.85</v>
       </c>
       <c r="I48" s="28" t="n">
-        <v>5.42</v>
+        <v>20.23</v>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="26" t="inlineStr">
         <is>
-          <t>한전산업</t>
+          <t>한컴위드</t>
         </is>
       </c>
       <c r="B49" s="25" t="n">
@@ -4698,25 +4710,25 @@
       </c>
       <c r="F49" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="G49" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="H49" s="28" t="n">
-        <v>2.29</v>
-      </c>
-      <c r="I49" s="27" t="n">
-        <v>-1.74</v>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="H49" s="27" t="n">
+        <v>-3.33</v>
+      </c>
+      <c r="I49" s="28" t="n">
+        <v>25.13</v>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="26" t="inlineStr">
         <is>
-          <t>한컴위드</t>
+          <t>한켐</t>
         </is>
       </c>
       <c r="B50" s="25" t="n">
@@ -4733,25 +4745,25 @@
       </c>
       <c r="F50" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="G50" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="H50" s="27" t="n">
-        <v>-3.77</v>
+        <v>-5.41</v>
       </c>
       <c r="I50" s="28" t="n">
-        <v>37.47</v>
+        <v>37.38</v>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="26" t="inlineStr">
         <is>
-          <t>한화엔진</t>
+          <t>한화솔루션</t>
         </is>
       </c>
       <c r="B51" s="25" t="n">
@@ -4768,19 +4780,19 @@
       </c>
       <c r="F51" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="G51" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="H51" s="28" t="n">
-        <v>11.85</v>
-      </c>
-      <c r="I51" s="28" t="n">
-        <v>11.27</v>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="H51" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="I51" s="27" t="n">
+        <v>-3.86</v>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
@@ -4803,19 +4815,19 @@
       </c>
       <c r="F52" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="G52" s="25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="H52" s="28" t="n">
-        <v>3.45</v>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="H52" s="27" t="n">
+        <v>-4.76</v>
       </c>
       <c r="I52" s="28" t="n">
-        <v>7.47</v>
+        <v>1.83</v>
       </c>
     </row>
   </sheetData>
@@ -4899,19 +4911,19 @@
         <v>1</v>
       </c>
       <c r="C3" s="36" t="n">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="D3" s="36" t="n">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="E3" s="36" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="F3" s="37" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="G3" s="37" t="inlineStr">
@@ -4930,19 +4942,19 @@
         <v>1</v>
       </c>
       <c r="C4" s="36" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="D4" s="36" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="E4" s="36" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="F4" s="37" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="G4" s="37" t="inlineStr">
@@ -4961,19 +4973,19 @@
         <v>1</v>
       </c>
       <c r="C5" s="36" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D5" s="36" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E5" s="36" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="F5" s="37" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="G5" s="37" t="inlineStr">
@@ -4985,26 +4997,26 @@
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="35" t="inlineStr">
         <is>
-          <t>방산</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="B6" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="36" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D6" s="36" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E6" s="36" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="F6" s="37" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="G6" s="37" t="inlineStr">
@@ -5016,26 +5028,26 @@
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="35" t="inlineStr">
         <is>
-          <t>원전</t>
+          <t>태양광</t>
         </is>
       </c>
       <c r="B7" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="36" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D7" s="36" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E7" s="36" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="F7" s="37" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="G7" s="37" t="inlineStr">
@@ -5047,26 +5059,26 @@
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="35" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>게임</t>
         </is>
       </c>
       <c r="B8" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="36" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D8" s="36" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="E8" s="36" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="F8" s="37" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="G8" s="37" t="inlineStr">
@@ -5085,19 +5097,19 @@
         <v>1</v>
       </c>
       <c r="C9" s="36" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D9" s="36" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E9" s="36" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="F9" s="37" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="G9" s="37" t="inlineStr">
@@ -5116,19 +5128,19 @@
         <v>1</v>
       </c>
       <c r="C10" s="36" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D10" s="36" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="E10" s="36" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="F10" s="37" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="G10" s="37" t="inlineStr">
@@ -5140,65 +5152,69 @@
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="35" t="inlineStr">
         <is>
+          <t>제약</t>
+        </is>
+      </c>
+      <c r="B11" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" s="36" t="n">
+        <v>7</v>
+      </c>
+      <c r="D11" s="36" t="n">
+        <v>7</v>
+      </c>
+      <c r="E11" s="36" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="F11" s="37" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="G11" s="37" t="inlineStr">
+        <is>
+          <t>⚡ 관심</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="35" t="inlineStr">
+        <is>
           <t>인공지능</t>
         </is>
       </c>
-      <c r="B11" s="36" t="n">
-        <v>1</v>
-      </c>
-      <c r="C11" s="36" t="n">
-        <v>17</v>
-      </c>
-      <c r="D11" s="36" t="n">
-        <v>17</v>
-      </c>
-      <c r="E11" s="36" t="inlineStr">
-        <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="F11" s="37" t="inlineStr">
-        <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="G11" s="37" t="inlineStr">
+      <c r="B12" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C12" s="36" t="n">
+        <v>19</v>
+      </c>
+      <c r="D12" s="36" t="n">
+        <v>19</v>
+      </c>
+      <c r="E12" s="36" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="F12" s="37" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="G12" s="37" t="inlineStr">
         <is>
           <t>⚡ 관심</t>
         </is>
       </c>
-    </row>
-    <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="26" t="inlineStr">
-        <is>
-          <t>이차전지</t>
-        </is>
-      </c>
-      <c r="B12" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="C12" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="D12" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" s="25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F12" s="29" t="inlineStr">
-        <is>
-          <t>감지 없음</t>
-        </is>
-      </c>
-      <c r="G12" s="29" t="inlineStr"/>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>AI반도체</t>
+          <t>이차전지</t>
         </is>
       </c>
       <c r="B13" s="25" t="n">
@@ -5225,7 +5241,7 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>수소</t>
+          <t>AI반도체</t>
         </is>
       </c>
       <c r="B14" s="25" t="n">
@@ -5252,7 +5268,7 @@
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>태양광</t>
+          <t>방산</t>
         </is>
       </c>
       <c r="B15" s="25" t="n">
@@ -5279,7 +5295,7 @@
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>게임</t>
+          <t>원전</t>
         </is>
       </c>
       <c r="B16" s="25" t="n">
@@ -5306,7 +5322,7 @@
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>엔터</t>
+          <t>수소</t>
         </is>
       </c>
       <c r="B17" s="25" t="n">
@@ -5333,7 +5349,7 @@
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="26" t="inlineStr">
         <is>
-          <t>핀테크</t>
+          <t>엔터</t>
         </is>
       </c>
       <c r="B18" s="25" t="n">
@@ -5360,7 +5376,7 @@
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>클라우드</t>
+          <t>핀테크</t>
         </is>
       </c>
       <c r="B19" s="25" t="n">
@@ -5387,7 +5403,7 @@
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="26" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>클라우드</t>
         </is>
       </c>
       <c r="B20" s="25" t="n">

</xml_diff>

<commit_message>
auto: 2026-09-20 07:22 자동 백업
</commit_message>
<xml_diff>
--- a/trend/stock_trend_history.xlsx
+++ b/trend/stock_trend_history.xlsx
@@ -694,7 +694,7 @@
     <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-09-19 06:54</t>
+          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-09-20 06:54</t>
         </is>
       </c>
     </row>
@@ -708,7 +708,7 @@
       </c>
       <c r="E3" s="3" t="n"/>
       <c r="G3" s="5" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H3" s="3" t="n"/>
       <c r="J3" s="6" t="n">
@@ -787,21 +787,21 @@
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-09-19) 상위: 반도체  점수 50.0점</t>
+          <t>⚡ 최신(2026-09-20) 상위: 반도체  점수 47.0점</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-09-19) 상위: 바이오  점수 20.0점</t>
+          <t>⚡ 최신(2026-09-20) 상위: 삼성전자  점수 17.0점</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-09-19) 상위: 삼성전자  점수 19.0점</t>
+          <t>⚡ 최신(2026-09-20) 상위: SK하이닉스  점수 15.0점</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="15" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B14" s="15" t="n">
@@ -928,10 +928,10 @@
         </is>
       </c>
       <c r="D14" s="15" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="E14" s="15" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="F14" s="15" t="n">
         <v>0</v>
@@ -947,7 +947,7 @@
       </c>
       <c r="J14" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급</t>
+          <t>네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K14" s="17" t="inlineStr">
@@ -959,7 +959,7 @@
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="15" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B15" s="15" t="n">
@@ -967,14 +967,14 @@
       </c>
       <c r="C15" s="16" t="inlineStr">
         <is>
-          <t>바이오</t>
+          <t>삼성전자</t>
         </is>
       </c>
       <c r="D15" s="15" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E15" s="15" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="F15" s="15" t="n">
         <v>0</v>
@@ -982,27 +982,25 @@
       <c r="G15" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H15" s="15" t="n">
+      <c r="H15" s="18" t="n">
+        <v>1.56</v>
+      </c>
+      <c r="I15" s="18" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="J15" s="17" t="inlineStr">
+        <is>
+          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K15" s="17" t="n">
         <v/>
-      </c>
-      <c r="I15" s="15" t="n">
-        <v/>
-      </c>
-      <c r="J15" s="17" t="inlineStr">
-        <is>
-          <t>매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급</t>
-        </is>
-      </c>
-      <c r="K15" s="17" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="15" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B16" s="15" t="n">
@@ -1010,14 +1008,14 @@
       </c>
       <c r="C16" s="16" t="inlineStr">
         <is>
-          <t>삼성전자</t>
+          <t>SK하이닉스</t>
         </is>
       </c>
       <c r="D16" s="15" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="E16" s="15" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="F16" s="15" t="n">
         <v>0</v>
@@ -1026,24 +1024,26 @@
         <v>0</v>
       </c>
       <c r="H16" s="18" t="n">
-        <v>1.56</v>
+        <v>4.7</v>
       </c>
       <c r="I16" s="18" t="n">
-        <v>0.19</v>
+        <v>2.04</v>
       </c>
       <c r="J16" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K16" s="17" t="n">
-        <v/>
+          <t>매일경제 기사 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K16" s="17" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B17" s="15" t="n">
@@ -1055,10 +1055,10 @@
         </is>
       </c>
       <c r="D17" s="15" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="E17" s="15" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="F17" s="15" t="n">
         <v>0</v>
@@ -1074,7 +1074,7 @@
       </c>
       <c r="J17" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
+          <t>매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K17" s="17" t="inlineStr">
@@ -1086,7 +1086,7 @@
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B18" s="15" t="n">
@@ -1094,14 +1094,14 @@
       </c>
       <c r="C18" s="16" t="inlineStr">
         <is>
-          <t>SK하이닉스</t>
+          <t>바이오</t>
         </is>
       </c>
       <c r="D18" s="15" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E18" s="15" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F18" s="15" t="n">
         <v>0</v>
@@ -1109,15 +1109,15 @@
       <c r="G18" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H18" s="18" t="n">
-        <v>4.7</v>
-      </c>
-      <c r="I18" s="18" t="n">
-        <v>2.04</v>
+      <c r="H18" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I18" s="15" t="n">
+        <v/>
       </c>
       <c r="J18" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+          <t>매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K18" s="17" t="inlineStr">
@@ -1129,7 +1129,7 @@
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B19" s="15" t="n">
@@ -1170,7 +1170,7 @@
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B20" s="15" t="n">
@@ -1178,14 +1178,14 @@
       </c>
       <c r="C20" s="16" t="inlineStr">
         <is>
-          <t>LG</t>
+          <t>게임</t>
         </is>
       </c>
       <c r="D20" s="15" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E20" s="15" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F20" s="15" t="n">
         <v>0</v>
@@ -1193,25 +1193,27 @@
       <c r="G20" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H20" s="19" t="n">
-        <v>-0.62</v>
-      </c>
-      <c r="I20" s="19" t="n">
-        <v>-0.36</v>
+      <c r="H20" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I20" s="15" t="n">
+        <v/>
       </c>
       <c r="J20" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K20" s="17" t="n">
-        <v/>
+          <t>네이버뉴스 기사 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K20" s="17" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="15" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B21" s="15" t="n">
@@ -1219,7 +1221,7 @@
       </c>
       <c r="C21" s="16" t="inlineStr">
         <is>
-          <t>한화시스템</t>
+          <t>현대차</t>
         </is>
       </c>
       <c r="D21" s="15" t="n">
@@ -1235,26 +1237,26 @@
         <v>0</v>
       </c>
       <c r="H21" s="18" t="n">
-        <v>0.38</v>
-      </c>
-      <c r="I21" s="18" t="n">
-        <v>12.69</v>
+        <v>0.55</v>
+      </c>
+      <c r="I21" s="19" t="n">
+        <v>-4.18</v>
       </c>
       <c r="J21" s="17" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K21" s="17" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="15" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B22" s="15" t="n">
@@ -1262,14 +1264,14 @@
       </c>
       <c r="C22" s="16" t="inlineStr">
         <is>
-          <t>미투온</t>
+          <t>LG</t>
         </is>
       </c>
       <c r="D22" s="15" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E22" s="15" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F22" s="15" t="n">
         <v>0</v>
@@ -1278,26 +1280,26 @@
         <v>0</v>
       </c>
       <c r="H22" s="19" t="n">
-        <v>-8.24</v>
-      </c>
-      <c r="I22" s="18" t="n">
-        <v>52.37</v>
+        <v>-0.62</v>
+      </c>
+      <c r="I22" s="19" t="n">
+        <v>-0.36</v>
       </c>
       <c r="J22" s="17" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +952% / 중요공시 2건 / 매일경제 헤드라인 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K22" s="17" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="15" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B23" s="15" t="n">
@@ -1328,7 +1330,7 @@
       </c>
       <c r="J23" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
+          <t>네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K23" s="17" t="inlineStr">
@@ -1340,7 +1342,7 @@
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="15" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B24" s="15" t="n">
@@ -1348,7 +1350,7 @@
       </c>
       <c r="C24" s="16" t="inlineStr">
         <is>
-          <t>스테이블코인</t>
+          <t>철강</t>
         </is>
       </c>
       <c r="D24" s="15" t="n">
@@ -1371,17 +1373,19 @@
       </c>
       <c r="J24" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K24" s="17" t="n">
-        <v/>
+          <t>매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K24" s="17" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="15" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B25" s="15" t="n">
@@ -1389,7 +1393,7 @@
       </c>
       <c r="C25" s="16" t="inlineStr">
         <is>
-          <t>게임</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="D25" s="15" t="n">
@@ -1412,60 +1416,62 @@
       </c>
       <c r="J25" s="17" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K25" s="17" t="n">
+          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K25" s="17" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="18" customHeight="1">
+      <c r="A26" s="20" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B26" s="20" t="n">
+        <v>13</v>
+      </c>
+      <c r="C26" s="21" t="inlineStr">
+        <is>
+          <t>Apple</t>
+        </is>
+      </c>
+      <c r="D26" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="E26" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="F26" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" s="20" t="n">
         <v/>
       </c>
-    </row>
-    <row r="26" ht="18" customHeight="1">
-      <c r="A26" s="15" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-      <c r="B26" s="15" t="n">
-        <v>13</v>
-      </c>
-      <c r="C26" s="16" t="inlineStr">
-        <is>
-          <t>로봇</t>
-        </is>
-      </c>
-      <c r="D26" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="E26" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="F26" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="G26" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H26" s="15" t="n">
+      <c r="I26" s="20" t="n">
         <v/>
       </c>
-      <c r="I26" s="15" t="n">
-        <v/>
-      </c>
-      <c r="J26" s="17" t="inlineStr">
-        <is>
-          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K26" s="17" t="inlineStr">
-        <is>
-          <t>네이버</t>
+      <c r="J26" s="22" t="inlineStr">
+        <is>
+          <t>Google 급상승 검색어 등장 (KR) / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K26" s="22" t="inlineStr">
+        <is>
+          <t>Google</t>
         </is>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="20" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B27" s="20" t="n">
@@ -1473,7 +1479,7 @@
       </c>
       <c r="C27" s="21" t="inlineStr">
         <is>
-          <t>전기차</t>
+          <t>원전</t>
         </is>
       </c>
       <c r="D27" s="20" t="n">
@@ -1496,7 +1502,7 @@
       </c>
       <c r="J27" s="22" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K27" s="22" t="inlineStr">
@@ -1508,7 +1514,7 @@
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="20" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B28" s="20" t="n">
@@ -1516,14 +1522,14 @@
       </c>
       <c r="C28" s="21" t="inlineStr">
         <is>
-          <t>태양광</t>
+          <t>진영</t>
         </is>
       </c>
       <c r="D28" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E28" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F28" s="20" t="n">
         <v>0</v>
@@ -1531,27 +1537,27 @@
       <c r="G28" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H28" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I28" s="20" t="n">
-        <v/>
+      <c r="H28" s="23" t="n">
+        <v>8.460000000000001</v>
+      </c>
+      <c r="I28" s="23" t="n">
+        <v>11.76</v>
       </c>
       <c r="J28" s="22" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+          <t>네이버 검색 당일 +96% / 중요공시 1건 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K28" s="22" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="20" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B29" s="20" t="n">
@@ -1594,7 +1600,7 @@
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="20" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B30" s="20" t="n">
@@ -1602,7 +1608,7 @@
       </c>
       <c r="C30" s="21" t="inlineStr">
         <is>
-          <t>프리티</t>
+          <t>더코디</t>
         </is>
       </c>
       <c r="D30" s="20" t="n">
@@ -1618,14 +1624,14 @@
         <v>0</v>
       </c>
       <c r="H30" s="24" t="n">
-        <v>-29.91</v>
+        <v>-29.89</v>
       </c>
       <c r="I30" s="24" t="n">
-        <v>-35.77</v>
+        <v>-44.49</v>
       </c>
       <c r="J30" s="22" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 3일 +200%</t>
+          <t>중요공시 10건 / 중요공시 3일 +67%</t>
         </is>
       </c>
       <c r="K30" s="22" t="inlineStr">
@@ -1637,7 +1643,7 @@
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="20" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B31" s="20" t="n">
@@ -1645,42 +1651,42 @@
       </c>
       <c r="C31" s="21" t="inlineStr">
         <is>
-          <t>조선</t>
+          <t>프리티</t>
         </is>
       </c>
       <c r="D31" s="20" t="n">
         <v>5</v>
       </c>
       <c r="E31" s="20" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F31" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G31" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H31" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I31" s="20" t="n">
-        <v/>
+      <c r="H31" s="24" t="n">
+        <v>-29.91</v>
+      </c>
+      <c r="I31" s="24" t="n">
+        <v>-35.77</v>
       </c>
       <c r="J31" s="22" t="inlineStr">
         <is>
-          <t>Google 급상승 검색어 등장 (KR)</t>
+          <t>중요공시 3건 / 중요공시 3일 +200%</t>
         </is>
       </c>
       <c r="K31" s="22" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="20" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B32" s="20" t="n">
@@ -1688,40 +1694,42 @@
       </c>
       <c r="C32" s="21" t="inlineStr">
         <is>
-          <t>현대차</t>
+          <t>한전산업</t>
         </is>
       </c>
       <c r="D32" s="20" t="n">
         <v>5</v>
       </c>
       <c r="E32" s="20" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F32" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G32" s="20" t="n">
         <v>0</v>
       </c>
       <c r="H32" s="23" t="n">
-        <v>0.55</v>
+        <v>0.31</v>
       </c>
       <c r="I32" s="24" t="n">
-        <v>-4.18</v>
+        <v>-4.05</v>
       </c>
       <c r="J32" s="22" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K32" s="22" t="n">
-        <v/>
+          <t>중요공시 3건 / 중요공시 3일 +200%</t>
+        </is>
+      </c>
+      <c r="K32" s="22" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="20" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B33" s="20" t="n">
@@ -1729,14 +1737,14 @@
       </c>
       <c r="C33" s="21" t="inlineStr">
         <is>
-          <t>뷰티스킨</t>
+          <t>한화시스템</t>
         </is>
       </c>
       <c r="D33" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E33" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F33" s="20" t="n">
         <v>0</v>
@@ -1745,26 +1753,26 @@
         <v>0</v>
       </c>
       <c r="H33" s="23" t="n">
-        <v>9.699999999999999</v>
+        <v>0.38</v>
       </c>
       <c r="I33" s="23" t="n">
-        <v>28.54</v>
+        <v>12.69</v>
       </c>
       <c r="J33" s="22" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +173% / 중요공시 1건</t>
+          <t>중요공시 1건 / 한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K33" s="22" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="20" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B34" s="20" t="n">
@@ -1772,7 +1780,7 @@
       </c>
       <c r="C34" s="21" t="inlineStr">
         <is>
-          <t>비츠로테크</t>
+          <t>미투온</t>
         </is>
       </c>
       <c r="D34" s="20" t="n">
@@ -1787,15 +1795,15 @@
       <c r="G34" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H34" s="23" t="n">
-        <v>1.66</v>
+      <c r="H34" s="24" t="n">
+        <v>-8.24</v>
       </c>
       <c r="I34" s="23" t="n">
-        <v>33.07</v>
+        <v>52.37</v>
       </c>
       <c r="J34" s="22" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +108% / 중요공시 1건</t>
+          <t>네이버 검색 당일 +1168% / 중요공시 2건</t>
         </is>
       </c>
       <c r="K34" s="22" t="inlineStr">
@@ -1807,7 +1815,7 @@
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="20" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B35" s="20" t="n">
@@ -1815,7 +1823,7 @@
       </c>
       <c r="C35" s="21" t="inlineStr">
         <is>
-          <t>대한항공</t>
+          <t>뷰티스킨</t>
         </is>
       </c>
       <c r="D35" s="20" t="n">
@@ -1830,25 +1838,27 @@
       <c r="G35" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H35" s="24" t="n">
-        <v>-1.35</v>
+      <c r="H35" s="23" t="n">
+        <v>9.699999999999999</v>
       </c>
       <c r="I35" s="23" t="n">
-        <v>0.6899999999999999</v>
+        <v>28.54</v>
       </c>
       <c r="J35" s="22" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K35" s="22" t="n">
-        <v/>
+          <t>네이버 검색 당일 +285% / 중요공시 1건</t>
+        </is>
+      </c>
+      <c r="K35" s="22" t="inlineStr">
+        <is>
+          <t>공시, 네이버</t>
+        </is>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="20" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B36" s="20" t="n">
@@ -1856,7 +1866,7 @@
       </c>
       <c r="C36" s="21" t="inlineStr">
         <is>
-          <t>한섬</t>
+          <t>비츠로테크</t>
         </is>
       </c>
       <c r="D36" s="20" t="n">
@@ -1872,14 +1882,14 @@
         <v>0</v>
       </c>
       <c r="H36" s="23" t="n">
-        <v>10.4</v>
+        <v>1.66</v>
       </c>
       <c r="I36" s="23" t="n">
-        <v>15.81</v>
+        <v>33.07</v>
       </c>
       <c r="J36" s="22" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 네이버뉴스 헤드라인 언급</t>
+          <t>네이버 검색 당일 +209% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K36" s="22" t="inlineStr">
@@ -1891,7 +1901,7 @@
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="20" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B37" s="20" t="n">
@@ -1899,7 +1909,7 @@
       </c>
       <c r="C37" s="21" t="inlineStr">
         <is>
-          <t>LS마린솔루션</t>
+          <t>엔에프씨</t>
         </is>
       </c>
       <c r="D37" s="20" t="n">
@@ -1915,26 +1925,24 @@
         <v>0</v>
       </c>
       <c r="H37" s="23" t="n">
-        <v>3.7</v>
+        <v>28.91</v>
       </c>
       <c r="I37" s="23" t="n">
-        <v>4.18</v>
+        <v>16.2</v>
       </c>
       <c r="J37" s="22" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K37" s="22" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K37" s="22" t="n">
+        <v/>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="20" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B38" s="20" t="n">
@@ -1942,7 +1950,7 @@
       </c>
       <c r="C38" s="21" t="inlineStr">
         <is>
-          <t>철강</t>
+          <t>스피어</t>
         </is>
       </c>
       <c r="D38" s="20" t="n">
@@ -1957,197 +1965,197 @@
       <c r="G38" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H38" s="20" t="n">
+      <c r="H38" s="23" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="I38" s="23" t="n">
+        <v>21.95</v>
+      </c>
+      <c r="J38" s="22" t="inlineStr">
+        <is>
+          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K38" s="22" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="18" customHeight="1">
+      <c r="A39" s="20" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B39" s="20" t="n">
+        <v>26</v>
+      </c>
+      <c r="C39" s="21" t="inlineStr">
+        <is>
+          <t>우진</t>
+        </is>
+      </c>
+      <c r="D39" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="E39" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F39" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G39" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H39" s="23" t="n">
+        <v>5.55</v>
+      </c>
+      <c r="I39" s="24" t="n">
+        <v>-0.45</v>
+      </c>
+      <c r="J39" s="22" t="inlineStr">
+        <is>
+          <t>중요공시 2건 / 네이버뉴스 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K39" s="22" t="inlineStr">
+        <is>
+          <t>공시, 네이버</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="18" customHeight="1">
+      <c r="A40" s="20" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B40" s="20" t="n">
+        <v>27</v>
+      </c>
+      <c r="C40" s="21" t="inlineStr">
+        <is>
+          <t>한전기술</t>
+        </is>
+      </c>
+      <c r="D40" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="E40" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F40" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G40" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H40" s="24" t="n">
+        <v>-2.6</v>
+      </c>
+      <c r="I40" s="24" t="n">
+        <v>-11.45</v>
+      </c>
+      <c r="J40" s="22" t="inlineStr">
+        <is>
+          <t>중요공시 1건 / 네이버뉴스 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K40" s="22" t="inlineStr">
+        <is>
+          <t>공시, 네이버</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="18" customHeight="1">
+      <c r="A41" s="20" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B41" s="20" t="n">
+        <v>28</v>
+      </c>
+      <c r="C41" s="21" t="inlineStr">
+        <is>
+          <t>LS마린솔루션</t>
+        </is>
+      </c>
+      <c r="D41" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="E41" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F41" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G41" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H41" s="23" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="I41" s="23" t="n">
+        <v>4.18</v>
+      </c>
+      <c r="J41" s="22" t="inlineStr">
+        <is>
+          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K41" s="22" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="18" customHeight="1">
+      <c r="A42" s="20" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B42" s="20" t="n">
+        <v>29</v>
+      </c>
+      <c r="C42" s="21" t="inlineStr">
+        <is>
+          <t>삼성증권</t>
+        </is>
+      </c>
+      <c r="D42" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="E42" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F42" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G42" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H42" s="24" t="n">
+        <v>-1.04</v>
+      </c>
+      <c r="I42" s="24" t="n">
+        <v>-2.06</v>
+      </c>
+      <c r="J42" s="22" t="inlineStr">
+        <is>
+          <t>매일경제 기사 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K42" s="22" t="n">
         <v/>
-      </c>
-      <c r="I38" s="20" t="n">
-        <v/>
-      </c>
-      <c r="J38" s="22" t="inlineStr">
-        <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K38" s="22" t="n">
-        <v/>
-      </c>
-    </row>
-    <row r="39" ht="18" customHeight="1">
-      <c r="A39" s="25" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-      <c r="B39" s="25" t="n">
-        <v>26</v>
-      </c>
-      <c r="C39" s="26" t="inlineStr">
-        <is>
-          <t>아이티센피엔에스</t>
-        </is>
-      </c>
-      <c r="D39" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="E39" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="F39" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="G39" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H39" s="27" t="n">
-        <v>-3.01</v>
-      </c>
-      <c r="I39" s="28" t="n">
-        <v>66.41</v>
-      </c>
-      <c r="J39" s="29" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +700%</t>
-        </is>
-      </c>
-      <c r="K39" s="29" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="18" customHeight="1">
-      <c r="A40" s="25" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-      <c r="B40" s="25" t="n">
-        <v>27</v>
-      </c>
-      <c r="C40" s="26" t="inlineStr">
-        <is>
-          <t>빛샘전자</t>
-        </is>
-      </c>
-      <c r="D40" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="E40" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="F40" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="G40" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H40" s="28" t="n">
-        <v>3.86</v>
-      </c>
-      <c r="I40" s="28" t="n">
-        <v>57.08</v>
-      </c>
-      <c r="J40" s="29" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +366%</t>
-        </is>
-      </c>
-      <c r="K40" s="29" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="18" customHeight="1">
-      <c r="A41" s="25" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-      <c r="B41" s="25" t="n">
-        <v>28</v>
-      </c>
-      <c r="C41" s="26" t="inlineStr">
-        <is>
-          <t>큐라티스</t>
-        </is>
-      </c>
-      <c r="D41" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="E41" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="F41" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="G41" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H41" s="27" t="n">
-        <v>-5.09</v>
-      </c>
-      <c r="I41" s="28" t="n">
-        <v>58.13</v>
-      </c>
-      <c r="J41" s="29" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +261%</t>
-        </is>
-      </c>
-      <c r="K41" s="29" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="18" customHeight="1">
-      <c r="A42" s="25" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-      <c r="B42" s="25" t="n">
-        <v>29</v>
-      </c>
-      <c r="C42" s="26" t="inlineStr">
-        <is>
-          <t>한켐</t>
-        </is>
-      </c>
-      <c r="D42" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="E42" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="F42" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="G42" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H42" s="27" t="n">
-        <v>-5.41</v>
-      </c>
-      <c r="I42" s="28" t="n">
-        <v>37.38</v>
-      </c>
-      <c r="J42" s="29" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +259%</t>
-        </is>
-      </c>
-      <c r="K42" s="29" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B43" s="25" t="n">
@@ -2155,7 +2163,7 @@
       </c>
       <c r="C43" s="26" t="inlineStr">
         <is>
-          <t>아톤</t>
+          <t>아이티센피엔에스</t>
         </is>
       </c>
       <c r="D43" s="25" t="n">
@@ -2171,14 +2179,14 @@
         <v>0</v>
       </c>
       <c r="H43" s="27" t="n">
-        <v>-3.27</v>
+        <v>-3.01</v>
       </c>
       <c r="I43" s="28" t="n">
-        <v>16.48</v>
+        <v>66.41</v>
       </c>
       <c r="J43" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +245%</t>
+          <t>네이버 검색 당일 +859%</t>
         </is>
       </c>
       <c r="K43" s="29" t="inlineStr">
@@ -2190,7 +2198,7 @@
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B44" s="25" t="n">
@@ -2198,7 +2206,7 @@
       </c>
       <c r="C44" s="26" t="inlineStr">
         <is>
-          <t>한국첨단소재</t>
+          <t>빛샘전자</t>
         </is>
       </c>
       <c r="D44" s="25" t="n">
@@ -2213,15 +2221,15 @@
       <c r="G44" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H44" s="27" t="n">
-        <v>-2.92</v>
+      <c r="H44" s="28" t="n">
+        <v>3.86</v>
       </c>
       <c r="I44" s="28" t="n">
-        <v>50.25</v>
+        <v>57.08</v>
       </c>
       <c r="J44" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +244%</t>
+          <t>네이버 검색 당일 +505%</t>
         </is>
       </c>
       <c r="K44" s="29" t="inlineStr">
@@ -2233,7 +2241,7 @@
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B45" s="25" t="n">
@@ -2241,7 +2249,7 @@
       </c>
       <c r="C45" s="26" t="inlineStr">
         <is>
-          <t>한컴위드</t>
+          <t>큐라티스</t>
         </is>
       </c>
       <c r="D45" s="25" t="n">
@@ -2257,14 +2265,14 @@
         <v>0</v>
       </c>
       <c r="H45" s="27" t="n">
-        <v>-3.33</v>
+        <v>-5.09</v>
       </c>
       <c r="I45" s="28" t="n">
-        <v>25.13</v>
+        <v>58.13</v>
       </c>
       <c r="J45" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +219%</t>
+          <t>네이버 검색 당일 +397%</t>
         </is>
       </c>
       <c r="K45" s="29" t="inlineStr">
@@ -2276,7 +2284,7 @@
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B46" s="25" t="n">
@@ -2284,7 +2292,7 @@
       </c>
       <c r="C46" s="26" t="inlineStr">
         <is>
-          <t>진양화학</t>
+          <t>한켐</t>
         </is>
       </c>
       <c r="D46" s="25" t="n">
@@ -2300,14 +2308,14 @@
         <v>0</v>
       </c>
       <c r="H46" s="27" t="n">
-        <v>-6.03</v>
+        <v>-5.41</v>
       </c>
       <c r="I46" s="28" t="n">
-        <v>22.47</v>
+        <v>37.38</v>
       </c>
       <c r="J46" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +132%</t>
+          <t>네이버 검색 당일 +341%</t>
         </is>
       </c>
       <c r="K46" s="29" t="inlineStr">
@@ -2319,7 +2327,7 @@
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B47" s="25" t="n">
@@ -2327,7 +2335,7 @@
       </c>
       <c r="C47" s="26" t="inlineStr">
         <is>
-          <t>티엠씨</t>
+          <t>아톤</t>
         </is>
       </c>
       <c r="D47" s="25" t="n">
@@ -2342,15 +2350,15 @@
       <c r="G47" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H47" s="28" t="n">
-        <v>7.8</v>
+      <c r="H47" s="27" t="n">
+        <v>-3.27</v>
       </c>
       <c r="I47" s="28" t="n">
-        <v>37.22</v>
+        <v>16.48</v>
       </c>
       <c r="J47" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +126%</t>
+          <t>네이버 검색 당일 +291%</t>
         </is>
       </c>
       <c r="K47" s="29" t="inlineStr">
@@ -2362,7 +2370,7 @@
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B48" s="25" t="n">
@@ -2370,7 +2378,7 @@
       </c>
       <c r="C48" s="26" t="inlineStr">
         <is>
-          <t>광전자</t>
+          <t>한국첨단소재</t>
         </is>
       </c>
       <c r="D48" s="25" t="n">
@@ -2385,15 +2393,15 @@
       <c r="G48" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H48" s="28" t="n">
-        <v>3.53</v>
+      <c r="H48" s="27" t="n">
+        <v>-2.92</v>
       </c>
       <c r="I48" s="28" t="n">
-        <v>33.67</v>
+        <v>50.25</v>
       </c>
       <c r="J48" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +118%</t>
+          <t>네이버 검색 당일 +288%</t>
         </is>
       </c>
       <c r="K48" s="29" t="inlineStr">
@@ -2405,7 +2413,7 @@
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B49" s="25" t="n">
@@ -2413,7 +2421,7 @@
       </c>
       <c r="C49" s="26" t="inlineStr">
         <is>
-          <t>한컴라이프케어</t>
+          <t>한컴위드</t>
         </is>
       </c>
       <c r="D49" s="25" t="n">
@@ -2428,15 +2436,15 @@
       <c r="G49" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H49" s="28" t="n">
-        <v>4.85</v>
+      <c r="H49" s="27" t="n">
+        <v>-3.33</v>
       </c>
       <c r="I49" s="28" t="n">
-        <v>20.23</v>
+        <v>25.13</v>
       </c>
       <c r="J49" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +116%</t>
+          <t>네이버 검색 당일 +269%</t>
         </is>
       </c>
       <c r="K49" s="29" t="inlineStr">
@@ -2448,7 +2456,7 @@
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B50" s="25" t="n">
@@ -2456,7 +2464,7 @@
       </c>
       <c r="C50" s="26" t="inlineStr">
         <is>
-          <t>진영</t>
+          <t>진양화학</t>
         </is>
       </c>
       <c r="D50" s="25" t="n">
@@ -2471,27 +2479,27 @@
       <c r="G50" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H50" s="28" t="n">
-        <v>8.460000000000001</v>
+      <c r="H50" s="27" t="n">
+        <v>-6.03</v>
       </c>
       <c r="I50" s="28" t="n">
-        <v>11.76</v>
+        <v>22.47</v>
       </c>
       <c r="J50" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +57% / 중요공시 1건</t>
+          <t>네이버 검색 당일 +214%</t>
         </is>
       </c>
       <c r="K50" s="29" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B51" s="25" t="n">
@@ -2499,7 +2507,7 @@
       </c>
       <c r="C51" s="26" t="inlineStr">
         <is>
-          <t>스피어</t>
+          <t>한컴라이프케어</t>
         </is>
       </c>
       <c r="D51" s="25" t="n">
@@ -2515,26 +2523,26 @@
         <v>0</v>
       </c>
       <c r="H51" s="28" t="n">
-        <v>1.45</v>
+        <v>4.85</v>
       </c>
       <c r="I51" s="28" t="n">
-        <v>21.95</v>
+        <v>20.23</v>
       </c>
       <c r="J51" s="29" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
+          <t>네이버 검색 당일 +201%</t>
         </is>
       </c>
       <c r="K51" s="29" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B52" s="25" t="n">
@@ -2542,7 +2550,7 @@
       </c>
       <c r="C52" s="26" t="inlineStr">
         <is>
-          <t>대한광통신</t>
+          <t>티엠씨</t>
         </is>
       </c>
       <c r="D52" s="25" t="n">
@@ -2558,14 +2566,14 @@
         <v>0</v>
       </c>
       <c r="H52" s="28" t="n">
-        <v>13.23</v>
+        <v>7.8</v>
       </c>
       <c r="I52" s="28" t="n">
-        <v>30.04</v>
+        <v>37.22</v>
       </c>
       <c r="J52" s="29" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급</t>
+          <t>네이버 검색 당일 +180%</t>
         </is>
       </c>
       <c r="K52" s="29" t="inlineStr">
@@ -2577,7 +2585,7 @@
     <row r="53" ht="18" customHeight="1">
       <c r="A53" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B53" s="25" t="n">
@@ -2585,7 +2593,7 @@
       </c>
       <c r="C53" s="26" t="inlineStr">
         <is>
-          <t>삼성중공업</t>
+          <t>센서뷰</t>
         </is>
       </c>
       <c r="D53" s="25" t="n">
@@ -2600,27 +2608,27 @@
       <c r="G53" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H53" s="27" t="n">
-        <v>-2.32</v>
-      </c>
-      <c r="I53" s="27" t="n">
-        <v>-1.64</v>
+      <c r="H53" s="28" t="n">
+        <v>7.05</v>
+      </c>
+      <c r="I53" s="28" t="n">
+        <v>56.85</v>
       </c>
       <c r="J53" s="29" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 한국경제 헤드라인 언급</t>
+          <t>네이버 검색 당일 +177%</t>
         </is>
       </c>
       <c r="K53" s="29" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="54" ht="18" customHeight="1">
       <c r="A54" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B54" s="25" t="n">
@@ -2628,7 +2636,7 @@
       </c>
       <c r="C54" s="26" t="inlineStr">
         <is>
-          <t>삼성전자우</t>
+          <t>나라스페이스테크놀로지</t>
         </is>
       </c>
       <c r="D54" s="25" t="n">
@@ -2644,24 +2652,26 @@
         <v>0</v>
       </c>
       <c r="H54" s="28" t="n">
-        <v>0.41</v>
+        <v>1.81</v>
       </c>
       <c r="I54" s="28" t="n">
-        <v>1.86</v>
+        <v>36.89</v>
       </c>
       <c r="J54" s="29" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K54" s="29" t="n">
-        <v/>
+          <t>네이버 검색 당일 +176%</t>
+        </is>
+      </c>
+      <c r="K54" s="29" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="55" ht="18" customHeight="1">
       <c r="A55" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B55" s="25" t="n">
@@ -2669,7 +2679,7 @@
       </c>
       <c r="C55" s="26" t="inlineStr">
         <is>
-          <t>엔에프씨</t>
+          <t>광전자</t>
         </is>
       </c>
       <c r="D55" s="25" t="n">
@@ -2685,24 +2695,26 @@
         <v>0</v>
       </c>
       <c r="H55" s="28" t="n">
-        <v>28.91</v>
+        <v>3.53</v>
       </c>
       <c r="I55" s="28" t="n">
-        <v>16.2</v>
+        <v>33.67</v>
       </c>
       <c r="J55" s="29" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K55" s="29" t="n">
-        <v/>
+          <t>네이버 검색 당일 +160%</t>
+        </is>
+      </c>
+      <c r="K55" s="29" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="56" ht="18" customHeight="1">
       <c r="A56" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B56" s="25" t="n">
@@ -2710,7 +2722,7 @@
       </c>
       <c r="C56" s="26" t="inlineStr">
         <is>
-          <t>현대약품</t>
+          <t>오션인더블유</t>
         </is>
       </c>
       <c r="D56" s="25" t="n">
@@ -2725,25 +2737,27 @@
       <c r="G56" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H56" s="27" t="n">
-        <v>-4.76</v>
+      <c r="H56" s="28" t="n">
+        <v>18.49</v>
       </c>
       <c r="I56" s="28" t="n">
-        <v>1.83</v>
+        <v>18.57</v>
       </c>
       <c r="J56" s="29" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K56" s="29" t="n">
-        <v/>
+          <t>네이버 검색 당일 +144%</t>
+        </is>
+      </c>
+      <c r="K56" s="29" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="57" ht="18" customHeight="1">
       <c r="A57" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B57" s="25" t="n">
@@ -2751,7 +2765,7 @@
       </c>
       <c r="C57" s="26" t="inlineStr">
         <is>
-          <t>대한전선</t>
+          <t>에이스테크</t>
         </is>
       </c>
       <c r="D57" s="25" t="n">
@@ -2767,14 +2781,14 @@
         <v>0</v>
       </c>
       <c r="H57" s="28" t="n">
-        <v>10.28</v>
+        <v>5.74</v>
       </c>
       <c r="I57" s="28" t="n">
-        <v>7.29</v>
+        <v>24.22</v>
       </c>
       <c r="J57" s="29" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급</t>
+          <t>네이버 검색 당일 +139%</t>
         </is>
       </c>
       <c r="K57" s="29" t="inlineStr">
@@ -2786,7 +2800,7 @@
     <row r="58" ht="18" customHeight="1">
       <c r="A58" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B58" s="25" t="n">
@@ -2794,7 +2808,7 @@
       </c>
       <c r="C58" s="26" t="inlineStr">
         <is>
-          <t>더코디</t>
+          <t>켄코아에어로스페이스</t>
         </is>
       </c>
       <c r="D58" s="25" t="n">
@@ -2809,27 +2823,27 @@
       <c r="G58" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H58" s="27" t="n">
-        <v>-29.89</v>
-      </c>
-      <c r="I58" s="27" t="n">
-        <v>-44.49</v>
+      <c r="H58" s="28" t="n">
+        <v>12.69</v>
+      </c>
+      <c r="I58" s="28" t="n">
+        <v>28.67</v>
       </c>
       <c r="J58" s="29" t="inlineStr">
         <is>
-          <t>중요공시 10건</t>
+          <t>네이버 검색 당일 +136%</t>
         </is>
       </c>
       <c r="K58" s="29" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="59" ht="18" customHeight="1">
       <c r="A59" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B59" s="25" t="n">
@@ -2837,7 +2851,7 @@
       </c>
       <c r="C59" s="26" t="inlineStr">
         <is>
-          <t>파이온엑스</t>
+          <t>아이씨티케이</t>
         </is>
       </c>
       <c r="D59" s="25" t="n">
@@ -2852,27 +2866,27 @@
       <c r="G59" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H59" s="27" t="n">
-        <v>-22.35</v>
-      </c>
-      <c r="I59" s="27" t="n">
-        <v>-33.73</v>
+      <c r="H59" s="28" t="n">
+        <v>3.95</v>
+      </c>
+      <c r="I59" s="28" t="n">
+        <v>29.94</v>
       </c>
       <c r="J59" s="29" t="inlineStr">
         <is>
-          <t>중요공시 4건</t>
+          <t>네이버 검색 당일 +119%</t>
         </is>
       </c>
       <c r="K59" s="29" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="60" ht="18" customHeight="1">
       <c r="A60" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B60" s="25" t="n">
@@ -2880,7 +2894,7 @@
       </c>
       <c r="C60" s="26" t="inlineStr">
         <is>
-          <t>아티스트컴퍼니</t>
+          <t>이엔셀</t>
         </is>
       </c>
       <c r="D60" s="25" t="n">
@@ -2895,27 +2909,27 @@
       <c r="G60" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H60" s="27" t="n">
-        <v>-3.18</v>
+      <c r="H60" s="28" t="n">
+        <v>30.15</v>
       </c>
       <c r="I60" s="28" t="n">
-        <v>11.13</v>
+        <v>25.6</v>
       </c>
       <c r="J60" s="29" t="inlineStr">
         <is>
-          <t>중요공시 3건</t>
+          <t>네이버 검색 당일 +114%</t>
         </is>
       </c>
       <c r="K60" s="29" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="61" ht="18" customHeight="1">
       <c r="A61" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B61" s="25" t="n">
@@ -2923,7 +2937,7 @@
       </c>
       <c r="C61" s="26" t="inlineStr">
         <is>
-          <t>한전산업</t>
+          <t>성호전자</t>
         </is>
       </c>
       <c r="D61" s="25" t="n">
@@ -2939,26 +2953,26 @@
         <v>0</v>
       </c>
       <c r="H61" s="28" t="n">
-        <v>0.31</v>
-      </c>
-      <c r="I61" s="27" t="n">
-        <v>-4.05</v>
+        <v>18.92</v>
+      </c>
+      <c r="I61" s="28" t="n">
+        <v>51.03</v>
       </c>
       <c r="J61" s="29" t="inlineStr">
         <is>
-          <t>중요공시 3건</t>
+          <t>네이버 검색 당일 +79% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K61" s="29" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="62" ht="18" customHeight="1">
       <c r="A62" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B62" s="25" t="n">
@@ -2966,30 +2980,30 @@
       </c>
       <c r="C62" s="26" t="inlineStr">
         <is>
-          <t>두산퓨얼셀</t>
+          <t>삼성중공업</t>
         </is>
       </c>
       <c r="D62" s="25" t="n">
         <v>3</v>
       </c>
       <c r="E62" s="25" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F62" s="25" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G62" s="25" t="n">
         <v>0</v>
       </c>
       <c r="H62" s="27" t="n">
-        <v>-1.57</v>
-      </c>
-      <c r="I62" s="28" t="n">
-        <v>2.87</v>
+        <v>-2.32</v>
+      </c>
+      <c r="I62" s="27" t="n">
+        <v>-1.64</v>
       </c>
       <c r="J62" s="29" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 3일 +100%</t>
+          <t>중요공시 1건 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K62" s="29" t="inlineStr">
@@ -3001,7 +3015,7 @@
     <row r="63" ht="18" customHeight="1">
       <c r="A63" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B63" s="25" t="n">
@@ -3009,7 +3023,7 @@
       </c>
       <c r="C63" s="26" t="inlineStr">
         <is>
-          <t>한화솔루션</t>
+          <t>삼성전자우</t>
         </is>
       </c>
       <c r="D63" s="25" t="n">
@@ -3024,21 +3038,19 @@
       <c r="G63" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H63" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="I63" s="27" t="n">
-        <v>-3.86</v>
+      <c r="H63" s="28" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="I63" s="28" t="n">
+        <v>1.86</v>
       </c>
       <c r="J63" s="29" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K63" s="29" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K63" s="29" t="n">
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -3134,22 +3146,22 @@
         <v>1</v>
       </c>
       <c r="C3" s="25" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="D3" s="25" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="E3" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F3" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G3" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="H3" s="25" t="n"/>
@@ -3158,95 +3170,99 @@
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="26" t="inlineStr">
         <is>
-          <t>바이오</t>
+          <t>삼성전자</t>
         </is>
       </c>
       <c r="B4" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C4" s="25" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="D4" s="25" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E4" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F4" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G4" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-      <c r="H4" s="25" t="n"/>
-      <c r="I4" s="25" t="n"/>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="H4" s="28" t="n">
+        <v>1.56</v>
+      </c>
+      <c r="I4" s="28" t="n">
+        <v>0.19</v>
+      </c>
     </row>
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="26" t="inlineStr">
         <is>
-          <t>삼성전자</t>
+          <t>SK하이닉스</t>
         </is>
       </c>
       <c r="B5" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="25" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="D5" s="25" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="E5" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F5" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G5" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="H5" s="28" t="n">
-        <v>1.56</v>
+        <v>4.7</v>
       </c>
       <c r="I5" s="28" t="n">
-        <v>0.19</v>
+        <v>2.04</v>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="26" t="inlineStr">
         <is>
-          <t>인공지능</t>
+          <t>바이오</t>
         </is>
       </c>
       <c r="B6" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="25" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="D6" s="25" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="E6" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F6" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G6" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="H6" s="25" t="n"/>
@@ -3255,37 +3271,33 @@
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="26" t="inlineStr">
         <is>
-          <t>SK하이닉스</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="B7" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="25" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D7" s="25" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E7" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F7" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G7" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-      <c r="H7" s="28" t="n">
-        <v>4.7</v>
-      </c>
-      <c r="I7" s="28" t="n">
-        <v>2.04</v>
-      </c>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="H7" s="25" t="n"/>
+      <c r="I7" s="25" t="n"/>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="26" t="inlineStr">
@@ -3307,12 +3319,12 @@
       </c>
       <c r="F8" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G8" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="H8" s="28" t="n">
@@ -3325,42 +3337,38 @@
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="26" t="inlineStr">
         <is>
-          <t>LG</t>
+          <t>게임</t>
         </is>
       </c>
       <c r="B9" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="25" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D9" s="25" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E9" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F9" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G9" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-      <c r="H9" s="27" t="n">
-        <v>-0.62</v>
-      </c>
-      <c r="I9" s="27" t="n">
-        <v>-0.36</v>
-      </c>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="H9" s="25" t="n"/>
+      <c r="I9" s="25" t="n"/>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="26" t="inlineStr">
         <is>
-          <t>한화시스템</t>
+          <t>LG</t>
         </is>
       </c>
       <c r="B10" s="25" t="n">
@@ -3377,51 +3385,55 @@
       </c>
       <c r="F10" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G10" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-      <c r="H10" s="28" t="n">
-        <v>0.38</v>
-      </c>
-      <c r="I10" s="28" t="n">
-        <v>12.69</v>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="H10" s="27" t="n">
+        <v>-0.62</v>
+      </c>
+      <c r="I10" s="27" t="n">
+        <v>-0.36</v>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="26" t="inlineStr">
         <is>
-          <t>게임</t>
+          <t>현대차</t>
         </is>
       </c>
       <c r="B11" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="25" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D11" s="25" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E11" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F11" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G11" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-      <c r="H11" s="25" t="n"/>
-      <c r="I11" s="25" t="n"/>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="H11" s="28" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="I11" s="27" t="n">
+        <v>-4.18</v>
+      </c>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="26" t="inlineStr">
@@ -3443,12 +3455,12 @@
       </c>
       <c r="F12" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G12" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="H12" s="25" t="n"/>
@@ -3457,7 +3469,7 @@
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>미투온</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="B13" s="25" t="n">
@@ -3474,25 +3486,21 @@
       </c>
       <c r="F13" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G13" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-      <c r="H13" s="27" t="n">
-        <v>-8.24</v>
-      </c>
-      <c r="I13" s="28" t="n">
-        <v>52.37</v>
-      </c>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="H13" s="25" t="n"/>
+      <c r="I13" s="25" t="n"/>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>스테이블코인</t>
+          <t>철강</t>
         </is>
       </c>
       <c r="B14" s="25" t="n">
@@ -3509,12 +3517,12 @@
       </c>
       <c r="F14" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G14" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="H14" s="25" t="n"/>
@@ -3523,29 +3531,29 @@
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>Apple</t>
         </is>
       </c>
       <c r="B15" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C15" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D15" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E15" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F15" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G15" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="H15" s="25" t="n"/>
@@ -3554,7 +3562,7 @@
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>전기차</t>
+          <t>원전</t>
         </is>
       </c>
       <c r="B16" s="25" t="n">
@@ -3571,12 +3579,12 @@
       </c>
       <c r="F16" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G16" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="H16" s="25" t="n"/>
@@ -3585,38 +3593,42 @@
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>태양광</t>
+          <t>GS건설</t>
         </is>
       </c>
       <c r="B17" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C17" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D17" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E17" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F17" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G17" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-      <c r="H17" s="25" t="n"/>
-      <c r="I17" s="25" t="n"/>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="H17" s="28" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="I17" s="27" t="n">
+        <v>-3.38</v>
+      </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="26" t="inlineStr">
         <is>
-          <t>GS건설</t>
+          <t>더코디</t>
         </is>
       </c>
       <c r="B18" s="25" t="n">
@@ -3633,25 +3645,25 @@
       </c>
       <c r="F18" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G18" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-      <c r="H18" s="28" t="n">
-        <v>1.5</v>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="H18" s="27" t="n">
+        <v>-29.89</v>
       </c>
       <c r="I18" s="27" t="n">
-        <v>-3.38</v>
+        <v>-44.49</v>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>조선</t>
+          <t>진영</t>
         </is>
       </c>
       <c r="B19" s="25" t="n">
@@ -3668,16 +3680,20 @@
       </c>
       <c r="F19" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G19" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-      <c r="H19" s="25" t="n"/>
-      <c r="I19" s="25" t="n"/>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="H19" s="28" t="n">
+        <v>8.460000000000001</v>
+      </c>
+      <c r="I19" s="28" t="n">
+        <v>11.76</v>
+      </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="26" t="inlineStr">
@@ -3699,12 +3715,12 @@
       </c>
       <c r="F20" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G20" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="H20" s="27" t="n">
@@ -3717,7 +3733,7 @@
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="26" t="inlineStr">
         <is>
-          <t>현대차</t>
+          <t>한전산업</t>
         </is>
       </c>
       <c r="B21" s="25" t="n">
@@ -3734,60 +3750,60 @@
       </c>
       <c r="F21" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G21" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="H21" s="28" t="n">
-        <v>0.55</v>
+        <v>0.31</v>
       </c>
       <c r="I21" s="27" t="n">
-        <v>-4.18</v>
+        <v>-4.05</v>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="26" t="inlineStr">
         <is>
-          <t>LS마린솔루션</t>
+          <t>한화시스템</t>
         </is>
       </c>
       <c r="B22" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C22" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D22" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E22" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F22" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G22" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="H22" s="28" t="n">
-        <v>3.7</v>
+        <v>0.38</v>
       </c>
       <c r="I22" s="28" t="n">
-        <v>4.18</v>
+        <v>12.69</v>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="26" t="inlineStr">
         <is>
-          <t>대한항공</t>
+          <t>LS마린솔루션</t>
         </is>
       </c>
       <c r="B23" s="25" t="n">
@@ -3804,25 +3820,25 @@
       </c>
       <c r="F23" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G23" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-      <c r="H23" s="27" t="n">
-        <v>-1.35</v>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="H23" s="28" t="n">
+        <v>3.7</v>
       </c>
       <c r="I23" s="28" t="n">
-        <v>0.6899999999999999</v>
+        <v>4.18</v>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="26" t="inlineStr">
         <is>
-          <t>뷰티스킨</t>
+          <t>미투온</t>
         </is>
       </c>
       <c r="B24" s="25" t="n">
@@ -3839,25 +3855,25 @@
       </c>
       <c r="F24" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G24" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-      <c r="H24" s="28" t="n">
-        <v>9.699999999999999</v>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="H24" s="27" t="n">
+        <v>-8.24</v>
       </c>
       <c r="I24" s="28" t="n">
-        <v>28.54</v>
+        <v>52.37</v>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="26" t="inlineStr">
         <is>
-          <t>비츠로테크</t>
+          <t>뷰티스킨</t>
         </is>
       </c>
       <c r="B25" s="25" t="n">
@@ -3874,25 +3890,25 @@
       </c>
       <c r="F25" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G25" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="H25" s="28" t="n">
-        <v>1.66</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="I25" s="28" t="n">
-        <v>33.07</v>
+        <v>28.54</v>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="26" t="inlineStr">
         <is>
-          <t>철강</t>
+          <t>비츠로테크</t>
         </is>
       </c>
       <c r="B26" s="25" t="n">
@@ -3909,21 +3925,25 @@
       </c>
       <c r="F26" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G26" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-      <c r="H26" s="25" t="n"/>
-      <c r="I26" s="25" t="n"/>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="H26" s="28" t="n">
+        <v>1.66</v>
+      </c>
+      <c r="I26" s="28" t="n">
+        <v>33.07</v>
+      </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="26" t="inlineStr">
         <is>
-          <t>한섬</t>
+          <t>삼성증권</t>
         </is>
       </c>
       <c r="B27" s="25" t="n">
@@ -3940,165 +3960,165 @@
       </c>
       <c r="F27" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G27" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-      <c r="H27" s="28" t="n">
-        <v>10.4</v>
-      </c>
-      <c r="I27" s="28" t="n">
-        <v>15.81</v>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="H27" s="27" t="n">
+        <v>-1.04</v>
+      </c>
+      <c r="I27" s="27" t="n">
+        <v>-2.06</v>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="26" t="inlineStr">
         <is>
-          <t>광전자</t>
+          <t>스피어</t>
         </is>
       </c>
       <c r="B28" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C28" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D28" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E28" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F28" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G28" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="H28" s="28" t="n">
-        <v>3.53</v>
+        <v>1.45</v>
       </c>
       <c r="I28" s="28" t="n">
-        <v>33.67</v>
+        <v>21.95</v>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="26" t="inlineStr">
         <is>
-          <t>대한광통신</t>
+          <t>엔에프씨</t>
         </is>
       </c>
       <c r="B29" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C29" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D29" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E29" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F29" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G29" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="H29" s="28" t="n">
-        <v>13.23</v>
+        <v>28.91</v>
       </c>
       <c r="I29" s="28" t="n">
-        <v>30.04</v>
+        <v>16.2</v>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="26" t="inlineStr">
         <is>
-          <t>대한전선</t>
+          <t>우진</t>
         </is>
       </c>
       <c r="B30" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C30" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D30" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E30" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F30" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G30" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="H30" s="28" t="n">
-        <v>10.28</v>
-      </c>
-      <c r="I30" s="28" t="n">
-        <v>7.29</v>
+        <v>5.55</v>
+      </c>
+      <c r="I30" s="27" t="n">
+        <v>-0.45</v>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="26" t="inlineStr">
         <is>
-          <t>더코디</t>
+          <t>한전기술</t>
         </is>
       </c>
       <c r="B31" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C31" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D31" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E31" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F31" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G31" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="H31" s="27" t="n">
-        <v>-29.89</v>
+        <v>-2.6</v>
       </c>
       <c r="I31" s="27" t="n">
-        <v>-44.49</v>
+        <v>-11.45</v>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="26" t="inlineStr">
         <is>
-          <t>두산퓨얼셀</t>
+          <t>광전자</t>
         </is>
       </c>
       <c r="B32" s="25" t="n">
@@ -4115,25 +4135,25 @@
       </c>
       <c r="F32" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G32" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-      <c r="H32" s="27" t="n">
-        <v>-1.57</v>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="H32" s="28" t="n">
+        <v>3.53</v>
       </c>
       <c r="I32" s="28" t="n">
-        <v>2.87</v>
+        <v>33.67</v>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="26" t="inlineStr">
         <is>
-          <t>빛샘전자</t>
+          <t>나라스페이스테크놀로지</t>
         </is>
       </c>
       <c r="B33" s="25" t="n">
@@ -4150,25 +4170,25 @@
       </c>
       <c r="F33" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G33" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="H33" s="28" t="n">
-        <v>3.86</v>
+        <v>1.81</v>
       </c>
       <c r="I33" s="28" t="n">
-        <v>57.08</v>
+        <v>36.89</v>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="26" t="inlineStr">
         <is>
-          <t>삼성전자우</t>
+          <t>빛샘전자</t>
         </is>
       </c>
       <c r="B34" s="25" t="n">
@@ -4185,25 +4205,25 @@
       </c>
       <c r="F34" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G34" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="H34" s="28" t="n">
-        <v>0.41</v>
+        <v>3.86</v>
       </c>
       <c r="I34" s="28" t="n">
-        <v>1.86</v>
+        <v>57.08</v>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="26" t="inlineStr">
         <is>
-          <t>삼성중공업</t>
+          <t>삼성전자우</t>
         </is>
       </c>
       <c r="B35" s="25" t="n">
@@ -4220,25 +4240,25 @@
       </c>
       <c r="F35" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G35" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-      <c r="H35" s="27" t="n">
-        <v>-2.32</v>
-      </c>
-      <c r="I35" s="27" t="n">
-        <v>-1.64</v>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="H35" s="28" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="I35" s="28" t="n">
+        <v>1.86</v>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="26" t="inlineStr">
         <is>
-          <t>스피어</t>
+          <t>삼성중공업</t>
         </is>
       </c>
       <c r="B36" s="25" t="n">
@@ -4255,25 +4275,25 @@
       </c>
       <c r="F36" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G36" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-      <c r="H36" s="28" t="n">
-        <v>1.45</v>
-      </c>
-      <c r="I36" s="28" t="n">
-        <v>21.95</v>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="H36" s="27" t="n">
+        <v>-2.32</v>
+      </c>
+      <c r="I36" s="27" t="n">
+        <v>-1.64</v>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="26" t="inlineStr">
         <is>
-          <t>아이티센피엔에스</t>
+          <t>성호전자</t>
         </is>
       </c>
       <c r="B37" s="25" t="n">
@@ -4290,25 +4310,25 @@
       </c>
       <c r="F37" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G37" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-      <c r="H37" s="27" t="n">
-        <v>-3.01</v>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="H37" s="28" t="n">
+        <v>18.92</v>
       </c>
       <c r="I37" s="28" t="n">
-        <v>66.41</v>
+        <v>51.03</v>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="26" t="inlineStr">
         <is>
-          <t>아톤</t>
+          <t>센서뷰</t>
         </is>
       </c>
       <c r="B38" s="25" t="n">
@@ -4325,25 +4345,25 @@
       </c>
       <c r="F38" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G38" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-      <c r="H38" s="27" t="n">
-        <v>-3.27</v>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="H38" s="28" t="n">
+        <v>7.05</v>
       </c>
       <c r="I38" s="28" t="n">
-        <v>16.48</v>
+        <v>56.85</v>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="26" t="inlineStr">
         <is>
-          <t>아티스트컴퍼니</t>
+          <t>아이씨티케이</t>
         </is>
       </c>
       <c r="B39" s="25" t="n">
@@ -4360,25 +4380,25 @@
       </c>
       <c r="F39" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G39" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-      <c r="H39" s="27" t="n">
-        <v>-3.18</v>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="H39" s="28" t="n">
+        <v>3.95</v>
       </c>
       <c r="I39" s="28" t="n">
-        <v>11.13</v>
+        <v>29.94</v>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="26" t="inlineStr">
         <is>
-          <t>엔에프씨</t>
+          <t>아이티센피엔에스</t>
         </is>
       </c>
       <c r="B40" s="25" t="n">
@@ -4395,25 +4415,25 @@
       </c>
       <c r="F40" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G40" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-      <c r="H40" s="28" t="n">
-        <v>28.91</v>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="H40" s="27" t="n">
+        <v>-3.01</v>
       </c>
       <c r="I40" s="28" t="n">
-        <v>16.2</v>
+        <v>66.41</v>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="26" t="inlineStr">
         <is>
-          <t>진양화학</t>
+          <t>아톤</t>
         </is>
       </c>
       <c r="B41" s="25" t="n">
@@ -4430,25 +4450,25 @@
       </c>
       <c r="F41" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G41" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="H41" s="27" t="n">
-        <v>-6.03</v>
+        <v>-3.27</v>
       </c>
       <c r="I41" s="28" t="n">
-        <v>22.47</v>
+        <v>16.48</v>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="26" t="inlineStr">
         <is>
-          <t>진영</t>
+          <t>에이스테크</t>
         </is>
       </c>
       <c r="B42" s="25" t="n">
@@ -4465,25 +4485,25 @@
       </c>
       <c r="F42" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G42" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="H42" s="28" t="n">
-        <v>8.460000000000001</v>
+        <v>5.74</v>
       </c>
       <c r="I42" s="28" t="n">
-        <v>11.76</v>
+        <v>24.22</v>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="26" t="inlineStr">
         <is>
-          <t>큐라티스</t>
+          <t>오션인더블유</t>
         </is>
       </c>
       <c r="B43" s="25" t="n">
@@ -4500,25 +4520,25 @@
       </c>
       <c r="F43" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G43" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-      <c r="H43" s="27" t="n">
-        <v>-5.09</v>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="H43" s="28" t="n">
+        <v>18.49</v>
       </c>
       <c r="I43" s="28" t="n">
-        <v>58.13</v>
+        <v>18.57</v>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="26" t="inlineStr">
         <is>
-          <t>티엠씨</t>
+          <t>이엔셀</t>
         </is>
       </c>
       <c r="B44" s="25" t="n">
@@ -4535,25 +4555,25 @@
       </c>
       <c r="F44" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G44" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="H44" s="28" t="n">
-        <v>7.8</v>
+        <v>30.15</v>
       </c>
       <c r="I44" s="28" t="n">
-        <v>37.22</v>
+        <v>25.6</v>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="26" t="inlineStr">
         <is>
-          <t>파이온엑스</t>
+          <t>진양화학</t>
         </is>
       </c>
       <c r="B45" s="25" t="n">
@@ -4570,25 +4590,25 @@
       </c>
       <c r="F45" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G45" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="H45" s="27" t="n">
-        <v>-22.35</v>
-      </c>
-      <c r="I45" s="27" t="n">
-        <v>-33.73</v>
+        <v>-6.03</v>
+      </c>
+      <c r="I45" s="28" t="n">
+        <v>22.47</v>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="26" t="inlineStr">
         <is>
-          <t>한국첨단소재</t>
+          <t>켄코아에어로스페이스</t>
         </is>
       </c>
       <c r="B46" s="25" t="n">
@@ -4605,25 +4625,25 @@
       </c>
       <c r="F46" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G46" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-      <c r="H46" s="27" t="n">
-        <v>-2.92</v>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="H46" s="28" t="n">
+        <v>12.69</v>
       </c>
       <c r="I46" s="28" t="n">
-        <v>50.25</v>
+        <v>28.67</v>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="26" t="inlineStr">
         <is>
-          <t>한전산업</t>
+          <t>큐라티스</t>
         </is>
       </c>
       <c r="B47" s="25" t="n">
@@ -4640,25 +4660,25 @@
       </c>
       <c r="F47" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G47" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-      <c r="H47" s="28" t="n">
-        <v>0.31</v>
-      </c>
-      <c r="I47" s="27" t="n">
-        <v>-4.05</v>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="H47" s="27" t="n">
+        <v>-5.09</v>
+      </c>
+      <c r="I47" s="28" t="n">
+        <v>58.13</v>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="26" t="inlineStr">
         <is>
-          <t>한컴라이프케어</t>
+          <t>티엠씨</t>
         </is>
       </c>
       <c r="B48" s="25" t="n">
@@ -4675,25 +4695,25 @@
       </c>
       <c r="F48" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G48" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="H48" s="28" t="n">
-        <v>4.85</v>
+        <v>7.8</v>
       </c>
       <c r="I48" s="28" t="n">
-        <v>20.23</v>
+        <v>37.22</v>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="26" t="inlineStr">
         <is>
-          <t>한컴위드</t>
+          <t>한국첨단소재</t>
         </is>
       </c>
       <c r="B49" s="25" t="n">
@@ -4710,25 +4730,25 @@
       </c>
       <c r="F49" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G49" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="H49" s="27" t="n">
-        <v>-3.33</v>
+        <v>-2.92</v>
       </c>
       <c r="I49" s="28" t="n">
-        <v>25.13</v>
+        <v>50.25</v>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="26" t="inlineStr">
         <is>
-          <t>한켐</t>
+          <t>한컴라이프케어</t>
         </is>
       </c>
       <c r="B50" s="25" t="n">
@@ -4745,25 +4765,25 @@
       </c>
       <c r="F50" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G50" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-      <c r="H50" s="27" t="n">
-        <v>-5.41</v>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="H50" s="28" t="n">
+        <v>4.85</v>
       </c>
       <c r="I50" s="28" t="n">
-        <v>37.38</v>
+        <v>20.23</v>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="26" t="inlineStr">
         <is>
-          <t>한화솔루션</t>
+          <t>한컴위드</t>
         </is>
       </c>
       <c r="B51" s="25" t="n">
@@ -4780,25 +4800,25 @@
       </c>
       <c r="F51" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G51" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-      <c r="H51" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="I51" s="27" t="n">
-        <v>-3.86</v>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="H51" s="27" t="n">
+        <v>-3.33</v>
+      </c>
+      <c r="I51" s="28" t="n">
+        <v>25.13</v>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="26" t="inlineStr">
         <is>
-          <t>현대약품</t>
+          <t>한켐</t>
         </is>
       </c>
       <c r="B52" s="25" t="n">
@@ -4815,19 +4835,19 @@
       </c>
       <c r="F52" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G52" s="25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="H52" s="27" t="n">
-        <v>-4.76</v>
+        <v>-5.41</v>
       </c>
       <c r="I52" s="28" t="n">
-        <v>1.83</v>
+        <v>37.38</v>
       </c>
     </row>
   </sheetData>
@@ -4911,19 +4931,19 @@
         <v>1</v>
       </c>
       <c r="C3" s="36" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="D3" s="36" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="E3" s="36" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="F3" s="37" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G3" s="37" t="inlineStr">
@@ -4942,19 +4962,19 @@
         <v>1</v>
       </c>
       <c r="C4" s="36" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="D4" s="36" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="E4" s="36" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="F4" s="37" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G4" s="37" t="inlineStr">
@@ -4966,7 +4986,7 @@
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="35" t="inlineStr">
         <is>
-          <t>전기차</t>
+          <t>원전</t>
         </is>
       </c>
       <c r="B5" s="36" t="n">
@@ -4980,12 +5000,12 @@
       </c>
       <c r="E5" s="36" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="F5" s="37" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G5" s="37" t="inlineStr">
@@ -5011,12 +5031,12 @@
       </c>
       <c r="E6" s="36" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="F6" s="37" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G6" s="37" t="inlineStr">
@@ -5028,26 +5048,26 @@
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="35" t="inlineStr">
         <is>
-          <t>태양광</t>
+          <t>게임</t>
         </is>
       </c>
       <c r="B7" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="36" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D7" s="36" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E7" s="36" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="F7" s="37" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G7" s="37" t="inlineStr">
@@ -5059,7 +5079,7 @@
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="35" t="inlineStr">
         <is>
-          <t>게임</t>
+          <t>철강</t>
         </is>
       </c>
       <c r="B8" s="36" t="n">
@@ -5073,12 +5093,12 @@
       </c>
       <c r="E8" s="36" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="F8" s="37" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G8" s="37" t="inlineStr">
@@ -5090,26 +5110,26 @@
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="35" t="inlineStr">
         <is>
-          <t>조선</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="B9" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="36" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D9" s="36" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E9" s="36" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="F9" s="37" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G9" s="37" t="inlineStr">
@@ -5121,26 +5141,26 @@
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="35" t="inlineStr">
         <is>
-          <t>철강</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="B10" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C10" s="36" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="D10" s="36" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="E10" s="36" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="F10" s="37" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G10" s="37" t="inlineStr">
@@ -5150,71 +5170,63 @@
       </c>
     </row>
     <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="35" t="inlineStr">
-        <is>
-          <t>제약</t>
-        </is>
-      </c>
-      <c r="B11" s="36" t="n">
-        <v>1</v>
-      </c>
-      <c r="C11" s="36" t="n">
-        <v>7</v>
-      </c>
-      <c r="D11" s="36" t="n">
-        <v>7</v>
-      </c>
-      <c r="E11" s="36" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-      <c r="F11" s="37" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-      <c r="G11" s="37" t="inlineStr">
-        <is>
-          <t>⚡ 관심</t>
-        </is>
-      </c>
+      <c r="A11" s="26" t="inlineStr">
+        <is>
+          <t>이차전지</t>
+        </is>
+      </c>
+      <c r="B11" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F11" s="29" t="inlineStr">
+        <is>
+          <t>감지 없음</t>
+        </is>
+      </c>
+      <c r="G11" s="29" t="inlineStr"/>
     </row>
     <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="35" t="inlineStr">
-        <is>
-          <t>인공지능</t>
-        </is>
-      </c>
-      <c r="B12" s="36" t="n">
-        <v>1</v>
-      </c>
-      <c r="C12" s="36" t="n">
-        <v>19</v>
-      </c>
-      <c r="D12" s="36" t="n">
-        <v>19</v>
-      </c>
-      <c r="E12" s="36" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-      <c r="F12" s="37" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-      <c r="G12" s="37" t="inlineStr">
-        <is>
-          <t>⚡ 관심</t>
-        </is>
-      </c>
+      <c r="A12" s="26" t="inlineStr">
+        <is>
+          <t>AI반도체</t>
+        </is>
+      </c>
+      <c r="B12" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F12" s="29" t="inlineStr">
+        <is>
+          <t>감지 없음</t>
+        </is>
+      </c>
+      <c r="G12" s="29" t="inlineStr"/>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>이차전지</t>
+          <t>전기차</t>
         </is>
       </c>
       <c r="B13" s="25" t="n">
@@ -5241,7 +5253,7 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>AI반도체</t>
+          <t>방산</t>
         </is>
       </c>
       <c r="B14" s="25" t="n">
@@ -5268,7 +5280,7 @@
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>방산</t>
+          <t>수소</t>
         </is>
       </c>
       <c r="B15" s="25" t="n">
@@ -5295,7 +5307,7 @@
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>원전</t>
+          <t>태양광</t>
         </is>
       </c>
       <c r="B16" s="25" t="n">
@@ -5322,7 +5334,7 @@
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>수소</t>
+          <t>엔터</t>
         </is>
       </c>
       <c r="B17" s="25" t="n">
@@ -5349,7 +5361,7 @@
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="26" t="inlineStr">
         <is>
-          <t>엔터</t>
+          <t>핀테크</t>
         </is>
       </c>
       <c r="B18" s="25" t="n">
@@ -5376,7 +5388,7 @@
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>핀테크</t>
+          <t>클라우드</t>
         </is>
       </c>
       <c r="B19" s="25" t="n">
@@ -5403,7 +5415,7 @@
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="26" t="inlineStr">
         <is>
-          <t>클라우드</t>
+          <t>조선</t>
         </is>
       </c>
       <c r="B20" s="25" t="n">

</xml_diff>

<commit_message>
auto: 2026-09-21 07:01 자동 백업
</commit_message>
<xml_diff>
--- a/trend/stock_trend_history.xlsx
+++ b/trend/stock_trend_history.xlsx
@@ -694,7 +694,7 @@
     <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-09-20 06:54</t>
+          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-09-21 06:54</t>
         </is>
       </c>
     </row>
@@ -708,7 +708,7 @@
       </c>
       <c r="E3" s="3" t="n"/>
       <c r="G3" s="5" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="H3" s="3" t="n"/>
       <c r="J3" s="6" t="n">
@@ -787,21 +787,21 @@
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-09-20) 상위: 반도체  점수 47.0점</t>
+          <t>⚡ 최신(2026-09-21) 상위: 반도체  점수 78.0점</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-09-20) 상위: 삼성전자  점수 17.0점</t>
+          <t>⚡ 최신(2026-09-21) 상위: 삼성전자  점수 34.0점</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-09-20) 상위: SK하이닉스  점수 15.0점</t>
+          <t>⚡ 최신(2026-09-21) 상위: 바이오  점수 22.0점</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="15" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B14" s="15" t="n">
@@ -928,10 +928,10 @@
         </is>
       </c>
       <c r="D14" s="15" t="n">
-        <v>47</v>
+        <v>78</v>
       </c>
       <c r="E14" s="15" t="n">
-        <v>47</v>
+        <v>78</v>
       </c>
       <c r="F14" s="15" t="n">
         <v>0</v>
@@ -947,7 +947,7 @@
       </c>
       <c r="J14" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K14" s="17" t="inlineStr">
@@ -959,7 +959,7 @@
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="15" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B15" s="15" t="n">
@@ -971,10 +971,10 @@
         </is>
       </c>
       <c r="D15" s="15" t="n">
-        <v>17</v>
+        <v>34</v>
       </c>
       <c r="E15" s="15" t="n">
-        <v>17</v>
+        <v>34</v>
       </c>
       <c r="F15" s="15" t="n">
         <v>0</v>
@@ -990,17 +990,19 @@
       </c>
       <c r="J15" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K15" s="17" t="n">
-        <v/>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K15" s="17" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="15" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B16" s="15" t="n">
@@ -1008,14 +1010,14 @@
       </c>
       <c r="C16" s="16" t="inlineStr">
         <is>
-          <t>SK하이닉스</t>
+          <t>바이오</t>
         </is>
       </c>
       <c r="D16" s="15" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="E16" s="15" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="F16" s="15" t="n">
         <v>0</v>
@@ -1023,15 +1025,15 @@
       <c r="G16" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H16" s="18" t="n">
-        <v>4.7</v>
-      </c>
-      <c r="I16" s="18" t="n">
-        <v>2.04</v>
+      <c r="H16" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I16" s="15" t="n">
+        <v/>
       </c>
       <c r="J16" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+          <t>네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K16" s="17" t="inlineStr">
@@ -1043,7 +1045,7 @@
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B17" s="15" t="n">
@@ -1055,10 +1057,10 @@
         </is>
       </c>
       <c r="D17" s="15" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E17" s="15" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F17" s="15" t="n">
         <v>0</v>
@@ -1074,7 +1076,7 @@
       </c>
       <c r="J17" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+          <t>매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K17" s="17" t="inlineStr">
@@ -1086,7 +1088,7 @@
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B18" s="15" t="n">
@@ -1094,14 +1096,14 @@
       </c>
       <c r="C18" s="16" t="inlineStr">
         <is>
-          <t>바이오</t>
+          <t>SK하이닉스</t>
         </is>
       </c>
       <c r="D18" s="15" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="E18" s="15" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F18" s="15" t="n">
         <v>0</v>
@@ -1109,15 +1111,15 @@
       <c r="G18" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H18" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I18" s="15" t="n">
-        <v/>
+      <c r="H18" s="18" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="I18" s="18" t="n">
+        <v>2.04</v>
       </c>
       <c r="J18" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 한국경제 헤드라인 언급</t>
+          <t>매일경제 기사 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급</t>
         </is>
       </c>
       <c r="K18" s="17" t="inlineStr">
@@ -1129,7 +1131,7 @@
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B19" s="15" t="n">
@@ -1137,7 +1139,7 @@
       </c>
       <c r="C19" s="16" t="inlineStr">
         <is>
-          <t>삼성전기</t>
+          <t>LG</t>
         </is>
       </c>
       <c r="D19" s="15" t="n">
@@ -1152,15 +1154,15 @@
       <c r="G19" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H19" s="18" t="n">
-        <v>2.74</v>
+      <c r="H19" s="19" t="n">
+        <v>-0.62</v>
       </c>
       <c r="I19" s="19" t="n">
-        <v>-0.86</v>
+        <v>-0.36</v>
       </c>
       <c r="J19" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K19" s="17" t="n">
@@ -1170,7 +1172,7 @@
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B20" s="15" t="n">
@@ -1178,7 +1180,7 @@
       </c>
       <c r="C20" s="16" t="inlineStr">
         <is>
-          <t>게임</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="D20" s="15" t="n">
@@ -1201,7 +1203,7 @@
       </c>
       <c r="J20" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 기사 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K20" s="17" t="inlineStr">
@@ -1213,7 +1215,7 @@
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="15" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B21" s="15" t="n">
@@ -1221,42 +1223,42 @@
       </c>
       <c r="C21" s="16" t="inlineStr">
         <is>
-          <t>현대차</t>
+          <t>GS건설</t>
         </is>
       </c>
       <c r="D21" s="15" t="n">
         <v>8</v>
       </c>
       <c r="E21" s="15" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="F21" s="15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G21" s="15" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H21" s="18" t="n">
-        <v>0.55</v>
+        <v>1.5</v>
       </c>
       <c r="I21" s="19" t="n">
-        <v>-4.18</v>
+        <v>-3.38</v>
       </c>
       <c r="J21" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>중요공시 3건 / 중요공시 3일 +50% / 중요공시 7일 +50%</t>
         </is>
       </c>
       <c r="K21" s="17" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="15" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B22" s="15" t="n">
@@ -1264,162 +1266,158 @@
       </c>
       <c r="C22" s="16" t="inlineStr">
         <is>
-          <t>LG</t>
+          <t>더코디</t>
         </is>
       </c>
       <c r="D22" s="15" t="n">
         <v>8</v>
       </c>
       <c r="E22" s="15" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="F22" s="15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G22" s="15" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H22" s="19" t="n">
-        <v>-0.62</v>
+        <v>-29.89</v>
       </c>
       <c r="I22" s="19" t="n">
-        <v>-0.36</v>
+        <v>-44.49</v>
       </c>
       <c r="J22" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>중요공시 10건 / 중요공시 3일 +100% / 중요공시 7일 +67%</t>
         </is>
       </c>
       <c r="K22" s="17" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="15" t="inlineStr">
-        <is>
-          <t>2026-09-20</t>
-        </is>
-      </c>
-      <c r="B23" s="15" t="n">
+      <c r="A23" s="20" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B23" s="20" t="n">
         <v>10</v>
       </c>
-      <c r="C23" s="16" t="inlineStr">
-        <is>
-          <t>제약</t>
-        </is>
-      </c>
-      <c r="D23" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="E23" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="F23" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="G23" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H23" s="15" t="n">
+      <c r="C23" s="21" t="inlineStr">
+        <is>
+          <t>로봇</t>
+        </is>
+      </c>
+      <c r="D23" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="E23" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="F23" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" s="20" t="n">
         <v/>
       </c>
-      <c r="I23" s="15" t="n">
+      <c r="I23" s="20" t="n">
         <v/>
       </c>
-      <c r="J23" s="17" t="inlineStr">
-        <is>
-          <t>네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
-        </is>
-      </c>
-      <c r="K23" s="17" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+      <c r="J23" s="22" t="inlineStr">
+        <is>
+          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K23" s="22" t="n">
+        <v/>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="15" t="inlineStr">
-        <is>
-          <t>2026-09-20</t>
-        </is>
-      </c>
-      <c r="B24" s="15" t="n">
+      <c r="A24" s="20" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B24" s="20" t="n">
         <v>11</v>
       </c>
-      <c r="C24" s="16" t="inlineStr">
-        <is>
-          <t>철강</t>
-        </is>
-      </c>
-      <c r="D24" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="E24" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="F24" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="G24" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H24" s="15" t="n">
+      <c r="C24" s="21" t="inlineStr">
+        <is>
+          <t>삼성전기</t>
+        </is>
+      </c>
+      <c r="D24" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="E24" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="F24" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" s="23" t="n">
+        <v>2.74</v>
+      </c>
+      <c r="I24" s="24" t="n">
+        <v>-0.86</v>
+      </c>
+      <c r="J24" s="22" t="inlineStr">
+        <is>
+          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K24" s="22" t="n">
         <v/>
       </c>
-      <c r="I24" s="15" t="n">
-        <v/>
-      </c>
-      <c r="J24" s="17" t="inlineStr">
-        <is>
-          <t>매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K24" s="17" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
-      </c>
     </row>
     <row r="25" ht="18" customHeight="1">
-      <c r="A25" s="15" t="inlineStr">
-        <is>
-          <t>2026-09-20</t>
-        </is>
-      </c>
-      <c r="B25" s="15" t="n">
+      <c r="A25" s="20" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B25" s="20" t="n">
         <v>12</v>
       </c>
-      <c r="C25" s="16" t="inlineStr">
-        <is>
-          <t>로봇</t>
-        </is>
-      </c>
-      <c r="D25" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="E25" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="F25" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="G25" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H25" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I25" s="15" t="n">
-        <v/>
-      </c>
-      <c r="J25" s="17" t="inlineStr">
-        <is>
-          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K25" s="17" t="inlineStr">
+      <c r="C25" s="21" t="inlineStr">
+        <is>
+          <t>SFA반도체</t>
+        </is>
+      </c>
+      <c r="D25" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="E25" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="F25" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" s="23" t="n">
+        <v>3.21</v>
+      </c>
+      <c r="I25" s="23" t="n">
+        <v>27.7</v>
+      </c>
+      <c r="J25" s="22" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +86% / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K25" s="22" t="inlineStr">
         <is>
           <t>네이버</t>
         </is>
@@ -1428,7 +1426,7 @@
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="20" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B26" s="20" t="n">
@@ -1436,14 +1434,14 @@
       </c>
       <c r="C26" s="21" t="inlineStr">
         <is>
-          <t>Apple</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="D26" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E26" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F26" s="20" t="n">
         <v>0</v>
@@ -1459,7 +1457,7 @@
       </c>
       <c r="J26" s="22" t="inlineStr">
         <is>
-          <t>Google 급상승 검색어 등장 (KR) / 매일경제 기사 언급</t>
+          <t>Google 급상승 검색어 등장 (KR)</t>
         </is>
       </c>
       <c r="K26" s="22" t="inlineStr">
@@ -1471,7 +1469,7 @@
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="20" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B27" s="20" t="n">
@@ -1479,14 +1477,14 @@
       </c>
       <c r="C27" s="21" t="inlineStr">
         <is>
-          <t>원전</t>
+          <t>GS</t>
         </is>
       </c>
       <c r="D27" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E27" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F27" s="20" t="n">
         <v>0</v>
@@ -1494,27 +1492,27 @@
       <c r="G27" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H27" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I27" s="20" t="n">
-        <v/>
+      <c r="H27" s="24" t="n">
+        <v>-0.18</v>
+      </c>
+      <c r="I27" s="24" t="n">
+        <v>-4.2</v>
       </c>
       <c r="J27" s="22" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+          <t>Google 급상승 검색어 등장 (US)</t>
         </is>
       </c>
       <c r="K27" s="22" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>Google</t>
         </is>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="20" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B28" s="20" t="n">
@@ -1522,7 +1520,7 @@
       </c>
       <c r="C28" s="21" t="inlineStr">
         <is>
-          <t>진영</t>
+          <t>게임</t>
         </is>
       </c>
       <c r="D28" s="20" t="n">
@@ -1537,27 +1535,25 @@
       <c r="G28" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H28" s="23" t="n">
-        <v>8.460000000000001</v>
-      </c>
-      <c r="I28" s="23" t="n">
-        <v>11.76</v>
+      <c r="H28" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I28" s="20" t="n">
+        <v/>
       </c>
       <c r="J28" s="22" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +96% / 중요공시 1건 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K28" s="22" t="inlineStr">
-        <is>
-          <t>공시, 네이버</t>
-        </is>
+          <t>한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K28" s="22" t="n">
+        <v/>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="20" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B29" s="20" t="n">
@@ -1565,42 +1561,40 @@
       </c>
       <c r="C29" s="21" t="inlineStr">
         <is>
-          <t>GS건설</t>
+          <t>현대차</t>
         </is>
       </c>
       <c r="D29" s="20" t="n">
         <v>5</v>
       </c>
       <c r="E29" s="20" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F29" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G29" s="20" t="n">
         <v>0</v>
       </c>
       <c r="H29" s="23" t="n">
-        <v>1.5</v>
+        <v>0.55</v>
       </c>
       <c r="I29" s="24" t="n">
-        <v>-3.38</v>
+        <v>-4.18</v>
       </c>
       <c r="J29" s="22" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 3일 +50%</t>
-        </is>
-      </c>
-      <c r="K29" s="22" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K29" s="22" t="n">
+        <v/>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="20" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B30" s="20" t="n">
@@ -1608,42 +1602,42 @@
       </c>
       <c r="C30" s="21" t="inlineStr">
         <is>
-          <t>더코디</t>
+          <t>미투온</t>
         </is>
       </c>
       <c r="D30" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E30" s="20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F30" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G30" s="20" t="n">
         <v>0</v>
       </c>
       <c r="H30" s="24" t="n">
-        <v>-29.89</v>
-      </c>
-      <c r="I30" s="24" t="n">
-        <v>-44.49</v>
+        <v>-8.24</v>
+      </c>
+      <c r="I30" s="23" t="n">
+        <v>52.37</v>
       </c>
       <c r="J30" s="22" t="inlineStr">
         <is>
-          <t>중요공시 10건 / 중요공시 3일 +67%</t>
+          <t>네이버 검색 당일 +1205% / 중요공시 2건</t>
         </is>
       </c>
       <c r="K30" s="22" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="20" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B31" s="20" t="n">
@@ -1651,42 +1645,42 @@
       </c>
       <c r="C31" s="21" t="inlineStr">
         <is>
-          <t>프리티</t>
+          <t>뷰티스킨</t>
         </is>
       </c>
       <c r="D31" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E31" s="20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F31" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G31" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H31" s="24" t="n">
-        <v>-29.91</v>
-      </c>
-      <c r="I31" s="24" t="n">
-        <v>-35.77</v>
+      <c r="H31" s="23" t="n">
+        <v>9.699999999999999</v>
+      </c>
+      <c r="I31" s="23" t="n">
+        <v>28.54</v>
       </c>
       <c r="J31" s="22" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 3일 +200%</t>
+          <t>네이버 검색 당일 +303% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K31" s="22" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="20" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B32" s="20" t="n">
@@ -1694,42 +1688,42 @@
       </c>
       <c r="C32" s="21" t="inlineStr">
         <is>
-          <t>한전산업</t>
+          <t>비츠로테크</t>
         </is>
       </c>
       <c r="D32" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E32" s="20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F32" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G32" s="20" t="n">
         <v>0</v>
       </c>
       <c r="H32" s="23" t="n">
-        <v>0.31</v>
-      </c>
-      <c r="I32" s="24" t="n">
-        <v>-4.05</v>
+        <v>1.66</v>
+      </c>
+      <c r="I32" s="23" t="n">
+        <v>33.07</v>
       </c>
       <c r="J32" s="22" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 3일 +200%</t>
+          <t>네이버 검색 당일 +228% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K32" s="22" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="20" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B33" s="20" t="n">
@@ -1737,14 +1731,14 @@
       </c>
       <c r="C33" s="21" t="inlineStr">
         <is>
-          <t>한화시스템</t>
+          <t>진영</t>
         </is>
       </c>
       <c r="D33" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E33" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F33" s="20" t="n">
         <v>0</v>
@@ -1753,26 +1747,26 @@
         <v>0</v>
       </c>
       <c r="H33" s="23" t="n">
-        <v>0.38</v>
+        <v>8.460000000000001</v>
       </c>
       <c r="I33" s="23" t="n">
-        <v>12.69</v>
+        <v>11.76</v>
       </c>
       <c r="J33" s="22" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
+          <t>네이버 검색 당일 +144% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K33" s="22" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="20" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B34" s="20" t="n">
@@ -1780,42 +1774,42 @@
       </c>
       <c r="C34" s="21" t="inlineStr">
         <is>
-          <t>미투온</t>
+          <t>금호건설</t>
         </is>
       </c>
       <c r="D34" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E34" s="20" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F34" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G34" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H34" s="24" t="n">
-        <v>-8.24</v>
-      </c>
-      <c r="I34" s="23" t="n">
-        <v>52.37</v>
+        <v>3</v>
+      </c>
+      <c r="H34" s="23" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="I34" s="24" t="n">
+        <v>-8.359999999999999</v>
       </c>
       <c r="J34" s="22" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +1168% / 중요공시 2건</t>
+          <t>중요공시 2건 / 중요공시 7일 +100%</t>
         </is>
       </c>
       <c r="K34" s="22" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="20" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B35" s="20" t="n">
@@ -1823,42 +1817,42 @@
       </c>
       <c r="C35" s="21" t="inlineStr">
         <is>
-          <t>뷰티스킨</t>
+          <t>현대건설</t>
         </is>
       </c>
       <c r="D35" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E35" s="20" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F35" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G35" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H35" s="23" t="n">
-        <v>9.699999999999999</v>
-      </c>
-      <c r="I35" s="23" t="n">
-        <v>28.54</v>
+        <v>3</v>
+      </c>
+      <c r="H35" s="24" t="n">
+        <v>-0.71</v>
+      </c>
+      <c r="I35" s="24" t="n">
+        <v>-6.89</v>
       </c>
       <c r="J35" s="22" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +285% / 중요공시 1건</t>
+          <t>중요공시 2건 / 중요공시 7일 +100%</t>
         </is>
       </c>
       <c r="K35" s="22" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="20" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B36" s="20" t="n">
@@ -1866,7 +1860,7 @@
       </c>
       <c r="C36" s="21" t="inlineStr">
         <is>
-          <t>비츠로테크</t>
+          <t>제주항공</t>
         </is>
       </c>
       <c r="D36" s="20" t="n">
@@ -1881,27 +1875,27 @@
       <c r="G36" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H36" s="23" t="n">
-        <v>1.66</v>
-      </c>
-      <c r="I36" s="23" t="n">
-        <v>33.07</v>
+      <c r="H36" s="24" t="n">
+        <v>-5.07</v>
+      </c>
+      <c r="I36" s="24" t="n">
+        <v>-7.07</v>
       </c>
       <c r="J36" s="22" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +209% / 중요공시 1건</t>
+          <t>중요공시 2건 / 매일경제 기사 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K36" s="22" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="20" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B37" s="20" t="n">
@@ -1909,7 +1903,7 @@
       </c>
       <c r="C37" s="21" t="inlineStr">
         <is>
-          <t>엔에프씨</t>
+          <t>LS마린솔루션</t>
         </is>
       </c>
       <c r="D37" s="20" t="n">
@@ -1925,24 +1919,26 @@
         <v>0</v>
       </c>
       <c r="H37" s="23" t="n">
-        <v>28.91</v>
+        <v>3.7</v>
       </c>
       <c r="I37" s="23" t="n">
-        <v>16.2</v>
+        <v>4.18</v>
       </c>
       <c r="J37" s="22" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K37" s="22" t="n">
-        <v/>
+          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K37" s="22" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="20" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B38" s="20" t="n">
@@ -1950,7 +1946,7 @@
       </c>
       <c r="C38" s="21" t="inlineStr">
         <is>
-          <t>스피어</t>
+          <t>DB</t>
         </is>
       </c>
       <c r="D38" s="20" t="n">
@@ -1966,196 +1962,198 @@
         <v>0</v>
       </c>
       <c r="H38" s="23" t="n">
-        <v>1.45</v>
-      </c>
-      <c r="I38" s="23" t="n">
-        <v>21.95</v>
+        <v>0.37</v>
+      </c>
+      <c r="I38" s="24" t="n">
+        <v>-1.21</v>
       </c>
       <c r="J38" s="22" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
+          <t>매일경제 헤드라인 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K38" s="22" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
-      <c r="A39" s="20" t="inlineStr">
-        <is>
-          <t>2026-09-20</t>
-        </is>
-      </c>
-      <c r="B39" s="20" t="n">
+      <c r="A39" s="25" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B39" s="25" t="n">
         <v>26</v>
       </c>
-      <c r="C39" s="21" t="inlineStr">
-        <is>
-          <t>우진</t>
-        </is>
-      </c>
-      <c r="D39" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E39" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F39" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G39" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H39" s="23" t="n">
-        <v>5.55</v>
-      </c>
-      <c r="I39" s="24" t="n">
-        <v>-0.45</v>
-      </c>
-      <c r="J39" s="22" t="inlineStr">
-        <is>
-          <t>중요공시 2건 / 네이버뉴스 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K39" s="22" t="inlineStr">
-        <is>
-          <t>공시, 네이버</t>
+      <c r="C39" s="26" t="inlineStr">
+        <is>
+          <t>아이티센피엔에스</t>
+        </is>
+      </c>
+      <c r="D39" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E39" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F39" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G39" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H39" s="27" t="n">
+        <v>-3.01</v>
+      </c>
+      <c r="I39" s="28" t="n">
+        <v>66.41</v>
+      </c>
+      <c r="J39" s="29" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +884%</t>
+        </is>
+      </c>
+      <c r="K39" s="29" t="inlineStr">
+        <is>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
-      <c r="A40" s="20" t="inlineStr">
-        <is>
-          <t>2026-09-20</t>
-        </is>
-      </c>
-      <c r="B40" s="20" t="n">
+      <c r="A40" s="25" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B40" s="25" t="n">
         <v>27</v>
       </c>
-      <c r="C40" s="21" t="inlineStr">
-        <is>
-          <t>한전기술</t>
-        </is>
-      </c>
-      <c r="D40" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E40" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F40" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G40" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H40" s="24" t="n">
-        <v>-2.6</v>
-      </c>
-      <c r="I40" s="24" t="n">
-        <v>-11.45</v>
-      </c>
-      <c r="J40" s="22" t="inlineStr">
-        <is>
-          <t>중요공시 1건 / 네이버뉴스 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K40" s="22" t="inlineStr">
-        <is>
-          <t>공시, 네이버</t>
+      <c r="C40" s="26" t="inlineStr">
+        <is>
+          <t>빛샘전자</t>
+        </is>
+      </c>
+      <c r="D40" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E40" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F40" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G40" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H40" s="28" t="n">
+        <v>3.86</v>
+      </c>
+      <c r="I40" s="28" t="n">
+        <v>57.08</v>
+      </c>
+      <c r="J40" s="29" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +531%</t>
+        </is>
+      </c>
+      <c r="K40" s="29" t="inlineStr">
+        <is>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
-      <c r="A41" s="20" t="inlineStr">
-        <is>
-          <t>2026-09-20</t>
-        </is>
-      </c>
-      <c r="B41" s="20" t="n">
+      <c r="A41" s="25" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B41" s="25" t="n">
         <v>28</v>
       </c>
-      <c r="C41" s="21" t="inlineStr">
-        <is>
-          <t>LS마린솔루션</t>
-        </is>
-      </c>
-      <c r="D41" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E41" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F41" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G41" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H41" s="23" t="n">
-        <v>3.7</v>
-      </c>
-      <c r="I41" s="23" t="n">
-        <v>4.18</v>
-      </c>
-      <c r="J41" s="22" t="inlineStr">
-        <is>
-          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K41" s="22" t="inlineStr">
-        <is>
-          <t>공시</t>
+      <c r="C41" s="26" t="inlineStr">
+        <is>
+          <t>큐라티스</t>
+        </is>
+      </c>
+      <c r="D41" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E41" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F41" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G41" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H41" s="27" t="n">
+        <v>-5.09</v>
+      </c>
+      <c r="I41" s="28" t="n">
+        <v>58.13</v>
+      </c>
+      <c r="J41" s="29" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +414%</t>
+        </is>
+      </c>
+      <c r="K41" s="29" t="inlineStr">
+        <is>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
-      <c r="A42" s="20" t="inlineStr">
-        <is>
-          <t>2026-09-20</t>
-        </is>
-      </c>
-      <c r="B42" s="20" t="n">
+      <c r="A42" s="25" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B42" s="25" t="n">
         <v>29</v>
       </c>
-      <c r="C42" s="21" t="inlineStr">
-        <is>
-          <t>삼성증권</t>
-        </is>
-      </c>
-      <c r="D42" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E42" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F42" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G42" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H42" s="24" t="n">
-        <v>-1.04</v>
-      </c>
-      <c r="I42" s="24" t="n">
-        <v>-2.06</v>
-      </c>
-      <c r="J42" s="22" t="inlineStr">
-        <is>
-          <t>매일경제 기사 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K42" s="22" t="n">
-        <v/>
+      <c r="C42" s="26" t="inlineStr">
+        <is>
+          <t>한켐</t>
+        </is>
+      </c>
+      <c r="D42" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E42" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F42" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G42" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H42" s="27" t="n">
+        <v>-5.41</v>
+      </c>
+      <c r="I42" s="28" t="n">
+        <v>37.38</v>
+      </c>
+      <c r="J42" s="29" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +355%</t>
+        </is>
+      </c>
+      <c r="K42" s="29" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B43" s="25" t="n">
@@ -2163,7 +2161,7 @@
       </c>
       <c r="C43" s="26" t="inlineStr">
         <is>
-          <t>아이티센피엔에스</t>
+          <t>아톤</t>
         </is>
       </c>
       <c r="D43" s="25" t="n">
@@ -2179,14 +2177,14 @@
         <v>0</v>
       </c>
       <c r="H43" s="27" t="n">
-        <v>-3.01</v>
+        <v>-3.27</v>
       </c>
       <c r="I43" s="28" t="n">
-        <v>66.41</v>
+        <v>16.48</v>
       </c>
       <c r="J43" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +859%</t>
+          <t>네이버 검색 당일 +302%</t>
         </is>
       </c>
       <c r="K43" s="29" t="inlineStr">
@@ -2198,7 +2196,7 @@
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B44" s="25" t="n">
@@ -2206,7 +2204,7 @@
       </c>
       <c r="C44" s="26" t="inlineStr">
         <is>
-          <t>빛샘전자</t>
+          <t>한국첨단소재</t>
         </is>
       </c>
       <c r="D44" s="25" t="n">
@@ -2221,15 +2219,15 @@
       <c r="G44" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H44" s="28" t="n">
-        <v>3.86</v>
+      <c r="H44" s="27" t="n">
+        <v>-2.92</v>
       </c>
       <c r="I44" s="28" t="n">
-        <v>57.08</v>
+        <v>50.25</v>
       </c>
       <c r="J44" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +505%</t>
+          <t>네이버 검색 당일 +296%</t>
         </is>
       </c>
       <c r="K44" s="29" t="inlineStr">
@@ -2241,7 +2239,7 @@
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B45" s="25" t="n">
@@ -2249,7 +2247,7 @@
       </c>
       <c r="C45" s="26" t="inlineStr">
         <is>
-          <t>큐라티스</t>
+          <t>한컴위드</t>
         </is>
       </c>
       <c r="D45" s="25" t="n">
@@ -2265,14 +2263,14 @@
         <v>0</v>
       </c>
       <c r="H45" s="27" t="n">
-        <v>-5.09</v>
+        <v>-3.33</v>
       </c>
       <c r="I45" s="28" t="n">
-        <v>58.13</v>
+        <v>25.13</v>
       </c>
       <c r="J45" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +397%</t>
+          <t>네이버 검색 당일 +280%</t>
         </is>
       </c>
       <c r="K45" s="29" t="inlineStr">
@@ -2284,7 +2282,7 @@
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B46" s="25" t="n">
@@ -2292,7 +2290,7 @@
       </c>
       <c r="C46" s="26" t="inlineStr">
         <is>
-          <t>한켐</t>
+          <t>한컴라이프케어</t>
         </is>
       </c>
       <c r="D46" s="25" t="n">
@@ -2307,15 +2305,15 @@
       <c r="G46" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H46" s="27" t="n">
-        <v>-5.41</v>
+      <c r="H46" s="28" t="n">
+        <v>4.85</v>
       </c>
       <c r="I46" s="28" t="n">
-        <v>37.38</v>
+        <v>20.23</v>
       </c>
       <c r="J46" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +341%</t>
+          <t>네이버 검색 당일 +226%</t>
         </is>
       </c>
       <c r="K46" s="29" t="inlineStr">
@@ -2327,7 +2325,7 @@
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B47" s="25" t="n">
@@ -2335,7 +2333,7 @@
       </c>
       <c r="C47" s="26" t="inlineStr">
         <is>
-          <t>아톤</t>
+          <t>진양화학</t>
         </is>
       </c>
       <c r="D47" s="25" t="n">
@@ -2351,14 +2349,14 @@
         <v>0</v>
       </c>
       <c r="H47" s="27" t="n">
-        <v>-3.27</v>
+        <v>-6.03</v>
       </c>
       <c r="I47" s="28" t="n">
-        <v>16.48</v>
+        <v>22.47</v>
       </c>
       <c r="J47" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +291%</t>
+          <t>네이버 검색 당일 +225%</t>
         </is>
       </c>
       <c r="K47" s="29" t="inlineStr">
@@ -2370,7 +2368,7 @@
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B48" s="25" t="n">
@@ -2378,7 +2376,7 @@
       </c>
       <c r="C48" s="26" t="inlineStr">
         <is>
-          <t>한국첨단소재</t>
+          <t>티엠씨</t>
         </is>
       </c>
       <c r="D48" s="25" t="n">
@@ -2393,15 +2391,15 @@
       <c r="G48" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H48" s="27" t="n">
-        <v>-2.92</v>
+      <c r="H48" s="28" t="n">
+        <v>7.8</v>
       </c>
       <c r="I48" s="28" t="n">
-        <v>50.25</v>
+        <v>37.22</v>
       </c>
       <c r="J48" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +288%</t>
+          <t>네이버 검색 당일 +195%</t>
         </is>
       </c>
       <c r="K48" s="29" t="inlineStr">
@@ -2413,7 +2411,7 @@
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B49" s="25" t="n">
@@ -2421,7 +2419,7 @@
       </c>
       <c r="C49" s="26" t="inlineStr">
         <is>
-          <t>한컴위드</t>
+          <t>센서뷰</t>
         </is>
       </c>
       <c r="D49" s="25" t="n">
@@ -2436,15 +2434,15 @@
       <c r="G49" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H49" s="27" t="n">
-        <v>-3.33</v>
+      <c r="H49" s="28" t="n">
+        <v>7.05</v>
       </c>
       <c r="I49" s="28" t="n">
-        <v>25.13</v>
+        <v>56.85</v>
       </c>
       <c r="J49" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +269%</t>
+          <t>네이버 검색 당일 +194%</t>
         </is>
       </c>
       <c r="K49" s="29" t="inlineStr">
@@ -2456,7 +2454,7 @@
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B50" s="25" t="n">
@@ -2464,7 +2462,7 @@
       </c>
       <c r="C50" s="26" t="inlineStr">
         <is>
-          <t>진양화학</t>
+          <t>나라스페이스테크놀로지</t>
         </is>
       </c>
       <c r="D50" s="25" t="n">
@@ -2479,15 +2477,15 @@
       <c r="G50" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H50" s="27" t="n">
-        <v>-6.03</v>
+      <c r="H50" s="28" t="n">
+        <v>1.81</v>
       </c>
       <c r="I50" s="28" t="n">
-        <v>22.47</v>
+        <v>36.89</v>
       </c>
       <c r="J50" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +214%</t>
+          <t>네이버 검색 당일 +191%</t>
         </is>
       </c>
       <c r="K50" s="29" t="inlineStr">
@@ -2499,7 +2497,7 @@
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B51" s="25" t="n">
@@ -2507,7 +2505,7 @@
       </c>
       <c r="C51" s="26" t="inlineStr">
         <is>
-          <t>한컴라이프케어</t>
+          <t>오션인더블유</t>
         </is>
       </c>
       <c r="D51" s="25" t="n">
@@ -2523,14 +2521,14 @@
         <v>0</v>
       </c>
       <c r="H51" s="28" t="n">
-        <v>4.85</v>
+        <v>18.49</v>
       </c>
       <c r="I51" s="28" t="n">
-        <v>20.23</v>
+        <v>18.57</v>
       </c>
       <c r="J51" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +201%</t>
+          <t>네이버 검색 당일 +179%</t>
         </is>
       </c>
       <c r="K51" s="29" t="inlineStr">
@@ -2542,7 +2540,7 @@
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B52" s="25" t="n">
@@ -2550,7 +2548,7 @@
       </c>
       <c r="C52" s="26" t="inlineStr">
         <is>
-          <t>티엠씨</t>
+          <t>광전자</t>
         </is>
       </c>
       <c r="D52" s="25" t="n">
@@ -2566,14 +2564,14 @@
         <v>0</v>
       </c>
       <c r="H52" s="28" t="n">
-        <v>7.8</v>
+        <v>3.53</v>
       </c>
       <c r="I52" s="28" t="n">
-        <v>37.22</v>
+        <v>33.67</v>
       </c>
       <c r="J52" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +180%</t>
+          <t>네이버 검색 당일 +166%</t>
         </is>
       </c>
       <c r="K52" s="29" t="inlineStr">
@@ -2585,7 +2583,7 @@
     <row r="53" ht="18" customHeight="1">
       <c r="A53" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B53" s="25" t="n">
@@ -2593,7 +2591,7 @@
       </c>
       <c r="C53" s="26" t="inlineStr">
         <is>
-          <t>센서뷰</t>
+          <t>켄코아에어로스페이스</t>
         </is>
       </c>
       <c r="D53" s="25" t="n">
@@ -2609,14 +2607,14 @@
         <v>0</v>
       </c>
       <c r="H53" s="28" t="n">
-        <v>7.05</v>
+        <v>12.69</v>
       </c>
       <c r="I53" s="28" t="n">
-        <v>56.85</v>
+        <v>28.67</v>
       </c>
       <c r="J53" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +177%</t>
+          <t>네이버 검색 당일 +158%</t>
         </is>
       </c>
       <c r="K53" s="29" t="inlineStr">
@@ -2628,7 +2626,7 @@
     <row r="54" ht="18" customHeight="1">
       <c r="A54" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B54" s="25" t="n">
@@ -2636,7 +2634,7 @@
       </c>
       <c r="C54" s="26" t="inlineStr">
         <is>
-          <t>나라스페이스테크놀로지</t>
+          <t>에이스테크</t>
         </is>
       </c>
       <c r="D54" s="25" t="n">
@@ -2652,14 +2650,14 @@
         <v>0</v>
       </c>
       <c r="H54" s="28" t="n">
-        <v>1.81</v>
+        <v>5.74</v>
       </c>
       <c r="I54" s="28" t="n">
-        <v>36.89</v>
+        <v>24.22</v>
       </c>
       <c r="J54" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +176%</t>
+          <t>네이버 검색 당일 +148%</t>
         </is>
       </c>
       <c r="K54" s="29" t="inlineStr">
@@ -2671,7 +2669,7 @@
     <row r="55" ht="18" customHeight="1">
       <c r="A55" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B55" s="25" t="n">
@@ -2679,7 +2677,7 @@
       </c>
       <c r="C55" s="26" t="inlineStr">
         <is>
-          <t>광전자</t>
+          <t>이엔셀</t>
         </is>
       </c>
       <c r="D55" s="25" t="n">
@@ -2695,14 +2693,14 @@
         <v>0</v>
       </c>
       <c r="H55" s="28" t="n">
-        <v>3.53</v>
+        <v>30.15</v>
       </c>
       <c r="I55" s="28" t="n">
-        <v>33.67</v>
+        <v>25.6</v>
       </c>
       <c r="J55" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +160%</t>
+          <t>네이버 검색 당일 +146%</t>
         </is>
       </c>
       <c r="K55" s="29" t="inlineStr">
@@ -2714,7 +2712,7 @@
     <row r="56" ht="18" customHeight="1">
       <c r="A56" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B56" s="25" t="n">
@@ -2722,7 +2720,7 @@
       </c>
       <c r="C56" s="26" t="inlineStr">
         <is>
-          <t>오션인더블유</t>
+          <t>아이씨티케이</t>
         </is>
       </c>
       <c r="D56" s="25" t="n">
@@ -2738,14 +2736,14 @@
         <v>0</v>
       </c>
       <c r="H56" s="28" t="n">
-        <v>18.49</v>
+        <v>3.95</v>
       </c>
       <c r="I56" s="28" t="n">
-        <v>18.57</v>
+        <v>29.94</v>
       </c>
       <c r="J56" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +144%</t>
+          <t>네이버 검색 당일 +133%</t>
         </is>
       </c>
       <c r="K56" s="29" t="inlineStr">
@@ -2757,7 +2755,7 @@
     <row r="57" ht="18" customHeight="1">
       <c r="A57" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B57" s="25" t="n">
@@ -2765,7 +2763,7 @@
       </c>
       <c r="C57" s="26" t="inlineStr">
         <is>
-          <t>에이스테크</t>
+          <t>우리넷</t>
         </is>
       </c>
       <c r="D57" s="25" t="n">
@@ -2781,14 +2779,14 @@
         <v>0</v>
       </c>
       <c r="H57" s="28" t="n">
-        <v>5.74</v>
+        <v>8.26</v>
       </c>
       <c r="I57" s="28" t="n">
-        <v>24.22</v>
+        <v>23.13</v>
       </c>
       <c r="J57" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +139%</t>
+          <t>네이버 검색 당일 +104%</t>
         </is>
       </c>
       <c r="K57" s="29" t="inlineStr">
@@ -2800,7 +2798,7 @@
     <row r="58" ht="18" customHeight="1">
       <c r="A58" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B58" s="25" t="n">
@@ -2808,7 +2806,7 @@
       </c>
       <c r="C58" s="26" t="inlineStr">
         <is>
-          <t>켄코아에어로스페이스</t>
+          <t>성호전자</t>
         </is>
       </c>
       <c r="D58" s="25" t="n">
@@ -2824,26 +2822,26 @@
         <v>0</v>
       </c>
       <c r="H58" s="28" t="n">
-        <v>12.69</v>
+        <v>18.92</v>
       </c>
       <c r="I58" s="28" t="n">
-        <v>28.67</v>
+        <v>51.03</v>
       </c>
       <c r="J58" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +136%</t>
+          <t>네이버 검색 당일 +92% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K58" s="29" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="59" ht="18" customHeight="1">
       <c r="A59" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B59" s="25" t="n">
@@ -2851,7 +2849,7 @@
       </c>
       <c r="C59" s="26" t="inlineStr">
         <is>
-          <t>아이씨티케이</t>
+          <t>스피어</t>
         </is>
       </c>
       <c r="D59" s="25" t="n">
@@ -2867,26 +2865,26 @@
         <v>0</v>
       </c>
       <c r="H59" s="28" t="n">
-        <v>3.95</v>
+        <v>1.45</v>
       </c>
       <c r="I59" s="28" t="n">
-        <v>29.94</v>
+        <v>21.95</v>
       </c>
       <c r="J59" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +119%</t>
+          <t>네이버 검색 당일 +50% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K59" s="29" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="60" ht="18" customHeight="1">
       <c r="A60" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B60" s="25" t="n">
@@ -2894,7 +2892,7 @@
       </c>
       <c r="C60" s="26" t="inlineStr">
         <is>
-          <t>이엔셀</t>
+          <t>삼성전자우</t>
         </is>
       </c>
       <c r="D60" s="25" t="n">
@@ -2910,26 +2908,24 @@
         <v>0</v>
       </c>
       <c r="H60" s="28" t="n">
-        <v>30.15</v>
+        <v>0.41</v>
       </c>
       <c r="I60" s="28" t="n">
-        <v>25.6</v>
+        <v>1.86</v>
       </c>
       <c r="J60" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +114%</t>
-        </is>
-      </c>
-      <c r="K60" s="29" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+          <t>매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K60" s="29" t="n">
+        <v/>
       </c>
     </row>
     <row r="61" ht="18" customHeight="1">
       <c r="A61" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B61" s="25" t="n">
@@ -2937,7 +2933,7 @@
       </c>
       <c r="C61" s="26" t="inlineStr">
         <is>
-          <t>성호전자</t>
+          <t>파이온엑스</t>
         </is>
       </c>
       <c r="D61" s="25" t="n">
@@ -2952,27 +2948,27 @@
       <c r="G61" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H61" s="28" t="n">
-        <v>18.92</v>
-      </c>
-      <c r="I61" s="28" t="n">
-        <v>51.03</v>
+      <c r="H61" s="27" t="n">
+        <v>-22.35</v>
+      </c>
+      <c r="I61" s="27" t="n">
+        <v>-33.73</v>
       </c>
       <c r="J61" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +79% / 중요공시 1건</t>
+          <t>중요공시 4건</t>
         </is>
       </c>
       <c r="K61" s="29" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="62" ht="18" customHeight="1">
       <c r="A62" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B62" s="25" t="n">
@@ -2980,7 +2976,7 @@
       </c>
       <c r="C62" s="26" t="inlineStr">
         <is>
-          <t>삼성중공업</t>
+          <t>프리티</t>
         </is>
       </c>
       <c r="D62" s="25" t="n">
@@ -2996,14 +2992,14 @@
         <v>0</v>
       </c>
       <c r="H62" s="27" t="n">
-        <v>-2.32</v>
+        <v>-29.91</v>
       </c>
       <c r="I62" s="27" t="n">
-        <v>-1.64</v>
+        <v>-35.77</v>
       </c>
       <c r="J62" s="29" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 한국경제 헤드라인 언급</t>
+          <t>중요공시 3건</t>
         </is>
       </c>
       <c r="K62" s="29" t="inlineStr">
@@ -3015,7 +3011,7 @@
     <row r="63" ht="18" customHeight="1">
       <c r="A63" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B63" s="25" t="n">
@@ -3023,7 +3019,7 @@
       </c>
       <c r="C63" s="26" t="inlineStr">
         <is>
-          <t>삼성전자우</t>
+          <t>아티스트컴퍼니</t>
         </is>
       </c>
       <c r="D63" s="25" t="n">
@@ -3038,19 +3034,21 @@
       <c r="G63" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H63" s="28" t="n">
-        <v>0.41</v>
+      <c r="H63" s="27" t="n">
+        <v>-3.18</v>
       </c>
       <c r="I63" s="28" t="n">
-        <v>1.86</v>
+        <v>11.13</v>
       </c>
       <c r="J63" s="29" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K63" s="29" t="n">
-        <v/>
+          <t>중요공시 3건</t>
+        </is>
+      </c>
+      <c r="K63" s="29" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -3146,22 +3144,22 @@
         <v>1</v>
       </c>
       <c r="C3" s="25" t="n">
-        <v>47</v>
+        <v>78</v>
       </c>
       <c r="D3" s="25" t="n">
-        <v>47</v>
+        <v>78</v>
       </c>
       <c r="E3" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F3" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G3" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="H3" s="25" t="n"/>
@@ -3177,22 +3175,22 @@
         <v>1</v>
       </c>
       <c r="C4" s="25" t="n">
-        <v>17</v>
+        <v>34</v>
       </c>
       <c r="D4" s="25" t="n">
-        <v>17</v>
+        <v>34</v>
       </c>
       <c r="E4" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F4" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G4" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="H4" s="28" t="n">
@@ -3205,64 +3203,60 @@
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="26" t="inlineStr">
         <is>
-          <t>SK하이닉스</t>
+          <t>바이오</t>
         </is>
       </c>
       <c r="B5" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="25" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="D5" s="25" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="E5" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F5" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G5" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
-        </is>
-      </c>
-      <c r="H5" s="28" t="n">
-        <v>4.7</v>
-      </c>
-      <c r="I5" s="28" t="n">
-        <v>2.04</v>
-      </c>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="H5" s="25" t="n"/>
+      <c r="I5" s="25" t="n"/>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="26" t="inlineStr">
         <is>
-          <t>바이오</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="B6" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="25" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="D6" s="25" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E6" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F6" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G6" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="H6" s="25" t="n"/>
@@ -3271,38 +3265,42 @@
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="26" t="inlineStr">
         <is>
-          <t>인공지능</t>
+          <t>SK하이닉스</t>
         </is>
       </c>
       <c r="B7" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="25" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D7" s="25" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="E7" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F7" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G7" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
-        </is>
-      </c>
-      <c r="H7" s="25" t="n"/>
-      <c r="I7" s="25" t="n"/>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="H7" s="28" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="I7" s="28" t="n">
+        <v>2.04</v>
+      </c>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="26" t="inlineStr">
         <is>
-          <t>삼성전기</t>
+          <t>LG</t>
         </is>
       </c>
       <c r="B8" s="25" t="n">
@@ -3319,25 +3317,25 @@
       </c>
       <c r="F8" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G8" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
-        </is>
-      </c>
-      <c r="H8" s="28" t="n">
-        <v>2.74</v>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="H8" s="27" t="n">
+        <v>-0.62</v>
       </c>
       <c r="I8" s="27" t="n">
-        <v>-0.86</v>
+        <v>-0.36</v>
       </c>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="26" t="inlineStr">
         <is>
-          <t>게임</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="B9" s="25" t="n">
@@ -3354,12 +3352,12 @@
       </c>
       <c r="F9" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G9" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="H9" s="25" t="n"/>
@@ -3368,7 +3366,7 @@
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="26" t="inlineStr">
         <is>
-          <t>LG</t>
+          <t>GS건설</t>
         </is>
       </c>
       <c r="B10" s="25" t="n">
@@ -3385,25 +3383,25 @@
       </c>
       <c r="F10" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G10" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
-        </is>
-      </c>
-      <c r="H10" s="27" t="n">
-        <v>-0.62</v>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="H10" s="28" t="n">
+        <v>1.5</v>
       </c>
       <c r="I10" s="27" t="n">
-        <v>-0.36</v>
+        <v>-3.38</v>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="26" t="inlineStr">
         <is>
-          <t>현대차</t>
+          <t>더코디</t>
         </is>
       </c>
       <c r="B11" s="25" t="n">
@@ -3420,19 +3418,19 @@
       </c>
       <c r="F11" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G11" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
-        </is>
-      </c>
-      <c r="H11" s="28" t="n">
-        <v>0.55</v>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="H11" s="27" t="n">
+        <v>-29.89</v>
       </c>
       <c r="I11" s="27" t="n">
-        <v>-4.18</v>
+        <v>-44.49</v>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1">
@@ -3445,22 +3443,22 @@
         <v>1</v>
       </c>
       <c r="C12" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D12" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E12" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F12" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G12" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="H12" s="25" t="n"/>
@@ -3469,91 +3467,99 @@
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>삼성전기</t>
         </is>
       </c>
       <c r="B13" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C13" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D13" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E13" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F13" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G13" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
-        </is>
-      </c>
-      <c r="H13" s="25" t="n"/>
-      <c r="I13" s="25" t="n"/>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="H13" s="28" t="n">
+        <v>2.74</v>
+      </c>
+      <c r="I13" s="27" t="n">
+        <v>-0.86</v>
+      </c>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>철강</t>
+          <t>GS</t>
         </is>
       </c>
       <c r="B14" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C14" s="25" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D14" s="25" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E14" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F14" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G14" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
-        </is>
-      </c>
-      <c r="H14" s="25" t="n"/>
-      <c r="I14" s="25" t="n"/>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="H14" s="27" t="n">
+        <v>-0.18</v>
+      </c>
+      <c r="I14" s="27" t="n">
+        <v>-4.2</v>
+      </c>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>Apple</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="B15" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C15" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D15" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E15" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F15" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G15" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="H15" s="25" t="n"/>
@@ -3562,38 +3568,42 @@
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>원전</t>
+          <t>SFA반도체</t>
         </is>
       </c>
       <c r="B16" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C16" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D16" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E16" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F16" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G16" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
-        </is>
-      </c>
-      <c r="H16" s="25" t="n"/>
-      <c r="I16" s="25" t="n"/>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="H16" s="28" t="n">
+        <v>3.21</v>
+      </c>
+      <c r="I16" s="28" t="n">
+        <v>27.7</v>
+      </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>GS건설</t>
+          <t>게임</t>
         </is>
       </c>
       <c r="B17" s="25" t="n">
@@ -3610,25 +3620,21 @@
       </c>
       <c r="F17" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G17" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
-        </is>
-      </c>
-      <c r="H17" s="28" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="I17" s="27" t="n">
-        <v>-3.38</v>
-      </c>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="H17" s="25" t="n"/>
+      <c r="I17" s="25" t="n"/>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="26" t="inlineStr">
         <is>
-          <t>더코디</t>
+          <t>현대차</t>
         </is>
       </c>
       <c r="B18" s="25" t="n">
@@ -3645,165 +3651,165 @@
       </c>
       <c r="F18" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G18" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
-        </is>
-      </c>
-      <c r="H18" s="27" t="n">
-        <v>-29.89</v>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="H18" s="28" t="n">
+        <v>0.55</v>
       </c>
       <c r="I18" s="27" t="n">
-        <v>-44.49</v>
+        <v>-4.18</v>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>진영</t>
+          <t>DB</t>
         </is>
       </c>
       <c r="B19" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C19" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D19" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E19" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F19" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G19" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="H19" s="28" t="n">
-        <v>8.460000000000001</v>
-      </c>
-      <c r="I19" s="28" t="n">
-        <v>11.76</v>
+        <v>0.37</v>
+      </c>
+      <c r="I19" s="27" t="n">
+        <v>-1.21</v>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="26" t="inlineStr">
         <is>
-          <t>프리티</t>
+          <t>LS마린솔루션</t>
         </is>
       </c>
       <c r="B20" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C20" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D20" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E20" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F20" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G20" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
-        </is>
-      </c>
-      <c r="H20" s="27" t="n">
-        <v>-29.91</v>
-      </c>
-      <c r="I20" s="27" t="n">
-        <v>-35.77</v>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="H20" s="28" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="I20" s="28" t="n">
+        <v>4.18</v>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="26" t="inlineStr">
         <is>
-          <t>한전산업</t>
+          <t>금호건설</t>
         </is>
       </c>
       <c r="B21" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C21" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D21" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E21" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F21" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G21" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="H21" s="28" t="n">
-        <v>0.31</v>
+        <v>0.22</v>
       </c>
       <c r="I21" s="27" t="n">
-        <v>-4.05</v>
+        <v>-8.359999999999999</v>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="26" t="inlineStr">
         <is>
-          <t>한화시스템</t>
+          <t>미투온</t>
         </is>
       </c>
       <c r="B22" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C22" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D22" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E22" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F22" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G22" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
-        </is>
-      </c>
-      <c r="H22" s="28" t="n">
-        <v>0.38</v>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="H22" s="27" t="n">
+        <v>-8.24</v>
       </c>
       <c r="I22" s="28" t="n">
-        <v>12.69</v>
+        <v>52.37</v>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="26" t="inlineStr">
         <is>
-          <t>LS마린솔루션</t>
+          <t>뷰티스킨</t>
         </is>
       </c>
       <c r="B23" s="25" t="n">
@@ -3820,25 +3826,25 @@
       </c>
       <c r="F23" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G23" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="H23" s="28" t="n">
-        <v>3.7</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="I23" s="28" t="n">
-        <v>4.18</v>
+        <v>28.54</v>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="26" t="inlineStr">
         <is>
-          <t>미투온</t>
+          <t>비츠로테크</t>
         </is>
       </c>
       <c r="B24" s="25" t="n">
@@ -3855,25 +3861,25 @@
       </c>
       <c r="F24" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G24" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
-        </is>
-      </c>
-      <c r="H24" s="27" t="n">
-        <v>-8.24</v>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="H24" s="28" t="n">
+        <v>1.66</v>
       </c>
       <c r="I24" s="28" t="n">
-        <v>52.37</v>
+        <v>33.07</v>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="26" t="inlineStr">
         <is>
-          <t>뷰티스킨</t>
+          <t>제주항공</t>
         </is>
       </c>
       <c r="B25" s="25" t="n">
@@ -3890,25 +3896,25 @@
       </c>
       <c r="F25" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G25" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
-        </is>
-      </c>
-      <c r="H25" s="28" t="n">
-        <v>9.699999999999999</v>
-      </c>
-      <c r="I25" s="28" t="n">
-        <v>28.54</v>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="H25" s="27" t="n">
+        <v>-5.07</v>
+      </c>
+      <c r="I25" s="27" t="n">
+        <v>-7.07</v>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="26" t="inlineStr">
         <is>
-          <t>비츠로테크</t>
+          <t>진영</t>
         </is>
       </c>
       <c r="B26" s="25" t="n">
@@ -3925,25 +3931,25 @@
       </c>
       <c r="F26" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G26" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="H26" s="28" t="n">
-        <v>1.66</v>
+        <v>8.460000000000001</v>
       </c>
       <c r="I26" s="28" t="n">
-        <v>33.07</v>
+        <v>11.76</v>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="26" t="inlineStr">
         <is>
-          <t>삼성증권</t>
+          <t>현대건설</t>
         </is>
       </c>
       <c r="B27" s="25" t="n">
@@ -3960,165 +3966,165 @@
       </c>
       <c r="F27" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G27" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="H27" s="27" t="n">
-        <v>-1.04</v>
+        <v>-0.71</v>
       </c>
       <c r="I27" s="27" t="n">
-        <v>-2.06</v>
+        <v>-6.89</v>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="26" t="inlineStr">
         <is>
-          <t>스피어</t>
+          <t>광전자</t>
         </is>
       </c>
       <c r="B28" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C28" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D28" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E28" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F28" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G28" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="H28" s="28" t="n">
-        <v>1.45</v>
+        <v>3.53</v>
       </c>
       <c r="I28" s="28" t="n">
-        <v>21.95</v>
+        <v>33.67</v>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="26" t="inlineStr">
         <is>
-          <t>엔에프씨</t>
+          <t>나라스페이스테크놀로지</t>
         </is>
       </c>
       <c r="B29" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C29" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D29" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E29" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F29" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G29" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="H29" s="28" t="n">
-        <v>28.91</v>
+        <v>1.81</v>
       </c>
       <c r="I29" s="28" t="n">
-        <v>16.2</v>
+        <v>36.89</v>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="26" t="inlineStr">
         <is>
-          <t>우진</t>
+          <t>빛샘전자</t>
         </is>
       </c>
       <c r="B30" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C30" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D30" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E30" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F30" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G30" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="H30" s="28" t="n">
-        <v>5.55</v>
-      </c>
-      <c r="I30" s="27" t="n">
-        <v>-0.45</v>
+        <v>3.86</v>
+      </c>
+      <c r="I30" s="28" t="n">
+        <v>57.08</v>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="26" t="inlineStr">
         <is>
-          <t>한전기술</t>
+          <t>삼성전자우</t>
         </is>
       </c>
       <c r="B31" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C31" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D31" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E31" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F31" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G31" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
-        </is>
-      </c>
-      <c r="H31" s="27" t="n">
-        <v>-2.6</v>
-      </c>
-      <c r="I31" s="27" t="n">
-        <v>-11.45</v>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="H31" s="28" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="I31" s="28" t="n">
+        <v>1.86</v>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="26" t="inlineStr">
         <is>
-          <t>광전자</t>
+          <t>성호전자</t>
         </is>
       </c>
       <c r="B32" s="25" t="n">
@@ -4135,25 +4141,25 @@
       </c>
       <c r="F32" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G32" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="H32" s="28" t="n">
-        <v>3.53</v>
+        <v>18.92</v>
       </c>
       <c r="I32" s="28" t="n">
-        <v>33.67</v>
+        <v>51.03</v>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="26" t="inlineStr">
         <is>
-          <t>나라스페이스테크놀로지</t>
+          <t>센서뷰</t>
         </is>
       </c>
       <c r="B33" s="25" t="n">
@@ -4170,25 +4176,25 @@
       </c>
       <c r="F33" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G33" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="H33" s="28" t="n">
-        <v>1.81</v>
+        <v>7.05</v>
       </c>
       <c r="I33" s="28" t="n">
-        <v>36.89</v>
+        <v>56.85</v>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="26" t="inlineStr">
         <is>
-          <t>빛샘전자</t>
+          <t>스피어</t>
         </is>
       </c>
       <c r="B34" s="25" t="n">
@@ -4205,25 +4211,25 @@
       </c>
       <c r="F34" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G34" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="H34" s="28" t="n">
-        <v>3.86</v>
+        <v>1.45</v>
       </c>
       <c r="I34" s="28" t="n">
-        <v>57.08</v>
+        <v>21.95</v>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="26" t="inlineStr">
         <is>
-          <t>삼성전자우</t>
+          <t>아이씨티케이</t>
         </is>
       </c>
       <c r="B35" s="25" t="n">
@@ -4240,25 +4246,25 @@
       </c>
       <c r="F35" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G35" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="H35" s="28" t="n">
-        <v>0.41</v>
+        <v>3.95</v>
       </c>
       <c r="I35" s="28" t="n">
-        <v>1.86</v>
+        <v>29.94</v>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="26" t="inlineStr">
         <is>
-          <t>삼성중공업</t>
+          <t>아이티센피엔에스</t>
         </is>
       </c>
       <c r="B36" s="25" t="n">
@@ -4275,25 +4281,25 @@
       </c>
       <c r="F36" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G36" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="H36" s="27" t="n">
-        <v>-2.32</v>
-      </c>
-      <c r="I36" s="27" t="n">
-        <v>-1.64</v>
+        <v>-3.01</v>
+      </c>
+      <c r="I36" s="28" t="n">
+        <v>66.41</v>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="26" t="inlineStr">
         <is>
-          <t>성호전자</t>
+          <t>아톤</t>
         </is>
       </c>
       <c r="B37" s="25" t="n">
@@ -4310,25 +4316,25 @@
       </c>
       <c r="F37" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G37" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
-        </is>
-      </c>
-      <c r="H37" s="28" t="n">
-        <v>18.92</v>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="H37" s="27" t="n">
+        <v>-3.27</v>
       </c>
       <c r="I37" s="28" t="n">
-        <v>51.03</v>
+        <v>16.48</v>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="26" t="inlineStr">
         <is>
-          <t>센서뷰</t>
+          <t>아티스트컴퍼니</t>
         </is>
       </c>
       <c r="B38" s="25" t="n">
@@ -4345,25 +4351,25 @@
       </c>
       <c r="F38" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G38" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
-        </is>
-      </c>
-      <c r="H38" s="28" t="n">
-        <v>7.05</v>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="H38" s="27" t="n">
+        <v>-3.18</v>
       </c>
       <c r="I38" s="28" t="n">
-        <v>56.85</v>
+        <v>11.13</v>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="26" t="inlineStr">
         <is>
-          <t>아이씨티케이</t>
+          <t>에이스테크</t>
         </is>
       </c>
       <c r="B39" s="25" t="n">
@@ -4380,25 +4386,25 @@
       </c>
       <c r="F39" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G39" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="H39" s="28" t="n">
-        <v>3.95</v>
+        <v>5.74</v>
       </c>
       <c r="I39" s="28" t="n">
-        <v>29.94</v>
+        <v>24.22</v>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="26" t="inlineStr">
         <is>
-          <t>아이티센피엔에스</t>
+          <t>오션인더블유</t>
         </is>
       </c>
       <c r="B40" s="25" t="n">
@@ -4415,25 +4421,25 @@
       </c>
       <c r="F40" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G40" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
-        </is>
-      </c>
-      <c r="H40" s="27" t="n">
-        <v>-3.01</v>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="H40" s="28" t="n">
+        <v>18.49</v>
       </c>
       <c r="I40" s="28" t="n">
-        <v>66.41</v>
+        <v>18.57</v>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="26" t="inlineStr">
         <is>
-          <t>아톤</t>
+          <t>우리넷</t>
         </is>
       </c>
       <c r="B41" s="25" t="n">
@@ -4450,25 +4456,25 @@
       </c>
       <c r="F41" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G41" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
-        </is>
-      </c>
-      <c r="H41" s="27" t="n">
-        <v>-3.27</v>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="H41" s="28" t="n">
+        <v>8.26</v>
       </c>
       <c r="I41" s="28" t="n">
-        <v>16.48</v>
+        <v>23.13</v>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="26" t="inlineStr">
         <is>
-          <t>에이스테크</t>
+          <t>이엔셀</t>
         </is>
       </c>
       <c r="B42" s="25" t="n">
@@ -4485,25 +4491,25 @@
       </c>
       <c r="F42" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G42" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="H42" s="28" t="n">
-        <v>5.74</v>
+        <v>30.15</v>
       </c>
       <c r="I42" s="28" t="n">
-        <v>24.22</v>
+        <v>25.6</v>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="26" t="inlineStr">
         <is>
-          <t>오션인더블유</t>
+          <t>진양화학</t>
         </is>
       </c>
       <c r="B43" s="25" t="n">
@@ -4520,25 +4526,25 @@
       </c>
       <c r="F43" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G43" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
-        </is>
-      </c>
-      <c r="H43" s="28" t="n">
-        <v>18.49</v>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="H43" s="27" t="n">
+        <v>-6.03</v>
       </c>
       <c r="I43" s="28" t="n">
-        <v>18.57</v>
+        <v>22.47</v>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="26" t="inlineStr">
         <is>
-          <t>이엔셀</t>
+          <t>켄코아에어로스페이스</t>
         </is>
       </c>
       <c r="B44" s="25" t="n">
@@ -4555,25 +4561,25 @@
       </c>
       <c r="F44" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G44" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="H44" s="28" t="n">
-        <v>30.15</v>
+        <v>12.69</v>
       </c>
       <c r="I44" s="28" t="n">
-        <v>25.6</v>
+        <v>28.67</v>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="26" t="inlineStr">
         <is>
-          <t>진양화학</t>
+          <t>큐라티스</t>
         </is>
       </c>
       <c r="B45" s="25" t="n">
@@ -4590,25 +4596,25 @@
       </c>
       <c r="F45" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G45" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="H45" s="27" t="n">
-        <v>-6.03</v>
+        <v>-5.09</v>
       </c>
       <c r="I45" s="28" t="n">
-        <v>22.47</v>
+        <v>58.13</v>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="26" t="inlineStr">
         <is>
-          <t>켄코아에어로스페이스</t>
+          <t>티엠씨</t>
         </is>
       </c>
       <c r="B46" s="25" t="n">
@@ -4625,25 +4631,25 @@
       </c>
       <c r="F46" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G46" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="H46" s="28" t="n">
-        <v>12.69</v>
+        <v>7.8</v>
       </c>
       <c r="I46" s="28" t="n">
-        <v>28.67</v>
+        <v>37.22</v>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="26" t="inlineStr">
         <is>
-          <t>큐라티스</t>
+          <t>파이온엑스</t>
         </is>
       </c>
       <c r="B47" s="25" t="n">
@@ -4660,25 +4666,25 @@
       </c>
       <c r="F47" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G47" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="H47" s="27" t="n">
-        <v>-5.09</v>
-      </c>
-      <c r="I47" s="28" t="n">
-        <v>58.13</v>
+        <v>-22.35</v>
+      </c>
+      <c r="I47" s="27" t="n">
+        <v>-33.73</v>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="26" t="inlineStr">
         <is>
-          <t>티엠씨</t>
+          <t>프리티</t>
         </is>
       </c>
       <c r="B48" s="25" t="n">
@@ -4695,19 +4701,19 @@
       </c>
       <c r="F48" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G48" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
-        </is>
-      </c>
-      <c r="H48" s="28" t="n">
-        <v>7.8</v>
-      </c>
-      <c r="I48" s="28" t="n">
-        <v>37.22</v>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="H48" s="27" t="n">
+        <v>-29.91</v>
+      </c>
+      <c r="I48" s="27" t="n">
+        <v>-35.77</v>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
@@ -4730,12 +4736,12 @@
       </c>
       <c r="F49" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G49" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="H49" s="27" t="n">
@@ -4765,12 +4771,12 @@
       </c>
       <c r="F50" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G50" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="H50" s="28" t="n">
@@ -4800,12 +4806,12 @@
       </c>
       <c r="F51" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G51" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="H51" s="27" t="n">
@@ -4835,12 +4841,12 @@
       </c>
       <c r="F52" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G52" s="25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="H52" s="27" t="n">
@@ -4931,19 +4937,19 @@
         <v>1</v>
       </c>
       <c r="C3" s="36" t="n">
-        <v>47</v>
+        <v>78</v>
       </c>
       <c r="D3" s="36" t="n">
-        <v>47</v>
+        <v>78</v>
       </c>
       <c r="E3" s="36" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="F3" s="37" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G3" s="37" t="inlineStr">
@@ -4962,19 +4968,19 @@
         <v>1</v>
       </c>
       <c r="C4" s="36" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="D4" s="36" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="E4" s="36" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="F4" s="37" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G4" s="37" t="inlineStr">
@@ -4986,7 +4992,7 @@
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="35" t="inlineStr">
         <is>
-          <t>원전</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="B5" s="36" t="n">
@@ -5000,12 +5006,12 @@
       </c>
       <c r="E5" s="36" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="F5" s="37" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G5" s="37" t="inlineStr">
@@ -5017,26 +5023,26 @@
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="35" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>게임</t>
         </is>
       </c>
       <c r="B6" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="36" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D6" s="36" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E6" s="36" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="F6" s="37" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G6" s="37" t="inlineStr">
@@ -5048,7 +5054,7 @@
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="35" t="inlineStr">
         <is>
-          <t>게임</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="B7" s="36" t="n">
@@ -5062,12 +5068,12 @@
       </c>
       <c r="E7" s="36" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="F7" s="37" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G7" s="37" t="inlineStr">
@@ -5079,26 +5085,26 @@
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="35" t="inlineStr">
         <is>
-          <t>철강</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="B8" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="36" t="n">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="D8" s="36" t="n">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="E8" s="36" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="F8" s="37" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G8" s="37" t="inlineStr">
@@ -5108,71 +5114,63 @@
       </c>
     </row>
     <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="35" t="inlineStr">
-        <is>
-          <t>제약</t>
-        </is>
-      </c>
-      <c r="B9" s="36" t="n">
-        <v>1</v>
-      </c>
-      <c r="C9" s="36" t="n">
-        <v>7</v>
-      </c>
-      <c r="D9" s="36" t="n">
-        <v>7</v>
-      </c>
-      <c r="E9" s="36" t="inlineStr">
-        <is>
-          <t>2026-09-20</t>
-        </is>
-      </c>
-      <c r="F9" s="37" t="inlineStr">
-        <is>
-          <t>2026-09-20</t>
-        </is>
-      </c>
-      <c r="G9" s="37" t="inlineStr">
-        <is>
-          <t>⚡ 관심</t>
-        </is>
-      </c>
+      <c r="A9" s="26" t="inlineStr">
+        <is>
+          <t>이차전지</t>
+        </is>
+      </c>
+      <c r="B9" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F9" s="29" t="inlineStr">
+        <is>
+          <t>감지 없음</t>
+        </is>
+      </c>
+      <c r="G9" s="29" t="inlineStr"/>
     </row>
     <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="35" t="inlineStr">
-        <is>
-          <t>인공지능</t>
-        </is>
-      </c>
-      <c r="B10" s="36" t="n">
-        <v>1</v>
-      </c>
-      <c r="C10" s="36" t="n">
-        <v>15</v>
-      </c>
-      <c r="D10" s="36" t="n">
-        <v>15</v>
-      </c>
-      <c r="E10" s="36" t="inlineStr">
-        <is>
-          <t>2026-09-20</t>
-        </is>
-      </c>
-      <c r="F10" s="37" t="inlineStr">
-        <is>
-          <t>2026-09-20</t>
-        </is>
-      </c>
-      <c r="G10" s="37" t="inlineStr">
-        <is>
-          <t>⚡ 관심</t>
-        </is>
-      </c>
+      <c r="A10" s="26" t="inlineStr">
+        <is>
+          <t>AI반도체</t>
+        </is>
+      </c>
+      <c r="B10" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F10" s="29" t="inlineStr">
+        <is>
+          <t>감지 없음</t>
+        </is>
+      </c>
+      <c r="G10" s="29" t="inlineStr"/>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="26" t="inlineStr">
         <is>
-          <t>이차전지</t>
+          <t>전기차</t>
         </is>
       </c>
       <c r="B11" s="25" t="n">
@@ -5199,7 +5197,7 @@
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="26" t="inlineStr">
         <is>
-          <t>AI반도체</t>
+          <t>방산</t>
         </is>
       </c>
       <c r="B12" s="25" t="n">
@@ -5226,7 +5224,7 @@
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>전기차</t>
+          <t>원전</t>
         </is>
       </c>
       <c r="B13" s="25" t="n">
@@ -5253,7 +5251,7 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>방산</t>
+          <t>수소</t>
         </is>
       </c>
       <c r="B14" s="25" t="n">
@@ -5280,7 +5278,7 @@
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>수소</t>
+          <t>태양광</t>
         </is>
       </c>
       <c r="B15" s="25" t="n">
@@ -5307,7 +5305,7 @@
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>태양광</t>
+          <t>엔터</t>
         </is>
       </c>
       <c r="B16" s="25" t="n">
@@ -5334,7 +5332,7 @@
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>엔터</t>
+          <t>핀테크</t>
         </is>
       </c>
       <c r="B17" s="25" t="n">
@@ -5361,7 +5359,7 @@
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="26" t="inlineStr">
         <is>
-          <t>핀테크</t>
+          <t>클라우드</t>
         </is>
       </c>
       <c r="B18" s="25" t="n">
@@ -5388,7 +5386,7 @@
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>클라우드</t>
+          <t>조선</t>
         </is>
       </c>
       <c r="B19" s="25" t="n">
@@ -5415,7 +5413,7 @@
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="26" t="inlineStr">
         <is>
-          <t>조선</t>
+          <t>철강</t>
         </is>
       </c>
       <c r="B20" s="25" t="n">

</xml_diff>

<commit_message>
auto: 2026-09-24 06:56 자동 백업
</commit_message>
<xml_diff>
--- a/trend/stock_trend_history.xlsx
+++ b/trend/stock_trend_history.xlsx
@@ -258,13 +258,13 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -694,7 +694,7 @@
     <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-09-23 06:54</t>
+          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-09-24 06:54</t>
         </is>
       </c>
     </row>
@@ -708,7 +708,7 @@
       </c>
       <c r="E3" s="3" t="n"/>
       <c r="G3" s="5" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="H3" s="3" t="n"/>
       <c r="J3" s="6" t="n">
@@ -787,21 +787,21 @@
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-09-23) 상위: 반도체  점수 75.0점</t>
+          <t>⚡ 최신(2026-09-24) 상위: 반도체  점수 51.0점</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-09-23) 상위: 원전  점수 24.0점</t>
+          <t>⚡ 최신(2026-09-24) 상위: 삼성전자  점수 32.0점</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-09-23) 상위: 삼성전자  점수 21.0점</t>
+          <t>⚡ 최신(2026-09-24) 상위: SK하이닉스  점수 18.0점</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="15" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B14" s="15" t="n">
@@ -928,10 +928,10 @@
         </is>
       </c>
       <c r="D14" s="15" t="n">
-        <v>75</v>
+        <v>51</v>
       </c>
       <c r="E14" s="15" t="n">
-        <v>75</v>
+        <v>51</v>
       </c>
       <c r="F14" s="15" t="n">
         <v>0</v>
@@ -947,7 +947,7 @@
       </c>
       <c r="J14" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+          <t>매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K14" s="17" t="inlineStr">
@@ -959,7 +959,7 @@
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="15" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B15" s="15" t="n">
@@ -967,14 +967,14 @@
       </c>
       <c r="C15" s="16" t="inlineStr">
         <is>
-          <t>원전</t>
+          <t>삼성전자</t>
         </is>
       </c>
       <c r="D15" s="15" t="n">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="E15" s="15" t="n">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="F15" s="15" t="n">
         <v>0</v>
@@ -982,25 +982,27 @@
       <c r="G15" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H15" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I15" s="15" t="n">
-        <v/>
+      <c r="H15" s="18" t="n">
+        <v>3.24</v>
+      </c>
+      <c r="I15" s="18" t="n">
+        <v>13.02</v>
       </c>
       <c r="J15" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K15" s="17" t="n">
-        <v/>
+          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K15" s="17" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="15" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B16" s="15" t="n">
@@ -1008,14 +1010,14 @@
       </c>
       <c r="C16" s="16" t="inlineStr">
         <is>
-          <t>삼성전자</t>
+          <t>SK하이닉스</t>
         </is>
       </c>
       <c r="D16" s="15" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E16" s="15" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F16" s="15" t="n">
         <v>0</v>
@@ -1024,24 +1026,26 @@
         <v>0</v>
       </c>
       <c r="H16" s="18" t="n">
-        <v>0.91</v>
+        <v>1.2</v>
       </c>
       <c r="I16" s="18" t="n">
-        <v>10.78</v>
+        <v>6.03</v>
       </c>
       <c r="J16" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K16" s="17" t="n">
-        <v/>
+          <t>매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K16" s="17" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B17" s="15" t="n">
@@ -1049,14 +1053,14 @@
       </c>
       <c r="C17" s="16" t="inlineStr">
         <is>
-          <t>SK하이닉스</t>
+          <t>원전</t>
         </is>
       </c>
       <c r="D17" s="15" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E17" s="15" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F17" s="15" t="n">
         <v>0</v>
@@ -1064,15 +1068,15 @@
       <c r="G17" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H17" s="19" t="n">
-        <v>-2.02</v>
-      </c>
-      <c r="I17" s="18" t="n">
-        <v>7.54</v>
+      <c r="H17" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I17" s="15" t="n">
+        <v/>
       </c>
       <c r="J17" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K17" s="17" t="n">
@@ -1082,7 +1086,7 @@
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B18" s="15" t="n">
@@ -1090,14 +1094,14 @@
       </c>
       <c r="C18" s="16" t="inlineStr">
         <is>
-          <t>LG</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="D18" s="15" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E18" s="15" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F18" s="15" t="n">
         <v>0</v>
@@ -1105,25 +1109,27 @@
       <c r="G18" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H18" s="18" t="n">
-        <v>3.66</v>
-      </c>
-      <c r="I18" s="18" t="n">
-        <v>2.38</v>
+      <c r="H18" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I18" s="15" t="n">
+        <v/>
       </c>
       <c r="J18" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K18" s="17" t="n">
-        <v/>
+          <t>매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K18" s="17" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B19" s="15" t="n">
@@ -1131,7 +1137,7 @@
       </c>
       <c r="C19" s="16" t="inlineStr">
         <is>
-          <t>인공지능</t>
+          <t>대한항공</t>
         </is>
       </c>
       <c r="D19" s="15" t="n">
@@ -1146,27 +1152,25 @@
       <c r="G19" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H19" s="15" t="n">
+      <c r="H19" s="19" t="n">
+        <v>-0.47</v>
+      </c>
+      <c r="I19" s="18" t="n">
+        <v>7.69</v>
+      </c>
+      <c r="J19" s="17" t="inlineStr">
+        <is>
+          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K19" s="17" t="n">
         <v/>
-      </c>
-      <c r="I19" s="15" t="n">
-        <v/>
-      </c>
-      <c r="J19" s="17" t="inlineStr">
-        <is>
-          <t>매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K19" s="17" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B20" s="15" t="n">
@@ -1174,14 +1178,14 @@
       </c>
       <c r="C20" s="16" t="inlineStr">
         <is>
-          <t>셀리드</t>
+          <t>LG전자</t>
         </is>
       </c>
       <c r="D20" s="15" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E20" s="15" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F20" s="15" t="n">
         <v>0</v>
@@ -1189,27 +1193,25 @@
       <c r="G20" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H20" s="18" t="n">
-        <v>14.94</v>
+      <c r="H20" s="19" t="n">
+        <v>-2.09</v>
       </c>
       <c r="I20" s="18" t="n">
-        <v>24.62</v>
+        <v>5.46</v>
       </c>
       <c r="J20" s="17" t="inlineStr">
         <is>
-          <t>중요공시 4건 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K20" s="17" t="inlineStr">
-        <is>
-          <t>네이버, 공시</t>
-        </is>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K20" s="17" t="n">
+        <v/>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="15" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B21" s="15" t="n">
@@ -1221,10 +1223,10 @@
         </is>
       </c>
       <c r="D21" s="15" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E21" s="15" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F21" s="15" t="n">
         <v>0</v>
@@ -1233,14 +1235,14 @@
         <v>0</v>
       </c>
       <c r="H21" s="18" t="n">
-        <v>3.98</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="I21" s="18" t="n">
-        <v>11.95</v>
+        <v>9.4</v>
       </c>
       <c r="J21" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K21" s="17" t="n">
@@ -1250,7 +1252,7 @@
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="15" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B22" s="15" t="n">
@@ -1258,14 +1260,14 @@
       </c>
       <c r="C22" s="16" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>카카오</t>
         </is>
       </c>
       <c r="D22" s="15" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E22" s="15" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F22" s="15" t="n">
         <v>0</v>
@@ -1273,25 +1275,27 @@
       <c r="G22" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H22" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I22" s="15" t="n">
-        <v/>
+      <c r="H22" s="19" t="n">
+        <v>-1.31</v>
+      </c>
+      <c r="I22" s="18" t="n">
+        <v>0.45</v>
       </c>
       <c r="J22" s="17" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K22" s="17" t="n">
-        <v/>
+          <t>매일경제 기사 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K22" s="17" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="15" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B23" s="15" t="n">
@@ -1299,14 +1303,14 @@
       </c>
       <c r="C23" s="16" t="inlineStr">
         <is>
-          <t>카카오</t>
+          <t>셀리드</t>
         </is>
       </c>
       <c r="D23" s="15" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E23" s="15" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F23" s="15" t="n">
         <v>0</v>
@@ -1314,25 +1318,27 @@
       <c r="G23" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H23" s="18" t="n">
-        <v>2.54</v>
-      </c>
-      <c r="I23" s="19" t="n">
-        <v>-1.3</v>
+      <c r="H23" s="19" t="n">
+        <v>-9.710000000000001</v>
+      </c>
+      <c r="I23" s="18" t="n">
+        <v>17.08</v>
       </c>
       <c r="J23" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K23" s="17" t="n">
-        <v/>
+          <t>중요공시 4건 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K23" s="17" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="15" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B24" s="15" t="n">
@@ -1340,42 +1346,42 @@
       </c>
       <c r="C24" s="16" t="inlineStr">
         <is>
-          <t>태양광</t>
+          <t>HJ중공업</t>
         </is>
       </c>
       <c r="D24" s="15" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E24" s="15" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="F24" s="15" t="n">
         <v>0</v>
       </c>
       <c r="G24" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H24" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I24" s="15" t="n">
-        <v/>
+        <v>3</v>
+      </c>
+      <c r="H24" s="19" t="n">
+        <v>-1.78</v>
+      </c>
+      <c r="I24" s="19" t="n">
+        <v>-0.67</v>
       </c>
       <c r="J24" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>중요공시 3건 / 중요공시 7일 +200% / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K24" s="17" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="15" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B25" s="15" t="n">
@@ -1383,42 +1389,42 @@
       </c>
       <c r="C25" s="16" t="inlineStr">
         <is>
-          <t>바이오</t>
+          <t>대우건설</t>
         </is>
       </c>
       <c r="D25" s="15" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E25" s="15" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="F25" s="15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G25" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H25" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I25" s="15" t="n">
-        <v/>
+        <v>3</v>
+      </c>
+      <c r="H25" s="19" t="n">
+        <v>-6.4</v>
+      </c>
+      <c r="I25" s="19" t="n">
+        <v>-4.89</v>
       </c>
       <c r="J25" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
+          <t>중요공시 3건 / 중요공시 3일 +50% / 중요공시 7일 +50%</t>
         </is>
       </c>
       <c r="K25" s="17" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="15" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B26" s="15" t="n">
@@ -1426,7 +1432,7 @@
       </c>
       <c r="C26" s="16" t="inlineStr">
         <is>
-          <t>금호건설</t>
+          <t>스피어</t>
         </is>
       </c>
       <c r="D26" s="15" t="n">
@@ -1441,15 +1447,15 @@
       <c r="G26" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="H26" s="19" t="n">
-        <v>-3.42</v>
-      </c>
-      <c r="I26" s="19" t="n">
-        <v>-1.78</v>
+      <c r="H26" s="18" t="n">
+        <v>3.76</v>
+      </c>
+      <c r="I26" s="18" t="n">
+        <v>15.23</v>
       </c>
       <c r="J26" s="17" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 3일 +50% / 중요공시 7일 +50%</t>
+          <t>중요공시 3건 / 중요공시 3일 +200% / 중요공시 7일 +200%</t>
         </is>
       </c>
       <c r="K26" s="17" t="inlineStr">
@@ -1461,7 +1467,7 @@
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="15" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B27" s="15" t="n">
@@ -1469,7 +1475,7 @@
       </c>
       <c r="C27" s="16" t="inlineStr">
         <is>
-          <t>대우건설</t>
+          <t>금호건설</t>
         </is>
       </c>
       <c r="D27" s="15" t="n">
@@ -1484,11 +1490,11 @@
       <c r="G27" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="H27" s="18" t="n">
-        <v>2.33</v>
+      <c r="H27" s="19" t="n">
+        <v>-1.73</v>
       </c>
       <c r="I27" s="19" t="n">
-        <v>-2.12</v>
+        <v>-5.09</v>
       </c>
       <c r="J27" s="17" t="inlineStr">
         <is>
@@ -1504,7 +1510,7 @@
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="15" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B28" s="15" t="n">
@@ -1512,7 +1518,7 @@
       </c>
       <c r="C28" s="16" t="inlineStr">
         <is>
-          <t>KT&amp;G</t>
+          <t>태양광</t>
         </is>
       </c>
       <c r="D28" s="15" t="n">
@@ -1527,15 +1533,15 @@
       <c r="G28" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H28" s="18" t="n">
-        <v>1.56</v>
-      </c>
-      <c r="I28" s="18" t="n">
-        <v>3.46</v>
+      <c r="H28" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I28" s="15" t="n">
+        <v/>
       </c>
       <c r="J28" s="17" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+          <t>매일경제 기사 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K28" s="17" t="n">
@@ -1543,222 +1549,224 @@
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
-      <c r="A29" s="20" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="B29" s="20" t="n">
+      <c r="A29" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B29" s="15" t="n">
         <v>16</v>
       </c>
-      <c r="C29" s="21" t="inlineStr">
-        <is>
-          <t>LG전자</t>
-        </is>
-      </c>
-      <c r="D29" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="E29" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="F29" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G29" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H29" s="22" t="n">
-        <v>5.91</v>
-      </c>
-      <c r="I29" s="22" t="n">
-        <v>6.44</v>
-      </c>
-      <c r="J29" s="23" t="inlineStr">
-        <is>
-          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K29" s="23" t="n">
+      <c r="C29" s="16" t="inlineStr">
+        <is>
+          <t>바이오</t>
+        </is>
+      </c>
+      <c r="D29" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="E29" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="F29" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" s="15" t="n">
         <v/>
       </c>
+      <c r="I29" s="15" t="n">
+        <v/>
+      </c>
+      <c r="J29" s="17" t="inlineStr">
+        <is>
+          <t>네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급</t>
+        </is>
+      </c>
+      <c r="K29" s="17" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="18" customHeight="1">
-      <c r="A30" s="20" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="B30" s="20" t="n">
+      <c r="A30" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B30" s="15" t="n">
         <v>17</v>
       </c>
-      <c r="C30" s="21" t="inlineStr">
-        <is>
-          <t>더코디</t>
-        </is>
-      </c>
-      <c r="D30" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="E30" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="F30" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G30" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="H30" s="24" t="n">
-        <v>-20.08</v>
-      </c>
-      <c r="I30" s="24" t="n">
-        <v>-40.46</v>
-      </c>
-      <c r="J30" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 9건 / 중요공시 7일 +50%</t>
-        </is>
-      </c>
-      <c r="K30" s="23" t="inlineStr">
+      <c r="C30" s="16" t="inlineStr">
+        <is>
+          <t>한화시스템</t>
+        </is>
+      </c>
+      <c r="D30" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="E30" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="F30" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="G30" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="H30" s="19" t="n">
+        <v>-4.12</v>
+      </c>
+      <c r="I30" s="18" t="n">
+        <v>7.98</v>
+      </c>
+      <c r="J30" s="17" t="inlineStr">
+        <is>
+          <t>중요공시 2건 / 중요공시 3일 +100% / 중요공시 7일 +100% / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K30" s="17" t="inlineStr">
         <is>
           <t>공시</t>
         </is>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
-      <c r="A31" s="20" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="B31" s="20" t="n">
+      <c r="A31" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B31" s="15" t="n">
         <v>18</v>
       </c>
-      <c r="C31" s="21" t="inlineStr">
-        <is>
-          <t>우성머티리얼스</t>
-        </is>
-      </c>
-      <c r="D31" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="E31" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="F31" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G31" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="H31" s="22" t="n">
-        <v>11.39</v>
-      </c>
-      <c r="I31" s="22" t="n">
-        <v>12.08</v>
-      </c>
-      <c r="J31" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 7건 / 중요공시 7일 +600%</t>
-        </is>
-      </c>
-      <c r="K31" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
+      <c r="C31" s="16" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="D31" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="E31" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="F31" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I31" s="15" t="n">
+        <v/>
+      </c>
+      <c r="J31" s="17" t="inlineStr">
+        <is>
+          <t>네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K31" s="17" t="inlineStr">
+        <is>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
-      <c r="A32" s="20" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="B32" s="20" t="n">
+      <c r="A32" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B32" s="15" t="n">
         <v>19</v>
       </c>
-      <c r="C32" s="21" t="inlineStr">
-        <is>
-          <t>GS건설</t>
-        </is>
-      </c>
-      <c r="D32" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="E32" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="F32" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G32" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="H32" s="22" t="n">
-        <v>1.9</v>
-      </c>
-      <c r="I32" s="24" t="n">
-        <v>-1.7</v>
-      </c>
-      <c r="J32" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 4건 / 중요공시 7일 +100%</t>
-        </is>
-      </c>
-      <c r="K32" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
+      <c r="C32" s="16" t="inlineStr">
+        <is>
+          <t>방산</t>
+        </is>
+      </c>
+      <c r="D32" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="E32" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="F32" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H32" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I32" s="15" t="n">
+        <v/>
+      </c>
+      <c r="J32" s="17" t="inlineStr">
+        <is>
+          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K32" s="17" t="inlineStr">
+        <is>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
-      <c r="A33" s="20" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="B33" s="20" t="n">
+      <c r="A33" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B33" s="15" t="n">
         <v>20</v>
       </c>
-      <c r="C33" s="21" t="inlineStr">
-        <is>
-          <t>HJ중공업</t>
-        </is>
-      </c>
-      <c r="D33" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="E33" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="F33" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G33" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="H33" s="24" t="n">
-        <v>-0.72</v>
-      </c>
-      <c r="I33" s="24" t="n">
-        <v>-0.79</v>
-      </c>
-      <c r="J33" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 3건 / 중요공시 7일 +200%</t>
-        </is>
-      </c>
-      <c r="K33" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
+      <c r="C33" s="16" t="inlineStr">
+        <is>
+          <t>제약</t>
+        </is>
+      </c>
+      <c r="D33" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="E33" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="F33" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H33" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I33" s="15" t="n">
+        <v/>
+      </c>
+      <c r="J33" s="17" t="inlineStr">
+        <is>
+          <t>네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
+        </is>
+      </c>
+      <c r="K33" s="17" t="inlineStr">
+        <is>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="20" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B34" s="20" t="n">
@@ -1766,30 +1774,30 @@
       </c>
       <c r="C34" s="21" t="inlineStr">
         <is>
-          <t>스피어</t>
+          <t>대양금속</t>
         </is>
       </c>
       <c r="D34" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E34" s="20" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F34" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G34" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="H34" s="24" t="n">
-        <v>-3.62</v>
+      <c r="H34" s="22" t="n">
+        <v>-14.85</v>
       </c>
       <c r="I34" s="22" t="n">
-        <v>12.16</v>
+        <v>-11.08</v>
       </c>
       <c r="J34" s="23" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 3일 +100% / 중요공시 7일 +100%</t>
+          <t>중요공시 3건 / 중요공시 7일 +200%</t>
         </is>
       </c>
       <c r="K34" s="23" t="inlineStr">
@@ -1801,7 +1809,7 @@
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="20" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B35" s="20" t="n">
@@ -1809,30 +1817,30 @@
       </c>
       <c r="C35" s="21" t="inlineStr">
         <is>
-          <t>비에이치아이</t>
+          <t>GS건설</t>
         </is>
       </c>
       <c r="D35" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E35" s="20" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F35" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G35" s="20" t="n">
         <v>3</v>
       </c>
       <c r="H35" s="22" t="n">
-        <v>3.22</v>
-      </c>
-      <c r="I35" s="24" t="n">
-        <v>-2.43</v>
+        <v>-7.33</v>
+      </c>
+      <c r="I35" s="22" t="n">
+        <v>-5.57</v>
       </c>
       <c r="J35" s="23" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 3일 +100% / 중요공시 7일 +100%</t>
+          <t>중요공시 4건 / 중요공시 7일 +100%</t>
         </is>
       </c>
       <c r="K35" s="23" t="inlineStr">
@@ -1844,7 +1852,7 @@
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="20" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B36" s="20" t="n">
@@ -1852,7 +1860,7 @@
       </c>
       <c r="C36" s="21" t="inlineStr">
         <is>
-          <t>스테이블코인</t>
+          <t>와이즈플래닛컴퍼니</t>
         </is>
       </c>
       <c r="D36" s="20" t="n">
@@ -1875,7 +1883,7 @@
       </c>
       <c r="J36" s="23" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K36" s="23" t="n">
@@ -1885,7 +1893,7 @@
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="20" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B37" s="20" t="n">
@@ -1893,40 +1901,42 @@
       </c>
       <c r="C37" s="21" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>비에이치아이</t>
         </is>
       </c>
       <c r="D37" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E37" s="20" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F37" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G37" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H37" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I37" s="20" t="n">
-        <v/>
+        <v>3</v>
+      </c>
+      <c r="H37" s="22" t="n">
+        <v>-5.76</v>
+      </c>
+      <c r="I37" s="22" t="n">
+        <v>-4.57</v>
       </c>
       <c r="J37" s="23" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K37" s="23" t="n">
-        <v/>
+          <t>중요공시 2건 / 중요공시 3일 +100% / 중요공시 7일 +100%</t>
+        </is>
+      </c>
+      <c r="K37" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="20" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B38" s="20" t="n">
@@ -1934,40 +1944,42 @@
       </c>
       <c r="C38" s="21" t="inlineStr">
         <is>
-          <t>현대차</t>
+          <t>삼성물산</t>
         </is>
       </c>
       <c r="D38" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E38" s="20" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F38" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G38" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H38" s="22" t="n">
-        <v>0.14</v>
+      <c r="H38" s="24" t="n">
+        <v>1.1</v>
       </c>
       <c r="I38" s="24" t="n">
-        <v>-2.03</v>
+        <v>4.84</v>
       </c>
       <c r="J38" s="23" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K38" s="23" t="n">
-        <v/>
+          <t>중요공시 2건 / 중요공시 3일 +100% / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K38" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="20" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B39" s="20" t="n">
@@ -1975,42 +1987,40 @@
       </c>
       <c r="C39" s="21" t="inlineStr">
         <is>
-          <t>우진</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="D39" s="20" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E39" s="20" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F39" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G39" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H39" s="24" t="n">
-        <v>-1.95</v>
-      </c>
-      <c r="I39" s="24" t="n">
-        <v>-2.87</v>
+      <c r="H39" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I39" s="20" t="n">
+        <v/>
       </c>
       <c r="J39" s="23" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 3일 +50%</t>
-        </is>
-      </c>
-      <c r="K39" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K39" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="20" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B40" s="20" t="n">
@@ -2018,7 +2028,7 @@
       </c>
       <c r="C40" s="21" t="inlineStr">
         <is>
-          <t>조선</t>
+          <t>두산에너빌리티</t>
         </is>
       </c>
       <c r="D40" s="20" t="n">
@@ -2033,11 +2043,11 @@
       <c r="G40" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H40" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I40" s="20" t="n">
-        <v/>
+      <c r="H40" s="22" t="n">
+        <v>-4.5</v>
+      </c>
+      <c r="I40" s="22" t="n">
+        <v>-1.66</v>
       </c>
       <c r="J40" s="23" t="inlineStr">
         <is>
@@ -2053,7 +2063,7 @@
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="20" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B41" s="20" t="n">
@@ -2061,42 +2071,42 @@
       </c>
       <c r="C41" s="21" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>우진</t>
         </is>
       </c>
       <c r="D41" s="20" t="n">
         <v>5</v>
       </c>
       <c r="E41" s="20" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F41" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G41" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H41" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I41" s="20" t="n">
-        <v/>
+      <c r="H41" s="22" t="n">
+        <v>-4.46</v>
+      </c>
+      <c r="I41" s="22" t="n">
+        <v>-2.59</v>
       </c>
       <c r="J41" s="23" t="inlineStr">
         <is>
-          <t>네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
+          <t>중요공시 3건 / 중요공시 3일 +50%</t>
         </is>
       </c>
       <c r="K41" s="23" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="20" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B42" s="20" t="n">
@@ -2104,7 +2114,7 @@
       </c>
       <c r="C42" s="21" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>포스코퓨처엠</t>
         </is>
       </c>
       <c r="D42" s="20" t="n">
@@ -2119,25 +2129,27 @@
       <c r="G42" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H42" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I42" s="20" t="n">
-        <v/>
+      <c r="H42" s="22" t="n">
+        <v>-2.96</v>
+      </c>
+      <c r="I42" s="22" t="n">
+        <v>-4.24</v>
       </c>
       <c r="J42" s="23" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K42" s="23" t="n">
-        <v/>
+          <t>중요공시 1건 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K42" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="20" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B43" s="20" t="n">
@@ -2145,7 +2157,7 @@
       </c>
       <c r="C43" s="21" t="inlineStr">
         <is>
-          <t>성호전자</t>
+          <t>노타</t>
         </is>
       </c>
       <c r="D43" s="20" t="n">
@@ -2160,27 +2172,25 @@
       <c r="G43" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H43" s="24" t="n">
-        <v>-0.37</v>
-      </c>
-      <c r="I43" s="22" t="n">
-        <v>59.59</v>
+      <c r="H43" s="22" t="n">
+        <v>-9.529999999999999</v>
+      </c>
+      <c r="I43" s="24" t="n">
+        <v>21.21</v>
       </c>
       <c r="J43" s="23" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K43" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K43" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="20" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B44" s="20" t="n">
@@ -2188,7 +2198,7 @@
       </c>
       <c r="C44" s="21" t="inlineStr">
         <is>
-          <t>코리아써키트</t>
+          <t>SG</t>
         </is>
       </c>
       <c r="D44" s="20" t="n">
@@ -2203,15 +2213,15 @@
       <c r="G44" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H44" s="22" t="n">
-        <v>25.52</v>
-      </c>
-      <c r="I44" s="22" t="n">
-        <v>32.53</v>
+      <c r="H44" s="24" t="n">
+        <v>7.27</v>
+      </c>
+      <c r="I44" s="24" t="n">
+        <v>8.619999999999999</v>
       </c>
       <c r="J44" s="23" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 한국경제 헤드라인 언급</t>
+          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K44" s="23" t="n">
@@ -2221,7 +2231,7 @@
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="20" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B45" s="20" t="n">
@@ -2229,253 +2239,255 @@
       </c>
       <c r="C45" s="21" t="inlineStr">
         <is>
-          <t>광진실업</t>
+          <t>스테이블코인</t>
         </is>
       </c>
       <c r="D45" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E45" s="20" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F45" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G45" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="H45" s="24" t="n">
-        <v>-12.46</v>
-      </c>
-      <c r="I45" s="24" t="n">
-        <v>-18.87</v>
+        <v>0</v>
+      </c>
+      <c r="H45" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I45" s="20" t="n">
+        <v/>
       </c>
       <c r="J45" s="23" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 7일 +100%</t>
-        </is>
-      </c>
-      <c r="K45" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K45" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
-      <c r="A46" s="20" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="B46" s="20" t="n">
+      <c r="A46" s="25" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B46" s="25" t="n">
         <v>33</v>
       </c>
-      <c r="C46" s="21" t="inlineStr">
-        <is>
-          <t>핑거</t>
-        </is>
-      </c>
-      <c r="D46" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E46" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F46" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G46" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H46" s="22" t="n">
-        <v>10.87</v>
-      </c>
-      <c r="I46" s="22" t="n">
-        <v>27.73</v>
-      </c>
-      <c r="J46" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 2건 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K46" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
+      <c r="C46" s="26" t="inlineStr">
+        <is>
+          <t>한국제17호스팩</t>
+        </is>
+      </c>
+      <c r="D46" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E46" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F46" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G46" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H46" s="27" t="n">
+        <v>-1.91</v>
+      </c>
+      <c r="I46" s="27" t="n">
+        <v>-1.91</v>
+      </c>
+      <c r="J46" s="28" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +4057%</t>
+        </is>
+      </c>
+      <c r="K46" s="28" t="inlineStr">
+        <is>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
-      <c r="A47" s="20" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="B47" s="20" t="n">
+      <c r="A47" s="25" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B47" s="25" t="n">
         <v>34</v>
       </c>
-      <c r="C47" s="21" t="inlineStr">
-        <is>
-          <t>자이에스앤디</t>
-        </is>
-      </c>
-      <c r="D47" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E47" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F47" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G47" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H47" s="22" t="n">
-        <v>3.08</v>
-      </c>
-      <c r="I47" s="24" t="n">
-        <v>-8.720000000000001</v>
-      </c>
-      <c r="J47" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 1건 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K47" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
+      <c r="C47" s="26" t="inlineStr">
+        <is>
+          <t>KB제34호스팩</t>
+        </is>
+      </c>
+      <c r="D47" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E47" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F47" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H47" s="27" t="n">
+        <v>-0.37</v>
+      </c>
+      <c r="I47" s="27" t="n">
+        <v>-0.37</v>
+      </c>
+      <c r="J47" s="28" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +2698%</t>
+        </is>
+      </c>
+      <c r="K47" s="28" t="inlineStr">
+        <is>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
-      <c r="A48" s="20" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="B48" s="20" t="n">
+      <c r="A48" s="25" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B48" s="25" t="n">
         <v>35</v>
       </c>
-      <c r="C48" s="21" t="inlineStr">
-        <is>
-          <t>디지털대성</t>
-        </is>
-      </c>
-      <c r="D48" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E48" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F48" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G48" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H48" s="22" t="n">
-        <v>1.06</v>
-      </c>
-      <c r="I48" s="22" t="n">
-        <v>7.43</v>
-      </c>
-      <c r="J48" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 1건 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K48" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
+      <c r="C48" s="26" t="inlineStr">
+        <is>
+          <t>네오사피엔스</t>
+        </is>
+      </c>
+      <c r="D48" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E48" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F48" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G48" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H48" s="27" t="n">
+        <v>-16.78</v>
+      </c>
+      <c r="I48" s="27" t="n">
+        <v>-32.79</v>
+      </c>
+      <c r="J48" s="28" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +810%</t>
+        </is>
+      </c>
+      <c r="K48" s="28" t="inlineStr">
+        <is>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
-      <c r="A49" s="20" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="B49" s="20" t="n">
+      <c r="A49" s="25" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B49" s="25" t="n">
         <v>36</v>
       </c>
-      <c r="C49" s="21" t="inlineStr">
-        <is>
-          <t>방산</t>
-        </is>
-      </c>
-      <c r="D49" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E49" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F49" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G49" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H49" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I49" s="20" t="n">
-        <v/>
-      </c>
-      <c r="J49" s="23" t="inlineStr">
-        <is>
-          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K49" s="23" t="n">
-        <v/>
+      <c r="C49" s="26" t="inlineStr">
+        <is>
+          <t>동국생명과학</t>
+        </is>
+      </c>
+      <c r="D49" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E49" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F49" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G49" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H49" s="27" t="n">
+        <v>-9.06</v>
+      </c>
+      <c r="I49" s="29" t="n">
+        <v>20.52</v>
+      </c>
+      <c r="J49" s="28" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +295%</t>
+        </is>
+      </c>
+      <c r="K49" s="28" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
-      <c r="A50" s="20" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="B50" s="20" t="n">
+      <c r="A50" s="25" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B50" s="25" t="n">
         <v>37</v>
       </c>
-      <c r="C50" s="21" t="inlineStr">
-        <is>
-          <t>카카오페이</t>
-        </is>
-      </c>
-      <c r="D50" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E50" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F50" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G50" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H50" s="22" t="n">
-        <v>1.61</v>
-      </c>
-      <c r="I50" s="24" t="n">
-        <v>-10.59</v>
-      </c>
-      <c r="J50" s="23" t="inlineStr">
-        <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K50" s="23" t="n">
-        <v/>
+      <c r="C50" s="26" t="inlineStr">
+        <is>
+          <t>토마토시스템</t>
+        </is>
+      </c>
+      <c r="D50" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E50" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F50" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G50" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H50" s="29" t="n">
+        <v>12.07</v>
+      </c>
+      <c r="I50" s="29" t="n">
+        <v>65.84999999999999</v>
+      </c>
+      <c r="J50" s="28" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +214%</t>
+        </is>
+      </c>
+      <c r="K50" s="28" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B51" s="25" t="n">
@@ -2483,7 +2495,7 @@
       </c>
       <c r="C51" s="26" t="inlineStr">
         <is>
-          <t>네오사피엔스</t>
+          <t>케이쓰리아이</t>
         </is>
       </c>
       <c r="D51" s="25" t="n">
@@ -2498,27 +2510,27 @@
       <c r="G51" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H51" s="27" t="n">
-        <v>-19.24</v>
-      </c>
-      <c r="I51" s="27" t="n">
-        <v>-19.24</v>
+      <c r="H51" s="29" t="n">
+        <v>11.96</v>
+      </c>
+      <c r="I51" s="29" t="n">
+        <v>26.25</v>
       </c>
       <c r="J51" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +598%</t>
+          <t>중요공시 3건</t>
         </is>
       </c>
       <c r="K51" s="28" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B52" s="25" t="n">
@@ -2526,7 +2538,7 @@
       </c>
       <c r="C52" s="26" t="inlineStr">
         <is>
-          <t>엠케이전자</t>
+          <t>한화솔루션</t>
         </is>
       </c>
       <c r="D52" s="25" t="n">
@@ -2542,14 +2554,14 @@
         <v>0</v>
       </c>
       <c r="H52" s="29" t="n">
-        <v>7.26</v>
+        <v>6.52</v>
       </c>
       <c r="I52" s="29" t="n">
-        <v>23.23</v>
+        <v>2.62</v>
       </c>
       <c r="J52" s="28" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급</t>
+          <t>한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K52" s="28" t="n">
@@ -2559,7 +2571,7 @@
     <row r="53" ht="18" customHeight="1">
       <c r="A53" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B53" s="25" t="n">
@@ -2567,7 +2579,7 @@
       </c>
       <c r="C53" s="26" t="inlineStr">
         <is>
-          <t>노타</t>
+          <t>삼성E&amp;A</t>
         </is>
       </c>
       <c r="D53" s="25" t="n">
@@ -2582,25 +2594,27 @@
       <c r="G53" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H53" s="29" t="n">
-        <v>28.93</v>
-      </c>
-      <c r="I53" s="29" t="n">
-        <v>32.96</v>
+      <c r="H53" s="27" t="n">
+        <v>-3.31</v>
+      </c>
+      <c r="I53" s="27" t="n">
+        <v>-1.2</v>
       </c>
       <c r="J53" s="28" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K53" s="28" t="n">
-        <v/>
+          <t>중요공시 1건 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K53" s="28" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="54" ht="18" customHeight="1">
       <c r="A54" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B54" s="25" t="n">
@@ -2608,7 +2622,7 @@
       </c>
       <c r="C54" s="26" t="inlineStr">
         <is>
-          <t>대한항공</t>
+          <t>더코디</t>
         </is>
       </c>
       <c r="D54" s="25" t="n">
@@ -2624,24 +2638,26 @@
         <v>0</v>
       </c>
       <c r="H54" s="29" t="n">
-        <v>8.949999999999999</v>
-      </c>
-      <c r="I54" s="29" t="n">
-        <v>7.84</v>
+        <v>5.14</v>
+      </c>
+      <c r="I54" s="27" t="n">
+        <v>-40.85</v>
       </c>
       <c r="J54" s="28" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K54" s="28" t="n">
-        <v/>
+          <t>중요공시 8건</t>
+        </is>
+      </c>
+      <c r="K54" s="28" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="55" ht="18" customHeight="1">
       <c r="A55" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B55" s="25" t="n">
@@ -2664,11 +2680,11 @@
       <c r="G55" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H55" s="27" t="n">
-        <v>-2.41</v>
+      <c r="H55" s="29" t="n">
+        <v>0.41</v>
       </c>
       <c r="I55" s="27" t="n">
-        <v>-11.08</v>
+        <v>-5.05</v>
       </c>
       <c r="J55" s="28" t="inlineStr">
         <is>
@@ -2684,7 +2700,7 @@
     <row r="56" ht="18" customHeight="1">
       <c r="A56" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B56" s="25" t="n">
@@ -2692,7 +2708,7 @@
       </c>
       <c r="C56" s="26" t="inlineStr">
         <is>
-          <t>앤씨앤</t>
+          <t>비케이홀딩스</t>
         </is>
       </c>
       <c r="D56" s="25" t="n">
@@ -2708,14 +2724,14 @@
         <v>0</v>
       </c>
       <c r="H56" s="27" t="n">
-        <v>-12.5</v>
-      </c>
-      <c r="I56" s="29" t="n">
-        <v>31.15</v>
+        <v>-15.35</v>
+      </c>
+      <c r="I56" s="27" t="n">
+        <v>-17.21</v>
       </c>
       <c r="J56" s="28" t="inlineStr">
         <is>
-          <t>중요공시 4건</t>
+          <t>중요공시 3건</t>
         </is>
       </c>
       <c r="K56" s="28" t="inlineStr">
@@ -2727,7 +2743,7 @@
     <row r="57" ht="18" customHeight="1">
       <c r="A57" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B57" s="25" t="n">
@@ -2735,7 +2751,7 @@
       </c>
       <c r="C57" s="26" t="inlineStr">
         <is>
-          <t>한전산업</t>
+          <t>앤씨앤</t>
         </is>
       </c>
       <c r="D57" s="25" t="n">
@@ -2751,10 +2767,10 @@
         <v>0</v>
       </c>
       <c r="H57" s="29" t="n">
-        <v>0.54</v>
-      </c>
-      <c r="I57" s="27" t="n">
-        <v>-0.31</v>
+        <v>5.18</v>
+      </c>
+      <c r="I57" s="29" t="n">
+        <v>35.4</v>
       </c>
       <c r="J57" s="28" t="inlineStr">
         <is>
@@ -2770,7 +2786,7 @@
     <row r="58" ht="18" customHeight="1">
       <c r="A58" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B58" s="25" t="n">
@@ -2793,11 +2809,11 @@
       <c r="G58" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H58" s="25" t="n">
-        <v>0</v>
+      <c r="H58" s="27" t="n">
+        <v>-1.3</v>
       </c>
       <c r="I58" s="27" t="n">
-        <v>-1.5</v>
+        <v>-2.16</v>
       </c>
       <c r="J58" s="28" t="inlineStr">
         <is>
@@ -2813,7 +2829,7 @@
     <row r="59" ht="18" customHeight="1">
       <c r="A59" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B59" s="25" t="n">
@@ -2821,30 +2837,30 @@
       </c>
       <c r="C59" s="26" t="inlineStr">
         <is>
-          <t>파이온엑스</t>
+          <t>모아데이타</t>
         </is>
       </c>
       <c r="D59" s="25" t="n">
         <v>3</v>
       </c>
       <c r="E59" s="25" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F59" s="25" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G59" s="25" t="n">
         <v>0</v>
       </c>
       <c r="H59" s="27" t="n">
-        <v>-28.48</v>
+        <v>-2.38</v>
       </c>
       <c r="I59" s="27" t="n">
-        <v>-57.95</v>
+        <v>-13.38</v>
       </c>
       <c r="J59" s="28" t="inlineStr">
         <is>
-          <t>중요공시 3건</t>
+          <t>중요공시 2건 / 중요공시 3일 +100%</t>
         </is>
       </c>
       <c r="K59" s="28" t="inlineStr">
@@ -2856,7 +2872,7 @@
     <row r="60" ht="18" customHeight="1">
       <c r="A60" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B60" s="25" t="n">
@@ -2864,7 +2880,7 @@
       </c>
       <c r="C60" s="26" t="inlineStr">
         <is>
-          <t>모아데이타</t>
+          <t>삼일씨엔에스</t>
         </is>
       </c>
       <c r="D60" s="25" t="n">
@@ -2879,11 +2895,11 @@
       <c r="G60" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H60" s="27" t="n">
-        <v>-4.18</v>
-      </c>
-      <c r="I60" s="25" t="n">
-        <v>0</v>
+      <c r="H60" s="29" t="n">
+        <v>5.45</v>
+      </c>
+      <c r="I60" s="29" t="n">
+        <v>9.49</v>
       </c>
       <c r="J60" s="28" t="inlineStr">
         <is>
@@ -2899,7 +2915,7 @@
     <row r="61" ht="18" customHeight="1">
       <c r="A61" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B61" s="25" t="n">
@@ -2923,10 +2939,10 @@
         <v>0</v>
       </c>
       <c r="H61" s="27" t="n">
-        <v>-1.87</v>
+        <v>-0.11</v>
       </c>
       <c r="I61" s="29" t="n">
-        <v>0.17</v>
+        <v>0.39</v>
       </c>
       <c r="J61" s="28" t="inlineStr">
         <is>
@@ -2942,7 +2958,7 @@
     <row r="62" ht="18" customHeight="1">
       <c r="A62" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B62" s="25" t="n">
@@ -2950,30 +2966,30 @@
       </c>
       <c r="C62" s="26" t="inlineStr">
         <is>
-          <t>아이엘</t>
+          <t>현대로템</t>
         </is>
       </c>
       <c r="D62" s="25" t="n">
         <v>3</v>
       </c>
       <c r="E62" s="25" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F62" s="25" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G62" s="25" t="n">
         <v>0</v>
       </c>
       <c r="H62" s="27" t="n">
-        <v>-0.86</v>
-      </c>
-      <c r="I62" s="29" t="n">
-        <v>9.279999999999999</v>
+        <v>-1.19</v>
+      </c>
+      <c r="I62" s="27" t="n">
+        <v>-2.59</v>
       </c>
       <c r="J62" s="28" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 3일 +100%</t>
+          <t>중요공시 2건 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K62" s="28" t="inlineStr">
@@ -2985,7 +3001,7 @@
     <row r="63" ht="18" customHeight="1">
       <c r="A63" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B63" s="25" t="n">
@@ -2993,35 +3009,35 @@
       </c>
       <c r="C63" s="26" t="inlineStr">
         <is>
-          <t>삼성물산</t>
+          <t>삼성SDI</t>
         </is>
       </c>
       <c r="D63" s="25" t="n">
         <v>3</v>
       </c>
       <c r="E63" s="25" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F63" s="25" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G63" s="25" t="n">
         <v>0</v>
       </c>
       <c r="H63" s="27" t="n">
-        <v>-1.09</v>
-      </c>
-      <c r="I63" s="29" t="n">
-        <v>4.44</v>
+        <v>-1.88</v>
+      </c>
+      <c r="I63" s="27" t="n">
+        <v>-4.58</v>
       </c>
       <c r="J63" s="28" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 3일 +100%</t>
+          <t>네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K63" s="28" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
@@ -3118,22 +3134,22 @@
         <v>1</v>
       </c>
       <c r="C3" s="25" t="n">
-        <v>75</v>
+        <v>51</v>
       </c>
       <c r="D3" s="25" t="n">
-        <v>75</v>
+        <v>51</v>
       </c>
       <c r="E3" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F3" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G3" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="H3" s="25" t="n"/>
@@ -3142,143 +3158,139 @@
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="26" t="inlineStr">
         <is>
-          <t>원전</t>
+          <t>삼성전자</t>
         </is>
       </c>
       <c r="B4" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C4" s="25" t="n">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="D4" s="25" t="n">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="E4" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F4" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G4" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="H4" s="25" t="n"/>
-      <c r="I4" s="25" t="n"/>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="H4" s="29" t="n">
+        <v>3.24</v>
+      </c>
+      <c r="I4" s="29" t="n">
+        <v>13.02</v>
+      </c>
     </row>
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="26" t="inlineStr">
         <is>
-          <t>삼성전자</t>
+          <t>SK하이닉스</t>
         </is>
       </c>
       <c r="B5" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="25" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D5" s="25" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E5" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F5" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G5" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="H5" s="29" t="n">
-        <v>0.91</v>
+        <v>1.2</v>
       </c>
       <c r="I5" s="29" t="n">
-        <v>10.78</v>
+        <v>6.03</v>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="26" t="inlineStr">
         <is>
-          <t>LG</t>
+          <t>원전</t>
         </is>
       </c>
       <c r="B6" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="25" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D6" s="25" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E6" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F6" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G6" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="H6" s="29" t="n">
-        <v>3.66</v>
-      </c>
-      <c r="I6" s="29" t="n">
-        <v>2.38</v>
-      </c>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="H6" s="25" t="n"/>
+      <c r="I6" s="25" t="n"/>
     </row>
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="26" t="inlineStr">
         <is>
-          <t>SK하이닉스</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="B7" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="25" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D7" s="25" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E7" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F7" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G7" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="H7" s="27" t="n">
-        <v>-2.02</v>
-      </c>
-      <c r="I7" s="29" t="n">
-        <v>7.54</v>
-      </c>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="H7" s="25" t="n"/>
+      <c r="I7" s="25" t="n"/>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="26" t="inlineStr">
         <is>
-          <t>인공지능</t>
+          <t>LG전자</t>
         </is>
       </c>
       <c r="B8" s="25" t="n">
@@ -3295,219 +3307,235 @@
       </c>
       <c r="F8" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G8" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="H8" s="25" t="n"/>
-      <c r="I8" s="25" t="n"/>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="H8" s="27" t="n">
+        <v>-2.09</v>
+      </c>
+      <c r="I8" s="29" t="n">
+        <v>5.46</v>
+      </c>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="26" t="inlineStr">
         <is>
-          <t>셀리드</t>
+          <t>대한항공</t>
         </is>
       </c>
       <c r="B9" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="25" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D9" s="25" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E9" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F9" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G9" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="H9" s="29" t="n">
-        <v>14.94</v>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="H9" s="27" t="n">
+        <v>-0.47</v>
       </c>
       <c r="I9" s="29" t="n">
-        <v>24.62</v>
+        <v>7.69</v>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="26" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>삼성전기</t>
         </is>
       </c>
       <c r="B10" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C10" s="25" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D10" s="25" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E10" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F10" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G10" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="H10" s="25" t="n"/>
-      <c r="I10" s="25" t="n"/>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="H10" s="29" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="I10" s="29" t="n">
+        <v>9.4</v>
+      </c>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="26" t="inlineStr">
         <is>
-          <t>삼성전기</t>
+          <t>카카오</t>
         </is>
       </c>
       <c r="B11" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="25" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D11" s="25" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E11" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F11" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G11" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="H11" s="29" t="n">
-        <v>3.98</v>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="H11" s="27" t="n">
+        <v>-1.31</v>
       </c>
       <c r="I11" s="29" t="n">
-        <v>11.95</v>
+        <v>0.45</v>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="26" t="inlineStr">
         <is>
-          <t>카카오</t>
+          <t>HJ중공업</t>
         </is>
       </c>
       <c r="B12" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C12" s="25" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D12" s="25" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E12" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F12" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G12" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="H12" s="29" t="n">
-        <v>2.54</v>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="H12" s="27" t="n">
+        <v>-1.78</v>
       </c>
       <c r="I12" s="27" t="n">
-        <v>-1.3</v>
+        <v>-0.67</v>
       </c>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>태양광</t>
+          <t>셀리드</t>
         </is>
       </c>
       <c r="B13" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C13" s="25" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D13" s="25" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E13" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F13" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G13" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="H13" s="25" t="n"/>
-      <c r="I13" s="25" t="n"/>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="H13" s="27" t="n">
+        <v>-9.710000000000001</v>
+      </c>
+      <c r="I13" s="29" t="n">
+        <v>17.08</v>
+      </c>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>바이오</t>
+          <t>금호건설</t>
         </is>
       </c>
       <c r="B14" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C14" s="25" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D14" s="25" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E14" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F14" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G14" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="H14" s="25" t="n"/>
-      <c r="I14" s="25" t="n"/>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="H14" s="27" t="n">
+        <v>-1.73</v>
+      </c>
+      <c r="I14" s="27" t="n">
+        <v>-5.09</v>
+      </c>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>KT&amp;G</t>
+          <t>대우건설</t>
         </is>
       </c>
       <c r="B15" s="25" t="n">
@@ -3524,25 +3552,25 @@
       </c>
       <c r="F15" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G15" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="H15" s="29" t="n">
-        <v>1.56</v>
-      </c>
-      <c r="I15" s="29" t="n">
-        <v>3.46</v>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="H15" s="27" t="n">
+        <v>-6.4</v>
+      </c>
+      <c r="I15" s="27" t="n">
+        <v>-4.89</v>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>금호건설</t>
+          <t>바이오</t>
         </is>
       </c>
       <c r="B16" s="25" t="n">
@@ -3559,25 +3587,21 @@
       </c>
       <c r="F16" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G16" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="H16" s="27" t="n">
-        <v>-3.42</v>
-      </c>
-      <c r="I16" s="27" t="n">
-        <v>-1.78</v>
-      </c>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="H16" s="25" t="n"/>
+      <c r="I16" s="25" t="n"/>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>대우건설</t>
+          <t>스피어</t>
         </is>
       </c>
       <c r="B17" s="25" t="n">
@@ -3594,47 +3618,47 @@
       </c>
       <c r="F17" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G17" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="H17" s="29" t="n">
-        <v>2.33</v>
-      </c>
-      <c r="I17" s="27" t="n">
-        <v>-2.12</v>
+        <v>3.76</v>
+      </c>
+      <c r="I17" s="29" t="n">
+        <v>15.23</v>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="26" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>태양광</t>
         </is>
       </c>
       <c r="B18" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C18" s="25" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D18" s="25" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E18" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F18" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G18" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="H18" s="25" t="n"/>
@@ -3643,147 +3667,135 @@
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>GS건설</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B19" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C19" s="25" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D19" s="25" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E19" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F19" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G19" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="H19" s="29" t="n">
-        <v>1.9</v>
-      </c>
-      <c r="I19" s="27" t="n">
-        <v>-1.7</v>
-      </c>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="H19" s="25" t="n"/>
+      <c r="I19" s="25" t="n"/>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="26" t="inlineStr">
         <is>
-          <t>HJ중공업</t>
+          <t>방산</t>
         </is>
       </c>
       <c r="B20" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C20" s="25" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D20" s="25" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E20" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F20" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G20" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="H20" s="27" t="n">
-        <v>-0.72</v>
-      </c>
-      <c r="I20" s="27" t="n">
-        <v>-0.79</v>
-      </c>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="H20" s="25" t="n"/>
+      <c r="I20" s="25" t="n"/>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="26" t="inlineStr">
         <is>
-          <t>LG전자</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="B21" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C21" s="25" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D21" s="25" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E21" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F21" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G21" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="H21" s="29" t="n">
-        <v>5.91</v>
-      </c>
-      <c r="I21" s="29" t="n">
-        <v>6.44</v>
-      </c>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="H21" s="25" t="n"/>
+      <c r="I21" s="25" t="n"/>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="26" t="inlineStr">
         <is>
-          <t>더코디</t>
+          <t>한화시스템</t>
         </is>
       </c>
       <c r="B22" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C22" s="25" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D22" s="25" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E22" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F22" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G22" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="H22" s="27" t="n">
-        <v>-20.08</v>
-      </c>
-      <c r="I22" s="27" t="n">
-        <v>-40.46</v>
+        <v>-4.12</v>
+      </c>
+      <c r="I22" s="29" t="n">
+        <v>7.98</v>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="26" t="inlineStr">
         <is>
-          <t>비에이치아이</t>
+          <t>GS건설</t>
         </is>
       </c>
       <c r="B23" s="25" t="n">
@@ -3800,25 +3812,25 @@
       </c>
       <c r="F23" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G23" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="H23" s="29" t="n">
-        <v>3.22</v>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="H23" s="27" t="n">
+        <v>-7.33</v>
       </c>
       <c r="I23" s="27" t="n">
-        <v>-2.43</v>
+        <v>-5.57</v>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="26" t="inlineStr">
         <is>
-          <t>스테이블코인</t>
+          <t>대양금속</t>
         </is>
       </c>
       <c r="B24" s="25" t="n">
@@ -3835,21 +3847,25 @@
       </c>
       <c r="F24" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G24" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="H24" s="25" t="n"/>
-      <c r="I24" s="25" t="n"/>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="H24" s="27" t="n">
+        <v>-14.85</v>
+      </c>
+      <c r="I24" s="27" t="n">
+        <v>-11.08</v>
+      </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="26" t="inlineStr">
         <is>
-          <t>스피어</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="B25" s="25" t="n">
@@ -3866,25 +3882,21 @@
       </c>
       <c r="F25" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G25" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="H25" s="27" t="n">
-        <v>-3.62</v>
-      </c>
-      <c r="I25" s="29" t="n">
-        <v>12.16</v>
-      </c>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="H25" s="25" t="n"/>
+      <c r="I25" s="25" t="n"/>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="26" t="inlineStr">
         <is>
-          <t>우성머티리얼스</t>
+          <t>비에이치아이</t>
         </is>
       </c>
       <c r="B26" s="25" t="n">
@@ -3901,25 +3913,25 @@
       </c>
       <c r="F26" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G26" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="H26" s="29" t="n">
-        <v>11.39</v>
-      </c>
-      <c r="I26" s="29" t="n">
-        <v>12.08</v>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="H26" s="27" t="n">
+        <v>-5.76</v>
+      </c>
+      <c r="I26" s="27" t="n">
+        <v>-4.57</v>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="26" t="inlineStr">
         <is>
-          <t>현대차</t>
+          <t>삼성물산</t>
         </is>
       </c>
       <c r="B27" s="25" t="n">
@@ -3936,47 +3948,47 @@
       </c>
       <c r="F27" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G27" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="H27" s="29" t="n">
-        <v>0.14</v>
-      </c>
-      <c r="I27" s="27" t="n">
-        <v>-2.03</v>
+        <v>1.1</v>
+      </c>
+      <c r="I27" s="29" t="n">
+        <v>4.84</v>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="26" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>와이즈플래닛컴퍼니</t>
         </is>
       </c>
       <c r="B28" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C28" s="25" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D28" s="25" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E28" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F28" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G28" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="H28" s="25" t="n"/>
@@ -3985,7 +3997,7 @@
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="26" t="inlineStr">
         <is>
-          <t>우진</t>
+          <t>두산에너빌리티</t>
         </is>
       </c>
       <c r="B29" s="25" t="n">
@@ -4002,25 +4014,25 @@
       </c>
       <c r="F29" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G29" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="H29" s="27" t="n">
-        <v>-1.95</v>
+        <v>-4.5</v>
       </c>
       <c r="I29" s="27" t="n">
-        <v>-2.87</v>
+        <v>-1.66</v>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="26" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>우진</t>
         </is>
       </c>
       <c r="B30" s="25" t="n">
@@ -4037,21 +4049,25 @@
       </c>
       <c r="F30" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G30" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="H30" s="25" t="n"/>
-      <c r="I30" s="25" t="n"/>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="H30" s="27" t="n">
+        <v>-4.46</v>
+      </c>
+      <c r="I30" s="27" t="n">
+        <v>-2.59</v>
+      </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="26" t="inlineStr">
         <is>
-          <t>조선</t>
+          <t>포스코퓨처엠</t>
         </is>
       </c>
       <c r="B31" s="25" t="n">
@@ -4068,21 +4084,25 @@
       </c>
       <c r="F31" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G31" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="H31" s="25" t="n"/>
-      <c r="I31" s="25" t="n"/>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="H31" s="27" t="n">
+        <v>-2.96</v>
+      </c>
+      <c r="I31" s="27" t="n">
+        <v>-4.24</v>
+      </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="26" t="inlineStr">
         <is>
-          <t>광진실업</t>
+          <t>SG</t>
         </is>
       </c>
       <c r="B32" s="25" t="n">
@@ -4099,25 +4119,25 @@
       </c>
       <c r="F32" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G32" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="H32" s="27" t="n">
-        <v>-12.46</v>
-      </c>
-      <c r="I32" s="27" t="n">
-        <v>-18.87</v>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="H32" s="29" t="n">
+        <v>7.27</v>
+      </c>
+      <c r="I32" s="29" t="n">
+        <v>8.619999999999999</v>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="26" t="inlineStr">
         <is>
-          <t>디지털대성</t>
+          <t>노타</t>
         </is>
       </c>
       <c r="B33" s="25" t="n">
@@ -4134,25 +4154,25 @@
       </c>
       <c r="F33" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G33" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="H33" s="29" t="n">
-        <v>1.06</v>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="H33" s="27" t="n">
+        <v>-9.529999999999999</v>
       </c>
       <c r="I33" s="29" t="n">
-        <v>7.43</v>
+        <v>21.21</v>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="26" t="inlineStr">
         <is>
-          <t>방산</t>
+          <t>스테이블코인</t>
         </is>
       </c>
       <c r="B34" s="25" t="n">
@@ -4169,12 +4189,12 @@
       </c>
       <c r="F34" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G34" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="H34" s="25" t="n"/>
@@ -4183,182 +4203,182 @@
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="26" t="inlineStr">
         <is>
-          <t>성호전자</t>
+          <t>KB제34호스팩</t>
         </is>
       </c>
       <c r="B35" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C35" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D35" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E35" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F35" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G35" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="H35" s="27" t="n">
         <v>-0.37</v>
       </c>
-      <c r="I35" s="29" t="n">
-        <v>59.59</v>
+      <c r="I35" s="27" t="n">
+        <v>-0.37</v>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="26" t="inlineStr">
         <is>
-          <t>자이에스앤디</t>
+          <t>네오사피엔스</t>
         </is>
       </c>
       <c r="B36" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C36" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D36" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E36" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F36" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G36" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="H36" s="29" t="n">
-        <v>3.08</v>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="H36" s="27" t="n">
+        <v>-16.78</v>
       </c>
       <c r="I36" s="27" t="n">
-        <v>-8.720000000000001</v>
+        <v>-32.79</v>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="26" t="inlineStr">
         <is>
-          <t>카카오페이</t>
+          <t>넥사다이내믹스</t>
         </is>
       </c>
       <c r="B37" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C37" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D37" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E37" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F37" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G37" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="H37" s="29" t="n">
-        <v>1.61</v>
+        <v>0.41</v>
       </c>
       <c r="I37" s="27" t="n">
-        <v>-10.59</v>
+        <v>-5.05</v>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="26" t="inlineStr">
         <is>
-          <t>코리아써키트</t>
+          <t>더코디</t>
         </is>
       </c>
       <c r="B38" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C38" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D38" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E38" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F38" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G38" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="H38" s="29" t="n">
-        <v>25.52</v>
-      </c>
-      <c r="I38" s="29" t="n">
-        <v>32.53</v>
+        <v>5.14</v>
+      </c>
+      <c r="I38" s="27" t="n">
+        <v>-40.85</v>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="26" t="inlineStr">
         <is>
-          <t>핑거</t>
+          <t>동국생명과학</t>
         </is>
       </c>
       <c r="B39" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C39" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D39" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E39" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F39" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G39" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="H39" s="29" t="n">
-        <v>10.87</v>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="H39" s="27" t="n">
+        <v>-9.06</v>
       </c>
       <c r="I39" s="29" t="n">
-        <v>27.73</v>
+        <v>20.52</v>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="26" t="inlineStr">
         <is>
-          <t>네오사피엔스</t>
+          <t>모아데이타</t>
         </is>
       </c>
       <c r="B40" s="25" t="n">
@@ -4375,25 +4395,25 @@
       </c>
       <c r="F40" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G40" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="H40" s="27" t="n">
-        <v>-19.24</v>
+        <v>-2.38</v>
       </c>
       <c r="I40" s="27" t="n">
-        <v>-19.24</v>
+        <v>-13.38</v>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="26" t="inlineStr">
         <is>
-          <t>넥사다이내믹스</t>
+          <t>비케이홀딩스</t>
         </is>
       </c>
       <c r="B41" s="25" t="n">
@@ -4410,25 +4430,25 @@
       </c>
       <c r="F41" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G41" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="H41" s="27" t="n">
-        <v>-2.41</v>
+        <v>-15.35</v>
       </c>
       <c r="I41" s="27" t="n">
-        <v>-11.08</v>
+        <v>-17.21</v>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="26" t="inlineStr">
         <is>
-          <t>노타</t>
+          <t>삼성E&amp;A</t>
         </is>
       </c>
       <c r="B42" s="25" t="n">
@@ -4445,25 +4465,25 @@
       </c>
       <c r="F42" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G42" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="H42" s="29" t="n">
-        <v>28.93</v>
-      </c>
-      <c r="I42" s="29" t="n">
-        <v>32.96</v>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="H42" s="27" t="n">
+        <v>-3.31</v>
+      </c>
+      <c r="I42" s="27" t="n">
+        <v>-1.2</v>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="26" t="inlineStr">
         <is>
-          <t>대한항공</t>
+          <t>삼성SDI</t>
         </is>
       </c>
       <c r="B43" s="25" t="n">
@@ -4480,25 +4500,25 @@
       </c>
       <c r="F43" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G43" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="H43" s="29" t="n">
-        <v>8.949999999999999</v>
-      </c>
-      <c r="I43" s="29" t="n">
-        <v>7.84</v>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="H43" s="27" t="n">
+        <v>-1.88</v>
+      </c>
+      <c r="I43" s="27" t="n">
+        <v>-4.58</v>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="26" t="inlineStr">
         <is>
-          <t>모아데이타</t>
+          <t>삼일씨엔에스</t>
         </is>
       </c>
       <c r="B44" s="25" t="n">
@@ -4515,25 +4535,25 @@
       </c>
       <c r="F44" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G44" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="H44" s="27" t="n">
-        <v>-4.18</v>
-      </c>
-      <c r="I44" s="25" t="n">
-        <v>0</v>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="H44" s="29" t="n">
+        <v>5.45</v>
+      </c>
+      <c r="I44" s="29" t="n">
+        <v>9.49</v>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="26" t="inlineStr">
         <is>
-          <t>삼성물산</t>
+          <t>서희건설</t>
         </is>
       </c>
       <c r="B45" s="25" t="n">
@@ -4550,25 +4570,25 @@
       </c>
       <c r="F45" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G45" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="H45" s="27" t="n">
-        <v>-1.09</v>
-      </c>
-      <c r="I45" s="29" t="n">
-        <v>4.44</v>
+        <v>-1.3</v>
+      </c>
+      <c r="I45" s="27" t="n">
+        <v>-2.16</v>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="26" t="inlineStr">
         <is>
-          <t>서희건설</t>
+          <t>셀트리온</t>
         </is>
       </c>
       <c r="B46" s="25" t="n">
@@ -4585,25 +4605,25 @@
       </c>
       <c r="F46" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G46" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="H46" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="I46" s="27" t="n">
-        <v>-1.5</v>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="H46" s="27" t="n">
+        <v>-0.11</v>
+      </c>
+      <c r="I46" s="29" t="n">
+        <v>0.39</v>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="26" t="inlineStr">
         <is>
-          <t>셀트리온</t>
+          <t>앤씨앤</t>
         </is>
       </c>
       <c r="B47" s="25" t="n">
@@ -4620,25 +4640,25 @@
       </c>
       <c r="F47" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G47" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="H47" s="27" t="n">
-        <v>-1.87</v>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="H47" s="29" t="n">
+        <v>5.18</v>
       </c>
       <c r="I47" s="29" t="n">
-        <v>0.17</v>
+        <v>35.4</v>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="26" t="inlineStr">
         <is>
-          <t>아이엘</t>
+          <t>케이쓰리아이</t>
         </is>
       </c>
       <c r="B48" s="25" t="n">
@@ -4655,25 +4675,25 @@
       </c>
       <c r="F48" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G48" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="H48" s="27" t="n">
-        <v>-0.86</v>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="H48" s="29" t="n">
+        <v>11.96</v>
       </c>
       <c r="I48" s="29" t="n">
-        <v>9.279999999999999</v>
+        <v>26.25</v>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="26" t="inlineStr">
         <is>
-          <t>앤씨앤</t>
+          <t>토마토시스템</t>
         </is>
       </c>
       <c r="B49" s="25" t="n">
@@ -4690,25 +4710,25 @@
       </c>
       <c r="F49" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G49" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="H49" s="27" t="n">
-        <v>-12.5</v>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="H49" s="29" t="n">
+        <v>12.07</v>
       </c>
       <c r="I49" s="29" t="n">
-        <v>31.15</v>
+        <v>65.84999999999999</v>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="26" t="inlineStr">
         <is>
-          <t>엠케이전자</t>
+          <t>한국제17호스팩</t>
         </is>
       </c>
       <c r="B50" s="25" t="n">
@@ -4725,25 +4745,25 @@
       </c>
       <c r="F50" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G50" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="H50" s="29" t="n">
-        <v>7.26</v>
-      </c>
-      <c r="I50" s="29" t="n">
-        <v>23.23</v>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="H50" s="27" t="n">
+        <v>-1.91</v>
+      </c>
+      <c r="I50" s="27" t="n">
+        <v>-1.91</v>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="26" t="inlineStr">
         <is>
-          <t>파이온엑스</t>
+          <t>한화솔루션</t>
         </is>
       </c>
       <c r="B51" s="25" t="n">
@@ -4760,25 +4780,25 @@
       </c>
       <c r="F51" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G51" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="H51" s="27" t="n">
-        <v>-28.48</v>
-      </c>
-      <c r="I51" s="27" t="n">
-        <v>-57.95</v>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="H51" s="29" t="n">
+        <v>6.52</v>
+      </c>
+      <c r="I51" s="29" t="n">
+        <v>2.62</v>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="26" t="inlineStr">
         <is>
-          <t>한전산업</t>
+          <t>현대로템</t>
         </is>
       </c>
       <c r="B52" s="25" t="n">
@@ -4795,19 +4815,19 @@
       </c>
       <c r="F52" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G52" s="25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="H52" s="29" t="n">
-        <v>0.54</v>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="H52" s="27" t="n">
+        <v>-1.19</v>
       </c>
       <c r="I52" s="27" t="n">
-        <v>-0.31</v>
+        <v>-2.59</v>
       </c>
     </row>
   </sheetData>
@@ -4891,19 +4911,19 @@
         <v>1</v>
       </c>
       <c r="C3" s="36" t="n">
-        <v>75</v>
+        <v>51</v>
       </c>
       <c r="D3" s="36" t="n">
-        <v>75</v>
+        <v>51</v>
       </c>
       <c r="E3" s="36" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="F3" s="37" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G3" s="37" t="inlineStr">
@@ -4922,19 +4942,19 @@
         <v>1</v>
       </c>
       <c r="C4" s="36" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D4" s="36" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E4" s="36" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="F4" s="37" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G4" s="37" t="inlineStr">
@@ -4953,19 +4973,19 @@
         <v>1</v>
       </c>
       <c r="C5" s="36" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D5" s="36" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E5" s="36" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="F5" s="37" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G5" s="37" t="inlineStr">
@@ -4984,19 +5004,19 @@
         <v>1</v>
       </c>
       <c r="C6" s="36" t="n">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="D6" s="36" t="n">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="E6" s="36" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="F6" s="37" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G6" s="37" t="inlineStr">
@@ -5015,19 +5035,19 @@
         <v>1</v>
       </c>
       <c r="C7" s="36" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="D7" s="36" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="E7" s="36" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="F7" s="37" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G7" s="37" t="inlineStr">
@@ -5046,19 +5066,19 @@
         <v>1</v>
       </c>
       <c r="C8" s="36" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D8" s="36" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E8" s="36" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="F8" s="37" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G8" s="37" t="inlineStr">
@@ -5070,26 +5090,26 @@
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="35" t="inlineStr">
         <is>
-          <t>조선</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="B9" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="36" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D9" s="36" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E9" s="36" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="F9" s="37" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G9" s="37" t="inlineStr">
@@ -5101,26 +5121,26 @@
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="35" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="B10" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C10" s="36" t="n">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="D10" s="36" t="n">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="E10" s="36" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="F10" s="37" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G10" s="37" t="inlineStr">
@@ -5132,26 +5152,26 @@
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="35" t="inlineStr">
         <is>
-          <t>인공지능</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B11" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="36" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="D11" s="36" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E11" s="36" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="F11" s="37" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G11" s="37" t="inlineStr">
@@ -5161,40 +5181,36 @@
       </c>
     </row>
     <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="35" t="inlineStr">
-        <is>
-          <t>AMD</t>
-        </is>
-      </c>
-      <c r="B12" s="36" t="n">
-        <v>1</v>
-      </c>
-      <c r="C12" s="36" t="n">
-        <v>6</v>
-      </c>
-      <c r="D12" s="36" t="n">
-        <v>6</v>
-      </c>
-      <c r="E12" s="36" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="F12" s="37" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="G12" s="37" t="inlineStr">
-        <is>
-          <t>⚡ 관심</t>
-        </is>
-      </c>
+      <c r="A12" s="26" t="inlineStr">
+        <is>
+          <t>이차전지</t>
+        </is>
+      </c>
+      <c r="B12" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F12" s="28" t="inlineStr">
+        <is>
+          <t>감지 없음</t>
+        </is>
+      </c>
+      <c r="G12" s="28" t="inlineStr"/>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>이차전지</t>
+          <t>AI반도체</t>
         </is>
       </c>
       <c r="B13" s="25" t="n">
@@ -5221,7 +5237,7 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>AI반도체</t>
+          <t>전기차</t>
         </is>
       </c>
       <c r="B14" s="25" t="n">
@@ -5248,7 +5264,7 @@
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>전기차</t>
+          <t>수소</t>
         </is>
       </c>
       <c r="B15" s="25" t="n">
@@ -5275,7 +5291,7 @@
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>수소</t>
+          <t>게임</t>
         </is>
       </c>
       <c r="B16" s="25" t="n">
@@ -5302,7 +5318,7 @@
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>게임</t>
+          <t>엔터</t>
         </is>
       </c>
       <c r="B17" s="25" t="n">
@@ -5329,7 +5345,7 @@
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="26" t="inlineStr">
         <is>
-          <t>엔터</t>
+          <t>핀테크</t>
         </is>
       </c>
       <c r="B18" s="25" t="n">
@@ -5356,7 +5372,7 @@
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>핀테크</t>
+          <t>클라우드</t>
         </is>
       </c>
       <c r="B19" s="25" t="n">
@@ -5383,7 +5399,7 @@
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="26" t="inlineStr">
         <is>
-          <t>클라우드</t>
+          <t>조선</t>
         </is>
       </c>
       <c r="B20" s="25" t="n">

</xml_diff>

<commit_message>
auto: 2026-09-25 07:08 자동 백업
</commit_message>
<xml_diff>
--- a/trend/stock_trend_history.xlsx
+++ b/trend/stock_trend_history.xlsx
@@ -261,11 +261,11 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -694,7 +694,7 @@
     <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-09-24 06:54</t>
+          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-09-25 06:54</t>
         </is>
       </c>
     </row>
@@ -708,7 +708,7 @@
       </c>
       <c r="E3" s="3" t="n"/>
       <c r="G3" s="5" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="H3" s="3" t="n"/>
       <c r="J3" s="6" t="n">
@@ -787,21 +787,21 @@
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-09-24) 상위: 반도체  점수 51.0점</t>
+          <t>⚡ 최신(2026-09-25) 상위: 반도체  점수 47.0점</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-09-24) 상위: 삼성전자  점수 32.0점</t>
+          <t>⚡ 최신(2026-09-25) 상위: 삼성전자  점수 30.0점</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-09-24) 상위: SK하이닉스  점수 18.0점</t>
+          <t>⚡ 최신(2026-09-25) 상위: 제약  점수 15.0점</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="15" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B14" s="15" t="n">
@@ -928,10 +928,10 @@
         </is>
       </c>
       <c r="D14" s="15" t="n">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="E14" s="15" t="n">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F14" s="15" t="n">
         <v>0</v>
@@ -947,7 +947,7 @@
       </c>
       <c r="J14" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급</t>
+          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K14" s="17" t="inlineStr">
@@ -959,7 +959,7 @@
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="15" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B15" s="15" t="n">
@@ -971,10 +971,10 @@
         </is>
       </c>
       <c r="D15" s="15" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="E15" s="15" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="F15" s="15" t="n">
         <v>0</v>
@@ -990,7 +990,7 @@
       </c>
       <c r="J15" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K15" s="17" t="inlineStr">
@@ -1002,7 +1002,7 @@
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="15" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B16" s="15" t="n">
@@ -1010,14 +1010,14 @@
       </c>
       <c r="C16" s="16" t="inlineStr">
         <is>
-          <t>SK하이닉스</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="D16" s="15" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="E16" s="15" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="F16" s="15" t="n">
         <v>0</v>
@@ -1025,15 +1025,15 @@
       <c r="G16" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H16" s="18" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="I16" s="18" t="n">
-        <v>6.03</v>
+      <c r="H16" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I16" s="15" t="n">
+        <v/>
       </c>
       <c r="J16" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 기사 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K16" s="17" t="inlineStr">
@@ -1045,7 +1045,7 @@
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B17" s="15" t="n">
@@ -1053,14 +1053,14 @@
       </c>
       <c r="C17" s="16" t="inlineStr">
         <is>
-          <t>원전</t>
+          <t>LG전자</t>
         </is>
       </c>
       <c r="D17" s="15" t="n">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="E17" s="15" t="n">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="F17" s="15" t="n">
         <v>0</v>
@@ -1068,15 +1068,15 @@
       <c r="G17" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H17" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I17" s="15" t="n">
-        <v/>
+      <c r="H17" s="19" t="n">
+        <v>-2.09</v>
+      </c>
+      <c r="I17" s="18" t="n">
+        <v>5.46</v>
       </c>
       <c r="J17" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급</t>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K17" s="17" t="n">
@@ -1086,7 +1086,7 @@
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B18" s="15" t="n">
@@ -1094,14 +1094,14 @@
       </c>
       <c r="C18" s="16" t="inlineStr">
         <is>
-          <t>인공지능</t>
+          <t>바이오</t>
         </is>
       </c>
       <c r="D18" s="15" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="E18" s="15" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="F18" s="15" t="n">
         <v>0</v>
@@ -1117,7 +1117,7 @@
       </c>
       <c r="J18" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K18" s="17" t="inlineStr">
@@ -1129,7 +1129,7 @@
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B19" s="15" t="n">
@@ -1137,14 +1137,14 @@
       </c>
       <c r="C19" s="16" t="inlineStr">
         <is>
-          <t>대한항공</t>
+          <t>셀리드</t>
         </is>
       </c>
       <c r="D19" s="15" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E19" s="15" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F19" s="15" t="n">
         <v>0</v>
@@ -1153,24 +1153,26 @@
         <v>0</v>
       </c>
       <c r="H19" s="19" t="n">
-        <v>-0.47</v>
+        <v>-9.710000000000001</v>
       </c>
       <c r="I19" s="18" t="n">
-        <v>7.69</v>
+        <v>17.08</v>
       </c>
       <c r="J19" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K19" s="17" t="n">
-        <v/>
+          <t>네이버 검색 당일 +63% / 중요공시 4건 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K19" s="17" t="inlineStr">
+        <is>
+          <t>네이버, 공시</t>
+        </is>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B20" s="15" t="n">
@@ -1178,14 +1180,14 @@
       </c>
       <c r="C20" s="16" t="inlineStr">
         <is>
-          <t>LG전자</t>
+          <t>대한항공</t>
         </is>
       </c>
       <c r="D20" s="15" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E20" s="15" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F20" s="15" t="n">
         <v>0</v>
@@ -1194,14 +1196,14 @@
         <v>0</v>
       </c>
       <c r="H20" s="19" t="n">
-        <v>-2.09</v>
+        <v>-0.47</v>
       </c>
       <c r="I20" s="18" t="n">
-        <v>5.46</v>
+        <v>7.69</v>
       </c>
       <c r="J20" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K20" s="17" t="n">
@@ -1211,7 +1213,7 @@
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="15" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B21" s="15" t="n">
@@ -1219,14 +1221,14 @@
       </c>
       <c r="C21" s="16" t="inlineStr">
         <is>
-          <t>삼성전기</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="D21" s="15" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E21" s="15" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F21" s="15" t="n">
         <v>0</v>
@@ -1234,25 +1236,27 @@
       <c r="G21" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H21" s="18" t="n">
-        <v>0.8100000000000001</v>
-      </c>
-      <c r="I21" s="18" t="n">
-        <v>9.4</v>
+      <c r="H21" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I21" s="15" t="n">
+        <v/>
       </c>
       <c r="J21" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K21" s="17" t="n">
-        <v/>
+          <t>매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
+        </is>
+      </c>
+      <c r="K21" s="17" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="15" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B22" s="15" t="n">
@@ -1260,7 +1264,7 @@
       </c>
       <c r="C22" s="16" t="inlineStr">
         <is>
-          <t>카카오</t>
+          <t>원전</t>
         </is>
       </c>
       <c r="D22" s="15" t="n">
@@ -1275,15 +1279,15 @@
       <c r="G22" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H22" s="19" t="n">
-        <v>-1.31</v>
-      </c>
-      <c r="I22" s="18" t="n">
-        <v>0.45</v>
+      <c r="H22" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I22" s="15" t="n">
+        <v/>
       </c>
       <c r="J22" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K22" s="17" t="inlineStr">
@@ -1295,7 +1299,7 @@
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="15" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B23" s="15" t="n">
@@ -1303,7 +1307,7 @@
       </c>
       <c r="C23" s="16" t="inlineStr">
         <is>
-          <t>셀리드</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="D23" s="15" t="n">
@@ -1318,27 +1322,25 @@
       <c r="G23" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H23" s="19" t="n">
-        <v>-9.710000000000001</v>
-      </c>
-      <c r="I23" s="18" t="n">
-        <v>17.08</v>
+      <c r="H23" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I23" s="15" t="n">
+        <v/>
       </c>
       <c r="J23" s="17" t="inlineStr">
         <is>
-          <t>중요공시 4건 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K23" s="17" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K23" s="17" t="n">
+        <v/>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="15" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B24" s="15" t="n">
@@ -1346,42 +1348,40 @@
       </c>
       <c r="C24" s="16" t="inlineStr">
         <is>
-          <t>HJ중공업</t>
+          <t>SK하이닉스</t>
         </is>
       </c>
       <c r="D24" s="15" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E24" s="15" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F24" s="15" t="n">
         <v>0</v>
       </c>
       <c r="G24" s="15" t="n">
-        <v>3</v>
-      </c>
-      <c r="H24" s="19" t="n">
-        <v>-1.78</v>
-      </c>
-      <c r="I24" s="19" t="n">
-        <v>-0.67</v>
+        <v>0</v>
+      </c>
+      <c r="H24" s="18" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="I24" s="18" t="n">
+        <v>6.03</v>
       </c>
       <c r="J24" s="17" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 7일 +200% / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K24" s="17" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K24" s="17" t="n">
+        <v/>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="15" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B25" s="15" t="n">
@@ -1389,7 +1389,7 @@
       </c>
       <c r="C25" s="16" t="inlineStr">
         <is>
-          <t>대우건설</t>
+          <t>스피어</t>
         </is>
       </c>
       <c r="D25" s="15" t="n">
@@ -1404,15 +1404,15 @@
       <c r="G25" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="H25" s="19" t="n">
-        <v>-6.4</v>
-      </c>
-      <c r="I25" s="19" t="n">
-        <v>-4.89</v>
+      <c r="H25" s="18" t="n">
+        <v>3.76</v>
+      </c>
+      <c r="I25" s="18" t="n">
+        <v>15.23</v>
       </c>
       <c r="J25" s="17" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 3일 +50% / 중요공시 7일 +50%</t>
+          <t>중요공시 3건 / 중요공시 3일 +200% / 중요공시 7일 +200%</t>
         </is>
       </c>
       <c r="K25" s="17" t="inlineStr">
@@ -1424,7 +1424,7 @@
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="15" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B26" s="15" t="n">
@@ -1432,7 +1432,7 @@
       </c>
       <c r="C26" s="16" t="inlineStr">
         <is>
-          <t>스피어</t>
+          <t>금호건설</t>
         </is>
       </c>
       <c r="D26" s="15" t="n">
@@ -1447,15 +1447,15 @@
       <c r="G26" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="H26" s="18" t="n">
-        <v>3.76</v>
-      </c>
-      <c r="I26" s="18" t="n">
-        <v>15.23</v>
+      <c r="H26" s="19" t="n">
+        <v>-1.73</v>
+      </c>
+      <c r="I26" s="19" t="n">
+        <v>-5.09</v>
       </c>
       <c r="J26" s="17" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 3일 +200% / 중요공시 7일 +200%</t>
+          <t>중요공시 3건 / 중요공시 3일 +50% / 중요공시 7일 +50%</t>
         </is>
       </c>
       <c r="K26" s="17" t="inlineStr">
@@ -1467,7 +1467,7 @@
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="15" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B27" s="15" t="n">
@@ -1475,42 +1475,42 @@
       </c>
       <c r="C27" s="16" t="inlineStr">
         <is>
-          <t>금호건설</t>
+          <t>현대차</t>
         </is>
       </c>
       <c r="D27" s="15" t="n">
         <v>8</v>
       </c>
       <c r="E27" s="15" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="F27" s="15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G27" s="15" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H27" s="19" t="n">
-        <v>-1.73</v>
+        <v>-1.38</v>
       </c>
       <c r="I27" s="19" t="n">
-        <v>-5.09</v>
+        <v>-1.52</v>
       </c>
       <c r="J27" s="17" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 3일 +50% / 중요공시 7일 +50%</t>
+          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K27" s="17" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="15" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B28" s="15" t="n">
@@ -1518,14 +1518,14 @@
       </c>
       <c r="C28" s="16" t="inlineStr">
         <is>
-          <t>태양광</t>
+          <t>와이즈플래닛컴퍼니</t>
         </is>
       </c>
       <c r="D28" s="15" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E28" s="15" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F28" s="15" t="n">
         <v>0</v>
@@ -1541,7 +1541,7 @@
       </c>
       <c r="J28" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급</t>
+          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K28" s="17" t="n">
@@ -1551,7 +1551,7 @@
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="15" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B29" s="15" t="n">
@@ -1559,14 +1559,14 @@
       </c>
       <c r="C29" s="16" t="inlineStr">
         <is>
-          <t>바이오</t>
+          <t>GS</t>
         </is>
       </c>
       <c r="D29" s="15" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E29" s="15" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F29" s="15" t="n">
         <v>0</v>
@@ -1574,199 +1574,199 @@
       <c r="G29" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H29" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I29" s="15" t="n">
-        <v/>
+      <c r="H29" s="18" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="I29" s="19" t="n">
+        <v>-0.72</v>
       </c>
       <c r="J29" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급</t>
+          <t>Google 급상승 검색어 등장 (US) / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K29" s="17" t="inlineStr">
         <is>
+          <t>Google</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="18" customHeight="1">
+      <c r="A30" s="20" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B30" s="20" t="n">
+        <v>17</v>
+      </c>
+      <c r="C30" s="21" t="inlineStr">
+        <is>
+          <t>노타</t>
+        </is>
+      </c>
+      <c r="D30" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="E30" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="F30" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" s="22" t="n">
+        <v>-9.529999999999999</v>
+      </c>
+      <c r="I30" s="23" t="n">
+        <v>21.21</v>
+      </c>
+      <c r="J30" s="24" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +152% / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K30" s="24" t="inlineStr">
+        <is>
           <t>네이버</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="18" customHeight="1">
-      <c r="A30" s="15" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B30" s="15" t="n">
-        <v>17</v>
-      </c>
-      <c r="C30" s="16" t="inlineStr">
-        <is>
-          <t>한화시스템</t>
-        </is>
-      </c>
-      <c r="D30" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="E30" s="15" t="n">
-        <v>2</v>
-      </c>
-      <c r="F30" s="15" t="n">
-        <v>2</v>
-      </c>
-      <c r="G30" s="15" t="n">
-        <v>3</v>
-      </c>
-      <c r="H30" s="19" t="n">
-        <v>-4.12</v>
-      </c>
-      <c r="I30" s="18" t="n">
-        <v>7.98</v>
-      </c>
-      <c r="J30" s="17" t="inlineStr">
-        <is>
-          <t>중요공시 2건 / 중요공시 3일 +100% / 중요공시 7일 +100% / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K30" s="17" t="inlineStr">
+    <row r="31" ht="18" customHeight="1">
+      <c r="A31" s="20" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B31" s="20" t="n">
+        <v>18</v>
+      </c>
+      <c r="C31" s="21" t="inlineStr">
+        <is>
+          <t>GS건설</t>
+        </is>
+      </c>
+      <c r="D31" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="E31" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="F31" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="H31" s="22" t="n">
+        <v>-7.33</v>
+      </c>
+      <c r="I31" s="22" t="n">
+        <v>-5.57</v>
+      </c>
+      <c r="J31" s="24" t="inlineStr">
+        <is>
+          <t>중요공시 3건 / 중요공시 7일 +50%</t>
+        </is>
+      </c>
+      <c r="K31" s="24" t="inlineStr">
         <is>
           <t>공시</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="18" customHeight="1">
-      <c r="A31" s="15" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B31" s="15" t="n">
-        <v>18</v>
-      </c>
-      <c r="C31" s="16" t="inlineStr">
-        <is>
-          <t>AMD</t>
-        </is>
-      </c>
-      <c r="D31" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="E31" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="F31" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="G31" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H31" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I31" s="15" t="n">
-        <v/>
-      </c>
-      <c r="J31" s="17" t="inlineStr">
-        <is>
-          <t>네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K31" s="17" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
-      </c>
-    </row>
     <row r="32" ht="18" customHeight="1">
-      <c r="A32" s="15" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B32" s="15" t="n">
+      <c r="A32" s="20" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B32" s="20" t="n">
         <v>19</v>
       </c>
-      <c r="C32" s="16" t="inlineStr">
-        <is>
-          <t>방산</t>
-        </is>
-      </c>
-      <c r="D32" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="E32" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="F32" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="G32" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H32" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I32" s="15" t="n">
-        <v/>
-      </c>
-      <c r="J32" s="17" t="inlineStr">
-        <is>
-          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K32" s="17" t="inlineStr">
-        <is>
-          <t>네이버</t>
+      <c r="C32" s="21" t="inlineStr">
+        <is>
+          <t>HJ중공업</t>
+        </is>
+      </c>
+      <c r="D32" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="E32" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="F32" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H32" s="22" t="n">
+        <v>-1.78</v>
+      </c>
+      <c r="I32" s="22" t="n">
+        <v>-0.67</v>
+      </c>
+      <c r="J32" s="24" t="inlineStr">
+        <is>
+          <t>중요공시 3건 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K32" s="24" t="inlineStr">
+        <is>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
-      <c r="A33" s="15" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B33" s="15" t="n">
+      <c r="A33" s="20" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B33" s="20" t="n">
         <v>20</v>
       </c>
-      <c r="C33" s="16" t="inlineStr">
-        <is>
-          <t>제약</t>
-        </is>
-      </c>
-      <c r="D33" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="E33" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="F33" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="G33" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H33" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I33" s="15" t="n">
-        <v/>
-      </c>
-      <c r="J33" s="17" t="inlineStr">
-        <is>
-          <t>네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
-        </is>
-      </c>
-      <c r="K33" s="17" t="inlineStr">
-        <is>
-          <t>네이버</t>
+      <c r="C33" s="21" t="inlineStr">
+        <is>
+          <t>비케이홀딩스</t>
+        </is>
+      </c>
+      <c r="D33" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="E33" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="F33" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="H33" s="22" t="n">
+        <v>-15.35</v>
+      </c>
+      <c r="I33" s="22" t="n">
+        <v>-17.21</v>
+      </c>
+      <c r="J33" s="24" t="inlineStr">
+        <is>
+          <t>중요공시 3건 / 중요공시 7일 +200%</t>
+        </is>
+      </c>
+      <c r="K33" s="24" t="inlineStr">
+        <is>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="20" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B34" s="20" t="n">
@@ -1774,33 +1774,33 @@
       </c>
       <c r="C34" s="21" t="inlineStr">
         <is>
-          <t>대양금속</t>
+          <t>한화시스템</t>
         </is>
       </c>
       <c r="D34" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E34" s="20" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F34" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G34" s="20" t="n">
         <v>3</v>
       </c>
       <c r="H34" s="22" t="n">
-        <v>-14.85</v>
-      </c>
-      <c r="I34" s="22" t="n">
-        <v>-11.08</v>
-      </c>
-      <c r="J34" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 3건 / 중요공시 7일 +200%</t>
-        </is>
-      </c>
-      <c r="K34" s="23" t="inlineStr">
+        <v>-4.12</v>
+      </c>
+      <c r="I34" s="23" t="n">
+        <v>7.98</v>
+      </c>
+      <c r="J34" s="24" t="inlineStr">
+        <is>
+          <t>중요공시 2건 / 중요공시 3일 +100% / 중요공시 7일 +100%</t>
+        </is>
+      </c>
+      <c r="K34" s="24" t="inlineStr">
         <is>
           <t>공시</t>
         </is>
@@ -1809,7 +1809,7 @@
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="20" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B35" s="20" t="n">
@@ -1817,33 +1817,33 @@
       </c>
       <c r="C35" s="21" t="inlineStr">
         <is>
-          <t>GS건설</t>
+          <t>비에이치아이</t>
         </is>
       </c>
       <c r="D35" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E35" s="20" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F35" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G35" s="20" t="n">
         <v>3</v>
       </c>
       <c r="H35" s="22" t="n">
-        <v>-7.33</v>
+        <v>-5.76</v>
       </c>
       <c r="I35" s="22" t="n">
-        <v>-5.57</v>
-      </c>
-      <c r="J35" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 4건 / 중요공시 7일 +100%</t>
-        </is>
-      </c>
-      <c r="K35" s="23" t="inlineStr">
+        <v>-4.57</v>
+      </c>
+      <c r="J35" s="24" t="inlineStr">
+        <is>
+          <t>중요공시 2건 / 중요공시 3일 +100% / 중요공시 7일 +100%</t>
+        </is>
+      </c>
+      <c r="K35" s="24" t="inlineStr">
         <is>
           <t>공시</t>
         </is>
@@ -1852,7 +1852,7 @@
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="20" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B36" s="20" t="n">
@@ -1860,40 +1860,42 @@
       </c>
       <c r="C36" s="21" t="inlineStr">
         <is>
-          <t>와이즈플래닛컴퍼니</t>
+          <t>삼성물산</t>
         </is>
       </c>
       <c r="D36" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E36" s="20" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F36" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G36" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H36" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I36" s="20" t="n">
-        <v/>
-      </c>
-      <c r="J36" s="23" t="inlineStr">
-        <is>
-          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K36" s="23" t="n">
-        <v/>
+      <c r="H36" s="23" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="I36" s="23" t="n">
+        <v>4.84</v>
+      </c>
+      <c r="J36" s="24" t="inlineStr">
+        <is>
+          <t>중요공시 2건 / 중요공시 3일 +100% / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K36" s="24" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="20" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B37" s="20" t="n">
@@ -1901,33 +1903,33 @@
       </c>
       <c r="C37" s="21" t="inlineStr">
         <is>
-          <t>비에이치아이</t>
+          <t>포스코퓨처엠</t>
         </is>
       </c>
       <c r="D37" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E37" s="20" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F37" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G37" s="20" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H37" s="22" t="n">
-        <v>-5.76</v>
+        <v>-2.96</v>
       </c>
       <c r="I37" s="22" t="n">
-        <v>-4.57</v>
-      </c>
-      <c r="J37" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 2건 / 중요공시 3일 +100% / 중요공시 7일 +100%</t>
-        </is>
-      </c>
-      <c r="K37" s="23" t="inlineStr">
+        <v>-4.24</v>
+      </c>
+      <c r="J37" s="24" t="inlineStr">
+        <is>
+          <t>중요공시 1건 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K37" s="24" t="inlineStr">
         <is>
           <t>공시</t>
         </is>
@@ -1936,7 +1938,7 @@
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="20" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B38" s="20" t="n">
@@ -1944,42 +1946,40 @@
       </c>
       <c r="C38" s="21" t="inlineStr">
         <is>
-          <t>삼성물산</t>
+          <t>카카오</t>
         </is>
       </c>
       <c r="D38" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E38" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F38" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G38" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H38" s="24" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="I38" s="24" t="n">
-        <v>4.84</v>
-      </c>
-      <c r="J38" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 2건 / 중요공시 3일 +100% / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K38" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+      <c r="H38" s="22" t="n">
+        <v>-1.31</v>
+      </c>
+      <c r="I38" s="23" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="J38" s="24" t="inlineStr">
+        <is>
+          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K38" s="24" t="n">
+        <v/>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="20" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B39" s="20" t="n">
@@ -1987,14 +1987,14 @@
       </c>
       <c r="C39" s="21" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>디에이테크놀로지</t>
         </is>
       </c>
       <c r="D39" s="20" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E39" s="20" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F39" s="20" t="n">
         <v>0</v>
@@ -2002,25 +2002,27 @@
       <c r="G39" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H39" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I39" s="20" t="n">
-        <v/>
-      </c>
-      <c r="J39" s="23" t="inlineStr">
-        <is>
-          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K39" s="23" t="n">
-        <v/>
+      <c r="H39" s="22" t="n">
+        <v>-96.68000000000001</v>
+      </c>
+      <c r="I39" s="22" t="n">
+        <v>-96.68000000000001</v>
+      </c>
+      <c r="J39" s="24" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +533% / 중요공시 2건</t>
+        </is>
+      </c>
+      <c r="K39" s="24" t="inlineStr">
+        <is>
+          <t>네이버, 공시</t>
+        </is>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="20" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B40" s="20" t="n">
@@ -2028,14 +2030,14 @@
       </c>
       <c r="C40" s="21" t="inlineStr">
         <is>
-          <t>두산에너빌리티</t>
+          <t>대양금속</t>
         </is>
       </c>
       <c r="D40" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E40" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F40" s="20" t="n">
         <v>0</v>
@@ -2044,26 +2046,26 @@
         <v>0</v>
       </c>
       <c r="H40" s="22" t="n">
-        <v>-4.5</v>
+        <v>-14.85</v>
       </c>
       <c r="I40" s="22" t="n">
-        <v>-1.66</v>
-      </c>
-      <c r="J40" s="23" t="inlineStr">
-        <is>
-          <t>Google 급상승 검색어 등장 (KR)</t>
-        </is>
-      </c>
-      <c r="K40" s="23" t="inlineStr">
-        <is>
-          <t>Google</t>
+        <v>-11.08</v>
+      </c>
+      <c r="J40" s="24" t="inlineStr">
+        <is>
+          <t>중요공시 3건</t>
+        </is>
+      </c>
+      <c r="K40" s="24" t="inlineStr">
+        <is>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="20" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B41" s="20" t="n">
@@ -2071,33 +2073,33 @@
       </c>
       <c r="C41" s="21" t="inlineStr">
         <is>
-          <t>우진</t>
+          <t>케이쓰리아이</t>
         </is>
       </c>
       <c r="D41" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E41" s="20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F41" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G41" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H41" s="22" t="n">
-        <v>-4.46</v>
-      </c>
-      <c r="I41" s="22" t="n">
-        <v>-2.59</v>
-      </c>
-      <c r="J41" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 3건 / 중요공시 3일 +50%</t>
-        </is>
-      </c>
-      <c r="K41" s="23" t="inlineStr">
+      <c r="H41" s="23" t="n">
+        <v>11.96</v>
+      </c>
+      <c r="I41" s="23" t="n">
+        <v>26.25</v>
+      </c>
+      <c r="J41" s="24" t="inlineStr">
+        <is>
+          <t>중요공시 3건</t>
+        </is>
+      </c>
+      <c r="K41" s="24" t="inlineStr">
         <is>
           <t>공시</t>
         </is>
@@ -2106,7 +2108,7 @@
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="20" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B42" s="20" t="n">
@@ -2114,14 +2116,14 @@
       </c>
       <c r="C42" s="21" t="inlineStr">
         <is>
-          <t>포스코퓨처엠</t>
+          <t>우리기술</t>
         </is>
       </c>
       <c r="D42" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E42" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F42" s="20" t="n">
         <v>0</v>
@@ -2130,26 +2132,26 @@
         <v>0</v>
       </c>
       <c r="H42" s="22" t="n">
-        <v>-2.96</v>
-      </c>
-      <c r="I42" s="22" t="n">
-        <v>-4.24</v>
-      </c>
-      <c r="J42" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 1건 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K42" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
+        <v>-3.35</v>
+      </c>
+      <c r="I42" s="23" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="J42" s="24" t="inlineStr">
+        <is>
+          <t>중요공시 2건 / 네이버뉴스 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K42" s="24" t="inlineStr">
+        <is>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="20" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B43" s="20" t="n">
@@ -2157,7 +2159,7 @@
       </c>
       <c r="C43" s="21" t="inlineStr">
         <is>
-          <t>노타</t>
+          <t>삼성제약</t>
         </is>
       </c>
       <c r="D43" s="20" t="n">
@@ -2173,24 +2175,26 @@
         <v>0</v>
       </c>
       <c r="H43" s="22" t="n">
-        <v>-9.529999999999999</v>
-      </c>
-      <c r="I43" s="24" t="n">
-        <v>21.21</v>
-      </c>
-      <c r="J43" s="23" t="inlineStr">
-        <is>
-          <t>매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K43" s="23" t="n">
-        <v/>
+        <v>-2.66</v>
+      </c>
+      <c r="I43" s="22" t="n">
+        <v>-8.380000000000001</v>
+      </c>
+      <c r="J43" s="24" t="inlineStr">
+        <is>
+          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K43" s="24" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="20" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B44" s="20" t="n">
@@ -2198,7 +2202,7 @@
       </c>
       <c r="C44" s="21" t="inlineStr">
         <is>
-          <t>SG</t>
+          <t>삼성전기</t>
         </is>
       </c>
       <c r="D44" s="20" t="n">
@@ -2213,25 +2217,25 @@
       <c r="G44" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H44" s="24" t="n">
-        <v>7.27</v>
-      </c>
-      <c r="I44" s="24" t="n">
-        <v>8.619999999999999</v>
-      </c>
-      <c r="J44" s="23" t="inlineStr">
-        <is>
-          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K44" s="23" t="n">
+      <c r="H44" s="23" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="I44" s="23" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="J44" s="24" t="inlineStr">
+        <is>
+          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K44" s="24" t="n">
         <v/>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="20" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B45" s="20" t="n">
@@ -2239,7 +2243,7 @@
       </c>
       <c r="C45" s="21" t="inlineStr">
         <is>
-          <t>스테이블코인</t>
+          <t>방산</t>
         </is>
       </c>
       <c r="D45" s="20" t="n">
@@ -2260,148 +2264,144 @@
       <c r="I45" s="20" t="n">
         <v/>
       </c>
-      <c r="J45" s="23" t="inlineStr">
+      <c r="J45" s="24" t="inlineStr">
+        <is>
+          <t>매일경제 기사 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K45" s="24" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="46" ht="18" customHeight="1">
+      <c r="A46" s="20" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B46" s="20" t="n">
+        <v>33</v>
+      </c>
+      <c r="C46" s="21" t="inlineStr">
+        <is>
+          <t>태양광</t>
+        </is>
+      </c>
+      <c r="D46" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="E46" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F46" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G46" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H46" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I46" s="20" t="n">
+        <v/>
+      </c>
+      <c r="J46" s="24" t="inlineStr">
+        <is>
+          <t>매일경제 기사 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K46" s="24" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="47" ht="18" customHeight="1">
+      <c r="A47" s="20" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B47" s="20" t="n">
+        <v>34</v>
+      </c>
+      <c r="C47" s="21" t="inlineStr">
+        <is>
+          <t>테스</t>
+        </is>
+      </c>
+      <c r="D47" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="E47" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F47" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H47" s="23" t="n">
+        <v>8.949999999999999</v>
+      </c>
+      <c r="I47" s="23" t="n">
+        <v>19.31</v>
+      </c>
+      <c r="J47" s="24" t="inlineStr">
+        <is>
+          <t>매일경제 헤드라인 언급 / 네이버뉴스 기사 언급</t>
+        </is>
+      </c>
+      <c r="K47" s="24" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="18" customHeight="1">
+      <c r="A48" s="20" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B48" s="20" t="n">
+        <v>35</v>
+      </c>
+      <c r="C48" s="21" t="inlineStr">
+        <is>
+          <t>스테이블코인</t>
+        </is>
+      </c>
+      <c r="D48" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="E48" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F48" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G48" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H48" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I48" s="20" t="n">
+        <v/>
+      </c>
+      <c r="J48" s="24" t="inlineStr">
         <is>
           <t>한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
-      <c r="K45" s="23" t="n">
+      <c r="K48" s="24" t="n">
         <v/>
-      </c>
-    </row>
-    <row r="46" ht="18" customHeight="1">
-      <c r="A46" s="25" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B46" s="25" t="n">
-        <v>33</v>
-      </c>
-      <c r="C46" s="26" t="inlineStr">
-        <is>
-          <t>한국제17호스팩</t>
-        </is>
-      </c>
-      <c r="D46" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="E46" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="F46" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="G46" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H46" s="27" t="n">
-        <v>-1.91</v>
-      </c>
-      <c r="I46" s="27" t="n">
-        <v>-1.91</v>
-      </c>
-      <c r="J46" s="28" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +4057%</t>
-        </is>
-      </c>
-      <c r="K46" s="28" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="18" customHeight="1">
-      <c r="A47" s="25" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B47" s="25" t="n">
-        <v>34</v>
-      </c>
-      <c r="C47" s="26" t="inlineStr">
-        <is>
-          <t>KB제34호스팩</t>
-        </is>
-      </c>
-      <c r="D47" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="E47" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="F47" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="G47" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H47" s="27" t="n">
-        <v>-0.37</v>
-      </c>
-      <c r="I47" s="27" t="n">
-        <v>-0.37</v>
-      </c>
-      <c r="J47" s="28" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +2698%</t>
-        </is>
-      </c>
-      <c r="K47" s="28" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="18" customHeight="1">
-      <c r="A48" s="25" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="B48" s="25" t="n">
-        <v>35</v>
-      </c>
-      <c r="C48" s="26" t="inlineStr">
-        <is>
-          <t>네오사피엔스</t>
-        </is>
-      </c>
-      <c r="D48" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="E48" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="F48" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="G48" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H48" s="27" t="n">
-        <v>-16.78</v>
-      </c>
-      <c r="I48" s="27" t="n">
-        <v>-32.79</v>
-      </c>
-      <c r="J48" s="28" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +810%</t>
-        </is>
-      </c>
-      <c r="K48" s="28" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B49" s="25" t="n">
@@ -2409,7 +2409,7 @@
       </c>
       <c r="C49" s="26" t="inlineStr">
         <is>
-          <t>동국생명과학</t>
+          <t>한국제17호스팩</t>
         </is>
       </c>
       <c r="D49" s="25" t="n">
@@ -2425,14 +2425,14 @@
         <v>0</v>
       </c>
       <c r="H49" s="27" t="n">
-        <v>-9.06</v>
-      </c>
-      <c r="I49" s="29" t="n">
-        <v>20.52</v>
+        <v>-1.91</v>
+      </c>
+      <c r="I49" s="27" t="n">
+        <v>-1.91</v>
       </c>
       <c r="J49" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +295%</t>
+          <t>네이버 검색 당일 +4633%</t>
         </is>
       </c>
       <c r="K49" s="28" t="inlineStr">
@@ -2444,7 +2444,7 @@
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B50" s="25" t="n">
@@ -2452,7 +2452,7 @@
       </c>
       <c r="C50" s="26" t="inlineStr">
         <is>
-          <t>토마토시스템</t>
+          <t>KB제34호스팩</t>
         </is>
       </c>
       <c r="D50" s="25" t="n">
@@ -2467,15 +2467,15 @@
       <c r="G50" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H50" s="29" t="n">
-        <v>12.07</v>
-      </c>
-      <c r="I50" s="29" t="n">
-        <v>65.84999999999999</v>
+      <c r="H50" s="27" t="n">
+        <v>-0.37</v>
+      </c>
+      <c r="I50" s="27" t="n">
+        <v>-0.37</v>
       </c>
       <c r="J50" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +214%</t>
+          <t>네이버 검색 당일 +3094%</t>
         </is>
       </c>
       <c r="K50" s="28" t="inlineStr">
@@ -2487,7 +2487,7 @@
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B51" s="25" t="n">
@@ -2495,7 +2495,7 @@
       </c>
       <c r="C51" s="26" t="inlineStr">
         <is>
-          <t>케이쓰리아이</t>
+          <t>네오사피엔스</t>
         </is>
       </c>
       <c r="D51" s="25" t="n">
@@ -2510,27 +2510,27 @@
       <c r="G51" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H51" s="29" t="n">
-        <v>11.96</v>
-      </c>
-      <c r="I51" s="29" t="n">
-        <v>26.25</v>
+      <c r="H51" s="27" t="n">
+        <v>-16.78</v>
+      </c>
+      <c r="I51" s="27" t="n">
+        <v>-32.79</v>
       </c>
       <c r="J51" s="28" t="inlineStr">
         <is>
-          <t>중요공시 3건</t>
+          <t>네이버 검색 당일 +930%</t>
         </is>
       </c>
       <c r="K51" s="28" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B52" s="25" t="n">
@@ -2538,7 +2538,7 @@
       </c>
       <c r="C52" s="26" t="inlineStr">
         <is>
-          <t>한화솔루션</t>
+          <t>동국생명과학</t>
         </is>
       </c>
       <c r="D52" s="25" t="n">
@@ -2553,25 +2553,27 @@
       <c r="G52" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H52" s="29" t="n">
-        <v>6.52</v>
+      <c r="H52" s="27" t="n">
+        <v>-9.06</v>
       </c>
       <c r="I52" s="29" t="n">
-        <v>2.62</v>
+        <v>20.52</v>
       </c>
       <c r="J52" s="28" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K52" s="28" t="n">
-        <v/>
+          <t>네이버 검색 당일 +554%</t>
+        </is>
+      </c>
+      <c r="K52" s="28" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="53" ht="18" customHeight="1">
       <c r="A53" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B53" s="25" t="n">
@@ -2579,7 +2581,7 @@
       </c>
       <c r="C53" s="26" t="inlineStr">
         <is>
-          <t>삼성E&amp;A</t>
+          <t>토마토시스템</t>
         </is>
       </c>
       <c r="D53" s="25" t="n">
@@ -2594,27 +2596,27 @@
       <c r="G53" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H53" s="27" t="n">
-        <v>-3.31</v>
-      </c>
-      <c r="I53" s="27" t="n">
-        <v>-1.2</v>
+      <c r="H53" s="29" t="n">
+        <v>12.07</v>
+      </c>
+      <c r="I53" s="29" t="n">
+        <v>65.84999999999999</v>
       </c>
       <c r="J53" s="28" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 한국경제 헤드라인 언급</t>
+          <t>네이버 검색 당일 +477%</t>
         </is>
       </c>
       <c r="K53" s="28" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="54" ht="18" customHeight="1">
       <c r="A54" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B54" s="25" t="n">
@@ -2622,7 +2624,7 @@
       </c>
       <c r="C54" s="26" t="inlineStr">
         <is>
-          <t>더코디</t>
+          <t>삼기에너지솔루션즈</t>
         </is>
       </c>
       <c r="D54" s="25" t="n">
@@ -2638,26 +2640,26 @@
         <v>0</v>
       </c>
       <c r="H54" s="29" t="n">
-        <v>5.14</v>
-      </c>
-      <c r="I54" s="27" t="n">
-        <v>-40.85</v>
+        <v>18.12</v>
+      </c>
+      <c r="I54" s="29" t="n">
+        <v>21.39</v>
       </c>
       <c r="J54" s="28" t="inlineStr">
         <is>
-          <t>중요공시 8건</t>
+          <t>네이버 검색 당일 +130%</t>
         </is>
       </c>
       <c r="K54" s="28" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="55" ht="18" customHeight="1">
       <c r="A55" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B55" s="25" t="n">
@@ -2665,7 +2667,7 @@
       </c>
       <c r="C55" s="26" t="inlineStr">
         <is>
-          <t>넥사다이내믹스</t>
+          <t>두산에너빌리티</t>
         </is>
       </c>
       <c r="D55" s="25" t="n">
@@ -2680,27 +2682,27 @@
       <c r="G55" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H55" s="29" t="n">
-        <v>0.41</v>
+      <c r="H55" s="27" t="n">
+        <v>-4.5</v>
       </c>
       <c r="I55" s="27" t="n">
-        <v>-5.05</v>
+        <v>-1.66</v>
       </c>
       <c r="J55" s="28" t="inlineStr">
         <is>
-          <t>중요공시 5건</t>
+          <t>네이버뉴스 헤드라인 언급</t>
         </is>
       </c>
       <c r="K55" s="28" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="56" ht="18" customHeight="1">
       <c r="A56" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B56" s="25" t="n">
@@ -2708,7 +2710,7 @@
       </c>
       <c r="C56" s="26" t="inlineStr">
         <is>
-          <t>비케이홀딩스</t>
+          <t>한화솔루션</t>
         </is>
       </c>
       <c r="D56" s="25" t="n">
@@ -2723,27 +2725,25 @@
       <c r="G56" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H56" s="27" t="n">
-        <v>-15.35</v>
-      </c>
-      <c r="I56" s="27" t="n">
-        <v>-17.21</v>
+      <c r="H56" s="29" t="n">
+        <v>6.52</v>
+      </c>
+      <c r="I56" s="29" t="n">
+        <v>2.62</v>
       </c>
       <c r="J56" s="28" t="inlineStr">
         <is>
-          <t>중요공시 3건</t>
-        </is>
-      </c>
-      <c r="K56" s="28" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K56" s="28" t="n">
+        <v/>
       </c>
     </row>
     <row r="57" ht="18" customHeight="1">
       <c r="A57" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B57" s="25" t="n">
@@ -2751,7 +2751,7 @@
       </c>
       <c r="C57" s="26" t="inlineStr">
         <is>
-          <t>앤씨앤</t>
+          <t>삼성E&amp;A</t>
         </is>
       </c>
       <c r="D57" s="25" t="n">
@@ -2766,15 +2766,15 @@
       <c r="G57" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H57" s="29" t="n">
-        <v>5.18</v>
-      </c>
-      <c r="I57" s="29" t="n">
-        <v>35.4</v>
+      <c r="H57" s="27" t="n">
+        <v>-3.31</v>
+      </c>
+      <c r="I57" s="27" t="n">
+        <v>-1.2</v>
       </c>
       <c r="J57" s="28" t="inlineStr">
         <is>
-          <t>중요공시 3건</t>
+          <t>중요공시 1건 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K57" s="28" t="inlineStr">
@@ -2786,7 +2786,7 @@
     <row r="58" ht="18" customHeight="1">
       <c r="A58" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B58" s="25" t="n">
@@ -2794,7 +2794,7 @@
       </c>
       <c r="C58" s="26" t="inlineStr">
         <is>
-          <t>서희건설</t>
+          <t>더코디</t>
         </is>
       </c>
       <c r="D58" s="25" t="n">
@@ -2809,15 +2809,15 @@
       <c r="G58" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H58" s="27" t="n">
-        <v>-1.3</v>
+      <c r="H58" s="29" t="n">
+        <v>5.14</v>
       </c>
       <c r="I58" s="27" t="n">
-        <v>-2.16</v>
+        <v>-40.85</v>
       </c>
       <c r="J58" s="28" t="inlineStr">
         <is>
-          <t>중요공시 3건</t>
+          <t>중요공시 6건</t>
         </is>
       </c>
       <c r="K58" s="28" t="inlineStr">
@@ -2829,7 +2829,7 @@
     <row r="59" ht="18" customHeight="1">
       <c r="A59" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B59" s="25" t="n">
@@ -2837,30 +2837,30 @@
       </c>
       <c r="C59" s="26" t="inlineStr">
         <is>
-          <t>모아데이타</t>
+          <t>넥사다이내믹스</t>
         </is>
       </c>
       <c r="D59" s="25" t="n">
         <v>3</v>
       </c>
       <c r="E59" s="25" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F59" s="25" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G59" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H59" s="27" t="n">
-        <v>-2.38</v>
+      <c r="H59" s="29" t="n">
+        <v>0.41</v>
       </c>
       <c r="I59" s="27" t="n">
-        <v>-13.38</v>
+        <v>-5.05</v>
       </c>
       <c r="J59" s="28" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 3일 +100%</t>
+          <t>중요공시 5건</t>
         </is>
       </c>
       <c r="K59" s="28" t="inlineStr">
@@ -2872,7 +2872,7 @@
     <row r="60" ht="18" customHeight="1">
       <c r="A60" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B60" s="25" t="n">
@@ -2880,30 +2880,30 @@
       </c>
       <c r="C60" s="26" t="inlineStr">
         <is>
-          <t>삼일씨엔에스</t>
+          <t>앤씨앤</t>
         </is>
       </c>
       <c r="D60" s="25" t="n">
         <v>3</v>
       </c>
       <c r="E60" s="25" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F60" s="25" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G60" s="25" t="n">
         <v>0</v>
       </c>
       <c r="H60" s="29" t="n">
-        <v>5.45</v>
+        <v>5.18</v>
       </c>
       <c r="I60" s="29" t="n">
-        <v>9.49</v>
+        <v>35.4</v>
       </c>
       <c r="J60" s="28" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 3일 +100%</t>
+          <t>중요공시 3건</t>
         </is>
       </c>
       <c r="K60" s="28" t="inlineStr">
@@ -2915,7 +2915,7 @@
     <row r="61" ht="18" customHeight="1">
       <c r="A61" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B61" s="25" t="n">
@@ -2923,30 +2923,30 @@
       </c>
       <c r="C61" s="26" t="inlineStr">
         <is>
-          <t>셀트리온</t>
+          <t>서희건설</t>
         </is>
       </c>
       <c r="D61" s="25" t="n">
         <v>3</v>
       </c>
       <c r="E61" s="25" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F61" s="25" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G61" s="25" t="n">
         <v>0</v>
       </c>
       <c r="H61" s="27" t="n">
-        <v>-0.11</v>
-      </c>
-      <c r="I61" s="29" t="n">
-        <v>0.39</v>
+        <v>-1.3</v>
+      </c>
+      <c r="I61" s="27" t="n">
+        <v>-2.16</v>
       </c>
       <c r="J61" s="28" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 3일 +100%</t>
+          <t>중요공시 3건</t>
         </is>
       </c>
       <c r="K61" s="28" t="inlineStr">
@@ -2958,7 +2958,7 @@
     <row r="62" ht="18" customHeight="1">
       <c r="A62" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B62" s="25" t="n">
@@ -2966,30 +2966,30 @@
       </c>
       <c r="C62" s="26" t="inlineStr">
         <is>
-          <t>현대로템</t>
+          <t>모아데이타</t>
         </is>
       </c>
       <c r="D62" s="25" t="n">
         <v>3</v>
       </c>
       <c r="E62" s="25" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F62" s="25" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G62" s="25" t="n">
         <v>0</v>
       </c>
       <c r="H62" s="27" t="n">
-        <v>-1.19</v>
+        <v>-2.38</v>
       </c>
       <c r="I62" s="27" t="n">
-        <v>-2.59</v>
+        <v>-13.38</v>
       </c>
       <c r="J62" s="28" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 한국경제 헤드라인 언급</t>
+          <t>중요공시 2건 / 중요공시 3일 +100%</t>
         </is>
       </c>
       <c r="K62" s="28" t="inlineStr">
@@ -3001,7 +3001,7 @@
     <row r="63" ht="18" customHeight="1">
       <c r="A63" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B63" s="25" t="n">
@@ -3009,35 +3009,35 @@
       </c>
       <c r="C63" s="26" t="inlineStr">
         <is>
-          <t>삼성SDI</t>
+          <t>삼일씨엔에스</t>
         </is>
       </c>
       <c r="D63" s="25" t="n">
         <v>3</v>
       </c>
       <c r="E63" s="25" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F63" s="25" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G63" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H63" s="27" t="n">
-        <v>-1.88</v>
-      </c>
-      <c r="I63" s="27" t="n">
-        <v>-4.58</v>
+      <c r="H63" s="29" t="n">
+        <v>5.45</v>
+      </c>
+      <c r="I63" s="29" t="n">
+        <v>9.49</v>
       </c>
       <c r="J63" s="28" t="inlineStr">
         <is>
-          <t>네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+          <t>중요공시 2건 / 중요공시 3일 +100%</t>
         </is>
       </c>
       <c r="K63" s="28" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
@@ -3134,22 +3134,22 @@
         <v>1</v>
       </c>
       <c r="C3" s="25" t="n">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="D3" s="25" t="n">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="E3" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F3" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="G3" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="H3" s="25" t="n"/>
@@ -3165,22 +3165,22 @@
         <v>1</v>
       </c>
       <c r="C4" s="25" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D4" s="25" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="E4" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F4" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="G4" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="H4" s="29" t="n">
@@ -3193,95 +3193,95 @@
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="26" t="inlineStr">
         <is>
-          <t>SK하이닉스</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="B5" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="25" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="D5" s="25" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="E5" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F5" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="G5" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="H5" s="29" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="I5" s="29" t="n">
-        <v>6.03</v>
-      </c>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="H5" s="25" t="n"/>
+      <c r="I5" s="25" t="n"/>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="26" t="inlineStr">
         <is>
-          <t>원전</t>
+          <t>LG전자</t>
         </is>
       </c>
       <c r="B6" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="25" t="n">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="D6" s="25" t="n">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="E6" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F6" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="G6" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="H6" s="25" t="n"/>
-      <c r="I6" s="25" t="n"/>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="H6" s="27" t="n">
+        <v>-2.09</v>
+      </c>
+      <c r="I6" s="29" t="n">
+        <v>5.46</v>
+      </c>
     </row>
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="26" t="inlineStr">
         <is>
-          <t>인공지능</t>
+          <t>바이오</t>
         </is>
       </c>
       <c r="B7" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="25" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="D7" s="25" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="E7" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F7" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="G7" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="H7" s="25" t="n"/>
@@ -3290,112 +3290,108 @@
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="26" t="inlineStr">
         <is>
-          <t>LG전자</t>
+          <t>대한항공</t>
         </is>
       </c>
       <c r="B8" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="25" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D8" s="25" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E8" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F8" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="G8" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="H8" s="27" t="n">
-        <v>-2.09</v>
+        <v>-0.47</v>
       </c>
       <c r="I8" s="29" t="n">
-        <v>5.46</v>
+        <v>7.69</v>
       </c>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="26" t="inlineStr">
         <is>
-          <t>대한항공</t>
+          <t>셀리드</t>
         </is>
       </c>
       <c r="B9" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="25" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D9" s="25" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E9" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F9" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="G9" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="H9" s="27" t="n">
-        <v>-0.47</v>
+        <v>-9.710000000000001</v>
       </c>
       <c r="I9" s="29" t="n">
-        <v>7.69</v>
+        <v>17.08</v>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="26" t="inlineStr">
         <is>
-          <t>삼성전기</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="B10" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C10" s="25" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D10" s="25" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E10" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F10" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="G10" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="H10" s="29" t="n">
-        <v>0.8100000000000001</v>
-      </c>
-      <c r="I10" s="29" t="n">
-        <v>9.4</v>
-      </c>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="H10" s="25" t="n"/>
+      <c r="I10" s="25" t="n"/>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="26" t="inlineStr">
         <is>
-          <t>카카오</t>
+          <t>원전</t>
         </is>
       </c>
       <c r="B11" s="25" t="n">
@@ -3412,25 +3408,21 @@
       </c>
       <c r="F11" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="G11" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="H11" s="27" t="n">
-        <v>-1.31</v>
-      </c>
-      <c r="I11" s="29" t="n">
-        <v>0.45</v>
-      </c>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="H11" s="25" t="n"/>
+      <c r="I11" s="25" t="n"/>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="26" t="inlineStr">
         <is>
-          <t>HJ중공업</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="B12" s="25" t="n">
@@ -3447,54 +3439,50 @@
       </c>
       <c r="F12" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="G12" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="H12" s="27" t="n">
-        <v>-1.78</v>
-      </c>
-      <c r="I12" s="27" t="n">
-        <v>-0.67</v>
-      </c>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="H12" s="25" t="n"/>
+      <c r="I12" s="25" t="n"/>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>셀리드</t>
+          <t>SK하이닉스</t>
         </is>
       </c>
       <c r="B13" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C13" s="25" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D13" s="25" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E13" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F13" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="G13" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="H13" s="27" t="n">
-        <v>-9.710000000000001</v>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="H13" s="29" t="n">
+        <v>1.2</v>
       </c>
       <c r="I13" s="29" t="n">
-        <v>17.08</v>
+        <v>6.03</v>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
@@ -3517,12 +3505,12 @@
       </c>
       <c r="F14" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="G14" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="H14" s="27" t="n">
@@ -3535,7 +3523,7 @@
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>대우건설</t>
+          <t>스피어</t>
         </is>
       </c>
       <c r="B15" s="25" t="n">
@@ -3552,25 +3540,25 @@
       </c>
       <c r="F15" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="G15" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="H15" s="27" t="n">
-        <v>-6.4</v>
-      </c>
-      <c r="I15" s="27" t="n">
-        <v>-4.89</v>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="H15" s="29" t="n">
+        <v>3.76</v>
+      </c>
+      <c r="I15" s="29" t="n">
+        <v>15.23</v>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>바이오</t>
+          <t>현대차</t>
         </is>
       </c>
       <c r="B16" s="25" t="n">
@@ -3587,78 +3575,82 @@
       </c>
       <c r="F16" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="G16" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="H16" s="25" t="n"/>
-      <c r="I16" s="25" t="n"/>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="H16" s="27" t="n">
+        <v>-1.38</v>
+      </c>
+      <c r="I16" s="27" t="n">
+        <v>-1.52</v>
+      </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>스피어</t>
+          <t>GS</t>
         </is>
       </c>
       <c r="B17" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C17" s="25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D17" s="25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E17" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F17" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="G17" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="H17" s="29" t="n">
-        <v>3.76</v>
-      </c>
-      <c r="I17" s="29" t="n">
-        <v>15.23</v>
+        <v>0.91</v>
+      </c>
+      <c r="I17" s="27" t="n">
+        <v>-0.72</v>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="26" t="inlineStr">
         <is>
-          <t>태양광</t>
+          <t>와이즈플래닛컴퍼니</t>
         </is>
       </c>
       <c r="B18" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C18" s="25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D18" s="25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E18" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F18" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="G18" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="H18" s="25" t="n"/>
@@ -3667,135 +3659,147 @@
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>GS건설</t>
         </is>
       </c>
       <c r="B19" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C19" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D19" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E19" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F19" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="G19" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="H19" s="25" t="n"/>
-      <c r="I19" s="25" t="n"/>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="H19" s="27" t="n">
+        <v>-7.33</v>
+      </c>
+      <c r="I19" s="27" t="n">
+        <v>-5.57</v>
+      </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="26" t="inlineStr">
         <is>
-          <t>방산</t>
+          <t>HJ중공업</t>
         </is>
       </c>
       <c r="B20" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C20" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D20" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E20" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F20" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="G20" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="H20" s="25" t="n"/>
-      <c r="I20" s="25" t="n"/>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="H20" s="27" t="n">
+        <v>-1.78</v>
+      </c>
+      <c r="I20" s="27" t="n">
+        <v>-0.67</v>
+      </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="26" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>노타</t>
         </is>
       </c>
       <c r="B21" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C21" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D21" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E21" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F21" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="G21" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="H21" s="25" t="n"/>
-      <c r="I21" s="25" t="n"/>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="H21" s="27" t="n">
+        <v>-9.529999999999999</v>
+      </c>
+      <c r="I21" s="29" t="n">
+        <v>21.21</v>
+      </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="26" t="inlineStr">
         <is>
-          <t>한화시스템</t>
+          <t>비에이치아이</t>
         </is>
       </c>
       <c r="B22" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C22" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D22" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E22" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F22" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="G22" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="H22" s="27" t="n">
-        <v>-4.12</v>
-      </c>
-      <c r="I22" s="29" t="n">
-        <v>7.98</v>
+        <v>-5.76</v>
+      </c>
+      <c r="I22" s="27" t="n">
+        <v>-4.57</v>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="26" t="inlineStr">
         <is>
-          <t>GS건설</t>
+          <t>비케이홀딩스</t>
         </is>
       </c>
       <c r="B23" s="25" t="n">
@@ -3812,25 +3816,25 @@
       </c>
       <c r="F23" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="G23" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="H23" s="27" t="n">
-        <v>-7.33</v>
+        <v>-15.35</v>
       </c>
       <c r="I23" s="27" t="n">
-        <v>-5.57</v>
+        <v>-17.21</v>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="26" t="inlineStr">
         <is>
-          <t>대양금속</t>
+          <t>삼성물산</t>
         </is>
       </c>
       <c r="B24" s="25" t="n">
@@ -3847,25 +3851,25 @@
       </c>
       <c r="F24" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="G24" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="H24" s="27" t="n">
-        <v>-14.85</v>
-      </c>
-      <c r="I24" s="27" t="n">
-        <v>-11.08</v>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="H24" s="29" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="I24" s="29" t="n">
+        <v>4.84</v>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="26" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>한화시스템</t>
         </is>
       </c>
       <c r="B25" s="25" t="n">
@@ -3882,227 +3886,231 @@
       </c>
       <c r="F25" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="G25" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="H25" s="25" t="n"/>
-      <c r="I25" s="25" t="n"/>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="H25" s="27" t="n">
+        <v>-4.12</v>
+      </c>
+      <c r="I25" s="29" t="n">
+        <v>7.98</v>
+      </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="26" t="inlineStr">
         <is>
-          <t>비에이치아이</t>
+          <t>카카오</t>
         </is>
       </c>
       <c r="B26" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C26" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D26" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E26" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F26" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="G26" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="H26" s="27" t="n">
-        <v>-5.76</v>
-      </c>
-      <c r="I26" s="27" t="n">
-        <v>-4.57</v>
+        <v>-1.31</v>
+      </c>
+      <c r="I26" s="29" t="n">
+        <v>0.45</v>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="26" t="inlineStr">
         <is>
-          <t>삼성물산</t>
+          <t>포스코퓨처엠</t>
         </is>
       </c>
       <c r="B27" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C27" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D27" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E27" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F27" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="G27" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="H27" s="29" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="I27" s="29" t="n">
-        <v>4.84</v>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="H27" s="27" t="n">
+        <v>-2.96</v>
+      </c>
+      <c r="I27" s="27" t="n">
+        <v>-4.24</v>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="26" t="inlineStr">
         <is>
-          <t>와이즈플래닛컴퍼니</t>
+          <t>대양금속</t>
         </is>
       </c>
       <c r="B28" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C28" s="25" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D28" s="25" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E28" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F28" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="G28" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="H28" s="25" t="n"/>
-      <c r="I28" s="25" t="n"/>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="H28" s="27" t="n">
+        <v>-14.85</v>
+      </c>
+      <c r="I28" s="27" t="n">
+        <v>-11.08</v>
+      </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="26" t="inlineStr">
         <is>
-          <t>두산에너빌리티</t>
+          <t>디에이테크놀로지</t>
         </is>
       </c>
       <c r="B29" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C29" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D29" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E29" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F29" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="G29" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="H29" s="27" t="n">
-        <v>-4.5</v>
+        <v>-96.68000000000001</v>
       </c>
       <c r="I29" s="27" t="n">
-        <v>-1.66</v>
+        <v>-96.68000000000001</v>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="26" t="inlineStr">
         <is>
-          <t>우진</t>
+          <t>방산</t>
         </is>
       </c>
       <c r="B30" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C30" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D30" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E30" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F30" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="G30" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="H30" s="27" t="n">
-        <v>-4.46</v>
-      </c>
-      <c r="I30" s="27" t="n">
-        <v>-2.59</v>
-      </c>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="H30" s="25" t="n"/>
+      <c r="I30" s="25" t="n"/>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="26" t="inlineStr">
         <is>
-          <t>포스코퓨처엠</t>
+          <t>삼성전기</t>
         </is>
       </c>
       <c r="B31" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C31" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D31" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E31" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F31" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="G31" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="H31" s="27" t="n">
-        <v>-2.96</v>
-      </c>
-      <c r="I31" s="27" t="n">
-        <v>-4.24</v>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="H31" s="29" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="I31" s="29" t="n">
+        <v>9.4</v>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="26" t="inlineStr">
         <is>
-          <t>SG</t>
+          <t>삼성제약</t>
         </is>
       </c>
       <c r="B32" s="25" t="n">
@@ -4119,25 +4127,25 @@
       </c>
       <c r="F32" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="G32" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="H32" s="29" t="n">
-        <v>7.27</v>
-      </c>
-      <c r="I32" s="29" t="n">
-        <v>8.619999999999999</v>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="H32" s="27" t="n">
+        <v>-2.66</v>
+      </c>
+      <c r="I32" s="27" t="n">
+        <v>-8.380000000000001</v>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="26" t="inlineStr">
         <is>
-          <t>노타</t>
+          <t>스테이블코인</t>
         </is>
       </c>
       <c r="B33" s="25" t="n">
@@ -4154,25 +4162,21 @@
       </c>
       <c r="F33" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="G33" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="H33" s="27" t="n">
-        <v>-9.529999999999999</v>
-      </c>
-      <c r="I33" s="29" t="n">
-        <v>21.21</v>
-      </c>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="H33" s="25" t="n"/>
+      <c r="I33" s="25" t="n"/>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="26" t="inlineStr">
         <is>
-          <t>스테이블코인</t>
+          <t>우리기술</t>
         </is>
       </c>
       <c r="B34" s="25" t="n">
@@ -4189,126 +4193,126 @@
       </c>
       <c r="F34" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="G34" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="H34" s="25" t="n"/>
-      <c r="I34" s="25" t="n"/>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="H34" s="27" t="n">
+        <v>-3.35</v>
+      </c>
+      <c r="I34" s="29" t="n">
+        <v>0.54</v>
+      </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="26" t="inlineStr">
         <is>
-          <t>KB제34호스팩</t>
+          <t>케이쓰리아이</t>
         </is>
       </c>
       <c r="B35" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C35" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D35" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E35" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F35" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="G35" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="H35" s="27" t="n">
-        <v>-0.37</v>
-      </c>
-      <c r="I35" s="27" t="n">
-        <v>-0.37</v>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="H35" s="29" t="n">
+        <v>11.96</v>
+      </c>
+      <c r="I35" s="29" t="n">
+        <v>26.25</v>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="26" t="inlineStr">
         <is>
-          <t>네오사피엔스</t>
+          <t>태양광</t>
         </is>
       </c>
       <c r="B36" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C36" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D36" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E36" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F36" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="G36" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="H36" s="27" t="n">
-        <v>-16.78</v>
-      </c>
-      <c r="I36" s="27" t="n">
-        <v>-32.79</v>
-      </c>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="H36" s="25" t="n"/>
+      <c r="I36" s="25" t="n"/>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="26" t="inlineStr">
         <is>
-          <t>넥사다이내믹스</t>
+          <t>테스</t>
         </is>
       </c>
       <c r="B37" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C37" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D37" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E37" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F37" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="G37" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="H37" s="29" t="n">
-        <v>0.41</v>
-      </c>
-      <c r="I37" s="27" t="n">
-        <v>-5.05</v>
+        <v>8.949999999999999</v>
+      </c>
+      <c r="I37" s="29" t="n">
+        <v>19.31</v>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="26" t="inlineStr">
         <is>
-          <t>더코디</t>
+          <t>KB제34호스팩</t>
         </is>
       </c>
       <c r="B38" s="25" t="n">
@@ -4325,25 +4329,25 @@
       </c>
       <c r="F38" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="G38" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="H38" s="29" t="n">
-        <v>5.14</v>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="H38" s="27" t="n">
+        <v>-0.37</v>
       </c>
       <c r="I38" s="27" t="n">
-        <v>-40.85</v>
+        <v>-0.37</v>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="26" t="inlineStr">
         <is>
-          <t>동국생명과학</t>
+          <t>네오사피엔스</t>
         </is>
       </c>
       <c r="B39" s="25" t="n">
@@ -4360,25 +4364,25 @@
       </c>
       <c r="F39" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="G39" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="H39" s="27" t="n">
-        <v>-9.06</v>
-      </c>
-      <c r="I39" s="29" t="n">
-        <v>20.52</v>
+        <v>-16.78</v>
+      </c>
+      <c r="I39" s="27" t="n">
+        <v>-32.79</v>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="26" t="inlineStr">
         <is>
-          <t>모아데이타</t>
+          <t>넥사다이내믹스</t>
         </is>
       </c>
       <c r="B40" s="25" t="n">
@@ -4395,25 +4399,25 @@
       </c>
       <c r="F40" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="G40" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="H40" s="27" t="n">
-        <v>-2.38</v>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="H40" s="29" t="n">
+        <v>0.41</v>
       </c>
       <c r="I40" s="27" t="n">
-        <v>-13.38</v>
+        <v>-5.05</v>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="26" t="inlineStr">
         <is>
-          <t>비케이홀딩스</t>
+          <t>더코디</t>
         </is>
       </c>
       <c r="B41" s="25" t="n">
@@ -4430,25 +4434,25 @@
       </c>
       <c r="F41" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="G41" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="H41" s="27" t="n">
-        <v>-15.35</v>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="H41" s="29" t="n">
+        <v>5.14</v>
       </c>
       <c r="I41" s="27" t="n">
-        <v>-17.21</v>
+        <v>-40.85</v>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="26" t="inlineStr">
         <is>
-          <t>삼성E&amp;A</t>
+          <t>동국생명과학</t>
         </is>
       </c>
       <c r="B42" s="25" t="n">
@@ -4465,25 +4469,25 @@
       </c>
       <c r="F42" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="G42" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="H42" s="27" t="n">
-        <v>-3.31</v>
-      </c>
-      <c r="I42" s="27" t="n">
-        <v>-1.2</v>
+        <v>-9.06</v>
+      </c>
+      <c r="I42" s="29" t="n">
+        <v>20.52</v>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="26" t="inlineStr">
         <is>
-          <t>삼성SDI</t>
+          <t>두산에너빌리티</t>
         </is>
       </c>
       <c r="B43" s="25" t="n">
@@ -4500,25 +4504,25 @@
       </c>
       <c r="F43" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="G43" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="H43" s="27" t="n">
-        <v>-1.88</v>
+        <v>-4.5</v>
       </c>
       <c r="I43" s="27" t="n">
-        <v>-4.58</v>
+        <v>-1.66</v>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="26" t="inlineStr">
         <is>
-          <t>삼일씨엔에스</t>
+          <t>모아데이타</t>
         </is>
       </c>
       <c r="B44" s="25" t="n">
@@ -4535,25 +4539,25 @@
       </c>
       <c r="F44" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="G44" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="H44" s="29" t="n">
-        <v>5.45</v>
-      </c>
-      <c r="I44" s="29" t="n">
-        <v>9.49</v>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="H44" s="27" t="n">
+        <v>-2.38</v>
+      </c>
+      <c r="I44" s="27" t="n">
+        <v>-13.38</v>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="26" t="inlineStr">
         <is>
-          <t>서희건설</t>
+          <t>삼기에너지솔루션즈</t>
         </is>
       </c>
       <c r="B45" s="25" t="n">
@@ -4570,25 +4574,25 @@
       </c>
       <c r="F45" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="G45" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="H45" s="27" t="n">
-        <v>-1.3</v>
-      </c>
-      <c r="I45" s="27" t="n">
-        <v>-2.16</v>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="H45" s="29" t="n">
+        <v>18.12</v>
+      </c>
+      <c r="I45" s="29" t="n">
+        <v>21.39</v>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="26" t="inlineStr">
         <is>
-          <t>셀트리온</t>
+          <t>삼성E&amp;A</t>
         </is>
       </c>
       <c r="B46" s="25" t="n">
@@ -4605,25 +4609,25 @@
       </c>
       <c r="F46" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="G46" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="H46" s="27" t="n">
-        <v>-0.11</v>
-      </c>
-      <c r="I46" s="29" t="n">
-        <v>0.39</v>
+        <v>-3.31</v>
+      </c>
+      <c r="I46" s="27" t="n">
+        <v>-1.2</v>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="26" t="inlineStr">
         <is>
-          <t>앤씨앤</t>
+          <t>삼일씨엔에스</t>
         </is>
       </c>
       <c r="B47" s="25" t="n">
@@ -4640,25 +4644,25 @@
       </c>
       <c r="F47" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="G47" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="H47" s="29" t="n">
-        <v>5.18</v>
+        <v>5.45</v>
       </c>
       <c r="I47" s="29" t="n">
-        <v>35.4</v>
+        <v>9.49</v>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="26" t="inlineStr">
         <is>
-          <t>케이쓰리아이</t>
+          <t>서희건설</t>
         </is>
       </c>
       <c r="B48" s="25" t="n">
@@ -4675,25 +4679,25 @@
       </c>
       <c r="F48" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="G48" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="H48" s="29" t="n">
-        <v>11.96</v>
-      </c>
-      <c r="I48" s="29" t="n">
-        <v>26.25</v>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="H48" s="27" t="n">
+        <v>-1.3</v>
+      </c>
+      <c r="I48" s="27" t="n">
+        <v>-2.16</v>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="26" t="inlineStr">
         <is>
-          <t>토마토시스템</t>
+          <t>앤씨앤</t>
         </is>
       </c>
       <c r="B49" s="25" t="n">
@@ -4710,25 +4714,25 @@
       </c>
       <c r="F49" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="G49" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="H49" s="29" t="n">
-        <v>12.07</v>
+        <v>5.18</v>
       </c>
       <c r="I49" s="29" t="n">
-        <v>65.84999999999999</v>
+        <v>35.4</v>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="26" t="inlineStr">
         <is>
-          <t>한국제17호스팩</t>
+          <t>토마토시스템</t>
         </is>
       </c>
       <c r="B50" s="25" t="n">
@@ -4745,25 +4749,25 @@
       </c>
       <c r="F50" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="G50" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="H50" s="27" t="n">
-        <v>-1.91</v>
-      </c>
-      <c r="I50" s="27" t="n">
-        <v>-1.91</v>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="H50" s="29" t="n">
+        <v>12.07</v>
+      </c>
+      <c r="I50" s="29" t="n">
+        <v>65.84999999999999</v>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="26" t="inlineStr">
         <is>
-          <t>한화솔루션</t>
+          <t>한국제17호스팩</t>
         </is>
       </c>
       <c r="B51" s="25" t="n">
@@ -4780,25 +4784,25 @@
       </c>
       <c r="F51" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="G51" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="H51" s="29" t="n">
-        <v>6.52</v>
-      </c>
-      <c r="I51" s="29" t="n">
-        <v>2.62</v>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="H51" s="27" t="n">
+        <v>-1.91</v>
+      </c>
+      <c r="I51" s="27" t="n">
+        <v>-1.91</v>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="26" t="inlineStr">
         <is>
-          <t>현대로템</t>
+          <t>한화솔루션</t>
         </is>
       </c>
       <c r="B52" s="25" t="n">
@@ -4815,19 +4819,19 @@
       </c>
       <c r="F52" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="G52" s="25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="H52" s="27" t="n">
-        <v>-1.19</v>
-      </c>
-      <c r="I52" s="27" t="n">
-        <v>-2.59</v>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="H52" s="29" t="n">
+        <v>6.52</v>
+      </c>
+      <c r="I52" s="29" t="n">
+        <v>2.62</v>
       </c>
     </row>
   </sheetData>
@@ -4911,19 +4915,19 @@
         <v>1</v>
       </c>
       <c r="C3" s="36" t="n">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="D3" s="36" t="n">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="E3" s="36" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="F3" s="37" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="G3" s="37" t="inlineStr">
@@ -4942,19 +4946,19 @@
         <v>1</v>
       </c>
       <c r="C4" s="36" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="D4" s="36" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E4" s="36" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="F4" s="37" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="G4" s="37" t="inlineStr">
@@ -4973,19 +4977,19 @@
         <v>1</v>
       </c>
       <c r="C5" s="36" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D5" s="36" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E5" s="36" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="F5" s="37" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="G5" s="37" t="inlineStr">
@@ -5004,19 +5008,19 @@
         <v>1</v>
       </c>
       <c r="C6" s="36" t="n">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="D6" s="36" t="n">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="E6" s="36" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="F6" s="37" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="G6" s="37" t="inlineStr">
@@ -5035,19 +5039,19 @@
         <v>1</v>
       </c>
       <c r="C7" s="36" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D7" s="36" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E7" s="36" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="F7" s="37" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="G7" s="37" t="inlineStr">
@@ -5066,19 +5070,19 @@
         <v>1</v>
       </c>
       <c r="C8" s="36" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D8" s="36" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="E8" s="36" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="F8" s="37" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="G8" s="37" t="inlineStr">
@@ -5097,19 +5101,19 @@
         <v>1</v>
       </c>
       <c r="C9" s="36" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="D9" s="36" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="E9" s="36" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="F9" s="37" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="G9" s="37" t="inlineStr">
@@ -5128,19 +5132,19 @@
         <v>1</v>
       </c>
       <c r="C10" s="36" t="n">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="D10" s="36" t="n">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="E10" s="36" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="F10" s="37" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="G10" s="37" t="inlineStr">
@@ -5150,40 +5154,36 @@
       </c>
     </row>
     <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="35" t="inlineStr">
-        <is>
-          <t>AMD</t>
-        </is>
-      </c>
-      <c r="B11" s="36" t="n">
-        <v>1</v>
-      </c>
-      <c r="C11" s="36" t="n">
-        <v>7</v>
-      </c>
-      <c r="D11" s="36" t="n">
-        <v>7</v>
-      </c>
-      <c r="E11" s="36" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="F11" s="37" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="G11" s="37" t="inlineStr">
-        <is>
-          <t>⚡ 관심</t>
-        </is>
-      </c>
+      <c r="A11" s="26" t="inlineStr">
+        <is>
+          <t>이차전지</t>
+        </is>
+      </c>
+      <c r="B11" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F11" s="28" t="inlineStr">
+        <is>
+          <t>감지 없음</t>
+        </is>
+      </c>
+      <c r="G11" s="28" t="inlineStr"/>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="26" t="inlineStr">
         <is>
-          <t>이차전지</t>
+          <t>AI반도체</t>
         </is>
       </c>
       <c r="B12" s="25" t="n">
@@ -5210,7 +5210,7 @@
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>AI반도체</t>
+          <t>전기차</t>
         </is>
       </c>
       <c r="B13" s="25" t="n">
@@ -5237,7 +5237,7 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>전기차</t>
+          <t>수소</t>
         </is>
       </c>
       <c r="B14" s="25" t="n">
@@ -5264,7 +5264,7 @@
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>수소</t>
+          <t>게임</t>
         </is>
       </c>
       <c r="B15" s="25" t="n">
@@ -5291,7 +5291,7 @@
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>게임</t>
+          <t>엔터</t>
         </is>
       </c>
       <c r="B16" s="25" t="n">
@@ -5318,7 +5318,7 @@
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>엔터</t>
+          <t>핀테크</t>
         </is>
       </c>
       <c r="B17" s="25" t="n">
@@ -5345,7 +5345,7 @@
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="26" t="inlineStr">
         <is>
-          <t>핀테크</t>
+          <t>클라우드</t>
         </is>
       </c>
       <c r="B18" s="25" t="n">
@@ -5372,7 +5372,7 @@
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>클라우드</t>
+          <t>조선</t>
         </is>
       </c>
       <c r="B19" s="25" t="n">
@@ -5399,7 +5399,7 @@
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="26" t="inlineStr">
         <is>
-          <t>조선</t>
+          <t>철강</t>
         </is>
       </c>
       <c r="B20" s="25" t="n">
@@ -5426,7 +5426,7 @@
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="26" t="inlineStr">
         <is>
-          <t>철강</t>
+          <t>의료기기</t>
         </is>
       </c>
       <c r="B21" s="25" t="n">
@@ -5453,7 +5453,7 @@
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="26" t="inlineStr">
         <is>
-          <t>의료기기</t>
+          <t>NVIDIA</t>
         </is>
       </c>
       <c r="B22" s="25" t="n">
@@ -5480,7 +5480,7 @@
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="26" t="inlineStr">
         <is>
-          <t>NVIDIA</t>
+          <t>Tesla</t>
         </is>
       </c>
       <c r="B23" s="25" t="n">
@@ -5507,7 +5507,7 @@
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="26" t="inlineStr">
         <is>
-          <t>Tesla</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B24" s="25" t="n">

</xml_diff>

<commit_message>
auto: 2026-09-27 07:21 자동 백업
</commit_message>
<xml_diff>
--- a/trend/stock_trend_history.xlsx
+++ b/trend/stock_trend_history.xlsx
@@ -261,11 +261,11 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -694,7 +694,7 @@
     <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-09-26 06:54</t>
+          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-09-27 06:54</t>
         </is>
       </c>
     </row>
@@ -708,7 +708,7 @@
       </c>
       <c r="E3" s="3" t="n"/>
       <c r="G3" s="5" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="H3" s="3" t="n"/>
       <c r="J3" s="6" t="n">
@@ -787,21 +787,21 @@
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-09-26) 상위: 반도체  점수 55.0점</t>
+          <t>⚡ 최신(2026-09-27) 상위: 반도체  점수 43.0점</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-09-26) 상위: 삼성전자  점수 29.0점</t>
+          <t>⚡ 최신(2026-09-27) 상위: 삼성전자  점수 35.0점</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-09-26) 상위: 인공지능  점수 18.0점</t>
+          <t>⚡ 최신(2026-09-27) 상위: 게임  점수 13.0점</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="15" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B14" s="15" t="n">
@@ -928,10 +928,10 @@
         </is>
       </c>
       <c r="D14" s="15" t="n">
-        <v>55</v>
+        <v>43</v>
       </c>
       <c r="E14" s="15" t="n">
-        <v>55</v>
+        <v>43</v>
       </c>
       <c r="F14" s="15" t="n">
         <v>0</v>
@@ -947,7 +947,7 @@
       </c>
       <c r="J14" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K14" s="17" t="inlineStr">
@@ -959,7 +959,7 @@
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="15" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B15" s="15" t="n">
@@ -971,10 +971,10 @@
         </is>
       </c>
       <c r="D15" s="15" t="n">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="E15" s="15" t="n">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="F15" s="15" t="n">
         <v>0</v>
@@ -986,11 +986,11 @@
         <v>3.24</v>
       </c>
       <c r="I15" s="18" t="n">
-        <v>13.02</v>
+        <v>11.91</v>
       </c>
       <c r="J15" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급</t>
+          <t>매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K15" s="17" t="inlineStr">
@@ -1002,7 +1002,7 @@
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="15" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B16" s="15" t="n">
@@ -1010,14 +1010,14 @@
       </c>
       <c r="C16" s="16" t="inlineStr">
         <is>
-          <t>인공지능</t>
+          <t>게임</t>
         </is>
       </c>
       <c r="D16" s="15" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E16" s="15" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="F16" s="15" t="n">
         <v>0</v>
@@ -1033,19 +1033,19 @@
       </c>
       <c r="J16" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급</t>
+          <t>Google 급상승 검색어 등장 (KR) / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K16" s="17" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>Google</t>
         </is>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B17" s="15" t="n">
@@ -1053,14 +1053,14 @@
       </c>
       <c r="C17" s="16" t="inlineStr">
         <is>
-          <t>게임</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="D17" s="15" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E17" s="15" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F17" s="15" t="n">
         <v>0</v>
@@ -1076,7 +1076,7 @@
       </c>
       <c r="J17" s="17" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
+          <t>네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K17" s="17" t="inlineStr">
@@ -1088,7 +1088,7 @@
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B18" s="15" t="n">
@@ -1096,7 +1096,7 @@
       </c>
       <c r="C18" s="16" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="D18" s="15" t="n">
@@ -1119,7 +1119,7 @@
       </c>
       <c r="J18" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 헤드라인 언급</t>
+          <t>매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K18" s="17" t="inlineStr">
@@ -1131,7 +1131,7 @@
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B19" s="15" t="n">
@@ -1158,7 +1158,7 @@
         <v>-0.47</v>
       </c>
       <c r="I19" s="18" t="n">
-        <v>7.69</v>
+        <v>6.6</v>
       </c>
       <c r="J19" s="17" t="inlineStr">
         <is>
@@ -1172,7 +1172,7 @@
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B20" s="15" t="n">
@@ -1198,12 +1198,12 @@
       <c r="H20" s="18" t="n">
         <v>3.76</v>
       </c>
-      <c r="I20" s="18" t="n">
-        <v>15.23</v>
+      <c r="I20" s="19" t="n">
+        <v>-2.7</v>
       </c>
       <c r="J20" s="17" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 3일 +200% / 중요공시 7일 +50%</t>
+          <t>중요공시 3건 / 중요공시 3일 +50% / 중요공시 7일 +50%</t>
         </is>
       </c>
       <c r="K20" s="17" t="inlineStr">
@@ -1215,7 +1215,7 @@
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="15" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B21" s="15" t="n">
@@ -1223,42 +1223,42 @@
       </c>
       <c r="C21" s="16" t="inlineStr">
         <is>
-          <t>셀리드</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="D21" s="15" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E21" s="15" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="F21" s="15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G21" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H21" s="19" t="n">
-        <v>-9.710000000000001</v>
-      </c>
-      <c r="I21" s="18" t="n">
-        <v>17.08</v>
+      <c r="H21" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I21" s="15" t="n">
+        <v/>
       </c>
       <c r="J21" s="17" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +73% / 중요공시 4건 / 중요공시 3일 +100%</t>
+          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K21" s="17" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="15" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B22" s="15" t="n">
@@ -1266,42 +1266,42 @@
       </c>
       <c r="C22" s="16" t="inlineStr">
         <is>
-          <t>대양금속</t>
+          <t>SK하이닉스</t>
         </is>
       </c>
       <c r="D22" s="15" t="n">
         <v>7</v>
       </c>
       <c r="E22" s="15" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F22" s="15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G22" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H22" s="19" t="n">
-        <v>-14.85</v>
-      </c>
-      <c r="I22" s="19" t="n">
-        <v>-11.08</v>
+      <c r="H22" s="18" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="I22" s="18" t="n">
+        <v>5.49</v>
       </c>
       <c r="J22" s="17" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +56% / 중요공시 3건 / 중요공시 3일 +200%</t>
+          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K22" s="17" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="15" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B23" s="15" t="n">
@@ -1328,7 +1328,7 @@
         <v>-1.78</v>
       </c>
       <c r="I23" s="19" t="n">
-        <v>-0.67</v>
+        <v>-5.1</v>
       </c>
       <c r="J23" s="17" t="inlineStr">
         <is>
@@ -1342,52 +1342,50 @@
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="15" t="inlineStr">
-        <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-      <c r="B24" s="15" t="n">
+      <c r="A24" s="20" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B24" s="20" t="n">
         <v>11</v>
       </c>
-      <c r="C24" s="16" t="inlineStr">
-        <is>
-          <t>태양광</t>
-        </is>
-      </c>
-      <c r="D24" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="E24" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="F24" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="G24" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H24" s="15" t="n">
+      <c r="C24" s="21" t="inlineStr">
+        <is>
+          <t>LG전자</t>
+        </is>
+      </c>
+      <c r="D24" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="E24" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="F24" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" s="22" t="n">
+        <v>-2.09</v>
+      </c>
+      <c r="I24" s="23" t="n">
+        <v>5.57</v>
+      </c>
+      <c r="J24" s="24" t="inlineStr">
+        <is>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K24" s="24" t="n">
         <v/>
-      </c>
-      <c r="I24" s="15" t="n">
-        <v/>
-      </c>
-      <c r="J24" s="17" t="inlineStr">
-        <is>
-          <t>매일경제 기사 언급 / 한국경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K24" s="17" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="20" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B25" s="20" t="n">
@@ -1395,7 +1393,7 @@
       </c>
       <c r="C25" s="21" t="inlineStr">
         <is>
-          <t>네오사피엔스</t>
+          <t>바이오</t>
         </is>
       </c>
       <c r="D25" s="20" t="n">
@@ -1410,18 +1408,18 @@
       <c r="G25" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H25" s="22" t="n">
-        <v>-16.78</v>
-      </c>
-      <c r="I25" s="22" t="n">
-        <v>-32.79</v>
-      </c>
-      <c r="J25" s="23" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +949% / 네이버뉴스 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K25" s="23" t="inlineStr">
+      <c r="H25" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I25" s="20" t="n">
+        <v/>
+      </c>
+      <c r="J25" s="24" t="inlineStr">
+        <is>
+          <t>네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
+        </is>
+      </c>
+      <c r="K25" s="24" t="inlineStr">
         <is>
           <t>네이버</t>
         </is>
@@ -1430,7 +1428,7 @@
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="20" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B26" s="20" t="n">
@@ -1438,14 +1436,14 @@
       </c>
       <c r="C26" s="21" t="inlineStr">
         <is>
-          <t>LG전자</t>
+          <t>셀리드</t>
         </is>
       </c>
       <c r="D26" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E26" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F26" s="20" t="n">
         <v>0</v>
@@ -1454,24 +1452,26 @@
         <v>0</v>
       </c>
       <c r="H26" s="22" t="n">
-        <v>-2.09</v>
-      </c>
-      <c r="I26" s="24" t="n">
-        <v>5.46</v>
-      </c>
-      <c r="J26" s="23" t="inlineStr">
-        <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K26" s="23" t="n">
-        <v/>
+        <v>-9.710000000000001</v>
+      </c>
+      <c r="I26" s="23" t="n">
+        <v>13.26</v>
+      </c>
+      <c r="J26" s="24" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +80% / 중요공시 4건</t>
+        </is>
+      </c>
+      <c r="K26" s="24" t="inlineStr">
+        <is>
+          <t>네이버, 공시</t>
+        </is>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="20" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B27" s="20" t="n">
@@ -1479,14 +1479,14 @@
       </c>
       <c r="C27" s="21" t="inlineStr">
         <is>
-          <t>바이오</t>
+          <t>케이쓰리아이</t>
         </is>
       </c>
       <c r="D27" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E27" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F27" s="20" t="n">
         <v>0</v>
@@ -1494,27 +1494,27 @@
       <c r="G27" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H27" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I27" s="20" t="n">
-        <v/>
-      </c>
-      <c r="J27" s="23" t="inlineStr">
-        <is>
-          <t>네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K27" s="23" t="inlineStr">
-        <is>
-          <t>네이버</t>
+      <c r="H27" s="23" t="n">
+        <v>11.96</v>
+      </c>
+      <c r="I27" s="23" t="n">
+        <v>23.71</v>
+      </c>
+      <c r="J27" s="24" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +70% / 중요공시 3건</t>
+        </is>
+      </c>
+      <c r="K27" s="24" t="inlineStr">
+        <is>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="20" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B28" s="20" t="n">
@@ -1522,14 +1522,14 @@
       </c>
       <c r="C28" s="21" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>대양금속</t>
         </is>
       </c>
       <c r="D28" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E28" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F28" s="20" t="n">
         <v>0</v>
@@ -1537,25 +1537,27 @@
       <c r="G28" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H28" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I28" s="20" t="n">
-        <v/>
-      </c>
-      <c r="J28" s="23" t="inlineStr">
-        <is>
-          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K28" s="23" t="n">
-        <v/>
+      <c r="H28" s="22" t="n">
+        <v>-14.85</v>
+      </c>
+      <c r="I28" s="22" t="n">
+        <v>-12.69</v>
+      </c>
+      <c r="J28" s="24" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +60% / 중요공시 3건</t>
+        </is>
+      </c>
+      <c r="K28" s="24" t="inlineStr">
+        <is>
+          <t>네이버, 공시</t>
+        </is>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="20" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B29" s="20" t="n">
@@ -1563,7 +1565,7 @@
       </c>
       <c r="C29" s="21" t="inlineStr">
         <is>
-          <t>케이쓰리아이</t>
+          <t>전기차</t>
         </is>
       </c>
       <c r="D29" s="20" t="n">
@@ -1578,27 +1580,27 @@
       <c r="G29" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H29" s="24" t="n">
-        <v>11.96</v>
-      </c>
-      <c r="I29" s="24" t="n">
-        <v>26.25</v>
-      </c>
-      <c r="J29" s="23" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +60% / 중요공시 3건</t>
-        </is>
-      </c>
-      <c r="K29" s="23" t="inlineStr">
-        <is>
-          <t>공시, 네이버</t>
+      <c r="H29" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I29" s="20" t="n">
+        <v/>
+      </c>
+      <c r="J29" s="24" t="inlineStr">
+        <is>
+          <t>매일경제 기사 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K29" s="24" t="inlineStr">
+        <is>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="20" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B30" s="20" t="n">
@@ -1606,42 +1608,40 @@
       </c>
       <c r="C30" s="21" t="inlineStr">
         <is>
-          <t>서희건설</t>
+          <t>카카오</t>
         </is>
       </c>
       <c r="D30" s="20" t="n">
         <v>5</v>
       </c>
       <c r="E30" s="20" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F30" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G30" s="20" t="n">
         <v>0</v>
       </c>
       <c r="H30" s="22" t="n">
-        <v>-1.3</v>
-      </c>
-      <c r="I30" s="22" t="n">
-        <v>-2.16</v>
-      </c>
-      <c r="J30" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 3건 / 중요공시 3일 +50%</t>
-        </is>
-      </c>
-      <c r="K30" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+        <v>-1.31</v>
+      </c>
+      <c r="I30" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="J30" s="24" t="inlineStr">
+        <is>
+          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K30" s="24" t="n">
+        <v/>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="20" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B31" s="20" t="n">
@@ -1649,14 +1649,14 @@
       </c>
       <c r="C31" s="21" t="inlineStr">
         <is>
-          <t>현대건설</t>
+          <t>디에이테크놀로지</t>
         </is>
       </c>
       <c r="D31" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E31" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F31" s="20" t="n">
         <v>0</v>
@@ -1665,26 +1665,26 @@
         <v>0</v>
       </c>
       <c r="H31" s="22" t="n">
-        <v>-7.21</v>
+        <v>-96.68000000000001</v>
       </c>
       <c r="I31" s="22" t="n">
-        <v>-1.37</v>
-      </c>
-      <c r="J31" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 1건 / 한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K31" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
+        <v>-96.68000000000001</v>
+      </c>
+      <c r="J31" s="24" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +628% / 중요공시 2건</t>
+        </is>
+      </c>
+      <c r="K31" s="24" t="inlineStr">
+        <is>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="20" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B32" s="20" t="n">
@@ -1692,14 +1692,14 @@
       </c>
       <c r="C32" s="21" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>와이즈플래닛컴퍼니</t>
         </is>
       </c>
       <c r="D32" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E32" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F32" s="20" t="n">
         <v>0</v>
@@ -1713,21 +1713,19 @@
       <c r="I32" s="20" t="n">
         <v/>
       </c>
-      <c r="J32" s="23" t="inlineStr">
-        <is>
-          <t>Google 급상승 검색어 등장 (US)</t>
-        </is>
-      </c>
-      <c r="K32" s="23" t="inlineStr">
-        <is>
-          <t>Google</t>
-        </is>
+      <c r="J32" s="24" t="inlineStr">
+        <is>
+          <t>매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K32" s="24" t="n">
+        <v/>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="20" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B33" s="20" t="n">
@@ -1735,40 +1733,42 @@
       </c>
       <c r="C33" s="21" t="inlineStr">
         <is>
-          <t>카카오</t>
+          <t>셀트리온</t>
         </is>
       </c>
       <c r="D33" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E33" s="20" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F33" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G33" s="20" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H33" s="22" t="n">
-        <v>-1.31</v>
-      </c>
-      <c r="I33" s="24" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="J33" s="23" t="inlineStr">
-        <is>
-          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K33" s="23" t="n">
-        <v/>
+        <v>-0.11</v>
+      </c>
+      <c r="I33" s="22" t="n">
+        <v>-1.77</v>
+      </c>
+      <c r="J33" s="24" t="inlineStr">
+        <is>
+          <t>중요공시 2건 / 중요공시 7일 +100%</t>
+        </is>
+      </c>
+      <c r="K33" s="24" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="20" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B34" s="20" t="n">
@@ -1776,14 +1776,14 @@
       </c>
       <c r="C34" s="21" t="inlineStr">
         <is>
-          <t>원전</t>
+          <t>삼성제약</t>
         </is>
       </c>
       <c r="D34" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E34" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F34" s="20" t="n">
         <v>0</v>
@@ -1791,25 +1791,27 @@
       <c r="G34" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H34" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I34" s="20" t="n">
-        <v/>
-      </c>
-      <c r="J34" s="23" t="inlineStr">
-        <is>
-          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K34" s="23" t="n">
-        <v/>
+      <c r="H34" s="22" t="n">
+        <v>-2.66</v>
+      </c>
+      <c r="I34" s="22" t="n">
+        <v>-6.91</v>
+      </c>
+      <c r="J34" s="24" t="inlineStr">
+        <is>
+          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K34" s="24" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="20" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B35" s="20" t="n">
@@ -1817,7 +1819,7 @@
       </c>
       <c r="C35" s="21" t="inlineStr">
         <is>
-          <t>디에이테크놀로지</t>
+          <t>태양광</t>
         </is>
       </c>
       <c r="D35" s="20" t="n">
@@ -1832,27 +1834,25 @@
       <c r="G35" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H35" s="22" t="n">
-        <v>-96.68000000000001</v>
-      </c>
-      <c r="I35" s="22" t="n">
-        <v>-96.68000000000001</v>
-      </c>
-      <c r="J35" s="23" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +593% / 중요공시 2건</t>
-        </is>
-      </c>
-      <c r="K35" s="23" t="inlineStr">
-        <is>
-          <t>공시, 네이버</t>
-        </is>
+      <c r="H35" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I35" s="20" t="n">
+        <v/>
+      </c>
+      <c r="J35" s="24" t="inlineStr">
+        <is>
+          <t>매일경제 기사 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K35" s="24" t="n">
+        <v/>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="20" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B36" s="20" t="n">
@@ -1860,7 +1860,7 @@
       </c>
       <c r="C36" s="21" t="inlineStr">
         <is>
-          <t>와이즈플래닛컴퍼니</t>
+          <t>엔터</t>
         </is>
       </c>
       <c r="D36" s="20" t="n">
@@ -1881,316 +1881,322 @@
       <c r="I36" s="20" t="n">
         <v/>
       </c>
-      <c r="J36" s="23" t="inlineStr">
-        <is>
-          <t>매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K36" s="23" t="n">
-        <v/>
+      <c r="J36" s="24" t="inlineStr">
+        <is>
+          <t>매일경제 헤드라인 언급 / 네이버뉴스 기사 언급</t>
+        </is>
+      </c>
+      <c r="K36" s="24" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
-      <c r="A37" s="20" t="inlineStr">
-        <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-      <c r="B37" s="20" t="n">
+      <c r="A37" s="25" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B37" s="25" t="n">
         <v>24</v>
       </c>
-      <c r="C37" s="21" t="inlineStr">
-        <is>
-          <t>삼일씨엔에스</t>
-        </is>
-      </c>
-      <c r="D37" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E37" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="F37" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G37" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="H37" s="24" t="n">
-        <v>5.45</v>
-      </c>
-      <c r="I37" s="24" t="n">
-        <v>9.49</v>
-      </c>
-      <c r="J37" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 2건 / 중요공시 7일 +100%</t>
-        </is>
-      </c>
-      <c r="K37" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
+      <c r="C37" s="26" t="inlineStr">
+        <is>
+          <t>한국제17호스팩</t>
+        </is>
+      </c>
+      <c r="D37" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E37" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F37" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H37" s="27" t="n">
+        <v>-1.91</v>
+      </c>
+      <c r="I37" s="27" t="n">
+        <v>-1.91</v>
+      </c>
+      <c r="J37" s="28" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +4732%</t>
+        </is>
+      </c>
+      <c r="K37" s="28" t="inlineStr">
+        <is>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
-      <c r="A38" s="20" t="inlineStr">
-        <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-      <c r="B38" s="20" t="n">
+      <c r="A38" s="25" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B38" s="25" t="n">
         <v>25</v>
       </c>
-      <c r="C38" s="21" t="inlineStr">
-        <is>
-          <t>비에이치아이</t>
-        </is>
-      </c>
-      <c r="D38" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E38" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="F38" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G38" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="H38" s="22" t="n">
-        <v>-5.76</v>
-      </c>
-      <c r="I38" s="22" t="n">
-        <v>-4.57</v>
-      </c>
-      <c r="J38" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 2건 / 중요공시 7일 +100%</t>
-        </is>
-      </c>
-      <c r="K38" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
+      <c r="C38" s="26" t="inlineStr">
+        <is>
+          <t>KB제34호스팩</t>
+        </is>
+      </c>
+      <c r="D38" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E38" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F38" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G38" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H38" s="27" t="n">
+        <v>-0.37</v>
+      </c>
+      <c r="I38" s="27" t="n">
+        <v>-0.37</v>
+      </c>
+      <c r="J38" s="28" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +3142%</t>
+        </is>
+      </c>
+      <c r="K38" s="28" t="inlineStr">
+        <is>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
-      <c r="A39" s="20" t="inlineStr">
-        <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-      <c r="B39" s="20" t="n">
+      <c r="A39" s="25" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B39" s="25" t="n">
         <v>26</v>
       </c>
-      <c r="C39" s="21" t="inlineStr">
-        <is>
-          <t>삼성제약</t>
-        </is>
-      </c>
-      <c r="D39" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E39" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F39" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G39" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H39" s="22" t="n">
-        <v>-2.66</v>
-      </c>
-      <c r="I39" s="22" t="n">
-        <v>-8.380000000000001</v>
-      </c>
-      <c r="J39" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K39" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
+      <c r="C39" s="26" t="inlineStr">
+        <is>
+          <t>네오사피엔스</t>
+        </is>
+      </c>
+      <c r="D39" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E39" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F39" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G39" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H39" s="27" t="n">
+        <v>-16.78</v>
+      </c>
+      <c r="I39" s="27" t="n">
+        <v>-32.79</v>
+      </c>
+      <c r="J39" s="28" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +961%</t>
+        </is>
+      </c>
+      <c r="K39" s="28" t="inlineStr">
+        <is>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
-      <c r="A40" s="20" t="inlineStr">
-        <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-      <c r="B40" s="20" t="n">
+      <c r="A40" s="25" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B40" s="25" t="n">
         <v>27</v>
       </c>
-      <c r="C40" s="21" t="inlineStr">
-        <is>
-          <t>GS</t>
-        </is>
-      </c>
-      <c r="D40" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E40" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F40" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G40" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H40" s="24" t="n">
-        <v>0.91</v>
-      </c>
-      <c r="I40" s="22" t="n">
-        <v>-0.72</v>
-      </c>
-      <c r="J40" s="23" t="inlineStr">
-        <is>
-          <t>네이버뉴스 기사 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K40" s="23" t="inlineStr">
+      <c r="C40" s="26" t="inlineStr">
+        <is>
+          <t>동국생명과학</t>
+        </is>
+      </c>
+      <c r="D40" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E40" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F40" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G40" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H40" s="27" t="n">
+        <v>-9.06</v>
+      </c>
+      <c r="I40" s="29" t="n">
+        <v>18.45</v>
+      </c>
+      <c r="J40" s="28" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +618%</t>
+        </is>
+      </c>
+      <c r="K40" s="28" t="inlineStr">
         <is>
           <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
-      <c r="A41" s="20" t="inlineStr">
-        <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-      <c r="B41" s="20" t="n">
+      <c r="A41" s="25" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B41" s="25" t="n">
         <v>28</v>
       </c>
-      <c r="C41" s="21" t="inlineStr">
-        <is>
-          <t>방산</t>
-        </is>
-      </c>
-      <c r="D41" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E41" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F41" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G41" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H41" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I41" s="20" t="n">
-        <v/>
-      </c>
-      <c r="J41" s="23" t="inlineStr">
-        <is>
-          <t>매일경제 기사 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K41" s="23" t="n">
-        <v/>
+      <c r="C41" s="26" t="inlineStr">
+        <is>
+          <t>토마토시스템</t>
+        </is>
+      </c>
+      <c r="D41" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E41" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F41" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G41" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H41" s="29" t="n">
+        <v>12.07</v>
+      </c>
+      <c r="I41" s="29" t="n">
+        <v>71.98999999999999</v>
+      </c>
+      <c r="J41" s="28" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +524%</t>
+        </is>
+      </c>
+      <c r="K41" s="28" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
-      <c r="A42" s="20" t="inlineStr">
-        <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-      <c r="B42" s="20" t="n">
+      <c r="A42" s="25" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B42" s="25" t="n">
         <v>29</v>
       </c>
-      <c r="C42" s="21" t="inlineStr">
-        <is>
-          <t>엔터</t>
-        </is>
-      </c>
-      <c r="D42" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E42" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F42" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G42" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H42" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I42" s="20" t="n">
-        <v/>
-      </c>
-      <c r="J42" s="23" t="inlineStr">
-        <is>
-          <t>매일경제 헤드라인 언급 / 네이버뉴스 기사 언급</t>
-        </is>
-      </c>
-      <c r="K42" s="23" t="inlineStr">
+      <c r="C42" s="26" t="inlineStr">
+        <is>
+          <t>노타</t>
+        </is>
+      </c>
+      <c r="D42" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E42" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F42" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G42" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H42" s="27" t="n">
+        <v>-9.529999999999999</v>
+      </c>
+      <c r="I42" s="29" t="n">
+        <v>17.85</v>
+      </c>
+      <c r="J42" s="28" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +176%</t>
+        </is>
+      </c>
+      <c r="K42" s="28" t="inlineStr">
         <is>
           <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
-      <c r="A43" s="20" t="inlineStr">
-        <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-      <c r="B43" s="20" t="n">
+      <c r="A43" s="25" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B43" s="25" t="n">
         <v>30</v>
       </c>
-      <c r="C43" s="21" t="inlineStr">
-        <is>
-          <t>스테이블코인</t>
-        </is>
-      </c>
-      <c r="D43" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E43" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F43" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G43" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H43" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I43" s="20" t="n">
-        <v/>
-      </c>
-      <c r="J43" s="23" t="inlineStr">
-        <is>
-          <t>한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K43" s="23" t="n">
-        <v/>
+      <c r="C43" s="26" t="inlineStr">
+        <is>
+          <t>삼기에너지솔루션즈</t>
+        </is>
+      </c>
+      <c r="D43" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E43" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F43" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G43" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H43" s="29" t="n">
+        <v>18.12</v>
+      </c>
+      <c r="I43" s="29" t="n">
+        <v>20.69</v>
+      </c>
+      <c r="J43" s="28" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +168%</t>
+        </is>
+      </c>
+      <c r="K43" s="28" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B44" s="25" t="n">
@@ -2198,7 +2204,7 @@
       </c>
       <c r="C44" s="26" t="inlineStr">
         <is>
-          <t>한국제17호스팩</t>
+          <t>HT로보틱스</t>
         </is>
       </c>
       <c r="D44" s="25" t="n">
@@ -2213,15 +2219,15 @@
       <c r="G44" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H44" s="27" t="n">
-        <v>-1.91</v>
-      </c>
-      <c r="I44" s="27" t="n">
-        <v>-1.91</v>
+      <c r="H44" s="29" t="n">
+        <v>30.09</v>
+      </c>
+      <c r="I44" s="29" t="n">
+        <v>25.86</v>
       </c>
       <c r="J44" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +4696%</t>
+          <t>네이버 검색 당일 +143%</t>
         </is>
       </c>
       <c r="K44" s="28" t="inlineStr">
@@ -2233,7 +2239,7 @@
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B45" s="25" t="n">
@@ -2241,7 +2247,7 @@
       </c>
       <c r="C45" s="26" t="inlineStr">
         <is>
-          <t>KB제34호스팩</t>
+          <t>더블유에스아이</t>
         </is>
       </c>
       <c r="D45" s="25" t="n">
@@ -2257,14 +2263,14 @@
         <v>0</v>
       </c>
       <c r="H45" s="27" t="n">
-        <v>-0.37</v>
-      </c>
-      <c r="I45" s="27" t="n">
-        <v>-0.37</v>
+        <v>-11.72</v>
+      </c>
+      <c r="I45" s="29" t="n">
+        <v>17.69</v>
       </c>
       <c r="J45" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +3123%</t>
+          <t>네이버 검색 당일 +116%</t>
         </is>
       </c>
       <c r="K45" s="28" t="inlineStr">
@@ -2276,7 +2282,7 @@
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B46" s="25" t="n">
@@ -2284,7 +2290,7 @@
       </c>
       <c r="C46" s="26" t="inlineStr">
         <is>
-          <t>동국생명과학</t>
+          <t>에이에프더블류</t>
         </is>
       </c>
       <c r="D46" s="25" t="n">
@@ -2299,27 +2305,27 @@
       <c r="G46" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H46" s="27" t="n">
-        <v>-9.06</v>
-      </c>
-      <c r="I46" s="29" t="n">
-        <v>20.52</v>
+      <c r="H46" s="29" t="n">
+        <v>19.1</v>
+      </c>
+      <c r="I46" s="27" t="n">
+        <v>-7.02</v>
       </c>
       <c r="J46" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +596%</t>
+          <t>네이버 검색 당일 +53% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K46" s="28" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B47" s="25" t="n">
@@ -2327,7 +2333,7 @@
       </c>
       <c r="C47" s="26" t="inlineStr">
         <is>
-          <t>토마토시스템</t>
+          <t>한화솔루션</t>
         </is>
       </c>
       <c r="D47" s="25" t="n">
@@ -2343,26 +2349,24 @@
         <v>0</v>
       </c>
       <c r="H47" s="29" t="n">
-        <v>12.07</v>
+        <v>6.52</v>
       </c>
       <c r="I47" s="29" t="n">
-        <v>65.84999999999999</v>
+        <v>2.62</v>
       </c>
       <c r="J47" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +507%</t>
-        </is>
-      </c>
-      <c r="K47" s="28" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+          <t>한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K47" s="28" t="n">
+        <v/>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B48" s="25" t="n">
@@ -2370,7 +2374,7 @@
       </c>
       <c r="C48" s="26" t="inlineStr">
         <is>
-          <t>노타</t>
+          <t>더코디</t>
         </is>
       </c>
       <c r="D48" s="25" t="n">
@@ -2385,27 +2389,27 @@
       <c r="G48" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H48" s="27" t="n">
-        <v>-9.529999999999999</v>
-      </c>
-      <c r="I48" s="29" t="n">
-        <v>21.21</v>
+      <c r="H48" s="29" t="n">
+        <v>5.14</v>
+      </c>
+      <c r="I48" s="27" t="n">
+        <v>-43.87</v>
       </c>
       <c r="J48" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +166%</t>
+          <t>중요공시 3건</t>
         </is>
       </c>
       <c r="K48" s="28" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B49" s="25" t="n">
@@ -2413,7 +2417,7 @@
       </c>
       <c r="C49" s="26" t="inlineStr">
         <is>
-          <t>삼기에너지솔루션즈</t>
+          <t>비케이홀딩스</t>
         </is>
       </c>
       <c r="D49" s="25" t="n">
@@ -2428,27 +2432,27 @@
       <c r="G49" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H49" s="29" t="n">
-        <v>18.12</v>
-      </c>
-      <c r="I49" s="29" t="n">
-        <v>21.39</v>
+      <c r="H49" s="27" t="n">
+        <v>-15.35</v>
+      </c>
+      <c r="I49" s="27" t="n">
+        <v>-17.3</v>
       </c>
       <c r="J49" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +153%</t>
+          <t>중요공시 3건</t>
         </is>
       </c>
       <c r="K49" s="28" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B50" s="25" t="n">
@@ -2456,7 +2460,7 @@
       </c>
       <c r="C50" s="26" t="inlineStr">
         <is>
-          <t>HT로보틱스</t>
+          <t>넥사다이내믹스</t>
         </is>
       </c>
       <c r="D50" s="25" t="n">
@@ -2472,26 +2476,26 @@
         <v>0</v>
       </c>
       <c r="H50" s="29" t="n">
-        <v>30.09</v>
-      </c>
-      <c r="I50" s="29" t="n">
-        <v>28.42</v>
+        <v>0.41</v>
+      </c>
+      <c r="I50" s="27" t="n">
+        <v>-6.74</v>
       </c>
       <c r="J50" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +120%</t>
+          <t>중요공시 3건</t>
         </is>
       </c>
       <c r="K50" s="28" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B51" s="25" t="n">
@@ -2499,7 +2503,7 @@
       </c>
       <c r="C51" s="26" t="inlineStr">
         <is>
-          <t>더블유에스아이</t>
+          <t>서희건설</t>
         </is>
       </c>
       <c r="D51" s="25" t="n">
@@ -2515,26 +2519,26 @@
         <v>0</v>
       </c>
       <c r="H51" s="27" t="n">
-        <v>-11.72</v>
-      </c>
-      <c r="I51" s="29" t="n">
-        <v>20.18</v>
+        <v>-1.3</v>
+      </c>
+      <c r="I51" s="27" t="n">
+        <v>-3.4</v>
       </c>
       <c r="J51" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +110%</t>
+          <t>중요공시 3건</t>
         </is>
       </c>
       <c r="K51" s="28" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B52" s="25" t="n">
@@ -2542,40 +2546,42 @@
       </c>
       <c r="C52" s="26" t="inlineStr">
         <is>
-          <t>한화솔루션</t>
+          <t>현대로템</t>
         </is>
       </c>
       <c r="D52" s="25" t="n">
         <v>3</v>
       </c>
       <c r="E52" s="25" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F52" s="25" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G52" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H52" s="29" t="n">
-        <v>6.52</v>
-      </c>
-      <c r="I52" s="29" t="n">
-        <v>2.62</v>
+      <c r="H52" s="27" t="n">
+        <v>-1.19</v>
+      </c>
+      <c r="I52" s="27" t="n">
+        <v>-5.04</v>
       </c>
       <c r="J52" s="28" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K52" s="28" t="n">
-        <v/>
+          <t>중요공시 2건 / 중요공시 3일 +100%</t>
+        </is>
+      </c>
+      <c r="K52" s="28" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="53" ht="18" customHeight="1">
       <c r="A53" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B53" s="25" t="n">
@@ -2583,7 +2589,7 @@
       </c>
       <c r="C53" s="26" t="inlineStr">
         <is>
-          <t>SK하이닉스</t>
+          <t>현대차</t>
         </is>
       </c>
       <c r="D53" s="25" t="n">
@@ -2598,27 +2604,25 @@
       <c r="G53" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H53" s="29" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="I53" s="29" t="n">
-        <v>6.03</v>
+      <c r="H53" s="27" t="n">
+        <v>-1.38</v>
+      </c>
+      <c r="I53" s="27" t="n">
+        <v>-2.06</v>
       </c>
       <c r="J53" s="28" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K53" s="28" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+          <t>매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K53" s="28" t="n">
+        <v/>
       </c>
     </row>
     <row r="54" ht="18" customHeight="1">
       <c r="A54" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B54" s="25" t="n">
@@ -2626,7 +2630,7 @@
       </c>
       <c r="C54" s="26" t="inlineStr">
         <is>
-          <t>더코디</t>
+          <t>조선</t>
         </is>
       </c>
       <c r="D54" s="25" t="n">
@@ -2641,27 +2645,27 @@
       <c r="G54" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H54" s="29" t="n">
-        <v>5.14</v>
-      </c>
-      <c r="I54" s="27" t="n">
-        <v>-40.85</v>
+      <c r="H54" s="25" t="n">
+        <v/>
+      </c>
+      <c r="I54" s="25" t="n">
+        <v/>
       </c>
       <c r="J54" s="28" t="inlineStr">
         <is>
-          <t>중요공시 3건</t>
+          <t>네이버뉴스 헤드라인 언급</t>
         </is>
       </c>
       <c r="K54" s="28" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="55" ht="18" customHeight="1">
       <c r="A55" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B55" s="25" t="n">
@@ -2669,7 +2673,7 @@
       </c>
       <c r="C55" s="26" t="inlineStr">
         <is>
-          <t>비케이홀딩스</t>
+          <t>OCI홀딩스</t>
         </is>
       </c>
       <c r="D55" s="25" t="n">
@@ -2684,27 +2688,25 @@
       <c r="G55" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H55" s="27" t="n">
-        <v>-15.35</v>
-      </c>
-      <c r="I55" s="27" t="n">
-        <v>-17.21</v>
+      <c r="H55" s="29" t="n">
+        <v>9.720000000000001</v>
+      </c>
+      <c r="I55" s="29" t="n">
+        <v>1.72</v>
       </c>
       <c r="J55" s="28" t="inlineStr">
         <is>
-          <t>중요공시 3건</t>
-        </is>
-      </c>
-      <c r="K55" s="28" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K55" s="28" t="n">
+        <v/>
       </c>
     </row>
     <row r="56" ht="18" customHeight="1">
       <c r="A56" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B56" s="25" t="n">
@@ -2712,7 +2714,7 @@
       </c>
       <c r="C56" s="26" t="inlineStr">
         <is>
-          <t>넥사다이내믹스</t>
+          <t>한국콜마</t>
         </is>
       </c>
       <c r="D56" s="25" t="n">
@@ -2728,26 +2730,26 @@
         <v>0</v>
       </c>
       <c r="H56" s="29" t="n">
-        <v>0.41</v>
+        <v>0.48</v>
       </c>
       <c r="I56" s="27" t="n">
-        <v>-5.05</v>
+        <v>-0.88</v>
       </c>
       <c r="J56" s="28" t="inlineStr">
         <is>
-          <t>중요공시 3건</t>
+          <t>네이버뉴스 헤드라인 언급</t>
         </is>
       </c>
       <c r="K56" s="28" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="57" ht="18" customHeight="1">
       <c r="A57" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B57" s="25" t="n">
@@ -2755,42 +2757,42 @@
       </c>
       <c r="C57" s="26" t="inlineStr">
         <is>
-          <t>현대로템</t>
+          <t>HLB</t>
         </is>
       </c>
       <c r="D57" s="25" t="n">
         <v>3</v>
       </c>
       <c r="E57" s="25" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F57" s="25" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G57" s="25" t="n">
         <v>0</v>
       </c>
       <c r="H57" s="27" t="n">
-        <v>-1.19</v>
+        <v>-0.32</v>
       </c>
       <c r="I57" s="27" t="n">
-        <v>-2.59</v>
+        <v>-2.36</v>
       </c>
       <c r="J57" s="28" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 3일 +100%</t>
+          <t>네이버뉴스 헤드라인 언급</t>
         </is>
       </c>
       <c r="K57" s="28" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="58" ht="18" customHeight="1">
       <c r="A58" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B58" s="25" t="n">
@@ -2798,7 +2800,7 @@
       </c>
       <c r="C58" s="26" t="inlineStr">
         <is>
-          <t>포스코퓨처엠</t>
+          <t>SK스퀘어</t>
         </is>
       </c>
       <c r="D58" s="25" t="n">
@@ -2813,27 +2815,25 @@
       <c r="G58" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H58" s="27" t="n">
-        <v>-2.96</v>
-      </c>
-      <c r="I58" s="27" t="n">
-        <v>-4.24</v>
+      <c r="H58" s="29" t="n">
+        <v>4.14</v>
+      </c>
+      <c r="I58" s="29" t="n">
+        <v>15.9</v>
       </c>
       <c r="J58" s="28" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K58" s="28" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K58" s="28" t="n">
+        <v/>
       </c>
     </row>
     <row r="59" ht="18" customHeight="1">
       <c r="A59" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B59" s="25" t="n">
@@ -2841,7 +2841,7 @@
       </c>
       <c r="C59" s="26" t="inlineStr">
         <is>
-          <t>파두</t>
+          <t>대성하이텍</t>
         </is>
       </c>
       <c r="D59" s="25" t="n">
@@ -2857,26 +2857,24 @@
         <v>0</v>
       </c>
       <c r="H59" s="29" t="n">
-        <v>12.59</v>
+        <v>15.65</v>
       </c>
       <c r="I59" s="29" t="n">
-        <v>37.27</v>
+        <v>19.29</v>
       </c>
       <c r="J59" s="28" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K59" s="28" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+          <t>매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K59" s="28" t="n">
+        <v/>
       </c>
     </row>
     <row r="60" ht="18" customHeight="1">
       <c r="A60" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B60" s="25" t="n">
@@ -2884,7 +2882,7 @@
       </c>
       <c r="C60" s="26" t="inlineStr">
         <is>
-          <t>이수페타시스</t>
+          <t>원전</t>
         </is>
       </c>
       <c r="D60" s="25" t="n">
@@ -2899,27 +2897,25 @@
       <c r="G60" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H60" s="29" t="n">
-        <v>5.02</v>
-      </c>
-      <c r="I60" s="29" t="n">
-        <v>10.88</v>
+      <c r="H60" s="25" t="n">
+        <v/>
+      </c>
+      <c r="I60" s="25" t="n">
+        <v/>
       </c>
       <c r="J60" s="28" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K60" s="28" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+          <t>매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K60" s="28" t="n">
+        <v/>
       </c>
     </row>
     <row r="61" ht="18" customHeight="1">
       <c r="A61" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B61" s="25" t="n">
@@ -2927,7 +2923,7 @@
       </c>
       <c r="C61" s="26" t="inlineStr">
         <is>
-          <t>테스</t>
+          <t>기아</t>
         </is>
       </c>
       <c r="D61" s="25" t="n">
@@ -2942,15 +2938,15 @@
       <c r="G61" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H61" s="29" t="n">
-        <v>8.949999999999999</v>
-      </c>
-      <c r="I61" s="29" t="n">
-        <v>19.31</v>
+      <c r="H61" s="27" t="n">
+        <v>-2.35</v>
+      </c>
+      <c r="I61" s="27" t="n">
+        <v>-4.28</v>
       </c>
       <c r="J61" s="28" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급</t>
+          <t>한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K61" s="28" t="n">
@@ -2960,7 +2956,7 @@
     <row r="62" ht="18" customHeight="1">
       <c r="A62" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B62" s="25" t="n">
@@ -2968,7 +2964,7 @@
       </c>
       <c r="C62" s="26" t="inlineStr">
         <is>
-          <t>OCI홀딩스</t>
+          <t>하이브</t>
         </is>
       </c>
       <c r="D62" s="25" t="n">
@@ -2984,10 +2980,10 @@
         <v>0</v>
       </c>
       <c r="H62" s="29" t="n">
-        <v>9.720000000000001</v>
-      </c>
-      <c r="I62" s="29" t="n">
-        <v>2.48</v>
+        <v>0.38</v>
+      </c>
+      <c r="I62" s="27" t="n">
+        <v>-5.51</v>
       </c>
       <c r="J62" s="28" t="inlineStr">
         <is>
@@ -3001,7 +2997,7 @@
     <row r="63" ht="18" customHeight="1">
       <c r="A63" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B63" s="25" t="n">
@@ -3009,7 +3005,7 @@
       </c>
       <c r="C63" s="26" t="inlineStr">
         <is>
-          <t>한국콜마</t>
+          <t>아모텍</t>
         </is>
       </c>
       <c r="D63" s="25" t="n">
@@ -3024,21 +3020,19 @@
       <c r="G63" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H63" s="29" t="n">
-        <v>0.48</v>
-      </c>
-      <c r="I63" s="27" t="n">
-        <v>-2.33</v>
+      <c r="H63" s="27" t="n">
+        <v>-0.31</v>
+      </c>
+      <c r="I63" s="29" t="n">
+        <v>20.99</v>
       </c>
       <c r="J63" s="28" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K63" s="28" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+          <t>매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K63" s="28" t="n">
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -3134,22 +3128,22 @@
         <v>1</v>
       </c>
       <c r="C3" s="25" t="n">
-        <v>55</v>
+        <v>43</v>
       </c>
       <c r="D3" s="25" t="n">
-        <v>55</v>
+        <v>43</v>
       </c>
       <c r="E3" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F3" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="G3" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="H3" s="25" t="n"/>
@@ -3165,57 +3159,57 @@
         <v>1</v>
       </c>
       <c r="C4" s="25" t="n">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="D4" s="25" t="n">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="E4" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F4" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="G4" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="H4" s="29" t="n">
         <v>3.24</v>
       </c>
       <c r="I4" s="29" t="n">
-        <v>13.02</v>
+        <v>11.91</v>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="26" t="inlineStr">
         <is>
-          <t>인공지능</t>
+          <t>게임</t>
         </is>
       </c>
       <c r="B5" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="25" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="D5" s="25" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E5" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F5" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="G5" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="H5" s="25" t="n"/>
@@ -3224,29 +3218,29 @@
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="26" t="inlineStr">
         <is>
-          <t>게임</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="B6" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="25" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D6" s="25" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E6" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F6" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="G6" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="H6" s="25" t="n"/>
@@ -3255,7 +3249,7 @@
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="26" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="B7" s="25" t="n">
@@ -3272,12 +3266,12 @@
       </c>
       <c r="F7" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="G7" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="H7" s="25" t="n"/>
@@ -3303,25 +3297,25 @@
       </c>
       <c r="F8" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="G8" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="H8" s="27" t="n">
         <v>-0.47</v>
       </c>
       <c r="I8" s="29" t="n">
-        <v>7.69</v>
+        <v>6.6</v>
       </c>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="26" t="inlineStr">
         <is>
-          <t>스피어</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="B9" s="25" t="n">
@@ -3338,60 +3332,56 @@
       </c>
       <c r="F9" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="G9" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-      <c r="H9" s="29" t="n">
-        <v>3.76</v>
-      </c>
-      <c r="I9" s="29" t="n">
-        <v>15.23</v>
-      </c>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="H9" s="25" t="n"/>
+      <c r="I9" s="25" t="n"/>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="26" t="inlineStr">
         <is>
-          <t>HJ중공업</t>
+          <t>스피어</t>
         </is>
       </c>
       <c r="B10" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C10" s="25" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D10" s="25" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E10" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F10" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="G10" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-      <c r="H10" s="27" t="n">
-        <v>-1.78</v>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="H10" s="29" t="n">
+        <v>3.76</v>
       </c>
       <c r="I10" s="27" t="n">
-        <v>-0.67</v>
+        <v>-2.7</v>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="26" t="inlineStr">
         <is>
-          <t>대양금속</t>
+          <t>HJ중공업</t>
         </is>
       </c>
       <c r="B11" s="25" t="n">
@@ -3408,25 +3398,25 @@
       </c>
       <c r="F11" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="G11" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="H11" s="27" t="n">
-        <v>-14.85</v>
+        <v>-1.78</v>
       </c>
       <c r="I11" s="27" t="n">
-        <v>-11.08</v>
+        <v>-5.1</v>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="26" t="inlineStr">
         <is>
-          <t>셀리드</t>
+          <t>SK하이닉스</t>
         </is>
       </c>
       <c r="B12" s="25" t="n">
@@ -3443,56 +3433,60 @@
       </c>
       <c r="F12" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="G12" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-      <c r="H12" s="27" t="n">
-        <v>-9.710000000000001</v>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="H12" s="29" t="n">
+        <v>1.2</v>
       </c>
       <c r="I12" s="29" t="n">
-        <v>17.08</v>
+        <v>5.49</v>
       </c>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>태양광</t>
+          <t>LG전자</t>
         </is>
       </c>
       <c r="B13" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C13" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D13" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E13" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F13" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="G13" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-      <c r="H13" s="25" t="n"/>
-      <c r="I13" s="25" t="n"/>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="H13" s="27" t="n">
+        <v>-2.09</v>
+      </c>
+      <c r="I13" s="29" t="n">
+        <v>5.57</v>
+      </c>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>LG전자</t>
+          <t>바이오</t>
         </is>
       </c>
       <c r="B14" s="25" t="n">
@@ -3509,113 +3503,113 @@
       </c>
       <c r="F14" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="G14" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-      <c r="H14" s="27" t="n">
-        <v>-2.09</v>
-      </c>
-      <c r="I14" s="29" t="n">
-        <v>5.46</v>
-      </c>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="H14" s="25" t="n"/>
+      <c r="I14" s="25" t="n"/>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>네오사피엔스</t>
+          <t>대양금속</t>
         </is>
       </c>
       <c r="B15" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C15" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D15" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E15" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F15" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="G15" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="H15" s="27" t="n">
-        <v>-16.78</v>
+        <v>-14.85</v>
       </c>
       <c r="I15" s="27" t="n">
-        <v>-32.79</v>
+        <v>-12.69</v>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>셀리드</t>
         </is>
       </c>
       <c r="B16" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C16" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D16" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E16" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F16" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="G16" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-      <c r="H16" s="25" t="n"/>
-      <c r="I16" s="25" t="n"/>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="H16" s="27" t="n">
+        <v>-9.710000000000001</v>
+      </c>
+      <c r="I16" s="29" t="n">
+        <v>13.26</v>
+      </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>바이오</t>
+          <t>전기차</t>
         </is>
       </c>
       <c r="B17" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C17" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D17" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E17" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F17" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="G17" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="H17" s="25" t="n"/>
@@ -3624,7 +3618,7 @@
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="26" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>카카오</t>
         </is>
       </c>
       <c r="B18" s="25" t="n">
@@ -3641,21 +3635,25 @@
       </c>
       <c r="F18" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="G18" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-      <c r="H18" s="25" t="n"/>
-      <c r="I18" s="25" t="n"/>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="H18" s="27" t="n">
+        <v>-1.31</v>
+      </c>
+      <c r="I18" s="25" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>서희건설</t>
+          <t>케이쓰리아이</t>
         </is>
       </c>
       <c r="B19" s="25" t="n">
@@ -3672,161 +3670,161 @@
       </c>
       <c r="F19" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="G19" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-      <c r="H19" s="27" t="n">
-        <v>-1.3</v>
-      </c>
-      <c r="I19" s="27" t="n">
-        <v>-2.16</v>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="H19" s="29" t="n">
+        <v>11.96</v>
+      </c>
+      <c r="I19" s="29" t="n">
+        <v>23.71</v>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="26" t="inlineStr">
         <is>
-          <t>원전</t>
+          <t>디에이테크놀로지</t>
         </is>
       </c>
       <c r="B20" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C20" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D20" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E20" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F20" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="G20" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-      <c r="H20" s="25" t="n"/>
-      <c r="I20" s="25" t="n"/>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="H20" s="27" t="n">
+        <v>-96.68000000000001</v>
+      </c>
+      <c r="I20" s="27" t="n">
+        <v>-96.68000000000001</v>
+      </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="26" t="inlineStr">
         <is>
-          <t>카카오</t>
+          <t>삼성제약</t>
         </is>
       </c>
       <c r="B21" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C21" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D21" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E21" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F21" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="G21" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="H21" s="27" t="n">
-        <v>-1.31</v>
-      </c>
-      <c r="I21" s="29" t="n">
-        <v>0.45</v>
+        <v>-2.66</v>
+      </c>
+      <c r="I21" s="27" t="n">
+        <v>-6.91</v>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="26" t="inlineStr">
         <is>
-          <t>케이쓰리아이</t>
+          <t>셀트리온</t>
         </is>
       </c>
       <c r="B22" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C22" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D22" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E22" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F22" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="G22" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-      <c r="H22" s="29" t="n">
-        <v>11.96</v>
-      </c>
-      <c r="I22" s="29" t="n">
-        <v>26.25</v>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="H22" s="27" t="n">
+        <v>-0.11</v>
+      </c>
+      <c r="I22" s="27" t="n">
+        <v>-1.77</v>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="26" t="inlineStr">
         <is>
-          <t>현대건설</t>
+          <t>엔터</t>
         </is>
       </c>
       <c r="B23" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C23" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D23" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E23" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F23" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="G23" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-      <c r="H23" s="27" t="n">
-        <v>-7.21</v>
-      </c>
-      <c r="I23" s="27" t="n">
-        <v>-1.37</v>
-      </c>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="H23" s="25" t="n"/>
+      <c r="I23" s="25" t="n"/>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="26" t="inlineStr">
         <is>
-          <t>GS</t>
+          <t>와이즈플래닛컴퍼니</t>
         </is>
       </c>
       <c r="B24" s="25" t="n">
@@ -3843,25 +3841,21 @@
       </c>
       <c r="F24" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="G24" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-      <c r="H24" s="29" t="n">
-        <v>0.91</v>
-      </c>
-      <c r="I24" s="27" t="n">
-        <v>-0.72</v>
-      </c>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="H24" s="25" t="n"/>
+      <c r="I24" s="25" t="n"/>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="26" t="inlineStr">
         <is>
-          <t>디에이테크놀로지</t>
+          <t>태양광</t>
         </is>
       </c>
       <c r="B25" s="25" t="n">
@@ -3878,254 +3872,266 @@
       </c>
       <c r="F25" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="G25" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-      <c r="H25" s="27" t="n">
-        <v>-96.68000000000001</v>
-      </c>
-      <c r="I25" s="27" t="n">
-        <v>-96.68000000000001</v>
-      </c>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="H25" s="25" t="n"/>
+      <c r="I25" s="25" t="n"/>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="26" t="inlineStr">
         <is>
-          <t>방산</t>
+          <t>HLB</t>
         </is>
       </c>
       <c r="B26" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C26" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D26" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E26" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F26" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="G26" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-      <c r="H26" s="25" t="n"/>
-      <c r="I26" s="25" t="n"/>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="H26" s="27" t="n">
+        <v>-0.32</v>
+      </c>
+      <c r="I26" s="27" t="n">
+        <v>-2.36</v>
+      </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="26" t="inlineStr">
         <is>
-          <t>비에이치아이</t>
+          <t>HT로보틱스</t>
         </is>
       </c>
       <c r="B27" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C27" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D27" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E27" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F27" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="G27" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-      <c r="H27" s="27" t="n">
-        <v>-5.76</v>
-      </c>
-      <c r="I27" s="27" t="n">
-        <v>-4.57</v>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="H27" s="29" t="n">
+        <v>30.09</v>
+      </c>
+      <c r="I27" s="29" t="n">
+        <v>25.86</v>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="26" t="inlineStr">
         <is>
-          <t>삼성제약</t>
+          <t>KB제34호스팩</t>
         </is>
       </c>
       <c r="B28" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C28" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D28" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E28" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F28" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="G28" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="H28" s="27" t="n">
-        <v>-2.66</v>
+        <v>-0.37</v>
       </c>
       <c r="I28" s="27" t="n">
-        <v>-8.380000000000001</v>
+        <v>-0.37</v>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="26" t="inlineStr">
         <is>
-          <t>삼일씨엔에스</t>
+          <t>OCI홀딩스</t>
         </is>
       </c>
       <c r="B29" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C29" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D29" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E29" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F29" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="G29" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="H29" s="29" t="n">
-        <v>5.45</v>
+        <v>9.720000000000001</v>
       </c>
       <c r="I29" s="29" t="n">
-        <v>9.49</v>
+        <v>1.72</v>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="26" t="inlineStr">
         <is>
-          <t>스테이블코인</t>
+          <t>SK스퀘어</t>
         </is>
       </c>
       <c r="B30" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C30" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D30" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E30" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F30" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="G30" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-      <c r="H30" s="25" t="n"/>
-      <c r="I30" s="25" t="n"/>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="H30" s="29" t="n">
+        <v>4.14</v>
+      </c>
+      <c r="I30" s="29" t="n">
+        <v>15.9</v>
+      </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="26" t="inlineStr">
         <is>
-          <t>엔터</t>
+          <t>기아</t>
         </is>
       </c>
       <c r="B31" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C31" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D31" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E31" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F31" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="G31" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-      <c r="H31" s="25" t="n"/>
-      <c r="I31" s="25" t="n"/>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="H31" s="27" t="n">
+        <v>-2.35</v>
+      </c>
+      <c r="I31" s="27" t="n">
+        <v>-4.28</v>
+      </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="26" t="inlineStr">
         <is>
-          <t>와이즈플래닛컴퍼니</t>
+          <t>네오사피엔스</t>
         </is>
       </c>
       <c r="B32" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C32" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D32" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E32" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F32" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="G32" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-      <c r="H32" s="25" t="n"/>
-      <c r="I32" s="25" t="n"/>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="H32" s="27" t="n">
+        <v>-16.78</v>
+      </c>
+      <c r="I32" s="27" t="n">
+        <v>-32.79</v>
+      </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="26" t="inlineStr">
         <is>
-          <t>HT로보틱스</t>
+          <t>넥사다이내믹스</t>
         </is>
       </c>
       <c r="B33" s="25" t="n">
@@ -4142,25 +4148,25 @@
       </c>
       <c r="F33" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="G33" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="H33" s="29" t="n">
-        <v>30.09</v>
-      </c>
-      <c r="I33" s="29" t="n">
-        <v>28.42</v>
+        <v>0.41</v>
+      </c>
+      <c r="I33" s="27" t="n">
+        <v>-6.74</v>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="26" t="inlineStr">
         <is>
-          <t>KB제34호스팩</t>
+          <t>노타</t>
         </is>
       </c>
       <c r="B34" s="25" t="n">
@@ -4177,25 +4183,25 @@
       </c>
       <c r="F34" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="G34" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="H34" s="27" t="n">
-        <v>-0.37</v>
-      </c>
-      <c r="I34" s="27" t="n">
-        <v>-0.37</v>
+        <v>-9.529999999999999</v>
+      </c>
+      <c r="I34" s="29" t="n">
+        <v>17.85</v>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="26" t="inlineStr">
         <is>
-          <t>OCI홀딩스</t>
+          <t>대성하이텍</t>
         </is>
       </c>
       <c r="B35" s="25" t="n">
@@ -4212,25 +4218,25 @@
       </c>
       <c r="F35" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="G35" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="H35" s="29" t="n">
-        <v>9.720000000000001</v>
+        <v>15.65</v>
       </c>
       <c r="I35" s="29" t="n">
-        <v>2.48</v>
+        <v>19.29</v>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="26" t="inlineStr">
         <is>
-          <t>SK하이닉스</t>
+          <t>더블유에스아이</t>
         </is>
       </c>
       <c r="B36" s="25" t="n">
@@ -4247,25 +4253,25 @@
       </c>
       <c r="F36" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="G36" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-      <c r="H36" s="29" t="n">
-        <v>1.2</v>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="H36" s="27" t="n">
+        <v>-11.72</v>
       </c>
       <c r="I36" s="29" t="n">
-        <v>6.03</v>
+        <v>17.69</v>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="26" t="inlineStr">
         <is>
-          <t>넥사다이내믹스</t>
+          <t>더코디</t>
         </is>
       </c>
       <c r="B37" s="25" t="n">
@@ -4282,25 +4288,25 @@
       </c>
       <c r="F37" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="G37" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="H37" s="29" t="n">
-        <v>0.41</v>
+        <v>5.14</v>
       </c>
       <c r="I37" s="27" t="n">
-        <v>-5.05</v>
+        <v>-43.87</v>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="26" t="inlineStr">
         <is>
-          <t>노타</t>
+          <t>동국생명과학</t>
         </is>
       </c>
       <c r="B38" s="25" t="n">
@@ -4317,25 +4323,25 @@
       </c>
       <c r="F38" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="G38" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="H38" s="27" t="n">
-        <v>-9.529999999999999</v>
+        <v>-9.06</v>
       </c>
       <c r="I38" s="29" t="n">
-        <v>21.21</v>
+        <v>18.45</v>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="26" t="inlineStr">
         <is>
-          <t>더블유에스아이</t>
+          <t>비케이홀딩스</t>
         </is>
       </c>
       <c r="B39" s="25" t="n">
@@ -4352,25 +4358,25 @@
       </c>
       <c r="F39" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="G39" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="H39" s="27" t="n">
-        <v>-11.72</v>
-      </c>
-      <c r="I39" s="29" t="n">
-        <v>20.18</v>
+        <v>-15.35</v>
+      </c>
+      <c r="I39" s="27" t="n">
+        <v>-17.3</v>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="26" t="inlineStr">
         <is>
-          <t>더코디</t>
+          <t>삼기에너지솔루션즈</t>
         </is>
       </c>
       <c r="B40" s="25" t="n">
@@ -4387,25 +4393,25 @@
       </c>
       <c r="F40" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="G40" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="H40" s="29" t="n">
-        <v>5.14</v>
-      </c>
-      <c r="I40" s="27" t="n">
-        <v>-40.85</v>
+        <v>18.12</v>
+      </c>
+      <c r="I40" s="29" t="n">
+        <v>20.69</v>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="26" t="inlineStr">
         <is>
-          <t>동국생명과학</t>
+          <t>서희건설</t>
         </is>
       </c>
       <c r="B41" s="25" t="n">
@@ -4422,25 +4428,25 @@
       </c>
       <c r="F41" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="G41" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="H41" s="27" t="n">
-        <v>-9.06</v>
-      </c>
-      <c r="I41" s="29" t="n">
-        <v>20.52</v>
+        <v>-1.3</v>
+      </c>
+      <c r="I41" s="27" t="n">
+        <v>-3.4</v>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="26" t="inlineStr">
         <is>
-          <t>비케이홀딩스</t>
+          <t>아모텍</t>
         </is>
       </c>
       <c r="B42" s="25" t="n">
@@ -4457,25 +4463,25 @@
       </c>
       <c r="F42" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="G42" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="H42" s="27" t="n">
-        <v>-15.35</v>
-      </c>
-      <c r="I42" s="27" t="n">
-        <v>-17.21</v>
+        <v>-0.31</v>
+      </c>
+      <c r="I42" s="29" t="n">
+        <v>20.99</v>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="26" t="inlineStr">
         <is>
-          <t>삼기에너지솔루션즈</t>
+          <t>에이에프더블류</t>
         </is>
       </c>
       <c r="B43" s="25" t="n">
@@ -4492,25 +4498,25 @@
       </c>
       <c r="F43" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="G43" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="H43" s="29" t="n">
-        <v>18.12</v>
-      </c>
-      <c r="I43" s="29" t="n">
-        <v>21.39</v>
+        <v>19.1</v>
+      </c>
+      <c r="I43" s="27" t="n">
+        <v>-7.02</v>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="26" t="inlineStr">
         <is>
-          <t>이수페타시스</t>
+          <t>원전</t>
         </is>
       </c>
       <c r="B44" s="25" t="n">
@@ -4527,25 +4533,21 @@
       </c>
       <c r="F44" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="G44" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-      <c r="H44" s="29" t="n">
-        <v>5.02</v>
-      </c>
-      <c r="I44" s="29" t="n">
-        <v>10.88</v>
-      </c>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="H44" s="25" t="n"/>
+      <c r="I44" s="25" t="n"/>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="26" t="inlineStr">
         <is>
-          <t>테스</t>
+          <t>조선</t>
         </is>
       </c>
       <c r="B45" s="25" t="n">
@@ -4562,20 +4564,16 @@
       </c>
       <c r="F45" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="G45" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-      <c r="H45" s="29" t="n">
-        <v>8.949999999999999</v>
-      </c>
-      <c r="I45" s="29" t="n">
-        <v>19.31</v>
-      </c>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="H45" s="25" t="n"/>
+      <c r="I45" s="25" t="n"/>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="26" t="inlineStr">
@@ -4597,25 +4595,25 @@
       </c>
       <c r="F46" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="G46" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="H46" s="29" t="n">
         <v>12.07</v>
       </c>
       <c r="I46" s="29" t="n">
-        <v>65.84999999999999</v>
+        <v>71.98999999999999</v>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="26" t="inlineStr">
         <is>
-          <t>파두</t>
+          <t>하이브</t>
         </is>
       </c>
       <c r="B47" s="25" t="n">
@@ -4632,25 +4630,25 @@
       </c>
       <c r="F47" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="G47" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="H47" s="29" t="n">
-        <v>12.59</v>
-      </c>
-      <c r="I47" s="29" t="n">
-        <v>37.27</v>
+        <v>0.38</v>
+      </c>
+      <c r="I47" s="27" t="n">
+        <v>-5.51</v>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="26" t="inlineStr">
         <is>
-          <t>포스코퓨처엠</t>
+          <t>한국제17호스팩</t>
         </is>
       </c>
       <c r="B48" s="25" t="n">
@@ -4667,25 +4665,25 @@
       </c>
       <c r="F48" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="G48" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="H48" s="27" t="n">
-        <v>-2.96</v>
+        <v>-1.91</v>
       </c>
       <c r="I48" s="27" t="n">
-        <v>-4.24</v>
+        <v>-1.91</v>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="26" t="inlineStr">
         <is>
-          <t>한국제17호스팩</t>
+          <t>한국콜마</t>
         </is>
       </c>
       <c r="B49" s="25" t="n">
@@ -4702,25 +4700,25 @@
       </c>
       <c r="F49" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="G49" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-      <c r="H49" s="27" t="n">
-        <v>-1.91</v>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="H49" s="29" t="n">
+        <v>0.48</v>
       </c>
       <c r="I49" s="27" t="n">
-        <v>-1.91</v>
+        <v>-0.88</v>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="26" t="inlineStr">
         <is>
-          <t>한국콜마</t>
+          <t>한화솔루션</t>
         </is>
       </c>
       <c r="B50" s="25" t="n">
@@ -4737,25 +4735,25 @@
       </c>
       <c r="F50" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="G50" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="H50" s="29" t="n">
-        <v>0.48</v>
-      </c>
-      <c r="I50" s="27" t="n">
-        <v>-2.33</v>
+        <v>6.52</v>
+      </c>
+      <c r="I50" s="29" t="n">
+        <v>2.62</v>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="26" t="inlineStr">
         <is>
-          <t>한화솔루션</t>
+          <t>현대로템</t>
         </is>
       </c>
       <c r="B51" s="25" t="n">
@@ -4772,25 +4770,25 @@
       </c>
       <c r="F51" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="G51" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-      <c r="H51" s="29" t="n">
-        <v>6.52</v>
-      </c>
-      <c r="I51" s="29" t="n">
-        <v>2.62</v>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="H51" s="27" t="n">
+        <v>-1.19</v>
+      </c>
+      <c r="I51" s="27" t="n">
+        <v>-5.04</v>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="26" t="inlineStr">
         <is>
-          <t>현대로템</t>
+          <t>현대차</t>
         </is>
       </c>
       <c r="B52" s="25" t="n">
@@ -4807,19 +4805,19 @@
       </c>
       <c r="F52" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="G52" s="25" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="H52" s="27" t="n">
-        <v>-1.19</v>
+        <v>-1.38</v>
       </c>
       <c r="I52" s="27" t="n">
-        <v>-2.59</v>
+        <v>-2.06</v>
       </c>
     </row>
   </sheetData>
@@ -4903,19 +4901,19 @@
         <v>1</v>
       </c>
       <c r="C3" s="36" t="n">
-        <v>55</v>
+        <v>43</v>
       </c>
       <c r="D3" s="36" t="n">
-        <v>55</v>
+        <v>43</v>
       </c>
       <c r="E3" s="36" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="F3" s="37" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="G3" s="37" t="inlineStr">
@@ -4941,12 +4939,12 @@
       </c>
       <c r="E4" s="36" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="F4" s="37" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="G4" s="37" t="inlineStr">
@@ -4958,26 +4956,26 @@
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="35" t="inlineStr">
         <is>
-          <t>방산</t>
+          <t>전기차</t>
         </is>
       </c>
       <c r="B5" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="36" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D5" s="36" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E5" s="36" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="F5" s="37" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="G5" s="37" t="inlineStr">
@@ -4996,19 +4994,19 @@
         <v>1</v>
       </c>
       <c r="C6" s="36" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D6" s="36" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E6" s="36" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="F6" s="37" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="G6" s="37" t="inlineStr">
@@ -5027,19 +5025,19 @@
         <v>1</v>
       </c>
       <c r="C7" s="36" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D7" s="36" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E7" s="36" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="F7" s="37" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="G7" s="37" t="inlineStr">
@@ -5058,19 +5056,19 @@
         <v>1</v>
       </c>
       <c r="C8" s="36" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D8" s="36" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E8" s="36" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="F8" s="37" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="G8" s="37" t="inlineStr">
@@ -5096,12 +5094,12 @@
       </c>
       <c r="E9" s="36" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="F9" s="37" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="G9" s="37" t="inlineStr">
@@ -5127,12 +5125,12 @@
       </c>
       <c r="E10" s="36" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="F10" s="37" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="G10" s="37" t="inlineStr">
@@ -5144,26 +5142,26 @@
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="35" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>조선</t>
         </is>
       </c>
       <c r="B11" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="36" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D11" s="36" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="E11" s="36" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="F11" s="37" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="G11" s="37" t="inlineStr">
@@ -5175,65 +5173,69 @@
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="35" t="inlineStr">
         <is>
+          <t>제약</t>
+        </is>
+      </c>
+      <c r="B12" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C12" s="36" t="n">
+        <v>12</v>
+      </c>
+      <c r="D12" s="36" t="n">
+        <v>12</v>
+      </c>
+      <c r="E12" s="36" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="F12" s="37" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="G12" s="37" t="inlineStr">
+        <is>
+          <t>⚡ 관심</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="35" t="inlineStr">
+        <is>
           <t>인공지능</t>
         </is>
       </c>
-      <c r="B12" s="36" t="n">
-        <v>1</v>
-      </c>
-      <c r="C12" s="36" t="n">
-        <v>18</v>
-      </c>
-      <c r="D12" s="36" t="n">
-        <v>18</v>
-      </c>
-      <c r="E12" s="36" t="inlineStr">
-        <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-      <c r="F12" s="37" t="inlineStr">
-        <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-      <c r="G12" s="37" t="inlineStr">
+      <c r="B13" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C13" s="36" t="n">
+        <v>10</v>
+      </c>
+      <c r="D13" s="36" t="n">
+        <v>10</v>
+      </c>
+      <c r="E13" s="36" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="F13" s="37" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="G13" s="37" t="inlineStr">
         <is>
           <t>⚡ 관심</t>
         </is>
       </c>
-    </row>
-    <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="26" t="inlineStr">
-        <is>
-          <t>이차전지</t>
-        </is>
-      </c>
-      <c r="B13" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="C13" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="D13" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="E13" s="25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F13" s="28" t="inlineStr">
-        <is>
-          <t>감지 없음</t>
-        </is>
-      </c>
-      <c r="G13" s="28" t="inlineStr"/>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>AI반도체</t>
+          <t>이차전지</t>
         </is>
       </c>
       <c r="B14" s="25" t="n">
@@ -5260,7 +5262,7 @@
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>전기차</t>
+          <t>AI반도체</t>
         </is>
       </c>
       <c r="B15" s="25" t="n">
@@ -5287,7 +5289,7 @@
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>수소</t>
+          <t>방산</t>
         </is>
       </c>
       <c r="B16" s="25" t="n">
@@ -5314,7 +5316,7 @@
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>핀테크</t>
+          <t>수소</t>
         </is>
       </c>
       <c r="B17" s="25" t="n">
@@ -5341,7 +5343,7 @@
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="26" t="inlineStr">
         <is>
-          <t>클라우드</t>
+          <t>핀테크</t>
         </is>
       </c>
       <c r="B18" s="25" t="n">
@@ -5368,7 +5370,7 @@
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>조선</t>
+          <t>클라우드</t>
         </is>
       </c>
       <c r="B19" s="25" t="n">

</xml_diff>

<commit_message>
auto: 2026-09-30 07:16 자동 백업
</commit_message>
<xml_diff>
--- a/trend/stock_trend_history.xlsx
+++ b/trend/stock_trend_history.xlsx
@@ -57,13 +57,13 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="002563EB"/>
+      <color rgb="00E53935"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00E53935"/>
+      <color rgb="002563EB"/>
       <sz val="10"/>
     </font>
     <font>
@@ -258,13 +258,13 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -694,7 +694,7 @@
     <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-09-29 06:54</t>
+          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-09-30 06:54</t>
         </is>
       </c>
     </row>
@@ -708,7 +708,7 @@
       </c>
       <c r="E3" s="3" t="n"/>
       <c r="G3" s="5" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H3" s="3" t="n"/>
       <c r="J3" s="6" t="n">
@@ -787,21 +787,21 @@
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-09-29) 상위: 반도체  점수 62.0점</t>
+          <t>⚡ 최신(2026-09-30) 상위: 반도체  점수 88.0점</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-09-29) 상위: 바이오  점수 26.0점</t>
+          <t>⚡ 최신(2026-09-30) 상위: 인공지능  점수 29.0점</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-09-29) 상위: 삼성전자  점수 24.0점</t>
+          <t>⚡ 최신(2026-09-30) 상위: 삼성전자  점수 20.0점</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="15" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B14" s="15" t="n">
@@ -928,10 +928,10 @@
         </is>
       </c>
       <c r="D14" s="15" t="n">
-        <v>62</v>
+        <v>88</v>
       </c>
       <c r="E14" s="15" t="n">
-        <v>62</v>
+        <v>88</v>
       </c>
       <c r="F14" s="15" t="n">
         <v>0</v>
@@ -947,7 +947,7 @@
       </c>
       <c r="J14" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 한국경제 헤드라인 언급</t>
+          <t>매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급</t>
         </is>
       </c>
       <c r="K14" s="17" t="inlineStr">
@@ -959,7 +959,7 @@
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="15" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B15" s="15" t="n">
@@ -967,14 +967,14 @@
       </c>
       <c r="C15" s="16" t="inlineStr">
         <is>
-          <t>바이오</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="D15" s="15" t="n">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="E15" s="15" t="n">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="F15" s="15" t="n">
         <v>0</v>
@@ -990,7 +990,7 @@
       </c>
       <c r="J15" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
+          <t>매일경제 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K15" s="17" t="inlineStr">
@@ -1002,7 +1002,7 @@
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="15" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B16" s="15" t="n">
@@ -1014,10 +1014,10 @@
         </is>
       </c>
       <c r="D16" s="15" t="n">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="E16" s="15" t="n">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="F16" s="15" t="n">
         <v>0</v>
@@ -1026,14 +1026,14 @@
         <v>0</v>
       </c>
       <c r="H16" s="18" t="n">
-        <v>-5.76</v>
-      </c>
-      <c r="I16" s="18" t="n">
-        <v>-1.82</v>
+        <v>1.85</v>
+      </c>
+      <c r="I16" s="15" t="n">
+        <v>0</v>
       </c>
       <c r="J16" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+          <t>네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K16" s="17" t="inlineStr">
@@ -1045,7 +1045,7 @@
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B17" s="15" t="n">
@@ -1053,14 +1053,14 @@
       </c>
       <c r="C17" s="16" t="inlineStr">
         <is>
-          <t>HLB</t>
+          <t>삼성전기</t>
         </is>
       </c>
       <c r="D17" s="15" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="E17" s="15" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="F17" s="15" t="n">
         <v>0</v>
@@ -1068,27 +1068,27 @@
       <c r="G17" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H17" s="19" t="n">
-        <v>27.86</v>
-      </c>
-      <c r="I17" s="19" t="n">
-        <v>24.45</v>
+      <c r="H17" s="18" t="n">
+        <v>3.96</v>
+      </c>
+      <c r="I17" s="18" t="n">
+        <v>8.24</v>
       </c>
       <c r="J17" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급</t>
+          <t>중요공시 1건 / 매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K17" s="17" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B18" s="15" t="n">
@@ -1096,7 +1096,7 @@
       </c>
       <c r="C18" s="16" t="inlineStr">
         <is>
-          <t>삼성전기</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="D18" s="15" t="n">
@@ -1111,27 +1111,25 @@
       <c r="G18" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H18" s="18" t="n">
-        <v>-0.67</v>
-      </c>
-      <c r="I18" s="19" t="n">
-        <v>4.12</v>
+      <c r="H18" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I18" s="15" t="n">
+        <v/>
       </c>
       <c r="J18" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K18" s="17" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K18" s="17" t="n">
+        <v/>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B19" s="15" t="n">
@@ -1143,10 +1141,10 @@
         </is>
       </c>
       <c r="D19" s="15" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E19" s="15" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="F19" s="15" t="n">
         <v>0</v>
@@ -1162,7 +1160,7 @@
       </c>
       <c r="J19" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급</t>
+          <t>매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K19" s="17" t="inlineStr">
@@ -1174,7 +1172,7 @@
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B20" s="15" t="n">
@@ -1182,14 +1180,14 @@
       </c>
       <c r="C20" s="16" t="inlineStr">
         <is>
-          <t>인공지능</t>
+          <t>바이오</t>
         </is>
       </c>
       <c r="D20" s="15" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="E20" s="15" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F20" s="15" t="n">
         <v>0</v>
@@ -1205,7 +1203,7 @@
       </c>
       <c r="J20" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+          <t>네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K20" s="17" t="inlineStr">
@@ -1217,7 +1215,7 @@
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="15" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B21" s="15" t="n">
@@ -1229,10 +1227,10 @@
         </is>
       </c>
       <c r="D21" s="15" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E21" s="15" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="F21" s="15" t="n">
         <v>0</v>
@@ -1241,14 +1239,14 @@
         <v>0</v>
       </c>
       <c r="H21" s="18" t="n">
-        <v>-5.48</v>
-      </c>
-      <c r="I21" s="18" t="n">
-        <v>-6.28</v>
+        <v>1.65</v>
+      </c>
+      <c r="I21" s="19" t="n">
+        <v>-4.74</v>
       </c>
       <c r="J21" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K21" s="17" t="inlineStr">
@@ -1260,7 +1258,7 @@
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="15" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B22" s="15" t="n">
@@ -1268,14 +1266,14 @@
       </c>
       <c r="C22" s="16" t="inlineStr">
         <is>
-          <t>태양광</t>
+          <t>LG전자</t>
         </is>
       </c>
       <c r="D22" s="15" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E22" s="15" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F22" s="15" t="n">
         <v>0</v>
@@ -1283,15 +1281,15 @@
       <c r="G22" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H22" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I22" s="15" t="n">
-        <v/>
+      <c r="H22" s="18" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="I22" s="18" t="n">
+        <v>6.4</v>
       </c>
       <c r="J22" s="17" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K22" s="17" t="n">
@@ -1301,7 +1299,7 @@
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="15" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B23" s="15" t="n">
@@ -1309,14 +1307,14 @@
       </c>
       <c r="C23" s="16" t="inlineStr">
         <is>
-          <t>전기차</t>
+          <t>방산</t>
         </is>
       </c>
       <c r="D23" s="15" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E23" s="15" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F23" s="15" t="n">
         <v>0</v>
@@ -1332,19 +1330,17 @@
       </c>
       <c r="J23" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K23" s="17" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+          <t>한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K23" s="17" t="n">
+        <v/>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="15" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B24" s="15" t="n">
@@ -1352,40 +1348,42 @@
       </c>
       <c r="C24" s="16" t="inlineStr">
         <is>
-          <t>OCI홀딩스</t>
+          <t>모아데이타</t>
         </is>
       </c>
       <c r="D24" s="15" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E24" s="15" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="F24" s="15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G24" s="15" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H24" s="19" t="n">
-        <v>12.35</v>
+        <v>-5.96</v>
       </c>
       <c r="I24" s="19" t="n">
-        <v>20.21</v>
+        <v>-22.05</v>
       </c>
       <c r="J24" s="17" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K24" s="17" t="n">
-        <v/>
+          <t>중요공시 4건 / 중요공시 3일 +100% / 중요공시 7일 +300%</t>
+        </is>
+      </c>
+      <c r="K24" s="17" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="15" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B25" s="15" t="n">
@@ -1393,42 +1391,42 @@
       </c>
       <c r="C25" s="16" t="inlineStr">
         <is>
-          <t>현대차</t>
+          <t>셀트리온</t>
         </is>
       </c>
       <c r="D25" s="15" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E25" s="15" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="F25" s="15" t="n">
         <v>0</v>
       </c>
       <c r="G25" s="15" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H25" s="18" t="n">
-        <v>-0.84</v>
-      </c>
-      <c r="I25" s="18" t="n">
-        <v>-2.07</v>
+        <v>0.62</v>
+      </c>
+      <c r="I25" s="19" t="n">
+        <v>-1.49</v>
       </c>
       <c r="J25" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 기사 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+          <t>중요공시 2건 / 중요공시 7일 +100% / 네이버뉴스 기사 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K25" s="17" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="15" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B26" s="15" t="n">
@@ -1436,30 +1434,30 @@
       </c>
       <c r="C26" s="16" t="inlineStr">
         <is>
-          <t>모아데이타</t>
+          <t>뷰노</t>
         </is>
       </c>
       <c r="D26" s="15" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E26" s="15" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="F26" s="15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G26" s="15" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H26" s="18" t="n">
-        <v>-11.38</v>
+        <v>14.92</v>
       </c>
       <c r="I26" s="18" t="n">
-        <v>-17.11</v>
+        <v>52.94</v>
       </c>
       <c r="J26" s="17" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 3일 +50% / 중요공시 7일 +200%</t>
+          <t>중요공시 1건 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K26" s="17" t="inlineStr">
@@ -1471,7 +1469,7 @@
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="15" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B27" s="15" t="n">
@@ -1479,85 +1477,83 @@
       </c>
       <c r="C27" s="16" t="inlineStr">
         <is>
-          <t>핑거</t>
+          <t>조선</t>
         </is>
       </c>
       <c r="D27" s="15" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E27" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="F27" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I27" s="15" t="n">
+        <v/>
+      </c>
+      <c r="J27" s="17" t="inlineStr">
+        <is>
+          <t>네이버뉴스 기사 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K27" s="17" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="18" customHeight="1">
+      <c r="A28" s="20" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B28" s="20" t="n">
+        <v>15</v>
+      </c>
+      <c r="C28" s="21" t="inlineStr">
+        <is>
+          <t>대덕전자</t>
+        </is>
+      </c>
+      <c r="D28" s="20" t="n">
         <v>6</v>
       </c>
-      <c r="F27" s="15" t="n">
-        <v>2</v>
-      </c>
-      <c r="G27" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H27" s="19" t="n">
-        <v>13.82</v>
-      </c>
-      <c r="I27" s="19" t="n">
-        <v>32.43</v>
-      </c>
-      <c r="J27" s="17" t="inlineStr">
-        <is>
-          <t>중요공시 4건 / 중요공시 3일 +100% / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K27" s="17" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="18" customHeight="1">
-      <c r="A28" s="15" t="inlineStr">
-        <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-      <c r="B28" s="15" t="n">
-        <v>15</v>
-      </c>
-      <c r="C28" s="16" t="inlineStr">
-        <is>
-          <t>게임</t>
-        </is>
-      </c>
-      <c r="D28" s="15" t="n">
-        <v>8</v>
-      </c>
-      <c r="E28" s="15" t="n">
-        <v>8</v>
-      </c>
-      <c r="F28" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="G28" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H28" s="15" t="n">
+      <c r="E28" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="F28" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" s="22" t="n">
+        <v>8.710000000000001</v>
+      </c>
+      <c r="I28" s="22" t="n">
+        <v>28.57</v>
+      </c>
+      <c r="J28" s="23" t="inlineStr">
+        <is>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K28" s="23" t="n">
         <v/>
-      </c>
-      <c r="I28" s="15" t="n">
-        <v/>
-      </c>
-      <c r="J28" s="17" t="inlineStr">
-        <is>
-          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K28" s="17" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="20" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B29" s="20" t="n">
@@ -1565,7 +1561,7 @@
       </c>
       <c r="C29" s="21" t="inlineStr">
         <is>
-          <t>한화솔루션</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="D29" s="20" t="n">
@@ -1580,15 +1576,15 @@
       <c r="G29" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H29" s="22" t="n">
-        <v>16.5</v>
-      </c>
-      <c r="I29" s="22" t="n">
-        <v>23.2</v>
+      <c r="H29" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I29" s="20" t="n">
+        <v/>
       </c>
       <c r="J29" s="23" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K29" s="23" t="n">
@@ -1598,7 +1594,7 @@
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="20" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B30" s="20" t="n">
@@ -1606,42 +1602,40 @@
       </c>
       <c r="C30" s="21" t="inlineStr">
         <is>
-          <t>스피어</t>
+          <t>DB</t>
         </is>
       </c>
       <c r="D30" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E30" s="20" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F30" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G30" s="20" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H30" s="24" t="n">
-        <v>-4.9</v>
-      </c>
-      <c r="I30" s="24" t="n">
-        <v>-4.9</v>
+        <v>-0.23</v>
+      </c>
+      <c r="I30" s="22" t="n">
+        <v>6.92</v>
       </c>
       <c r="J30" s="23" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 7일 +200%</t>
-        </is>
-      </c>
-      <c r="K30" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K30" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="20" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B31" s="20" t="n">
@@ -1649,42 +1643,40 @@
       </c>
       <c r="C31" s="21" t="inlineStr">
         <is>
-          <t>삼성제약</t>
+          <t>태양광</t>
         </is>
       </c>
       <c r="D31" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E31" s="20" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F31" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G31" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H31" s="22" t="n">
-        <v>4.38</v>
-      </c>
-      <c r="I31" s="24" t="n">
-        <v>-0.15</v>
+      <c r="H31" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I31" s="20" t="n">
+        <v/>
       </c>
       <c r="J31" s="23" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 3일 +100% / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K31" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K31" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="20" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B32" s="20" t="n">
@@ -1692,30 +1684,30 @@
       </c>
       <c r="C32" s="21" t="inlineStr">
         <is>
-          <t>현대로템</t>
+          <t>더코디</t>
         </is>
       </c>
       <c r="D32" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E32" s="20" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F32" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G32" s="20" t="n">
         <v>0</v>
       </c>
       <c r="H32" s="24" t="n">
-        <v>-0.43</v>
+        <v>-10.85</v>
       </c>
       <c r="I32" s="24" t="n">
-        <v>-3.57</v>
+        <v>-8.130000000000001</v>
       </c>
       <c r="J32" s="23" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+          <t>중요공시 5건 / 중요공시 3일 +67%</t>
         </is>
       </c>
       <c r="K32" s="23" t="inlineStr">
@@ -1727,7 +1719,7 @@
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="20" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B33" s="20" t="n">
@@ -1735,40 +1727,42 @@
       </c>
       <c r="C33" s="21" t="inlineStr">
         <is>
-          <t>기아</t>
+          <t>앤씨앤</t>
         </is>
       </c>
       <c r="D33" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E33" s="20" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F33" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G33" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H33" s="22" t="n">
-        <v>0.77</v>
+      <c r="H33" s="24" t="n">
+        <v>-18.6</v>
       </c>
       <c r="I33" s="24" t="n">
-        <v>-2.74</v>
+        <v>-12.5</v>
       </c>
       <c r="J33" s="23" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K33" s="23" t="n">
-        <v/>
+          <t>중요공시 3건 / 중요공시 3일 +50%</t>
+        </is>
+      </c>
+      <c r="K33" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="20" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B34" s="20" t="n">
@@ -1776,14 +1770,14 @@
       </c>
       <c r="C34" s="21" t="inlineStr">
         <is>
-          <t>수소</t>
+          <t>OCI홀딩스</t>
         </is>
       </c>
       <c r="D34" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E34" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F34" s="20" t="n">
         <v>0</v>
@@ -1791,25 +1785,27 @@
       <c r="G34" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H34" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I34" s="20" t="n">
-        <v/>
+      <c r="H34" s="24" t="n">
+        <v>-5.6</v>
+      </c>
+      <c r="I34" s="22" t="n">
+        <v>13.47</v>
       </c>
       <c r="J34" s="23" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K34" s="23" t="n">
-        <v/>
+          <t>중요공시 1건 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K34" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="20" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B35" s="20" t="n">
@@ -1817,7 +1813,7 @@
       </c>
       <c r="C35" s="21" t="inlineStr">
         <is>
-          <t>셀리드</t>
+          <t>삼성SDI</t>
         </is>
       </c>
       <c r="D35" s="20" t="n">
@@ -1832,27 +1828,25 @@
       <c r="G35" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H35" s="22" t="n">
-        <v>2.11</v>
-      </c>
-      <c r="I35" s="22" t="n">
-        <v>5.98</v>
+      <c r="H35" s="24" t="n">
+        <v>-2.08</v>
+      </c>
+      <c r="I35" s="24" t="n">
+        <v>-3.54</v>
       </c>
       <c r="J35" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +92% / 중요공시 3건</t>
-        </is>
-      </c>
-      <c r="K35" s="23" t="inlineStr">
-        <is>
-          <t>공시, 네이버</t>
-        </is>
+          <t>매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K35" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="20" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B36" s="20" t="n">
@@ -1860,7 +1854,7 @@
       </c>
       <c r="C36" s="21" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>게임</t>
         </is>
       </c>
       <c r="D36" s="20" t="n">
@@ -1875,25 +1869,27 @@
       <c r="G36" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H36" s="22" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="I36" s="22" t="n">
-        <v>5.55</v>
+      <c r="H36" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I36" s="20" t="n">
+        <v/>
       </c>
       <c r="J36" s="23" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K36" s="23" t="n">
-        <v/>
+          <t>네이버뉴스 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K36" s="23" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="20" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B37" s="20" t="n">
@@ -1901,7 +1897,7 @@
       </c>
       <c r="C37" s="21" t="inlineStr">
         <is>
-          <t>방산</t>
+          <t>엔터</t>
         </is>
       </c>
       <c r="D37" s="20" t="n">
@@ -1924,19 +1920,17 @@
       </c>
       <c r="J37" s="23" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 한국경제 헤드라인 언급 / 네이버뉴스 기사 언급</t>
-        </is>
-      </c>
-      <c r="K37" s="23" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K37" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="20" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B38" s="20" t="n">
@@ -1944,14 +1938,14 @@
       </c>
       <c r="C38" s="21" t="inlineStr">
         <is>
-          <t>LG전자</t>
+          <t>테라뷰</t>
         </is>
       </c>
       <c r="D38" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E38" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F38" s="20" t="n">
         <v>0</v>
@@ -1960,24 +1954,26 @@
         <v>0</v>
       </c>
       <c r="H38" s="22" t="n">
-        <v>1.9</v>
+        <v>30.98</v>
       </c>
       <c r="I38" s="22" t="n">
-        <v>5.67</v>
+        <v>23.9</v>
       </c>
       <c r="J38" s="23" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K38" s="23" t="n">
-        <v/>
+          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K38" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="20" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B39" s="20" t="n">
@@ -1985,42 +1981,42 @@
       </c>
       <c r="C39" s="21" t="inlineStr">
         <is>
-          <t>스테이블코인</t>
+          <t>스피어</t>
         </is>
       </c>
       <c r="D39" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E39" s="20" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F39" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G39" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H39" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I39" s="20" t="n">
-        <v/>
+        <v>3</v>
+      </c>
+      <c r="H39" s="24" t="n">
+        <v>-4.26</v>
+      </c>
+      <c r="I39" s="24" t="n">
+        <v>-8.960000000000001</v>
       </c>
       <c r="J39" s="23" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 기사 언급</t>
+          <t>중요공시 2건 / 중요공시 7일 +100%</t>
         </is>
       </c>
       <c r="K39" s="23" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="20" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B40" s="20" t="n">
@@ -2028,7 +2024,7 @@
       </c>
       <c r="C40" s="21" t="inlineStr">
         <is>
-          <t>루닛</t>
+          <t>미래산업</t>
         </is>
       </c>
       <c r="D40" s="20" t="n">
@@ -2044,14 +2040,14 @@
         <v>0</v>
       </c>
       <c r="H40" s="22" t="n">
-        <v>13.78</v>
+        <v>7.68</v>
       </c>
       <c r="I40" s="22" t="n">
-        <v>9.67</v>
+        <v>25.37</v>
       </c>
       <c r="J40" s="23" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 3일 +100%</t>
+          <t>중요공시 2건 / 중요공시 3일 +100% / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K40" s="23" t="inlineStr">
@@ -2063,7 +2059,7 @@
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="20" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B41" s="20" t="n">
@@ -2071,7 +2067,7 @@
       </c>
       <c r="C41" s="21" t="inlineStr">
         <is>
-          <t>에코프로</t>
+          <t>한미반도체</t>
         </is>
       </c>
       <c r="D41" s="20" t="n">
@@ -2087,26 +2083,26 @@
         <v>0</v>
       </c>
       <c r="H41" s="22" t="n">
-        <v>1.5</v>
+        <v>8.15</v>
       </c>
       <c r="I41" s="22" t="n">
-        <v>1.25</v>
+        <v>5.44</v>
       </c>
       <c r="J41" s="23" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 네이버뉴스 헤드라인 언급</t>
+          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K41" s="23" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="20" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B42" s="20" t="n">
@@ -2114,7 +2110,7 @@
       </c>
       <c r="C42" s="21" t="inlineStr">
         <is>
-          <t>KT</t>
+          <t>티로보틱스</t>
         </is>
       </c>
       <c r="D42" s="20" t="n">
@@ -2129,59 +2125,61 @@
       <c r="G42" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H42" s="24" t="n">
-        <v>-0.19</v>
-      </c>
-      <c r="I42" s="24" t="n">
-        <v>-0.9399999999999999</v>
+      <c r="H42" s="22" t="n">
+        <v>5.49</v>
+      </c>
+      <c r="I42" s="22" t="n">
+        <v>12.03</v>
       </c>
       <c r="J42" s="23" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K42" s="23" t="n">
-        <v/>
+          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K42" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
-      <c r="A43" s="25" t="inlineStr">
-        <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-      <c r="B43" s="25" t="n">
+      <c r="A43" s="20" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B43" s="20" t="n">
         <v>30</v>
       </c>
-      <c r="C43" s="26" t="inlineStr">
-        <is>
-          <t>네오사피엔스</t>
-        </is>
-      </c>
-      <c r="D43" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="E43" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="F43" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="G43" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H43" s="27" t="n">
-        <v>-16.94</v>
-      </c>
-      <c r="I43" s="27" t="n">
-        <v>-44.17</v>
-      </c>
-      <c r="J43" s="28" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +986%</t>
-        </is>
-      </c>
-      <c r="K43" s="28" t="inlineStr">
+      <c r="C43" s="21" t="inlineStr">
+        <is>
+          <t>현대차</t>
+        </is>
+      </c>
+      <c r="D43" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="E43" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F43" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G43" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H43" s="24" t="n">
+        <v>-0.99</v>
+      </c>
+      <c r="I43" s="24" t="n">
+        <v>-3.04</v>
+      </c>
+      <c r="J43" s="23" t="inlineStr">
+        <is>
+          <t>네이버뉴스 기사 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K43" s="23" t="inlineStr">
         <is>
           <t>네이버</t>
         </is>
@@ -2190,7 +2188,7 @@
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B44" s="25" t="n">
@@ -2198,7 +2196,7 @@
       </c>
       <c r="C44" s="26" t="inlineStr">
         <is>
-          <t>디에이테크놀로지</t>
+          <t>현대바이오랜드</t>
         </is>
       </c>
       <c r="D44" s="25" t="n">
@@ -2214,14 +2212,14 @@
         <v>0</v>
       </c>
       <c r="H44" s="27" t="n">
-        <v>-30.69</v>
+        <v>25.03</v>
       </c>
       <c r="I44" s="27" t="n">
-        <v>-97.7</v>
+        <v>45.2</v>
       </c>
       <c r="J44" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +690%</t>
+          <t>네이버 검색 당일 +189%</t>
         </is>
       </c>
       <c r="K44" s="28" t="inlineStr">
@@ -2233,7 +2231,7 @@
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B45" s="25" t="n">
@@ -2241,7 +2239,7 @@
       </c>
       <c r="C45" s="26" t="inlineStr">
         <is>
-          <t>동국생명과학</t>
+          <t>베노티앤알</t>
         </is>
       </c>
       <c r="D45" s="25" t="n">
@@ -2256,27 +2254,27 @@
       <c r="G45" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H45" s="29" t="n">
-        <v>19.93</v>
-      </c>
-      <c r="I45" s="29" t="n">
-        <v>39.08</v>
+      <c r="H45" s="27" t="n">
+        <v>7.73</v>
+      </c>
+      <c r="I45" s="27" t="n">
+        <v>40.46</v>
       </c>
       <c r="J45" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +670%</t>
+          <t>중요공시 3건</t>
         </is>
       </c>
       <c r="K45" s="28" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B46" s="25" t="n">
@@ -2284,7 +2282,7 @@
       </c>
       <c r="C46" s="26" t="inlineStr">
         <is>
-          <t>토마토시스템</t>
+          <t>HLB제약</t>
         </is>
       </c>
       <c r="D46" s="25" t="n">
@@ -2299,27 +2297,25 @@
       <c r="G46" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H46" s="29" t="n">
-        <v>7.54</v>
-      </c>
-      <c r="I46" s="29" t="n">
-        <v>56.67</v>
+      <c r="H46" s="27" t="n">
+        <v>29.94</v>
+      </c>
+      <c r="I46" s="27" t="n">
+        <v>69.61</v>
       </c>
       <c r="J46" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +564%</t>
-        </is>
-      </c>
-      <c r="K46" s="28" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+          <t>매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K46" s="28" t="n">
+        <v/>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B47" s="25" t="n">
@@ -2327,7 +2323,7 @@
       </c>
       <c r="C47" s="26" t="inlineStr">
         <is>
-          <t>삼기에너지솔루션즈</t>
+          <t>글로벌테크놀로지</t>
         </is>
       </c>
       <c r="D47" s="25" t="n">
@@ -2342,27 +2338,25 @@
       <c r="G47" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H47" s="27" t="n">
-        <v>-0.96</v>
-      </c>
-      <c r="I47" s="29" t="n">
-        <v>22.76</v>
+      <c r="H47" s="25" t="n">
+        <v/>
+      </c>
+      <c r="I47" s="25" t="n">
+        <v/>
       </c>
       <c r="J47" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +198%</t>
-        </is>
-      </c>
-      <c r="K47" s="28" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+          <t>한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K47" s="28" t="n">
+        <v/>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B48" s="25" t="n">
@@ -2370,42 +2364,42 @@
       </c>
       <c r="C48" s="26" t="inlineStr">
         <is>
-          <t>HT로보틱스</t>
+          <t>루닛</t>
         </is>
       </c>
       <c r="D48" s="25" t="n">
         <v>3</v>
       </c>
       <c r="E48" s="25" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F48" s="25" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G48" s="25" t="n">
         <v>0</v>
       </c>
       <c r="H48" s="27" t="n">
-        <v>-2</v>
-      </c>
-      <c r="I48" s="29" t="n">
-        <v>28.04</v>
+        <v>5.25</v>
+      </c>
+      <c r="I48" s="27" t="n">
+        <v>15.43</v>
       </c>
       <c r="J48" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +196%</t>
+          <t>중요공시 2건 / 중요공시 3일 +100%</t>
         </is>
       </c>
       <c r="K48" s="28" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B49" s="25" t="n">
@@ -2413,7 +2407,7 @@
       </c>
       <c r="C49" s="26" t="inlineStr">
         <is>
-          <t>더블유에스아이</t>
+          <t>HLB</t>
         </is>
       </c>
       <c r="D49" s="25" t="n">
@@ -2428,27 +2422,25 @@
       <c r="G49" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H49" s="29" t="n">
-        <v>10.12</v>
-      </c>
-      <c r="I49" s="29" t="n">
-        <v>25.48</v>
+      <c r="H49" s="27" t="n">
+        <v>3.15</v>
+      </c>
+      <c r="I49" s="27" t="n">
+        <v>28.37</v>
       </c>
       <c r="J49" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +129%</t>
-        </is>
-      </c>
-      <c r="K49" s="28" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+          <t>매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K49" s="28" t="n">
+        <v/>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B50" s="25" t="n">
@@ -2456,42 +2448,42 @@
       </c>
       <c r="C50" s="26" t="inlineStr">
         <is>
-          <t>블루엠텍</t>
+          <t>아리바이오홀딩스</t>
         </is>
       </c>
       <c r="D50" s="25" t="n">
         <v>3</v>
       </c>
       <c r="E50" s="25" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F50" s="25" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G50" s="25" t="n">
         <v>0</v>
       </c>
       <c r="H50" s="29" t="n">
-        <v>3.51</v>
+        <v>-25.47</v>
       </c>
       <c r="I50" s="29" t="n">
-        <v>1.45</v>
+        <v>-24.04</v>
       </c>
       <c r="J50" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +110%</t>
+          <t>중요공시 2건 / 중요공시 3일 +100%</t>
         </is>
       </c>
       <c r="K50" s="28" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B51" s="25" t="n">
@@ -2499,7 +2491,7 @@
       </c>
       <c r="C51" s="26" t="inlineStr">
         <is>
-          <t>삼성전자우</t>
+          <t>MDS테크</t>
         </is>
       </c>
       <c r="D51" s="25" t="n">
@@ -2515,10 +2507,10 @@
         <v>0</v>
       </c>
       <c r="H51" s="27" t="n">
-        <v>-7.43</v>
+        <v>11.21</v>
       </c>
       <c r="I51" s="27" t="n">
-        <v>-2.38</v>
+        <v>11.21</v>
       </c>
       <c r="J51" s="28" t="inlineStr">
         <is>
@@ -2532,7 +2524,7 @@
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B52" s="25" t="n">
@@ -2540,30 +2532,30 @@
       </c>
       <c r="C52" s="26" t="inlineStr">
         <is>
-          <t>미래산업</t>
+          <t>IBKS제25호스팩</t>
         </is>
       </c>
       <c r="D52" s="25" t="n">
         <v>3</v>
       </c>
       <c r="E52" s="25" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F52" s="25" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G52" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H52" s="29" t="n">
-        <v>9.82</v>
-      </c>
-      <c r="I52" s="29" t="n">
-        <v>16.42</v>
+      <c r="H52" s="27" t="n">
+        <v>2.06</v>
+      </c>
+      <c r="I52" s="27" t="n">
+        <v>2.06</v>
       </c>
       <c r="J52" s="28" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 3일 +100%</t>
+          <t>중요공시 5건</t>
         </is>
       </c>
       <c r="K52" s="28" t="inlineStr">
@@ -2575,7 +2567,7 @@
     <row r="53" ht="18" customHeight="1">
       <c r="A53" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B53" s="25" t="n">
@@ -2583,7 +2575,7 @@
       </c>
       <c r="C53" s="26" t="inlineStr">
         <is>
-          <t>더코디</t>
+          <t>비케이홀딩스</t>
         </is>
       </c>
       <c r="D53" s="25" t="n">
@@ -2599,14 +2591,14 @@
         <v>0</v>
       </c>
       <c r="H53" s="29" t="n">
-        <v>22.64</v>
+        <v>-27.91</v>
       </c>
       <c r="I53" s="29" t="n">
-        <v>3.06</v>
+        <v>-42.06</v>
       </c>
       <c r="J53" s="28" t="inlineStr">
         <is>
-          <t>중요공시 3건</t>
+          <t>중요공시 4건</t>
         </is>
       </c>
       <c r="K53" s="28" t="inlineStr">
@@ -2618,7 +2610,7 @@
     <row r="54" ht="18" customHeight="1">
       <c r="A54" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B54" s="25" t="n">
@@ -2626,7 +2618,7 @@
       </c>
       <c r="C54" s="26" t="inlineStr">
         <is>
-          <t>앤씨앤</t>
+          <t>모아라이프플러스</t>
         </is>
       </c>
       <c r="D54" s="25" t="n">
@@ -2641,11 +2633,11 @@
       <c r="G54" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H54" s="29" t="n">
-        <v>16.81</v>
-      </c>
-      <c r="I54" s="29" t="n">
-        <v>7.5</v>
+      <c r="H54" s="27" t="n">
+        <v>4.03</v>
+      </c>
+      <c r="I54" s="27" t="n">
+        <v>4.26</v>
       </c>
       <c r="J54" s="28" t="inlineStr">
         <is>
@@ -2661,7 +2653,7 @@
     <row r="55" ht="18" customHeight="1">
       <c r="A55" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B55" s="25" t="n">
@@ -2669,30 +2661,30 @@
       </c>
       <c r="C55" s="26" t="inlineStr">
         <is>
-          <t>디티앤씨알오</t>
+          <t>한화오션</t>
         </is>
       </c>
       <c r="D55" s="25" t="n">
         <v>3</v>
       </c>
       <c r="E55" s="25" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F55" s="25" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G55" s="25" t="n">
         <v>0</v>
       </c>
       <c r="H55" s="29" t="n">
-        <v>14.38</v>
+        <v>-1.74</v>
       </c>
       <c r="I55" s="29" t="n">
-        <v>14.04</v>
+        <v>-4.12</v>
       </c>
       <c r="J55" s="28" t="inlineStr">
         <is>
-          <t>중요공시 3건</t>
+          <t>중요공시 2건 / 중요공시 3일 +100%</t>
         </is>
       </c>
       <c r="K55" s="28" t="inlineStr">
@@ -2704,7 +2696,7 @@
     <row r="56" ht="18" customHeight="1">
       <c r="A56" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B56" s="25" t="n">
@@ -2712,7 +2704,7 @@
       </c>
       <c r="C56" s="26" t="inlineStr">
         <is>
-          <t>케이쓰리아이</t>
+          <t>라메디텍</t>
         </is>
       </c>
       <c r="D56" s="25" t="n">
@@ -2728,26 +2720,24 @@
         <v>0</v>
       </c>
       <c r="H56" s="27" t="n">
-        <v>-2.44</v>
-      </c>
-      <c r="I56" s="29" t="n">
-        <v>10.82</v>
+        <v>29.53</v>
+      </c>
+      <c r="I56" s="27" t="n">
+        <v>50.28</v>
       </c>
       <c r="J56" s="28" t="inlineStr">
         <is>
-          <t>중요공시 3건</t>
-        </is>
-      </c>
-      <c r="K56" s="28" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K56" s="28" t="n">
+        <v/>
       </c>
     </row>
     <row r="57" ht="18" customHeight="1">
       <c r="A57" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B57" s="25" t="n">
@@ -2755,42 +2745,40 @@
       </c>
       <c r="C57" s="26" t="inlineStr">
         <is>
-          <t>한화오션</t>
+          <t>네이버</t>
         </is>
       </c>
       <c r="D57" s="25" t="n">
         <v>3</v>
       </c>
       <c r="E57" s="25" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F57" s="25" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G57" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H57" s="27" t="n">
-        <v>-0.25</v>
-      </c>
-      <c r="I57" s="27" t="n">
-        <v>-2.42</v>
+      <c r="H57" s="25" t="n">
+        <v/>
+      </c>
+      <c r="I57" s="25" t="n">
+        <v/>
       </c>
       <c r="J57" s="28" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 3일 +100%</t>
-        </is>
-      </c>
-      <c r="K57" s="28" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K57" s="28" t="n">
+        <v/>
       </c>
     </row>
     <row r="58" ht="18" customHeight="1">
       <c r="A58" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B58" s="25" t="n">
@@ -2798,7 +2786,7 @@
       </c>
       <c r="C58" s="26" t="inlineStr">
         <is>
-          <t>알테오젠</t>
+          <t>기아</t>
         </is>
       </c>
       <c r="D58" s="25" t="n">
@@ -2813,27 +2801,25 @@
       <c r="G58" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H58" s="27" t="n">
-        <v>-0.2</v>
-      </c>
-      <c r="I58" s="27" t="n">
-        <v>-1.95</v>
+      <c r="H58" s="29" t="n">
+        <v>-0.9399999999999999</v>
+      </c>
+      <c r="I58" s="29" t="n">
+        <v>-3.65</v>
       </c>
       <c r="J58" s="28" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K58" s="28" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+          <t>매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K58" s="28" t="n">
+        <v/>
       </c>
     </row>
     <row r="59" ht="18" customHeight="1">
       <c r="A59" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B59" s="25" t="n">
@@ -2841,7 +2827,7 @@
       </c>
       <c r="C59" s="26" t="inlineStr">
         <is>
-          <t>에코프로비엠</t>
+          <t>카카오</t>
         </is>
       </c>
       <c r="D59" s="25" t="n">
@@ -2857,14 +2843,14 @@
         <v>0</v>
       </c>
       <c r="H59" s="29" t="n">
-        <v>4.74</v>
-      </c>
-      <c r="I59" s="29" t="n">
-        <v>6.35</v>
+        <v>-0.59</v>
+      </c>
+      <c r="I59" s="27" t="n">
+        <v>1.05</v>
       </c>
       <c r="J59" s="28" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급</t>
+          <t>네이버뉴스 기사 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K59" s="28" t="inlineStr">
@@ -2876,7 +2862,7 @@
     <row r="60" ht="18" customHeight="1">
       <c r="A60" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B60" s="25" t="n">
@@ -2884,7 +2870,7 @@
       </c>
       <c r="C60" s="26" t="inlineStr">
         <is>
-          <t>엔터</t>
+          <t>KT</t>
         </is>
       </c>
       <c r="D60" s="25" t="n">
@@ -2899,11 +2885,11 @@
       <c r="G60" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H60" s="25" t="n">
-        <v/>
-      </c>
-      <c r="I60" s="25" t="n">
-        <v/>
+      <c r="H60" s="29" t="n">
+        <v>-0.38</v>
+      </c>
+      <c r="I60" s="29" t="n">
+        <v>-1.31</v>
       </c>
       <c r="J60" s="28" t="inlineStr">
         <is>
@@ -2917,7 +2903,7 @@
     <row r="61" ht="18" customHeight="1">
       <c r="A61" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B61" s="25" t="n">
@@ -2925,7 +2911,7 @@
       </c>
       <c r="C61" s="26" t="inlineStr">
         <is>
-          <t>프롬바이오</t>
+          <t>KT&amp;G</t>
         </is>
       </c>
       <c r="D61" s="25" t="n">
@@ -2941,14 +2927,14 @@
         <v>0</v>
       </c>
       <c r="H61" s="27" t="n">
-        <v>-10.98</v>
+        <v>0.86</v>
       </c>
       <c r="I61" s="27" t="n">
-        <v>-23.43</v>
+        <v>1.44</v>
       </c>
       <c r="J61" s="28" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급</t>
+          <t>매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K61" s="28" t="n">
@@ -2958,7 +2944,7 @@
     <row r="62" ht="18" customHeight="1">
       <c r="A62" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B62" s="25" t="n">
@@ -2966,14 +2952,14 @@
       </c>
       <c r="C62" s="26" t="inlineStr">
         <is>
-          <t>제주반도체</t>
+          <t>한국비엔씨</t>
         </is>
       </c>
       <c r="D62" s="25" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E62" s="25" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F62" s="25" t="n">
         <v>0</v>
@@ -2981,25 +2967,27 @@
       <c r="G62" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H62" s="27" t="n">
-        <v>-5</v>
+      <c r="H62" s="29" t="n">
+        <v>-3.8</v>
       </c>
       <c r="I62" s="27" t="n">
-        <v>-2.37</v>
+        <v>14.01</v>
       </c>
       <c r="J62" s="28" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K62" s="28" t="n">
-        <v/>
+          <t>네이버 검색 당일 +80%</t>
+        </is>
+      </c>
+      <c r="K62" s="28" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="63" ht="18" customHeight="1">
       <c r="A63" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B63" s="25" t="n">
@@ -3007,14 +2995,14 @@
       </c>
       <c r="C63" s="26" t="inlineStr">
         <is>
-          <t>NH투자증권</t>
+          <t>현대로템</t>
         </is>
       </c>
       <c r="D63" s="25" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E63" s="25" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F63" s="25" t="n">
         <v>0</v>
@@ -3022,19 +3010,21 @@
       <c r="G63" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H63" s="27" t="n">
-        <v>-0.57</v>
-      </c>
-      <c r="I63" s="27" t="n">
-        <v>-1.89</v>
+      <c r="H63" s="29" t="n">
+        <v>-3.27</v>
+      </c>
+      <c r="I63" s="29" t="n">
+        <v>-6.72</v>
       </c>
       <c r="J63" s="28" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K63" s="28" t="n">
-        <v/>
+          <t>중요공시 1건 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K63" s="28" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -3130,22 +3120,22 @@
         <v>1</v>
       </c>
       <c r="C3" s="25" t="n">
-        <v>62</v>
+        <v>88</v>
       </c>
       <c r="D3" s="25" t="n">
-        <v>62</v>
+        <v>88</v>
       </c>
       <c r="E3" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F3" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G3" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="H3" s="25" t="n"/>
@@ -3154,29 +3144,29 @@
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="26" t="inlineStr">
         <is>
-          <t>바이오</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="B4" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C4" s="25" t="n">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="D4" s="25" t="n">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="E4" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F4" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G4" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="H4" s="25" t="n"/>
@@ -3192,70 +3182,70 @@
         <v>1</v>
       </c>
       <c r="C5" s="25" t="n">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D5" s="25" t="n">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="E5" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F5" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G5" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="H5" s="27" t="n">
-        <v>-5.76</v>
-      </c>
-      <c r="I5" s="27" t="n">
-        <v>-1.82</v>
+        <v>1.85</v>
+      </c>
+      <c r="I5" s="25" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="26" t="inlineStr">
         <is>
-          <t>HLB</t>
+          <t>삼성전기</t>
         </is>
       </c>
       <c r="B6" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="25" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="D6" s="25" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="E6" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F6" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G6" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-      <c r="H6" s="29" t="n">
-        <v>27.86</v>
-      </c>
-      <c r="I6" s="29" t="n">
-        <v>24.45</v>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="H6" s="27" t="n">
+        <v>3.96</v>
+      </c>
+      <c r="I6" s="27" t="n">
+        <v>8.24</v>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="26" t="inlineStr">
         <is>
-          <t>삼성전기</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="B7" s="25" t="n">
@@ -3272,20 +3262,16 @@
       </c>
       <c r="F7" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G7" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-      <c r="H7" s="27" t="n">
-        <v>-0.67</v>
-      </c>
-      <c r="I7" s="29" t="n">
-        <v>4.12</v>
-      </c>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="H7" s="25" t="n"/>
+      <c r="I7" s="25" t="n"/>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="26" t="inlineStr">
@@ -3297,22 +3283,22 @@
         <v>1</v>
       </c>
       <c r="C8" s="25" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="D8" s="25" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E8" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F8" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G8" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="H8" s="25" t="n"/>
@@ -3321,29 +3307,29 @@
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="26" t="inlineStr">
         <is>
-          <t>인공지능</t>
+          <t>바이오</t>
         </is>
       </c>
       <c r="B9" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="25" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="D9" s="25" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="E9" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F9" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G9" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="H9" s="25" t="n"/>
@@ -3352,95 +3338,99 @@
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="26" t="inlineStr">
         <is>
-          <t>SK하이닉스</t>
+          <t>LG전자</t>
         </is>
       </c>
       <c r="B10" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C10" s="25" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="D10" s="25" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E10" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F10" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G10" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="H10" s="27" t="n">
-        <v>-5.48</v>
+        <v>0.7</v>
       </c>
       <c r="I10" s="27" t="n">
-        <v>-6.28</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="26" t="inlineStr">
         <is>
-          <t>전기차</t>
+          <t>SK하이닉스</t>
         </is>
       </c>
       <c r="B11" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="25" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D11" s="25" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E11" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F11" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G11" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-      <c r="H11" s="25" t="n"/>
-      <c r="I11" s="25" t="n"/>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="H11" s="27" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="I11" s="29" t="n">
+        <v>-4.74</v>
+      </c>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="26" t="inlineStr">
         <is>
-          <t>태양광</t>
+          <t>방산</t>
         </is>
       </c>
       <c r="B12" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C12" s="25" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D12" s="25" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E12" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F12" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G12" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="H12" s="25" t="n"/>
@@ -3449,178 +3439,174 @@
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>OCI홀딩스</t>
+          <t>모아데이타</t>
         </is>
       </c>
       <c r="B13" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C13" s="25" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D13" s="25" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E13" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F13" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G13" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="H13" s="29" t="n">
-        <v>12.35</v>
+        <v>-5.96</v>
       </c>
       <c r="I13" s="29" t="n">
-        <v>20.21</v>
+        <v>-22.05</v>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>현대차</t>
+          <t>셀트리온</t>
         </is>
       </c>
       <c r="B14" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C14" s="25" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D14" s="25" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E14" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F14" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G14" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="H14" s="27" t="n">
-        <v>-0.84</v>
-      </c>
-      <c r="I14" s="27" t="n">
-        <v>-2.07</v>
+        <v>0.62</v>
+      </c>
+      <c r="I14" s="29" t="n">
+        <v>-1.49</v>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>게임</t>
+          <t>뷰노</t>
         </is>
       </c>
       <c r="B15" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C15" s="25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D15" s="25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E15" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F15" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G15" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-      <c r="H15" s="25" t="n"/>
-      <c r="I15" s="25" t="n"/>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="H15" s="27" t="n">
+        <v>14.92</v>
+      </c>
+      <c r="I15" s="27" t="n">
+        <v>52.94</v>
+      </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>모아데이타</t>
+          <t>조선</t>
         </is>
       </c>
       <c r="B16" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C16" s="25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D16" s="25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E16" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F16" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G16" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-      <c r="H16" s="27" t="n">
-        <v>-11.38</v>
-      </c>
-      <c r="I16" s="27" t="n">
-        <v>-17.11</v>
-      </c>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="H16" s="25" t="n"/>
+      <c r="I16" s="25" t="n"/>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>핑거</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B17" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C17" s="25" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D17" s="25" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E17" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F17" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G17" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-      <c r="H17" s="29" t="n">
-        <v>13.82</v>
-      </c>
-      <c r="I17" s="29" t="n">
-        <v>32.43</v>
-      </c>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="H17" s="25" t="n"/>
+      <c r="I17" s="25" t="n"/>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="26" t="inlineStr">
         <is>
-          <t>기아</t>
+          <t>DB</t>
         </is>
       </c>
       <c r="B18" s="25" t="n">
@@ -3637,25 +3623,25 @@
       </c>
       <c r="F18" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G18" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="H18" s="29" t="n">
-        <v>0.77</v>
+        <v>-0.23</v>
       </c>
       <c r="I18" s="27" t="n">
-        <v>-2.74</v>
+        <v>6.92</v>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>삼성제약</t>
+          <t>대덕전자</t>
         </is>
       </c>
       <c r="B19" s="25" t="n">
@@ -3672,25 +3658,25 @@
       </c>
       <c r="F19" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G19" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-      <c r="H19" s="29" t="n">
-        <v>4.38</v>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="H19" s="27" t="n">
+        <v>8.710000000000001</v>
       </c>
       <c r="I19" s="27" t="n">
-        <v>-0.15</v>
+        <v>28.57</v>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="26" t="inlineStr">
         <is>
-          <t>수소</t>
+          <t>태양광</t>
         </is>
       </c>
       <c r="B20" s="25" t="n">
@@ -3707,12 +3693,12 @@
       </c>
       <c r="F20" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G20" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="H20" s="25" t="n"/>
@@ -3721,112 +3707,108 @@
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="26" t="inlineStr">
         <is>
-          <t>스피어</t>
+          <t>OCI홀딩스</t>
         </is>
       </c>
       <c r="B21" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C21" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D21" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E21" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F21" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G21" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-      <c r="H21" s="27" t="n">
-        <v>-4.9</v>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="H21" s="29" t="n">
+        <v>-5.6</v>
       </c>
       <c r="I21" s="27" t="n">
-        <v>-4.9</v>
+        <v>13.47</v>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="26" t="inlineStr">
         <is>
-          <t>한화솔루션</t>
+          <t>게임</t>
         </is>
       </c>
       <c r="B22" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C22" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D22" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E22" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F22" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G22" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-      <c r="H22" s="29" t="n">
-        <v>16.5</v>
-      </c>
-      <c r="I22" s="29" t="n">
-        <v>23.2</v>
-      </c>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="H22" s="25" t="n"/>
+      <c r="I22" s="25" t="n"/>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="26" t="inlineStr">
         <is>
-          <t>현대로템</t>
+          <t>더코디</t>
         </is>
       </c>
       <c r="B23" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C23" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D23" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E23" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F23" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G23" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-      <c r="H23" s="27" t="n">
-        <v>-0.43</v>
-      </c>
-      <c r="I23" s="27" t="n">
-        <v>-3.57</v>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="H23" s="29" t="n">
+        <v>-10.85</v>
+      </c>
+      <c r="I23" s="29" t="n">
+        <v>-8.130000000000001</v>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="26" t="inlineStr">
         <is>
-          <t>LG전자</t>
+          <t>삼성SDI</t>
         </is>
       </c>
       <c r="B24" s="25" t="n">
@@ -3843,25 +3825,25 @@
       </c>
       <c r="F24" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G24" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="H24" s="29" t="n">
-        <v>1.9</v>
+        <v>-2.08</v>
       </c>
       <c r="I24" s="29" t="n">
-        <v>5.67</v>
+        <v>-3.54</v>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="26" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>앤씨앤</t>
         </is>
       </c>
       <c r="B25" s="25" t="n">
@@ -3878,25 +3860,25 @@
       </c>
       <c r="F25" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G25" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="H25" s="29" t="n">
-        <v>1.4</v>
+        <v>-18.6</v>
       </c>
       <c r="I25" s="29" t="n">
-        <v>5.55</v>
+        <v>-12.5</v>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="26" t="inlineStr">
         <is>
-          <t>방산</t>
+          <t>엔터</t>
         </is>
       </c>
       <c r="B26" s="25" t="n">
@@ -3913,12 +3895,12 @@
       </c>
       <c r="F26" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G26" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="H26" s="25" t="n"/>
@@ -3927,73 +3909,77 @@
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="26" t="inlineStr">
         <is>
-          <t>셀리드</t>
+          <t>미래산업</t>
         </is>
       </c>
       <c r="B27" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C27" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D27" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E27" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F27" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G27" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-      <c r="H27" s="29" t="n">
-        <v>2.11</v>
-      </c>
-      <c r="I27" s="29" t="n">
-        <v>5.98</v>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="H27" s="27" t="n">
+        <v>7.68</v>
+      </c>
+      <c r="I27" s="27" t="n">
+        <v>25.37</v>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="26" t="inlineStr">
         <is>
-          <t>스테이블코인</t>
+          <t>스피어</t>
         </is>
       </c>
       <c r="B28" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C28" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D28" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E28" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F28" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G28" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-      <c r="H28" s="25" t="n"/>
-      <c r="I28" s="25" t="n"/>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="H28" s="29" t="n">
+        <v>-4.26</v>
+      </c>
+      <c r="I28" s="29" t="n">
+        <v>-8.960000000000001</v>
+      </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="26" t="inlineStr">
         <is>
-          <t>KT</t>
+          <t>테라뷰</t>
         </is>
       </c>
       <c r="B29" s="25" t="n">
@@ -4010,25 +3996,25 @@
       </c>
       <c r="F29" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G29" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="H29" s="27" t="n">
-        <v>-0.19</v>
+        <v>30.98</v>
       </c>
       <c r="I29" s="27" t="n">
-        <v>-0.9399999999999999</v>
+        <v>23.9</v>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="26" t="inlineStr">
         <is>
-          <t>루닛</t>
+          <t>티로보틱스</t>
         </is>
       </c>
       <c r="B30" s="25" t="n">
@@ -4045,25 +4031,25 @@
       </c>
       <c r="F30" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G30" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-      <c r="H30" s="29" t="n">
-        <v>13.78</v>
-      </c>
-      <c r="I30" s="29" t="n">
-        <v>9.67</v>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="H30" s="27" t="n">
+        <v>5.49</v>
+      </c>
+      <c r="I30" s="27" t="n">
+        <v>12.03</v>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="26" t="inlineStr">
         <is>
-          <t>에코프로</t>
+          <t>한미반도체</t>
         </is>
       </c>
       <c r="B31" s="25" t="n">
@@ -4080,60 +4066,60 @@
       </c>
       <c r="F31" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G31" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-      <c r="H31" s="29" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="I31" s="29" t="n">
-        <v>1.25</v>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="H31" s="27" t="n">
+        <v>8.15</v>
+      </c>
+      <c r="I31" s="27" t="n">
+        <v>5.44</v>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="26" t="inlineStr">
         <is>
-          <t>HT로보틱스</t>
+          <t>현대차</t>
         </is>
       </c>
       <c r="B32" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C32" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D32" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E32" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F32" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G32" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-      <c r="H32" s="27" t="n">
-        <v>-2</v>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="H32" s="29" t="n">
+        <v>-0.99</v>
       </c>
       <c r="I32" s="29" t="n">
-        <v>28.04</v>
+        <v>-3.04</v>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="26" t="inlineStr">
         <is>
-          <t>NH투자증권</t>
+          <t>HLB</t>
         </is>
       </c>
       <c r="B33" s="25" t="n">
@@ -4150,25 +4136,25 @@
       </c>
       <c r="F33" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G33" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="H33" s="27" t="n">
-        <v>-0.57</v>
+        <v>3.15</v>
       </c>
       <c r="I33" s="27" t="n">
-        <v>-1.89</v>
+        <v>28.37</v>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="26" t="inlineStr">
         <is>
-          <t>네오사피엔스</t>
+          <t>HLB제약</t>
         </is>
       </c>
       <c r="B34" s="25" t="n">
@@ -4185,25 +4171,25 @@
       </c>
       <c r="F34" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G34" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="H34" s="27" t="n">
-        <v>-16.94</v>
+        <v>29.94</v>
       </c>
       <c r="I34" s="27" t="n">
-        <v>-44.17</v>
+        <v>69.61</v>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="26" t="inlineStr">
         <is>
-          <t>더블유에스아이</t>
+          <t>IBKS제25호스팩</t>
         </is>
       </c>
       <c r="B35" s="25" t="n">
@@ -4220,25 +4206,25 @@
       </c>
       <c r="F35" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G35" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-      <c r="H35" s="29" t="n">
-        <v>10.12</v>
-      </c>
-      <c r="I35" s="29" t="n">
-        <v>25.48</v>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="H35" s="27" t="n">
+        <v>2.06</v>
+      </c>
+      <c r="I35" s="27" t="n">
+        <v>2.06</v>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="26" t="inlineStr">
         <is>
-          <t>더코디</t>
+          <t>KT</t>
         </is>
       </c>
       <c r="B36" s="25" t="n">
@@ -4255,25 +4241,25 @@
       </c>
       <c r="F36" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G36" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="H36" s="29" t="n">
-        <v>22.64</v>
+        <v>-0.38</v>
       </c>
       <c r="I36" s="29" t="n">
-        <v>3.06</v>
+        <v>-1.31</v>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="26" t="inlineStr">
         <is>
-          <t>동국생명과학</t>
+          <t>KT&amp;G</t>
         </is>
       </c>
       <c r="B37" s="25" t="n">
@@ -4290,25 +4276,25 @@
       </c>
       <c r="F37" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G37" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-      <c r="H37" s="29" t="n">
-        <v>19.93</v>
-      </c>
-      <c r="I37" s="29" t="n">
-        <v>39.08</v>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="H37" s="27" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="I37" s="27" t="n">
+        <v>1.44</v>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="26" t="inlineStr">
         <is>
-          <t>디에이테크놀로지</t>
+          <t>MDS테크</t>
         </is>
       </c>
       <c r="B38" s="25" t="n">
@@ -4325,25 +4311,25 @@
       </c>
       <c r="F38" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G38" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="H38" s="27" t="n">
-        <v>-30.69</v>
+        <v>11.21</v>
       </c>
       <c r="I38" s="27" t="n">
-        <v>-97.7</v>
+        <v>11.21</v>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="26" t="inlineStr">
         <is>
-          <t>디티앤씨알오</t>
+          <t>글로벌테크놀로지</t>
         </is>
       </c>
       <c r="B39" s="25" t="n">
@@ -4360,25 +4346,21 @@
       </c>
       <c r="F39" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G39" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-      <c r="H39" s="29" t="n">
-        <v>14.38</v>
-      </c>
-      <c r="I39" s="29" t="n">
-        <v>14.04</v>
-      </c>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="H39" s="25" t="n"/>
+      <c r="I39" s="25" t="n"/>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="26" t="inlineStr">
         <is>
-          <t>미래산업</t>
+          <t>기아</t>
         </is>
       </c>
       <c r="B40" s="25" t="n">
@@ -4395,25 +4377,25 @@
       </c>
       <c r="F40" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G40" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="H40" s="29" t="n">
-        <v>9.82</v>
+        <v>-0.9399999999999999</v>
       </c>
       <c r="I40" s="29" t="n">
-        <v>16.42</v>
+        <v>-3.65</v>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="26" t="inlineStr">
         <is>
-          <t>블루엠텍</t>
+          <t>네이버</t>
         </is>
       </c>
       <c r="B41" s="25" t="n">
@@ -4430,25 +4412,21 @@
       </c>
       <c r="F41" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G41" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-      <c r="H41" s="29" t="n">
-        <v>3.51</v>
-      </c>
-      <c r="I41" s="29" t="n">
-        <v>1.45</v>
-      </c>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="H41" s="25" t="n"/>
+      <c r="I41" s="25" t="n"/>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="26" t="inlineStr">
         <is>
-          <t>삼기에너지솔루션즈</t>
+          <t>라메디텍</t>
         </is>
       </c>
       <c r="B42" s="25" t="n">
@@ -4465,25 +4443,25 @@
       </c>
       <c r="F42" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G42" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="H42" s="27" t="n">
-        <v>-0.96</v>
-      </c>
-      <c r="I42" s="29" t="n">
-        <v>22.76</v>
+        <v>29.53</v>
+      </c>
+      <c r="I42" s="27" t="n">
+        <v>50.28</v>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="26" t="inlineStr">
         <is>
-          <t>삼성전자우</t>
+          <t>루닛</t>
         </is>
       </c>
       <c r="B43" s="25" t="n">
@@ -4500,25 +4478,25 @@
       </c>
       <c r="F43" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G43" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="H43" s="27" t="n">
-        <v>-7.43</v>
+        <v>5.25</v>
       </c>
       <c r="I43" s="27" t="n">
-        <v>-2.38</v>
+        <v>15.43</v>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="26" t="inlineStr">
         <is>
-          <t>알테오젠</t>
+          <t>모아라이프플러스</t>
         </is>
       </c>
       <c r="B44" s="25" t="n">
@@ -4535,25 +4513,25 @@
       </c>
       <c r="F44" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G44" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="H44" s="27" t="n">
-        <v>-0.2</v>
+        <v>4.03</v>
       </c>
       <c r="I44" s="27" t="n">
-        <v>-1.95</v>
+        <v>4.26</v>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="26" t="inlineStr">
         <is>
-          <t>앤씨앤</t>
+          <t>베노티앤알</t>
         </is>
       </c>
       <c r="B45" s="25" t="n">
@@ -4570,25 +4548,25 @@
       </c>
       <c r="F45" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G45" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-      <c r="H45" s="29" t="n">
-        <v>16.81</v>
-      </c>
-      <c r="I45" s="29" t="n">
-        <v>7.5</v>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="H45" s="27" t="n">
+        <v>7.73</v>
+      </c>
+      <c r="I45" s="27" t="n">
+        <v>40.46</v>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="26" t="inlineStr">
         <is>
-          <t>에코프로비엠</t>
+          <t>비케이홀딩스</t>
         </is>
       </c>
       <c r="B46" s="25" t="n">
@@ -4605,25 +4583,25 @@
       </c>
       <c r="F46" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G46" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="H46" s="29" t="n">
-        <v>4.74</v>
+        <v>-27.91</v>
       </c>
       <c r="I46" s="29" t="n">
-        <v>6.35</v>
+        <v>-42.06</v>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="26" t="inlineStr">
         <is>
-          <t>엔터</t>
+          <t>아리바이오홀딩스</t>
         </is>
       </c>
       <c r="B47" s="25" t="n">
@@ -4640,21 +4618,25 @@
       </c>
       <c r="F47" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G47" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-      <c r="H47" s="25" t="n"/>
-      <c r="I47" s="25" t="n"/>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="H47" s="29" t="n">
+        <v>-25.47</v>
+      </c>
+      <c r="I47" s="29" t="n">
+        <v>-24.04</v>
+      </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="26" t="inlineStr">
         <is>
-          <t>제주반도체</t>
+          <t>카카오</t>
         </is>
       </c>
       <c r="B48" s="25" t="n">
@@ -4671,25 +4653,25 @@
       </c>
       <c r="F48" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G48" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-      <c r="H48" s="27" t="n">
-        <v>-5</v>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="H48" s="29" t="n">
+        <v>-0.59</v>
       </c>
       <c r="I48" s="27" t="n">
-        <v>-2.37</v>
+        <v>1.05</v>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="26" t="inlineStr">
         <is>
-          <t>케이쓰리아이</t>
+          <t>한화오션</t>
         </is>
       </c>
       <c r="B49" s="25" t="n">
@@ -4706,25 +4688,25 @@
       </c>
       <c r="F49" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G49" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-      <c r="H49" s="27" t="n">
-        <v>-2.44</v>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="H49" s="29" t="n">
+        <v>-1.74</v>
       </c>
       <c r="I49" s="29" t="n">
-        <v>10.82</v>
+        <v>-4.12</v>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="26" t="inlineStr">
         <is>
-          <t>토마토시스템</t>
+          <t>현대바이오랜드</t>
         </is>
       </c>
       <c r="B50" s="25" t="n">
@@ -4741,89 +4723,89 @@
       </c>
       <c r="F50" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G50" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-      <c r="H50" s="29" t="n">
-        <v>7.54</v>
-      </c>
-      <c r="I50" s="29" t="n">
-        <v>56.67</v>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="H50" s="27" t="n">
+        <v>25.03</v>
+      </c>
+      <c r="I50" s="27" t="n">
+        <v>45.2</v>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="26" t="inlineStr">
         <is>
-          <t>프롬바이오</t>
+          <t>한국비엔씨</t>
         </is>
       </c>
       <c r="B51" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C51" s="25" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D51" s="25" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E51" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F51" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G51" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-      <c r="H51" s="27" t="n">
-        <v>-10.98</v>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="H51" s="29" t="n">
+        <v>-3.8</v>
       </c>
       <c r="I51" s="27" t="n">
-        <v>-23.43</v>
+        <v>14.01</v>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="26" t="inlineStr">
         <is>
-          <t>한화오션</t>
+          <t>현대로템</t>
         </is>
       </c>
       <c r="B52" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C52" s="25" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D52" s="25" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E52" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F52" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G52" s="25" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-      <c r="H52" s="27" t="n">
-        <v>-0.25</v>
-      </c>
-      <c r="I52" s="27" t="n">
-        <v>-2.42</v>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="H52" s="29" t="n">
+        <v>-3.27</v>
+      </c>
+      <c r="I52" s="29" t="n">
+        <v>-6.72</v>
       </c>
     </row>
   </sheetData>
@@ -4907,19 +4889,19 @@
         <v>1</v>
       </c>
       <c r="C3" s="36" t="n">
-        <v>62</v>
+        <v>88</v>
       </c>
       <c r="D3" s="36" t="n">
-        <v>62</v>
+        <v>88</v>
       </c>
       <c r="E3" s="36" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F3" s="37" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G3" s="37" t="inlineStr">
@@ -4938,19 +4920,19 @@
         <v>1</v>
       </c>
       <c r="C4" s="36" t="n">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="D4" s="36" t="n">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="E4" s="36" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F4" s="37" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G4" s="37" t="inlineStr">
@@ -4962,26 +4944,26 @@
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="35" t="inlineStr">
         <is>
-          <t>전기차</t>
+          <t>방산</t>
         </is>
       </c>
       <c r="B5" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="36" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D5" s="36" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E5" s="36" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F5" s="37" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G5" s="37" t="inlineStr">
@@ -4993,26 +4975,26 @@
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="35" t="inlineStr">
         <is>
-          <t>방산</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="B6" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="36" t="n">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="D6" s="36" t="n">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="E6" s="36" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F6" s="37" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G6" s="37" t="inlineStr">
@@ -5024,7 +5006,7 @@
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="35" t="inlineStr">
         <is>
-          <t>수소</t>
+          <t>태양광</t>
         </is>
       </c>
       <c r="B7" s="36" t="n">
@@ -5038,12 +5020,12 @@
       </c>
       <c r="E7" s="36" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F7" s="37" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G7" s="37" t="inlineStr">
@@ -5055,26 +5037,26 @@
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="35" t="inlineStr">
         <is>
-          <t>태양광</t>
+          <t>게임</t>
         </is>
       </c>
       <c r="B8" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="36" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="D8" s="36" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="E8" s="36" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F8" s="37" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G8" s="37" t="inlineStr">
@@ -5086,26 +5068,26 @@
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="35" t="inlineStr">
         <is>
-          <t>게임</t>
+          <t>엔터</t>
         </is>
       </c>
       <c r="B9" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="36" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D9" s="36" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E9" s="36" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F9" s="37" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G9" s="37" t="inlineStr">
@@ -5117,26 +5099,26 @@
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="35" t="inlineStr">
         <is>
-          <t>엔터</t>
+          <t>조선</t>
         </is>
       </c>
       <c r="B10" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C10" s="36" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="D10" s="36" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E10" s="36" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F10" s="37" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G10" s="37" t="inlineStr">
@@ -5155,19 +5137,19 @@
         <v>1</v>
       </c>
       <c r="C11" s="36" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="D11" s="36" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E11" s="36" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F11" s="37" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G11" s="37" t="inlineStr">
@@ -5186,19 +5168,19 @@
         <v>1</v>
       </c>
       <c r="C12" s="36" t="n">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="D12" s="36" t="n">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="E12" s="36" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F12" s="37" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G12" s="37" t="inlineStr">
@@ -5208,36 +5190,40 @@
       </c>
     </row>
     <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="26" t="inlineStr">
-        <is>
-          <t>이차전지</t>
-        </is>
-      </c>
-      <c r="B13" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="C13" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="D13" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="E13" s="25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F13" s="28" t="inlineStr">
-        <is>
-          <t>감지 없음</t>
-        </is>
-      </c>
-      <c r="G13" s="28" t="inlineStr"/>
+      <c r="A13" s="35" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="B13" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C13" s="36" t="n">
+        <v>6</v>
+      </c>
+      <c r="D13" s="36" t="n">
+        <v>6</v>
+      </c>
+      <c r="E13" s="36" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="F13" s="37" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="G13" s="37" t="inlineStr">
+        <is>
+          <t>⚡ 관심</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>AI반도체</t>
+          <t>이차전지</t>
         </is>
       </c>
       <c r="B14" s="25" t="n">
@@ -5264,7 +5250,7 @@
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>원전</t>
+          <t>AI반도체</t>
         </is>
       </c>
       <c r="B15" s="25" t="n">
@@ -5291,7 +5277,7 @@
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>전기차</t>
         </is>
       </c>
       <c r="B16" s="25" t="n">
@@ -5318,7 +5304,7 @@
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>핀테크</t>
+          <t>원전</t>
         </is>
       </c>
       <c r="B17" s="25" t="n">
@@ -5345,7 +5331,7 @@
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="26" t="inlineStr">
         <is>
-          <t>클라우드</t>
+          <t>수소</t>
         </is>
       </c>
       <c r="B18" s="25" t="n">
@@ -5372,7 +5358,7 @@
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>조선</t>
+          <t>핀테크</t>
         </is>
       </c>
       <c r="B19" s="25" t="n">
@@ -5399,7 +5385,7 @@
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="26" t="inlineStr">
         <is>
-          <t>철강</t>
+          <t>클라우드</t>
         </is>
       </c>
       <c r="B20" s="25" t="n">
@@ -5426,7 +5412,7 @@
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="26" t="inlineStr">
         <is>
-          <t>의료기기</t>
+          <t>철강</t>
         </is>
       </c>
       <c r="B21" s="25" t="n">
@@ -5453,7 +5439,7 @@
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="26" t="inlineStr">
         <is>
-          <t>NVIDIA</t>
+          <t>의료기기</t>
         </is>
       </c>
       <c r="B22" s="25" t="n">
@@ -5480,7 +5466,7 @@
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="26" t="inlineStr">
         <is>
-          <t>Tesla</t>
+          <t>NVIDIA</t>
         </is>
       </c>
       <c r="B23" s="25" t="n">
@@ -5507,7 +5493,7 @@
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="26" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>Tesla</t>
         </is>
       </c>
       <c r="B24" s="25" t="n">

</xml_diff>

<commit_message>
auto: 2026-10-04 07:15 자동 백업
</commit_message>
<xml_diff>
--- a/trend/stock_trend_history.xlsx
+++ b/trend/stock_trend_history.xlsx
@@ -258,13 +258,13 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -694,7 +694,7 @@
     <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-10-03 06:54</t>
+          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-10-04 06:54</t>
         </is>
       </c>
     </row>
@@ -708,7 +708,7 @@
       </c>
       <c r="E3" s="3" t="n"/>
       <c r="G3" s="5" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="H3" s="3" t="n"/>
       <c r="J3" s="6" t="n">
@@ -787,21 +787,21 @@
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-10-03) 상위: 반도체  점수 43.0점</t>
+          <t>⚡ 최신(2026-10-04) 상위: 반도체  점수 48.0점</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-10-03) 상위: 삼성전자  점수 29.0점</t>
+          <t>⚡ 최신(2026-10-04) 상위: 삼성전자  점수 35.0점</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-10-03) 상위: 인공지능  점수 25.0점</t>
+          <t>⚡ 최신(2026-10-04) 상위: 인공지능  점수 24.0점</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="15" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B14" s="15" t="n">
@@ -928,10 +928,10 @@
         </is>
       </c>
       <c r="D14" s="15" t="n">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="E14" s="15" t="n">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="F14" s="15" t="n">
         <v>0</v>
@@ -947,7 +947,7 @@
       </c>
       <c r="J14" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K14" s="17" t="inlineStr">
@@ -959,7 +959,7 @@
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="15" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B15" s="15" t="n">
@@ -971,10 +971,10 @@
         </is>
       </c>
       <c r="D15" s="15" t="n">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="E15" s="15" t="n">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="F15" s="15" t="n">
         <v>0</v>
@@ -985,12 +985,12 @@
       <c r="H15" s="18" t="n">
         <v>0.55</v>
       </c>
-      <c r="I15" s="19" t="n">
-        <v>-3.66</v>
+      <c r="I15" s="18" t="n">
+        <v>2.22</v>
       </c>
       <c r="J15" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K15" s="17" t="inlineStr">
@@ -1002,7 +1002,7 @@
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="15" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B16" s="15" t="n">
@@ -1014,10 +1014,10 @@
         </is>
       </c>
       <c r="D16" s="15" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E16" s="15" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F16" s="15" t="n">
         <v>0</v>
@@ -1033,7 +1033,7 @@
       </c>
       <c r="J16" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+          <t>매일경제 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K16" s="17" t="inlineStr">
@@ -1045,7 +1045,7 @@
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B17" s="15" t="n">
@@ -1057,10 +1057,10 @@
         </is>
       </c>
       <c r="D17" s="15" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E17" s="15" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="F17" s="15" t="n">
         <v>0</v>
@@ -1072,7 +1072,7 @@
         <v>-0.57</v>
       </c>
       <c r="I17" s="19" t="n">
-        <v>-2.8</v>
+        <v>-1.98</v>
       </c>
       <c r="J17" s="17" t="inlineStr">
         <is>
@@ -1086,7 +1086,7 @@
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B18" s="15" t="n">
@@ -1094,14 +1094,14 @@
       </c>
       <c r="C18" s="16" t="inlineStr">
         <is>
-          <t>바이오</t>
+          <t>원전</t>
         </is>
       </c>
       <c r="D18" s="15" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E18" s="15" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F18" s="15" t="n">
         <v>0</v>
@@ -1117,7 +1117,7 @@
       </c>
       <c r="J18" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 한국경제 헤드라인 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K18" s="17" t="inlineStr">
@@ -1129,7 +1129,7 @@
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B19" s="15" t="n">
@@ -1137,14 +1137,14 @@
       </c>
       <c r="C19" s="16" t="inlineStr">
         <is>
-          <t>철강</t>
+          <t>바이오</t>
         </is>
       </c>
       <c r="D19" s="15" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E19" s="15" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F19" s="15" t="n">
         <v>0</v>
@@ -1160,7 +1160,7 @@
       </c>
       <c r="J19" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K19" s="17" t="inlineStr">
@@ -1172,7 +1172,7 @@
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B20" s="15" t="n">
@@ -1184,10 +1184,10 @@
         </is>
       </c>
       <c r="D20" s="15" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E20" s="15" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F20" s="15" t="n">
         <v>0</v>
@@ -1203,7 +1203,7 @@
       </c>
       <c r="J20" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K20" s="17" t="inlineStr">
@@ -1215,7 +1215,7 @@
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="15" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B21" s="15" t="n">
@@ -1223,7 +1223,7 @@
       </c>
       <c r="C21" s="16" t="inlineStr">
         <is>
-          <t>SK하이닉스</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="D21" s="15" t="n">
@@ -1238,15 +1238,15 @@
       <c r="G21" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H21" s="18" t="n">
-        <v>0.77</v>
-      </c>
-      <c r="I21" s="19" t="n">
-        <v>-1.13</v>
+      <c r="H21" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I21" s="15" t="n">
+        <v/>
       </c>
       <c r="J21" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K21" s="17" t="inlineStr">
@@ -1258,7 +1258,7 @@
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="15" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B22" s="15" t="n">
@@ -1266,14 +1266,14 @@
       </c>
       <c r="C22" s="16" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>한창</t>
         </is>
       </c>
       <c r="D22" s="15" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E22" s="15" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F22" s="15" t="n">
         <v>0</v>
@@ -1281,27 +1281,27 @@
       <c r="G22" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H22" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I22" s="15" t="n">
-        <v/>
+      <c r="H22" s="19" t="n">
+        <v>-91.06999999999999</v>
+      </c>
+      <c r="I22" s="19" t="n">
+        <v>-91.06999999999999</v>
       </c>
       <c r="J22" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+          <t>네이버 검색 당일 +143% / 중요공시 1건 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K22" s="17" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="15" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B23" s="15" t="n">
@@ -1309,42 +1309,42 @@
       </c>
       <c r="C23" s="16" t="inlineStr">
         <is>
-          <t>삼성E&amp;A</t>
+          <t>SK하이닉스</t>
         </is>
       </c>
       <c r="D23" s="15" t="n">
         <v>7</v>
       </c>
       <c r="E23" s="15" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="F23" s="15" t="n">
         <v>0</v>
       </c>
       <c r="G23" s="15" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H23" s="18" t="n">
-        <v>0.84</v>
-      </c>
-      <c r="I23" s="19" t="n">
-        <v>-3.53</v>
+        <v>0.77</v>
+      </c>
+      <c r="I23" s="18" t="n">
+        <v>4.6</v>
       </c>
       <c r="J23" s="17" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 7일 +100% / 매일경제 헤드라인 언급</t>
+          <t>네이버뉴스 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K23" s="17" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="15" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B24" s="15" t="n">
@@ -1352,83 +1352,83 @@
       </c>
       <c r="C24" s="16" t="inlineStr">
         <is>
-          <t>에스제이그룹</t>
+          <t>삼성E&amp;A</t>
         </is>
       </c>
       <c r="D24" s="15" t="n">
         <v>7</v>
       </c>
       <c r="E24" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="F24" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="H24" s="18" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="I24" s="19" t="n">
+        <v>-4.11</v>
+      </c>
+      <c r="J24" s="17" t="inlineStr">
+        <is>
+          <t>중요공시 2건 / 중요공시 7일 +100% / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K24" s="17" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B25" s="15" t="n">
+        <v>12</v>
+      </c>
+      <c r="C25" s="16" t="inlineStr">
+        <is>
+          <t>철강</t>
+        </is>
+      </c>
+      <c r="D25" s="15" t="n">
         <v>7</v>
       </c>
-      <c r="F24" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="G24" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H24" s="18" t="n">
-        <v>29.96</v>
-      </c>
-      <c r="I24" s="18" t="n">
-        <v>26.45</v>
-      </c>
-      <c r="J24" s="17" t="inlineStr">
-        <is>
-          <t>중요공시 1건 / 네이버뉴스 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K24" s="17" t="inlineStr">
-        <is>
-          <t>공시, 네이버</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="18" customHeight="1">
-      <c r="A25" s="20" t="inlineStr">
-        <is>
-          <t>2026-10-03</t>
-        </is>
-      </c>
-      <c r="B25" s="20" t="n">
-        <v>12</v>
-      </c>
-      <c r="C25" s="21" t="inlineStr">
-        <is>
-          <t>SG</t>
-        </is>
-      </c>
-      <c r="D25" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="E25" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="F25" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G25" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H25" s="22" t="n">
-        <v>-5.15</v>
-      </c>
-      <c r="I25" s="22" t="n">
-        <v>-8.68</v>
-      </c>
-      <c r="J25" s="23" t="inlineStr">
-        <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K25" s="23" t="n">
+      <c r="E25" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="F25" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I25" s="15" t="n">
+        <v/>
+      </c>
+      <c r="J25" s="17" t="inlineStr">
+        <is>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K25" s="17" t="n">
         <v/>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="20" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B26" s="20" t="n">
@@ -1436,42 +1436,42 @@
       </c>
       <c r="C26" s="21" t="inlineStr">
         <is>
-          <t>티엠씨</t>
+          <t>세미파이브</t>
         </is>
       </c>
       <c r="D26" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E26" s="20" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F26" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G26" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H26" s="24" t="n">
-        <v>29.68</v>
-      </c>
-      <c r="I26" s="24" t="n">
-        <v>28.86</v>
+      <c r="H26" s="22" t="n">
+        <v>1.72</v>
+      </c>
+      <c r="I26" s="22" t="n">
+        <v>28.88</v>
       </c>
       <c r="J26" s="23" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급</t>
+          <t>네이버 검색 당일 +437% / 중요공시 2건 / 중요공시 3일 +100%</t>
         </is>
       </c>
       <c r="K26" s="23" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="20" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B27" s="20" t="n">
@@ -1479,42 +1479,40 @@
       </c>
       <c r="C27" s="21" t="inlineStr">
         <is>
-          <t>모아데이타</t>
+          <t>SG</t>
         </is>
       </c>
       <c r="D27" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E27" s="20" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F27" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G27" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="H27" s="22" t="n">
-        <v>-3.6</v>
-      </c>
-      <c r="I27" s="22" t="n">
-        <v>-13.01</v>
+        <v>0</v>
+      </c>
+      <c r="H27" s="24" t="n">
+        <v>-5.15</v>
+      </c>
+      <c r="I27" s="24" t="n">
+        <v>-2.64</v>
       </c>
       <c r="J27" s="23" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 7일 +50%</t>
-        </is>
-      </c>
-      <c r="K27" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K27" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="20" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B28" s="20" t="n">
@@ -1522,30 +1520,30 @@
       </c>
       <c r="C28" s="21" t="inlineStr">
         <is>
-          <t>아리바이오홀딩스</t>
+          <t>모아데이타</t>
         </is>
       </c>
       <c r="D28" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E28" s="20" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F28" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G28" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="H28" s="22" t="n">
-        <v>-2.23</v>
-      </c>
-      <c r="I28" s="22" t="n">
-        <v>-22.77</v>
+      <c r="H28" s="24" t="n">
+        <v>-3.6</v>
+      </c>
+      <c r="I28" s="24" t="n">
+        <v>-1.83</v>
       </c>
       <c r="J28" s="23" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 3일 +100% / 중요공시 7일 +100%</t>
+          <t>중요공시 3건 / 중요공시 7일 +50%</t>
         </is>
       </c>
       <c r="K28" s="23" t="inlineStr">
@@ -1557,7 +1555,7 @@
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="20" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B29" s="20" t="n">
@@ -1565,42 +1563,42 @@
       </c>
       <c r="C29" s="21" t="inlineStr">
         <is>
-          <t>선도전기</t>
+          <t>머큐리</t>
         </is>
       </c>
       <c r="D29" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E29" s="20" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F29" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G29" s="20" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H29" s="22" t="n">
-        <v>-1.82</v>
+        <v>29.8</v>
       </c>
       <c r="I29" s="22" t="n">
-        <v>-4.44</v>
+        <v>28.21</v>
       </c>
       <c r="J29" s="23" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 3일 +100% / 중요공시 7일 +100%</t>
+          <t>네이버 검색 당일 +69% / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K29" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="20" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B30" s="20" t="n">
@@ -1608,40 +1606,42 @@
       </c>
       <c r="C30" s="21" t="inlineStr">
         <is>
-          <t>원전</t>
+          <t>팬오션</t>
         </is>
       </c>
       <c r="D30" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E30" s="20" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F30" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G30" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H30" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I30" s="20" t="n">
-        <v/>
+      <c r="H30" s="22" t="n">
+        <v>6.47</v>
+      </c>
+      <c r="I30" s="22" t="n">
+        <v>9.84</v>
       </c>
       <c r="J30" s="23" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K30" s="23" t="n">
-        <v/>
+          <t>네이버 검색 당일 +67% / 중요공시 2건 / 중요공시 3일 +100%</t>
+        </is>
+      </c>
+      <c r="K30" s="23" t="inlineStr">
+        <is>
+          <t>네이버, 공시</t>
+        </is>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="20" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B31" s="20" t="n">
@@ -1649,42 +1649,42 @@
       </c>
       <c r="C31" s="21" t="inlineStr">
         <is>
-          <t>더코디</t>
+          <t>두산에너빌리티</t>
         </is>
       </c>
       <c r="D31" s="20" t="n">
         <v>5</v>
       </c>
       <c r="E31" s="20" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F31" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G31" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H31" s="22" t="n">
-        <v>-1.27</v>
+      <c r="H31" s="24" t="n">
+        <v>-1.09</v>
       </c>
       <c r="I31" s="22" t="n">
-        <v>-2.96</v>
+        <v>0.37</v>
       </c>
       <c r="J31" s="23" t="inlineStr">
         <is>
-          <t>중요공시 6건 / 중요공시 3일 +100%</t>
+          <t>중요공시 1건 / 네이버뉴스 헤드라인 언급</t>
         </is>
       </c>
       <c r="K31" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="20" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B32" s="20" t="n">
@@ -1692,42 +1692,42 @@
       </c>
       <c r="C32" s="21" t="inlineStr">
         <is>
-          <t>에이전트AI</t>
+          <t>퀀텀레일</t>
         </is>
       </c>
       <c r="D32" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E32" s="20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F32" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G32" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H32" s="22" t="n">
-        <v>-2.34</v>
-      </c>
-      <c r="I32" s="22" t="n">
-        <v>-39.85</v>
+      <c r="H32" s="24" t="n">
+        <v>-1.63</v>
+      </c>
+      <c r="I32" s="24" t="n">
+        <v>-51.68</v>
       </c>
       <c r="J32" s="23" t="inlineStr">
         <is>
-          <t>중요공시 5건 / 중요공시 3일 +400%</t>
+          <t>네이버 검색 당일 +1711% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K32" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="20" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B33" s="20" t="n">
@@ -1735,14 +1735,14 @@
       </c>
       <c r="C33" s="21" t="inlineStr">
         <is>
-          <t>삼성전기</t>
+          <t>나인테크</t>
         </is>
       </c>
       <c r="D33" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E33" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F33" s="20" t="n">
         <v>0</v>
@@ -1750,27 +1750,27 @@
       <c r="G33" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H33" s="24" t="n">
-        <v>1.48</v>
-      </c>
-      <c r="I33" s="24" t="n">
-        <v>5.06</v>
+      <c r="H33" s="22" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="I33" s="22" t="n">
+        <v>28.05</v>
       </c>
       <c r="J33" s="23" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+          <t>네이버 검색 당일 +437% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K33" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="20" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B34" s="20" t="n">
@@ -1778,14 +1778,14 @@
       </c>
       <c r="C34" s="21" t="inlineStr">
         <is>
-          <t>에코프로</t>
+          <t>한국파마</t>
         </is>
       </c>
       <c r="D34" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E34" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F34" s="20" t="n">
         <v>0</v>
@@ -1793,27 +1793,27 @@
       <c r="G34" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H34" s="24" t="n">
-        <v>5.07</v>
-      </c>
-      <c r="I34" s="24" t="n">
-        <v>11.24</v>
+      <c r="H34" s="22" t="n">
+        <v>13.42</v>
+      </c>
+      <c r="I34" s="22" t="n">
+        <v>19.06</v>
       </c>
       <c r="J34" s="23" t="inlineStr">
         <is>
-          <t>Google 급상승 검색어 등장 (KR)</t>
+          <t>네이버 검색 당일 +202% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K34" s="23" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="20" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B35" s="20" t="n">
@@ -1821,14 +1821,14 @@
       </c>
       <c r="C35" s="21" t="inlineStr">
         <is>
-          <t>에코프로머티</t>
+          <t>한화솔루션</t>
         </is>
       </c>
       <c r="D35" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E35" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F35" s="20" t="n">
         <v>0</v>
@@ -1836,27 +1836,27 @@
       <c r="G35" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H35" s="24" t="n">
-        <v>3.8</v>
-      </c>
-      <c r="I35" s="24" t="n">
-        <v>8.99</v>
+      <c r="H35" s="22" t="n">
+        <v>5.71</v>
+      </c>
+      <c r="I35" s="22" t="n">
+        <v>5.4</v>
       </c>
       <c r="J35" s="23" t="inlineStr">
         <is>
-          <t>Google 급상승 검색어 등장 (KR)</t>
+          <t>네이버 검색 당일 +156% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K35" s="23" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="20" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B36" s="20" t="n">
@@ -1864,14 +1864,14 @@
       </c>
       <c r="C36" s="21" t="inlineStr">
         <is>
-          <t>에코프로에이치엔</t>
+          <t>고영</t>
         </is>
       </c>
       <c r="D36" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E36" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F36" s="20" t="n">
         <v>0</v>
@@ -1879,27 +1879,27 @@
       <c r="G36" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H36" s="24" t="n">
-        <v>1.02</v>
-      </c>
-      <c r="I36" s="24" t="n">
-        <v>13.73</v>
+      <c r="H36" s="22" t="n">
+        <v>1.47</v>
+      </c>
+      <c r="I36" s="22" t="n">
+        <v>19.41</v>
       </c>
       <c r="J36" s="23" t="inlineStr">
         <is>
-          <t>Google 급상승 검색어 등장 (KR)</t>
+          <t>네이버 검색 당일 +111% / 중요공시 2건</t>
         </is>
       </c>
       <c r="K36" s="23" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="20" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B37" s="20" t="n">
@@ -1907,14 +1907,14 @@
       </c>
       <c r="C37" s="21" t="inlineStr">
         <is>
-          <t>에코프로비엠</t>
+          <t>삼성중공업</t>
         </is>
       </c>
       <c r="D37" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E37" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F37" s="20" t="n">
         <v>0</v>
@@ -1922,27 +1922,27 @@
       <c r="G37" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H37" s="24" t="n">
-        <v>1.58</v>
+      <c r="H37" s="22" t="n">
+        <v>0.91</v>
       </c>
       <c r="I37" s="24" t="n">
-        <v>9.57</v>
+        <v>-1.14</v>
       </c>
       <c r="J37" s="23" t="inlineStr">
         <is>
-          <t>Google 급상승 검색어 등장 (KR)</t>
+          <t>네이버 검색 당일 +53% / 중요공시 2건 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K37" s="23" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="20" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B38" s="20" t="n">
@@ -1950,14 +1950,14 @@
       </c>
       <c r="C38" s="21" t="inlineStr">
         <is>
-          <t>LG전자</t>
+          <t>성호전자</t>
         </is>
       </c>
       <c r="D38" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E38" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F38" s="20" t="n">
         <v>0</v>
@@ -1965,25 +1965,27 @@
       <c r="G38" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H38" s="24" t="n">
-        <v>1.65</v>
-      </c>
-      <c r="I38" s="24" t="n">
-        <v>2.38</v>
+      <c r="H38" s="22" t="n">
+        <v>11.35</v>
+      </c>
+      <c r="I38" s="22" t="n">
+        <v>27.13</v>
       </c>
       <c r="J38" s="23" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K38" s="23" t="n">
-        <v/>
+          <t>네이버뉴스 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K38" s="23" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="20" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B39" s="20" t="n">
@@ -1991,7 +1993,7 @@
       </c>
       <c r="C39" s="21" t="inlineStr">
         <is>
-          <t>퀀텀레일</t>
+          <t>빛샘전자</t>
         </is>
       </c>
       <c r="D39" s="20" t="n">
@@ -2007,26 +2009,26 @@
         <v>0</v>
       </c>
       <c r="H39" s="22" t="n">
-        <v>-1.63</v>
+        <v>11.65</v>
       </c>
       <c r="I39" s="22" t="n">
-        <v>-58.04</v>
+        <v>26.1</v>
       </c>
       <c r="J39" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +1443% / 중요공시 1건</t>
+          <t>네이버뉴스 헤드라인 언급</t>
         </is>
       </c>
       <c r="K39" s="23" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="20" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B40" s="20" t="n">
@@ -2034,7 +2036,7 @@
       </c>
       <c r="C40" s="21" t="inlineStr">
         <is>
-          <t>나인테크</t>
+          <t>우리기술</t>
         </is>
       </c>
       <c r="D40" s="20" t="n">
@@ -2049,27 +2051,27 @@
       <c r="G40" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H40" s="24" t="n">
-        <v>0.71</v>
-      </c>
-      <c r="I40" s="24" t="n">
-        <v>29.52</v>
+      <c r="H40" s="22" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="I40" s="22" t="n">
+        <v>1.19</v>
       </c>
       <c r="J40" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +364% / 중요공시 1건</t>
+          <t>중요공시 1건 / 네이버뉴스 헤드라인 언급</t>
         </is>
       </c>
       <c r="K40" s="23" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="20" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B41" s="20" t="n">
@@ -2077,42 +2079,42 @@
       </c>
       <c r="C41" s="21" t="inlineStr">
         <is>
-          <t>세미파이브</t>
+          <t>에이에프더블류</t>
         </is>
       </c>
       <c r="D41" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E41" s="20" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F41" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G41" s="20" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H41" s="24" t="n">
-        <v>1.72</v>
+        <v>-5.13</v>
       </c>
       <c r="I41" s="24" t="n">
-        <v>27.38</v>
+        <v>-51.32</v>
       </c>
       <c r="J41" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +344% / 중요공시 2건</t>
+          <t>중요공시 2건 / 중요공시 7일 +100%</t>
         </is>
       </c>
       <c r="K41" s="23" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="20" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B42" s="20" t="n">
@@ -2120,42 +2122,42 @@
       </c>
       <c r="C42" s="21" t="inlineStr">
         <is>
-          <t>한화솔루션</t>
+          <t>아리바이오홀딩스</t>
         </is>
       </c>
       <c r="D42" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E42" s="20" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F42" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G42" s="20" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H42" s="24" t="n">
-        <v>5.71</v>
+        <v>-2.23</v>
       </c>
       <c r="I42" s="24" t="n">
-        <v>22.79</v>
+        <v>-22.96</v>
       </c>
       <c r="J42" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +110% / 중요공시 1건</t>
+          <t>중요공시 2건 / 중요공시 7일 +100%</t>
         </is>
       </c>
       <c r="K42" s="23" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="20" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B43" s="20" t="n">
@@ -2163,30 +2165,30 @@
       </c>
       <c r="C43" s="21" t="inlineStr">
         <is>
-          <t>한화생명</t>
+          <t>선도전기</t>
         </is>
       </c>
       <c r="D43" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E43" s="20" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F43" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G43" s="20" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H43" s="24" t="n">
-        <v>0.38</v>
-      </c>
-      <c r="I43" s="22" t="n">
-        <v>-6.34</v>
+        <v>-1.82</v>
+      </c>
+      <c r="I43" s="24" t="n">
+        <v>-1.82</v>
       </c>
       <c r="J43" s="23" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 매일경제 헤드라인 언급</t>
+          <t>중요공시 2건 / 중요공시 7일 +100%</t>
         </is>
       </c>
       <c r="K43" s="23" t="inlineStr">
@@ -2198,7 +2200,7 @@
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="20" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B44" s="20" t="n">
@@ -2206,30 +2208,30 @@
       </c>
       <c r="C44" s="21" t="inlineStr">
         <is>
-          <t>팬오션</t>
+          <t>루닛</t>
         </is>
       </c>
       <c r="D44" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E44" s="20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F44" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G44" s="20" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H44" s="24" t="n">
-        <v>6.47</v>
+        <v>-5.03</v>
       </c>
       <c r="I44" s="24" t="n">
-        <v>11.41</v>
+        <v>-5.88</v>
       </c>
       <c r="J44" s="23" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 3일 +100%</t>
+          <t>중요공시 2건 / 중요공시 7일 +100%</t>
         </is>
       </c>
       <c r="K44" s="23" t="inlineStr">
@@ -2241,7 +2243,7 @@
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="20" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B45" s="20" t="n">
@@ -2249,30 +2251,30 @@
       </c>
       <c r="C45" s="21" t="inlineStr">
         <is>
-          <t>두산에너빌리티</t>
+          <t>한화오션</t>
         </is>
       </c>
       <c r="D45" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E45" s="20" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F45" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G45" s="20" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H45" s="22" t="n">
-        <v>-1.09</v>
-      </c>
-      <c r="I45" s="22" t="n">
-        <v>-1.57</v>
+        <v>0.13</v>
+      </c>
+      <c r="I45" s="24" t="n">
+        <v>-2.24</v>
       </c>
       <c r="J45" s="23" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
+          <t>중요공시 2건 / 중요공시 7일 +100%</t>
         </is>
       </c>
       <c r="K45" s="23" t="inlineStr">
@@ -2284,7 +2286,7 @@
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="20" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B46" s="20" t="n">
@@ -2292,30 +2294,30 @@
       </c>
       <c r="C46" s="21" t="inlineStr">
         <is>
-          <t>한창</t>
+          <t>광진실업</t>
         </is>
       </c>
       <c r="D46" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E46" s="20" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F46" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G46" s="20" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H46" s="22" t="n">
-        <v>-91.06999999999999</v>
-      </c>
-      <c r="I46" s="22" t="n">
-        <v>-91.06999999999999</v>
+        <v>0.49</v>
+      </c>
+      <c r="I46" s="24" t="n">
+        <v>-18.6</v>
       </c>
       <c r="J46" s="23" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 한국경제 헤드라인 언급</t>
+          <t>중요공시 2건 / 중요공시 7일 +100%</t>
         </is>
       </c>
       <c r="K46" s="23" t="inlineStr">
@@ -2327,7 +2329,7 @@
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="20" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B47" s="20" t="n">
@@ -2335,7 +2337,7 @@
       </c>
       <c r="C47" s="21" t="inlineStr">
         <is>
-          <t>한화오션</t>
+          <t>미래산업</t>
         </is>
       </c>
       <c r="D47" s="20" t="n">
@@ -2350,11 +2352,11 @@
       <c r="G47" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="H47" s="24" t="n">
-        <v>0.13</v>
+      <c r="H47" s="22" t="n">
+        <v>0.6</v>
       </c>
       <c r="I47" s="22" t="n">
-        <v>-2.48</v>
+        <v>16.62</v>
       </c>
       <c r="J47" s="23" t="inlineStr">
         <is>
@@ -2370,7 +2372,7 @@
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="20" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B48" s="20" t="n">
@@ -2378,42 +2380,42 @@
       </c>
       <c r="C48" s="21" t="inlineStr">
         <is>
-          <t>미래산업</t>
+          <t>SK이노베이션</t>
         </is>
       </c>
       <c r="D48" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E48" s="20" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F48" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G48" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="H48" s="24" t="n">
-        <v>0.6</v>
+        <v>0</v>
+      </c>
+      <c r="H48" s="22" t="n">
+        <v>7.23</v>
       </c>
       <c r="I48" s="24" t="n">
-        <v>28.07</v>
+        <v>-4.78</v>
       </c>
       <c r="J48" s="23" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 7일 +100%</t>
+          <t>중요공시 1건 / 네이버뉴스 헤드라인 언급</t>
         </is>
       </c>
       <c r="K48" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="20" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B49" s="20" t="n">
@@ -2421,7 +2423,7 @@
       </c>
       <c r="C49" s="21" t="inlineStr">
         <is>
-          <t>일진전기</t>
+          <t>에스제이그룹</t>
         </is>
       </c>
       <c r="D49" s="20" t="n">
@@ -2436,11 +2438,11 @@
       <c r="G49" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H49" s="24" t="n">
-        <v>3.24</v>
-      </c>
-      <c r="I49" s="24" t="n">
-        <v>5.13</v>
+      <c r="H49" s="22" t="n">
+        <v>29.96</v>
+      </c>
+      <c r="I49" s="22" t="n">
+        <v>30.39</v>
       </c>
       <c r="J49" s="23" t="inlineStr">
         <is>
@@ -2456,7 +2458,7 @@
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="20" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B50" s="20" t="n">
@@ -2464,7 +2466,7 @@
       </c>
       <c r="C50" s="21" t="inlineStr">
         <is>
-          <t>씨싸이트</t>
+          <t>전기차</t>
         </is>
       </c>
       <c r="D50" s="20" t="n">
@@ -2479,27 +2481,25 @@
       <c r="G50" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H50" s="22" t="n">
-        <v>-4.62</v>
-      </c>
-      <c r="I50" s="24" t="n">
-        <v>52.19</v>
+      <c r="H50" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I50" s="20" t="n">
+        <v/>
       </c>
       <c r="J50" s="23" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 네이버뉴스 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K50" s="23" t="inlineStr">
-        <is>
-          <t>공시, 네이버</t>
-        </is>
+          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K50" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="20" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B51" s="20" t="n">
@@ -2507,7 +2507,7 @@
       </c>
       <c r="C51" s="21" t="inlineStr">
         <is>
-          <t>현대로템</t>
+          <t>스테이블코인</t>
         </is>
       </c>
       <c r="D51" s="20" t="n">
@@ -2522,27 +2522,25 @@
       <c r="G51" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H51" s="24" t="n">
-        <v>3.21</v>
-      </c>
-      <c r="I51" s="22" t="n">
-        <v>-0.77</v>
+      <c r="H51" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I51" s="20" t="n">
+        <v/>
       </c>
       <c r="J51" s="23" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 네이버뉴스 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K51" s="23" t="inlineStr">
-        <is>
-          <t>공시, 네이버</t>
-        </is>
+          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K51" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="20" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B52" s="20" t="n">
@@ -2550,7 +2548,7 @@
       </c>
       <c r="C52" s="21" t="inlineStr">
         <is>
-          <t>파두</t>
+          <t>현대건설</t>
         </is>
       </c>
       <c r="D52" s="20" t="n">
@@ -2565,15 +2563,15 @@
       <c r="G52" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H52" s="22" t="n">
-        <v>-2.58</v>
+      <c r="H52" s="24" t="n">
+        <v>-2.22</v>
       </c>
       <c r="I52" s="24" t="n">
-        <v>6.76</v>
+        <v>-6.9</v>
       </c>
       <c r="J52" s="23" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 한국경제 헤드라인 언급</t>
+          <t>한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K52" s="23" t="n">
@@ -2581,132 +2579,138 @@
       </c>
     </row>
     <row r="53" ht="18" customHeight="1">
-      <c r="A53" s="20" t="inlineStr">
-        <is>
-          <t>2026-10-03</t>
-        </is>
-      </c>
-      <c r="B53" s="20" t="n">
+      <c r="A53" s="25" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B53" s="25" t="n">
         <v>40</v>
       </c>
-      <c r="C53" s="21" t="inlineStr">
-        <is>
-          <t>전기차</t>
-        </is>
-      </c>
-      <c r="D53" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E53" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F53" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G53" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H53" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I53" s="20" t="n">
-        <v/>
-      </c>
-      <c r="J53" s="23" t="inlineStr">
-        <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K53" s="23" t="n">
-        <v/>
+      <c r="C53" s="26" t="inlineStr">
+        <is>
+          <t>브릴스</t>
+        </is>
+      </c>
+      <c r="D53" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E53" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F53" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G53" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H53" s="27" t="n">
+        <v>9.81</v>
+      </c>
+      <c r="I53" s="27" t="n">
+        <v>9.81</v>
+      </c>
+      <c r="J53" s="28" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +2242%</t>
+        </is>
+      </c>
+      <c r="K53" s="28" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="54" ht="18" customHeight="1">
-      <c r="A54" s="20" t="inlineStr">
-        <is>
-          <t>2026-10-03</t>
-        </is>
-      </c>
-      <c r="B54" s="20" t="n">
+      <c r="A54" s="25" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B54" s="25" t="n">
         <v>41</v>
       </c>
-      <c r="C54" s="21" t="inlineStr">
-        <is>
-          <t>스테이블코인</t>
-        </is>
-      </c>
-      <c r="D54" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E54" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F54" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G54" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H54" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I54" s="20" t="n">
-        <v/>
-      </c>
-      <c r="J54" s="23" t="inlineStr">
-        <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K54" s="23" t="n">
-        <v/>
+      <c r="C54" s="26" t="inlineStr">
+        <is>
+          <t>현대바이오랜드</t>
+        </is>
+      </c>
+      <c r="D54" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E54" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F54" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G54" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H54" s="29" t="n">
+        <v>-3.29</v>
+      </c>
+      <c r="I54" s="27" t="n">
+        <v>10.25</v>
+      </c>
+      <c r="J54" s="28" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +1609%</t>
+        </is>
+      </c>
+      <c r="K54" s="28" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="55" ht="18" customHeight="1">
-      <c r="A55" s="20" t="inlineStr">
-        <is>
-          <t>2026-10-03</t>
-        </is>
-      </c>
-      <c r="B55" s="20" t="n">
+      <c r="A55" s="25" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B55" s="25" t="n">
         <v>42</v>
       </c>
-      <c r="C55" s="21" t="inlineStr">
-        <is>
-          <t>NH투자증권</t>
-        </is>
-      </c>
-      <c r="D55" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E55" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F55" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G55" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H55" s="24" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="I55" s="24" t="n">
-        <v>2.87</v>
-      </c>
-      <c r="J55" s="23" t="inlineStr">
-        <is>
-          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K55" s="23" t="n">
-        <v/>
+      <c r="C55" s="26" t="inlineStr">
+        <is>
+          <t>코스모로보틱스</t>
+        </is>
+      </c>
+      <c r="D55" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E55" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F55" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G55" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H55" s="29" t="n">
+        <v>-8.460000000000001</v>
+      </c>
+      <c r="I55" s="29" t="n">
+        <v>-30.64</v>
+      </c>
+      <c r="J55" s="28" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +1375%</t>
+        </is>
+      </c>
+      <c r="K55" s="28" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="56" ht="18" customHeight="1">
       <c r="A56" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B56" s="25" t="n">
@@ -2714,7 +2718,7 @@
       </c>
       <c r="C56" s="26" t="inlineStr">
         <is>
-          <t>브릴스</t>
+          <t>글로벌테크놀로지</t>
         </is>
       </c>
       <c r="D56" s="25" t="n">
@@ -2729,15 +2733,15 @@
       <c r="G56" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H56" s="27" t="n">
-        <v>9.81</v>
+      <c r="H56" s="29" t="n">
+        <v>-8.550000000000001</v>
       </c>
       <c r="I56" s="27" t="n">
-        <v>9.81</v>
+        <v>2.48</v>
       </c>
       <c r="J56" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +1597%</t>
+          <t>네이버 검색 당일 +1355%</t>
         </is>
       </c>
       <c r="K56" s="28" t="inlineStr">
@@ -2749,7 +2753,7 @@
     <row r="57" ht="18" customHeight="1">
       <c r="A57" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B57" s="25" t="n">
@@ -2757,7 +2761,7 @@
       </c>
       <c r="C57" s="26" t="inlineStr">
         <is>
-          <t>현대바이오랜드</t>
+          <t>덕산넵코어스</t>
         </is>
       </c>
       <c r="D57" s="25" t="n">
@@ -2773,14 +2777,14 @@
         <v>0</v>
       </c>
       <c r="H57" s="29" t="n">
-        <v>-3.29</v>
-      </c>
-      <c r="I57" s="27" t="n">
-        <v>23.76</v>
+        <v>-1.75</v>
+      </c>
+      <c r="I57" s="29" t="n">
+        <v>-3.09</v>
       </c>
       <c r="J57" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +1461%</t>
+          <t>네이버 검색 당일 +1294%</t>
         </is>
       </c>
       <c r="K57" s="28" t="inlineStr">
@@ -2792,7 +2796,7 @@
     <row r="58" ht="18" customHeight="1">
       <c r="A58" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B58" s="25" t="n">
@@ -2800,7 +2804,7 @@
       </c>
       <c r="C58" s="26" t="inlineStr">
         <is>
-          <t>글로벌테크놀로지</t>
+          <t>빅웨이브로보틱스</t>
         </is>
       </c>
       <c r="D58" s="25" t="n">
@@ -2815,15 +2819,15 @@
       <c r="G58" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H58" s="29" t="n">
-        <v>-8.550000000000001</v>
+      <c r="H58" s="27" t="n">
+        <v>2.75</v>
       </c>
       <c r="I58" s="27" t="n">
-        <v>2.48</v>
+        <v>17.38</v>
       </c>
       <c r="J58" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +1238%</t>
+          <t>네이버 검색 당일 +1242%</t>
         </is>
       </c>
       <c r="K58" s="28" t="inlineStr">
@@ -2835,7 +2839,7 @@
     <row r="59" ht="18" customHeight="1">
       <c r="A59" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B59" s="25" t="n">
@@ -2843,7 +2847,7 @@
       </c>
       <c r="C59" s="26" t="inlineStr">
         <is>
-          <t>코스모로보틱스</t>
+          <t>덕우전자</t>
         </is>
       </c>
       <c r="D59" s="25" t="n">
@@ -2858,15 +2862,15 @@
       <c r="G59" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H59" s="29" t="n">
-        <v>-8.460000000000001</v>
-      </c>
-      <c r="I59" s="29" t="n">
-        <v>-30.94</v>
+      <c r="H59" s="27" t="n">
+        <v>17.91</v>
+      </c>
+      <c r="I59" s="27" t="n">
+        <v>53.62</v>
       </c>
       <c r="J59" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +1174%</t>
+          <t>네이버 검색 당일 +975%</t>
         </is>
       </c>
       <c r="K59" s="28" t="inlineStr">
@@ -2878,7 +2882,7 @@
     <row r="60" ht="18" customHeight="1">
       <c r="A60" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B60" s="25" t="n">
@@ -2886,7 +2890,7 @@
       </c>
       <c r="C60" s="26" t="inlineStr">
         <is>
-          <t>덕산넵코어스</t>
+          <t>부산주공</t>
         </is>
       </c>
       <c r="D60" s="25" t="n">
@@ -2902,14 +2906,14 @@
         <v>0</v>
       </c>
       <c r="H60" s="29" t="n">
-        <v>-1.75</v>
+        <v>-32.5</v>
       </c>
       <c r="I60" s="29" t="n">
-        <v>-3.09</v>
+        <v>-94.44</v>
       </c>
       <c r="J60" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +1124%</t>
+          <t>네이버 검색 당일 +721%</t>
         </is>
       </c>
       <c r="K60" s="28" t="inlineStr">
@@ -2921,7 +2925,7 @@
     <row r="61" ht="18" customHeight="1">
       <c r="A61" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B61" s="25" t="n">
@@ -2929,7 +2933,7 @@
       </c>
       <c r="C61" s="26" t="inlineStr">
         <is>
-          <t>빅웨이브로보틱스</t>
+          <t>원일티엔아이</t>
         </is>
       </c>
       <c r="D61" s="25" t="n">
@@ -2945,14 +2949,14 @@
         <v>0</v>
       </c>
       <c r="H61" s="27" t="n">
-        <v>2.75</v>
+        <v>18.34</v>
       </c>
       <c r="I61" s="27" t="n">
-        <v>17.38</v>
+        <v>54.33</v>
       </c>
       <c r="J61" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +1117%</t>
+          <t>네이버 검색 당일 +596%</t>
         </is>
       </c>
       <c r="K61" s="28" t="inlineStr">
@@ -2964,7 +2968,7 @@
     <row r="62" ht="18" customHeight="1">
       <c r="A62" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B62" s="25" t="n">
@@ -2972,7 +2976,7 @@
       </c>
       <c r="C62" s="26" t="inlineStr">
         <is>
-          <t>부산주공</t>
+          <t>KBI동양철관</t>
         </is>
       </c>
       <c r="D62" s="25" t="n">
@@ -2988,14 +2992,14 @@
         <v>0</v>
       </c>
       <c r="H62" s="29" t="n">
-        <v>-32.5</v>
-      </c>
-      <c r="I62" s="29" t="n">
-        <v>-94.44</v>
+        <v>-4.36</v>
+      </c>
+      <c r="I62" s="27" t="n">
+        <v>16.03</v>
       </c>
       <c r="J62" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +582%</t>
+          <t>네이버 검색 당일 +515%</t>
         </is>
       </c>
       <c r="K62" s="28" t="inlineStr">
@@ -3007,7 +3011,7 @@
     <row r="63" ht="18" customHeight="1">
       <c r="A63" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B63" s="25" t="n">
@@ -3015,7 +3019,7 @@
       </c>
       <c r="C63" s="26" t="inlineStr">
         <is>
-          <t>KBI동양철관</t>
+          <t>윈팩</t>
         </is>
       </c>
       <c r="D63" s="25" t="n">
@@ -3030,15 +3034,15 @@
       <c r="G63" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H63" s="29" t="n">
-        <v>-4.36</v>
+      <c r="H63" s="27" t="n">
+        <v>4.95</v>
       </c>
       <c r="I63" s="27" t="n">
-        <v>18.86</v>
+        <v>72.38</v>
       </c>
       <c r="J63" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +409%</t>
+          <t>네이버 검색 당일 +448%</t>
         </is>
       </c>
       <c r="K63" s="28" t="inlineStr">
@@ -3140,22 +3144,22 @@
         <v>1</v>
       </c>
       <c r="C3" s="25" t="n">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="D3" s="25" t="n">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="E3" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F3" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="G3" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="H3" s="25" t="n"/>
@@ -3171,29 +3175,29 @@
         <v>1</v>
       </c>
       <c r="C4" s="25" t="n">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="D4" s="25" t="n">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="E4" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F4" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="G4" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="H4" s="27" t="n">
         <v>0.55</v>
       </c>
-      <c r="I4" s="29" t="n">
-        <v>-3.66</v>
+      <c r="I4" s="27" t="n">
+        <v>2.22</v>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
@@ -3206,22 +3210,22 @@
         <v>1</v>
       </c>
       <c r="C5" s="25" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D5" s="25" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E5" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F5" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="G5" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="H5" s="25" t="n"/>
@@ -3237,29 +3241,29 @@
         <v>1</v>
       </c>
       <c r="C6" s="25" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D6" s="25" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E6" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F6" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="G6" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="H6" s="29" t="n">
         <v>-0.57</v>
       </c>
       <c r="I6" s="29" t="n">
-        <v>-2.8</v>
+        <v>-1.98</v>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1">
@@ -3272,22 +3276,22 @@
         <v>1</v>
       </c>
       <c r="C7" s="25" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D7" s="25" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E7" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F7" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="G7" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="H7" s="25" t="n"/>
@@ -3296,29 +3300,29 @@
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="26" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>원전</t>
         </is>
       </c>
       <c r="B8" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="25" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D8" s="25" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E8" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F8" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="G8" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="H8" s="25" t="n"/>
@@ -3327,29 +3331,29 @@
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="26" t="inlineStr">
         <is>
-          <t>철강</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="B9" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="25" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D9" s="25" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E9" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F9" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="G9" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="H9" s="25" t="n"/>
@@ -3358,7 +3362,7 @@
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="26" t="inlineStr">
         <is>
-          <t>SK하이닉스</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="B10" s="25" t="n">
@@ -3375,51 +3379,51 @@
       </c>
       <c r="F10" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="G10" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
-        </is>
-      </c>
-      <c r="H10" s="27" t="n">
-        <v>0.77</v>
-      </c>
-      <c r="I10" s="29" t="n">
-        <v>-1.13</v>
-      </c>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="H10" s="25" t="n"/>
+      <c r="I10" s="25" t="n"/>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="26" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>SK하이닉스</t>
         </is>
       </c>
       <c r="B11" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D11" s="25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E11" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F11" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="G11" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
-        </is>
-      </c>
-      <c r="H11" s="25" t="n"/>
-      <c r="I11" s="25" t="n"/>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="H11" s="27" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="I11" s="27" t="n">
+        <v>4.6</v>
+      </c>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="26" t="inlineStr">
@@ -3441,25 +3445,25 @@
       </c>
       <c r="F12" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="G12" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="H12" s="27" t="n">
         <v>0.84</v>
       </c>
       <c r="I12" s="29" t="n">
-        <v>-3.53</v>
+        <v>-4.11</v>
       </c>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>에스제이그룹</t>
+          <t>철강</t>
         </is>
       </c>
       <c r="B13" s="25" t="n">
@@ -3476,60 +3480,56 @@
       </c>
       <c r="F13" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="G13" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
-        </is>
-      </c>
-      <c r="H13" s="27" t="n">
-        <v>29.96</v>
-      </c>
-      <c r="I13" s="27" t="n">
-        <v>26.45</v>
-      </c>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="H13" s="25" t="n"/>
+      <c r="I13" s="25" t="n"/>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>SG</t>
+          <t>한창</t>
         </is>
       </c>
       <c r="B14" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C14" s="25" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D14" s="25" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E14" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F14" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="G14" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="H14" s="29" t="n">
-        <v>-5.15</v>
+        <v>-91.06999999999999</v>
       </c>
       <c r="I14" s="29" t="n">
-        <v>-8.68</v>
+        <v>-91.06999999999999</v>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>모아데이타</t>
+          <t>SG</t>
         </is>
       </c>
       <c r="B15" s="25" t="n">
@@ -3546,25 +3546,25 @@
       </c>
       <c r="F15" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="G15" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="H15" s="29" t="n">
-        <v>-3.6</v>
+        <v>-5.15</v>
       </c>
       <c r="I15" s="29" t="n">
-        <v>-13.01</v>
+        <v>-2.64</v>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>선도전기</t>
+          <t>모아데이타</t>
         </is>
       </c>
       <c r="B16" s="25" t="n">
@@ -3581,25 +3581,25 @@
       </c>
       <c r="F16" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="G16" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="H16" s="29" t="n">
-        <v>-1.82</v>
+        <v>-3.6</v>
       </c>
       <c r="I16" s="29" t="n">
-        <v>-4.44</v>
+        <v>-1.83</v>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>아리바이오홀딩스</t>
+          <t>세미파이브</t>
         </is>
       </c>
       <c r="B17" s="25" t="n">
@@ -3616,91 +3616,95 @@
       </c>
       <c r="F17" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="G17" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
-        </is>
-      </c>
-      <c r="H17" s="29" t="n">
-        <v>-2.23</v>
-      </c>
-      <c r="I17" s="29" t="n">
-        <v>-22.77</v>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="H17" s="27" t="n">
+        <v>1.72</v>
+      </c>
+      <c r="I17" s="27" t="n">
+        <v>28.88</v>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="26" t="inlineStr">
         <is>
-          <t>원전</t>
+          <t>두산에너빌리티</t>
         </is>
       </c>
       <c r="B18" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C18" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D18" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E18" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F18" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="G18" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
-        </is>
-      </c>
-      <c r="H18" s="25" t="n"/>
-      <c r="I18" s="25" t="n"/>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="H18" s="29" t="n">
+        <v>-1.09</v>
+      </c>
+      <c r="I18" s="27" t="n">
+        <v>0.37</v>
+      </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>티엠씨</t>
+          <t>머큐리</t>
         </is>
       </c>
       <c r="B19" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C19" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D19" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E19" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F19" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="G19" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="H19" s="27" t="n">
-        <v>29.68</v>
+        <v>29.8</v>
       </c>
       <c r="I19" s="27" t="n">
-        <v>28.86</v>
+        <v>28.21</v>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="26" t="inlineStr">
         <is>
-          <t>LG전자</t>
+          <t>팬오션</t>
         </is>
       </c>
       <c r="B20" s="25" t="n">
@@ -3717,270 +3721,270 @@
       </c>
       <c r="F20" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="G20" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="H20" s="27" t="n">
-        <v>1.65</v>
+        <v>6.47</v>
       </c>
       <c r="I20" s="27" t="n">
-        <v>2.38</v>
+        <v>9.84</v>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="26" t="inlineStr">
         <is>
-          <t>더코디</t>
+          <t>SK이노베이션</t>
         </is>
       </c>
       <c r="B21" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C21" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D21" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E21" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F21" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="G21" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
-        </is>
-      </c>
-      <c r="H21" s="29" t="n">
-        <v>-1.27</v>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="H21" s="27" t="n">
+        <v>7.23</v>
       </c>
       <c r="I21" s="29" t="n">
-        <v>-2.96</v>
+        <v>-4.78</v>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="26" t="inlineStr">
         <is>
-          <t>삼성전기</t>
+          <t>고영</t>
         </is>
       </c>
       <c r="B22" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C22" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D22" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E22" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F22" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="G22" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="H22" s="27" t="n">
-        <v>1.48</v>
+        <v>1.47</v>
       </c>
       <c r="I22" s="27" t="n">
-        <v>5.06</v>
+        <v>19.41</v>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="26" t="inlineStr">
         <is>
-          <t>에이전트AI</t>
+          <t>광진실업</t>
         </is>
       </c>
       <c r="B23" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C23" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D23" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E23" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F23" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="G23" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
-        </is>
-      </c>
-      <c r="H23" s="29" t="n">
-        <v>-2.34</v>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="H23" s="27" t="n">
+        <v>0.49</v>
       </c>
       <c r="I23" s="29" t="n">
-        <v>-39.85</v>
+        <v>-18.6</v>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="26" t="inlineStr">
         <is>
-          <t>에코프로</t>
+          <t>나인테크</t>
         </is>
       </c>
       <c r="B24" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C24" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D24" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E24" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F24" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="G24" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="H24" s="27" t="n">
-        <v>5.07</v>
+        <v>0.71</v>
       </c>
       <c r="I24" s="27" t="n">
-        <v>11.24</v>
+        <v>28.05</v>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="26" t="inlineStr">
         <is>
-          <t>에코프로머티</t>
+          <t>루닛</t>
         </is>
       </c>
       <c r="B25" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C25" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D25" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E25" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F25" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="G25" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
-        </is>
-      </c>
-      <c r="H25" s="27" t="n">
-        <v>3.8</v>
-      </c>
-      <c r="I25" s="27" t="n">
-        <v>8.99</v>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="H25" s="29" t="n">
+        <v>-5.03</v>
+      </c>
+      <c r="I25" s="29" t="n">
+        <v>-5.88</v>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="26" t="inlineStr">
         <is>
-          <t>에코프로비엠</t>
+          <t>미래산업</t>
         </is>
       </c>
       <c r="B26" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C26" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D26" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E26" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F26" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="G26" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="H26" s="27" t="n">
-        <v>1.58</v>
+        <v>0.6</v>
       </c>
       <c r="I26" s="27" t="n">
-        <v>9.57</v>
+        <v>16.62</v>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="26" t="inlineStr">
         <is>
-          <t>에코프로에이치엔</t>
+          <t>빛샘전자</t>
         </is>
       </c>
       <c r="B27" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C27" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D27" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E27" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F27" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="G27" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="H27" s="27" t="n">
-        <v>1.02</v>
+        <v>11.65</v>
       </c>
       <c r="I27" s="27" t="n">
-        <v>13.73</v>
+        <v>26.1</v>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="26" t="inlineStr">
         <is>
-          <t>NH투자증권</t>
+          <t>삼성중공업</t>
         </is>
       </c>
       <c r="B28" s="25" t="n">
@@ -3997,25 +4001,25 @@
       </c>
       <c r="F28" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="G28" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="H28" s="27" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="I28" s="27" t="n">
-        <v>2.87</v>
+        <v>0.91</v>
+      </c>
+      <c r="I28" s="29" t="n">
+        <v>-1.14</v>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="26" t="inlineStr">
         <is>
-          <t>나인테크</t>
+          <t>선도전기</t>
         </is>
       </c>
       <c r="B29" s="25" t="n">
@@ -4032,25 +4036,25 @@
       </c>
       <c r="F29" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="G29" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
-        </is>
-      </c>
-      <c r="H29" s="27" t="n">
-        <v>0.71</v>
-      </c>
-      <c r="I29" s="27" t="n">
-        <v>29.52</v>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="H29" s="29" t="n">
+        <v>-1.82</v>
+      </c>
+      <c r="I29" s="29" t="n">
+        <v>-1.82</v>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="26" t="inlineStr">
         <is>
-          <t>두산에너빌리티</t>
+          <t>성호전자</t>
         </is>
       </c>
       <c r="B30" s="25" t="n">
@@ -4067,25 +4071,25 @@
       </c>
       <c r="F30" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="G30" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
-        </is>
-      </c>
-      <c r="H30" s="29" t="n">
-        <v>-1.09</v>
-      </c>
-      <c r="I30" s="29" t="n">
-        <v>-1.57</v>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="H30" s="27" t="n">
+        <v>11.35</v>
+      </c>
+      <c r="I30" s="27" t="n">
+        <v>27.13</v>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="26" t="inlineStr">
         <is>
-          <t>미래산업</t>
+          <t>스테이블코인</t>
         </is>
       </c>
       <c r="B31" s="25" t="n">
@@ -4102,25 +4106,21 @@
       </c>
       <c r="F31" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="G31" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
-        </is>
-      </c>
-      <c r="H31" s="27" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="I31" s="27" t="n">
-        <v>28.07</v>
-      </c>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="H31" s="25" t="n"/>
+      <c r="I31" s="25" t="n"/>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="26" t="inlineStr">
         <is>
-          <t>세미파이브</t>
+          <t>아리바이오홀딩스</t>
         </is>
       </c>
       <c r="B32" s="25" t="n">
@@ -4137,25 +4137,25 @@
       </c>
       <c r="F32" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="G32" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
-        </is>
-      </c>
-      <c r="H32" s="27" t="n">
-        <v>1.72</v>
-      </c>
-      <c r="I32" s="27" t="n">
-        <v>27.38</v>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="H32" s="29" t="n">
+        <v>-2.23</v>
+      </c>
+      <c r="I32" s="29" t="n">
+        <v>-22.96</v>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="26" t="inlineStr">
         <is>
-          <t>스테이블코인</t>
+          <t>에스제이그룹</t>
         </is>
       </c>
       <c r="B33" s="25" t="n">
@@ -4172,21 +4172,25 @@
       </c>
       <c r="F33" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="G33" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
-        </is>
-      </c>
-      <c r="H33" s="25" t="n"/>
-      <c r="I33" s="25" t="n"/>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="H33" s="27" t="n">
+        <v>29.96</v>
+      </c>
+      <c r="I33" s="27" t="n">
+        <v>30.39</v>
+      </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="26" t="inlineStr">
         <is>
-          <t>씨싸이트</t>
+          <t>에이에프더블류</t>
         </is>
       </c>
       <c r="B34" s="25" t="n">
@@ -4203,25 +4207,25 @@
       </c>
       <c r="F34" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="G34" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="H34" s="29" t="n">
-        <v>-4.62</v>
-      </c>
-      <c r="I34" s="27" t="n">
-        <v>52.19</v>
+        <v>-5.13</v>
+      </c>
+      <c r="I34" s="29" t="n">
+        <v>-51.32</v>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="26" t="inlineStr">
         <is>
-          <t>일진전기</t>
+          <t>우리기술</t>
         </is>
       </c>
       <c r="B35" s="25" t="n">
@@ -4238,19 +4242,19 @@
       </c>
       <c r="F35" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="G35" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="H35" s="27" t="n">
-        <v>3.24</v>
+        <v>1.75</v>
       </c>
       <c r="I35" s="27" t="n">
-        <v>5.13</v>
+        <v>1.19</v>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
@@ -4273,12 +4277,12 @@
       </c>
       <c r="F36" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="G36" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="H36" s="25" t="n"/>
@@ -4304,25 +4308,25 @@
       </c>
       <c r="F37" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="G37" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="H37" s="29" t="n">
         <v>-1.63</v>
       </c>
       <c r="I37" s="29" t="n">
-        <v>-58.04</v>
+        <v>-51.68</v>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="26" t="inlineStr">
         <is>
-          <t>파두</t>
+          <t>한국파마</t>
         </is>
       </c>
       <c r="B38" s="25" t="n">
@@ -4339,25 +4343,25 @@
       </c>
       <c r="F38" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="G38" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
-        </is>
-      </c>
-      <c r="H38" s="29" t="n">
-        <v>-2.58</v>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="H38" s="27" t="n">
+        <v>13.42</v>
       </c>
       <c r="I38" s="27" t="n">
-        <v>6.76</v>
+        <v>19.06</v>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="26" t="inlineStr">
         <is>
-          <t>팬오션</t>
+          <t>한화솔루션</t>
         </is>
       </c>
       <c r="B39" s="25" t="n">
@@ -4374,25 +4378,25 @@
       </c>
       <c r="F39" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="G39" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="H39" s="27" t="n">
-        <v>6.47</v>
+        <v>5.71</v>
       </c>
       <c r="I39" s="27" t="n">
-        <v>11.41</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="26" t="inlineStr">
         <is>
-          <t>한창</t>
+          <t>한화오션</t>
         </is>
       </c>
       <c r="B40" s="25" t="n">
@@ -4409,25 +4413,25 @@
       </c>
       <c r="F40" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="G40" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
-        </is>
-      </c>
-      <c r="H40" s="29" t="n">
-        <v>-91.06999999999999</v>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="H40" s="27" t="n">
+        <v>0.13</v>
       </c>
       <c r="I40" s="29" t="n">
-        <v>-91.06999999999999</v>
+        <v>-2.24</v>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="26" t="inlineStr">
         <is>
-          <t>한화생명</t>
+          <t>현대건설</t>
         </is>
       </c>
       <c r="B41" s="25" t="n">
@@ -4444,130 +4448,130 @@
       </c>
       <c r="F41" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="G41" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
-        </is>
-      </c>
-      <c r="H41" s="27" t="n">
-        <v>0.38</v>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="H41" s="29" t="n">
+        <v>-2.22</v>
       </c>
       <c r="I41" s="29" t="n">
-        <v>-6.34</v>
+        <v>-6.9</v>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="26" t="inlineStr">
         <is>
-          <t>한화솔루션</t>
+          <t>KBI동양철관</t>
         </is>
       </c>
       <c r="B42" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C42" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D42" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E42" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F42" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="G42" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
-        </is>
-      </c>
-      <c r="H42" s="27" t="n">
-        <v>5.71</v>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="H42" s="29" t="n">
+        <v>-4.36</v>
       </c>
       <c r="I42" s="27" t="n">
-        <v>22.79</v>
+        <v>16.03</v>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="26" t="inlineStr">
         <is>
-          <t>한화오션</t>
+          <t>글로벌테크놀로지</t>
         </is>
       </c>
       <c r="B43" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C43" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D43" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E43" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F43" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="G43" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
-        </is>
-      </c>
-      <c r="H43" s="27" t="n">
-        <v>0.13</v>
-      </c>
-      <c r="I43" s="29" t="n">
-        <v>-2.48</v>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="H43" s="29" t="n">
+        <v>-8.550000000000001</v>
+      </c>
+      <c r="I43" s="27" t="n">
+        <v>2.48</v>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="26" t="inlineStr">
         <is>
-          <t>현대로템</t>
+          <t>덕산넵코어스</t>
         </is>
       </c>
       <c r="B44" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C44" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D44" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E44" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F44" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="G44" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
-        </is>
-      </c>
-      <c r="H44" s="27" t="n">
-        <v>3.21</v>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="H44" s="29" t="n">
+        <v>-1.75</v>
       </c>
       <c r="I44" s="29" t="n">
-        <v>-0.77</v>
+        <v>-3.09</v>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="26" t="inlineStr">
         <is>
-          <t>KBI동양철관</t>
+          <t>덕우전자</t>
         </is>
       </c>
       <c r="B45" s="25" t="n">
@@ -4584,25 +4588,25 @@
       </c>
       <c r="F45" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="G45" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
-        </is>
-      </c>
-      <c r="H45" s="29" t="n">
-        <v>-4.36</v>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="H45" s="27" t="n">
+        <v>17.91</v>
       </c>
       <c r="I45" s="27" t="n">
-        <v>18.86</v>
+        <v>53.62</v>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="26" t="inlineStr">
         <is>
-          <t>글로벌테크놀로지</t>
+          <t>부산주공</t>
         </is>
       </c>
       <c r="B46" s="25" t="n">
@@ -4619,25 +4623,25 @@
       </c>
       <c r="F46" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="G46" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="H46" s="29" t="n">
-        <v>-8.550000000000001</v>
-      </c>
-      <c r="I46" s="27" t="n">
-        <v>2.48</v>
+        <v>-32.5</v>
+      </c>
+      <c r="I46" s="29" t="n">
+        <v>-94.44</v>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="26" t="inlineStr">
         <is>
-          <t>덕산넵코어스</t>
+          <t>브릴스</t>
         </is>
       </c>
       <c r="B47" s="25" t="n">
@@ -4654,25 +4658,25 @@
       </c>
       <c r="F47" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="G47" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
-        </is>
-      </c>
-      <c r="H47" s="29" t="n">
-        <v>-1.75</v>
-      </c>
-      <c r="I47" s="29" t="n">
-        <v>-3.09</v>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="H47" s="27" t="n">
+        <v>9.81</v>
+      </c>
+      <c r="I47" s="27" t="n">
+        <v>9.81</v>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="26" t="inlineStr">
         <is>
-          <t>부산주공</t>
+          <t>빅웨이브로보틱스</t>
         </is>
       </c>
       <c r="B48" s="25" t="n">
@@ -4689,25 +4693,25 @@
       </c>
       <c r="F48" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="G48" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
-        </is>
-      </c>
-      <c r="H48" s="29" t="n">
-        <v>-32.5</v>
-      </c>
-      <c r="I48" s="29" t="n">
-        <v>-94.44</v>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="H48" s="27" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="I48" s="27" t="n">
+        <v>17.38</v>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="26" t="inlineStr">
         <is>
-          <t>브릴스</t>
+          <t>원일티엔아이</t>
         </is>
       </c>
       <c r="B49" s="25" t="n">
@@ -4724,25 +4728,25 @@
       </c>
       <c r="F49" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="G49" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="H49" s="27" t="n">
-        <v>9.81</v>
+        <v>18.34</v>
       </c>
       <c r="I49" s="27" t="n">
-        <v>9.81</v>
+        <v>54.33</v>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="26" t="inlineStr">
         <is>
-          <t>빅웨이브로보틱스</t>
+          <t>윈팩</t>
         </is>
       </c>
       <c r="B50" s="25" t="n">
@@ -4759,19 +4763,19 @@
       </c>
       <c r="F50" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="G50" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="H50" s="27" t="n">
-        <v>2.75</v>
+        <v>4.95</v>
       </c>
       <c r="I50" s="27" t="n">
-        <v>17.38</v>
+        <v>72.38</v>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
@@ -4794,19 +4798,19 @@
       </c>
       <c r="F51" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="G51" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="H51" s="29" t="n">
         <v>-8.460000000000001</v>
       </c>
       <c r="I51" s="29" t="n">
-        <v>-30.94</v>
+        <v>-30.64</v>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
@@ -4829,19 +4833,19 @@
       </c>
       <c r="F52" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="G52" s="25" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="H52" s="29" t="n">
         <v>-3.29</v>
       </c>
       <c r="I52" s="27" t="n">
-        <v>23.76</v>
+        <v>10.25</v>
       </c>
     </row>
   </sheetData>
@@ -4925,19 +4929,19 @@
         <v>1</v>
       </c>
       <c r="C3" s="36" t="n">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="D3" s="36" t="n">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="E3" s="36" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="F3" s="37" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="G3" s="37" t="inlineStr">
@@ -4956,19 +4960,19 @@
         <v>1</v>
       </c>
       <c r="C4" s="36" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D4" s="36" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E4" s="36" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="F4" s="37" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="G4" s="37" t="inlineStr">
@@ -4994,12 +4998,12 @@
       </c>
       <c r="E5" s="36" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="F5" s="37" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="G5" s="37" t="inlineStr">
@@ -5018,19 +5022,19 @@
         <v>1</v>
       </c>
       <c r="C6" s="36" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="D6" s="36" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="E6" s="36" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="F6" s="37" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="G6" s="37" t="inlineStr">
@@ -5049,19 +5053,19 @@
         <v>1</v>
       </c>
       <c r="C7" s="36" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D7" s="36" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E7" s="36" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="F7" s="37" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="G7" s="37" t="inlineStr">
@@ -5080,19 +5084,19 @@
         <v>1</v>
       </c>
       <c r="C8" s="36" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D8" s="36" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="E8" s="36" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="F8" s="37" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="G8" s="37" t="inlineStr">
@@ -5111,19 +5115,19 @@
         <v>1</v>
       </c>
       <c r="C9" s="36" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D9" s="36" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E9" s="36" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="F9" s="37" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="G9" s="37" t="inlineStr">
@@ -5142,19 +5146,19 @@
         <v>1</v>
       </c>
       <c r="C10" s="36" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D10" s="36" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E10" s="36" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="F10" s="37" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="G10" s="37" t="inlineStr">

</xml_diff>

<commit_message>
auto: 2026-10-05 07:23 자동 백업
</commit_message>
<xml_diff>
--- a/trend/stock_trend_history.xlsx
+++ b/trend/stock_trend_history.xlsx
@@ -694,7 +694,7 @@
     <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-10-04 06:54</t>
+          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-10-05 06:54</t>
         </is>
       </c>
     </row>
@@ -708,7 +708,7 @@
       </c>
       <c r="E3" s="3" t="n"/>
       <c r="G3" s="5" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H3" s="3" t="n"/>
       <c r="J3" s="6" t="n">
@@ -787,21 +787,21 @@
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-10-04) 상위: 반도체  점수 48.0점</t>
+          <t>⚡ 최신(2026-10-05) 상위: 반도체  점수 51.0점</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-10-04) 상위: 삼성전자  점수 35.0점</t>
+          <t>⚡ 최신(2026-10-05) 상위: 삼성전자  점수 43.0점</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-10-04) 상위: 인공지능  점수 24.0점</t>
+          <t>⚡ 최신(2026-10-05) 상위: 인공지능  점수 24.0점</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="15" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B14" s="15" t="n">
@@ -928,10 +928,10 @@
         </is>
       </c>
       <c r="D14" s="15" t="n">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="E14" s="15" t="n">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="F14" s="15" t="n">
         <v>0</v>
@@ -947,7 +947,7 @@
       </c>
       <c r="J14" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+          <t>네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K14" s="17" t="inlineStr">
@@ -959,7 +959,7 @@
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="15" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B15" s="15" t="n">
@@ -971,10 +971,10 @@
         </is>
       </c>
       <c r="D15" s="15" t="n">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="E15" s="15" t="n">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="F15" s="15" t="n">
         <v>0</v>
@@ -990,7 +990,7 @@
       </c>
       <c r="J15" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급</t>
         </is>
       </c>
       <c r="K15" s="17" t="inlineStr">
@@ -1002,7 +1002,7 @@
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="15" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B16" s="15" t="n">
@@ -1033,7 +1033,7 @@
       </c>
       <c r="J16" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급</t>
+          <t>매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K16" s="17" t="inlineStr">
@@ -1045,7 +1045,7 @@
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B17" s="15" t="n">
@@ -1057,10 +1057,10 @@
         </is>
       </c>
       <c r="D17" s="15" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="E17" s="15" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="F17" s="15" t="n">
         <v>0</v>
@@ -1076,7 +1076,7 @@
       </c>
       <c r="J17" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K17" s="17" t="n">
@@ -1086,7 +1086,7 @@
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B18" s="15" t="n">
@@ -1094,14 +1094,14 @@
       </c>
       <c r="C18" s="16" t="inlineStr">
         <is>
-          <t>원전</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="D18" s="15" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E18" s="15" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F18" s="15" t="n">
         <v>0</v>
@@ -1117,7 +1117,7 @@
       </c>
       <c r="J18" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급</t>
         </is>
       </c>
       <c r="K18" s="17" t="inlineStr">
@@ -1129,7 +1129,7 @@
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B19" s="15" t="n">
@@ -1137,14 +1137,14 @@
       </c>
       <c r="C19" s="16" t="inlineStr">
         <is>
-          <t>바이오</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="D19" s="15" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E19" s="15" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F19" s="15" t="n">
         <v>0</v>
@@ -1160,7 +1160,7 @@
       </c>
       <c r="J19" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 한국경제 헤드라인 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K19" s="17" t="inlineStr">
@@ -1172,7 +1172,7 @@
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B20" s="15" t="n">
@@ -1180,14 +1180,14 @@
       </c>
       <c r="C20" s="16" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>바이오</t>
         </is>
       </c>
       <c r="D20" s="15" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E20" s="15" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F20" s="15" t="n">
         <v>0</v>
@@ -1203,7 +1203,7 @@
       </c>
       <c r="J20" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K20" s="17" t="inlineStr">
@@ -1215,7 +1215,7 @@
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="15" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B21" s="15" t="n">
@@ -1223,7 +1223,7 @@
       </c>
       <c r="C21" s="16" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>SK하이닉스</t>
         </is>
       </c>
       <c r="D21" s="15" t="n">
@@ -1238,15 +1238,15 @@
       <c r="G21" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H21" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I21" s="15" t="n">
-        <v/>
+      <c r="H21" s="18" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="I21" s="18" t="n">
+        <v>4.6</v>
       </c>
       <c r="J21" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+          <t>매일경제 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K21" s="17" t="inlineStr">
@@ -1258,7 +1258,7 @@
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="15" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B22" s="15" t="n">
@@ -1266,42 +1266,42 @@
       </c>
       <c r="C22" s="16" t="inlineStr">
         <is>
-          <t>한창</t>
+          <t>삼성E&amp;A</t>
         </is>
       </c>
       <c r="D22" s="15" t="n">
         <v>7</v>
       </c>
       <c r="E22" s="15" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="F22" s="15" t="n">
         <v>0</v>
       </c>
       <c r="G22" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H22" s="19" t="n">
-        <v>-91.06999999999999</v>
+        <v>3</v>
+      </c>
+      <c r="H22" s="18" t="n">
+        <v>0.84</v>
       </c>
       <c r="I22" s="19" t="n">
-        <v>-91.06999999999999</v>
+        <v>-4.11</v>
       </c>
       <c r="J22" s="17" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +143% / 중요공시 1건 / 한국경제 헤드라인 언급</t>
+          <t>중요공시 2건 / 중요공시 7일 +100% / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K22" s="17" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="15" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B23" s="15" t="n">
@@ -1309,7 +1309,7 @@
       </c>
       <c r="C23" s="16" t="inlineStr">
         <is>
-          <t>SK하이닉스</t>
+          <t>원전</t>
         </is>
       </c>
       <c r="D23" s="15" t="n">
@@ -1324,27 +1324,25 @@
       <c r="G23" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H23" s="18" t="n">
-        <v>0.77</v>
-      </c>
-      <c r="I23" s="18" t="n">
-        <v>4.6</v>
+      <c r="H23" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I23" s="15" t="n">
+        <v/>
       </c>
       <c r="J23" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K23" s="17" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K23" s="17" t="n">
+        <v/>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="15" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B24" s="15" t="n">
@@ -1352,83 +1350,83 @@
       </c>
       <c r="C24" s="16" t="inlineStr">
         <is>
-          <t>삼성E&amp;A</t>
+          <t>스테이블코인</t>
         </is>
       </c>
       <c r="D24" s="15" t="n">
         <v>7</v>
       </c>
       <c r="E24" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="F24" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I24" s="15" t="n">
+        <v/>
+      </c>
+      <c r="J24" s="17" t="inlineStr">
+        <is>
+          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K24" s="17" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="20" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B25" s="20" t="n">
+        <v>12</v>
+      </c>
+      <c r="C25" s="21" t="inlineStr">
+        <is>
+          <t>세미파이브</t>
+        </is>
+      </c>
+      <c r="D25" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="E25" s="20" t="n">
         <v>4</v>
       </c>
-      <c r="F24" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="G24" s="15" t="n">
-        <v>3</v>
-      </c>
-      <c r="H24" s="18" t="n">
-        <v>0.84</v>
-      </c>
-      <c r="I24" s="19" t="n">
-        <v>-4.11</v>
-      </c>
-      <c r="J24" s="17" t="inlineStr">
-        <is>
-          <t>중요공시 2건 / 중요공시 7일 +100% / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K24" s="17" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="18" customHeight="1">
-      <c r="A25" s="15" t="inlineStr">
-        <is>
-          <t>2026-10-04</t>
-        </is>
-      </c>
-      <c r="B25" s="15" t="n">
-        <v>12</v>
-      </c>
-      <c r="C25" s="16" t="inlineStr">
-        <is>
-          <t>철강</t>
-        </is>
-      </c>
-      <c r="D25" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="E25" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="F25" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="G25" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H25" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I25" s="15" t="n">
-        <v/>
-      </c>
-      <c r="J25" s="17" t="inlineStr">
-        <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K25" s="17" t="n">
-        <v/>
+      <c r="F25" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="G25" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" s="22" t="n">
+        <v>1.72</v>
+      </c>
+      <c r="I25" s="22" t="n">
+        <v>28.88</v>
+      </c>
+      <c r="J25" s="23" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +458% / 중요공시 2건 / 중요공시 3일 +100%</t>
+        </is>
+      </c>
+      <c r="K25" s="23" t="inlineStr">
+        <is>
+          <t>공시, 네이버</t>
+        </is>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="20" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B26" s="20" t="n">
@@ -1436,7 +1434,7 @@
       </c>
       <c r="C26" s="21" t="inlineStr">
         <is>
-          <t>세미파이브</t>
+          <t>삼성중공업</t>
         </is>
       </c>
       <c r="D26" s="20" t="n">
@@ -1452,26 +1450,26 @@
         <v>0</v>
       </c>
       <c r="H26" s="22" t="n">
-        <v>1.72</v>
-      </c>
-      <c r="I26" s="22" t="n">
-        <v>28.88</v>
+        <v>0.91</v>
+      </c>
+      <c r="I26" s="24" t="n">
+        <v>-1.14</v>
       </c>
       <c r="J26" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +437% / 중요공시 2건 / 중요공시 3일 +100%</t>
+          <t>네이버 검색 당일 +57% / 중요공시 2건 / 중요공시 3일 +100% / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K26" s="23" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="20" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B27" s="20" t="n">
@@ -1479,7 +1477,7 @@
       </c>
       <c r="C27" s="21" t="inlineStr">
         <is>
-          <t>SG</t>
+          <t>대한항공</t>
         </is>
       </c>
       <c r="D27" s="20" t="n">
@@ -1495,24 +1493,26 @@
         <v>0</v>
       </c>
       <c r="H27" s="24" t="n">
-        <v>-5.15</v>
+        <v>-0.64</v>
       </c>
       <c r="I27" s="24" t="n">
-        <v>-2.64</v>
+        <v>-1.91</v>
       </c>
       <c r="J27" s="23" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K27" s="23" t="n">
-        <v/>
+          <t>중요공시 2건 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K27" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="20" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B28" s="20" t="n">
@@ -1520,42 +1520,40 @@
       </c>
       <c r="C28" s="21" t="inlineStr">
         <is>
-          <t>모아데이타</t>
+          <t>SG</t>
         </is>
       </c>
       <c r="D28" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E28" s="20" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F28" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G28" s="20" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H28" s="24" t="n">
-        <v>-3.6</v>
+        <v>-5.15</v>
       </c>
       <c r="I28" s="24" t="n">
-        <v>-1.83</v>
+        <v>-2.64</v>
       </c>
       <c r="J28" s="23" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 7일 +50%</t>
-        </is>
-      </c>
-      <c r="K28" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K28" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="20" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B29" s="20" t="n">
@@ -1563,42 +1561,42 @@
       </c>
       <c r="C29" s="21" t="inlineStr">
         <is>
-          <t>머큐리</t>
+          <t>모아데이타</t>
         </is>
       </c>
       <c r="D29" s="20" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E29" s="20" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F29" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G29" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H29" s="22" t="n">
-        <v>29.8</v>
-      </c>
-      <c r="I29" s="22" t="n">
-        <v>28.21</v>
+        <v>3</v>
+      </c>
+      <c r="H29" s="24" t="n">
+        <v>-3.6</v>
+      </c>
+      <c r="I29" s="24" t="n">
+        <v>-1.83</v>
       </c>
       <c r="J29" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +69% / 매일경제 헤드라인 언급</t>
+          <t>중요공시 3건 / 중요공시 7일 +50%</t>
         </is>
       </c>
       <c r="K29" s="23" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="20" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B30" s="20" t="n">
@@ -1606,42 +1604,42 @@
       </c>
       <c r="C30" s="21" t="inlineStr">
         <is>
-          <t>팬오션</t>
+          <t>루닛</t>
         </is>
       </c>
       <c r="D30" s="20" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E30" s="20" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F30" s="20" t="n">
         <v>2</v>
       </c>
       <c r="G30" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H30" s="22" t="n">
-        <v>6.47</v>
-      </c>
-      <c r="I30" s="22" t="n">
-        <v>9.84</v>
+        <v>3</v>
+      </c>
+      <c r="H30" s="24" t="n">
+        <v>-5.03</v>
+      </c>
+      <c r="I30" s="24" t="n">
+        <v>-5.88</v>
       </c>
       <c r="J30" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +67% / 중요공시 2건 / 중요공시 3일 +100%</t>
+          <t>중요공시 2건 / 중요공시 3일 +100% / 중요공시 7일 +100%</t>
         </is>
       </c>
       <c r="K30" s="23" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="20" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B31" s="20" t="n">
@@ -1649,14 +1647,14 @@
       </c>
       <c r="C31" s="21" t="inlineStr">
         <is>
-          <t>두산에너빌리티</t>
+          <t>전기차</t>
         </is>
       </c>
       <c r="D31" s="20" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E31" s="20" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F31" s="20" t="n">
         <v>0</v>
@@ -1664,27 +1662,25 @@
       <c r="G31" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H31" s="24" t="n">
-        <v>-1.09</v>
-      </c>
-      <c r="I31" s="22" t="n">
-        <v>0.37</v>
+      <c r="H31" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I31" s="20" t="n">
+        <v/>
       </c>
       <c r="J31" s="23" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 네이버뉴스 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K31" s="23" t="inlineStr">
-        <is>
-          <t>네이버, 공시</t>
-        </is>
+          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K31" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="20" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B32" s="20" t="n">
@@ -1692,14 +1688,14 @@
       </c>
       <c r="C32" s="21" t="inlineStr">
         <is>
-          <t>퀀텀레일</t>
+          <t>머큐리</t>
         </is>
       </c>
       <c r="D32" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E32" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F32" s="20" t="n">
         <v>0</v>
@@ -1707,27 +1703,27 @@
       <c r="G32" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H32" s="24" t="n">
-        <v>-1.63</v>
-      </c>
-      <c r="I32" s="24" t="n">
-        <v>-51.68</v>
+      <c r="H32" s="22" t="n">
+        <v>29.8</v>
+      </c>
+      <c r="I32" s="22" t="n">
+        <v>28.21</v>
       </c>
       <c r="J32" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +1711% / 중요공시 1건</t>
+          <t>네이버 검색 당일 +99% / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K32" s="23" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="20" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B33" s="20" t="n">
@@ -1735,42 +1731,42 @@
       </c>
       <c r="C33" s="21" t="inlineStr">
         <is>
-          <t>나인테크</t>
+          <t>팬오션</t>
         </is>
       </c>
       <c r="D33" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E33" s="20" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F33" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G33" s="20" t="n">
         <v>0</v>
       </c>
       <c r="H33" s="22" t="n">
-        <v>0.71</v>
+        <v>6.47</v>
       </c>
       <c r="I33" s="22" t="n">
-        <v>28.05</v>
+        <v>9.84</v>
       </c>
       <c r="J33" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +437% / 중요공시 1건</t>
+          <t>네이버 검색 당일 +76% / 중요공시 2건 / 중요공시 3일 +100%</t>
         </is>
       </c>
       <c r="K33" s="23" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="20" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B34" s="20" t="n">
@@ -1778,42 +1774,42 @@
       </c>
       <c r="C34" s="21" t="inlineStr">
         <is>
-          <t>한국파마</t>
+          <t>더코디</t>
         </is>
       </c>
       <c r="D34" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E34" s="20" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F34" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G34" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H34" s="22" t="n">
-        <v>13.42</v>
-      </c>
-      <c r="I34" s="22" t="n">
-        <v>19.06</v>
+      <c r="H34" s="24" t="n">
+        <v>-1.27</v>
+      </c>
+      <c r="I34" s="24" t="n">
+        <v>-20.87</v>
       </c>
       <c r="J34" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +202% / 중요공시 1건</t>
+          <t>중요공시 6건 / 중요공시 3일 +100%</t>
         </is>
       </c>
       <c r="K34" s="23" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="20" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B35" s="20" t="n">
@@ -1821,14 +1817,14 @@
       </c>
       <c r="C35" s="21" t="inlineStr">
         <is>
-          <t>한화솔루션</t>
+          <t>GS</t>
         </is>
       </c>
       <c r="D35" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E35" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F35" s="20" t="n">
         <v>0</v>
@@ -1837,26 +1833,26 @@
         <v>0</v>
       </c>
       <c r="H35" s="22" t="n">
-        <v>5.71</v>
-      </c>
-      <c r="I35" s="22" t="n">
-        <v>5.4</v>
+        <v>2.94</v>
+      </c>
+      <c r="I35" s="24" t="n">
+        <v>-8.050000000000001</v>
       </c>
       <c r="J35" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +156% / 중요공시 1건</t>
+          <t>Google 급상승 검색어 등장 (US)</t>
         </is>
       </c>
       <c r="K35" s="23" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>Google</t>
         </is>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="20" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B36" s="20" t="n">
@@ -1864,7 +1860,7 @@
       </c>
       <c r="C36" s="21" t="inlineStr">
         <is>
-          <t>고영</t>
+          <t>퀀텀레일</t>
         </is>
       </c>
       <c r="D36" s="20" t="n">
@@ -1879,27 +1875,27 @@
       <c r="G36" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H36" s="22" t="n">
-        <v>1.47</v>
-      </c>
-      <c r="I36" s="22" t="n">
-        <v>19.41</v>
+      <c r="H36" s="24" t="n">
+        <v>-1.63</v>
+      </c>
+      <c r="I36" s="24" t="n">
+        <v>-51.68</v>
       </c>
       <c r="J36" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +111% / 중요공시 2건</t>
+          <t>네이버 검색 당일 +1785% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K36" s="23" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="20" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B37" s="20" t="n">
@@ -1907,7 +1903,7 @@
       </c>
       <c r="C37" s="21" t="inlineStr">
         <is>
-          <t>삼성중공업</t>
+          <t>나인테크</t>
         </is>
       </c>
       <c r="D37" s="20" t="n">
@@ -1923,26 +1919,26 @@
         <v>0</v>
       </c>
       <c r="H37" s="22" t="n">
-        <v>0.91</v>
-      </c>
-      <c r="I37" s="24" t="n">
-        <v>-1.14</v>
+        <v>0.71</v>
+      </c>
+      <c r="I37" s="22" t="n">
+        <v>28.05</v>
       </c>
       <c r="J37" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +53% / 중요공시 2건 / 매일경제 기사 언급</t>
+          <t>네이버 검색 당일 +451% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K37" s="23" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="20" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B38" s="20" t="n">
@@ -1950,7 +1946,7 @@
       </c>
       <c r="C38" s="21" t="inlineStr">
         <is>
-          <t>성호전자</t>
+          <t>한국파마</t>
         </is>
       </c>
       <c r="D38" s="20" t="n">
@@ -1966,26 +1962,26 @@
         <v>0</v>
       </c>
       <c r="H38" s="22" t="n">
-        <v>11.35</v>
+        <v>13.42</v>
       </c>
       <c r="I38" s="22" t="n">
-        <v>27.13</v>
+        <v>19.06</v>
       </c>
       <c r="J38" s="23" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급</t>
+          <t>네이버 검색 당일 +229% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K38" s="23" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="20" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B39" s="20" t="n">
@@ -1993,7 +1989,7 @@
       </c>
       <c r="C39" s="21" t="inlineStr">
         <is>
-          <t>빛샘전자</t>
+          <t>한창</t>
         </is>
       </c>
       <c r="D39" s="20" t="n">
@@ -2008,27 +2004,27 @@
       <c r="G39" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H39" s="22" t="n">
-        <v>11.65</v>
-      </c>
-      <c r="I39" s="22" t="n">
-        <v>26.1</v>
+      <c r="H39" s="24" t="n">
+        <v>-91.06999999999999</v>
+      </c>
+      <c r="I39" s="24" t="n">
+        <v>-91.06999999999999</v>
       </c>
       <c r="J39" s="23" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급</t>
+          <t>네이버 검색 당일 +197% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K39" s="23" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="20" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B40" s="20" t="n">
@@ -2036,7 +2032,7 @@
       </c>
       <c r="C40" s="21" t="inlineStr">
         <is>
-          <t>우리기술</t>
+          <t>한화솔루션</t>
         </is>
       </c>
       <c r="D40" s="20" t="n">
@@ -2052,26 +2048,26 @@
         <v>0</v>
       </c>
       <c r="H40" s="22" t="n">
-        <v>1.75</v>
+        <v>5.71</v>
       </c>
       <c r="I40" s="22" t="n">
-        <v>1.19</v>
+        <v>5.4</v>
       </c>
       <c r="J40" s="23" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 네이버뉴스 헤드라인 언급</t>
+          <t>네이버 검색 당일 +163% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K40" s="23" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="20" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B41" s="20" t="n">
@@ -2079,42 +2075,42 @@
       </c>
       <c r="C41" s="21" t="inlineStr">
         <is>
-          <t>에이에프더블류</t>
+          <t>고영</t>
         </is>
       </c>
       <c r="D41" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E41" s="20" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F41" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G41" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="H41" s="24" t="n">
-        <v>-5.13</v>
-      </c>
-      <c r="I41" s="24" t="n">
-        <v>-51.32</v>
+        <v>0</v>
+      </c>
+      <c r="H41" s="22" t="n">
+        <v>1.47</v>
+      </c>
+      <c r="I41" s="22" t="n">
+        <v>19.41</v>
       </c>
       <c r="J41" s="23" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 7일 +100%</t>
+          <t>네이버 검색 당일 +121% / 중요공시 2건</t>
         </is>
       </c>
       <c r="K41" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="20" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B42" s="20" t="n">
@@ -2122,7 +2118,7 @@
       </c>
       <c r="C42" s="21" t="inlineStr">
         <is>
-          <t>아리바이오홀딩스</t>
+          <t>에이에프더블류</t>
         </is>
       </c>
       <c r="D42" s="20" t="n">
@@ -2138,10 +2134,10 @@
         <v>3</v>
       </c>
       <c r="H42" s="24" t="n">
-        <v>-2.23</v>
+        <v>-5.13</v>
       </c>
       <c r="I42" s="24" t="n">
-        <v>-22.96</v>
+        <v>-51.32</v>
       </c>
       <c r="J42" s="23" t="inlineStr">
         <is>
@@ -2157,7 +2153,7 @@
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="20" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B43" s="20" t="n">
@@ -2165,7 +2161,7 @@
       </c>
       <c r="C43" s="21" t="inlineStr">
         <is>
-          <t>선도전기</t>
+          <t>아리바이오홀딩스</t>
         </is>
       </c>
       <c r="D43" s="20" t="n">
@@ -2181,10 +2177,10 @@
         <v>3</v>
       </c>
       <c r="H43" s="24" t="n">
-        <v>-1.82</v>
+        <v>-2.23</v>
       </c>
       <c r="I43" s="24" t="n">
-        <v>-1.82</v>
+        <v>-22.96</v>
       </c>
       <c r="J43" s="23" t="inlineStr">
         <is>
@@ -2200,7 +2196,7 @@
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="20" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B44" s="20" t="n">
@@ -2208,7 +2204,7 @@
       </c>
       <c r="C44" s="21" t="inlineStr">
         <is>
-          <t>루닛</t>
+          <t>선도전기</t>
         </is>
       </c>
       <c r="D44" s="20" t="n">
@@ -2224,10 +2220,10 @@
         <v>3</v>
       </c>
       <c r="H44" s="24" t="n">
-        <v>-5.03</v>
+        <v>-1.82</v>
       </c>
       <c r="I44" s="24" t="n">
-        <v>-5.88</v>
+        <v>-1.82</v>
       </c>
       <c r="J44" s="23" t="inlineStr">
         <is>
@@ -2243,7 +2239,7 @@
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="20" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B45" s="20" t="n">
@@ -2286,7 +2282,7 @@
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="20" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B46" s="20" t="n">
@@ -2294,7 +2290,7 @@
       </c>
       <c r="C46" s="21" t="inlineStr">
         <is>
-          <t>광진실업</t>
+          <t>미래산업</t>
         </is>
       </c>
       <c r="D46" s="20" t="n">
@@ -2310,10 +2306,10 @@
         <v>3</v>
       </c>
       <c r="H46" s="22" t="n">
-        <v>0.49</v>
-      </c>
-      <c r="I46" s="24" t="n">
-        <v>-18.6</v>
+        <v>0.6</v>
+      </c>
+      <c r="I46" s="22" t="n">
+        <v>16.62</v>
       </c>
       <c r="J46" s="23" t="inlineStr">
         <is>
@@ -2329,7 +2325,7 @@
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="20" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B47" s="20" t="n">
@@ -2337,251 +2333,255 @@
       </c>
       <c r="C47" s="21" t="inlineStr">
         <is>
-          <t>미래산업</t>
+          <t>게임</t>
         </is>
       </c>
       <c r="D47" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E47" s="20" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F47" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G47" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="H47" s="22" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="I47" s="22" t="n">
-        <v>16.62</v>
+        <v>0</v>
+      </c>
+      <c r="H47" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I47" s="20" t="n">
+        <v/>
       </c>
       <c r="J47" s="23" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 7일 +100%</t>
-        </is>
-      </c>
-      <c r="K47" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K47" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
-      <c r="A48" s="20" t="inlineStr">
-        <is>
-          <t>2026-10-04</t>
-        </is>
-      </c>
-      <c r="B48" s="20" t="n">
+      <c r="A48" s="25" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B48" s="25" t="n">
         <v>35</v>
       </c>
-      <c r="C48" s="21" t="inlineStr">
-        <is>
-          <t>SK이노베이션</t>
-        </is>
-      </c>
-      <c r="D48" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E48" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F48" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G48" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H48" s="22" t="n">
-        <v>7.23</v>
-      </c>
-      <c r="I48" s="24" t="n">
-        <v>-4.78</v>
-      </c>
-      <c r="J48" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 1건 / 네이버뉴스 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K48" s="23" t="inlineStr">
-        <is>
-          <t>네이버, 공시</t>
+      <c r="C48" s="26" t="inlineStr">
+        <is>
+          <t>브릴스</t>
+        </is>
+      </c>
+      <c r="D48" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E48" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F48" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G48" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H48" s="27" t="n">
+        <v>9.81</v>
+      </c>
+      <c r="I48" s="27" t="n">
+        <v>9.81</v>
+      </c>
+      <c r="J48" s="28" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +2323%</t>
+        </is>
+      </c>
+      <c r="K48" s="28" t="inlineStr">
+        <is>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
-      <c r="A49" s="20" t="inlineStr">
-        <is>
-          <t>2026-10-04</t>
-        </is>
-      </c>
-      <c r="B49" s="20" t="n">
+      <c r="A49" s="25" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B49" s="25" t="n">
         <v>36</v>
       </c>
-      <c r="C49" s="21" t="inlineStr">
-        <is>
-          <t>에스제이그룹</t>
-        </is>
-      </c>
-      <c r="D49" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E49" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F49" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G49" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H49" s="22" t="n">
-        <v>29.96</v>
-      </c>
-      <c r="I49" s="22" t="n">
-        <v>30.39</v>
-      </c>
-      <c r="J49" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 1건 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K49" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
+      <c r="C49" s="26" t="inlineStr">
+        <is>
+          <t>현대바이오랜드</t>
+        </is>
+      </c>
+      <c r="D49" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E49" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F49" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G49" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H49" s="29" t="n">
+        <v>-3.29</v>
+      </c>
+      <c r="I49" s="27" t="n">
+        <v>10.25</v>
+      </c>
+      <c r="J49" s="28" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +1636%</t>
+        </is>
+      </c>
+      <c r="K49" s="28" t="inlineStr">
+        <is>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
-      <c r="A50" s="20" t="inlineStr">
-        <is>
-          <t>2026-10-04</t>
-        </is>
-      </c>
-      <c r="B50" s="20" t="n">
+      <c r="A50" s="25" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B50" s="25" t="n">
         <v>37</v>
       </c>
-      <c r="C50" s="21" t="inlineStr">
-        <is>
-          <t>전기차</t>
-        </is>
-      </c>
-      <c r="D50" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E50" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F50" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G50" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H50" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I50" s="20" t="n">
-        <v/>
-      </c>
-      <c r="J50" s="23" t="inlineStr">
-        <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K50" s="23" t="n">
-        <v/>
+      <c r="C50" s="26" t="inlineStr">
+        <is>
+          <t>코스모로보틱스</t>
+        </is>
+      </c>
+      <c r="D50" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E50" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F50" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G50" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H50" s="29" t="n">
+        <v>-8.460000000000001</v>
+      </c>
+      <c r="I50" s="29" t="n">
+        <v>-30.64</v>
+      </c>
+      <c r="J50" s="28" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +1408%</t>
+        </is>
+      </c>
+      <c r="K50" s="28" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
-      <c r="A51" s="20" t="inlineStr">
-        <is>
-          <t>2026-10-04</t>
-        </is>
-      </c>
-      <c r="B51" s="20" t="n">
+      <c r="A51" s="25" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B51" s="25" t="n">
         <v>38</v>
       </c>
-      <c r="C51" s="21" t="inlineStr">
-        <is>
-          <t>스테이블코인</t>
-        </is>
-      </c>
-      <c r="D51" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E51" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F51" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G51" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H51" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I51" s="20" t="n">
-        <v/>
-      </c>
-      <c r="J51" s="23" t="inlineStr">
-        <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K51" s="23" t="n">
-        <v/>
+      <c r="C51" s="26" t="inlineStr">
+        <is>
+          <t>글로벌테크놀로지</t>
+        </is>
+      </c>
+      <c r="D51" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E51" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F51" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G51" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H51" s="29" t="n">
+        <v>-8.550000000000001</v>
+      </c>
+      <c r="I51" s="27" t="n">
+        <v>2.48</v>
+      </c>
+      <c r="J51" s="28" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +1378%</t>
+        </is>
+      </c>
+      <c r="K51" s="28" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
-      <c r="A52" s="20" t="inlineStr">
-        <is>
-          <t>2026-10-04</t>
-        </is>
-      </c>
-      <c r="B52" s="20" t="n">
+      <c r="A52" s="25" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B52" s="25" t="n">
         <v>39</v>
       </c>
-      <c r="C52" s="21" t="inlineStr">
-        <is>
-          <t>현대건설</t>
-        </is>
-      </c>
-      <c r="D52" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E52" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F52" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G52" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H52" s="24" t="n">
-        <v>-2.22</v>
-      </c>
-      <c r="I52" s="24" t="n">
-        <v>-6.9</v>
-      </c>
-      <c r="J52" s="23" t="inlineStr">
-        <is>
-          <t>한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K52" s="23" t="n">
-        <v/>
+      <c r="C52" s="26" t="inlineStr">
+        <is>
+          <t>덕산넵코어스</t>
+        </is>
+      </c>
+      <c r="D52" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E52" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F52" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G52" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H52" s="29" t="n">
+        <v>-1.75</v>
+      </c>
+      <c r="I52" s="29" t="n">
+        <v>-3.09</v>
+      </c>
+      <c r="J52" s="28" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +1323%</t>
+        </is>
+      </c>
+      <c r="K52" s="28" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="53" ht="18" customHeight="1">
       <c r="A53" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B53" s="25" t="n">
@@ -2589,7 +2589,7 @@
       </c>
       <c r="C53" s="26" t="inlineStr">
         <is>
-          <t>브릴스</t>
+          <t>빅웨이브로보틱스</t>
         </is>
       </c>
       <c r="D53" s="25" t="n">
@@ -2605,14 +2605,14 @@
         <v>0</v>
       </c>
       <c r="H53" s="27" t="n">
-        <v>9.81</v>
+        <v>2.75</v>
       </c>
       <c r="I53" s="27" t="n">
-        <v>9.81</v>
+        <v>17.38</v>
       </c>
       <c r="J53" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +2242%</t>
+          <t>네이버 검색 당일 +1263%</t>
         </is>
       </c>
       <c r="K53" s="28" t="inlineStr">
@@ -2624,7 +2624,7 @@
     <row r="54" ht="18" customHeight="1">
       <c r="A54" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B54" s="25" t="n">
@@ -2632,7 +2632,7 @@
       </c>
       <c r="C54" s="26" t="inlineStr">
         <is>
-          <t>현대바이오랜드</t>
+          <t>덕우전자</t>
         </is>
       </c>
       <c r="D54" s="25" t="n">
@@ -2647,15 +2647,15 @@
       <c r="G54" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H54" s="29" t="n">
-        <v>-3.29</v>
+      <c r="H54" s="27" t="n">
+        <v>17.91</v>
       </c>
       <c r="I54" s="27" t="n">
-        <v>10.25</v>
+        <v>53.62</v>
       </c>
       <c r="J54" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +1609%</t>
+          <t>네이버 검색 당일 +1066%</t>
         </is>
       </c>
       <c r="K54" s="28" t="inlineStr">
@@ -2667,7 +2667,7 @@
     <row r="55" ht="18" customHeight="1">
       <c r="A55" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B55" s="25" t="n">
@@ -2675,7 +2675,7 @@
       </c>
       <c r="C55" s="26" t="inlineStr">
         <is>
-          <t>코스모로보틱스</t>
+          <t>부산주공</t>
         </is>
       </c>
       <c r="D55" s="25" t="n">
@@ -2691,14 +2691,14 @@
         <v>0</v>
       </c>
       <c r="H55" s="29" t="n">
-        <v>-8.460000000000001</v>
+        <v>-32.5</v>
       </c>
       <c r="I55" s="29" t="n">
-        <v>-30.64</v>
+        <v>-94.44</v>
       </c>
       <c r="J55" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +1375%</t>
+          <t>네이버 검색 당일 +769%</t>
         </is>
       </c>
       <c r="K55" s="28" t="inlineStr">
@@ -2710,7 +2710,7 @@
     <row r="56" ht="18" customHeight="1">
       <c r="A56" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B56" s="25" t="n">
@@ -2718,7 +2718,7 @@
       </c>
       <c r="C56" s="26" t="inlineStr">
         <is>
-          <t>글로벌테크놀로지</t>
+          <t>원일티엔아이</t>
         </is>
       </c>
       <c r="D56" s="25" t="n">
@@ -2733,15 +2733,15 @@
       <c r="G56" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H56" s="29" t="n">
-        <v>-8.550000000000001</v>
+      <c r="H56" s="27" t="n">
+        <v>18.34</v>
       </c>
       <c r="I56" s="27" t="n">
-        <v>2.48</v>
+        <v>54.33</v>
       </c>
       <c r="J56" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +1355%</t>
+          <t>네이버 검색 당일 +645%</t>
         </is>
       </c>
       <c r="K56" s="28" t="inlineStr">
@@ -2753,7 +2753,7 @@
     <row r="57" ht="18" customHeight="1">
       <c r="A57" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B57" s="25" t="n">
@@ -2761,7 +2761,7 @@
       </c>
       <c r="C57" s="26" t="inlineStr">
         <is>
-          <t>덕산넵코어스</t>
+          <t>KBI동양철관</t>
         </is>
       </c>
       <c r="D57" s="25" t="n">
@@ -2777,14 +2777,14 @@
         <v>0</v>
       </c>
       <c r="H57" s="29" t="n">
-        <v>-1.75</v>
-      </c>
-      <c r="I57" s="29" t="n">
-        <v>-3.09</v>
+        <v>-4.36</v>
+      </c>
+      <c r="I57" s="27" t="n">
+        <v>16.03</v>
       </c>
       <c r="J57" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +1294%</t>
+          <t>네이버 검색 당일 +547%</t>
         </is>
       </c>
       <c r="K57" s="28" t="inlineStr">
@@ -2796,7 +2796,7 @@
     <row r="58" ht="18" customHeight="1">
       <c r="A58" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B58" s="25" t="n">
@@ -2804,7 +2804,7 @@
       </c>
       <c r="C58" s="26" t="inlineStr">
         <is>
-          <t>빅웨이브로보틱스</t>
+          <t>윈팩</t>
         </is>
       </c>
       <c r="D58" s="25" t="n">
@@ -2820,14 +2820,14 @@
         <v>0</v>
       </c>
       <c r="H58" s="27" t="n">
-        <v>2.75</v>
+        <v>4.95</v>
       </c>
       <c r="I58" s="27" t="n">
-        <v>17.38</v>
+        <v>72.38</v>
       </c>
       <c r="J58" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +1242%</t>
+          <t>네이버 검색 당일 +472%</t>
         </is>
       </c>
       <c r="K58" s="28" t="inlineStr">
@@ -2839,7 +2839,7 @@
     <row r="59" ht="18" customHeight="1">
       <c r="A59" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B59" s="25" t="n">
@@ -2847,7 +2847,7 @@
       </c>
       <c r="C59" s="26" t="inlineStr">
         <is>
-          <t>덕우전자</t>
+          <t>피제이전자</t>
         </is>
       </c>
       <c r="D59" s="25" t="n">
@@ -2863,14 +2863,14 @@
         <v>0</v>
       </c>
       <c r="H59" s="27" t="n">
-        <v>17.91</v>
+        <v>30.5</v>
       </c>
       <c r="I59" s="27" t="n">
-        <v>53.62</v>
+        <v>29.32</v>
       </c>
       <c r="J59" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +975%</t>
+          <t>네이버 검색 당일 +444%</t>
         </is>
       </c>
       <c r="K59" s="28" t="inlineStr">
@@ -2882,7 +2882,7 @@
     <row r="60" ht="18" customHeight="1">
       <c r="A60" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B60" s="25" t="n">
@@ -2890,7 +2890,7 @@
       </c>
       <c r="C60" s="26" t="inlineStr">
         <is>
-          <t>부산주공</t>
+          <t>LK삼양</t>
         </is>
       </c>
       <c r="D60" s="25" t="n">
@@ -2905,15 +2905,15 @@
       <c r="G60" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H60" s="29" t="n">
-        <v>-32.5</v>
-      </c>
-      <c r="I60" s="29" t="n">
-        <v>-94.44</v>
+      <c r="H60" s="27" t="n">
+        <v>18.37</v>
+      </c>
+      <c r="I60" s="27" t="n">
+        <v>18.08</v>
       </c>
       <c r="J60" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +721%</t>
+          <t>네이버 검색 당일 +406%</t>
         </is>
       </c>
       <c r="K60" s="28" t="inlineStr">
@@ -2925,7 +2925,7 @@
     <row r="61" ht="18" customHeight="1">
       <c r="A61" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B61" s="25" t="n">
@@ -2933,7 +2933,7 @@
       </c>
       <c r="C61" s="26" t="inlineStr">
         <is>
-          <t>원일티엔아이</t>
+          <t>한국비엔씨</t>
         </is>
       </c>
       <c r="D61" s="25" t="n">
@@ -2948,15 +2948,15 @@
       <c r="G61" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H61" s="27" t="n">
-        <v>18.34</v>
-      </c>
-      <c r="I61" s="27" t="n">
-        <v>54.33</v>
+      <c r="H61" s="29" t="n">
+        <v>-3.07</v>
+      </c>
+      <c r="I61" s="29" t="n">
+        <v>-7.74</v>
       </c>
       <c r="J61" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +596%</t>
+          <t>네이버 검색 당일 +339%</t>
         </is>
       </c>
       <c r="K61" s="28" t="inlineStr">
@@ -2968,7 +2968,7 @@
     <row r="62" ht="18" customHeight="1">
       <c r="A62" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B62" s="25" t="n">
@@ -2976,7 +2976,7 @@
       </c>
       <c r="C62" s="26" t="inlineStr">
         <is>
-          <t>KBI동양철관</t>
+          <t>에이프릴바이오</t>
         </is>
       </c>
       <c r="D62" s="25" t="n">
@@ -2992,14 +2992,14 @@
         <v>0</v>
       </c>
       <c r="H62" s="29" t="n">
-        <v>-4.36</v>
-      </c>
-      <c r="I62" s="27" t="n">
-        <v>16.03</v>
+        <v>-21.12</v>
+      </c>
+      <c r="I62" s="29" t="n">
+        <v>-9.390000000000001</v>
       </c>
       <c r="J62" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +515%</t>
+          <t>네이버 검색 당일 +283%</t>
         </is>
       </c>
       <c r="K62" s="28" t="inlineStr">
@@ -3011,7 +3011,7 @@
     <row r="63" ht="18" customHeight="1">
       <c r="A63" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B63" s="25" t="n">
@@ -3019,7 +3019,7 @@
       </c>
       <c r="C63" s="26" t="inlineStr">
         <is>
-          <t>윈팩</t>
+          <t>세미티에스</t>
         </is>
       </c>
       <c r="D63" s="25" t="n">
@@ -3035,14 +3035,14 @@
         <v>0</v>
       </c>
       <c r="H63" s="27" t="n">
-        <v>4.95</v>
+        <v>2.06</v>
       </c>
       <c r="I63" s="27" t="n">
-        <v>72.38</v>
+        <v>27.22</v>
       </c>
       <c r="J63" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +448%</t>
+          <t>네이버 검색 당일 +222%</t>
         </is>
       </c>
       <c r="K63" s="28" t="inlineStr">
@@ -3144,22 +3144,22 @@
         <v>1</v>
       </c>
       <c r="C3" s="25" t="n">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="D3" s="25" t="n">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="E3" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F3" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G3" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="H3" s="25" t="n"/>
@@ -3175,22 +3175,22 @@
         <v>1</v>
       </c>
       <c r="C4" s="25" t="n">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="D4" s="25" t="n">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="E4" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F4" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G4" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="H4" s="27" t="n">
@@ -3220,12 +3220,12 @@
       </c>
       <c r="F5" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G5" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="H5" s="25" t="n"/>
@@ -3241,22 +3241,22 @@
         <v>1</v>
       </c>
       <c r="C6" s="25" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="D6" s="25" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="E6" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F6" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G6" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="H6" s="29" t="n">
@@ -3269,29 +3269,29 @@
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="26" t="inlineStr">
         <is>
-          <t>바이오</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="B7" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="25" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D7" s="25" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E7" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F7" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G7" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="H7" s="25" t="n"/>
@@ -3300,29 +3300,29 @@
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="26" t="inlineStr">
         <is>
-          <t>원전</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="B8" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="25" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D8" s="25" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E8" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F8" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G8" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="H8" s="25" t="n"/>
@@ -3331,29 +3331,29 @@
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="26" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>바이오</t>
         </is>
       </c>
       <c r="B9" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="25" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D9" s="25" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E9" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F9" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G9" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="H9" s="25" t="n"/>
@@ -3362,7 +3362,7 @@
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="26" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>SK하이닉스</t>
         </is>
       </c>
       <c r="B10" s="25" t="n">
@@ -3379,21 +3379,25 @@
       </c>
       <c r="F10" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G10" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
-        </is>
-      </c>
-      <c r="H10" s="25" t="n"/>
-      <c r="I10" s="25" t="n"/>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="H10" s="27" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="I10" s="27" t="n">
+        <v>4.6</v>
+      </c>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="26" t="inlineStr">
         <is>
-          <t>SK하이닉스</t>
+          <t>삼성E&amp;A</t>
         </is>
       </c>
       <c r="B11" s="25" t="n">
@@ -3410,25 +3414,25 @@
       </c>
       <c r="F11" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G11" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="H11" s="27" t="n">
-        <v>0.77</v>
-      </c>
-      <c r="I11" s="27" t="n">
-        <v>4.6</v>
+        <v>0.84</v>
+      </c>
+      <c r="I11" s="29" t="n">
+        <v>-4.11</v>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="26" t="inlineStr">
         <is>
-          <t>삼성E&amp;A</t>
+          <t>스테이블코인</t>
         </is>
       </c>
       <c r="B12" s="25" t="n">
@@ -3445,25 +3449,21 @@
       </c>
       <c r="F12" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G12" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
-        </is>
-      </c>
-      <c r="H12" s="27" t="n">
-        <v>0.84</v>
-      </c>
-      <c r="I12" s="29" t="n">
-        <v>-4.11</v>
-      </c>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="H12" s="25" t="n"/>
+      <c r="I12" s="25" t="n"/>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>철강</t>
+          <t>원전</t>
         </is>
       </c>
       <c r="B13" s="25" t="n">
@@ -3480,12 +3480,12 @@
       </c>
       <c r="F13" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G13" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="H13" s="25" t="n"/>
@@ -3494,42 +3494,42 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>한창</t>
+          <t>SG</t>
         </is>
       </c>
       <c r="B14" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C14" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D14" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E14" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F14" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G14" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="H14" s="29" t="n">
-        <v>-91.06999999999999</v>
+        <v>-5.15</v>
       </c>
       <c r="I14" s="29" t="n">
-        <v>-91.06999999999999</v>
+        <v>-2.64</v>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>SG</t>
+          <t>대한항공</t>
         </is>
       </c>
       <c r="B15" s="25" t="n">
@@ -3546,25 +3546,25 @@
       </c>
       <c r="F15" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G15" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="H15" s="29" t="n">
-        <v>-5.15</v>
+        <v>-0.64</v>
       </c>
       <c r="I15" s="29" t="n">
-        <v>-2.64</v>
+        <v>-1.91</v>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>모아데이타</t>
+          <t>루닛</t>
         </is>
       </c>
       <c r="B16" s="25" t="n">
@@ -3581,25 +3581,25 @@
       </c>
       <c r="F16" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G16" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="H16" s="29" t="n">
-        <v>-3.6</v>
+        <v>-5.03</v>
       </c>
       <c r="I16" s="29" t="n">
-        <v>-1.83</v>
+        <v>-5.88</v>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>세미파이브</t>
+          <t>모아데이타</t>
         </is>
       </c>
       <c r="B17" s="25" t="n">
@@ -3616,270 +3616,266 @@
       </c>
       <c r="F17" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G17" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
-        </is>
-      </c>
-      <c r="H17" s="27" t="n">
-        <v>1.72</v>
-      </c>
-      <c r="I17" s="27" t="n">
-        <v>28.88</v>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="H17" s="29" t="n">
+        <v>-3.6</v>
+      </c>
+      <c r="I17" s="29" t="n">
+        <v>-1.83</v>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="26" t="inlineStr">
         <is>
-          <t>두산에너빌리티</t>
+          <t>삼성중공업</t>
         </is>
       </c>
       <c r="B18" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C18" s="25" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D18" s="25" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E18" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F18" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G18" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
-        </is>
-      </c>
-      <c r="H18" s="29" t="n">
-        <v>-1.09</v>
-      </c>
-      <c r="I18" s="27" t="n">
-        <v>0.37</v>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="H18" s="27" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="I18" s="29" t="n">
+        <v>-1.14</v>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>머큐리</t>
+          <t>세미파이브</t>
         </is>
       </c>
       <c r="B19" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C19" s="25" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D19" s="25" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E19" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F19" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G19" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="H19" s="27" t="n">
-        <v>29.8</v>
+        <v>1.72</v>
       </c>
       <c r="I19" s="27" t="n">
-        <v>28.21</v>
+        <v>28.88</v>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="26" t="inlineStr">
         <is>
-          <t>팬오션</t>
+          <t>전기차</t>
         </is>
       </c>
       <c r="B20" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C20" s="25" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D20" s="25" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E20" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F20" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G20" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
-        </is>
-      </c>
-      <c r="H20" s="27" t="n">
-        <v>6.47</v>
-      </c>
-      <c r="I20" s="27" t="n">
-        <v>9.84</v>
-      </c>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="H20" s="25" t="n"/>
+      <c r="I20" s="25" t="n"/>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="26" t="inlineStr">
         <is>
-          <t>SK이노베이션</t>
+          <t>GS</t>
         </is>
       </c>
       <c r="B21" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C21" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D21" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E21" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F21" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G21" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="H21" s="27" t="n">
-        <v>7.23</v>
+        <v>2.94</v>
       </c>
       <c r="I21" s="29" t="n">
-        <v>-4.78</v>
+        <v>-8.050000000000001</v>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="26" t="inlineStr">
         <is>
-          <t>고영</t>
+          <t>더코디</t>
         </is>
       </c>
       <c r="B22" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C22" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D22" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E22" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F22" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G22" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
-        </is>
-      </c>
-      <c r="H22" s="27" t="n">
-        <v>1.47</v>
-      </c>
-      <c r="I22" s="27" t="n">
-        <v>19.41</v>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="H22" s="29" t="n">
+        <v>-1.27</v>
+      </c>
+      <c r="I22" s="29" t="n">
+        <v>-20.87</v>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="26" t="inlineStr">
         <is>
-          <t>광진실업</t>
+          <t>머큐리</t>
         </is>
       </c>
       <c r="B23" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C23" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D23" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E23" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F23" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G23" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="H23" s="27" t="n">
-        <v>0.49</v>
-      </c>
-      <c r="I23" s="29" t="n">
-        <v>-18.6</v>
+        <v>29.8</v>
+      </c>
+      <c r="I23" s="27" t="n">
+        <v>28.21</v>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="26" t="inlineStr">
         <is>
-          <t>나인테크</t>
+          <t>팬오션</t>
         </is>
       </c>
       <c r="B24" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C24" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D24" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E24" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F24" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G24" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="H24" s="27" t="n">
-        <v>0.71</v>
+        <v>6.47</v>
       </c>
       <c r="I24" s="27" t="n">
-        <v>28.05</v>
+        <v>9.84</v>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="26" t="inlineStr">
         <is>
-          <t>루닛</t>
+          <t>게임</t>
         </is>
       </c>
       <c r="B25" s="25" t="n">
@@ -3896,25 +3892,21 @@
       </c>
       <c r="F25" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G25" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
-        </is>
-      </c>
-      <c r="H25" s="29" t="n">
-        <v>-5.03</v>
-      </c>
-      <c r="I25" s="29" t="n">
-        <v>-5.88</v>
-      </c>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="H25" s="25" t="n"/>
+      <c r="I25" s="25" t="n"/>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="26" t="inlineStr">
         <is>
-          <t>미래산업</t>
+          <t>고영</t>
         </is>
       </c>
       <c r="B26" s="25" t="n">
@@ -3931,25 +3923,25 @@
       </c>
       <c r="F26" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G26" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="H26" s="27" t="n">
-        <v>0.6</v>
+        <v>1.47</v>
       </c>
       <c r="I26" s="27" t="n">
-        <v>16.62</v>
+        <v>19.41</v>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="26" t="inlineStr">
         <is>
-          <t>빛샘전자</t>
+          <t>나인테크</t>
         </is>
       </c>
       <c r="B27" s="25" t="n">
@@ -3966,25 +3958,25 @@
       </c>
       <c r="F27" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G27" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="H27" s="27" t="n">
-        <v>11.65</v>
+        <v>0.71</v>
       </c>
       <c r="I27" s="27" t="n">
-        <v>26.1</v>
+        <v>28.05</v>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="26" t="inlineStr">
         <is>
-          <t>삼성중공업</t>
+          <t>미래산업</t>
         </is>
       </c>
       <c r="B28" s="25" t="n">
@@ -4001,19 +3993,19 @@
       </c>
       <c r="F28" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G28" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="H28" s="27" t="n">
-        <v>0.91</v>
-      </c>
-      <c r="I28" s="29" t="n">
-        <v>-1.14</v>
+        <v>0.6</v>
+      </c>
+      <c r="I28" s="27" t="n">
+        <v>16.62</v>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
@@ -4036,12 +4028,12 @@
       </c>
       <c r="F29" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G29" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="H29" s="29" t="n">
@@ -4054,7 +4046,7 @@
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="26" t="inlineStr">
         <is>
-          <t>성호전자</t>
+          <t>아리바이오홀딩스</t>
         </is>
       </c>
       <c r="B30" s="25" t="n">
@@ -4071,25 +4063,25 @@
       </c>
       <c r="F30" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G30" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
-        </is>
-      </c>
-      <c r="H30" s="27" t="n">
-        <v>11.35</v>
-      </c>
-      <c r="I30" s="27" t="n">
-        <v>27.13</v>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="H30" s="29" t="n">
+        <v>-2.23</v>
+      </c>
+      <c r="I30" s="29" t="n">
+        <v>-22.96</v>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="26" t="inlineStr">
         <is>
-          <t>스테이블코인</t>
+          <t>에이에프더블류</t>
         </is>
       </c>
       <c r="B31" s="25" t="n">
@@ -4106,21 +4098,25 @@
       </c>
       <c r="F31" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G31" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
-        </is>
-      </c>
-      <c r="H31" s="25" t="n"/>
-      <c r="I31" s="25" t="n"/>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="H31" s="29" t="n">
+        <v>-5.13</v>
+      </c>
+      <c r="I31" s="29" t="n">
+        <v>-51.32</v>
+      </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="26" t="inlineStr">
         <is>
-          <t>아리바이오홀딩스</t>
+          <t>퀀텀레일</t>
         </is>
       </c>
       <c r="B32" s="25" t="n">
@@ -4137,25 +4133,25 @@
       </c>
       <c r="F32" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G32" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="H32" s="29" t="n">
-        <v>-2.23</v>
+        <v>-1.63</v>
       </c>
       <c r="I32" s="29" t="n">
-        <v>-22.96</v>
+        <v>-51.68</v>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="26" t="inlineStr">
         <is>
-          <t>에스제이그룹</t>
+          <t>한국파마</t>
         </is>
       </c>
       <c r="B33" s="25" t="n">
@@ -4172,25 +4168,25 @@
       </c>
       <c r="F33" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G33" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="H33" s="27" t="n">
-        <v>29.96</v>
+        <v>13.42</v>
       </c>
       <c r="I33" s="27" t="n">
-        <v>30.39</v>
+        <v>19.06</v>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="26" t="inlineStr">
         <is>
-          <t>에이에프더블류</t>
+          <t>한창</t>
         </is>
       </c>
       <c r="B34" s="25" t="n">
@@ -4207,25 +4203,25 @@
       </c>
       <c r="F34" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G34" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="H34" s="29" t="n">
-        <v>-5.13</v>
+        <v>-91.06999999999999</v>
       </c>
       <c r="I34" s="29" t="n">
-        <v>-51.32</v>
+        <v>-91.06999999999999</v>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="26" t="inlineStr">
         <is>
-          <t>우리기술</t>
+          <t>한화솔루션</t>
         </is>
       </c>
       <c r="B35" s="25" t="n">
@@ -4242,25 +4238,25 @@
       </c>
       <c r="F35" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G35" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="H35" s="27" t="n">
-        <v>1.75</v>
+        <v>5.71</v>
       </c>
       <c r="I35" s="27" t="n">
-        <v>1.19</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="26" t="inlineStr">
         <is>
-          <t>전기차</t>
+          <t>한화오션</t>
         </is>
       </c>
       <c r="B36" s="25" t="n">
@@ -4277,196 +4273,200 @@
       </c>
       <c r="F36" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G36" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
-        </is>
-      </c>
-      <c r="H36" s="25" t="n"/>
-      <c r="I36" s="25" t="n"/>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="H36" s="27" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="I36" s="29" t="n">
+        <v>-2.24</v>
+      </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="26" t="inlineStr">
         <is>
-          <t>퀀텀레일</t>
+          <t>KBI동양철관</t>
         </is>
       </c>
       <c r="B37" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C37" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D37" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E37" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F37" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G37" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="H37" s="29" t="n">
-        <v>-1.63</v>
-      </c>
-      <c r="I37" s="29" t="n">
-        <v>-51.68</v>
+        <v>-4.36</v>
+      </c>
+      <c r="I37" s="27" t="n">
+        <v>16.03</v>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="26" t="inlineStr">
         <is>
-          <t>한국파마</t>
+          <t>LK삼양</t>
         </is>
       </c>
       <c r="B38" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C38" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D38" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E38" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F38" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G38" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="H38" s="27" t="n">
-        <v>13.42</v>
+        <v>18.37</v>
       </c>
       <c r="I38" s="27" t="n">
-        <v>19.06</v>
+        <v>18.08</v>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="26" t="inlineStr">
         <is>
-          <t>한화솔루션</t>
+          <t>글로벌테크놀로지</t>
         </is>
       </c>
       <c r="B39" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C39" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D39" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E39" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F39" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G39" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
-        </is>
-      </c>
-      <c r="H39" s="27" t="n">
-        <v>5.71</v>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="H39" s="29" t="n">
+        <v>-8.550000000000001</v>
       </c>
       <c r="I39" s="27" t="n">
-        <v>5.4</v>
+        <v>2.48</v>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="26" t="inlineStr">
         <is>
-          <t>한화오션</t>
+          <t>덕산넵코어스</t>
         </is>
       </c>
       <c r="B40" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C40" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D40" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E40" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F40" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G40" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
-        </is>
-      </c>
-      <c r="H40" s="27" t="n">
-        <v>0.13</v>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="H40" s="29" t="n">
+        <v>-1.75</v>
       </c>
       <c r="I40" s="29" t="n">
-        <v>-2.24</v>
+        <v>-3.09</v>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="26" t="inlineStr">
         <is>
-          <t>현대건설</t>
+          <t>덕우전자</t>
         </is>
       </c>
       <c r="B41" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C41" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D41" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E41" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F41" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G41" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
-        </is>
-      </c>
-      <c r="H41" s="29" t="n">
-        <v>-2.22</v>
-      </c>
-      <c r="I41" s="29" t="n">
-        <v>-6.9</v>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="H41" s="27" t="n">
+        <v>17.91</v>
+      </c>
+      <c r="I41" s="27" t="n">
+        <v>53.62</v>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="26" t="inlineStr">
         <is>
-          <t>KBI동양철관</t>
+          <t>부산주공</t>
         </is>
       </c>
       <c r="B42" s="25" t="n">
@@ -4483,25 +4483,25 @@
       </c>
       <c r="F42" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G42" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="H42" s="29" t="n">
-        <v>-4.36</v>
-      </c>
-      <c r="I42" s="27" t="n">
-        <v>16.03</v>
+        <v>-32.5</v>
+      </c>
+      <c r="I42" s="29" t="n">
+        <v>-94.44</v>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="26" t="inlineStr">
         <is>
-          <t>글로벌테크놀로지</t>
+          <t>브릴스</t>
         </is>
       </c>
       <c r="B43" s="25" t="n">
@@ -4518,25 +4518,25 @@
       </c>
       <c r="F43" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G43" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
-        </is>
-      </c>
-      <c r="H43" s="29" t="n">
-        <v>-8.550000000000001</v>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="H43" s="27" t="n">
+        <v>9.81</v>
       </c>
       <c r="I43" s="27" t="n">
-        <v>2.48</v>
+        <v>9.81</v>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="26" t="inlineStr">
         <is>
-          <t>덕산넵코어스</t>
+          <t>빅웨이브로보틱스</t>
         </is>
       </c>
       <c r="B44" s="25" t="n">
@@ -4553,25 +4553,25 @@
       </c>
       <c r="F44" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G44" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
-        </is>
-      </c>
-      <c r="H44" s="29" t="n">
-        <v>-1.75</v>
-      </c>
-      <c r="I44" s="29" t="n">
-        <v>-3.09</v>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="H44" s="27" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="I44" s="27" t="n">
+        <v>17.38</v>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="26" t="inlineStr">
         <is>
-          <t>덕우전자</t>
+          <t>세미티에스</t>
         </is>
       </c>
       <c r="B45" s="25" t="n">
@@ -4588,25 +4588,25 @@
       </c>
       <c r="F45" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G45" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="H45" s="27" t="n">
-        <v>17.91</v>
+        <v>2.06</v>
       </c>
       <c r="I45" s="27" t="n">
-        <v>53.62</v>
+        <v>27.22</v>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="26" t="inlineStr">
         <is>
-          <t>부산주공</t>
+          <t>에이프릴바이오</t>
         </is>
       </c>
       <c r="B46" s="25" t="n">
@@ -4623,25 +4623,25 @@
       </c>
       <c r="F46" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G46" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="H46" s="29" t="n">
-        <v>-32.5</v>
+        <v>-21.12</v>
       </c>
       <c r="I46" s="29" t="n">
-        <v>-94.44</v>
+        <v>-9.390000000000001</v>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="26" t="inlineStr">
         <is>
-          <t>브릴스</t>
+          <t>원일티엔아이</t>
         </is>
       </c>
       <c r="B47" s="25" t="n">
@@ -4658,25 +4658,25 @@
       </c>
       <c r="F47" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G47" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="H47" s="27" t="n">
-        <v>9.81</v>
+        <v>18.34</v>
       </c>
       <c r="I47" s="27" t="n">
-        <v>9.81</v>
+        <v>54.33</v>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="26" t="inlineStr">
         <is>
-          <t>빅웨이브로보틱스</t>
+          <t>윈팩</t>
         </is>
       </c>
       <c r="B48" s="25" t="n">
@@ -4693,25 +4693,25 @@
       </c>
       <c r="F48" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G48" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="H48" s="27" t="n">
-        <v>2.75</v>
+        <v>4.95</v>
       </c>
       <c r="I48" s="27" t="n">
-        <v>17.38</v>
+        <v>72.38</v>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="26" t="inlineStr">
         <is>
-          <t>원일티엔아이</t>
+          <t>코스모로보틱스</t>
         </is>
       </c>
       <c r="B49" s="25" t="n">
@@ -4728,25 +4728,25 @@
       </c>
       <c r="F49" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G49" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
-        </is>
-      </c>
-      <c r="H49" s="27" t="n">
-        <v>18.34</v>
-      </c>
-      <c r="I49" s="27" t="n">
-        <v>54.33</v>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="H49" s="29" t="n">
+        <v>-8.460000000000001</v>
+      </c>
+      <c r="I49" s="29" t="n">
+        <v>-30.64</v>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="26" t="inlineStr">
         <is>
-          <t>윈팩</t>
+          <t>피제이전자</t>
         </is>
       </c>
       <c r="B50" s="25" t="n">
@@ -4763,25 +4763,25 @@
       </c>
       <c r="F50" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G50" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="H50" s="27" t="n">
-        <v>4.95</v>
+        <v>30.5</v>
       </c>
       <c r="I50" s="27" t="n">
-        <v>72.38</v>
+        <v>29.32</v>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="26" t="inlineStr">
         <is>
-          <t>코스모로보틱스</t>
+          <t>한국비엔씨</t>
         </is>
       </c>
       <c r="B51" s="25" t="n">
@@ -4798,19 +4798,19 @@
       </c>
       <c r="F51" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G51" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="H51" s="29" t="n">
-        <v>-8.460000000000001</v>
+        <v>-3.07</v>
       </c>
       <c r="I51" s="29" t="n">
-        <v>-30.64</v>
+        <v>-7.74</v>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
@@ -4833,12 +4833,12 @@
       </c>
       <c r="F52" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G52" s="25" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="H52" s="29" t="n">
@@ -4929,19 +4929,19 @@
         <v>1</v>
       </c>
       <c r="C3" s="36" t="n">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="D3" s="36" t="n">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="E3" s="36" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="F3" s="37" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G3" s="37" t="inlineStr">
@@ -4960,19 +4960,19 @@
         <v>1</v>
       </c>
       <c r="C4" s="36" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D4" s="36" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E4" s="36" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="F4" s="37" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G4" s="37" t="inlineStr">
@@ -4991,19 +4991,19 @@
         <v>1</v>
       </c>
       <c r="C5" s="36" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D5" s="36" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E5" s="36" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="F5" s="37" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G5" s="37" t="inlineStr">
@@ -5022,19 +5022,19 @@
         <v>1</v>
       </c>
       <c r="C6" s="36" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="D6" s="36" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="E6" s="36" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="F6" s="37" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G6" s="37" t="inlineStr">
@@ -5053,19 +5053,19 @@
         <v>1</v>
       </c>
       <c r="C7" s="36" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D7" s="36" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E7" s="36" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="F7" s="37" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G7" s="37" t="inlineStr">
@@ -5077,26 +5077,26 @@
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="35" t="inlineStr">
         <is>
-          <t>철강</t>
+          <t>게임</t>
         </is>
       </c>
       <c r="B8" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="36" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D8" s="36" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E8" s="36" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="F8" s="37" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G8" s="37" t="inlineStr">
@@ -5115,19 +5115,19 @@
         <v>1</v>
       </c>
       <c r="C9" s="36" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D9" s="36" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E9" s="36" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="F9" s="37" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G9" s="37" t="inlineStr">
@@ -5153,12 +5153,12 @@
       </c>
       <c r="E10" s="36" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="F10" s="37" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G10" s="37" t="inlineStr">
@@ -5305,7 +5305,7 @@
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>게임</t>
+          <t>엔터</t>
         </is>
       </c>
       <c r="B16" s="25" t="n">
@@ -5332,7 +5332,7 @@
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>엔터</t>
+          <t>핀테크</t>
         </is>
       </c>
       <c r="B17" s="25" t="n">
@@ -5359,7 +5359,7 @@
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="26" t="inlineStr">
         <is>
-          <t>핀테크</t>
+          <t>클라우드</t>
         </is>
       </c>
       <c r="B18" s="25" t="n">
@@ -5386,7 +5386,7 @@
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>클라우드</t>
+          <t>조선</t>
         </is>
       </c>
       <c r="B19" s="25" t="n">
@@ -5413,7 +5413,7 @@
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="26" t="inlineStr">
         <is>
-          <t>조선</t>
+          <t>철강</t>
         </is>
       </c>
       <c r="B20" s="25" t="n">

</xml_diff>

<commit_message>
auto: 2026-10-06 07:01 자동 백업
</commit_message>
<xml_diff>
--- a/trend/stock_trend_history.xlsx
+++ b/trend/stock_trend_history.xlsx
@@ -258,13 +258,13 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -694,7 +694,7 @@
     <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-10-05 06:54</t>
+          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-10-06 06:54</t>
         </is>
       </c>
     </row>
@@ -708,7 +708,7 @@
       </c>
       <c r="E3" s="3" t="n"/>
       <c r="G3" s="5" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="H3" s="3" t="n"/>
       <c r="J3" s="6" t="n">
@@ -787,21 +787,21 @@
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-10-05) 상위: 반도체  점수 51.0점</t>
+          <t>⚡ 최신(2026-10-06) 상위: 반도체  점수 60.0점</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-10-05) 상위: 삼성전자  점수 43.0점</t>
+          <t>⚡ 최신(2026-10-06) 상위: 삼성전자  점수 33.0점</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-10-05) 상위: 인공지능  점수 24.0점</t>
+          <t>⚡ 최신(2026-10-06) 상위: 인공지능  점수 22.0점</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="15" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B14" s="15" t="n">
@@ -928,10 +928,10 @@
         </is>
       </c>
       <c r="D14" s="15" t="n">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="E14" s="15" t="n">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="F14" s="15" t="n">
         <v>0</v>
@@ -947,7 +947,7 @@
       </c>
       <c r="J14" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K14" s="17" t="inlineStr">
@@ -959,7 +959,7 @@
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="15" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B15" s="15" t="n">
@@ -971,10 +971,10 @@
         </is>
       </c>
       <c r="D15" s="15" t="n">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="E15" s="15" t="n">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="F15" s="15" t="n">
         <v>0</v>
@@ -990,19 +990,19 @@
       </c>
       <c r="J15" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급</t>
+          <t>Google 급상승 검색어 등장 (KR) / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K15" s="17" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>네이버, Google</t>
         </is>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="15" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B16" s="15" t="n">
@@ -1014,10 +1014,10 @@
         </is>
       </c>
       <c r="D16" s="15" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E16" s="15" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="F16" s="15" t="n">
         <v>0</v>
@@ -1033,7 +1033,7 @@
       </c>
       <c r="J16" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급</t>
+          <t>매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K16" s="17" t="inlineStr">
@@ -1045,7 +1045,7 @@
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B17" s="15" t="n">
@@ -1053,14 +1053,14 @@
       </c>
       <c r="C17" s="16" t="inlineStr">
         <is>
-          <t>현대차</t>
+          <t>바이오</t>
         </is>
       </c>
       <c r="D17" s="15" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E17" s="15" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F17" s="15" t="n">
         <v>0</v>
@@ -1068,25 +1068,27 @@
       <c r="G17" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H17" s="19" t="n">
-        <v>-0.57</v>
-      </c>
-      <c r="I17" s="19" t="n">
-        <v>-1.98</v>
+      <c r="H17" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I17" s="15" t="n">
+        <v/>
       </c>
       <c r="J17" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K17" s="17" t="n">
-        <v/>
+          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
+        </is>
+      </c>
+      <c r="K17" s="17" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B18" s="15" t="n">
@@ -1098,10 +1100,10 @@
         </is>
       </c>
       <c r="D18" s="15" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E18" s="15" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="F18" s="15" t="n">
         <v>0</v>
@@ -1117,7 +1119,7 @@
       </c>
       <c r="J18" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K18" s="17" t="inlineStr">
@@ -1129,7 +1131,7 @@
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B19" s="15" t="n">
@@ -1141,10 +1143,10 @@
         </is>
       </c>
       <c r="D19" s="15" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E19" s="15" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="F19" s="15" t="n">
         <v>0</v>
@@ -1160,19 +1162,17 @@
       </c>
       <c r="J19" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K19" s="17" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K19" s="17" t="n">
+        <v/>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B20" s="15" t="n">
@@ -1180,14 +1180,14 @@
       </c>
       <c r="C20" s="16" t="inlineStr">
         <is>
-          <t>바이오</t>
+          <t>현대차</t>
         </is>
       </c>
       <c r="D20" s="15" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="E20" s="15" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F20" s="15" t="n">
         <v>0</v>
@@ -1195,27 +1195,25 @@
       <c r="G20" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H20" s="15" t="n">
+      <c r="H20" s="19" t="n">
+        <v>-0.57</v>
+      </c>
+      <c r="I20" s="19" t="n">
+        <v>-1.98</v>
+      </c>
+      <c r="J20" s="17" t="inlineStr">
+        <is>
+          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K20" s="17" t="n">
         <v/>
-      </c>
-      <c r="I20" s="15" t="n">
-        <v/>
-      </c>
-      <c r="J20" s="17" t="inlineStr">
-        <is>
-          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
-        </is>
-      </c>
-      <c r="K20" s="17" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="15" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B21" s="15" t="n">
@@ -1223,14 +1221,14 @@
       </c>
       <c r="C21" s="16" t="inlineStr">
         <is>
-          <t>SK하이닉스</t>
+          <t>스테이블코인</t>
         </is>
       </c>
       <c r="D21" s="15" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E21" s="15" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F21" s="15" t="n">
         <v>0</v>
@@ -1238,27 +1236,25 @@
       <c r="G21" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H21" s="18" t="n">
-        <v>0.77</v>
-      </c>
-      <c r="I21" s="18" t="n">
-        <v>4.6</v>
+      <c r="H21" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I21" s="15" t="n">
+        <v/>
       </c>
       <c r="J21" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
-        </is>
-      </c>
-      <c r="K21" s="17" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+          <t>한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K21" s="17" t="n">
+        <v/>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="15" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B22" s="15" t="n">
@@ -1266,42 +1262,40 @@
       </c>
       <c r="C22" s="16" t="inlineStr">
         <is>
-          <t>삼성E&amp;A</t>
+          <t>원전</t>
         </is>
       </c>
       <c r="D22" s="15" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="E22" s="15" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="F22" s="15" t="n">
         <v>0</v>
       </c>
       <c r="G22" s="15" t="n">
-        <v>3</v>
-      </c>
-      <c r="H22" s="18" t="n">
-        <v>0.84</v>
-      </c>
-      <c r="I22" s="19" t="n">
-        <v>-4.11</v>
+        <v>0</v>
+      </c>
+      <c r="H22" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I22" s="15" t="n">
+        <v/>
       </c>
       <c r="J22" s="17" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 7일 +100% / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K22" s="17" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K22" s="17" t="n">
+        <v/>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="15" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B23" s="15" t="n">
@@ -1309,14 +1303,14 @@
       </c>
       <c r="C23" s="16" t="inlineStr">
         <is>
-          <t>원전</t>
+          <t>전기차</t>
         </is>
       </c>
       <c r="D23" s="15" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="E23" s="15" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F23" s="15" t="n">
         <v>0</v>
@@ -1332,17 +1326,19 @@
       </c>
       <c r="J23" s="17" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K23" s="17" t="n">
-        <v/>
+          <t>네이버뉴스 기사 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K23" s="17" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="15" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B24" s="15" t="n">
@@ -1350,14 +1346,14 @@
       </c>
       <c r="C24" s="16" t="inlineStr">
         <is>
-          <t>스테이블코인</t>
+          <t>방산</t>
         </is>
       </c>
       <c r="D24" s="15" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E24" s="15" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F24" s="15" t="n">
         <v>0</v>
@@ -1373,7 +1369,7 @@
       </c>
       <c r="J24" s="17" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K24" s="17" t="n">
@@ -1381,95 +1377,95 @@
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
-      <c r="A25" s="20" t="inlineStr">
-        <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
-      <c r="B25" s="20" t="n">
+      <c r="A25" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B25" s="15" t="n">
         <v>12</v>
       </c>
-      <c r="C25" s="21" t="inlineStr">
-        <is>
-          <t>세미파이브</t>
-        </is>
-      </c>
-      <c r="D25" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="E25" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F25" s="20" t="n">
-        <v>2</v>
-      </c>
-      <c r="G25" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H25" s="22" t="n">
-        <v>1.72</v>
-      </c>
-      <c r="I25" s="22" t="n">
-        <v>28.88</v>
-      </c>
-      <c r="J25" s="23" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +458% / 중요공시 2건 / 중요공시 3일 +100%</t>
-        </is>
-      </c>
-      <c r="K25" s="23" t="inlineStr">
-        <is>
-          <t>공시, 네이버</t>
+      <c r="C25" s="16" t="inlineStr">
+        <is>
+          <t>한화솔루션</t>
+        </is>
+      </c>
+      <c r="D25" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="E25" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="F25" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" s="18" t="n">
+        <v>5.71</v>
+      </c>
+      <c r="I25" s="18" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="J25" s="17" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +168% / 중요공시 1건 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K25" s="17" t="inlineStr">
+        <is>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
-      <c r="A26" s="20" t="inlineStr">
-        <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
-      <c r="B26" s="20" t="n">
+      <c r="A26" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B26" s="15" t="n">
         <v>13</v>
       </c>
-      <c r="C26" s="21" t="inlineStr">
-        <is>
-          <t>삼성중공업</t>
-        </is>
-      </c>
-      <c r="D26" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="E26" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F26" s="20" t="n">
-        <v>2</v>
-      </c>
-      <c r="G26" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H26" s="22" t="n">
-        <v>0.91</v>
-      </c>
-      <c r="I26" s="24" t="n">
-        <v>-1.14</v>
-      </c>
-      <c r="J26" s="23" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +57% / 중요공시 2건 / 중요공시 3일 +100% / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K26" s="23" t="inlineStr">
-        <is>
-          <t>공시, 네이버</t>
+      <c r="C26" s="16" t="inlineStr">
+        <is>
+          <t>대한항공</t>
+        </is>
+      </c>
+      <c r="D26" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="E26" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="F26" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" s="19" t="n">
+        <v>-0.64</v>
+      </c>
+      <c r="I26" s="19" t="n">
+        <v>-1.91</v>
+      </c>
+      <c r="J26" s="17" t="inlineStr">
+        <is>
+          <t>중요공시 2건 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K26" s="17" t="inlineStr">
+        <is>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="20" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B27" s="20" t="n">
@@ -1477,7 +1473,7 @@
       </c>
       <c r="C27" s="21" t="inlineStr">
         <is>
-          <t>대한항공</t>
+          <t>삼성전자우</t>
         </is>
       </c>
       <c r="D27" s="20" t="n">
@@ -1492,27 +1488,27 @@
       <c r="G27" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H27" s="24" t="n">
-        <v>-0.64</v>
-      </c>
-      <c r="I27" s="24" t="n">
-        <v>-1.91</v>
+      <c r="H27" s="22" t="n">
+        <v>-0.25</v>
+      </c>
+      <c r="I27" s="22" t="n">
+        <v>-1.95</v>
       </c>
       <c r="J27" s="23" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+          <t>Google 급상승 검색어 등장 (KR)</t>
         </is>
       </c>
       <c r="K27" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>Google</t>
         </is>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="20" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B28" s="20" t="n">
@@ -1520,40 +1516,42 @@
       </c>
       <c r="C28" s="21" t="inlineStr">
         <is>
-          <t>SG</t>
+          <t>더코디</t>
         </is>
       </c>
       <c r="D28" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E28" s="20" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F28" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G28" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H28" s="24" t="n">
-        <v>-5.15</v>
-      </c>
-      <c r="I28" s="24" t="n">
-        <v>-2.64</v>
+        <v>3</v>
+      </c>
+      <c r="H28" s="22" t="n">
+        <v>-1.27</v>
+      </c>
+      <c r="I28" s="22" t="n">
+        <v>-20.87</v>
       </c>
       <c r="J28" s="23" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K28" s="23" t="n">
-        <v/>
+          <t>중요공시 6건 / 중요공시 7일 +100%</t>
+        </is>
+      </c>
+      <c r="K28" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="20" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B29" s="20" t="n">
@@ -1561,42 +1559,40 @@
       </c>
       <c r="C29" s="21" t="inlineStr">
         <is>
-          <t>모아데이타</t>
+          <t>AI반도체</t>
         </is>
       </c>
       <c r="D29" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E29" s="20" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F29" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G29" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="H29" s="24" t="n">
-        <v>-3.6</v>
-      </c>
-      <c r="I29" s="24" t="n">
-        <v>-1.83</v>
+        <v>0</v>
+      </c>
+      <c r="H29" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I29" s="20" t="n">
+        <v/>
       </c>
       <c r="J29" s="23" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 7일 +50%</t>
-        </is>
-      </c>
-      <c r="K29" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K29" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="20" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B30" s="20" t="n">
@@ -1604,42 +1600,40 @@
       </c>
       <c r="C30" s="21" t="inlineStr">
         <is>
-          <t>루닛</t>
+          <t>LG전자</t>
         </is>
       </c>
       <c r="D30" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E30" s="20" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F30" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G30" s="20" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H30" s="24" t="n">
-        <v>-5.03</v>
+        <v>1.65</v>
       </c>
       <c r="I30" s="24" t="n">
-        <v>-5.88</v>
+        <v>0.47</v>
       </c>
       <c r="J30" s="23" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 3일 +100% / 중요공시 7일 +100%</t>
-        </is>
-      </c>
-      <c r="K30" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K30" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="20" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B31" s="20" t="n">
@@ -1647,7 +1641,7 @@
       </c>
       <c r="C31" s="21" t="inlineStr">
         <is>
-          <t>전기차</t>
+          <t>케이뱅크</t>
         </is>
       </c>
       <c r="D31" s="20" t="n">
@@ -1662,15 +1656,15 @@
       <c r="G31" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H31" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I31" s="20" t="n">
-        <v/>
+      <c r="H31" s="22" t="n">
+        <v>-0.19</v>
+      </c>
+      <c r="I31" s="22" t="n">
+        <v>-1.82</v>
       </c>
       <c r="J31" s="23" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>한국경제 헤드라인 언급 / 매일경제 기사 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K31" s="23" t="n">
@@ -1680,7 +1674,7 @@
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="20" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B32" s="20" t="n">
@@ -1688,7 +1682,7 @@
       </c>
       <c r="C32" s="21" t="inlineStr">
         <is>
-          <t>머큐리</t>
+          <t>SK하이닉스</t>
         </is>
       </c>
       <c r="D32" s="20" t="n">
@@ -1703,27 +1697,25 @@
       <c r="G32" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H32" s="22" t="n">
-        <v>29.8</v>
-      </c>
-      <c r="I32" s="22" t="n">
-        <v>28.21</v>
+      <c r="H32" s="24" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="I32" s="24" t="n">
+        <v>4.6</v>
       </c>
       <c r="J32" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +99% / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K32" s="23" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+          <t>매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K32" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="20" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B33" s="20" t="n">
@@ -1731,42 +1723,40 @@
       </c>
       <c r="C33" s="21" t="inlineStr">
         <is>
-          <t>팬오션</t>
+          <t>SG</t>
         </is>
       </c>
       <c r="D33" s="20" t="n">
         <v>5</v>
       </c>
       <c r="E33" s="20" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F33" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G33" s="20" t="n">
         <v>0</v>
       </c>
       <c r="H33" s="22" t="n">
-        <v>6.47</v>
+        <v>-5.15</v>
       </c>
       <c r="I33" s="22" t="n">
-        <v>9.84</v>
+        <v>-2.64</v>
       </c>
       <c r="J33" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +76% / 중요공시 2건 / 중요공시 3일 +100%</t>
-        </is>
-      </c>
-      <c r="K33" s="23" t="inlineStr">
-        <is>
-          <t>공시, 네이버</t>
-        </is>
+          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K33" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="20" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B34" s="20" t="n">
@@ -1774,7 +1764,7 @@
       </c>
       <c r="C34" s="21" t="inlineStr">
         <is>
-          <t>더코디</t>
+          <t>삼성바이오로직스</t>
         </is>
       </c>
       <c r="D34" s="20" t="n">
@@ -1789,15 +1779,15 @@
       <c r="G34" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H34" s="24" t="n">
-        <v>-1.27</v>
-      </c>
-      <c r="I34" s="24" t="n">
-        <v>-20.87</v>
+      <c r="H34" s="22" t="n">
+        <v>-3.6</v>
+      </c>
+      <c r="I34" s="22" t="n">
+        <v>-0.96</v>
       </c>
       <c r="J34" s="23" t="inlineStr">
         <is>
-          <t>중요공시 6건 / 중요공시 3일 +100%</t>
+          <t>중요공시 3건 / 중요공시 3일 +50%</t>
         </is>
       </c>
       <c r="K34" s="23" t="inlineStr">
@@ -1809,7 +1799,7 @@
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="20" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B35" s="20" t="n">
@@ -1832,10 +1822,10 @@
       <c r="G35" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H35" s="22" t="n">
+      <c r="H35" s="24" t="n">
         <v>2.94</v>
       </c>
-      <c r="I35" s="24" t="n">
+      <c r="I35" s="22" t="n">
         <v>-8.050000000000001</v>
       </c>
       <c r="J35" s="23" t="inlineStr">
@@ -1852,7 +1842,7 @@
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="20" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B36" s="20" t="n">
@@ -1875,27 +1865,27 @@
       <c r="G36" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H36" s="24" t="n">
+      <c r="H36" s="22" t="n">
         <v>-1.63</v>
       </c>
-      <c r="I36" s="24" t="n">
+      <c r="I36" s="22" t="n">
         <v>-51.68</v>
       </c>
       <c r="J36" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +1785% / 중요공시 1건</t>
+          <t>네이버 검색 당일 +1842% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K36" s="23" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="20" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B37" s="20" t="n">
@@ -1903,7 +1893,7 @@
       </c>
       <c r="C37" s="21" t="inlineStr">
         <is>
-          <t>나인테크</t>
+          <t>세미파이브</t>
         </is>
       </c>
       <c r="D37" s="20" t="n">
@@ -1918,27 +1908,27 @@
       <c r="G37" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H37" s="22" t="n">
-        <v>0.71</v>
-      </c>
-      <c r="I37" s="22" t="n">
-        <v>28.05</v>
+      <c r="H37" s="24" t="n">
+        <v>1.72</v>
+      </c>
+      <c r="I37" s="24" t="n">
+        <v>28.88</v>
       </c>
       <c r="J37" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +451% / 중요공시 1건</t>
+          <t>네이버 검색 당일 +476% / 중요공시 2건</t>
         </is>
       </c>
       <c r="K37" s="23" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="20" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B38" s="20" t="n">
@@ -1946,7 +1936,7 @@
       </c>
       <c r="C38" s="21" t="inlineStr">
         <is>
-          <t>한국파마</t>
+          <t>나인테크</t>
         </is>
       </c>
       <c r="D38" s="20" t="n">
@@ -1961,27 +1951,27 @@
       <c r="G38" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H38" s="22" t="n">
-        <v>13.42</v>
-      </c>
-      <c r="I38" s="22" t="n">
-        <v>19.06</v>
+      <c r="H38" s="24" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="I38" s="24" t="n">
+        <v>28.05</v>
       </c>
       <c r="J38" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +229% / 중요공시 1건</t>
+          <t>네이버 검색 당일 +459% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K38" s="23" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="20" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B39" s="20" t="n">
@@ -1989,7 +1979,7 @@
       </c>
       <c r="C39" s="21" t="inlineStr">
         <is>
-          <t>한창</t>
+          <t>한국파마</t>
         </is>
       </c>
       <c r="D39" s="20" t="n">
@@ -2005,26 +1995,26 @@
         <v>0</v>
       </c>
       <c r="H39" s="24" t="n">
-        <v>-91.06999999999999</v>
+        <v>13.42</v>
       </c>
       <c r="I39" s="24" t="n">
-        <v>-91.06999999999999</v>
+        <v>19.06</v>
       </c>
       <c r="J39" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +197% / 중요공시 1건</t>
+          <t>네이버 검색 당일 +249% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K39" s="23" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="20" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B40" s="20" t="n">
@@ -2032,7 +2022,7 @@
       </c>
       <c r="C40" s="21" t="inlineStr">
         <is>
-          <t>한화솔루션</t>
+          <t>고영</t>
         </is>
       </c>
       <c r="D40" s="20" t="n">
@@ -2047,27 +2037,27 @@
       <c r="G40" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H40" s="22" t="n">
-        <v>5.71</v>
-      </c>
-      <c r="I40" s="22" t="n">
-        <v>5.4</v>
+      <c r="H40" s="24" t="n">
+        <v>1.47</v>
+      </c>
+      <c r="I40" s="24" t="n">
+        <v>19.41</v>
       </c>
       <c r="J40" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +163% / 중요공시 1건</t>
+          <t>네이버 검색 당일 +128% / 중요공시 2건</t>
         </is>
       </c>
       <c r="K40" s="23" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="20" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B41" s="20" t="n">
@@ -2075,7 +2065,7 @@
       </c>
       <c r="C41" s="21" t="inlineStr">
         <is>
-          <t>고영</t>
+          <t>오텍</t>
         </is>
       </c>
       <c r="D41" s="20" t="n">
@@ -2090,27 +2080,27 @@
       <c r="G41" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H41" s="22" t="n">
-        <v>1.47</v>
-      </c>
-      <c r="I41" s="22" t="n">
-        <v>19.41</v>
+      <c r="H41" s="24" t="n">
+        <v>8.32</v>
+      </c>
+      <c r="I41" s="24" t="n">
+        <v>13.69</v>
       </c>
       <c r="J41" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +121% / 중요공시 2건</t>
+          <t>네이버 검색 당일 +109% / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K41" s="23" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="20" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B42" s="20" t="n">
@@ -2118,42 +2108,42 @@
       </c>
       <c r="C42" s="21" t="inlineStr">
         <is>
-          <t>에이에프더블류</t>
+          <t>티엠씨</t>
         </is>
       </c>
       <c r="D42" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E42" s="20" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F42" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G42" s="20" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H42" s="24" t="n">
-        <v>-5.13</v>
+        <v>29.68</v>
       </c>
       <c r="I42" s="24" t="n">
-        <v>-51.32</v>
+        <v>33.33</v>
       </c>
       <c r="J42" s="23" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 7일 +100%</t>
+          <t>네이버 검색 당일 +79% / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K42" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="20" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B43" s="20" t="n">
@@ -2161,42 +2151,42 @@
       </c>
       <c r="C43" s="21" t="inlineStr">
         <is>
-          <t>아리바이오홀딩스</t>
+          <t>삼성중공업</t>
         </is>
       </c>
       <c r="D43" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E43" s="20" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F43" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G43" s="20" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H43" s="24" t="n">
-        <v>-2.23</v>
-      </c>
-      <c r="I43" s="24" t="n">
-        <v>-22.96</v>
+        <v>0.91</v>
+      </c>
+      <c r="I43" s="22" t="n">
+        <v>-1.14</v>
       </c>
       <c r="J43" s="23" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 7일 +100%</t>
+          <t>네이버 검색 당일 +60% / 중요공시 2건 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K43" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="20" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B44" s="20" t="n">
@@ -2204,7 +2194,7 @@
       </c>
       <c r="C44" s="21" t="inlineStr">
         <is>
-          <t>선도전기</t>
+          <t>에이에프더블류</t>
         </is>
       </c>
       <c r="D44" s="20" t="n">
@@ -2219,11 +2209,11 @@
       <c r="G44" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="H44" s="24" t="n">
-        <v>-1.82</v>
-      </c>
-      <c r="I44" s="24" t="n">
-        <v>-1.82</v>
+      <c r="H44" s="22" t="n">
+        <v>-5.13</v>
+      </c>
+      <c r="I44" s="22" t="n">
+        <v>-51.32</v>
       </c>
       <c r="J44" s="23" t="inlineStr">
         <is>
@@ -2239,7 +2229,7 @@
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="20" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B45" s="20" t="n">
@@ -2247,7 +2237,7 @@
       </c>
       <c r="C45" s="21" t="inlineStr">
         <is>
-          <t>한화오션</t>
+          <t>아리바이오홀딩스</t>
         </is>
       </c>
       <c r="D45" s="20" t="n">
@@ -2263,10 +2253,10 @@
         <v>3</v>
       </c>
       <c r="H45" s="22" t="n">
-        <v>0.13</v>
-      </c>
-      <c r="I45" s="24" t="n">
-        <v>-2.24</v>
+        <v>-2.23</v>
+      </c>
+      <c r="I45" s="22" t="n">
+        <v>-22.96</v>
       </c>
       <c r="J45" s="23" t="inlineStr">
         <is>
@@ -2282,7 +2272,7 @@
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="20" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B46" s="20" t="n">
@@ -2290,7 +2280,7 @@
       </c>
       <c r="C46" s="21" t="inlineStr">
         <is>
-          <t>미래산업</t>
+          <t>삼성E&amp;A</t>
         </is>
       </c>
       <c r="D46" s="20" t="n">
@@ -2305,11 +2295,11 @@
       <c r="G46" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="H46" s="22" t="n">
-        <v>0.6</v>
+      <c r="H46" s="24" t="n">
+        <v>0.84</v>
       </c>
       <c r="I46" s="22" t="n">
-        <v>16.62</v>
+        <v>-4.11</v>
       </c>
       <c r="J46" s="23" t="inlineStr">
         <is>
@@ -2325,7 +2315,7 @@
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="20" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B47" s="20" t="n">
@@ -2333,83 +2323,83 @@
       </c>
       <c r="C47" s="21" t="inlineStr">
         <is>
-          <t>게임</t>
+          <t>선도전기</t>
         </is>
       </c>
       <c r="D47" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E47" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="F47" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="H47" s="22" t="n">
+        <v>-1.82</v>
+      </c>
+      <c r="I47" s="22" t="n">
+        <v>-1.82</v>
+      </c>
+      <c r="J47" s="23" t="inlineStr">
+        <is>
+          <t>중요공시 2건 / 중요공시 7일 +100%</t>
+        </is>
+      </c>
+      <c r="K47" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="18" customHeight="1">
+      <c r="A48" s="20" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B48" s="20" t="n">
+        <v>35</v>
+      </c>
+      <c r="C48" s="21" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
+      </c>
+      <c r="D48" s="20" t="n">
         <v>4</v>
       </c>
-      <c r="F47" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G47" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H47" s="20" t="n">
+      <c r="E48" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F48" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G48" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H48" s="20" t="n">
         <v/>
       </c>
-      <c r="I47" s="20" t="n">
+      <c r="I48" s="20" t="n">
         <v/>
       </c>
-      <c r="J47" s="23" t="inlineStr">
+      <c r="J48" s="23" t="inlineStr">
         <is>
           <t>한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
-      <c r="K47" s="23" t="n">
+      <c r="K48" s="23" t="n">
         <v/>
-      </c>
-    </row>
-    <row r="48" ht="18" customHeight="1">
-      <c r="A48" s="25" t="inlineStr">
-        <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
-      <c r="B48" s="25" t="n">
-        <v>35</v>
-      </c>
-      <c r="C48" s="26" t="inlineStr">
-        <is>
-          <t>브릴스</t>
-        </is>
-      </c>
-      <c r="D48" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="E48" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="F48" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="G48" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H48" s="27" t="n">
-        <v>9.81</v>
-      </c>
-      <c r="I48" s="27" t="n">
-        <v>9.81</v>
-      </c>
-      <c r="J48" s="28" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +2323%</t>
-        </is>
-      </c>
-      <c r="K48" s="28" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B49" s="25" t="n">
@@ -2417,7 +2407,7 @@
       </c>
       <c r="C49" s="26" t="inlineStr">
         <is>
-          <t>현대바이오랜드</t>
+          <t>브릴스</t>
         </is>
       </c>
       <c r="D49" s="25" t="n">
@@ -2432,15 +2422,15 @@
       <c r="G49" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H49" s="29" t="n">
-        <v>-3.29</v>
+      <c r="H49" s="27" t="n">
+        <v>9.81</v>
       </c>
       <c r="I49" s="27" t="n">
-        <v>10.25</v>
+        <v>9.81</v>
       </c>
       <c r="J49" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +1636%</t>
+          <t>네이버 검색 당일 +2379%</t>
         </is>
       </c>
       <c r="K49" s="28" t="inlineStr">
@@ -2452,7 +2442,7 @@
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B50" s="25" t="n">
@@ -2460,7 +2450,7 @@
       </c>
       <c r="C50" s="26" t="inlineStr">
         <is>
-          <t>코스모로보틱스</t>
+          <t>현대바이오랜드</t>
         </is>
       </c>
       <c r="D50" s="25" t="n">
@@ -2476,14 +2466,14 @@
         <v>0</v>
       </c>
       <c r="H50" s="29" t="n">
-        <v>-8.460000000000001</v>
-      </c>
-      <c r="I50" s="29" t="n">
-        <v>-30.64</v>
+        <v>-3.29</v>
+      </c>
+      <c r="I50" s="27" t="n">
+        <v>10.25</v>
       </c>
       <c r="J50" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +1408%</t>
+          <t>네이버 검색 당일 +1656%</t>
         </is>
       </c>
       <c r="K50" s="28" t="inlineStr">
@@ -2495,7 +2485,7 @@
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B51" s="25" t="n">
@@ -2503,7 +2493,7 @@
       </c>
       <c r="C51" s="26" t="inlineStr">
         <is>
-          <t>글로벌테크놀로지</t>
+          <t>코스모로보틱스</t>
         </is>
       </c>
       <c r="D51" s="25" t="n">
@@ -2519,14 +2509,14 @@
         <v>0</v>
       </c>
       <c r="H51" s="29" t="n">
-        <v>-8.550000000000001</v>
-      </c>
-      <c r="I51" s="27" t="n">
-        <v>2.48</v>
+        <v>-8.460000000000001</v>
+      </c>
+      <c r="I51" s="29" t="n">
+        <v>-30.64</v>
       </c>
       <c r="J51" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +1378%</t>
+          <t>네이버 검색 당일 +1429%</t>
         </is>
       </c>
       <c r="K51" s="28" t="inlineStr">
@@ -2538,7 +2528,7 @@
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B52" s="25" t="n">
@@ -2546,7 +2536,7 @@
       </c>
       <c r="C52" s="26" t="inlineStr">
         <is>
-          <t>덕산넵코어스</t>
+          <t>글로벌테크놀로지</t>
         </is>
       </c>
       <c r="D52" s="25" t="n">
@@ -2562,14 +2552,14 @@
         <v>0</v>
       </c>
       <c r="H52" s="29" t="n">
-        <v>-1.75</v>
-      </c>
-      <c r="I52" s="29" t="n">
-        <v>-3.09</v>
+        <v>-8.550000000000001</v>
+      </c>
+      <c r="I52" s="27" t="n">
+        <v>2.48</v>
       </c>
       <c r="J52" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +1323%</t>
+          <t>네이버 검색 당일 +1394%</t>
         </is>
       </c>
       <c r="K52" s="28" t="inlineStr">
@@ -2581,7 +2571,7 @@
     <row r="53" ht="18" customHeight="1">
       <c r="A53" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B53" s="25" t="n">
@@ -2589,7 +2579,7 @@
       </c>
       <c r="C53" s="26" t="inlineStr">
         <is>
-          <t>빅웨이브로보틱스</t>
+          <t>덕산넵코어스</t>
         </is>
       </c>
       <c r="D53" s="25" t="n">
@@ -2604,15 +2594,15 @@
       <c r="G53" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H53" s="27" t="n">
-        <v>2.75</v>
-      </c>
-      <c r="I53" s="27" t="n">
-        <v>17.38</v>
+      <c r="H53" s="29" t="n">
+        <v>-1.75</v>
+      </c>
+      <c r="I53" s="29" t="n">
+        <v>-3.09</v>
       </c>
       <c r="J53" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +1263%</t>
+          <t>네이버 검색 당일 +1344%</t>
         </is>
       </c>
       <c r="K53" s="28" t="inlineStr">
@@ -2624,7 +2614,7 @@
     <row r="54" ht="18" customHeight="1">
       <c r="A54" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B54" s="25" t="n">
@@ -2632,7 +2622,7 @@
       </c>
       <c r="C54" s="26" t="inlineStr">
         <is>
-          <t>덕우전자</t>
+          <t>빅웨이브로보틱스</t>
         </is>
       </c>
       <c r="D54" s="25" t="n">
@@ -2648,14 +2638,14 @@
         <v>0</v>
       </c>
       <c r="H54" s="27" t="n">
-        <v>17.91</v>
+        <v>2.75</v>
       </c>
       <c r="I54" s="27" t="n">
-        <v>53.62</v>
+        <v>17.38</v>
       </c>
       <c r="J54" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +1066%</t>
+          <t>네이버 검색 당일 +1278%</t>
         </is>
       </c>
       <c r="K54" s="28" t="inlineStr">
@@ -2667,7 +2657,7 @@
     <row r="55" ht="18" customHeight="1">
       <c r="A55" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B55" s="25" t="n">
@@ -2675,7 +2665,7 @@
       </c>
       <c r="C55" s="26" t="inlineStr">
         <is>
-          <t>부산주공</t>
+          <t>덕우전자</t>
         </is>
       </c>
       <c r="D55" s="25" t="n">
@@ -2690,15 +2680,15 @@
       <c r="G55" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H55" s="29" t="n">
-        <v>-32.5</v>
-      </c>
-      <c r="I55" s="29" t="n">
-        <v>-94.44</v>
+      <c r="H55" s="27" t="n">
+        <v>17.91</v>
+      </c>
+      <c r="I55" s="27" t="n">
+        <v>53.62</v>
       </c>
       <c r="J55" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +769%</t>
+          <t>네이버 검색 당일 +1134%</t>
         </is>
       </c>
       <c r="K55" s="28" t="inlineStr">
@@ -2710,7 +2700,7 @@
     <row r="56" ht="18" customHeight="1">
       <c r="A56" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B56" s="25" t="n">
@@ -2718,7 +2708,7 @@
       </c>
       <c r="C56" s="26" t="inlineStr">
         <is>
-          <t>원일티엔아이</t>
+          <t>부산주공</t>
         </is>
       </c>
       <c r="D56" s="25" t="n">
@@ -2733,15 +2723,15 @@
       <c r="G56" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H56" s="27" t="n">
-        <v>18.34</v>
-      </c>
-      <c r="I56" s="27" t="n">
-        <v>54.33</v>
+      <c r="H56" s="29" t="n">
+        <v>-32.5</v>
+      </c>
+      <c r="I56" s="29" t="n">
+        <v>-94.44</v>
       </c>
       <c r="J56" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +645%</t>
+          <t>네이버 검색 당일 +804%</t>
         </is>
       </c>
       <c r="K56" s="28" t="inlineStr">
@@ -2753,7 +2743,7 @@
     <row r="57" ht="18" customHeight="1">
       <c r="A57" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B57" s="25" t="n">
@@ -2761,7 +2751,7 @@
       </c>
       <c r="C57" s="26" t="inlineStr">
         <is>
-          <t>KBI동양철관</t>
+          <t>원일티엔아이</t>
         </is>
       </c>
       <c r="D57" s="25" t="n">
@@ -2776,15 +2766,15 @@
       <c r="G57" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H57" s="29" t="n">
-        <v>-4.36</v>
+      <c r="H57" s="27" t="n">
+        <v>18.34</v>
       </c>
       <c r="I57" s="27" t="n">
-        <v>16.03</v>
+        <v>54.33</v>
       </c>
       <c r="J57" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +547%</t>
+          <t>네이버 검색 당일 +679%</t>
         </is>
       </c>
       <c r="K57" s="28" t="inlineStr">
@@ -2796,7 +2786,7 @@
     <row r="58" ht="18" customHeight="1">
       <c r="A58" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B58" s="25" t="n">
@@ -2804,7 +2794,7 @@
       </c>
       <c r="C58" s="26" t="inlineStr">
         <is>
-          <t>윈팩</t>
+          <t>KBI동양철관</t>
         </is>
       </c>
       <c r="D58" s="25" t="n">
@@ -2819,15 +2809,15 @@
       <c r="G58" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H58" s="27" t="n">
-        <v>4.95</v>
+      <c r="H58" s="29" t="n">
+        <v>-4.36</v>
       </c>
       <c r="I58" s="27" t="n">
-        <v>72.38</v>
+        <v>16.03</v>
       </c>
       <c r="J58" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +472%</t>
+          <t>네이버 검색 당일 +567%</t>
         </is>
       </c>
       <c r="K58" s="28" t="inlineStr">
@@ -2839,7 +2829,7 @@
     <row r="59" ht="18" customHeight="1">
       <c r="A59" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B59" s="25" t="n">
@@ -2870,7 +2860,7 @@
       </c>
       <c r="J59" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +444%</t>
+          <t>네이버 검색 당일 +537%</t>
         </is>
       </c>
       <c r="K59" s="28" t="inlineStr">
@@ -2882,7 +2872,7 @@
     <row r="60" ht="18" customHeight="1">
       <c r="A60" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B60" s="25" t="n">
@@ -2890,7 +2880,7 @@
       </c>
       <c r="C60" s="26" t="inlineStr">
         <is>
-          <t>LK삼양</t>
+          <t>윈팩</t>
         </is>
       </c>
       <c r="D60" s="25" t="n">
@@ -2906,14 +2896,14 @@
         <v>0</v>
       </c>
       <c r="H60" s="27" t="n">
-        <v>18.37</v>
+        <v>4.95</v>
       </c>
       <c r="I60" s="27" t="n">
-        <v>18.08</v>
+        <v>72.38</v>
       </c>
       <c r="J60" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +406%</t>
+          <t>네이버 검색 당일 +488%</t>
         </is>
       </c>
       <c r="K60" s="28" t="inlineStr">
@@ -2925,7 +2915,7 @@
     <row r="61" ht="18" customHeight="1">
       <c r="A61" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B61" s="25" t="n">
@@ -2933,7 +2923,7 @@
       </c>
       <c r="C61" s="26" t="inlineStr">
         <is>
-          <t>한국비엔씨</t>
+          <t>LK삼양</t>
         </is>
       </c>
       <c r="D61" s="25" t="n">
@@ -2948,15 +2938,15 @@
       <c r="G61" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H61" s="29" t="n">
-        <v>-3.07</v>
-      </c>
-      <c r="I61" s="29" t="n">
-        <v>-7.74</v>
+      <c r="H61" s="27" t="n">
+        <v>18.37</v>
+      </c>
+      <c r="I61" s="27" t="n">
+        <v>18.08</v>
       </c>
       <c r="J61" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +339%</t>
+          <t>네이버 검색 당일 +419%</t>
         </is>
       </c>
       <c r="K61" s="28" t="inlineStr">
@@ -2968,7 +2958,7 @@
     <row r="62" ht="18" customHeight="1">
       <c r="A62" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B62" s="25" t="n">
@@ -2976,7 +2966,7 @@
       </c>
       <c r="C62" s="26" t="inlineStr">
         <is>
-          <t>에이프릴바이오</t>
+          <t>한국비엔씨</t>
         </is>
       </c>
       <c r="D62" s="25" t="n">
@@ -2992,14 +2982,14 @@
         <v>0</v>
       </c>
       <c r="H62" s="29" t="n">
-        <v>-21.12</v>
+        <v>-3.07</v>
       </c>
       <c r="I62" s="29" t="n">
-        <v>-9.390000000000001</v>
+        <v>-7.74</v>
       </c>
       <c r="J62" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +283%</t>
+          <t>네이버 검색 당일 +344%</t>
         </is>
       </c>
       <c r="K62" s="28" t="inlineStr">
@@ -3011,7 +3001,7 @@
     <row r="63" ht="18" customHeight="1">
       <c r="A63" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B63" s="25" t="n">
@@ -3019,7 +3009,7 @@
       </c>
       <c r="C63" s="26" t="inlineStr">
         <is>
-          <t>세미티에스</t>
+          <t>에이프릴바이오</t>
         </is>
       </c>
       <c r="D63" s="25" t="n">
@@ -3034,15 +3024,15 @@
       <c r="G63" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H63" s="27" t="n">
-        <v>2.06</v>
-      </c>
-      <c r="I63" s="27" t="n">
-        <v>27.22</v>
+      <c r="H63" s="29" t="n">
+        <v>-21.12</v>
+      </c>
+      <c r="I63" s="29" t="n">
+        <v>-9.390000000000001</v>
       </c>
       <c r="J63" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +222%</t>
+          <t>네이버 검색 당일 +299%</t>
         </is>
       </c>
       <c r="K63" s="28" t="inlineStr">
@@ -3144,22 +3134,22 @@
         <v>1</v>
       </c>
       <c r="C3" s="25" t="n">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="D3" s="25" t="n">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="E3" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F3" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="G3" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="H3" s="25" t="n"/>
@@ -3175,22 +3165,22 @@
         <v>1</v>
       </c>
       <c r="C4" s="25" t="n">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="D4" s="25" t="n">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="E4" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F4" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="G4" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="H4" s="27" t="n">
@@ -3210,22 +3200,22 @@
         <v>1</v>
       </c>
       <c r="C5" s="25" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D5" s="25" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E5" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F5" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="G5" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="H5" s="25" t="n"/>
@@ -3234,37 +3224,33 @@
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="26" t="inlineStr">
         <is>
-          <t>현대차</t>
+          <t>바이오</t>
         </is>
       </c>
       <c r="B6" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="25" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D6" s="25" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E6" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F6" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="G6" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
-      <c r="H6" s="29" t="n">
-        <v>-0.57</v>
-      </c>
-      <c r="I6" s="29" t="n">
-        <v>-1.98</v>
-      </c>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H6" s="25" t="n"/>
+      <c r="I6" s="25" t="n"/>
     </row>
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="26" t="inlineStr">
@@ -3276,22 +3262,22 @@
         <v>1</v>
       </c>
       <c r="C7" s="25" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D7" s="25" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E7" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F7" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="G7" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="H7" s="25" t="n"/>
@@ -3307,22 +3293,22 @@
         <v>1</v>
       </c>
       <c r="C8" s="25" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D8" s="25" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E8" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F8" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="G8" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="H8" s="25" t="n"/>
@@ -3331,130 +3317,126 @@
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="26" t="inlineStr">
         <is>
-          <t>바이오</t>
+          <t>현대차</t>
         </is>
       </c>
       <c r="B9" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="25" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D9" s="25" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="E9" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F9" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="G9" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
-      <c r="H9" s="25" t="n"/>
-      <c r="I9" s="25" t="n"/>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H9" s="29" t="n">
+        <v>-0.57</v>
+      </c>
+      <c r="I9" s="29" t="n">
+        <v>-1.98</v>
+      </c>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="26" t="inlineStr">
         <is>
-          <t>SK하이닉스</t>
+          <t>스테이블코인</t>
         </is>
       </c>
       <c r="B10" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C10" s="25" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D10" s="25" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E10" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F10" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="G10" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
-      <c r="H10" s="27" t="n">
-        <v>0.77</v>
-      </c>
-      <c r="I10" s="27" t="n">
-        <v>4.6</v>
-      </c>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H10" s="25" t="n"/>
+      <c r="I10" s="25" t="n"/>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="26" t="inlineStr">
         <is>
-          <t>삼성E&amp;A</t>
+          <t>원전</t>
         </is>
       </c>
       <c r="B11" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="25" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="D11" s="25" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="E11" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F11" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="G11" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
-      <c r="H11" s="27" t="n">
-        <v>0.84</v>
-      </c>
-      <c r="I11" s="29" t="n">
-        <v>-4.11</v>
-      </c>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H11" s="25" t="n"/>
+      <c r="I11" s="25" t="n"/>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="26" t="inlineStr">
         <is>
-          <t>스테이블코인</t>
+          <t>전기차</t>
         </is>
       </c>
       <c r="B12" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C12" s="25" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D12" s="25" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="E12" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F12" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="G12" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="H12" s="25" t="n"/>
@@ -3463,29 +3445,29 @@
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>원전</t>
+          <t>방산</t>
         </is>
       </c>
       <c r="B13" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C13" s="25" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D13" s="25" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E13" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F13" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="G13" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="H13" s="25" t="n"/>
@@ -3494,77 +3476,77 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>SG</t>
+          <t>대한항공</t>
         </is>
       </c>
       <c r="B14" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C14" s="25" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D14" s="25" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E14" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F14" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="G14" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="H14" s="29" t="n">
-        <v>-5.15</v>
+        <v>-0.64</v>
       </c>
       <c r="I14" s="29" t="n">
-        <v>-2.64</v>
+        <v>-1.91</v>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>대한항공</t>
+          <t>한화솔루션</t>
         </is>
       </c>
       <c r="B15" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C15" s="25" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D15" s="25" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E15" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F15" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="G15" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
-      <c r="H15" s="29" t="n">
-        <v>-0.64</v>
-      </c>
-      <c r="I15" s="29" t="n">
-        <v>-1.91</v>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H15" s="27" t="n">
+        <v>5.71</v>
+      </c>
+      <c r="I15" s="27" t="n">
+        <v>5.4</v>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>루닛</t>
+          <t>AI반도체</t>
         </is>
       </c>
       <c r="B16" s="25" t="n">
@@ -3581,25 +3563,21 @@
       </c>
       <c r="F16" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="G16" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
-      <c r="H16" s="29" t="n">
-        <v>-5.03</v>
-      </c>
-      <c r="I16" s="29" t="n">
-        <v>-5.88</v>
-      </c>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H16" s="25" t="n"/>
+      <c r="I16" s="25" t="n"/>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>모아데이타</t>
+          <t>LG전자</t>
         </is>
       </c>
       <c r="B17" s="25" t="n">
@@ -3616,25 +3594,25 @@
       </c>
       <c r="F17" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="G17" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
-      <c r="H17" s="29" t="n">
-        <v>-3.6</v>
-      </c>
-      <c r="I17" s="29" t="n">
-        <v>-1.83</v>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H17" s="27" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="I17" s="27" t="n">
+        <v>0.47</v>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="26" t="inlineStr">
         <is>
-          <t>삼성중공업</t>
+          <t>더코디</t>
         </is>
       </c>
       <c r="B18" s="25" t="n">
@@ -3651,25 +3629,25 @@
       </c>
       <c r="F18" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="G18" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
-      <c r="H18" s="27" t="n">
-        <v>0.91</v>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H18" s="29" t="n">
+        <v>-1.27</v>
       </c>
       <c r="I18" s="29" t="n">
-        <v>-1.14</v>
+        <v>-20.87</v>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>세미파이브</t>
+          <t>삼성전자우</t>
         </is>
       </c>
       <c r="B19" s="25" t="n">
@@ -3686,25 +3664,25 @@
       </c>
       <c r="F19" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="G19" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
-      <c r="H19" s="27" t="n">
-        <v>1.72</v>
-      </c>
-      <c r="I19" s="27" t="n">
-        <v>28.88</v>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H19" s="29" t="n">
+        <v>-0.25</v>
+      </c>
+      <c r="I19" s="29" t="n">
+        <v>-1.95</v>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="26" t="inlineStr">
         <is>
-          <t>전기차</t>
+          <t>케이뱅크</t>
         </is>
       </c>
       <c r="B20" s="25" t="n">
@@ -3721,16 +3699,20 @@
       </c>
       <c r="F20" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="G20" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
-      <c r="H20" s="25" t="n"/>
-      <c r="I20" s="25" t="n"/>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H20" s="29" t="n">
+        <v>-0.19</v>
+      </c>
+      <c r="I20" s="29" t="n">
+        <v>-1.82</v>
+      </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="26" t="inlineStr">
@@ -3752,12 +3734,12 @@
       </c>
       <c r="F21" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="G21" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="H21" s="27" t="n">
@@ -3770,7 +3752,7 @@
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="26" t="inlineStr">
         <is>
-          <t>더코디</t>
+          <t>SG</t>
         </is>
       </c>
       <c r="B22" s="25" t="n">
@@ -3787,25 +3769,25 @@
       </c>
       <c r="F22" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="G22" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="H22" s="29" t="n">
-        <v>-1.27</v>
+        <v>-5.15</v>
       </c>
       <c r="I22" s="29" t="n">
-        <v>-20.87</v>
+        <v>-2.64</v>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="26" t="inlineStr">
         <is>
-          <t>머큐리</t>
+          <t>SK하이닉스</t>
         </is>
       </c>
       <c r="B23" s="25" t="n">
@@ -3822,25 +3804,25 @@
       </c>
       <c r="F23" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="G23" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="H23" s="27" t="n">
-        <v>29.8</v>
+        <v>0.77</v>
       </c>
       <c r="I23" s="27" t="n">
-        <v>28.21</v>
+        <v>4.6</v>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="26" t="inlineStr">
         <is>
-          <t>팬오션</t>
+          <t>삼성바이오로직스</t>
         </is>
       </c>
       <c r="B24" s="25" t="n">
@@ -3857,25 +3839,25 @@
       </c>
       <c r="F24" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="G24" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
-      <c r="H24" s="27" t="n">
-        <v>6.47</v>
-      </c>
-      <c r="I24" s="27" t="n">
-        <v>9.84</v>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H24" s="29" t="n">
+        <v>-3.6</v>
+      </c>
+      <c r="I24" s="29" t="n">
+        <v>-0.96</v>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="26" t="inlineStr">
         <is>
-          <t>게임</t>
+          <t>고영</t>
         </is>
       </c>
       <c r="B25" s="25" t="n">
@@ -3892,21 +3874,25 @@
       </c>
       <c r="F25" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="G25" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
-      <c r="H25" s="25" t="n"/>
-      <c r="I25" s="25" t="n"/>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H25" s="27" t="n">
+        <v>1.47</v>
+      </c>
+      <c r="I25" s="27" t="n">
+        <v>19.41</v>
+      </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="26" t="inlineStr">
         <is>
-          <t>고영</t>
+          <t>나인테크</t>
         </is>
       </c>
       <c r="B26" s="25" t="n">
@@ -3923,25 +3909,25 @@
       </c>
       <c r="F26" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="G26" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="H26" s="27" t="n">
-        <v>1.47</v>
+        <v>0.71</v>
       </c>
       <c r="I26" s="27" t="n">
-        <v>19.41</v>
+        <v>28.05</v>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="26" t="inlineStr">
         <is>
-          <t>나인테크</t>
+          <t>네이버</t>
         </is>
       </c>
       <c r="B27" s="25" t="n">
@@ -3958,25 +3944,21 @@
       </c>
       <c r="F27" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="G27" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
-      <c r="H27" s="27" t="n">
-        <v>0.71</v>
-      </c>
-      <c r="I27" s="27" t="n">
-        <v>28.05</v>
-      </c>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H27" s="25" t="n"/>
+      <c r="I27" s="25" t="n"/>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="26" t="inlineStr">
         <is>
-          <t>미래산업</t>
+          <t>삼성E&amp;A</t>
         </is>
       </c>
       <c r="B28" s="25" t="n">
@@ -3993,25 +3975,25 @@
       </c>
       <c r="F28" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="G28" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="H28" s="27" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="I28" s="27" t="n">
-        <v>16.62</v>
+        <v>0.84</v>
+      </c>
+      <c r="I28" s="29" t="n">
+        <v>-4.11</v>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="26" t="inlineStr">
         <is>
-          <t>선도전기</t>
+          <t>삼성중공업</t>
         </is>
       </c>
       <c r="B29" s="25" t="n">
@@ -4028,25 +4010,25 @@
       </c>
       <c r="F29" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="G29" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
-      <c r="H29" s="29" t="n">
-        <v>-1.82</v>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H29" s="27" t="n">
+        <v>0.91</v>
       </c>
       <c r="I29" s="29" t="n">
-        <v>-1.82</v>
+        <v>-1.14</v>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="26" t="inlineStr">
         <is>
-          <t>아리바이오홀딩스</t>
+          <t>선도전기</t>
         </is>
       </c>
       <c r="B30" s="25" t="n">
@@ -4063,25 +4045,25 @@
       </c>
       <c r="F30" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="G30" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="H30" s="29" t="n">
-        <v>-2.23</v>
+        <v>-1.82</v>
       </c>
       <c r="I30" s="29" t="n">
-        <v>-22.96</v>
+        <v>-1.82</v>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="26" t="inlineStr">
         <is>
-          <t>에이에프더블류</t>
+          <t>세미파이브</t>
         </is>
       </c>
       <c r="B31" s="25" t="n">
@@ -4098,25 +4080,25 @@
       </c>
       <c r="F31" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="G31" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
-      <c r="H31" s="29" t="n">
-        <v>-5.13</v>
-      </c>
-      <c r="I31" s="29" t="n">
-        <v>-51.32</v>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H31" s="27" t="n">
+        <v>1.72</v>
+      </c>
+      <c r="I31" s="27" t="n">
+        <v>28.88</v>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="26" t="inlineStr">
         <is>
-          <t>퀀텀레일</t>
+          <t>아리바이오홀딩스</t>
         </is>
       </c>
       <c r="B32" s="25" t="n">
@@ -4133,25 +4115,25 @@
       </c>
       <c r="F32" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="G32" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="H32" s="29" t="n">
-        <v>-1.63</v>
+        <v>-2.23</v>
       </c>
       <c r="I32" s="29" t="n">
-        <v>-51.68</v>
+        <v>-22.96</v>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="26" t="inlineStr">
         <is>
-          <t>한국파마</t>
+          <t>에이에프더블류</t>
         </is>
       </c>
       <c r="B33" s="25" t="n">
@@ -4168,25 +4150,25 @@
       </c>
       <c r="F33" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="G33" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
-      <c r="H33" s="27" t="n">
-        <v>13.42</v>
-      </c>
-      <c r="I33" s="27" t="n">
-        <v>19.06</v>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H33" s="29" t="n">
+        <v>-5.13</v>
+      </c>
+      <c r="I33" s="29" t="n">
+        <v>-51.32</v>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="26" t="inlineStr">
         <is>
-          <t>한창</t>
+          <t>오텍</t>
         </is>
       </c>
       <c r="B34" s="25" t="n">
@@ -4203,25 +4185,25 @@
       </c>
       <c r="F34" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="G34" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
-      <c r="H34" s="29" t="n">
-        <v>-91.06999999999999</v>
-      </c>
-      <c r="I34" s="29" t="n">
-        <v>-91.06999999999999</v>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H34" s="27" t="n">
+        <v>8.32</v>
+      </c>
+      <c r="I34" s="27" t="n">
+        <v>13.69</v>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="26" t="inlineStr">
         <is>
-          <t>한화솔루션</t>
+          <t>퀀텀레일</t>
         </is>
       </c>
       <c r="B35" s="25" t="n">
@@ -4238,25 +4220,25 @@
       </c>
       <c r="F35" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="G35" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
-      <c r="H35" s="27" t="n">
-        <v>5.71</v>
-      </c>
-      <c r="I35" s="27" t="n">
-        <v>5.4</v>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H35" s="29" t="n">
+        <v>-1.63</v>
+      </c>
+      <c r="I35" s="29" t="n">
+        <v>-51.68</v>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="26" t="inlineStr">
         <is>
-          <t>한화오션</t>
+          <t>티엠씨</t>
         </is>
       </c>
       <c r="B36" s="25" t="n">
@@ -4273,60 +4255,60 @@
       </c>
       <c r="F36" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="G36" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="H36" s="27" t="n">
-        <v>0.13</v>
-      </c>
-      <c r="I36" s="29" t="n">
-        <v>-2.24</v>
+        <v>29.68</v>
+      </c>
+      <c r="I36" s="27" t="n">
+        <v>33.33</v>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="26" t="inlineStr">
         <is>
-          <t>KBI동양철관</t>
+          <t>한국파마</t>
         </is>
       </c>
       <c r="B37" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C37" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D37" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E37" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F37" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="G37" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
-      <c r="H37" s="29" t="n">
-        <v>-4.36</v>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H37" s="27" t="n">
+        <v>13.42</v>
       </c>
       <c r="I37" s="27" t="n">
-        <v>16.03</v>
+        <v>19.06</v>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="26" t="inlineStr">
         <is>
-          <t>LK삼양</t>
+          <t>KBI동양철관</t>
         </is>
       </c>
       <c r="B38" s="25" t="n">
@@ -4343,25 +4325,25 @@
       </c>
       <c r="F38" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="G38" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
-      <c r="H38" s="27" t="n">
-        <v>18.37</v>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H38" s="29" t="n">
+        <v>-4.36</v>
       </c>
       <c r="I38" s="27" t="n">
-        <v>18.08</v>
+        <v>16.03</v>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="26" t="inlineStr">
         <is>
-          <t>글로벌테크놀로지</t>
+          <t>LK삼양</t>
         </is>
       </c>
       <c r="B39" s="25" t="n">
@@ -4378,25 +4360,25 @@
       </c>
       <c r="F39" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="G39" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
-      <c r="H39" s="29" t="n">
-        <v>-8.550000000000001</v>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H39" s="27" t="n">
+        <v>18.37</v>
       </c>
       <c r="I39" s="27" t="n">
-        <v>2.48</v>
+        <v>18.08</v>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="26" t="inlineStr">
         <is>
-          <t>덕산넵코어스</t>
+          <t>글로벌테크놀로지</t>
         </is>
       </c>
       <c r="B40" s="25" t="n">
@@ -4413,25 +4395,25 @@
       </c>
       <c r="F40" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="G40" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="H40" s="29" t="n">
-        <v>-1.75</v>
-      </c>
-      <c r="I40" s="29" t="n">
-        <v>-3.09</v>
+        <v>-8.550000000000001</v>
+      </c>
+      <c r="I40" s="27" t="n">
+        <v>2.48</v>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="26" t="inlineStr">
         <is>
-          <t>덕우전자</t>
+          <t>덕산넵코어스</t>
         </is>
       </c>
       <c r="B41" s="25" t="n">
@@ -4448,25 +4430,25 @@
       </c>
       <c r="F41" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="G41" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
-      <c r="H41" s="27" t="n">
-        <v>17.91</v>
-      </c>
-      <c r="I41" s="27" t="n">
-        <v>53.62</v>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H41" s="29" t="n">
+        <v>-1.75</v>
+      </c>
+      <c r="I41" s="29" t="n">
+        <v>-3.09</v>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="26" t="inlineStr">
         <is>
-          <t>부산주공</t>
+          <t>덕우전자</t>
         </is>
       </c>
       <c r="B42" s="25" t="n">
@@ -4483,25 +4465,25 @@
       </c>
       <c r="F42" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="G42" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
-      <c r="H42" s="29" t="n">
-        <v>-32.5</v>
-      </c>
-      <c r="I42" s="29" t="n">
-        <v>-94.44</v>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H42" s="27" t="n">
+        <v>17.91</v>
+      </c>
+      <c r="I42" s="27" t="n">
+        <v>53.62</v>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="26" t="inlineStr">
         <is>
-          <t>브릴스</t>
+          <t>부산주공</t>
         </is>
       </c>
       <c r="B43" s="25" t="n">
@@ -4518,25 +4500,25 @@
       </c>
       <c r="F43" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="G43" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
-      <c r="H43" s="27" t="n">
-        <v>9.81</v>
-      </c>
-      <c r="I43" s="27" t="n">
-        <v>9.81</v>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H43" s="29" t="n">
+        <v>-32.5</v>
+      </c>
+      <c r="I43" s="29" t="n">
+        <v>-94.44</v>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="26" t="inlineStr">
         <is>
-          <t>빅웨이브로보틱스</t>
+          <t>브릴스</t>
         </is>
       </c>
       <c r="B44" s="25" t="n">
@@ -4553,25 +4535,25 @@
       </c>
       <c r="F44" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="G44" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="H44" s="27" t="n">
-        <v>2.75</v>
+        <v>9.81</v>
       </c>
       <c r="I44" s="27" t="n">
-        <v>17.38</v>
+        <v>9.81</v>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="26" t="inlineStr">
         <is>
-          <t>세미티에스</t>
+          <t>빅웨이브로보틱스</t>
         </is>
       </c>
       <c r="B45" s="25" t="n">
@@ -4588,19 +4570,19 @@
       </c>
       <c r="F45" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="G45" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="H45" s="27" t="n">
-        <v>2.06</v>
+        <v>2.75</v>
       </c>
       <c r="I45" s="27" t="n">
-        <v>27.22</v>
+        <v>17.38</v>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
@@ -4623,12 +4605,12 @@
       </c>
       <c r="F46" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="G46" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="H46" s="29" t="n">
@@ -4658,12 +4640,12 @@
       </c>
       <c r="F47" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="G47" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="H47" s="27" t="n">
@@ -4693,12 +4675,12 @@
       </c>
       <c r="F48" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="G48" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="H48" s="27" t="n">
@@ -4728,12 +4710,12 @@
       </c>
       <c r="F49" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="G49" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="H49" s="29" t="n">
@@ -4763,12 +4745,12 @@
       </c>
       <c r="F50" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="G50" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="H50" s="27" t="n">
@@ -4798,12 +4780,12 @@
       </c>
       <c r="F51" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="G51" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="H51" s="29" t="n">
@@ -4833,12 +4815,12 @@
       </c>
       <c r="F52" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="G52" s="25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="H52" s="29" t="n">
@@ -4929,19 +4911,19 @@
         <v>1</v>
       </c>
       <c r="C3" s="36" t="n">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="D3" s="36" t="n">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="E3" s="36" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="F3" s="37" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="G3" s="37" t="inlineStr">
@@ -4960,19 +4942,19 @@
         <v>1</v>
       </c>
       <c r="C4" s="36" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D4" s="36" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E4" s="36" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="F4" s="37" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="G4" s="37" t="inlineStr">
@@ -4984,7 +4966,7 @@
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="35" t="inlineStr">
         <is>
-          <t>전기차</t>
+          <t>AI반도체</t>
         </is>
       </c>
       <c r="B5" s="36" t="n">
@@ -4998,12 +4980,12 @@
       </c>
       <c r="E5" s="36" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="F5" s="37" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="G5" s="37" t="inlineStr">
@@ -5015,26 +4997,26 @@
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="35" t="inlineStr">
         <is>
-          <t>원전</t>
+          <t>전기차</t>
         </is>
       </c>
       <c r="B6" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="36" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D6" s="36" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="E6" s="36" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="F6" s="37" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="G6" s="37" t="inlineStr">
@@ -5046,26 +5028,26 @@
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="35" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>방산</t>
         </is>
       </c>
       <c r="B7" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="36" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D7" s="36" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E7" s="36" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="F7" s="37" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="G7" s="37" t="inlineStr">
@@ -5077,26 +5059,26 @@
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="35" t="inlineStr">
         <is>
-          <t>게임</t>
+          <t>원전</t>
         </is>
       </c>
       <c r="B8" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="36" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="D8" s="36" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="E8" s="36" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="F8" s="37" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="G8" s="37" t="inlineStr">
@@ -5108,26 +5090,26 @@
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="35" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="B9" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="36" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D9" s="36" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E9" s="36" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="F9" s="37" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="G9" s="37" t="inlineStr">
@@ -5139,65 +5121,69 @@
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="35" t="inlineStr">
         <is>
+          <t>제약</t>
+        </is>
+      </c>
+      <c r="B10" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" s="36" t="n">
+        <v>14</v>
+      </c>
+      <c r="D10" s="36" t="n">
+        <v>14</v>
+      </c>
+      <c r="E10" s="36" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="F10" s="37" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="G10" s="37" t="inlineStr">
+        <is>
+          <t>⚡ 관심</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="35" t="inlineStr">
+        <is>
           <t>인공지능</t>
         </is>
       </c>
-      <c r="B10" s="36" t="n">
-        <v>1</v>
-      </c>
-      <c r="C10" s="36" t="n">
-        <v>24</v>
-      </c>
-      <c r="D10" s="36" t="n">
-        <v>24</v>
-      </c>
-      <c r="E10" s="36" t="inlineStr">
-        <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
-      <c r="F10" s="37" t="inlineStr">
-        <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
-      <c r="G10" s="37" t="inlineStr">
+      <c r="B11" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" s="36" t="n">
+        <v>22</v>
+      </c>
+      <c r="D11" s="36" t="n">
+        <v>22</v>
+      </c>
+      <c r="E11" s="36" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="F11" s="37" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="G11" s="37" t="inlineStr">
         <is>
           <t>⚡ 관심</t>
         </is>
       </c>
-    </row>
-    <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="26" t="inlineStr">
-        <is>
-          <t>이차전지</t>
-        </is>
-      </c>
-      <c r="B11" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="C11" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="D11" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" s="25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F11" s="28" t="inlineStr">
-        <is>
-          <t>감지 없음</t>
-        </is>
-      </c>
-      <c r="G11" s="28" t="inlineStr"/>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="26" t="inlineStr">
         <is>
-          <t>AI반도체</t>
+          <t>이차전지</t>
         </is>
       </c>
       <c r="B12" s="25" t="n">
@@ -5224,7 +5210,7 @@
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>방산</t>
+          <t>수소</t>
         </is>
       </c>
       <c r="B13" s="25" t="n">
@@ -5251,7 +5237,7 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>수소</t>
+          <t>태양광</t>
         </is>
       </c>
       <c r="B14" s="25" t="n">
@@ -5278,7 +5264,7 @@
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>태양광</t>
+          <t>게임</t>
         </is>
       </c>
       <c r="B15" s="25" t="n">

</xml_diff>

<commit_message>
auto: 2026-10-10 07:04 자동 백업
</commit_message>
<xml_diff>
--- a/trend/stock_trend_history.xlsx
+++ b/trend/stock_trend_history.xlsx
@@ -258,14 +258,14 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -694,7 +694,7 @@
     <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-10-09 06:54</t>
+          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-10-10 06:54</t>
         </is>
       </c>
     </row>
@@ -787,21 +787,21 @@
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-10-09) 상위: 반도체  점수 63.0점</t>
+          <t>⚡ 최신(2026-10-10) 상위: 반도체  점수 88.0점</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-10-09) 상위: 삼성전자  점수 37.0점</t>
+          <t>⚡ 최신(2026-10-10) 상위: 인공지능  점수 28.0점</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-10-09) 상위: LG  점수 32.0점</t>
+          <t>⚡ 최신(2026-10-10) 상위: 삼성전자  점수 23.0점</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="15" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B14" s="15" t="n">
@@ -928,10 +928,10 @@
         </is>
       </c>
       <c r="D14" s="15" t="n">
-        <v>63</v>
+        <v>88</v>
       </c>
       <c r="E14" s="15" t="n">
-        <v>63</v>
+        <v>88</v>
       </c>
       <c r="F14" s="15" t="n">
         <v>0</v>
@@ -947,7 +947,7 @@
       </c>
       <c r="J14" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급</t>
         </is>
       </c>
       <c r="K14" s="17" t="inlineStr">
@@ -959,7 +959,7 @@
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="15" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B15" s="15" t="n">
@@ -967,14 +967,14 @@
       </c>
       <c r="C15" s="16" t="inlineStr">
         <is>
-          <t>삼성전자</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="D15" s="15" t="n">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="E15" s="15" t="n">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="F15" s="15" t="n">
         <v>0</v>
@@ -982,27 +982,27 @@
       <c r="G15" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H15" s="18" t="n">
-        <v>-2.23</v>
-      </c>
-      <c r="I15" s="18" t="n">
-        <v>-2.41</v>
+      <c r="H15" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I15" s="15" t="n">
+        <v/>
       </c>
       <c r="J15" s="17" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K15" s="17" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="15" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B16" s="15" t="n">
@@ -1010,14 +1010,14 @@
       </c>
       <c r="C16" s="16" t="inlineStr">
         <is>
-          <t>LG</t>
+          <t>삼성전자</t>
         </is>
       </c>
       <c r="D16" s="15" t="n">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="E16" s="15" t="n">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="F16" s="15" t="n">
         <v>0</v>
@@ -1026,26 +1026,26 @@
         <v>0</v>
       </c>
       <c r="H16" s="18" t="n">
-        <v>-1.9</v>
+        <v>-2.23</v>
       </c>
       <c r="I16" s="18" t="n">
-        <v>-2.17</v>
+        <v>-2.41</v>
       </c>
       <c r="J16" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>중요공시 1건 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K16" s="17" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B17" s="15" t="n">
@@ -1053,14 +1053,14 @@
       </c>
       <c r="C17" s="16" t="inlineStr">
         <is>
-          <t>전기차</t>
+          <t>LG</t>
         </is>
       </c>
       <c r="D17" s="15" t="n">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="E17" s="15" t="n">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="F17" s="15" t="n">
         <v>0</v>
@@ -1068,27 +1068,25 @@
       <c r="G17" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H17" s="15" t="n">
+      <c r="H17" s="18" t="n">
+        <v>-1.9</v>
+      </c>
+      <c r="I17" s="18" t="n">
+        <v>-2.17</v>
+      </c>
+      <c r="J17" s="17" t="inlineStr">
+        <is>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K17" s="17" t="n">
         <v/>
-      </c>
-      <c r="I17" s="15" t="n">
-        <v/>
-      </c>
-      <c r="J17" s="17" t="inlineStr">
-        <is>
-          <t>매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K17" s="17" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B18" s="15" t="n">
@@ -1096,14 +1094,14 @@
       </c>
       <c r="C18" s="16" t="inlineStr">
         <is>
-          <t>LG전자</t>
+          <t>전기차</t>
         </is>
       </c>
       <c r="D18" s="15" t="n">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="E18" s="15" t="n">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="F18" s="15" t="n">
         <v>0</v>
@@ -1111,27 +1109,25 @@
       <c r="G18" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H18" s="18" t="n">
-        <v>-3.83</v>
-      </c>
-      <c r="I18" s="18" t="n">
-        <v>-5.85</v>
+      <c r="H18" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I18" s="15" t="n">
+        <v/>
       </c>
       <c r="J18" s="17" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K18" s="17" t="inlineStr">
-        <is>
-          <t>네이버, 공시</t>
-        </is>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K18" s="17" t="n">
+        <v/>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B19" s="15" t="n">
@@ -1139,14 +1135,14 @@
       </c>
       <c r="C19" s="16" t="inlineStr">
         <is>
-          <t>인공지능</t>
+          <t>바이오</t>
         </is>
       </c>
       <c r="D19" s="15" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="E19" s="15" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="F19" s="15" t="n">
         <v>0</v>
@@ -1162,7 +1158,7 @@
       </c>
       <c r="J19" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K19" s="17" t="inlineStr">
@@ -1174,7 +1170,7 @@
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B20" s="15" t="n">
@@ -1182,14 +1178,14 @@
       </c>
       <c r="C20" s="16" t="inlineStr">
         <is>
-          <t>SK하이닉스</t>
+          <t>LG전자</t>
         </is>
       </c>
       <c r="D20" s="15" t="n">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="E20" s="15" t="n">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="F20" s="15" t="n">
         <v>0</v>
@@ -1198,26 +1194,26 @@
         <v>0</v>
       </c>
       <c r="H20" s="18" t="n">
-        <v>-1.69</v>
+        <v>-3.83</v>
       </c>
       <c r="I20" s="18" t="n">
-        <v>-5.44</v>
+        <v>-5.85</v>
       </c>
       <c r="J20" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
+          <t>중요공시 1건 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K20" s="17" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="15" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B21" s="15" t="n">
@@ -1225,14 +1221,14 @@
       </c>
       <c r="C21" s="16" t="inlineStr">
         <is>
-          <t>바이오</t>
+          <t>현대차</t>
         </is>
       </c>
       <c r="D21" s="15" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E21" s="15" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F21" s="15" t="n">
         <v>0</v>
@@ -1240,27 +1236,25 @@
       <c r="G21" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H21" s="15" t="n">
+      <c r="H21" s="18" t="n">
+        <v>-3.57</v>
+      </c>
+      <c r="I21" s="18" t="n">
+        <v>-6.48</v>
+      </c>
+      <c r="J21" s="17" t="inlineStr">
+        <is>
+          <t>한국경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K21" s="17" t="n">
         <v/>
-      </c>
-      <c r="I21" s="15" t="n">
-        <v/>
-      </c>
-      <c r="J21" s="17" t="inlineStr">
-        <is>
-          <t>네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 기사 언급</t>
-        </is>
-      </c>
-      <c r="K21" s="17" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="15" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B22" s="15" t="n">
@@ -1268,7 +1262,7 @@
       </c>
       <c r="C22" s="16" t="inlineStr">
         <is>
-          <t>펩트론</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="D22" s="15" t="n">
@@ -1283,25 +1277,27 @@
       <c r="G22" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H22" s="18" t="n">
-        <v>-5.57</v>
-      </c>
-      <c r="I22" s="18" t="n">
-        <v>-30.52</v>
+      <c r="H22" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I22" s="15" t="n">
+        <v/>
       </c>
       <c r="J22" s="17" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K22" s="17" t="n">
-        <v/>
+          <t>Google 급상승 검색어 등장 (KR) / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K22" s="17" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="15" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B23" s="15" t="n">
@@ -1309,14 +1305,14 @@
       </c>
       <c r="C23" s="16" t="inlineStr">
         <is>
-          <t>HD현대</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="D23" s="15" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E23" s="15" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F23" s="15" t="n">
         <v>0</v>
@@ -1324,27 +1320,27 @@
       <c r="G23" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H23" s="18" t="n">
-        <v>-4.08</v>
-      </c>
-      <c r="I23" s="18" t="n">
-        <v>-11.15</v>
+      <c r="H23" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I23" s="15" t="n">
+        <v/>
       </c>
       <c r="J23" s="17" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K23" s="17" t="inlineStr">
         <is>
-          <t>네이버, 공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="15" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B24" s="15" t="n">
@@ -1352,14 +1348,14 @@
       </c>
       <c r="C24" s="16" t="inlineStr">
         <is>
-          <t>현대차</t>
+          <t>SK하이닉스</t>
         </is>
       </c>
       <c r="D24" s="15" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E24" s="15" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F24" s="15" t="n">
         <v>0</v>
@@ -1368,24 +1364,26 @@
         <v>0</v>
       </c>
       <c r="H24" s="18" t="n">
-        <v>-3.57</v>
+        <v>-1.69</v>
       </c>
       <c r="I24" s="18" t="n">
-        <v>-6.48</v>
+        <v>-5.44</v>
       </c>
       <c r="J24" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K24" s="17" t="n">
-        <v/>
+          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K24" s="17" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="15" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B25" s="15" t="n">
@@ -1393,30 +1391,30 @@
       </c>
       <c r="C25" s="16" t="inlineStr">
         <is>
-          <t>더코디</t>
+          <t>한화오션</t>
         </is>
       </c>
       <c r="D25" s="15" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E25" s="15" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F25" s="15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G25" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="H25" s="19" t="n">
-        <v>7.28</v>
+      <c r="H25" s="18" t="n">
+        <v>-3.1</v>
       </c>
       <c r="I25" s="18" t="n">
-        <v>-22.45</v>
+        <v>-8.880000000000001</v>
       </c>
       <c r="J25" s="17" t="inlineStr">
         <is>
-          <t>중요공시 9건 / 중요공시 3일 +50% / 중요공시 7일 +200%</t>
+          <t>중요공시 4건 / 중요공시 7일 +100% / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K25" s="17" t="inlineStr">
@@ -1428,7 +1426,7 @@
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="15" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B26" s="15" t="n">
@@ -1436,7 +1434,7 @@
       </c>
       <c r="C26" s="16" t="inlineStr">
         <is>
-          <t>한화오션</t>
+          <t>스피어</t>
         </is>
       </c>
       <c r="D26" s="15" t="n">
@@ -1451,15 +1449,15 @@
       <c r="G26" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="H26" s="18" t="n">
-        <v>-3.1</v>
-      </c>
-      <c r="I26" s="18" t="n">
-        <v>-8.880000000000001</v>
+      <c r="H26" s="19" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="I26" s="19" t="n">
+        <v>15.72</v>
       </c>
       <c r="J26" s="17" t="inlineStr">
         <is>
-          <t>중요공시 4건 / 중요공시 3일 +100% / 중요공시 7일 +100%</t>
+          <t>중요공시 3건 / 중요공시 3일 +200% / 중요공시 7일 +50%</t>
         </is>
       </c>
       <c r="K26" s="17" t="inlineStr">
@@ -1471,7 +1469,7 @@
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="15" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B27" s="15" t="n">
@@ -1479,40 +1477,42 @@
       </c>
       <c r="C27" s="16" t="inlineStr">
         <is>
-          <t>TSMC</t>
+          <t>더코디</t>
         </is>
       </c>
       <c r="D27" s="15" t="n">
         <v>8</v>
       </c>
       <c r="E27" s="15" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="F27" s="15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G27" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H27" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I27" s="15" t="n">
-        <v/>
+        <v>3</v>
+      </c>
+      <c r="H27" s="19" t="n">
+        <v>7.28</v>
+      </c>
+      <c r="I27" s="18" t="n">
+        <v>-22.45</v>
       </c>
       <c r="J27" s="17" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K27" s="17" t="n">
-        <v/>
+          <t>중요공시 9건 / 중요공시 3일 +50% / 중요공시 7일 +80%</t>
+        </is>
+      </c>
+      <c r="K27" s="17" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="15" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B28" s="15" t="n">
@@ -1520,14 +1520,14 @@
       </c>
       <c r="C28" s="16" t="inlineStr">
         <is>
-          <t>주성엔지니어링</t>
+          <t>TSMC</t>
         </is>
       </c>
       <c r="D28" s="15" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E28" s="15" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F28" s="15" t="n">
         <v>0</v>
@@ -1535,27 +1535,25 @@
       <c r="G28" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H28" s="19" t="n">
-        <v>4.77</v>
-      </c>
-      <c r="I28" s="19" t="n">
-        <v>13.33</v>
+      <c r="H28" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I28" s="15" t="n">
+        <v/>
       </c>
       <c r="J28" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K28" s="17" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+          <t>한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K28" s="17" t="n">
+        <v/>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="20" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B29" s="20" t="n">
@@ -1563,7 +1561,7 @@
       </c>
       <c r="C29" s="21" t="inlineStr">
         <is>
-          <t>리노공업</t>
+          <t>삼표시멘트</t>
         </is>
       </c>
       <c r="D29" s="20" t="n">
@@ -1579,17 +1577,17 @@
         <v>0</v>
       </c>
       <c r="H29" s="22" t="n">
-        <v>3.17</v>
-      </c>
-      <c r="I29" s="22" t="n">
-        <v>19.13</v>
-      </c>
-      <c r="J29" s="23" t="inlineStr">
-        <is>
-          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K29" s="23" t="inlineStr">
+        <v>-12.77</v>
+      </c>
+      <c r="I29" s="23" t="n">
+        <v>5.24</v>
+      </c>
+      <c r="J29" s="24" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +155% / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K29" s="24" t="inlineStr">
         <is>
           <t>네이버</t>
         </is>
@@ -1598,7 +1596,7 @@
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="20" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B30" s="20" t="n">
@@ -1606,7 +1604,7 @@
       </c>
       <c r="C30" s="21" t="inlineStr">
         <is>
-          <t>알테오젠</t>
+          <t>주성엔지니어링</t>
         </is>
       </c>
       <c r="D30" s="20" t="n">
@@ -1621,27 +1619,25 @@
       <c r="G30" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H30" s="24" t="n">
-        <v>-5.5</v>
-      </c>
-      <c r="I30" s="24" t="n">
-        <v>-5.87</v>
-      </c>
-      <c r="J30" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 6건 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K30" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+      <c r="H30" s="23" t="n">
+        <v>4.77</v>
+      </c>
+      <c r="I30" s="23" t="n">
+        <v>13.33</v>
+      </c>
+      <c r="J30" s="24" t="inlineStr">
+        <is>
+          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K30" s="24" t="n">
+        <v/>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="20" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B31" s="20" t="n">
@@ -1649,7 +1645,7 @@
       </c>
       <c r="C31" s="21" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>삼성전기</t>
         </is>
       </c>
       <c r="D31" s="20" t="n">
@@ -1664,27 +1660,27 @@
       <c r="G31" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H31" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I31" s="20" t="n">
-        <v/>
-      </c>
-      <c r="J31" s="23" t="inlineStr">
-        <is>
-          <t>네이버뉴스 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K31" s="23" t="inlineStr">
-        <is>
-          <t>네이버</t>
+      <c r="H31" s="22" t="n">
+        <v>-2.99</v>
+      </c>
+      <c r="I31" s="23" t="n">
+        <v>2.97</v>
+      </c>
+      <c r="J31" s="24" t="inlineStr">
+        <is>
+          <t>중요공시 1건 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K31" s="24" t="inlineStr">
+        <is>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="20" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B32" s="20" t="n">
@@ -1692,14 +1688,14 @@
       </c>
       <c r="C32" s="21" t="inlineStr">
         <is>
-          <t>삼표시멘트</t>
+          <t>펩트론</t>
         </is>
       </c>
       <c r="D32" s="20" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E32" s="20" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F32" s="20" t="n">
         <v>0</v>
@@ -1707,27 +1703,25 @@
       <c r="G32" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H32" s="24" t="n">
-        <v>-12.77</v>
+      <c r="H32" s="22" t="n">
+        <v>-5.57</v>
       </c>
       <c r="I32" s="22" t="n">
-        <v>5.24</v>
-      </c>
-      <c r="J32" s="23" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +72% / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K32" s="23" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+        <v>-30.52</v>
+      </c>
+      <c r="J32" s="24" t="inlineStr">
+        <is>
+          <t>한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K32" s="24" t="n">
+        <v/>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="20" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B33" s="20" t="n">
@@ -1735,42 +1729,42 @@
       </c>
       <c r="C33" s="21" t="inlineStr">
         <is>
-          <t>스피어</t>
+          <t>GS</t>
         </is>
       </c>
       <c r="D33" s="20" t="n">
         <v>5</v>
       </c>
       <c r="E33" s="20" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F33" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G33" s="20" t="n">
         <v>0</v>
       </c>
       <c r="H33" s="22" t="n">
-        <v>0.2</v>
+        <v>-4.55</v>
       </c>
       <c r="I33" s="22" t="n">
-        <v>15.72</v>
-      </c>
-      <c r="J33" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 3건 / 중요공시 3일 +200%</t>
-        </is>
-      </c>
-      <c r="K33" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
+        <v>-1.69</v>
+      </c>
+      <c r="J33" s="24" t="inlineStr">
+        <is>
+          <t>Google 급상승 검색어 등장 (US)</t>
+        </is>
+      </c>
+      <c r="K33" s="24" t="inlineStr">
+        <is>
+          <t>Google</t>
         </is>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="20" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B34" s="20" t="n">
@@ -1778,14 +1772,14 @@
       </c>
       <c r="C34" s="21" t="inlineStr">
         <is>
-          <t>한미약품</t>
+          <t>국제약품</t>
         </is>
       </c>
       <c r="D34" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E34" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F34" s="20" t="n">
         <v>0</v>
@@ -1793,27 +1787,27 @@
       <c r="G34" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H34" s="24" t="n">
-        <v>-9.74</v>
-      </c>
-      <c r="I34" s="24" t="n">
-        <v>-3.31</v>
-      </c>
-      <c r="J34" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 1건 / 매일경제 기사 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K34" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
+      <c r="H34" s="22" t="n">
+        <v>-4.4</v>
+      </c>
+      <c r="I34" s="23" t="n">
+        <v>31.52</v>
+      </c>
+      <c r="J34" s="24" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +902% / 중요공시 2건</t>
+        </is>
+      </c>
+      <c r="K34" s="24" t="inlineStr">
+        <is>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="20" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B35" s="20" t="n">
@@ -1821,42 +1815,42 @@
       </c>
       <c r="C35" s="21" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>대양금속</t>
         </is>
       </c>
       <c r="D35" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E35" s="20" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F35" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G35" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H35" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I35" s="20" t="n">
-        <v/>
-      </c>
-      <c r="J35" s="23" t="inlineStr">
-        <is>
-          <t>네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K35" s="23" t="inlineStr">
-        <is>
-          <t>네이버</t>
+        <v>3</v>
+      </c>
+      <c r="H35" s="22" t="n">
+        <v>-6.73</v>
+      </c>
+      <c r="I35" s="22" t="n">
+        <v>-21.09</v>
+      </c>
+      <c r="J35" s="24" t="inlineStr">
+        <is>
+          <t>중요공시 2건 / 중요공시 7일 +100%</t>
+        </is>
+      </c>
+      <c r="K35" s="24" t="inlineStr">
+        <is>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="20" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B36" s="20" t="n">
@@ -1864,14 +1858,14 @@
       </c>
       <c r="C36" s="21" t="inlineStr">
         <is>
-          <t>삼성SDI</t>
+          <t>수소</t>
         </is>
       </c>
       <c r="D36" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E36" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F36" s="20" t="n">
         <v>0</v>
@@ -1879,27 +1873,25 @@
       <c r="G36" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H36" s="22" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="I36" s="22" t="n">
-        <v>10.53</v>
-      </c>
-      <c r="J36" s="23" t="inlineStr">
-        <is>
-          <t>네이버뉴스 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K36" s="23" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+      <c r="H36" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I36" s="20" t="n">
+        <v/>
+      </c>
+      <c r="J36" s="24" t="inlineStr">
+        <is>
+          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K36" s="24" t="n">
+        <v/>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="20" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B37" s="20" t="n">
@@ -1907,14 +1899,14 @@
       </c>
       <c r="C37" s="21" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>게임</t>
         </is>
       </c>
       <c r="D37" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E37" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F37" s="20" t="n">
         <v>0</v>
@@ -1928,316 +1920,322 @@
       <c r="I37" s="20" t="n">
         <v/>
       </c>
-      <c r="J37" s="23" t="inlineStr">
-        <is>
-          <t>매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K37" s="23" t="n">
-        <v/>
+      <c r="J37" s="24" t="inlineStr">
+        <is>
+          <t>매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K37" s="24" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
-      <c r="A38" s="20" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="B38" s="20" t="n">
+      <c r="A38" s="25" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B38" s="25" t="n">
         <v>25</v>
       </c>
-      <c r="C38" s="21" t="inlineStr">
-        <is>
-          <t>태양광</t>
-        </is>
-      </c>
-      <c r="D38" s="20" t="n">
-        <v>5</v>
-      </c>
-      <c r="E38" s="20" t="n">
-        <v>5</v>
-      </c>
-      <c r="F38" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G38" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H38" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I38" s="20" t="n">
-        <v/>
-      </c>
-      <c r="J38" s="23" t="inlineStr">
-        <is>
-          <t>네이버뉴스 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K38" s="23" t="inlineStr">
+      <c r="C38" s="26" t="inlineStr">
+        <is>
+          <t>빅텐츠</t>
+        </is>
+      </c>
+      <c r="D38" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E38" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F38" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G38" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H38" s="27" t="n">
+        <v>-18.27</v>
+      </c>
+      <c r="I38" s="27" t="n">
+        <v>-12.71</v>
+      </c>
+      <c r="J38" s="28" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +37760%</t>
+        </is>
+      </c>
+      <c r="K38" s="28" t="inlineStr">
         <is>
           <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
-      <c r="A39" s="20" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="B39" s="20" t="n">
+      <c r="A39" s="25" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B39" s="25" t="n">
         <v>26</v>
       </c>
-      <c r="C39" s="21" t="inlineStr">
-        <is>
-          <t>삼성생명</t>
-        </is>
-      </c>
-      <c r="D39" s="20" t="n">
-        <v>5</v>
-      </c>
-      <c r="E39" s="20" t="n">
-        <v>5</v>
-      </c>
-      <c r="F39" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G39" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H39" s="24" t="n">
-        <v>-3.05</v>
-      </c>
-      <c r="I39" s="24" t="n">
-        <v>-4.59</v>
-      </c>
-      <c r="J39" s="23" t="inlineStr">
-        <is>
-          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K39" s="23" t="n">
-        <v/>
+      <c r="C39" s="26" t="inlineStr">
+        <is>
+          <t>비아트론</t>
+        </is>
+      </c>
+      <c r="D39" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E39" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F39" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G39" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H39" s="27" t="n">
+        <v>-9.609999999999999</v>
+      </c>
+      <c r="I39" s="29" t="n">
+        <v>28.12</v>
+      </c>
+      <c r="J39" s="28" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +232%</t>
+        </is>
+      </c>
+      <c r="K39" s="28" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
-      <c r="A40" s="20" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="B40" s="20" t="n">
+      <c r="A40" s="25" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B40" s="25" t="n">
         <v>27</v>
       </c>
-      <c r="C40" s="21" t="inlineStr">
-        <is>
-          <t>국제약품</t>
-        </is>
-      </c>
-      <c r="D40" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E40" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F40" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G40" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H40" s="24" t="n">
-        <v>-4.4</v>
-      </c>
-      <c r="I40" s="22" t="n">
-        <v>31.52</v>
-      </c>
-      <c r="J40" s="23" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +438% / 중요공시 2건</t>
-        </is>
-      </c>
-      <c r="K40" s="23" t="inlineStr">
-        <is>
-          <t>네이버, 공시</t>
+      <c r="C40" s="26" t="inlineStr">
+        <is>
+          <t>녹십자엠에스</t>
+        </is>
+      </c>
+      <c r="D40" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E40" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F40" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G40" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H40" s="27" t="n">
+        <v>-14.53</v>
+      </c>
+      <c r="I40" s="29" t="n">
+        <v>12.39</v>
+      </c>
+      <c r="J40" s="28" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +186%</t>
+        </is>
+      </c>
+      <c r="K40" s="28" t="inlineStr">
+        <is>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
-      <c r="A41" s="20" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="B41" s="20" t="n">
+      <c r="A41" s="25" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B41" s="25" t="n">
         <v>28</v>
       </c>
-      <c r="C41" s="21" t="inlineStr">
-        <is>
-          <t>빛과전자</t>
-        </is>
-      </c>
-      <c r="D41" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E41" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F41" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G41" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H41" s="24" t="n">
-        <v>-4.49</v>
-      </c>
-      <c r="I41" s="22" t="n">
-        <v>18.83</v>
-      </c>
-      <c r="J41" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K41" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
+      <c r="C41" s="26" t="inlineStr">
+        <is>
+          <t>라온시큐어</t>
+        </is>
+      </c>
+      <c r="D41" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E41" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F41" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G41" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H41" s="27" t="n">
+        <v>-5.14</v>
+      </c>
+      <c r="I41" s="29" t="n">
+        <v>39.35</v>
+      </c>
+      <c r="J41" s="28" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +183%</t>
+        </is>
+      </c>
+      <c r="K41" s="28" t="inlineStr">
+        <is>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
-      <c r="A42" s="20" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="B42" s="20" t="n">
+      <c r="A42" s="25" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B42" s="25" t="n">
         <v>29</v>
       </c>
-      <c r="C42" s="21" t="inlineStr">
-        <is>
-          <t>조선</t>
-        </is>
-      </c>
-      <c r="D42" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E42" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F42" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G42" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H42" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I42" s="20" t="n">
-        <v/>
-      </c>
-      <c r="J42" s="23" t="inlineStr">
-        <is>
-          <t>네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K42" s="23" t="inlineStr">
+      <c r="C42" s="26" t="inlineStr">
+        <is>
+          <t>아톤</t>
+        </is>
+      </c>
+      <c r="D42" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E42" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F42" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G42" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H42" s="27" t="n">
+        <v>-3.4</v>
+      </c>
+      <c r="I42" s="29" t="n">
+        <v>22.51</v>
+      </c>
+      <c r="J42" s="28" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +174%</t>
+        </is>
+      </c>
+      <c r="K42" s="28" t="inlineStr">
         <is>
           <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
-      <c r="A43" s="20" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="B43" s="20" t="n">
+      <c r="A43" s="25" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B43" s="25" t="n">
         <v>30</v>
       </c>
-      <c r="C43" s="21" t="inlineStr">
-        <is>
-          <t>신한지주</t>
-        </is>
-      </c>
-      <c r="D43" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E43" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F43" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G43" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H43" s="24" t="n">
-        <v>-2.91</v>
-      </c>
-      <c r="I43" s="24" t="n">
-        <v>-6.1</v>
-      </c>
-      <c r="J43" s="23" t="inlineStr">
-        <is>
-          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급</t>
-        </is>
-      </c>
-      <c r="K43" s="23" t="inlineStr">
+      <c r="C43" s="26" t="inlineStr">
+        <is>
+          <t>국전</t>
+        </is>
+      </c>
+      <c r="D43" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E43" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F43" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G43" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H43" s="29" t="n">
+        <v>3.18</v>
+      </c>
+      <c r="I43" s="29" t="n">
+        <v>27.51</v>
+      </c>
+      <c r="J43" s="28" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +105%</t>
+        </is>
+      </c>
+      <c r="K43" s="28" t="inlineStr">
         <is>
           <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
-      <c r="A44" s="20" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="B44" s="20" t="n">
+      <c r="A44" s="25" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B44" s="25" t="n">
         <v>31</v>
       </c>
-      <c r="C44" s="21" t="inlineStr">
-        <is>
-          <t>수소</t>
-        </is>
-      </c>
-      <c r="D44" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E44" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F44" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G44" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H44" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I44" s="20" t="n">
-        <v/>
-      </c>
-      <c r="J44" s="23" t="inlineStr">
-        <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K44" s="23" t="n">
-        <v/>
+      <c r="C44" s="26" t="inlineStr">
+        <is>
+          <t>대성산업</t>
+        </is>
+      </c>
+      <c r="D44" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E44" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F44" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G44" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H44" s="27" t="n">
+        <v>-9.98</v>
+      </c>
+      <c r="I44" s="29" t="n">
+        <v>12.61</v>
+      </c>
+      <c r="J44" s="28" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +90% / 중요공시 2건</t>
+        </is>
+      </c>
+      <c r="K44" s="28" t="inlineStr">
+        <is>
+          <t>공시, 네이버</t>
+        </is>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B45" s="25" t="n">
@@ -2245,7 +2243,7 @@
       </c>
       <c r="C45" s="26" t="inlineStr">
         <is>
-          <t>빅텐츠</t>
+          <t>우원개발</t>
         </is>
       </c>
       <c r="D45" s="25" t="n">
@@ -2260,27 +2258,27 @@
       <c r="G45" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H45" s="27" t="n">
-        <v>-18.27</v>
-      </c>
-      <c r="I45" s="27" t="n">
-        <v>-12.71</v>
+      <c r="H45" s="29" t="n">
+        <v>2.74</v>
+      </c>
+      <c r="I45" s="29" t="n">
+        <v>3.31</v>
       </c>
       <c r="J45" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +720%</t>
+          <t>중요공시 3건</t>
         </is>
       </c>
       <c r="K45" s="28" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B46" s="25" t="n">
@@ -2288,42 +2286,42 @@
       </c>
       <c r="C46" s="26" t="inlineStr">
         <is>
-          <t>라온시큐어</t>
+          <t>모아데이타</t>
         </is>
       </c>
       <c r="D46" s="25" t="n">
         <v>3</v>
       </c>
       <c r="E46" s="25" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F46" s="25" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G46" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H46" s="27" t="n">
-        <v>-5.14</v>
+      <c r="H46" s="29" t="n">
+        <v>29.56</v>
       </c>
       <c r="I46" s="29" t="n">
-        <v>39.35</v>
+        <v>30.85</v>
       </c>
       <c r="J46" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +127%</t>
+          <t>중요공시 2건 / 중요공시 3일 +100%</t>
         </is>
       </c>
       <c r="K46" s="28" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B47" s="25" t="n">
@@ -2331,7 +2329,7 @@
       </c>
       <c r="C47" s="26" t="inlineStr">
         <is>
-          <t>아톤</t>
+          <t>대한전선</t>
         </is>
       </c>
       <c r="D47" s="25" t="n">
@@ -2347,14 +2345,14 @@
         <v>0</v>
       </c>
       <c r="H47" s="27" t="n">
-        <v>-3.4</v>
-      </c>
-      <c r="I47" s="29" t="n">
-        <v>22.51</v>
+        <v>-4.71</v>
+      </c>
+      <c r="I47" s="27" t="n">
+        <v>-5.03</v>
       </c>
       <c r="J47" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +125%</t>
+          <t>네이버뉴스 헤드라인 언급</t>
         </is>
       </c>
       <c r="K47" s="28" t="inlineStr">
@@ -2366,7 +2364,7 @@
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B48" s="25" t="n">
@@ -2374,7 +2372,7 @@
       </c>
       <c r="C48" s="26" t="inlineStr">
         <is>
-          <t>이수페타시스</t>
+          <t>알테오젠</t>
         </is>
       </c>
       <c r="D48" s="25" t="n">
@@ -2389,27 +2387,27 @@
       <c r="G48" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H48" s="29" t="n">
-        <v>3.05</v>
-      </c>
-      <c r="I48" s="29" t="n">
-        <v>8.32</v>
+      <c r="H48" s="27" t="n">
+        <v>-5.5</v>
+      </c>
+      <c r="I48" s="27" t="n">
+        <v>-5.87</v>
       </c>
       <c r="J48" s="28" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급</t>
+          <t>중요공시 6건</t>
         </is>
       </c>
       <c r="K48" s="28" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B49" s="25" t="n">
@@ -2417,7 +2415,7 @@
       </c>
       <c r="C49" s="26" t="inlineStr">
         <is>
-          <t>DB</t>
+          <t>엔켐</t>
         </is>
       </c>
       <c r="D49" s="25" t="n">
@@ -2432,25 +2430,27 @@
       <c r="G49" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H49" s="29" t="n">
-        <v>12.72</v>
+      <c r="H49" s="27" t="n">
+        <v>-5.42</v>
       </c>
       <c r="I49" s="29" t="n">
-        <v>19.96</v>
+        <v>5.57</v>
       </c>
       <c r="J49" s="28" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K49" s="28" t="n">
-        <v/>
+          <t>중요공시 3건</t>
+        </is>
+      </c>
+      <c r="K49" s="28" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B50" s="25" t="n">
@@ -2458,7 +2458,7 @@
       </c>
       <c r="C50" s="26" t="inlineStr">
         <is>
-          <t>우원개발</t>
+          <t>LS에코에너지</t>
         </is>
       </c>
       <c r="D50" s="25" t="n">
@@ -2474,26 +2474,26 @@
         <v>0</v>
       </c>
       <c r="H50" s="29" t="n">
-        <v>2.74</v>
+        <v>6.89</v>
       </c>
       <c r="I50" s="29" t="n">
-        <v>3.31</v>
+        <v>16.83</v>
       </c>
       <c r="J50" s="28" t="inlineStr">
         <is>
-          <t>중요공시 3건</t>
+          <t>네이버뉴스 헤드라인 언급</t>
         </is>
       </c>
       <c r="K50" s="28" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B51" s="25" t="n">
@@ -2501,7 +2501,7 @@
       </c>
       <c r="C51" s="26" t="inlineStr">
         <is>
-          <t>엔켐</t>
+          <t>일진전기</t>
         </is>
       </c>
       <c r="D51" s="25" t="n">
@@ -2517,26 +2517,26 @@
         <v>0</v>
       </c>
       <c r="H51" s="27" t="n">
-        <v>-5.42</v>
-      </c>
-      <c r="I51" s="29" t="n">
-        <v>5.57</v>
+        <v>-5.75</v>
+      </c>
+      <c r="I51" s="27" t="n">
+        <v>-0.73</v>
       </c>
       <c r="J51" s="28" t="inlineStr">
         <is>
-          <t>중요공시 3건</t>
+          <t>네이버뉴스 헤드라인 언급</t>
         </is>
       </c>
       <c r="K51" s="28" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B52" s="25" t="n">
@@ -2544,7 +2544,7 @@
       </c>
       <c r="C52" s="26" t="inlineStr">
         <is>
-          <t>삼성전기</t>
+          <t>AI반도체</t>
         </is>
       </c>
       <c r="D52" s="25" t="n">
@@ -2559,27 +2559,25 @@
       <c r="G52" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H52" s="27" t="n">
-        <v>-2.99</v>
-      </c>
-      <c r="I52" s="29" t="n">
-        <v>2.97</v>
+      <c r="H52" s="25" t="n">
+        <v/>
+      </c>
+      <c r="I52" s="25" t="n">
+        <v/>
       </c>
       <c r="J52" s="28" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K52" s="28" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K52" s="28" t="n">
+        <v/>
       </c>
     </row>
     <row r="53" ht="18" customHeight="1">
       <c r="A53" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B53" s="25" t="n">
@@ -2587,7 +2585,7 @@
       </c>
       <c r="C53" s="26" t="inlineStr">
         <is>
-          <t>에코프로</t>
+          <t>조선</t>
         </is>
       </c>
       <c r="D53" s="25" t="n">
@@ -2602,11 +2600,11 @@
       <c r="G53" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H53" s="29" t="n">
-        <v>0.22</v>
-      </c>
-      <c r="I53" s="29" t="n">
-        <v>13.86</v>
+      <c r="H53" s="25" t="n">
+        <v/>
+      </c>
+      <c r="I53" s="25" t="n">
+        <v/>
       </c>
       <c r="J53" s="28" t="inlineStr">
         <is>
@@ -2622,7 +2620,7 @@
     <row r="54" ht="18" customHeight="1">
       <c r="A54" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B54" s="25" t="n">
@@ -2630,7 +2628,7 @@
       </c>
       <c r="C54" s="26" t="inlineStr">
         <is>
-          <t>에코프로비엠</t>
+          <t>유바이오로직스</t>
         </is>
       </c>
       <c r="D54" s="25" t="n">
@@ -2645,27 +2643,25 @@
       <c r="G54" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H54" s="29" t="n">
-        <v>1.69</v>
+      <c r="H54" s="27" t="n">
+        <v>-0.47</v>
       </c>
       <c r="I54" s="29" t="n">
-        <v>16.06</v>
+        <v>1.44</v>
       </c>
       <c r="J54" s="28" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K54" s="28" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+          <t>매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K54" s="28" t="n">
+        <v/>
       </c>
     </row>
     <row r="55" ht="18" customHeight="1">
       <c r="A55" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B55" s="25" t="n">
@@ -2673,7 +2669,7 @@
       </c>
       <c r="C55" s="26" t="inlineStr">
         <is>
-          <t>삼성에스디에스</t>
+          <t>SK스퀘어</t>
         </is>
       </c>
       <c r="D55" s="25" t="n">
@@ -2689,26 +2685,24 @@
         <v>0</v>
       </c>
       <c r="H55" s="27" t="n">
-        <v>-5.27</v>
+        <v>-6.78</v>
       </c>
       <c r="I55" s="27" t="n">
-        <v>-10.25</v>
+        <v>-6.45</v>
       </c>
       <c r="J55" s="28" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K55" s="28" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+          <t>매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K55" s="28" t="n">
+        <v/>
       </c>
     </row>
     <row r="56" ht="18" customHeight="1">
       <c r="A56" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B56" s="25" t="n">
@@ -2716,7 +2710,7 @@
       </c>
       <c r="C56" s="26" t="inlineStr">
         <is>
-          <t>기아</t>
+          <t>한양디지텍</t>
         </is>
       </c>
       <c r="D56" s="25" t="n">
@@ -2731,27 +2725,25 @@
       <c r="G56" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H56" s="27" t="n">
-        <v>-2.1</v>
-      </c>
-      <c r="I56" s="27" t="n">
-        <v>-5.81</v>
+      <c r="H56" s="29" t="n">
+        <v>7.01</v>
+      </c>
+      <c r="I56" s="29" t="n">
+        <v>21.91</v>
       </c>
       <c r="J56" s="28" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K56" s="28" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+          <t>매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K56" s="28" t="n">
+        <v/>
       </c>
     </row>
     <row r="57" ht="18" customHeight="1">
       <c r="A57" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B57" s="25" t="n">
@@ -2759,7 +2751,7 @@
       </c>
       <c r="C57" s="26" t="inlineStr">
         <is>
-          <t>유바이오로직스</t>
+          <t>한컴</t>
         </is>
       </c>
       <c r="D57" s="25" t="n">
@@ -2775,14 +2767,14 @@
         <v>0</v>
       </c>
       <c r="H57" s="27" t="n">
-        <v>-0.47</v>
+        <v>-1.48</v>
       </c>
       <c r="I57" s="29" t="n">
-        <v>1.44</v>
+        <v>1.29</v>
       </c>
       <c r="J57" s="28" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급</t>
+          <t>한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K57" s="28" t="n">
@@ -2792,7 +2784,7 @@
     <row r="58" ht="18" customHeight="1">
       <c r="A58" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B58" s="25" t="n">
@@ -2800,7 +2792,7 @@
       </c>
       <c r="C58" s="26" t="inlineStr">
         <is>
-          <t>유진테크놀로지</t>
+          <t>SK이터닉스</t>
         </is>
       </c>
       <c r="D58" s="25" t="n">
@@ -2815,27 +2807,25 @@
       <c r="G58" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H58" s="29" t="n">
-        <v>30</v>
-      </c>
-      <c r="I58" s="29" t="n">
-        <v>24.87</v>
+      <c r="H58" s="27" t="n">
+        <v>-5.71</v>
+      </c>
+      <c r="I58" s="27" t="n">
+        <v>-7.23</v>
       </c>
       <c r="J58" s="28" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K58" s="28" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+          <t>매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K58" s="28" t="n">
+        <v/>
       </c>
     </row>
     <row r="59" ht="18" customHeight="1">
       <c r="A59" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B59" s="25" t="n">
@@ -2843,7 +2833,7 @@
       </c>
       <c r="C59" s="26" t="inlineStr">
         <is>
-          <t>SK스퀘어</t>
+          <t>현대로템</t>
         </is>
       </c>
       <c r="D59" s="25" t="n">
@@ -2859,14 +2849,14 @@
         <v>0</v>
       </c>
       <c r="H59" s="27" t="n">
-        <v>-6.78</v>
+        <v>-2.87</v>
       </c>
       <c r="I59" s="27" t="n">
-        <v>-6.45</v>
+        <v>-7.42</v>
       </c>
       <c r="J59" s="28" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급</t>
+          <t>한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K59" s="28" t="n">
@@ -2876,7 +2866,7 @@
     <row r="60" ht="18" customHeight="1">
       <c r="A60" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B60" s="25" t="n">
@@ -2884,7 +2874,7 @@
       </c>
       <c r="C60" s="26" t="inlineStr">
         <is>
-          <t>심텍</t>
+          <t>방산</t>
         </is>
       </c>
       <c r="D60" s="25" t="n">
@@ -2899,11 +2889,11 @@
       <c r="G60" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H60" s="29" t="n">
-        <v>0.89</v>
-      </c>
-      <c r="I60" s="29" t="n">
-        <v>13.5</v>
+      <c r="H60" s="25" t="n">
+        <v/>
+      </c>
+      <c r="I60" s="25" t="n">
+        <v/>
       </c>
       <c r="J60" s="28" t="inlineStr">
         <is>
@@ -2917,7 +2907,7 @@
     <row r="61" ht="18" customHeight="1">
       <c r="A61" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B61" s="25" t="n">
@@ -2925,7 +2915,7 @@
       </c>
       <c r="C61" s="26" t="inlineStr">
         <is>
-          <t>대덕전자</t>
+          <t>동양</t>
         </is>
       </c>
       <c r="D61" s="25" t="n">
@@ -2940,11 +2930,11 @@
       <c r="G61" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H61" s="29" t="n">
-        <v>5.21</v>
-      </c>
-      <c r="I61" s="29" t="n">
-        <v>19.12</v>
+      <c r="H61" s="27" t="n">
+        <v>-0.45</v>
+      </c>
+      <c r="I61" s="27" t="n">
+        <v>-2.37</v>
       </c>
       <c r="J61" s="28" t="inlineStr">
         <is>
@@ -2958,7 +2948,7 @@
     <row r="62" ht="18" customHeight="1">
       <c r="A62" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B62" s="25" t="n">
@@ -2966,7 +2956,7 @@
       </c>
       <c r="C62" s="26" t="inlineStr">
         <is>
-          <t>한양디지텍</t>
+          <t>동양고속</t>
         </is>
       </c>
       <c r="D62" s="25" t="n">
@@ -2982,14 +2972,14 @@
         <v>0</v>
       </c>
       <c r="H62" s="29" t="n">
-        <v>7.01</v>
+        <v>27.18</v>
       </c>
       <c r="I62" s="29" t="n">
-        <v>21.91</v>
+        <v>58.64</v>
       </c>
       <c r="J62" s="28" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급</t>
+          <t>한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K62" s="28" t="n">
@@ -2999,7 +2989,7 @@
     <row r="63" ht="18" customHeight="1">
       <c r="A63" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B63" s="25" t="n">
@@ -3007,7 +2997,7 @@
       </c>
       <c r="C63" s="26" t="inlineStr">
         <is>
-          <t>SK이터닉스</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="D63" s="25" t="n">
@@ -3022,15 +3012,15 @@
       <c r="G63" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H63" s="27" t="n">
-        <v>-5.71</v>
-      </c>
-      <c r="I63" s="27" t="n">
-        <v>-7.23</v>
+      <c r="H63" s="25" t="n">
+        <v/>
+      </c>
+      <c r="I63" s="25" t="n">
+        <v/>
       </c>
       <c r="J63" s="28" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급</t>
+          <t>한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K63" s="28" t="n">
@@ -3130,22 +3120,22 @@
         <v>1</v>
       </c>
       <c r="C3" s="25" t="n">
-        <v>63</v>
+        <v>88</v>
       </c>
       <c r="D3" s="25" t="n">
-        <v>63</v>
+        <v>88</v>
       </c>
       <c r="E3" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F3" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="G3" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="H3" s="25" t="n"/>
@@ -3154,165 +3144,161 @@
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="26" t="inlineStr">
         <is>
-          <t>삼성전자</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="B4" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C4" s="25" t="n">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="D4" s="25" t="n">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="E4" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F4" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="G4" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="H4" s="27" t="n">
-        <v>-2.23</v>
-      </c>
-      <c r="I4" s="27" t="n">
-        <v>-2.41</v>
-      </c>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="H4" s="25" t="n"/>
+      <c r="I4" s="25" t="n"/>
     </row>
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="26" t="inlineStr">
         <is>
-          <t>LG</t>
+          <t>삼성전자</t>
         </is>
       </c>
       <c r="B5" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="25" t="n">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="D5" s="25" t="n">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="E5" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F5" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="G5" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="H5" s="27" t="n">
-        <v>-1.9</v>
+        <v>-2.23</v>
       </c>
       <c r="I5" s="27" t="n">
-        <v>-2.17</v>
+        <v>-2.41</v>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="26" t="inlineStr">
         <is>
-          <t>전기차</t>
+          <t>LG</t>
         </is>
       </c>
       <c r="B6" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="25" t="n">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="D6" s="25" t="n">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="E6" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F6" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="G6" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="H6" s="25" t="n"/>
-      <c r="I6" s="25" t="n"/>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="H6" s="27" t="n">
+        <v>-1.9</v>
+      </c>
+      <c r="I6" s="27" t="n">
+        <v>-2.17</v>
+      </c>
     </row>
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="26" t="inlineStr">
         <is>
-          <t>LG전자</t>
+          <t>전기차</t>
         </is>
       </c>
       <c r="B7" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="25" t="n">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="D7" s="25" t="n">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="E7" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F7" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="G7" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="H7" s="27" t="n">
-        <v>-3.83</v>
-      </c>
-      <c r="I7" s="27" t="n">
-        <v>-5.85</v>
-      </c>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="H7" s="25" t="n"/>
+      <c r="I7" s="25" t="n"/>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="26" t="inlineStr">
         <is>
-          <t>인공지능</t>
+          <t>바이오</t>
         </is>
       </c>
       <c r="B8" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="25" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="D8" s="25" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="E8" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F8" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="G8" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="H8" s="25" t="n"/>
@@ -3321,73 +3307,77 @@
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="26" t="inlineStr">
         <is>
-          <t>SK하이닉스</t>
+          <t>LG전자</t>
         </is>
       </c>
       <c r="B9" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="25" t="n">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="D9" s="25" t="n">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="E9" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F9" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="G9" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="H9" s="27" t="n">
-        <v>-1.69</v>
+        <v>-3.83</v>
       </c>
       <c r="I9" s="27" t="n">
-        <v>-5.44</v>
+        <v>-5.85</v>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="26" t="inlineStr">
         <is>
-          <t>바이오</t>
+          <t>현대차</t>
         </is>
       </c>
       <c r="B10" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C10" s="25" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D10" s="25" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E10" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F10" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="G10" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="H10" s="25" t="n"/>
-      <c r="I10" s="25" t="n"/>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="H10" s="27" t="n">
+        <v>-3.57</v>
+      </c>
+      <c r="I10" s="27" t="n">
+        <v>-6.48</v>
+      </c>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="26" t="inlineStr">
         <is>
-          <t>펩트론</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="B11" s="25" t="n">
@@ -3404,126 +3394,122 @@
       </c>
       <c r="F11" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="G11" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="H11" s="27" t="n">
-        <v>-5.57</v>
-      </c>
-      <c r="I11" s="27" t="n">
-        <v>-30.52</v>
-      </c>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="H11" s="25" t="n"/>
+      <c r="I11" s="25" t="n"/>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="26" t="inlineStr">
         <is>
-          <t>HD현대</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="B12" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C12" s="25" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D12" s="25" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E12" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F12" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="G12" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="H12" s="27" t="n">
-        <v>-4.08</v>
-      </c>
-      <c r="I12" s="27" t="n">
-        <v>-11.15</v>
-      </c>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="H12" s="25" t="n"/>
+      <c r="I12" s="25" t="n"/>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>현대차</t>
+          <t>SK하이닉스</t>
         </is>
       </c>
       <c r="B13" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C13" s="25" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D13" s="25" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E13" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F13" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="G13" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="H13" s="27" t="n">
-        <v>-3.57</v>
+        <v>-1.69</v>
       </c>
       <c r="I13" s="27" t="n">
-        <v>-6.48</v>
+        <v>-5.44</v>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>TSMC</t>
+          <t>한화오션</t>
         </is>
       </c>
       <c r="B14" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C14" s="25" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D14" s="25" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E14" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F14" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="G14" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="H14" s="25" t="n"/>
-      <c r="I14" s="25" t="n"/>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="H14" s="27" t="n">
+        <v>-3.1</v>
+      </c>
+      <c r="I14" s="27" t="n">
+        <v>-8.880000000000001</v>
+      </c>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>더코디</t>
+          <t>TSMC</t>
         </is>
       </c>
       <c r="B15" s="25" t="n">
@@ -3540,25 +3526,21 @@
       </c>
       <c r="F15" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="G15" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="H15" s="29" t="n">
-        <v>7.28</v>
-      </c>
-      <c r="I15" s="27" t="n">
-        <v>-22.45</v>
-      </c>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="H15" s="25" t="n"/>
+      <c r="I15" s="25" t="n"/>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>한화오션</t>
+          <t>더코디</t>
         </is>
       </c>
       <c r="B16" s="25" t="n">
@@ -3575,60 +3557,60 @@
       </c>
       <c r="F16" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="G16" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="H16" s="27" t="n">
-        <v>-3.1</v>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="H16" s="29" t="n">
+        <v>7.28</v>
       </c>
       <c r="I16" s="27" t="n">
-        <v>-8.880000000000001</v>
+        <v>-22.45</v>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>주성엔지니어링</t>
+          <t>스피어</t>
         </is>
       </c>
       <c r="B17" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C17" s="25" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D17" s="25" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E17" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F17" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="G17" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="H17" s="29" t="n">
-        <v>4.77</v>
+        <v>0.2</v>
       </c>
       <c r="I17" s="29" t="n">
-        <v>13.33</v>
+        <v>15.72</v>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="26" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>삼성전기</t>
         </is>
       </c>
       <c r="B18" s="25" t="n">
@@ -3645,21 +3627,25 @@
       </c>
       <c r="F18" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="G18" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="H18" s="25" t="n"/>
-      <c r="I18" s="25" t="n"/>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="H18" s="27" t="n">
+        <v>-2.99</v>
+      </c>
+      <c r="I18" s="29" t="n">
+        <v>2.97</v>
+      </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>리노공업</t>
+          <t>삼표시멘트</t>
         </is>
       </c>
       <c r="B19" s="25" t="n">
@@ -3676,25 +3662,25 @@
       </c>
       <c r="F19" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="G19" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="H19" s="29" t="n">
-        <v>3.17</v>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="H19" s="27" t="n">
+        <v>-12.77</v>
       </c>
       <c r="I19" s="29" t="n">
-        <v>19.13</v>
+        <v>5.24</v>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="26" t="inlineStr">
         <is>
-          <t>알테오젠</t>
+          <t>주성엔지니어링</t>
         </is>
       </c>
       <c r="B20" s="25" t="n">
@@ -3711,56 +3697,60 @@
       </c>
       <c r="F20" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="G20" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="H20" s="27" t="n">
-        <v>-5.5</v>
-      </c>
-      <c r="I20" s="27" t="n">
-        <v>-5.87</v>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="H20" s="29" t="n">
+        <v>4.77</v>
+      </c>
+      <c r="I20" s="29" t="n">
+        <v>13.33</v>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="26" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>펩트론</t>
         </is>
       </c>
       <c r="B21" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C21" s="25" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D21" s="25" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E21" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F21" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="G21" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="H21" s="25" t="n"/>
-      <c r="I21" s="25" t="n"/>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="H21" s="27" t="n">
+        <v>-5.57</v>
+      </c>
+      <c r="I21" s="27" t="n">
+        <v>-30.52</v>
+      </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="26" t="inlineStr">
         <is>
-          <t>삼성SDI</t>
+          <t>GS</t>
         </is>
       </c>
       <c r="B22" s="25" t="n">
@@ -3777,152 +3767,148 @@
       </c>
       <c r="F22" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="G22" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="H22" s="29" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="I22" s="29" t="n">
-        <v>10.53</v>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="H22" s="27" t="n">
+        <v>-4.55</v>
+      </c>
+      <c r="I22" s="27" t="n">
+        <v>-1.69</v>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="26" t="inlineStr">
         <is>
-          <t>삼성생명</t>
+          <t>게임</t>
         </is>
       </c>
       <c r="B23" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C23" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D23" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E23" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F23" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="G23" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="H23" s="27" t="n">
-        <v>-3.05</v>
-      </c>
-      <c r="I23" s="27" t="n">
-        <v>-4.59</v>
-      </c>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="H23" s="25" t="n"/>
+      <c r="I23" s="25" t="n"/>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="26" t="inlineStr">
         <is>
-          <t>삼표시멘트</t>
+          <t>국제약품</t>
         </is>
       </c>
       <c r="B24" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C24" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D24" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E24" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F24" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="G24" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="H24" s="27" t="n">
-        <v>-12.77</v>
+        <v>-4.4</v>
       </c>
       <c r="I24" s="29" t="n">
-        <v>5.24</v>
+        <v>31.52</v>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="26" t="inlineStr">
         <is>
-          <t>스피어</t>
+          <t>대양금속</t>
         </is>
       </c>
       <c r="B25" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C25" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D25" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E25" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F25" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="G25" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="H25" s="29" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="I25" s="29" t="n">
-        <v>15.72</v>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="H25" s="27" t="n">
+        <v>-6.73</v>
+      </c>
+      <c r="I25" s="27" t="n">
+        <v>-21.09</v>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="26" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>수소</t>
         </is>
       </c>
       <c r="B26" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C26" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D26" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E26" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F26" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="G26" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="H26" s="25" t="n"/>
@@ -3931,29 +3917,29 @@
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="26" t="inlineStr">
         <is>
-          <t>태양광</t>
+          <t>AI반도체</t>
         </is>
       </c>
       <c r="B27" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C27" s="25" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D27" s="25" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E27" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F27" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="G27" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="H27" s="25" t="n"/>
@@ -3962,209 +3948,213 @@
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="26" t="inlineStr">
         <is>
-          <t>한미약품</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B28" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C28" s="25" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D28" s="25" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E28" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F28" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="G28" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="H28" s="27" t="n">
-        <v>-9.74</v>
-      </c>
-      <c r="I28" s="27" t="n">
-        <v>-3.31</v>
-      </c>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="H28" s="25" t="n"/>
+      <c r="I28" s="25" t="n"/>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="26" t="inlineStr">
         <is>
-          <t>국제약품</t>
+          <t>LS에코에너지</t>
         </is>
       </c>
       <c r="B29" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C29" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D29" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E29" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F29" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="G29" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="H29" s="27" t="n">
-        <v>-4.4</v>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="H29" s="29" t="n">
+        <v>6.89</v>
       </c>
       <c r="I29" s="29" t="n">
-        <v>31.52</v>
+        <v>16.83</v>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="26" t="inlineStr">
         <is>
-          <t>빛과전자</t>
+          <t>SK스퀘어</t>
         </is>
       </c>
       <c r="B30" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C30" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D30" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E30" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F30" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="G30" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="H30" s="27" t="n">
-        <v>-4.49</v>
-      </c>
-      <c r="I30" s="29" t="n">
-        <v>18.83</v>
+        <v>-6.78</v>
+      </c>
+      <c r="I30" s="27" t="n">
+        <v>-6.45</v>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="26" t="inlineStr">
         <is>
-          <t>수소</t>
+          <t>SK이터닉스</t>
         </is>
       </c>
       <c r="B31" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C31" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D31" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E31" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F31" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="G31" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="H31" s="25" t="n"/>
-      <c r="I31" s="25" t="n"/>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="H31" s="27" t="n">
+        <v>-5.71</v>
+      </c>
+      <c r="I31" s="27" t="n">
+        <v>-7.23</v>
+      </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="26" t="inlineStr">
         <is>
-          <t>신한지주</t>
+          <t>국전</t>
         </is>
       </c>
       <c r="B32" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C32" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D32" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E32" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F32" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="G32" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="H32" s="27" t="n">
-        <v>-2.91</v>
-      </c>
-      <c r="I32" s="27" t="n">
-        <v>-6.1</v>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="H32" s="29" t="n">
+        <v>3.18</v>
+      </c>
+      <c r="I32" s="29" t="n">
+        <v>27.51</v>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="26" t="inlineStr">
         <is>
-          <t>조선</t>
+          <t>녹십자엠에스</t>
         </is>
       </c>
       <c r="B33" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C33" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D33" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E33" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F33" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="G33" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="H33" s="25" t="n"/>
-      <c r="I33" s="25" t="n"/>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="H33" s="27" t="n">
+        <v>-14.53</v>
+      </c>
+      <c r="I33" s="29" t="n">
+        <v>12.39</v>
+      </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="26" t="inlineStr">
         <is>
-          <t>DB</t>
+          <t>대성산업</t>
         </is>
       </c>
       <c r="B34" s="25" t="n">
@@ -4181,25 +4171,25 @@
       </c>
       <c r="F34" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="G34" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="H34" s="29" t="n">
-        <v>12.72</v>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="H34" s="27" t="n">
+        <v>-9.98</v>
       </c>
       <c r="I34" s="29" t="n">
-        <v>19.96</v>
+        <v>12.61</v>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="26" t="inlineStr">
         <is>
-          <t>SK스퀘어</t>
+          <t>대한전선</t>
         </is>
       </c>
       <c r="B35" s="25" t="n">
@@ -4216,25 +4206,25 @@
       </c>
       <c r="F35" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="G35" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="H35" s="27" t="n">
-        <v>-6.78</v>
+        <v>-4.71</v>
       </c>
       <c r="I35" s="27" t="n">
-        <v>-6.45</v>
+        <v>-5.03</v>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="26" t="inlineStr">
         <is>
-          <t>SK이터닉스</t>
+          <t>동양</t>
         </is>
       </c>
       <c r="B36" s="25" t="n">
@@ -4251,25 +4241,25 @@
       </c>
       <c r="F36" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="G36" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="H36" s="27" t="n">
-        <v>-5.71</v>
+        <v>-0.45</v>
       </c>
       <c r="I36" s="27" t="n">
-        <v>-7.23</v>
+        <v>-2.37</v>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="26" t="inlineStr">
         <is>
-          <t>기아</t>
+          <t>동양고속</t>
         </is>
       </c>
       <c r="B37" s="25" t="n">
@@ -4286,25 +4276,25 @@
       </c>
       <c r="F37" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="G37" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="H37" s="27" t="n">
-        <v>-2.1</v>
-      </c>
-      <c r="I37" s="27" t="n">
-        <v>-5.81</v>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="H37" s="29" t="n">
+        <v>27.18</v>
+      </c>
+      <c r="I37" s="29" t="n">
+        <v>58.64</v>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="26" t="inlineStr">
         <is>
-          <t>대덕전자</t>
+          <t>라온시큐어</t>
         </is>
       </c>
       <c r="B38" s="25" t="n">
@@ -4321,25 +4311,25 @@
       </c>
       <c r="F38" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="G38" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="H38" s="29" t="n">
-        <v>5.21</v>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="H38" s="27" t="n">
+        <v>-5.14</v>
       </c>
       <c r="I38" s="29" t="n">
-        <v>19.12</v>
+        <v>39.35</v>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="26" t="inlineStr">
         <is>
-          <t>라온시큐어</t>
+          <t>모아데이타</t>
         </is>
       </c>
       <c r="B39" s="25" t="n">
@@ -4356,25 +4346,25 @@
       </c>
       <c r="F39" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="G39" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="H39" s="27" t="n">
-        <v>-5.14</v>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="H39" s="29" t="n">
+        <v>29.56</v>
       </c>
       <c r="I39" s="29" t="n">
-        <v>39.35</v>
+        <v>30.85</v>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="26" t="inlineStr">
         <is>
-          <t>빅텐츠</t>
+          <t>방산</t>
         </is>
       </c>
       <c r="B40" s="25" t="n">
@@ -4391,25 +4381,21 @@
       </c>
       <c r="F40" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="G40" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="H40" s="27" t="n">
-        <v>-18.27</v>
-      </c>
-      <c r="I40" s="27" t="n">
-        <v>-12.71</v>
-      </c>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="H40" s="25" t="n"/>
+      <c r="I40" s="25" t="n"/>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="26" t="inlineStr">
         <is>
-          <t>삼성에스디에스</t>
+          <t>비아트론</t>
         </is>
       </c>
       <c r="B41" s="25" t="n">
@@ -4426,25 +4412,25 @@
       </c>
       <c r="F41" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="G41" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="H41" s="27" t="n">
-        <v>-5.27</v>
-      </c>
-      <c r="I41" s="27" t="n">
-        <v>-10.25</v>
+        <v>-9.609999999999999</v>
+      </c>
+      <c r="I41" s="29" t="n">
+        <v>28.12</v>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="26" t="inlineStr">
         <is>
-          <t>삼성전기</t>
+          <t>빅텐츠</t>
         </is>
       </c>
       <c r="B42" s="25" t="n">
@@ -4461,25 +4447,25 @@
       </c>
       <c r="F42" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="G42" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="H42" s="27" t="n">
-        <v>-2.99</v>
-      </c>
-      <c r="I42" s="29" t="n">
-        <v>2.97</v>
+        <v>-18.27</v>
+      </c>
+      <c r="I42" s="27" t="n">
+        <v>-12.71</v>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="26" t="inlineStr">
         <is>
-          <t>심텍</t>
+          <t>아톤</t>
         </is>
       </c>
       <c r="B43" s="25" t="n">
@@ -4496,25 +4482,25 @@
       </c>
       <c r="F43" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="G43" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="H43" s="29" t="n">
-        <v>0.89</v>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="H43" s="27" t="n">
+        <v>-3.4</v>
       </c>
       <c r="I43" s="29" t="n">
-        <v>13.5</v>
+        <v>22.51</v>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="26" t="inlineStr">
         <is>
-          <t>아톤</t>
+          <t>알테오젠</t>
         </is>
       </c>
       <c r="B44" s="25" t="n">
@@ -4531,25 +4517,25 @@
       </c>
       <c r="F44" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="G44" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="H44" s="27" t="n">
-        <v>-3.4</v>
-      </c>
-      <c r="I44" s="29" t="n">
-        <v>22.51</v>
+        <v>-5.5</v>
+      </c>
+      <c r="I44" s="27" t="n">
+        <v>-5.87</v>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="26" t="inlineStr">
         <is>
-          <t>에코프로</t>
+          <t>엔켐</t>
         </is>
       </c>
       <c r="B45" s="25" t="n">
@@ -4566,25 +4552,25 @@
       </c>
       <c r="F45" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="G45" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="H45" s="29" t="n">
-        <v>0.22</v>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="H45" s="27" t="n">
+        <v>-5.42</v>
       </c>
       <c r="I45" s="29" t="n">
-        <v>13.86</v>
+        <v>5.57</v>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="26" t="inlineStr">
         <is>
-          <t>에코프로비엠</t>
+          <t>우원개발</t>
         </is>
       </c>
       <c r="B46" s="25" t="n">
@@ -4601,25 +4587,25 @@
       </c>
       <c r="F46" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="G46" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="H46" s="29" t="n">
-        <v>1.69</v>
+        <v>2.74</v>
       </c>
       <c r="I46" s="29" t="n">
-        <v>16.06</v>
+        <v>3.31</v>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="26" t="inlineStr">
         <is>
-          <t>엔켐</t>
+          <t>유바이오로직스</t>
         </is>
       </c>
       <c r="B47" s="25" t="n">
@@ -4636,25 +4622,25 @@
       </c>
       <c r="F47" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="G47" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="H47" s="27" t="n">
-        <v>-5.42</v>
+        <v>-0.47</v>
       </c>
       <c r="I47" s="29" t="n">
-        <v>5.57</v>
+        <v>1.44</v>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="26" t="inlineStr">
         <is>
-          <t>우원개발</t>
+          <t>일진전기</t>
         </is>
       </c>
       <c r="B48" s="25" t="n">
@@ -4671,25 +4657,25 @@
       </c>
       <c r="F48" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="G48" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="H48" s="29" t="n">
-        <v>2.74</v>
-      </c>
-      <c r="I48" s="29" t="n">
-        <v>3.31</v>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="H48" s="27" t="n">
+        <v>-5.75</v>
+      </c>
+      <c r="I48" s="27" t="n">
+        <v>-0.73</v>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="26" t="inlineStr">
         <is>
-          <t>유바이오로직스</t>
+          <t>조선</t>
         </is>
       </c>
       <c r="B49" s="25" t="n">
@@ -4706,25 +4692,21 @@
       </c>
       <c r="F49" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="G49" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="H49" s="27" t="n">
-        <v>-0.47</v>
-      </c>
-      <c r="I49" s="29" t="n">
-        <v>1.44</v>
-      </c>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="H49" s="25" t="n"/>
+      <c r="I49" s="25" t="n"/>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="26" t="inlineStr">
         <is>
-          <t>유진테크놀로지</t>
+          <t>한양디지텍</t>
         </is>
       </c>
       <c r="B50" s="25" t="n">
@@ -4741,25 +4723,25 @@
       </c>
       <c r="F50" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="G50" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="H50" s="29" t="n">
-        <v>30</v>
+        <v>7.01</v>
       </c>
       <c r="I50" s="29" t="n">
-        <v>24.87</v>
+        <v>21.91</v>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="26" t="inlineStr">
         <is>
-          <t>이수페타시스</t>
+          <t>한컴</t>
         </is>
       </c>
       <c r="B51" s="25" t="n">
@@ -4776,25 +4758,25 @@
       </c>
       <c r="F51" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="G51" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="H51" s="29" t="n">
-        <v>3.05</v>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="H51" s="27" t="n">
+        <v>-1.48</v>
       </c>
       <c r="I51" s="29" t="n">
-        <v>8.32</v>
+        <v>1.29</v>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="26" t="inlineStr">
         <is>
-          <t>한양디지텍</t>
+          <t>현대로템</t>
         </is>
       </c>
       <c r="B52" s="25" t="n">
@@ -4811,19 +4793,19 @@
       </c>
       <c r="F52" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="G52" s="25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="H52" s="29" t="n">
-        <v>7.01</v>
-      </c>
-      <c r="I52" s="29" t="n">
-        <v>21.91</v>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="H52" s="27" t="n">
+        <v>-2.87</v>
+      </c>
+      <c r="I52" s="27" t="n">
+        <v>-7.42</v>
       </c>
     </row>
   </sheetData>
@@ -4907,19 +4889,19 @@
         <v>1</v>
       </c>
       <c r="C3" s="36" t="n">
-        <v>63</v>
+        <v>88</v>
       </c>
       <c r="D3" s="36" t="n">
-        <v>63</v>
+        <v>88</v>
       </c>
       <c r="E3" s="36" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="F3" s="37" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="G3" s="37" t="inlineStr">
@@ -4938,19 +4920,19 @@
         <v>1</v>
       </c>
       <c r="C4" s="36" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D4" s="36" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E4" s="36" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="F4" s="37" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="G4" s="37" t="inlineStr">
@@ -4962,26 +4944,26 @@
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="35" t="inlineStr">
         <is>
-          <t>전기차</t>
+          <t>AI반도체</t>
         </is>
       </c>
       <c r="B5" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="36" t="n">
-        <v>28</v>
+        <v>3</v>
       </c>
       <c r="D5" s="36" t="n">
-        <v>28</v>
+        <v>3</v>
       </c>
       <c r="E5" s="36" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="F5" s="37" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="G5" s="37" t="inlineStr">
@@ -4993,26 +4975,26 @@
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="35" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>전기차</t>
         </is>
       </c>
       <c r="B6" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="36" t="n">
-        <v>5</v>
+        <v>17</v>
       </c>
       <c r="D6" s="36" t="n">
-        <v>5</v>
+        <v>17</v>
       </c>
       <c r="E6" s="36" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="F6" s="37" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="G6" s="37" t="inlineStr">
@@ -5024,26 +5006,26 @@
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="35" t="inlineStr">
         <is>
-          <t>수소</t>
+          <t>방산</t>
         </is>
       </c>
       <c r="B7" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="36" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D7" s="36" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E7" s="36" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="F7" s="37" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="G7" s="37" t="inlineStr">
@@ -5055,26 +5037,26 @@
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="35" t="inlineStr">
         <is>
-          <t>태양광</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="B8" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="36" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D8" s="36" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="E8" s="36" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="F8" s="37" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="G8" s="37" t="inlineStr">
@@ -5086,7 +5068,7 @@
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="35" t="inlineStr">
         <is>
-          <t>조선</t>
+          <t>수소</t>
         </is>
       </c>
       <c r="B9" s="36" t="n">
@@ -5100,12 +5082,12 @@
       </c>
       <c r="E9" s="36" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="F9" s="37" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="G9" s="37" t="inlineStr">
@@ -5117,26 +5099,26 @@
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="35" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>게임</t>
         </is>
       </c>
       <c r="B10" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C10" s="36" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D10" s="36" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E10" s="36" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="F10" s="37" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="G10" s="37" t="inlineStr">
@@ -5148,26 +5130,26 @@
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="35" t="inlineStr">
         <is>
-          <t>인공지능</t>
+          <t>조선</t>
         </is>
       </c>
       <c r="B11" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="36" t="n">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="D11" s="36" t="n">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="E11" s="36" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="F11" s="37" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="G11" s="37" t="inlineStr">
@@ -5179,92 +5161,100 @@
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="35" t="inlineStr">
         <is>
+          <t>제약</t>
+        </is>
+      </c>
+      <c r="B12" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C12" s="36" t="n">
+        <v>11</v>
+      </c>
+      <c r="D12" s="36" t="n">
+        <v>11</v>
+      </c>
+      <c r="E12" s="36" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="F12" s="37" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="G12" s="37" t="inlineStr">
+        <is>
+          <t>⚡ 관심</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="35" t="inlineStr">
+        <is>
+          <t>인공지능</t>
+        </is>
+      </c>
+      <c r="B13" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C13" s="36" t="n">
+        <v>28</v>
+      </c>
+      <c r="D13" s="36" t="n">
+        <v>28</v>
+      </c>
+      <c r="E13" s="36" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="F13" s="37" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="G13" s="37" t="inlineStr">
+        <is>
+          <t>⚡ 관심</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="A14" s="35" t="inlineStr">
+        <is>
           <t>AMD</t>
         </is>
       </c>
-      <c r="B12" s="36" t="n">
-        <v>1</v>
-      </c>
-      <c r="C12" s="36" t="n">
-        <v>6</v>
-      </c>
-      <c r="D12" s="36" t="n">
-        <v>6</v>
-      </c>
-      <c r="E12" s="36" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="F12" s="37" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="G12" s="37" t="inlineStr">
+      <c r="B14" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C14" s="36" t="n">
+        <v>3</v>
+      </c>
+      <c r="D14" s="36" t="n">
+        <v>3</v>
+      </c>
+      <c r="E14" s="36" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="F14" s="37" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="G14" s="37" t="inlineStr">
         <is>
           <t>⚡ 관심</t>
         </is>
       </c>
-    </row>
-    <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="26" t="inlineStr">
-        <is>
-          <t>이차전지</t>
-        </is>
-      </c>
-      <c r="B13" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="C13" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="D13" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="E13" s="25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F13" s="28" t="inlineStr">
-        <is>
-          <t>감지 없음</t>
-        </is>
-      </c>
-      <c r="G13" s="28" t="inlineStr"/>
-    </row>
-    <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="26" t="inlineStr">
-        <is>
-          <t>AI반도체</t>
-        </is>
-      </c>
-      <c r="B14" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="C14" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="D14" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="E14" s="25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F14" s="28" t="inlineStr">
-        <is>
-          <t>감지 없음</t>
-        </is>
-      </c>
-      <c r="G14" s="28" t="inlineStr"/>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>방산</t>
+          <t>이차전지</t>
         </is>
       </c>
       <c r="B15" s="25" t="n">
@@ -5318,7 +5308,7 @@
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>게임</t>
+          <t>태양광</t>
         </is>
       </c>
       <c r="B17" s="25" t="n">

</xml_diff>

<commit_message>
auto: 2026-10-12 07:20 자동 백업
</commit_message>
<xml_diff>
--- a/trend/stock_trend_history.xlsx
+++ b/trend/stock_trend_history.xlsx
@@ -258,11 +258,11 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -273,11 +273,11 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -691,7 +691,7 @@
     <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-10-11 06:55</t>
+          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-10-12 06:54</t>
         </is>
       </c>
     </row>
@@ -784,21 +784,21 @@
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-10-11) 상위: 반도체  점수 92.0점</t>
+          <t>⚡ 최신(2026-10-12) 상위: 반도체  점수 93.0점</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-10-11) 상위: 삼성전자  점수 38.0점</t>
+          <t>⚡ 최신(2026-10-12) 상위: 삼성전자  점수 31.0점</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-10-11) 상위: 인공지능  점수 29.0점</t>
+          <t>⚡ 최신(2026-10-12) 상위: 인공지능  점수 26.0점</t>
         </is>
       </c>
     </row>
@@ -913,7 +913,7 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="15" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B14" s="15" t="n">
@@ -925,10 +925,10 @@
         </is>
       </c>
       <c r="D14" s="15" t="n">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E14" s="15" t="n">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F14" s="15" t="n">
         <v>0</v>
@@ -944,7 +944,7 @@
       </c>
       <c r="J14" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K14" s="17" t="inlineStr">
@@ -956,7 +956,7 @@
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="15" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B15" s="15" t="n">
@@ -968,10 +968,10 @@
         </is>
       </c>
       <c r="D15" s="15" t="n">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="E15" s="15" t="n">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="F15" s="15" t="n">
         <v>0</v>
@@ -983,23 +983,23 @@
         <v>-2.23</v>
       </c>
       <c r="I15" s="18" t="n">
-        <v>-4.19</v>
+        <v>-4.71</v>
       </c>
       <c r="J15" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급</t>
+          <t>중요공시 1건 / 네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K15" s="17" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="15" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B16" s="15" t="n">
@@ -1011,10 +1011,10 @@
         </is>
       </c>
       <c r="D16" s="15" t="n">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="E16" s="15" t="n">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F16" s="15" t="n">
         <v>0</v>
@@ -1030,7 +1030,7 @@
       </c>
       <c r="J16" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+          <t>매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K16" s="17" t="inlineStr">
@@ -1042,7 +1042,7 @@
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B17" s="15" t="n">
@@ -1050,14 +1050,14 @@
       </c>
       <c r="C17" s="16" t="inlineStr">
         <is>
-          <t>전기차</t>
+          <t>LG</t>
         </is>
       </c>
       <c r="D17" s="15" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E17" s="15" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="F17" s="15" t="n">
         <v>0</v>
@@ -1065,27 +1065,25 @@
       <c r="G17" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H17" s="15" t="n">
+      <c r="H17" s="18" t="n">
+        <v>-1.9</v>
+      </c>
+      <c r="I17" s="18" t="n">
+        <v>-2.69</v>
+      </c>
+      <c r="J17" s="17" t="inlineStr">
+        <is>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K17" s="17" t="n">
         <v/>
-      </c>
-      <c r="I17" s="15" t="n">
-        <v/>
-      </c>
-      <c r="J17" s="17" t="inlineStr">
-        <is>
-          <t>매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K17" s="17" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B18" s="15" t="n">
@@ -1093,14 +1091,14 @@
       </c>
       <c r="C18" s="16" t="inlineStr">
         <is>
-          <t>LG</t>
+          <t>조선</t>
         </is>
       </c>
       <c r="D18" s="15" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E18" s="15" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="F18" s="15" t="n">
         <v>0</v>
@@ -1108,25 +1106,27 @@
       <c r="G18" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H18" s="18" t="n">
-        <v>-1.9</v>
-      </c>
-      <c r="I18" s="18" t="n">
-        <v>-1.28</v>
+      <c r="H18" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I18" s="15" t="n">
+        <v/>
       </c>
       <c r="J18" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K18" s="17" t="n">
-        <v/>
+          <t>Google 급상승 검색어 등장 (KR) / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K18" s="17" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B19" s="15" t="n">
@@ -1134,14 +1134,14 @@
       </c>
       <c r="C19" s="16" t="inlineStr">
         <is>
-          <t>SK하이닉스</t>
+          <t>방산</t>
         </is>
       </c>
       <c r="D19" s="15" t="n">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="E19" s="15" t="n">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="F19" s="15" t="n">
         <v>0</v>
@@ -1149,27 +1149,25 @@
       <c r="G19" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H19" s="18" t="n">
-        <v>-1.69</v>
-      </c>
-      <c r="I19" s="18" t="n">
-        <v>-7.77</v>
+      <c r="H19" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I19" s="15" t="n">
+        <v/>
       </c>
       <c r="J19" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K19" s="17" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K19" s="17" t="n">
+        <v/>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B20" s="15" t="n">
@@ -1177,14 +1175,14 @@
       </c>
       <c r="C20" s="16" t="inlineStr">
         <is>
-          <t>LG전자</t>
+          <t>현대차</t>
         </is>
       </c>
       <c r="D20" s="15" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E20" s="15" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="F20" s="15" t="n">
         <v>0</v>
@@ -1193,14 +1191,14 @@
         <v>0</v>
       </c>
       <c r="H20" s="18" t="n">
-        <v>-3.83</v>
+        <v>-3.57</v>
       </c>
       <c r="I20" s="18" t="n">
-        <v>-5.19</v>
+        <v>-6.48</v>
       </c>
       <c r="J20" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+          <t>한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K20" s="17" t="n">
@@ -1210,7 +1208,7 @@
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="15" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B21" s="15" t="n">
@@ -1218,14 +1216,14 @@
       </c>
       <c r="C21" s="16" t="inlineStr">
         <is>
-          <t>바이오</t>
+          <t>SK하이닉스</t>
         </is>
       </c>
       <c r="D21" s="15" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E21" s="15" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F21" s="15" t="n">
         <v>0</v>
@@ -1233,15 +1231,15 @@
       <c r="G21" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H21" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I21" s="15" t="n">
-        <v/>
+      <c r="H21" s="18" t="n">
+        <v>-1.69</v>
+      </c>
+      <c r="I21" s="18" t="n">
+        <v>-8.470000000000001</v>
       </c>
       <c r="J21" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
+          <t>매일경제 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K21" s="17" t="inlineStr">
@@ -1253,7 +1251,7 @@
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="15" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B22" s="15" t="n">
@@ -1261,14 +1259,14 @@
       </c>
       <c r="C22" s="16" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>LG전자</t>
         </is>
       </c>
       <c r="D22" s="15" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E22" s="15" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="F22" s="15" t="n">
         <v>0</v>
@@ -1276,27 +1274,27 @@
       <c r="G22" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H22" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I22" s="15" t="n">
-        <v/>
+      <c r="H22" s="18" t="n">
+        <v>-3.83</v>
+      </c>
+      <c r="I22" s="18" t="n">
+        <v>-6.73</v>
       </c>
       <c r="J22" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 헤드라인 언급</t>
+          <t>중요공시 1건 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K22" s="17" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="15" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B23" s="15" t="n">
@@ -1304,14 +1302,14 @@
       </c>
       <c r="C23" s="16" t="inlineStr">
         <is>
-          <t>방산</t>
+          <t>바이오</t>
         </is>
       </c>
       <c r="D23" s="15" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E23" s="15" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F23" s="15" t="n">
         <v>0</v>
@@ -1327,17 +1325,19 @@
       </c>
       <c r="J23" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K23" s="17" t="n">
-        <v/>
+          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
+        </is>
+      </c>
+      <c r="K23" s="17" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="15" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B24" s="15" t="n">
@@ -1345,14 +1345,14 @@
       </c>
       <c r="C24" s="16" t="inlineStr">
         <is>
-          <t>현대차</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="D24" s="15" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E24" s="15" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F24" s="15" t="n">
         <v>0</v>
@@ -1360,15 +1360,15 @@
       <c r="G24" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H24" s="18" t="n">
-        <v>-3.57</v>
-      </c>
-      <c r="I24" s="18" t="n">
-        <v>-7.02</v>
+      <c r="H24" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I24" s="15" t="n">
+        <v/>
       </c>
       <c r="J24" s="17" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+          <t>한국경제 헤드라인 언급 / 매일경제 기사 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K24" s="17" t="n">
@@ -1378,7 +1378,7 @@
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="15" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B25" s="15" t="n">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="C25" s="16" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="D25" s="15" t="n">
@@ -1409,7 +1409,7 @@
       </c>
       <c r="J25" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 기사 언급 / 한국경제 헤드라인 언급</t>
+          <t>네이버뉴스 기사 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K25" s="17" t="inlineStr">
@@ -1421,7 +1421,7 @@
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="15" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B26" s="15" t="n">
@@ -1429,7 +1429,7 @@
       </c>
       <c r="C26" s="16" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>GS</t>
         </is>
       </c>
       <c r="D26" s="15" t="n">
@@ -1444,15 +1444,15 @@
       <c r="G26" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H26" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I26" s="15" t="n">
-        <v/>
+      <c r="H26" s="18" t="n">
+        <v>-4.55</v>
+      </c>
+      <c r="I26" s="18" t="n">
+        <v>-0.29</v>
       </c>
       <c r="J26" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 네이버뉴스 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>네이버뉴스 기사 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K26" s="17" t="inlineStr">
@@ -1464,7 +1464,7 @@
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="19" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B27" s="19" t="n">
@@ -1472,7 +1472,7 @@
       </c>
       <c r="C27" s="20" t="inlineStr">
         <is>
-          <t>삼표시멘트</t>
+          <t>빅텐츠</t>
         </is>
       </c>
       <c r="D27" s="19" t="n">
@@ -1488,26 +1488,26 @@
         <v>0</v>
       </c>
       <c r="H27" s="21" t="n">
-        <v>-12.77</v>
-      </c>
-      <c r="I27" s="22" t="n">
-        <v>1.19</v>
-      </c>
-      <c r="J27" s="23" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +169% / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K27" s="23" t="inlineStr">
-        <is>
-          <t>네이버</t>
+        <v>-18.27</v>
+      </c>
+      <c r="I27" s="21" t="n">
+        <v>-11.47</v>
+      </c>
+      <c r="J27" s="22" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +57401% / 중요공시 5건</t>
+        </is>
+      </c>
+      <c r="K27" s="22" t="inlineStr">
+        <is>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="19" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B28" s="19" t="n">
@@ -1519,10 +1519,10 @@
         </is>
       </c>
       <c r="D28" s="19" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E28" s="19" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F28" s="19" t="n">
         <v>0</v>
@@ -1530,25 +1530,25 @@
       <c r="G28" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="H28" s="22" t="n">
+      <c r="H28" s="23" t="n">
         <v>4.77</v>
       </c>
-      <c r="I28" s="22" t="n">
-        <v>9.56</v>
-      </c>
-      <c r="J28" s="23" t="inlineStr">
-        <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K28" s="23" t="n">
+      <c r="I28" s="23" t="n">
+        <v>10.02</v>
+      </c>
+      <c r="J28" s="22" t="inlineStr">
+        <is>
+          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K28" s="22" t="n">
         <v/>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="19" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B29" s="19" t="n">
@@ -1556,42 +1556,42 @@
       </c>
       <c r="C29" s="20" t="inlineStr">
         <is>
-          <t>AI반도체</t>
+          <t>한화오션</t>
         </is>
       </c>
       <c r="D29" s="19" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E29" s="19" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F29" s="19" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G29" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="H29" s="19" t="n">
-        <v/>
-      </c>
-      <c r="I29" s="19" t="n">
-        <v/>
-      </c>
-      <c r="J29" s="23" t="inlineStr">
-        <is>
-          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K29" s="23" t="inlineStr">
-        <is>
-          <t>네이버</t>
+      <c r="H29" s="21" t="n">
+        <v>-3.1</v>
+      </c>
+      <c r="I29" s="21" t="n">
+        <v>-8.77</v>
+      </c>
+      <c r="J29" s="22" t="inlineStr">
+        <is>
+          <t>중요공시 4건 / 중요공시 3일 +100%</t>
+        </is>
+      </c>
+      <c r="K29" s="22" t="inlineStr">
+        <is>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="19" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B30" s="19" t="n">
@@ -1599,7 +1599,7 @@
       </c>
       <c r="C30" s="20" t="inlineStr">
         <is>
-          <t>SG</t>
+          <t>기업은행</t>
         </is>
       </c>
       <c r="D30" s="19" t="n">
@@ -1615,17 +1615,17 @@
         <v>0</v>
       </c>
       <c r="H30" s="21" t="n">
-        <v>-3.87</v>
+        <v>-1</v>
       </c>
       <c r="I30" s="21" t="n">
-        <v>-10.47</v>
-      </c>
-      <c r="J30" s="23" t="inlineStr">
+        <v>-1.97</v>
+      </c>
+      <c r="J30" s="22" t="inlineStr">
         <is>
           <t>Google 급상승 검색어 등장 (KR)</t>
         </is>
       </c>
-      <c r="K30" s="23" t="inlineStr">
+      <c r="K30" s="22" t="inlineStr">
         <is>
           <t>Google</t>
         </is>
@@ -1634,7 +1634,7 @@
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="19" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B31" s="19" t="n">
@@ -1642,7 +1642,7 @@
       </c>
       <c r="C31" s="20" t="inlineStr">
         <is>
-          <t>삼성전기</t>
+          <t>원전</t>
         </is>
       </c>
       <c r="D31" s="19" t="n">
@@ -1657,25 +1657,25 @@
       <c r="G31" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="H31" s="21" t="n">
-        <v>-2.99</v>
-      </c>
-      <c r="I31" s="22" t="n">
-        <v>0.32</v>
-      </c>
-      <c r="J31" s="23" t="inlineStr">
-        <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K31" s="23" t="n">
+      <c r="H31" s="19" t="n">
+        <v/>
+      </c>
+      <c r="I31" s="19" t="n">
+        <v/>
+      </c>
+      <c r="J31" s="22" t="inlineStr">
+        <is>
+          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K31" s="22" t="n">
         <v/>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="19" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B32" s="19" t="n">
@@ -1683,14 +1683,14 @@
       </c>
       <c r="C32" s="20" t="inlineStr">
         <is>
-          <t>TSMC</t>
+          <t>국제약품</t>
         </is>
       </c>
       <c r="D32" s="19" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E32" s="19" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F32" s="19" t="n">
         <v>0</v>
@@ -1698,25 +1698,27 @@
       <c r="G32" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="H32" s="19" t="n">
-        <v/>
-      </c>
-      <c r="I32" s="19" t="n">
-        <v/>
-      </c>
-      <c r="J32" s="23" t="inlineStr">
-        <is>
-          <t>한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K32" s="23" t="n">
-        <v/>
+      <c r="H32" s="21" t="n">
+        <v>-4.4</v>
+      </c>
+      <c r="I32" s="23" t="n">
+        <v>28.14</v>
+      </c>
+      <c r="J32" s="22" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +1048% / 중요공시 2건</t>
+        </is>
+      </c>
+      <c r="K32" s="22" t="inlineStr">
+        <is>
+          <t>공시, 네이버</t>
+        </is>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="19" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B33" s="19" t="n">
@@ -1724,7 +1726,7 @@
       </c>
       <c r="C33" s="20" t="inlineStr">
         <is>
-          <t>태양광</t>
+          <t>국전</t>
         </is>
       </c>
       <c r="D33" s="19" t="n">
@@ -1739,18 +1741,18 @@
       <c r="G33" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="H33" s="19" t="n">
-        <v/>
-      </c>
-      <c r="I33" s="19" t="n">
-        <v/>
-      </c>
-      <c r="J33" s="23" t="inlineStr">
-        <is>
-          <t>매일경제 기사 언급 / 네이버뉴스 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K33" s="23" t="inlineStr">
+      <c r="H33" s="23" t="n">
+        <v>3.18</v>
+      </c>
+      <c r="I33" s="23" t="n">
+        <v>23.21</v>
+      </c>
+      <c r="J33" s="22" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +148% / 네이버뉴스 기사 언급</t>
+        </is>
+      </c>
+      <c r="K33" s="22" t="inlineStr">
         <is>
           <t>네이버</t>
         </is>
@@ -1759,7 +1761,7 @@
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="19" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B34" s="19" t="n">
@@ -1767,7 +1769,7 @@
       </c>
       <c r="C34" s="20" t="inlineStr">
         <is>
-          <t>수소</t>
+          <t>대성산업</t>
         </is>
       </c>
       <c r="D34" s="19" t="n">
@@ -1782,25 +1784,27 @@
       <c r="G34" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="H34" s="19" t="n">
-        <v/>
-      </c>
-      <c r="I34" s="19" t="n">
-        <v/>
-      </c>
-      <c r="J34" s="23" t="inlineStr">
-        <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K34" s="23" t="n">
-        <v/>
+      <c r="H34" s="21" t="n">
+        <v>-9.98</v>
+      </c>
+      <c r="I34" s="23" t="n">
+        <v>8.84</v>
+      </c>
+      <c r="J34" s="22" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +110% / 중요공시 2건</t>
+        </is>
+      </c>
+      <c r="K34" s="22" t="inlineStr">
+        <is>
+          <t>공시, 네이버</t>
+        </is>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="19" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B35" s="19" t="n">
@@ -1808,7 +1812,7 @@
       </c>
       <c r="C35" s="20" t="inlineStr">
         <is>
-          <t>클라우드</t>
+          <t>삼성전기</t>
         </is>
       </c>
       <c r="D35" s="19" t="n">
@@ -1823,70 +1827,68 @@
       <c r="G35" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="H35" s="19" t="n">
+      <c r="H35" s="21" t="n">
+        <v>-2.99</v>
+      </c>
+      <c r="I35" s="21" t="n">
+        <v>-1.14</v>
+      </c>
+      <c r="J35" s="22" t="inlineStr">
+        <is>
+          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K35" s="22" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="18" customHeight="1">
+      <c r="A36" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B36" s="19" t="n">
+        <v>23</v>
+      </c>
+      <c r="C36" s="20" t="inlineStr">
+        <is>
+          <t>전기차</t>
+        </is>
+      </c>
+      <c r="D36" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="E36" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="F36" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" s="19" t="n">
         <v/>
       </c>
-      <c r="I35" s="19" t="n">
+      <c r="I36" s="19" t="n">
         <v/>
       </c>
-      <c r="J35" s="23" t="inlineStr">
-        <is>
-          <t>한국경제 헤드라인 언급 / 네이버뉴스 기사 언급</t>
-        </is>
-      </c>
-      <c r="K35" s="23" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="18" customHeight="1">
-      <c r="A36" s="24" t="inlineStr">
-        <is>
-          <t>2026-10-11</t>
-        </is>
-      </c>
-      <c r="B36" s="24" t="n">
-        <v>23</v>
-      </c>
-      <c r="C36" s="25" t="inlineStr">
-        <is>
-          <t>빅텐츠</t>
-        </is>
-      </c>
-      <c r="D36" s="24" t="n">
-        <v>3</v>
-      </c>
-      <c r="E36" s="24" t="n">
-        <v>3</v>
-      </c>
-      <c r="F36" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="G36" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="H36" s="26" t="n">
-        <v>-18.27</v>
-      </c>
-      <c r="I36" s="26" t="n">
-        <v>-13.73</v>
-      </c>
-      <c r="J36" s="27" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +51107%</t>
-        </is>
-      </c>
-      <c r="K36" s="27" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+      <c r="J36" s="22" t="inlineStr">
+        <is>
+          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K36" s="22" t="n">
+        <v/>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B37" s="24" t="n">
@@ -1894,7 +1896,7 @@
       </c>
       <c r="C37" s="25" t="inlineStr">
         <is>
-          <t>국제약품</t>
+          <t>비아트론</t>
         </is>
       </c>
       <c r="D37" s="24" t="n">
@@ -1910,17 +1912,17 @@
         <v>0</v>
       </c>
       <c r="H37" s="26" t="n">
-        <v>-4.4</v>
-      </c>
-      <c r="I37" s="28" t="n">
-        <v>30.31</v>
-      </c>
-      <c r="J37" s="27" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +980%</t>
-        </is>
-      </c>
-      <c r="K37" s="27" t="inlineStr">
+        <v>-9.609999999999999</v>
+      </c>
+      <c r="I37" s="27" t="n">
+        <v>18.71</v>
+      </c>
+      <c r="J37" s="28" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +304%</t>
+        </is>
+      </c>
+      <c r="K37" s="28" t="inlineStr">
         <is>
           <t>네이버</t>
         </is>
@@ -1929,7 +1931,7 @@
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B38" s="24" t="n">
@@ -1937,7 +1939,7 @@
       </c>
       <c r="C38" s="25" t="inlineStr">
         <is>
-          <t>비아트론</t>
+          <t>녹십자엠에스</t>
         </is>
       </c>
       <c r="D38" s="24" t="n">
@@ -1953,17 +1955,17 @@
         <v>0</v>
       </c>
       <c r="H38" s="26" t="n">
-        <v>-9.609999999999999</v>
-      </c>
-      <c r="I38" s="28" t="n">
-        <v>25.09</v>
-      </c>
-      <c r="J38" s="27" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +269%</t>
-        </is>
-      </c>
-      <c r="K38" s="27" t="inlineStr">
+        <v>-14.53</v>
+      </c>
+      <c r="I38" s="27" t="n">
+        <v>9.869999999999999</v>
+      </c>
+      <c r="J38" s="28" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +214%</t>
+        </is>
+      </c>
+      <c r="K38" s="28" t="inlineStr">
         <is>
           <t>네이버</t>
         </is>
@@ -1972,7 +1974,7 @@
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B39" s="24" t="n">
@@ -1980,7 +1982,7 @@
       </c>
       <c r="C39" s="25" t="inlineStr">
         <is>
-          <t>녹십자엠에스</t>
+          <t>라온시큐어</t>
         </is>
       </c>
       <c r="D39" s="24" t="n">
@@ -1996,17 +1998,17 @@
         <v>0</v>
       </c>
       <c r="H39" s="26" t="n">
-        <v>-14.53</v>
-      </c>
-      <c r="I39" s="28" t="n">
-        <v>9.539999999999999</v>
-      </c>
-      <c r="J39" s="27" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +200%</t>
-        </is>
-      </c>
-      <c r="K39" s="27" t="inlineStr">
+        <v>-5.14</v>
+      </c>
+      <c r="I39" s="27" t="n">
+        <v>31.22</v>
+      </c>
+      <c r="J39" s="28" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +207%</t>
+        </is>
+      </c>
+      <c r="K39" s="28" t="inlineStr">
         <is>
           <t>네이버</t>
         </is>
@@ -2015,7 +2017,7 @@
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B40" s="24" t="n">
@@ -2023,7 +2025,7 @@
       </c>
       <c r="C40" s="25" t="inlineStr">
         <is>
-          <t>라온시큐어</t>
+          <t>아톤</t>
         </is>
       </c>
       <c r="D40" s="24" t="n">
@@ -2039,17 +2041,17 @@
         <v>0</v>
       </c>
       <c r="H40" s="26" t="n">
-        <v>-5.14</v>
-      </c>
-      <c r="I40" s="28" t="n">
-        <v>38.73</v>
-      </c>
-      <c r="J40" s="27" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +195%</t>
-        </is>
-      </c>
-      <c r="K40" s="27" t="inlineStr">
+        <v>-3.4</v>
+      </c>
+      <c r="I40" s="27" t="n">
+        <v>14.76</v>
+      </c>
+      <c r="J40" s="28" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +192%</t>
+        </is>
+      </c>
+      <c r="K40" s="28" t="inlineStr">
         <is>
           <t>네이버</t>
         </is>
@@ -2058,7 +2060,7 @@
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B41" s="24" t="n">
@@ -2066,7 +2068,7 @@
       </c>
       <c r="C41" s="25" t="inlineStr">
         <is>
-          <t>아톤</t>
+          <t>삼표시멘트</t>
         </is>
       </c>
       <c r="D41" s="24" t="n">
@@ -2082,17 +2084,17 @@
         <v>0</v>
       </c>
       <c r="H41" s="26" t="n">
-        <v>-3.4</v>
-      </c>
-      <c r="I41" s="28" t="n">
-        <v>21.15</v>
-      </c>
-      <c r="J41" s="27" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +184%</t>
-        </is>
-      </c>
-      <c r="K41" s="27" t="inlineStr">
+        <v>-12.77</v>
+      </c>
+      <c r="I41" s="26" t="n">
+        <v>-0.29</v>
+      </c>
+      <c r="J41" s="28" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +178%</t>
+        </is>
+      </c>
+      <c r="K41" s="28" t="inlineStr">
         <is>
           <t>네이버</t>
         </is>
@@ -2101,7 +2103,7 @@
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B42" s="24" t="n">
@@ -2109,7 +2111,7 @@
       </c>
       <c r="C42" s="25" t="inlineStr">
         <is>
-          <t>국전</t>
+          <t>SM C&amp;C</t>
         </is>
       </c>
       <c r="D42" s="24" t="n">
@@ -2124,18 +2126,18 @@
       <c r="G42" s="24" t="n">
         <v>0</v>
       </c>
-      <c r="H42" s="28" t="n">
-        <v>3.18</v>
-      </c>
-      <c r="I42" s="28" t="n">
-        <v>24.26</v>
-      </c>
-      <c r="J42" s="27" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +128%</t>
-        </is>
-      </c>
-      <c r="K42" s="27" t="inlineStr">
+      <c r="H42" s="26" t="n">
+        <v>-7.86</v>
+      </c>
+      <c r="I42" s="26" t="n">
+        <v>-13.42</v>
+      </c>
+      <c r="J42" s="28" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +120%</t>
+        </is>
+      </c>
+      <c r="K42" s="28" t="inlineStr">
         <is>
           <t>네이버</t>
         </is>
@@ -2144,7 +2146,7 @@
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B43" s="24" t="n">
@@ -2152,7 +2154,7 @@
       </c>
       <c r="C43" s="25" t="inlineStr">
         <is>
-          <t>대성산업</t>
+          <t>HLB바이오스텝</t>
         </is>
       </c>
       <c r="D43" s="24" t="n">
@@ -2167,18 +2169,18 @@
       <c r="G43" s="24" t="n">
         <v>0</v>
       </c>
-      <c r="H43" s="26" t="n">
-        <v>-9.98</v>
-      </c>
-      <c r="I43" s="28" t="n">
-        <v>10.69</v>
-      </c>
-      <c r="J43" s="27" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +102%</t>
-        </is>
-      </c>
-      <c r="K43" s="27" t="inlineStr">
+      <c r="H43" s="27" t="n">
+        <v>29.97</v>
+      </c>
+      <c r="I43" s="27" t="n">
+        <v>118.72</v>
+      </c>
+      <c r="J43" s="28" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +108%</t>
+        </is>
+      </c>
+      <c r="K43" s="28" t="inlineStr">
         <is>
           <t>네이버</t>
         </is>
@@ -2187,7 +2189,7 @@
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B44" s="24" t="n">
@@ -2195,7 +2197,7 @@
       </c>
       <c r="C44" s="25" t="inlineStr">
         <is>
-          <t>DB</t>
+          <t>에이엔피</t>
         </is>
       </c>
       <c r="D44" s="24" t="n">
@@ -2210,25 +2212,27 @@
       <c r="G44" s="24" t="n">
         <v>0</v>
       </c>
-      <c r="H44" s="28" t="n">
-        <v>12.72</v>
-      </c>
-      <c r="I44" s="28" t="n">
-        <v>12.44</v>
-      </c>
-      <c r="J44" s="27" t="inlineStr">
-        <is>
-          <t>매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K44" s="27" t="n">
-        <v/>
+      <c r="H44" s="27" t="n">
+        <v>29.69</v>
+      </c>
+      <c r="I44" s="27" t="n">
+        <v>23.27</v>
+      </c>
+      <c r="J44" s="28" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +51% / 중요공시 1건</t>
+        </is>
+      </c>
+      <c r="K44" s="28" t="inlineStr">
+        <is>
+          <t>공시, 네이버</t>
+        </is>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B45" s="24" t="n">
@@ -2236,7 +2240,7 @@
       </c>
       <c r="C45" s="25" t="inlineStr">
         <is>
-          <t>카카오</t>
+          <t>스피어</t>
         </is>
       </c>
       <c r="D45" s="24" t="n">
@@ -2251,27 +2255,27 @@
       <c r="G45" s="24" t="n">
         <v>0</v>
       </c>
-      <c r="H45" s="26" t="n">
-        <v>-1.52</v>
-      </c>
-      <c r="I45" s="26" t="n">
-        <v>-3.57</v>
-      </c>
-      <c r="J45" s="27" t="inlineStr">
-        <is>
-          <t>네이버뉴스 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K45" s="27" t="inlineStr">
-        <is>
-          <t>네이버</t>
+      <c r="H45" s="27" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="I45" s="27" t="n">
+        <v>2.83</v>
+      </c>
+      <c r="J45" s="28" t="inlineStr">
+        <is>
+          <t>중요공시 3건</t>
+        </is>
+      </c>
+      <c r="K45" s="28" t="inlineStr">
+        <is>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B46" s="24" t="n">
@@ -2279,7 +2283,7 @@
       </c>
       <c r="C46" s="25" t="inlineStr">
         <is>
-          <t>조선</t>
+          <t>우원개발</t>
         </is>
       </c>
       <c r="D46" s="24" t="n">
@@ -2294,25 +2298,27 @@
       <c r="G46" s="24" t="n">
         <v>0</v>
       </c>
-      <c r="H46" s="24" t="n">
-        <v/>
-      </c>
-      <c r="I46" s="24" t="n">
-        <v/>
-      </c>
-      <c r="J46" s="27" t="inlineStr">
-        <is>
-          <t>매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K46" s="27" t="n">
-        <v/>
+      <c r="H46" s="27" t="n">
+        <v>2.74</v>
+      </c>
+      <c r="I46" s="27" t="n">
+        <v>1.81</v>
+      </c>
+      <c r="J46" s="28" t="inlineStr">
+        <is>
+          <t>중요공시 3건</t>
+        </is>
+      </c>
+      <c r="K46" s="28" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B47" s="24" t="n">
@@ -2320,7 +2326,7 @@
       </c>
       <c r="C47" s="25" t="inlineStr">
         <is>
-          <t>유바이오로직스</t>
+          <t>DB</t>
         </is>
       </c>
       <c r="D47" s="24" t="n">
@@ -2335,25 +2341,25 @@
       <c r="G47" s="24" t="n">
         <v>0</v>
       </c>
-      <c r="H47" s="26" t="n">
-        <v>-0.47</v>
-      </c>
-      <c r="I47" s="26" t="n">
-        <v>-0.93</v>
-      </c>
-      <c r="J47" s="27" t="inlineStr">
+      <c r="H47" s="27" t="n">
+        <v>12.72</v>
+      </c>
+      <c r="I47" s="27" t="n">
+        <v>11.88</v>
+      </c>
+      <c r="J47" s="28" t="inlineStr">
         <is>
           <t>매일경제 헤드라인 언급</t>
         </is>
       </c>
-      <c r="K47" s="27" t="n">
+      <c r="K47" s="28" t="n">
         <v/>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B48" s="24" t="n">
@@ -2361,7 +2367,7 @@
       </c>
       <c r="C48" s="25" t="inlineStr">
         <is>
-          <t>SK스퀘어</t>
+          <t>삼성전자우</t>
         </is>
       </c>
       <c r="D48" s="24" t="n">
@@ -2377,24 +2383,26 @@
         <v>0</v>
       </c>
       <c r="H48" s="26" t="n">
-        <v>-6.78</v>
+        <v>-1.42</v>
       </c>
       <c r="I48" s="26" t="n">
-        <v>-7.91</v>
-      </c>
-      <c r="J48" s="27" t="inlineStr">
-        <is>
-          <t>매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K48" s="27" t="n">
-        <v/>
+        <v>-3.47</v>
+      </c>
+      <c r="J48" s="28" t="inlineStr">
+        <is>
+          <t>네이버뉴스 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K48" s="28" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B49" s="24" t="n">
@@ -2402,7 +2410,7 @@
       </c>
       <c r="C49" s="25" t="inlineStr">
         <is>
-          <t>한양디지텍</t>
+          <t>더코디</t>
         </is>
       </c>
       <c r="D49" s="24" t="n">
@@ -2417,25 +2425,27 @@
       <c r="G49" s="24" t="n">
         <v>0</v>
       </c>
-      <c r="H49" s="28" t="n">
-        <v>7.01</v>
-      </c>
-      <c r="I49" s="28" t="n">
-        <v>8.19</v>
-      </c>
-      <c r="J49" s="27" t="inlineStr">
-        <is>
-          <t>매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K49" s="27" t="n">
-        <v/>
+      <c r="H49" s="27" t="n">
+        <v>7.28</v>
+      </c>
+      <c r="I49" s="26" t="n">
+        <v>-15.36</v>
+      </c>
+      <c r="J49" s="28" t="inlineStr">
+        <is>
+          <t>중요공시 9건</t>
+        </is>
+      </c>
+      <c r="K49" s="28" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B50" s="24" t="n">
@@ -2443,7 +2453,7 @@
       </c>
       <c r="C50" s="25" t="inlineStr">
         <is>
-          <t>한컴</t>
+          <t>알테오젠</t>
         </is>
       </c>
       <c r="D50" s="24" t="n">
@@ -2459,24 +2469,26 @@
         <v>0</v>
       </c>
       <c r="H50" s="26" t="n">
-        <v>-1.48</v>
+        <v>-5.5</v>
       </c>
       <c r="I50" s="26" t="n">
-        <v>-0.4</v>
-      </c>
-      <c r="J50" s="27" t="inlineStr">
-        <is>
-          <t>한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K50" s="27" t="n">
-        <v/>
+        <v>-7.32</v>
+      </c>
+      <c r="J50" s="28" t="inlineStr">
+        <is>
+          <t>중요공시 6건</t>
+        </is>
+      </c>
+      <c r="K50" s="28" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B51" s="24" t="n">
@@ -2484,7 +2496,7 @@
       </c>
       <c r="C51" s="25" t="inlineStr">
         <is>
-          <t>SK이터닉스</t>
+          <t>엔켐</t>
         </is>
       </c>
       <c r="D51" s="24" t="n">
@@ -2500,24 +2512,26 @@
         <v>0</v>
       </c>
       <c r="H51" s="26" t="n">
-        <v>-5.71</v>
+        <v>-5.42</v>
       </c>
       <c r="I51" s="26" t="n">
-        <v>-6.48</v>
-      </c>
-      <c r="J51" s="27" t="inlineStr">
-        <is>
-          <t>매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K51" s="27" t="n">
-        <v/>
+        <v>-4.8</v>
+      </c>
+      <c r="J51" s="28" t="inlineStr">
+        <is>
+          <t>중요공시 3건</t>
+        </is>
+      </c>
+      <c r="K51" s="28" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B52" s="24" t="n">
@@ -2525,7 +2539,7 @@
       </c>
       <c r="C52" s="25" t="inlineStr">
         <is>
-          <t>동양</t>
+          <t>AI반도체</t>
         </is>
       </c>
       <c r="D52" s="24" t="n">
@@ -2540,25 +2554,25 @@
       <c r="G52" s="24" t="n">
         <v>0</v>
       </c>
-      <c r="H52" s="26" t="n">
-        <v>-0.45</v>
-      </c>
-      <c r="I52" s="26" t="n">
-        <v>-0.89</v>
-      </c>
-      <c r="J52" s="27" t="inlineStr">
-        <is>
-          <t>한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K52" s="27" t="n">
+      <c r="H52" s="24" t="n">
+        <v/>
+      </c>
+      <c r="I52" s="24" t="n">
+        <v/>
+      </c>
+      <c r="J52" s="28" t="inlineStr">
+        <is>
+          <t>매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K52" s="28" t="n">
         <v/>
       </c>
     </row>
     <row r="53" ht="18" customHeight="1">
       <c r="A53" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B53" s="24" t="n">
@@ -2566,7 +2580,7 @@
       </c>
       <c r="C53" s="25" t="inlineStr">
         <is>
-          <t>동양고속</t>
+          <t>한컴</t>
         </is>
       </c>
       <c r="D53" s="24" t="n">
@@ -2581,25 +2595,25 @@
       <c r="G53" s="24" t="n">
         <v>0</v>
       </c>
-      <c r="H53" s="28" t="n">
-        <v>27.18</v>
-      </c>
-      <c r="I53" s="28" t="n">
-        <v>58.3</v>
-      </c>
-      <c r="J53" s="27" t="inlineStr">
+      <c r="H53" s="26" t="n">
+        <v>-1.48</v>
+      </c>
+      <c r="I53" s="27" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="J53" s="28" t="inlineStr">
         <is>
           <t>한국경제 헤드라인 언급</t>
         </is>
       </c>
-      <c r="K53" s="27" t="n">
+      <c r="K53" s="28" t="n">
         <v/>
       </c>
     </row>
     <row r="54" ht="18" customHeight="1">
       <c r="A54" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B54" s="24" t="n">
@@ -2607,7 +2621,7 @@
       </c>
       <c r="C54" s="25" t="inlineStr">
         <is>
-          <t>한화오션</t>
+          <t>GS건설</t>
         </is>
       </c>
       <c r="D54" s="24" t="n">
@@ -2623,24 +2637,24 @@
         <v>0</v>
       </c>
       <c r="H54" s="26" t="n">
-        <v>-3.1</v>
+        <v>-3.05</v>
       </c>
       <c r="I54" s="26" t="n">
-        <v>-8.65</v>
-      </c>
-      <c r="J54" s="27" t="inlineStr">
+        <v>-4.07</v>
+      </c>
+      <c r="J54" s="28" t="inlineStr">
         <is>
           <t>한국경제 헤드라인 언급</t>
         </is>
       </c>
-      <c r="K54" s="27" t="n">
+      <c r="K54" s="28" t="n">
         <v/>
       </c>
     </row>
     <row r="55" ht="18" customHeight="1">
       <c r="A55" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B55" s="24" t="n">
@@ -2648,7 +2662,7 @@
       </c>
       <c r="C55" s="25" t="inlineStr">
         <is>
-          <t>삼성생명</t>
+          <t>철강</t>
         </is>
       </c>
       <c r="D55" s="24" t="n">
@@ -2663,25 +2677,25 @@
       <c r="G55" s="24" t="n">
         <v>0</v>
       </c>
-      <c r="H55" s="26" t="n">
-        <v>-3.05</v>
-      </c>
-      <c r="I55" s="26" t="n">
-        <v>-4.42</v>
-      </c>
-      <c r="J55" s="27" t="inlineStr">
-        <is>
-          <t>매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K55" s="27" t="n">
+      <c r="H55" s="24" t="n">
+        <v/>
+      </c>
+      <c r="I55" s="24" t="n">
+        <v/>
+      </c>
+      <c r="J55" s="28" t="inlineStr">
+        <is>
+          <t>매일경제 기사 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K55" s="28" t="n">
         <v/>
       </c>
     </row>
     <row r="56" ht="18" customHeight="1">
       <c r="A56" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B56" s="24" t="n">
@@ -2689,14 +2703,14 @@
       </c>
       <c r="C56" s="25" t="inlineStr">
         <is>
-          <t>HLB바이오스텝</t>
+          <t>TSMC</t>
         </is>
       </c>
       <c r="D56" s="24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E56" s="24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F56" s="24" t="n">
         <v>0</v>
@@ -2704,27 +2718,25 @@
       <c r="G56" s="24" t="n">
         <v>0</v>
       </c>
-      <c r="H56" s="28" t="n">
-        <v>29.97</v>
-      </c>
-      <c r="I56" s="28" t="n">
-        <v>108.25</v>
-      </c>
-      <c r="J56" s="27" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +99%</t>
-        </is>
-      </c>
-      <c r="K56" s="27" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+      <c r="H56" s="24" t="n">
+        <v/>
+      </c>
+      <c r="I56" s="24" t="n">
+        <v/>
+      </c>
+      <c r="J56" s="28" t="inlineStr">
+        <is>
+          <t>한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K56" s="28" t="n">
+        <v/>
       </c>
     </row>
     <row r="57" ht="18" customHeight="1">
       <c r="A57" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B57" s="24" t="n">
@@ -2747,18 +2759,18 @@
       <c r="G57" s="24" t="n">
         <v>0</v>
       </c>
-      <c r="H57" s="28" t="n">
+      <c r="H57" s="27" t="n">
         <v>20.23</v>
       </c>
-      <c r="I57" s="28" t="n">
-        <v>37.95</v>
-      </c>
-      <c r="J57" s="27" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +51%</t>
-        </is>
-      </c>
-      <c r="K57" s="27" t="inlineStr">
+      <c r="I57" s="27" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="J57" s="28" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +62%</t>
+        </is>
+      </c>
+      <c r="K57" s="28" t="inlineStr">
         <is>
           <t>네이버</t>
         </is>
@@ -2767,7 +2779,7 @@
     <row r="58" ht="18" customHeight="1">
       <c r="A58" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B58" s="24" t="n">
@@ -2790,18 +2802,18 @@
       <c r="G58" s="24" t="n">
         <v>0</v>
       </c>
-      <c r="H58" s="28" t="n">
+      <c r="H58" s="27" t="n">
         <v>6.55</v>
       </c>
-      <c r="I58" s="28" t="n">
-        <v>12.16</v>
-      </c>
-      <c r="J58" s="27" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +51%</t>
-        </is>
-      </c>
-      <c r="K58" s="27" t="inlineStr">
+      <c r="I58" s="27" t="n">
+        <v>10.02</v>
+      </c>
+      <c r="J58" s="28" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +59%</t>
+        </is>
+      </c>
+      <c r="K58" s="28" t="inlineStr">
         <is>
           <t>네이버</t>
         </is>
@@ -2810,7 +2822,7 @@
     <row r="59" ht="18" customHeight="1">
       <c r="A59" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B59" s="24" t="n">
@@ -2818,7 +2830,7 @@
       </c>
       <c r="C59" s="25" t="inlineStr">
         <is>
-          <t>HPSP</t>
+          <t>빛과전자</t>
         </is>
       </c>
       <c r="D59" s="24" t="n">
@@ -2834,24 +2846,26 @@
         <v>0</v>
       </c>
       <c r="H59" s="26" t="n">
-        <v>-2.44</v>
-      </c>
-      <c r="I59" s="26" t="n">
-        <v>-8.050000000000001</v>
-      </c>
-      <c r="J59" s="27" t="inlineStr">
-        <is>
-          <t>매일경제 기사 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K59" s="27" t="n">
-        <v/>
+        <v>-4.49</v>
+      </c>
+      <c r="I59" s="27" t="n">
+        <v>11.14</v>
+      </c>
+      <c r="J59" s="28" t="inlineStr">
+        <is>
+          <t>중요공시 1건</t>
+        </is>
+      </c>
+      <c r="K59" s="28" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="60" ht="18" customHeight="1">
       <c r="A60" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B60" s="24" t="n">
@@ -2859,7 +2873,7 @@
       </c>
       <c r="C60" s="25" t="inlineStr">
         <is>
-          <t>삼성SDI</t>
+          <t>한화머시너리앤서비스홀딩스</t>
         </is>
       </c>
       <c r="D60" s="24" t="n">
@@ -2874,25 +2888,27 @@
       <c r="G60" s="24" t="n">
         <v>0</v>
       </c>
-      <c r="H60" s="28" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="I60" s="28" t="n">
-        <v>9.67</v>
-      </c>
-      <c r="J60" s="27" t="inlineStr">
-        <is>
-          <t>매일경제 기사 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K60" s="27" t="n">
-        <v/>
+      <c r="H60" s="26" t="n">
+        <v>-0.16</v>
+      </c>
+      <c r="I60" s="27" t="n">
+        <v>7.76</v>
+      </c>
+      <c r="J60" s="28" t="inlineStr">
+        <is>
+          <t>중요공시 1건 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K60" s="28" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="61" ht="18" customHeight="1">
       <c r="A61" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B61" s="24" t="n">
@@ -2900,7 +2916,7 @@
       </c>
       <c r="C61" s="25" t="inlineStr">
         <is>
-          <t>한미약품</t>
+          <t>HPSP</t>
         </is>
       </c>
       <c r="D61" s="24" t="n">
@@ -2916,26 +2932,24 @@
         <v>0</v>
       </c>
       <c r="H61" s="26" t="n">
-        <v>-9.74</v>
+        <v>-2.44</v>
       </c>
       <c r="I61" s="26" t="n">
-        <v>-3.6</v>
-      </c>
-      <c r="J61" s="27" t="inlineStr">
-        <is>
-          <t>네이버뉴스 기사 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K61" s="27" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+        <v>-3.32</v>
+      </c>
+      <c r="J61" s="28" t="inlineStr">
+        <is>
+          <t>매일경제 기사 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K61" s="28" t="n">
+        <v/>
       </c>
     </row>
     <row r="62" ht="18" customHeight="1">
       <c r="A62" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B62" s="24" t="n">
@@ -2943,7 +2957,7 @@
       </c>
       <c r="C62" s="25" t="inlineStr">
         <is>
-          <t>현대지에프홀딩스</t>
+          <t>한미반도체</t>
         </is>
       </c>
       <c r="D62" s="24" t="n">
@@ -2958,25 +2972,27 @@
       <c r="G62" s="24" t="n">
         <v>0</v>
       </c>
-      <c r="H62" s="28" t="n">
-        <v>4.73</v>
-      </c>
-      <c r="I62" s="28" t="n">
-        <v>2.15</v>
-      </c>
-      <c r="J62" s="27" t="inlineStr">
-        <is>
-          <t>한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K62" s="27" t="n">
-        <v/>
+      <c r="H62" s="26" t="n">
+        <v>-0.38</v>
+      </c>
+      <c r="I62" s="26" t="n">
+        <v>-3.31</v>
+      </c>
+      <c r="J62" s="28" t="inlineStr">
+        <is>
+          <t>중요공시 1건 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K62" s="28" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="63" ht="18" customHeight="1">
       <c r="A63" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B63" s="24" t="n">
@@ -2984,14 +3000,14 @@
       </c>
       <c r="C63" s="25" t="inlineStr">
         <is>
-          <t>KT</t>
+          <t>제이앤티씨</t>
         </is>
       </c>
       <c r="D63" s="24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E63" s="24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F63" s="24" t="n">
         <v>0</v>
@@ -2999,18 +3015,16 @@
       <c r="G63" s="24" t="n">
         <v>0</v>
       </c>
-      <c r="H63" s="28" t="n">
-        <v>0.39</v>
-      </c>
-      <c r="I63" s="26" t="n">
-        <v>-1.16</v>
-      </c>
-      <c r="J63" s="27" t="inlineStr">
-        <is>
-          <t>한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K63" s="27" t="n">
+      <c r="H63" s="27" t="n">
+        <v>5.26</v>
+      </c>
+      <c r="I63" s="27" t="n">
+        <v>23.85</v>
+      </c>
+      <c r="J63" s="28" t="n">
+        <v/>
+      </c>
+      <c r="K63" s="28" t="n">
         <v/>
       </c>
     </row>
@@ -3107,22 +3121,22 @@
         <v>1</v>
       </c>
       <c r="C3" s="24" t="n">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D3" s="24" t="n">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E3" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F3" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G3" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="H3" s="24" t="n"/>
@@ -3138,29 +3152,29 @@
         <v>1</v>
       </c>
       <c r="C4" s="24" t="n">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="D4" s="24" t="n">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="E4" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F4" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G4" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="H4" s="26" t="n">
         <v>-2.23</v>
       </c>
       <c r="I4" s="26" t="n">
-        <v>-4.19</v>
+        <v>-4.71</v>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
@@ -3173,22 +3187,22 @@
         <v>1</v>
       </c>
       <c r="C5" s="24" t="n">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D5" s="24" t="n">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="E5" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F5" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G5" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="H5" s="24" t="n"/>
@@ -3197,227 +3211,231 @@
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="25" t="inlineStr">
         <is>
-          <t>전기차</t>
+          <t>LG</t>
         </is>
       </c>
       <c r="B6" s="24" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="24" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="D6" s="24" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E6" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F6" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G6" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
-        </is>
-      </c>
-      <c r="H6" s="24" t="n"/>
-      <c r="I6" s="24" t="n"/>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="H6" s="26" t="n">
+        <v>-1.9</v>
+      </c>
+      <c r="I6" s="26" t="n">
+        <v>-2.69</v>
+      </c>
     </row>
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="25" t="inlineStr">
         <is>
-          <t>LG</t>
+          <t>조선</t>
         </is>
       </c>
       <c r="B7" s="24" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="24" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D7" s="24" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E7" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F7" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G7" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
-        </is>
-      </c>
-      <c r="H7" s="26" t="n">
-        <v>-1.9</v>
-      </c>
-      <c r="I7" s="26" t="n">
-        <v>-1.28</v>
-      </c>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="H7" s="24" t="n"/>
+      <c r="I7" s="24" t="n"/>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="25" t="inlineStr">
         <is>
-          <t>SK하이닉스</t>
+          <t>방산</t>
         </is>
       </c>
       <c r="B8" s="24" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="24" t="n">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="D8" s="24" t="n">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="E8" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F8" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G8" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
-        </is>
-      </c>
-      <c r="H8" s="26" t="n">
-        <v>-1.69</v>
-      </c>
-      <c r="I8" s="26" t="n">
-        <v>-7.77</v>
-      </c>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="H8" s="24" t="n"/>
+      <c r="I8" s="24" t="n"/>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="25" t="inlineStr">
         <is>
-          <t>LG전자</t>
+          <t>현대차</t>
         </is>
       </c>
       <c r="B9" s="24" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="24" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D9" s="24" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E9" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F9" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G9" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="H9" s="26" t="n">
-        <v>-3.83</v>
+        <v>-3.57</v>
       </c>
       <c r="I9" s="26" t="n">
-        <v>-5.19</v>
+        <v>-6.48</v>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="25" t="inlineStr">
         <is>
-          <t>바이오</t>
+          <t>LG전자</t>
         </is>
       </c>
       <c r="B10" s="24" t="n">
         <v>1</v>
       </c>
       <c r="C10" s="24" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="D10" s="24" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E10" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F10" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G10" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
-        </is>
-      </c>
-      <c r="H10" s="24" t="n"/>
-      <c r="I10" s="24" t="n"/>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="H10" s="26" t="n">
+        <v>-3.83</v>
+      </c>
+      <c r="I10" s="26" t="n">
+        <v>-6.73</v>
+      </c>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="25" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>SK하이닉스</t>
         </is>
       </c>
       <c r="B11" s="24" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="24" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D11" s="24" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E11" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F11" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G11" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
-        </is>
-      </c>
-      <c r="H11" s="24" t="n"/>
-      <c r="I11" s="24" t="n"/>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="H11" s="26" t="n">
+        <v>-1.69</v>
+      </c>
+      <c r="I11" s="26" t="n">
+        <v>-8.470000000000001</v>
+      </c>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="25" t="inlineStr">
         <is>
-          <t>방산</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="B12" s="24" t="n">
         <v>1</v>
       </c>
       <c r="C12" s="24" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D12" s="24" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E12" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F12" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G12" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="H12" s="24" t="n"/>
@@ -3426,42 +3444,38 @@
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="25" t="inlineStr">
         <is>
-          <t>현대차</t>
+          <t>바이오</t>
         </is>
       </c>
       <c r="B13" s="24" t="n">
         <v>1</v>
       </c>
       <c r="C13" s="24" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D13" s="24" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E13" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F13" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G13" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
-        </is>
-      </c>
-      <c r="H13" s="26" t="n">
-        <v>-3.57</v>
-      </c>
-      <c r="I13" s="26" t="n">
-        <v>-7.02</v>
-      </c>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="H13" s="24" t="n"/>
+      <c r="I13" s="24" t="n"/>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="25" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>GS</t>
         </is>
       </c>
       <c r="B14" s="24" t="n">
@@ -3478,21 +3492,25 @@
       </c>
       <c r="F14" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G14" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
-        </is>
-      </c>
-      <c r="H14" s="24" t="n"/>
-      <c r="I14" s="24" t="n"/>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="H14" s="26" t="n">
+        <v>-4.55</v>
+      </c>
+      <c r="I14" s="26" t="n">
+        <v>-0.29</v>
+      </c>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="25" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="B15" s="24" t="n">
@@ -3509,12 +3527,12 @@
       </c>
       <c r="F15" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G15" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="H15" s="24" t="n"/>
@@ -3523,7 +3541,7 @@
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="25" t="inlineStr">
         <is>
-          <t>AI반도체</t>
+          <t>빅텐츠</t>
         </is>
       </c>
       <c r="B16" s="24" t="n">
@@ -3540,91 +3558,91 @@
       </c>
       <c r="F16" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G16" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
-        </is>
-      </c>
-      <c r="H16" s="24" t="n"/>
-      <c r="I16" s="24" t="n"/>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="H16" s="26" t="n">
+        <v>-18.27</v>
+      </c>
+      <c r="I16" s="26" t="n">
+        <v>-11.47</v>
+      </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="25" t="inlineStr">
         <is>
-          <t>삼표시멘트</t>
+          <t>기업은행</t>
         </is>
       </c>
       <c r="B17" s="24" t="n">
         <v>1</v>
       </c>
       <c r="C17" s="24" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D17" s="24" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E17" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F17" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G17" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="H17" s="26" t="n">
-        <v>-12.77</v>
-      </c>
-      <c r="I17" s="28" t="n">
-        <v>1.19</v>
+        <v>-1</v>
+      </c>
+      <c r="I17" s="26" t="n">
+        <v>-1.97</v>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="25" t="inlineStr">
         <is>
-          <t>주성엔지니어링</t>
+          <t>원전</t>
         </is>
       </c>
       <c r="B18" s="24" t="n">
         <v>1</v>
       </c>
       <c r="C18" s="24" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D18" s="24" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E18" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F18" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G18" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
-        </is>
-      </c>
-      <c r="H18" s="28" t="n">
-        <v>4.77</v>
-      </c>
-      <c r="I18" s="28" t="n">
-        <v>9.56</v>
-      </c>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="H18" s="24" t="n"/>
+      <c r="I18" s="24" t="n"/>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="25" t="inlineStr">
         <is>
-          <t>SG</t>
+          <t>주성엔지니어링</t>
         </is>
       </c>
       <c r="B19" s="24" t="n">
@@ -3641,25 +3659,25 @@
       </c>
       <c r="F19" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G19" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
-        </is>
-      </c>
-      <c r="H19" s="26" t="n">
-        <v>-3.87</v>
-      </c>
-      <c r="I19" s="26" t="n">
-        <v>-10.47</v>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="H19" s="27" t="n">
+        <v>4.77</v>
+      </c>
+      <c r="I19" s="27" t="n">
+        <v>10.02</v>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="25" t="inlineStr">
         <is>
-          <t>TSMC</t>
+          <t>한화오션</t>
         </is>
       </c>
       <c r="B20" s="24" t="n">
@@ -3676,56 +3694,60 @@
       </c>
       <c r="F20" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G20" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
-        </is>
-      </c>
-      <c r="H20" s="24" t="n"/>
-      <c r="I20" s="24" t="n"/>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="H20" s="26" t="n">
+        <v>-3.1</v>
+      </c>
+      <c r="I20" s="26" t="n">
+        <v>-8.77</v>
+      </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="25" t="inlineStr">
         <is>
-          <t>삼성전기</t>
+          <t>국전</t>
         </is>
       </c>
       <c r="B21" s="24" t="n">
         <v>1</v>
       </c>
       <c r="C21" s="24" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D21" s="24" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E21" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F21" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G21" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
-        </is>
-      </c>
-      <c r="H21" s="26" t="n">
-        <v>-2.99</v>
-      </c>
-      <c r="I21" s="28" t="n">
-        <v>0.32</v>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="H21" s="27" t="n">
+        <v>3.18</v>
+      </c>
+      <c r="I21" s="27" t="n">
+        <v>23.21</v>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="25" t="inlineStr">
         <is>
-          <t>수소</t>
+          <t>국제약품</t>
         </is>
       </c>
       <c r="B22" s="24" t="n">
@@ -3742,21 +3764,25 @@
       </c>
       <c r="F22" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G22" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
-        </is>
-      </c>
-      <c r="H22" s="24" t="n"/>
-      <c r="I22" s="24" t="n"/>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="H22" s="26" t="n">
+        <v>-4.4</v>
+      </c>
+      <c r="I22" s="27" t="n">
+        <v>28.14</v>
+      </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="25" t="inlineStr">
         <is>
-          <t>클라우드</t>
+          <t>대성산업</t>
         </is>
       </c>
       <c r="B23" s="24" t="n">
@@ -3773,21 +3799,25 @@
       </c>
       <c r="F23" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G23" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
-        </is>
-      </c>
-      <c r="H23" s="24" t="n"/>
-      <c r="I23" s="24" t="n"/>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="H23" s="26" t="n">
+        <v>-9.98</v>
+      </c>
+      <c r="I23" s="27" t="n">
+        <v>8.84</v>
+      </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="25" t="inlineStr">
         <is>
-          <t>태양광</t>
+          <t>삼성전기</t>
         </is>
       </c>
       <c r="B24" s="24" t="n">
@@ -3804,56 +3834,56 @@
       </c>
       <c r="F24" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G24" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
-        </is>
-      </c>
-      <c r="H24" s="24" t="n"/>
-      <c r="I24" s="24" t="n"/>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="H24" s="26" t="n">
+        <v>-2.99</v>
+      </c>
+      <c r="I24" s="26" t="n">
+        <v>-1.14</v>
+      </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="25" t="inlineStr">
         <is>
-          <t>DB</t>
+          <t>전기차</t>
         </is>
       </c>
       <c r="B25" s="24" t="n">
         <v>1</v>
       </c>
       <c r="C25" s="24" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D25" s="24" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E25" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F25" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G25" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
-        </is>
-      </c>
-      <c r="H25" s="28" t="n">
-        <v>12.72</v>
-      </c>
-      <c r="I25" s="28" t="n">
-        <v>12.44</v>
-      </c>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="H25" s="24" t="n"/>
+      <c r="I25" s="24" t="n"/>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="25" t="inlineStr">
         <is>
-          <t>SK스퀘어</t>
+          <t>AI반도체</t>
         </is>
       </c>
       <c r="B26" s="24" t="n">
@@ -3870,25 +3900,21 @@
       </c>
       <c r="F26" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G26" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
-        </is>
-      </c>
-      <c r="H26" s="26" t="n">
-        <v>-6.78</v>
-      </c>
-      <c r="I26" s="26" t="n">
-        <v>-7.91</v>
-      </c>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="H26" s="24" t="n"/>
+      <c r="I26" s="24" t="n"/>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="25" t="inlineStr">
         <is>
-          <t>SK이터닉스</t>
+          <t>DB</t>
         </is>
       </c>
       <c r="B27" s="24" t="n">
@@ -3905,25 +3931,25 @@
       </c>
       <c r="F27" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G27" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
-        </is>
-      </c>
-      <c r="H27" s="26" t="n">
-        <v>-5.71</v>
-      </c>
-      <c r="I27" s="26" t="n">
-        <v>-6.48</v>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="H27" s="27" t="n">
+        <v>12.72</v>
+      </c>
+      <c r="I27" s="27" t="n">
+        <v>11.88</v>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="25" t="inlineStr">
         <is>
-          <t>국전</t>
+          <t>GS건설</t>
         </is>
       </c>
       <c r="B28" s="24" t="n">
@@ -3940,25 +3966,25 @@
       </c>
       <c r="F28" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G28" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
-        </is>
-      </c>
-      <c r="H28" s="28" t="n">
-        <v>3.18</v>
-      </c>
-      <c r="I28" s="28" t="n">
-        <v>24.26</v>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="H28" s="26" t="n">
+        <v>-3.05</v>
+      </c>
+      <c r="I28" s="26" t="n">
+        <v>-4.07</v>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="25" t="inlineStr">
         <is>
-          <t>국제약품</t>
+          <t>HLB바이오스텝</t>
         </is>
       </c>
       <c r="B29" s="24" t="n">
@@ -3975,25 +4001,25 @@
       </c>
       <c r="F29" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G29" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
-        </is>
-      </c>
-      <c r="H29" s="26" t="n">
-        <v>-4.4</v>
-      </c>
-      <c r="I29" s="28" t="n">
-        <v>30.31</v>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="H29" s="27" t="n">
+        <v>29.97</v>
+      </c>
+      <c r="I29" s="27" t="n">
+        <v>118.72</v>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="25" t="inlineStr">
         <is>
-          <t>녹십자엠에스</t>
+          <t>SM C&amp;C</t>
         </is>
       </c>
       <c r="B30" s="24" t="n">
@@ -4010,25 +4036,25 @@
       </c>
       <c r="F30" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G30" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="H30" s="26" t="n">
-        <v>-14.53</v>
-      </c>
-      <c r="I30" s="28" t="n">
-        <v>9.539999999999999</v>
+        <v>-7.86</v>
+      </c>
+      <c r="I30" s="26" t="n">
+        <v>-13.42</v>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="25" t="inlineStr">
         <is>
-          <t>대성산업</t>
+          <t>TSMC</t>
         </is>
       </c>
       <c r="B31" s="24" t="n">
@@ -4045,25 +4071,21 @@
       </c>
       <c r="F31" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G31" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
-        </is>
-      </c>
-      <c r="H31" s="26" t="n">
-        <v>-9.98</v>
-      </c>
-      <c r="I31" s="28" t="n">
-        <v>10.69</v>
-      </c>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="H31" s="24" t="n"/>
+      <c r="I31" s="24" t="n"/>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="25" t="inlineStr">
         <is>
-          <t>동양</t>
+          <t>녹십자엠에스</t>
         </is>
       </c>
       <c r="B32" s="24" t="n">
@@ -4080,25 +4102,25 @@
       </c>
       <c r="F32" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G32" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="H32" s="26" t="n">
-        <v>-0.45</v>
-      </c>
-      <c r="I32" s="26" t="n">
-        <v>-0.89</v>
+        <v>-14.53</v>
+      </c>
+      <c r="I32" s="27" t="n">
+        <v>9.869999999999999</v>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="25" t="inlineStr">
         <is>
-          <t>동양고속</t>
+          <t>더코디</t>
         </is>
       </c>
       <c r="B33" s="24" t="n">
@@ -4115,19 +4137,19 @@
       </c>
       <c r="F33" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G33" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
-        </is>
-      </c>
-      <c r="H33" s="28" t="n">
-        <v>27.18</v>
-      </c>
-      <c r="I33" s="28" t="n">
-        <v>58.3</v>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="H33" s="27" t="n">
+        <v>7.28</v>
+      </c>
+      <c r="I33" s="26" t="n">
+        <v>-15.36</v>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
@@ -4150,19 +4172,19 @@
       </c>
       <c r="F34" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G34" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="H34" s="26" t="n">
         <v>-5.14</v>
       </c>
-      <c r="I34" s="28" t="n">
-        <v>38.73</v>
+      <c r="I34" s="27" t="n">
+        <v>31.22</v>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
@@ -4185,25 +4207,25 @@
       </c>
       <c r="F35" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G35" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="H35" s="26" t="n">
         <v>-9.609999999999999</v>
       </c>
-      <c r="I35" s="28" t="n">
-        <v>25.09</v>
+      <c r="I35" s="27" t="n">
+        <v>18.71</v>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="25" t="inlineStr">
         <is>
-          <t>빅텐츠</t>
+          <t>삼성전자우</t>
         </is>
       </c>
       <c r="B36" s="24" t="n">
@@ -4220,25 +4242,25 @@
       </c>
       <c r="F36" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G36" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="H36" s="26" t="n">
-        <v>-18.27</v>
+        <v>-1.42</v>
       </c>
       <c r="I36" s="26" t="n">
-        <v>-13.73</v>
+        <v>-3.47</v>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="25" t="inlineStr">
         <is>
-          <t>삼성생명</t>
+          <t>삼표시멘트</t>
         </is>
       </c>
       <c r="B37" s="24" t="n">
@@ -4255,25 +4277,25 @@
       </c>
       <c r="F37" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G37" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="H37" s="26" t="n">
-        <v>-3.05</v>
+        <v>-12.77</v>
       </c>
       <c r="I37" s="26" t="n">
-        <v>-4.42</v>
+        <v>-0.29</v>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="25" t="inlineStr">
         <is>
-          <t>아톤</t>
+          <t>스피어</t>
         </is>
       </c>
       <c r="B38" s="24" t="n">
@@ -4290,25 +4312,25 @@
       </c>
       <c r="F38" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G38" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
-        </is>
-      </c>
-      <c r="H38" s="26" t="n">
-        <v>-3.4</v>
-      </c>
-      <c r="I38" s="28" t="n">
-        <v>21.15</v>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="H38" s="27" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="I38" s="27" t="n">
+        <v>2.83</v>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="25" t="inlineStr">
         <is>
-          <t>유바이오로직스</t>
+          <t>아톤</t>
         </is>
       </c>
       <c r="B39" s="24" t="n">
@@ -4325,25 +4347,25 @@
       </c>
       <c r="F39" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G39" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="H39" s="26" t="n">
-        <v>-0.47</v>
-      </c>
-      <c r="I39" s="26" t="n">
-        <v>-0.93</v>
+        <v>-3.4</v>
+      </c>
+      <c r="I39" s="27" t="n">
+        <v>14.76</v>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="25" t="inlineStr">
         <is>
-          <t>조선</t>
+          <t>알테오젠</t>
         </is>
       </c>
       <c r="B40" s="24" t="n">
@@ -4360,21 +4382,25 @@
       </c>
       <c r="F40" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G40" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
-        </is>
-      </c>
-      <c r="H40" s="24" t="n"/>
-      <c r="I40" s="24" t="n"/>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="H40" s="26" t="n">
+        <v>-5.5</v>
+      </c>
+      <c r="I40" s="26" t="n">
+        <v>-7.32</v>
+      </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="25" t="inlineStr">
         <is>
-          <t>카카오</t>
+          <t>에이엔피</t>
         </is>
       </c>
       <c r="B41" s="24" t="n">
@@ -4391,25 +4417,25 @@
       </c>
       <c r="F41" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G41" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
-        </is>
-      </c>
-      <c r="H41" s="26" t="n">
-        <v>-1.52</v>
-      </c>
-      <c r="I41" s="26" t="n">
-        <v>-3.57</v>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="H41" s="27" t="n">
+        <v>29.69</v>
+      </c>
+      <c r="I41" s="27" t="n">
+        <v>23.27</v>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="25" t="inlineStr">
         <is>
-          <t>한양디지텍</t>
+          <t>엔켐</t>
         </is>
       </c>
       <c r="B42" s="24" t="n">
@@ -4426,25 +4452,25 @@
       </c>
       <c r="F42" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G42" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
-        </is>
-      </c>
-      <c r="H42" s="28" t="n">
-        <v>7.01</v>
-      </c>
-      <c r="I42" s="28" t="n">
-        <v>8.19</v>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="H42" s="26" t="n">
+        <v>-5.42</v>
+      </c>
+      <c r="I42" s="26" t="n">
+        <v>-4.8</v>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="25" t="inlineStr">
         <is>
-          <t>한컴</t>
+          <t>우원개발</t>
         </is>
       </c>
       <c r="B43" s="24" t="n">
@@ -4461,25 +4487,25 @@
       </c>
       <c r="F43" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G43" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
-        </is>
-      </c>
-      <c r="H43" s="26" t="n">
-        <v>-1.48</v>
-      </c>
-      <c r="I43" s="26" t="n">
-        <v>-0.4</v>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="H43" s="27" t="n">
+        <v>2.74</v>
+      </c>
+      <c r="I43" s="27" t="n">
+        <v>1.81</v>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="25" t="inlineStr">
         <is>
-          <t>한화오션</t>
+          <t>철강</t>
         </is>
       </c>
       <c r="B44" s="24" t="n">
@@ -4496,54 +4522,50 @@
       </c>
       <c r="F44" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G44" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
-        </is>
-      </c>
-      <c r="H44" s="26" t="n">
-        <v>-3.1</v>
-      </c>
-      <c r="I44" s="26" t="n">
-        <v>-8.65</v>
-      </c>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="H44" s="24" t="n"/>
+      <c r="I44" s="24" t="n"/>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="25" t="inlineStr">
         <is>
-          <t>HLB바이오스텝</t>
+          <t>한컴</t>
         </is>
       </c>
       <c r="B45" s="24" t="n">
         <v>1</v>
       </c>
       <c r="C45" s="24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D45" s="24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E45" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F45" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G45" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
-        </is>
-      </c>
-      <c r="H45" s="28" t="n">
-        <v>29.97</v>
-      </c>
-      <c r="I45" s="28" t="n">
-        <v>108.25</v>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="H45" s="26" t="n">
+        <v>-1.48</v>
+      </c>
+      <c r="I45" s="27" t="n">
+        <v>0.7</v>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
@@ -4566,25 +4588,25 @@
       </c>
       <c r="F46" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G46" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="H46" s="26" t="n">
         <v>-2.44</v>
       </c>
       <c r="I46" s="26" t="n">
-        <v>-8.050000000000001</v>
+        <v>-3.32</v>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="25" t="inlineStr">
         <is>
-          <t>KT</t>
+          <t>동국산업</t>
         </is>
       </c>
       <c r="B47" s="24" t="n">
@@ -4601,25 +4623,25 @@
       </c>
       <c r="F47" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G47" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
-        </is>
-      </c>
-      <c r="H47" s="28" t="n">
-        <v>0.39</v>
-      </c>
-      <c r="I47" s="26" t="n">
-        <v>-1.16</v>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="H47" s="27" t="n">
+        <v>20.23</v>
+      </c>
+      <c r="I47" s="27" t="n">
+        <v>16.9</v>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="25" t="inlineStr">
         <is>
-          <t>동국산업</t>
+          <t>빛과전자</t>
         </is>
       </c>
       <c r="B48" s="24" t="n">
@@ -4636,25 +4658,25 @@
       </c>
       <c r="F48" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G48" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
-        </is>
-      </c>
-      <c r="H48" s="28" t="n">
-        <v>20.23</v>
-      </c>
-      <c r="I48" s="28" t="n">
-        <v>37.95</v>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="H48" s="26" t="n">
+        <v>-4.49</v>
+      </c>
+      <c r="I48" s="27" t="n">
+        <v>11.14</v>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="25" t="inlineStr">
         <is>
-          <t>삼성SDI</t>
+          <t>알루코</t>
         </is>
       </c>
       <c r="B49" s="24" t="n">
@@ -4671,25 +4693,25 @@
       </c>
       <c r="F49" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G49" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
-        </is>
-      </c>
-      <c r="H49" s="28" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="I49" s="28" t="n">
-        <v>9.67</v>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="H49" s="27" t="n">
+        <v>6.55</v>
+      </c>
+      <c r="I49" s="27" t="n">
+        <v>10.02</v>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="25" t="inlineStr">
         <is>
-          <t>알루코</t>
+          <t>한미반도체</t>
         </is>
       </c>
       <c r="B50" s="24" t="n">
@@ -4706,25 +4728,25 @@
       </c>
       <c r="F50" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G50" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
-        </is>
-      </c>
-      <c r="H50" s="28" t="n">
-        <v>6.55</v>
-      </c>
-      <c r="I50" s="28" t="n">
-        <v>12.16</v>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="H50" s="26" t="n">
+        <v>-0.38</v>
+      </c>
+      <c r="I50" s="26" t="n">
+        <v>-3.31</v>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="25" t="inlineStr">
         <is>
-          <t>한미약품</t>
+          <t>한화머시너리앤서비스홀딩스</t>
         </is>
       </c>
       <c r="B51" s="24" t="n">
@@ -4741,54 +4763,54 @@
       </c>
       <c r="F51" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G51" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="H51" s="26" t="n">
-        <v>-9.74</v>
-      </c>
-      <c r="I51" s="26" t="n">
-        <v>-3.6</v>
+        <v>-0.16</v>
+      </c>
+      <c r="I51" s="27" t="n">
+        <v>7.76</v>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="25" t="inlineStr">
         <is>
-          <t>현대지에프홀딩스</t>
+          <t>제이앤티씨</t>
         </is>
       </c>
       <c r="B52" s="24" t="n">
         <v>1</v>
       </c>
       <c r="C52" s="24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D52" s="24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E52" s="31" t="n">
         <v>1</v>
       </c>
       <c r="F52" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G52" s="24" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
-        </is>
-      </c>
-      <c r="H52" s="28" t="n">
-        <v>4.73</v>
-      </c>
-      <c r="I52" s="28" t="n">
-        <v>2.15</v>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="H52" s="27" t="n">
+        <v>5.26</v>
+      </c>
+      <c r="I52" s="27" t="n">
+        <v>23.85</v>
       </c>
     </row>
   </sheetData>
@@ -4872,19 +4894,19 @@
         <v>1</v>
       </c>
       <c r="C3" s="35" t="n">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D3" s="35" t="n">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E3" s="35" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="F3" s="36" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G3" s="36" t="inlineStr">
@@ -4903,19 +4925,19 @@
         <v>1</v>
       </c>
       <c r="C4" s="35" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="D4" s="35" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E4" s="35" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="F4" s="36" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G4" s="36" t="inlineStr">
@@ -4934,19 +4956,19 @@
         <v>1</v>
       </c>
       <c r="C5" s="35" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D5" s="35" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E5" s="35" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="F5" s="36" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G5" s="36" t="inlineStr">
@@ -4965,19 +4987,19 @@
         <v>1</v>
       </c>
       <c r="C6" s="35" t="n">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="D6" s="35" t="n">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="E6" s="35" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="F6" s="36" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G6" s="36" t="inlineStr">
@@ -5003,12 +5025,12 @@
       </c>
       <c r="E7" s="35" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="F7" s="36" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G7" s="36" t="inlineStr">
@@ -5020,26 +5042,26 @@
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="34" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>원전</t>
         </is>
       </c>
       <c r="B8" s="35" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="35" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D8" s="35" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E8" s="35" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="F8" s="36" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G8" s="36" t="inlineStr">
@@ -5051,26 +5073,26 @@
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="34" t="inlineStr">
         <is>
-          <t>수소</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="B9" s="35" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="35" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D9" s="35" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="E9" s="35" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="F9" s="36" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G9" s="36" t="inlineStr">
@@ -5082,26 +5104,26 @@
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="34" t="inlineStr">
         <is>
-          <t>태양광</t>
+          <t>조선</t>
         </is>
       </c>
       <c r="B10" s="35" t="n">
         <v>1</v>
       </c>
       <c r="C10" s="35" t="n">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="D10" s="35" t="n">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="E10" s="35" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="F10" s="36" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G10" s="36" t="inlineStr">
@@ -5113,26 +5135,26 @@
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="34" t="inlineStr">
         <is>
-          <t>클라우드</t>
+          <t>철강</t>
         </is>
       </c>
       <c r="B11" s="35" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="35" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D11" s="35" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E11" s="35" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="F11" s="36" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G11" s="36" t="inlineStr">
@@ -5144,26 +5166,26 @@
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="34" t="inlineStr">
         <is>
-          <t>조선</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="B12" s="35" t="n">
         <v>1</v>
       </c>
       <c r="C12" s="35" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="D12" s="35" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E12" s="35" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="F12" s="36" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G12" s="36" t="inlineStr">
@@ -5175,26 +5197,26 @@
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="34" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="B13" s="35" t="n">
         <v>1</v>
       </c>
       <c r="C13" s="35" t="n">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="D13" s="35" t="n">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="E13" s="35" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="F13" s="36" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G13" s="36" t="inlineStr">
@@ -5204,71 +5226,63 @@
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="34" t="inlineStr">
-        <is>
-          <t>인공지능</t>
-        </is>
-      </c>
-      <c r="B14" s="35" t="n">
-        <v>1</v>
-      </c>
-      <c r="C14" s="35" t="n">
-        <v>29</v>
-      </c>
-      <c r="D14" s="35" t="n">
-        <v>29</v>
-      </c>
-      <c r="E14" s="35" t="inlineStr">
-        <is>
-          <t>2026-10-11</t>
-        </is>
-      </c>
-      <c r="F14" s="36" t="inlineStr">
-        <is>
-          <t>2026-10-11</t>
-        </is>
-      </c>
-      <c r="G14" s="36" t="inlineStr">
-        <is>
-          <t>⚡ 관심</t>
-        </is>
-      </c>
+      <c r="A14" s="25" t="inlineStr">
+        <is>
+          <t>이차전지</t>
+        </is>
+      </c>
+      <c r="B14" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F14" s="28" t="inlineStr">
+        <is>
+          <t>감지 없음</t>
+        </is>
+      </c>
+      <c r="G14" s="28" t="inlineStr"/>
     </row>
     <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="34" t="inlineStr">
-        <is>
-          <t>AMD</t>
-        </is>
-      </c>
-      <c r="B15" s="35" t="n">
-        <v>1</v>
-      </c>
-      <c r="C15" s="35" t="n">
-        <v>7</v>
-      </c>
-      <c r="D15" s="35" t="n">
-        <v>7</v>
-      </c>
-      <c r="E15" s="35" t="inlineStr">
-        <is>
-          <t>2026-10-11</t>
-        </is>
-      </c>
-      <c r="F15" s="36" t="inlineStr">
-        <is>
-          <t>2026-10-11</t>
-        </is>
-      </c>
-      <c r="G15" s="36" t="inlineStr">
-        <is>
-          <t>⚡ 관심</t>
-        </is>
-      </c>
+      <c r="A15" s="25" t="inlineStr">
+        <is>
+          <t>수소</t>
+        </is>
+      </c>
+      <c r="B15" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F15" s="28" t="inlineStr">
+        <is>
+          <t>감지 없음</t>
+        </is>
+      </c>
+      <c r="G15" s="28" t="inlineStr"/>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="25" t="inlineStr">
         <is>
-          <t>이차전지</t>
+          <t>태양광</t>
         </is>
       </c>
       <c r="B16" s="24" t="n">
@@ -5285,17 +5299,17 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F16" s="27" t="inlineStr">
+      <c r="F16" s="28" t="inlineStr">
         <is>
           <t>감지 없음</t>
         </is>
       </c>
-      <c r="G16" s="27" t="inlineStr"/>
+      <c r="G16" s="28" t="inlineStr"/>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="25" t="inlineStr">
         <is>
-          <t>원전</t>
+          <t>게임</t>
         </is>
       </c>
       <c r="B17" s="24" t="n">
@@ -5312,17 +5326,17 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F17" s="27" t="inlineStr">
+      <c r="F17" s="28" t="inlineStr">
         <is>
           <t>감지 없음</t>
         </is>
       </c>
-      <c r="G17" s="27" t="inlineStr"/>
+      <c r="G17" s="28" t="inlineStr"/>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="25" t="inlineStr">
         <is>
-          <t>게임</t>
+          <t>엔터</t>
         </is>
       </c>
       <c r="B18" s="24" t="n">
@@ -5339,17 +5353,17 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F18" s="27" t="inlineStr">
+      <c r="F18" s="28" t="inlineStr">
         <is>
           <t>감지 없음</t>
         </is>
       </c>
-      <c r="G18" s="27" t="inlineStr"/>
+      <c r="G18" s="28" t="inlineStr"/>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="25" t="inlineStr">
         <is>
-          <t>엔터</t>
+          <t>핀테크</t>
         </is>
       </c>
       <c r="B19" s="24" t="n">
@@ -5366,17 +5380,17 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F19" s="27" t="inlineStr">
+      <c r="F19" s="28" t="inlineStr">
         <is>
           <t>감지 없음</t>
         </is>
       </c>
-      <c r="G19" s="27" t="inlineStr"/>
+      <c r="G19" s="28" t="inlineStr"/>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="25" t="inlineStr">
         <is>
-          <t>핀테크</t>
+          <t>클라우드</t>
         </is>
       </c>
       <c r="B20" s="24" t="n">
@@ -5393,17 +5407,17 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F20" s="27" t="inlineStr">
+      <c r="F20" s="28" t="inlineStr">
         <is>
           <t>감지 없음</t>
         </is>
       </c>
-      <c r="G20" s="27" t="inlineStr"/>
+      <c r="G20" s="28" t="inlineStr"/>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="25" t="inlineStr">
         <is>
-          <t>철강</t>
+          <t>의료기기</t>
         </is>
       </c>
       <c r="B21" s="24" t="n">
@@ -5420,17 +5434,17 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F21" s="27" t="inlineStr">
+      <c r="F21" s="28" t="inlineStr">
         <is>
           <t>감지 없음</t>
         </is>
       </c>
-      <c r="G21" s="27" t="inlineStr"/>
+      <c r="G21" s="28" t="inlineStr"/>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="25" t="inlineStr">
         <is>
-          <t>의료기기</t>
+          <t>NVIDIA</t>
         </is>
       </c>
       <c r="B22" s="24" t="n">
@@ -5447,17 +5461,17 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F22" s="27" t="inlineStr">
+      <c r="F22" s="28" t="inlineStr">
         <is>
           <t>감지 없음</t>
         </is>
       </c>
-      <c r="G22" s="27" t="inlineStr"/>
+      <c r="G22" s="28" t="inlineStr"/>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="25" t="inlineStr">
         <is>
-          <t>NVIDIA</t>
+          <t>Tesla</t>
         </is>
       </c>
       <c r="B23" s="24" t="n">
@@ -5474,17 +5488,17 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F23" s="27" t="inlineStr">
+      <c r="F23" s="28" t="inlineStr">
         <is>
           <t>감지 없음</t>
         </is>
       </c>
-      <c r="G23" s="27" t="inlineStr"/>
+      <c r="G23" s="28" t="inlineStr"/>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="25" t="inlineStr">
         <is>
-          <t>Tesla</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B24" s="24" t="n">
@@ -5501,12 +5515,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F24" s="27" t="inlineStr">
+      <c r="F24" s="28" t="inlineStr">
         <is>
           <t>감지 없음</t>
         </is>
       </c>
-      <c r="G24" s="27" t="inlineStr"/>
+      <c r="G24" s="28" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
auto: 2026-10-18 07:09 자동 백업
</commit_message>
<xml_diff>
--- a/trend/stock_trend_history.xlsx
+++ b/trend/stock_trend_history.xlsx
@@ -261,11 +261,11 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -694,7 +694,7 @@
     <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-10-17 06:54</t>
+          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-10-18 06:53</t>
         </is>
       </c>
     </row>
@@ -787,21 +787,21 @@
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-10-17) 상위: 반도체  점수 53.0점</t>
+          <t>⚡ 최신(2026-10-18) 상위: 반도체  점수 50.0점</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-10-17) 상위: 삼성전자  점수 22.0점</t>
+          <t>⚡ 최신(2026-10-18) 상위: 바이오  점수 22.0점</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-10-17) 상위: 바이오  점수 22.0점</t>
+          <t>⚡ 최신(2026-10-18) 상위: 삼성전자  점수 20.0점</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="15" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B14" s="15" t="n">
@@ -928,10 +928,10 @@
         </is>
       </c>
       <c r="D14" s="15" t="n">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="E14" s="15" t="n">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="F14" s="15" t="n">
         <v>0</v>
@@ -947,7 +947,7 @@
       </c>
       <c r="J14" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+          <t>매일경제 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K14" s="17" t="inlineStr">
@@ -959,7 +959,7 @@
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="15" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B15" s="15" t="n">
@@ -967,7 +967,7 @@
       </c>
       <c r="C15" s="16" t="inlineStr">
         <is>
-          <t>삼성전자</t>
+          <t>바이오</t>
         </is>
       </c>
       <c r="D15" s="15" t="n">
@@ -982,27 +982,27 @@
       <c r="G15" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H15" s="18" t="n">
-        <v>4.58</v>
-      </c>
-      <c r="I15" s="19" t="n">
-        <v>-17.49</v>
+      <c r="H15" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I15" s="15" t="n">
+        <v/>
       </c>
       <c r="J15" s="17" t="inlineStr">
         <is>
-          <t>중요공시 1건 / Google 급상승 검색어 등장 (KR) / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
+          <t>매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급</t>
         </is>
       </c>
       <c r="K15" s="17" t="inlineStr">
         <is>
-          <t>공시, Google, 네이버</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="15" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B16" s="15" t="n">
@@ -1010,14 +1010,14 @@
       </c>
       <c r="C16" s="16" t="inlineStr">
         <is>
-          <t>바이오</t>
+          <t>삼성전자</t>
         </is>
       </c>
       <c r="D16" s="15" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E16" s="15" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F16" s="15" t="n">
         <v>0</v>
@@ -1025,27 +1025,27 @@
       <c r="G16" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H16" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I16" s="15" t="n">
-        <v/>
+      <c r="H16" s="18" t="n">
+        <v>4.58</v>
+      </c>
+      <c r="I16" s="19" t="n">
+        <v>-17.49</v>
       </c>
       <c r="J16" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 한국경제 헤드라인 언급 / 네이버뉴스 기사 언급</t>
+          <t>네이버 검색 당일 +87% / 중요공시 1건 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K16" s="17" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B17" s="15" t="n">
@@ -1088,7 +1088,7 @@
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B18" s="15" t="n">
@@ -1096,14 +1096,14 @@
       </c>
       <c r="C18" s="16" t="inlineStr">
         <is>
-          <t>인공지능</t>
+          <t>SK하이닉스</t>
         </is>
       </c>
       <c r="D18" s="15" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E18" s="15" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F18" s="15" t="n">
         <v>0</v>
@@ -1111,15 +1111,15 @@
       <c r="G18" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H18" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I18" s="15" t="n">
-        <v/>
+      <c r="H18" s="18" t="n">
+        <v>2.18</v>
+      </c>
+      <c r="I18" s="19" t="n">
+        <v>-24.97</v>
       </c>
       <c r="J18" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급</t>
+          <t>네이버 검색 당일 +138% / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K18" s="17" t="inlineStr">
@@ -1131,7 +1131,7 @@
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B19" s="15" t="n">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="C19" s="16" t="inlineStr">
         <is>
-          <t>방산</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="D19" s="15" t="n">
@@ -1162,7 +1162,7 @@
       </c>
       <c r="J19" s="17" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>매일경제 기사 언급 / 매일경제 기사 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K19" s="17" t="n">
@@ -1172,7 +1172,7 @@
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B20" s="15" t="n">
@@ -1184,10 +1184,10 @@
         </is>
       </c>
       <c r="D20" s="15" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E20" s="15" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F20" s="15" t="n">
         <v>2</v>
@@ -1203,7 +1203,7 @@
       </c>
       <c r="J20" s="17" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +81% / 중요공시 6건 / 중요공시 3일 +200% / 중요공시 7일 +500%</t>
+          <t>네이버 검색 당일 +119% / 중요공시 6건 / 중요공시 3일 +500% / 중요공시 7일 +200%</t>
         </is>
       </c>
       <c r="K20" s="17" t="inlineStr">
@@ -1215,7 +1215,7 @@
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="15" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B21" s="15" t="n">
@@ -1223,14 +1223,14 @@
       </c>
       <c r="C21" s="16" t="inlineStr">
         <is>
-          <t>삼성전기</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="D21" s="15" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E21" s="15" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F21" s="15" t="n">
         <v>0</v>
@@ -1238,27 +1238,27 @@
       <c r="G21" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H21" s="18" t="n">
-        <v>5.53</v>
-      </c>
-      <c r="I21" s="19" t="n">
-        <v>-24.05</v>
+      <c r="H21" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I21" s="15" t="n">
+        <v/>
       </c>
       <c r="J21" s="17" t="inlineStr">
         <is>
-          <t>Google 급상승 검색어 등장 (KR) / 네이버뉴스 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+          <t>매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K21" s="17" t="inlineStr">
         <is>
-          <t>Google, 네이버</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="15" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B22" s="15" t="n">
@@ -1266,14 +1266,14 @@
       </c>
       <c r="C22" s="16" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>방산</t>
         </is>
       </c>
       <c r="D22" s="15" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E22" s="15" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F22" s="15" t="n">
         <v>0</v>
@@ -1289,19 +1289,17 @@
       </c>
       <c r="J22" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급</t>
-        </is>
-      </c>
-      <c r="K22" s="17" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+          <t>한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K22" s="17" t="n">
+        <v/>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="15" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B23" s="15" t="n">
@@ -1309,14 +1307,14 @@
       </c>
       <c r="C23" s="16" t="inlineStr">
         <is>
-          <t>삼성바이오로직스</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="D23" s="15" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E23" s="15" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F23" s="15" t="n">
         <v>0</v>
@@ -1324,27 +1322,27 @@
       <c r="G23" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H23" s="18" t="n">
-        <v>4.03</v>
-      </c>
-      <c r="I23" s="18" t="n">
-        <v>5.82</v>
+      <c r="H23" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I23" s="15" t="n">
+        <v/>
       </c>
       <c r="J23" s="17" t="inlineStr">
         <is>
-          <t>중요공시 2건 / Google 급상승 검색어 등장 (KR) / 한국경제 헤드라인 언급</t>
+          <t>매일경제 기사 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K23" s="17" t="inlineStr">
         <is>
-          <t>공시, Google</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="15" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B24" s="15" t="n">
@@ -1352,14 +1350,14 @@
       </c>
       <c r="C24" s="16" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>우진엔텍</t>
         </is>
       </c>
       <c r="D24" s="15" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E24" s="15" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="F24" s="15" t="n">
         <v>0</v>
@@ -1367,25 +1365,27 @@
       <c r="G24" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H24" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I24" s="15" t="n">
-        <v/>
+      <c r="H24" s="19" t="n">
+        <v>-19.25</v>
+      </c>
+      <c r="I24" s="19" t="n">
+        <v>-19.25</v>
       </c>
       <c r="J24" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 매일경제 기사 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K24" s="17" t="n">
-        <v/>
+          <t>네이버 검색 당일 +173% / 중요공시 1건 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K24" s="17" t="inlineStr">
+        <is>
+          <t>공시, 네이버</t>
+        </is>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="15" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B25" s="15" t="n">
@@ -1393,42 +1393,42 @@
       </c>
       <c r="C25" s="16" t="inlineStr">
         <is>
-          <t>SK하이닉스</t>
+          <t>모아라이프플러스</t>
         </is>
       </c>
       <c r="D25" s="15" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E25" s="15" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="F25" s="15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G25" s="15" t="n">
         <v>0</v>
       </c>
       <c r="H25" s="18" t="n">
-        <v>2.18</v>
-      </c>
-      <c r="I25" s="19" t="n">
-        <v>-24.97</v>
+        <v>8.33</v>
+      </c>
+      <c r="I25" s="18" t="n">
+        <v>0.78</v>
       </c>
       <c r="J25" s="17" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +88% / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급</t>
+          <t>네이버 검색 당일 +99% / 중요공시 7건 / 중요공시 3일 +75%</t>
         </is>
       </c>
       <c r="K25" s="17" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="15" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B26" s="15" t="n">
@@ -1436,42 +1436,42 @@
       </c>
       <c r="C26" s="16" t="inlineStr">
         <is>
-          <t>넥사다이내믹스</t>
+          <t>카카오</t>
         </is>
       </c>
       <c r="D26" s="15" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E26" s="15" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="F26" s="15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G26" s="15" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H26" s="18" t="n">
-        <v>2.78</v>
-      </c>
-      <c r="I26" s="18" t="n">
-        <v>12.15</v>
+        <v>2.76</v>
+      </c>
+      <c r="I26" s="19" t="n">
+        <v>-2.16</v>
       </c>
       <c r="J26" s="17" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 3일 +200% / 중요공시 7일 +200%</t>
+          <t>네이버 검색 당일 +53% / Google 급상승 검색어 등장 (KR)</t>
         </is>
       </c>
       <c r="K26" s="17" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>Google, 네이버</t>
         </is>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="15" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B27" s="15" t="n">
@@ -1514,7 +1514,7 @@
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="20" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B28" s="20" t="n">
@@ -1522,7 +1522,7 @@
       </c>
       <c r="C28" s="21" t="inlineStr">
         <is>
-          <t>삼성중공업</t>
+          <t>LG유플러스</t>
         </is>
       </c>
       <c r="D28" s="20" t="n">
@@ -1538,26 +1538,24 @@
         <v>0</v>
       </c>
       <c r="H28" s="22" t="n">
-        <v>2.73</v>
-      </c>
-      <c r="I28" s="23" t="n">
-        <v>-2.49</v>
-      </c>
-      <c r="J28" s="24" t="inlineStr">
-        <is>
-          <t>Google 급상승 검색어 등장 (KR)</t>
-        </is>
-      </c>
-      <c r="K28" s="24" t="inlineStr">
-        <is>
-          <t>Google</t>
-        </is>
+        <v>3.06</v>
+      </c>
+      <c r="I28" s="22" t="n">
+        <v>7.48</v>
+      </c>
+      <c r="J28" s="23" t="inlineStr">
+        <is>
+          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K28" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="20" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B29" s="20" t="n">
@@ -1565,7 +1563,7 @@
       </c>
       <c r="C29" s="21" t="inlineStr">
         <is>
-          <t>삼성전자우</t>
+          <t>한화솔루션</t>
         </is>
       </c>
       <c r="D29" s="20" t="n">
@@ -1581,26 +1579,24 @@
         <v>0</v>
       </c>
       <c r="H29" s="22" t="n">
-        <v>8.539999999999999</v>
-      </c>
-      <c r="I29" s="23" t="n">
-        <v>-13.11</v>
-      </c>
-      <c r="J29" s="24" t="inlineStr">
-        <is>
-          <t>Google 급상승 검색어 등장 (KR)</t>
-        </is>
-      </c>
-      <c r="K29" s="24" t="inlineStr">
-        <is>
-          <t>Google</t>
-        </is>
+        <v>6.08</v>
+      </c>
+      <c r="I29" s="24" t="n">
+        <v>-12.04</v>
+      </c>
+      <c r="J29" s="23" t="inlineStr">
+        <is>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K29" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="20" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B30" s="20" t="n">
@@ -1608,33 +1604,33 @@
       </c>
       <c r="C30" s="21" t="inlineStr">
         <is>
-          <t>한화시스템</t>
+          <t>LG에너지솔루션</t>
         </is>
       </c>
       <c r="D30" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E30" s="20" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F30" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G30" s="20" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H30" s="22" t="n">
-        <v>9.08</v>
+        <v>2.67</v>
       </c>
       <c r="I30" s="22" t="n">
-        <v>4.95</v>
-      </c>
-      <c r="J30" s="24" t="inlineStr">
-        <is>
-          <t>중요공시 1건 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K30" s="24" t="inlineStr">
+        <v>0.12</v>
+      </c>
+      <c r="J30" s="23" t="inlineStr">
+        <is>
+          <t>중요공시 2건 / 중요공시 3일 +100% / 중요공시 7일 +100%</t>
+        </is>
+      </c>
+      <c r="K30" s="23" t="inlineStr">
         <is>
           <t>공시</t>
         </is>
@@ -1643,7 +1639,7 @@
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="20" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B31" s="20" t="n">
@@ -1651,7 +1647,7 @@
       </c>
       <c r="C31" s="21" t="inlineStr">
         <is>
-          <t>LG유플러스</t>
+          <t>피에스케이홀딩스</t>
         </is>
       </c>
       <c r="D31" s="20" t="n">
@@ -1667,24 +1663,24 @@
         <v>0</v>
       </c>
       <c r="H31" s="22" t="n">
-        <v>3.06</v>
-      </c>
-      <c r="I31" s="22" t="n">
-        <v>7.48</v>
-      </c>
-      <c r="J31" s="24" t="inlineStr">
-        <is>
-          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K31" s="24" t="n">
+        <v>10.96</v>
+      </c>
+      <c r="I31" s="24" t="n">
+        <v>-4.82</v>
+      </c>
+      <c r="J31" s="23" t="inlineStr">
+        <is>
+          <t>한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K31" s="23" t="n">
         <v/>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="20" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B32" s="20" t="n">
@@ -1692,7 +1688,7 @@
       </c>
       <c r="C32" s="21" t="inlineStr">
         <is>
-          <t>한화솔루션</t>
+          <t>피에스케이</t>
         </is>
       </c>
       <c r="D32" s="20" t="n">
@@ -1708,24 +1704,24 @@
         <v>0</v>
       </c>
       <c r="H32" s="22" t="n">
-        <v>6.08</v>
-      </c>
-      <c r="I32" s="23" t="n">
-        <v>-12.04</v>
-      </c>
-      <c r="J32" s="24" t="inlineStr">
-        <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K32" s="24" t="n">
+        <v>12.72</v>
+      </c>
+      <c r="I32" s="24" t="n">
+        <v>-10.82</v>
+      </c>
+      <c r="J32" s="23" t="inlineStr">
+        <is>
+          <t>한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K32" s="23" t="n">
         <v/>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="20" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B33" s="20" t="n">
@@ -1733,42 +1729,42 @@
       </c>
       <c r="C33" s="21" t="inlineStr">
         <is>
-          <t>LG에너지솔루션</t>
+          <t>동국제약</t>
         </is>
       </c>
       <c r="D33" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E33" s="20" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F33" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G33" s="20" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H33" s="22" t="n">
-        <v>2.67</v>
+        <v>4.34</v>
       </c>
       <c r="I33" s="22" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="J33" s="24" t="inlineStr">
-        <is>
-          <t>중요공시 2건 / 중요공시 3일 +100% / 중요공시 7일 +100%</t>
-        </is>
-      </c>
-      <c r="K33" s="24" t="inlineStr">
-        <is>
-          <t>공시</t>
+        <v>12.98</v>
+      </c>
+      <c r="J33" s="23" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +58% / 네이버뉴스 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K33" s="23" t="inlineStr">
+        <is>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="20" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B34" s="20" t="n">
@@ -1776,14 +1772,14 @@
       </c>
       <c r="C34" s="21" t="inlineStr">
         <is>
-          <t>삼성물산</t>
+          <t>두산에너빌리티</t>
         </is>
       </c>
       <c r="D34" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E34" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F34" s="20" t="n">
         <v>0</v>
@@ -1792,26 +1788,24 @@
         <v>0</v>
       </c>
       <c r="H34" s="22" t="n">
-        <v>7.78</v>
-      </c>
-      <c r="I34" s="23" t="n">
-        <v>-11.25</v>
-      </c>
-      <c r="J34" s="24" t="inlineStr">
-        <is>
-          <t>중요공시 1건 / Google 급상승 검색어 등장 (KR)</t>
-        </is>
-      </c>
-      <c r="K34" s="24" t="inlineStr">
-        <is>
-          <t>공시, Google</t>
-        </is>
+        <v>4.89</v>
+      </c>
+      <c r="I34" s="24" t="n">
+        <v>-16.04</v>
+      </c>
+      <c r="J34" s="23" t="inlineStr">
+        <is>
+          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K34" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="20" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B35" s="20" t="n">
@@ -1819,14 +1813,14 @@
       </c>
       <c r="C35" s="21" t="inlineStr">
         <is>
-          <t>삼성SDI</t>
+          <t>우리로</t>
         </is>
       </c>
       <c r="D35" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E35" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F35" s="20" t="n">
         <v>0</v>
@@ -1835,26 +1829,26 @@
         <v>0</v>
       </c>
       <c r="H35" s="22" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="I35" s="23" t="n">
-        <v>-6.53</v>
-      </c>
-      <c r="J35" s="24" t="inlineStr">
-        <is>
-          <t>Google 급상승 검색어 등장 (KR) / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K35" s="24" t="inlineStr">
-        <is>
-          <t>Google</t>
+        <v>18.59</v>
+      </c>
+      <c r="I35" s="22" t="n">
+        <v>7.33</v>
+      </c>
+      <c r="J35" s="23" t="inlineStr">
+        <is>
+          <t>중요공시 1건 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K35" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="20" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B36" s="20" t="n">
@@ -1862,42 +1856,42 @@
       </c>
       <c r="C36" s="21" t="inlineStr">
         <is>
-          <t>철강</t>
+          <t>엘앤씨바이오</t>
         </is>
       </c>
       <c r="D36" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E36" s="20" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F36" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G36" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H36" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I36" s="20" t="n">
-        <v/>
-      </c>
-      <c r="J36" s="24" t="inlineStr">
-        <is>
-          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K36" s="24" t="inlineStr">
-        <is>
-          <t>네이버</t>
+      <c r="H36" s="22" t="n">
+        <v>22.98</v>
+      </c>
+      <c r="I36" s="22" t="n">
+        <v>22.76</v>
+      </c>
+      <c r="J36" s="23" t="inlineStr">
+        <is>
+          <t>중요공시 3건 / 중요공시 3일 +50%</t>
+        </is>
+      </c>
+      <c r="K36" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="20" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B37" s="20" t="n">
@@ -1905,40 +1899,42 @@
       </c>
       <c r="C37" s="21" t="inlineStr">
         <is>
-          <t>피에스케이</t>
+          <t>넥사다이내믹스</t>
         </is>
       </c>
       <c r="D37" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E37" s="20" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F37" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G37" s="20" t="n">
         <v>0</v>
       </c>
       <c r="H37" s="22" t="n">
-        <v>12.72</v>
-      </c>
-      <c r="I37" s="23" t="n">
-        <v>-10.82</v>
-      </c>
-      <c r="J37" s="24" t="inlineStr">
-        <is>
-          <t>한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K37" s="24" t="n">
-        <v/>
+        <v>2.78</v>
+      </c>
+      <c r="I37" s="22" t="n">
+        <v>12.15</v>
+      </c>
+      <c r="J37" s="23" t="inlineStr">
+        <is>
+          <t>중요공시 3건 / 중요공시 3일 +200%</t>
+        </is>
+      </c>
+      <c r="K37" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="20" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B38" s="20" t="n">
@@ -1946,40 +1942,42 @@
       </c>
       <c r="C38" s="21" t="inlineStr">
         <is>
-          <t>피에스케이홀딩스</t>
+          <t>에코프로비엠</t>
         </is>
       </c>
       <c r="D38" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E38" s="20" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F38" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G38" s="20" t="n">
         <v>0</v>
       </c>
       <c r="H38" s="22" t="n">
-        <v>10.96</v>
-      </c>
-      <c r="I38" s="23" t="n">
-        <v>-4.82</v>
-      </c>
-      <c r="J38" s="24" t="inlineStr">
-        <is>
-          <t>한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K38" s="24" t="n">
-        <v/>
+        <v>3.7</v>
+      </c>
+      <c r="I38" s="24" t="n">
+        <v>-15.81</v>
+      </c>
+      <c r="J38" s="23" t="inlineStr">
+        <is>
+          <t>중요공시 3건 / 중요공시 3일 +50%</t>
+        </is>
+      </c>
+      <c r="K38" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="20" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B39" s="20" t="n">
@@ -1987,42 +1985,42 @@
       </c>
       <c r="C39" s="21" t="inlineStr">
         <is>
-          <t>모아라이프플러스</t>
+          <t>본느</t>
         </is>
       </c>
       <c r="D39" s="20" t="n">
         <v>5</v>
       </c>
       <c r="E39" s="20" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F39" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G39" s="20" t="n">
         <v>0</v>
       </c>
       <c r="H39" s="22" t="n">
-        <v>8.33</v>
-      </c>
-      <c r="I39" s="22" t="n">
-        <v>0.78</v>
-      </c>
-      <c r="J39" s="24" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +56% / 중요공시 7건</t>
-        </is>
-      </c>
-      <c r="K39" s="24" t="inlineStr">
-        <is>
-          <t>공시, 네이버</t>
+        <v>6.93</v>
+      </c>
+      <c r="I39" s="24" t="n">
+        <v>-17.93</v>
+      </c>
+      <c r="J39" s="23" t="inlineStr">
+        <is>
+          <t>중요공시 3건 / 중요공시 3일 +200%</t>
+        </is>
+      </c>
+      <c r="K39" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="20" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B40" s="20" t="n">
@@ -2030,42 +2028,42 @@
       </c>
       <c r="C40" s="21" t="inlineStr">
         <is>
-          <t>엘앤씨바이오</t>
+          <t>카카오뱅크</t>
         </is>
       </c>
       <c r="D40" s="20" t="n">
         <v>5</v>
       </c>
       <c r="E40" s="20" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F40" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G40" s="20" t="n">
         <v>0</v>
       </c>
       <c r="H40" s="22" t="n">
-        <v>22.98</v>
+        <v>1.8</v>
       </c>
       <c r="I40" s="22" t="n">
-        <v>22.76</v>
-      </c>
-      <c r="J40" s="24" t="inlineStr">
-        <is>
-          <t>중요공시 3건 / 중요공시 3일 +50%</t>
-        </is>
-      </c>
-      <c r="K40" s="24" t="inlineStr">
-        <is>
-          <t>공시</t>
+        <v>4.25</v>
+      </c>
+      <c r="J40" s="23" t="inlineStr">
+        <is>
+          <t>Google 급상승 검색어 등장 (KR)</t>
+        </is>
+      </c>
+      <c r="K40" s="23" t="inlineStr">
+        <is>
+          <t>Google</t>
         </is>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="20" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B41" s="20" t="n">
@@ -2073,42 +2071,40 @@
       </c>
       <c r="C41" s="21" t="inlineStr">
         <is>
-          <t>본느</t>
+          <t>하이트진로</t>
         </is>
       </c>
       <c r="D41" s="20" t="n">
         <v>5</v>
       </c>
       <c r="E41" s="20" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F41" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G41" s="20" t="n">
         <v>0</v>
       </c>
       <c r="H41" s="22" t="n">
-        <v>6.93</v>
-      </c>
-      <c r="I41" s="23" t="n">
-        <v>-17.93</v>
-      </c>
-      <c r="J41" s="24" t="inlineStr">
-        <is>
-          <t>중요공시 3건 / 중요공시 3일 +200%</t>
-        </is>
-      </c>
-      <c r="K41" s="24" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+        <v>1.43</v>
+      </c>
+      <c r="I41" s="22" t="n">
+        <v>5.76</v>
+      </c>
+      <c r="J41" s="23" t="inlineStr">
+        <is>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K41" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="20" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B42" s="20" t="n">
@@ -2116,7 +2112,7 @@
       </c>
       <c r="C42" s="21" t="inlineStr">
         <is>
-          <t>삼성E&amp;A</t>
+          <t>네이버</t>
         </is>
       </c>
       <c r="D42" s="20" t="n">
@@ -2131,27 +2127,25 @@
       <c r="G42" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H42" s="22" t="n">
-        <v>4.43</v>
-      </c>
-      <c r="I42" s="23" t="n">
-        <v>-8.98</v>
-      </c>
-      <c r="J42" s="24" t="inlineStr">
-        <is>
-          <t>Google 급상승 검색어 등장 (KR)</t>
-        </is>
-      </c>
-      <c r="K42" s="24" t="inlineStr">
-        <is>
-          <t>Google</t>
-        </is>
+      <c r="H42" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I42" s="20" t="n">
+        <v/>
+      </c>
+      <c r="J42" s="23" t="inlineStr">
+        <is>
+          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K42" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="20" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B43" s="20" t="n">
@@ -2159,7 +2153,7 @@
       </c>
       <c r="C43" s="21" t="inlineStr">
         <is>
-          <t>삼성생명</t>
+          <t>삼성전기</t>
         </is>
       </c>
       <c r="D43" s="20" t="n">
@@ -2175,26 +2169,24 @@
         <v>0</v>
       </c>
       <c r="H43" s="22" t="n">
-        <v>5.78</v>
-      </c>
-      <c r="I43" s="23" t="n">
-        <v>-11.85</v>
-      </c>
-      <c r="J43" s="24" t="inlineStr">
-        <is>
-          <t>Google 급상승 검색어 등장 (KR)</t>
-        </is>
-      </c>
-      <c r="K43" s="24" t="inlineStr">
-        <is>
-          <t>Google</t>
-        </is>
+        <v>5.53</v>
+      </c>
+      <c r="I43" s="24" t="n">
+        <v>-24.05</v>
+      </c>
+      <c r="J43" s="23" t="inlineStr">
+        <is>
+          <t>한국경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K43" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="20" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B44" s="20" t="n">
@@ -2202,14 +2194,14 @@
       </c>
       <c r="C44" s="21" t="inlineStr">
         <is>
-          <t>삼성증권</t>
+          <t>하이퍼코퍼레이션</t>
         </is>
       </c>
       <c r="D44" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E44" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F44" s="20" t="n">
         <v>0</v>
@@ -2217,27 +2209,27 @@
       <c r="G44" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H44" s="22" t="n">
-        <v>3.95</v>
-      </c>
-      <c r="I44" s="23" t="n">
-        <v>-8.029999999999999</v>
-      </c>
-      <c r="J44" s="24" t="inlineStr">
-        <is>
-          <t>Google 급상승 검색어 등장 (KR)</t>
-        </is>
-      </c>
-      <c r="K44" s="24" t="inlineStr">
-        <is>
-          <t>Google</t>
+      <c r="H44" s="24" t="n">
+        <v>-24.66</v>
+      </c>
+      <c r="I44" s="22" t="n">
+        <v>73.84999999999999</v>
+      </c>
+      <c r="J44" s="23" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +928% / 중요공시 1건</t>
+        </is>
+      </c>
+      <c r="K44" s="23" t="inlineStr">
+        <is>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="20" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B45" s="20" t="n">
@@ -2245,14 +2237,14 @@
       </c>
       <c r="C45" s="21" t="inlineStr">
         <is>
-          <t>태양광</t>
+          <t>HMM</t>
         </is>
       </c>
       <c r="D45" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E45" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F45" s="20" t="n">
         <v>0</v>
@@ -2260,18 +2252,18 @@
       <c r="G45" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H45" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I45" s="20" t="n">
-        <v/>
-      </c>
-      <c r="J45" s="24" t="inlineStr">
-        <is>
-          <t>네이버뉴스 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K45" s="24" t="inlineStr">
+      <c r="H45" s="22" t="n">
+        <v>1.51</v>
+      </c>
+      <c r="I45" s="22" t="n">
+        <v>13.19</v>
+      </c>
+      <c r="J45" s="23" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +218% / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K45" s="23" t="inlineStr">
         <is>
           <t>네이버</t>
         </is>
@@ -2280,7 +2272,7 @@
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="20" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B46" s="20" t="n">
@@ -2288,14 +2280,14 @@
       </c>
       <c r="C46" s="21" t="inlineStr">
         <is>
-          <t>하이트진로</t>
+          <t>금호건설</t>
         </is>
       </c>
       <c r="D46" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E46" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F46" s="20" t="n">
         <v>0</v>
@@ -2304,24 +2296,26 @@
         <v>0</v>
       </c>
       <c r="H46" s="22" t="n">
-        <v>1.43</v>
-      </c>
-      <c r="I46" s="22" t="n">
-        <v>5.76</v>
-      </c>
-      <c r="J46" s="24" t="inlineStr">
-        <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K46" s="24" t="n">
-        <v/>
+        <v>5.12</v>
+      </c>
+      <c r="I46" s="24" t="n">
+        <v>-6.89</v>
+      </c>
+      <c r="J46" s="23" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +218% / 중요공시 1건</t>
+        </is>
+      </c>
+      <c r="K46" s="23" t="inlineStr">
+        <is>
+          <t>공시, 네이버</t>
+        </is>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="20" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B47" s="20" t="n">
@@ -2329,14 +2323,14 @@
       </c>
       <c r="C47" s="21" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>형지글로벌</t>
         </is>
       </c>
       <c r="D47" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E47" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F47" s="20" t="n">
         <v>0</v>
@@ -2344,25 +2338,27 @@
       <c r="G47" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H47" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I47" s="20" t="n">
-        <v/>
-      </c>
-      <c r="J47" s="24" t="inlineStr">
-        <is>
-          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K47" s="24" t="n">
-        <v/>
+      <c r="H47" s="24" t="n">
+        <v>-18.32</v>
+      </c>
+      <c r="I47" s="24" t="n">
+        <v>-4.29</v>
+      </c>
+      <c r="J47" s="23" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +185% / 중요공시 1건</t>
+        </is>
+      </c>
+      <c r="K47" s="23" t="inlineStr">
+        <is>
+          <t>공시, 네이버</t>
+        </is>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="20" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B48" s="20" t="n">
@@ -2370,7 +2366,7 @@
       </c>
       <c r="C48" s="21" t="inlineStr">
         <is>
-          <t>하이퍼코퍼레이션</t>
+          <t>뉴인텍</t>
         </is>
       </c>
       <c r="D48" s="20" t="n">
@@ -2385,18 +2381,18 @@
       <c r="G48" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H48" s="23" t="n">
-        <v>-24.66</v>
+      <c r="H48" s="24" t="n">
+        <v>-13.33</v>
       </c>
       <c r="I48" s="22" t="n">
-        <v>73.84999999999999</v>
-      </c>
-      <c r="J48" s="24" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +677% / 중요공시 1건</t>
-        </is>
-      </c>
-      <c r="K48" s="24" t="inlineStr">
+        <v>39.09</v>
+      </c>
+      <c r="J48" s="23" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +181% / 중요공시 1건</t>
+        </is>
+      </c>
+      <c r="K48" s="23" t="inlineStr">
         <is>
           <t>공시, 네이버</t>
         </is>
@@ -2405,7 +2401,7 @@
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="20" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B49" s="20" t="n">
@@ -2413,7 +2409,7 @@
       </c>
       <c r="C49" s="21" t="inlineStr">
         <is>
-          <t>금호건설</t>
+          <t>롯데손해보험</t>
         </is>
       </c>
       <c r="D49" s="20" t="n">
@@ -2428,18 +2424,18 @@
       <c r="G49" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H49" s="22" t="n">
-        <v>5.12</v>
-      </c>
-      <c r="I49" s="23" t="n">
-        <v>-6.89</v>
-      </c>
-      <c r="J49" s="24" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +178% / 중요공시 1건</t>
-        </is>
-      </c>
-      <c r="K49" s="24" t="inlineStr">
+      <c r="H49" s="24" t="n">
+        <v>-0.59</v>
+      </c>
+      <c r="I49" s="22" t="n">
+        <v>10.24</v>
+      </c>
+      <c r="J49" s="23" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +159% / 중요공시 1건</t>
+        </is>
+      </c>
+      <c r="K49" s="23" t="inlineStr">
         <is>
           <t>공시, 네이버</t>
         </is>
@@ -2448,7 +2444,7 @@
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="20" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B50" s="20" t="n">
@@ -2456,7 +2452,7 @@
       </c>
       <c r="C50" s="21" t="inlineStr">
         <is>
-          <t>HMM</t>
+          <t>에이엔피</t>
         </is>
       </c>
       <c r="D50" s="20" t="n">
@@ -2472,26 +2468,26 @@
         <v>0</v>
       </c>
       <c r="H50" s="22" t="n">
-        <v>1.51</v>
+        <v>12.93</v>
       </c>
       <c r="I50" s="22" t="n">
-        <v>13.19</v>
-      </c>
-      <c r="J50" s="24" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +162% / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K50" s="24" t="inlineStr">
-        <is>
-          <t>네이버</t>
+        <v>71.89</v>
+      </c>
+      <c r="J50" s="23" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +132% / 중요공시 1건</t>
+        </is>
+      </c>
+      <c r="K50" s="23" t="inlineStr">
+        <is>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="20" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B51" s="20" t="n">
@@ -2499,7 +2495,7 @@
       </c>
       <c r="C51" s="21" t="inlineStr">
         <is>
-          <t>형지글로벌</t>
+          <t>한화시스템</t>
         </is>
       </c>
       <c r="D51" s="20" t="n">
@@ -2514,27 +2510,27 @@
       <c r="G51" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H51" s="23" t="n">
-        <v>-18.32</v>
-      </c>
-      <c r="I51" s="23" t="n">
-        <v>-4.29</v>
-      </c>
-      <c r="J51" s="24" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +136% / 중요공시 1건</t>
-        </is>
-      </c>
-      <c r="K51" s="24" t="inlineStr">
-        <is>
-          <t>공시, 네이버</t>
+      <c r="H51" s="22" t="n">
+        <v>9.08</v>
+      </c>
+      <c r="I51" s="22" t="n">
+        <v>4.95</v>
+      </c>
+      <c r="J51" s="23" t="inlineStr">
+        <is>
+          <t>중요공시 1건 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K51" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="20" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B52" s="20" t="n">
@@ -2542,42 +2538,42 @@
       </c>
       <c r="C52" s="21" t="inlineStr">
         <is>
-          <t>롯데손해보험</t>
+          <t>대우건설</t>
         </is>
       </c>
       <c r="D52" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E52" s="20" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F52" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G52" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H52" s="23" t="n">
-        <v>-0.59</v>
-      </c>
-      <c r="I52" s="22" t="n">
-        <v>10.24</v>
-      </c>
-      <c r="J52" s="24" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +128% / 중요공시 1건</t>
-        </is>
-      </c>
-      <c r="K52" s="24" t="inlineStr">
-        <is>
-          <t>공시, 네이버</t>
+      <c r="H52" s="22" t="n">
+        <v>3.57</v>
+      </c>
+      <c r="I52" s="24" t="n">
+        <v>-10.9</v>
+      </c>
+      <c r="J52" s="23" t="inlineStr">
+        <is>
+          <t>중요공시 2건 / 중요공시 3일 +100%</t>
+        </is>
+      </c>
+      <c r="K52" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="53" ht="18" customHeight="1">
       <c r="A53" s="20" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B53" s="20" t="n">
@@ -2585,7 +2581,7 @@
       </c>
       <c r="C53" s="21" t="inlineStr">
         <is>
-          <t>뉴인텍</t>
+          <t>뉴파워프라즈마</t>
         </is>
       </c>
       <c r="D53" s="20" t="n">
@@ -2600,27 +2596,25 @@
       <c r="G53" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H53" s="23" t="n">
-        <v>-13.33</v>
-      </c>
-      <c r="I53" s="22" t="n">
-        <v>39.09</v>
-      </c>
-      <c r="J53" s="24" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +108% / 중요공시 1건</t>
-        </is>
-      </c>
-      <c r="K53" s="24" t="inlineStr">
-        <is>
-          <t>공시, 네이버</t>
-        </is>
+      <c r="H53" s="22" t="n">
+        <v>12.84</v>
+      </c>
+      <c r="I53" s="24" t="n">
+        <v>-15.86</v>
+      </c>
+      <c r="J53" s="23" t="inlineStr">
+        <is>
+          <t>매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K53" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="54" ht="18" customHeight="1">
       <c r="A54" s="20" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B54" s="20" t="n">
@@ -2628,7 +2622,7 @@
       </c>
       <c r="C54" s="21" t="inlineStr">
         <is>
-          <t>TS트릴리온</t>
+          <t>대한항공</t>
         </is>
       </c>
       <c r="D54" s="20" t="n">
@@ -2643,25 +2637,27 @@
       <c r="G54" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H54" s="22" t="n">
-        <v>21.72</v>
-      </c>
-      <c r="I54" s="22" t="n">
-        <v>29.47</v>
-      </c>
-      <c r="J54" s="24" t="inlineStr">
-        <is>
-          <t>한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K54" s="24" t="n">
-        <v/>
+      <c r="H54" s="24" t="n">
+        <v>-9.25</v>
+      </c>
+      <c r="I54" s="24" t="n">
+        <v>-13.11</v>
+      </c>
+      <c r="J54" s="23" t="inlineStr">
+        <is>
+          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K54" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="55" ht="18" customHeight="1">
       <c r="A55" s="20" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B55" s="20" t="n">
@@ -2669,40 +2665,42 @@
       </c>
       <c r="C55" s="21" t="inlineStr">
         <is>
-          <t>두산에너빌리티</t>
+          <t>태영건설</t>
         </is>
       </c>
       <c r="D55" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E55" s="20" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F55" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G55" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H55" s="22" t="n">
-        <v>4.89</v>
-      </c>
-      <c r="I55" s="23" t="n">
-        <v>-16.04</v>
-      </c>
-      <c r="J55" s="24" t="inlineStr">
-        <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K55" s="24" t="n">
-        <v/>
+        <v>3</v>
+      </c>
+      <c r="H55" s="24" t="n">
+        <v>-1.32</v>
+      </c>
+      <c r="I55" s="24" t="n">
+        <v>-3.81</v>
+      </c>
+      <c r="J55" s="23" t="inlineStr">
+        <is>
+          <t>중요공시 2건 / 중요공시 7일 +100%</t>
+        </is>
+      </c>
+      <c r="K55" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="56" ht="18" customHeight="1">
       <c r="A56" s="20" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B56" s="20" t="n">
@@ -2710,33 +2708,33 @@
       </c>
       <c r="C56" s="21" t="inlineStr">
         <is>
-          <t>우리로</t>
+          <t>테라뷰</t>
         </is>
       </c>
       <c r="D56" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E56" s="20" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F56" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G56" s="20" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H56" s="22" t="n">
-        <v>18.59</v>
-      </c>
-      <c r="I56" s="22" t="n">
-        <v>7.33</v>
-      </c>
-      <c r="J56" s="24" t="inlineStr">
-        <is>
-          <t>중요공시 1건 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K56" s="24" t="inlineStr">
+        <v>4.5</v>
+      </c>
+      <c r="I56" s="24" t="n">
+        <v>-17.4</v>
+      </c>
+      <c r="J56" s="23" t="inlineStr">
+        <is>
+          <t>중요공시 2건 / 중요공시 7일 +100%</t>
+        </is>
+      </c>
+      <c r="K56" s="23" t="inlineStr">
         <is>
           <t>공시</t>
         </is>
@@ -2745,7 +2743,7 @@
     <row r="57" ht="18" customHeight="1">
       <c r="A57" s="20" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B57" s="20" t="n">
@@ -2753,7 +2751,7 @@
       </c>
       <c r="C57" s="21" t="inlineStr">
         <is>
-          <t>대한항공</t>
+          <t>클라우드</t>
         </is>
       </c>
       <c r="D57" s="20" t="n">
@@ -2768,27 +2766,27 @@
       <c r="G57" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H57" s="23" t="n">
-        <v>-9.25</v>
-      </c>
-      <c r="I57" s="23" t="n">
-        <v>-13.11</v>
-      </c>
-      <c r="J57" s="24" t="inlineStr">
-        <is>
-          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K57" s="24" t="inlineStr">
-        <is>
-          <t>공시</t>
+      <c r="H57" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I57" s="20" t="n">
+        <v/>
+      </c>
+      <c r="J57" s="23" t="inlineStr">
+        <is>
+          <t>네이버뉴스 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K57" s="23" t="inlineStr">
+        <is>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="58" ht="18" customHeight="1">
       <c r="A58" s="20" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B58" s="20" t="n">
@@ -2796,7 +2794,7 @@
       </c>
       <c r="C58" s="21" t="inlineStr">
         <is>
-          <t>우진엔텍</t>
+          <t>삼성증권</t>
         </is>
       </c>
       <c r="D58" s="20" t="n">
@@ -2811,27 +2809,27 @@
       <c r="G58" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H58" s="23" t="n">
-        <v>-19.25</v>
-      </c>
-      <c r="I58" s="23" t="n">
-        <v>-19.25</v>
-      </c>
-      <c r="J58" s="24" t="inlineStr">
-        <is>
-          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K58" s="24" t="inlineStr">
-        <is>
-          <t>공시</t>
+      <c r="H58" s="22" t="n">
+        <v>3.95</v>
+      </c>
+      <c r="I58" s="24" t="n">
+        <v>-8.029999999999999</v>
+      </c>
+      <c r="J58" s="23" t="inlineStr">
+        <is>
+          <t>네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K58" s="23" t="inlineStr">
+        <is>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="59" ht="18" customHeight="1">
       <c r="A59" s="20" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B59" s="20" t="n">
@@ -2839,42 +2837,42 @@
       </c>
       <c r="C59" s="21" t="inlineStr">
         <is>
-          <t>테라뷰</t>
+          <t>하이브</t>
         </is>
       </c>
       <c r="D59" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E59" s="20" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F59" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G59" s="20" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H59" s="22" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="I59" s="23" t="n">
-        <v>-17.4</v>
-      </c>
-      <c r="J59" s="24" t="inlineStr">
-        <is>
-          <t>중요공시 2건 / 중요공시 7일 +100%</t>
-        </is>
-      </c>
-      <c r="K59" s="24" t="inlineStr">
-        <is>
-          <t>공시</t>
+        <v>8.23</v>
+      </c>
+      <c r="I59" s="22" t="n">
+        <v>8.23</v>
+      </c>
+      <c r="J59" s="23" t="inlineStr">
+        <is>
+          <t>한국경제 헤드라인 언급 / 네이버뉴스 기사 언급</t>
+        </is>
+      </c>
+      <c r="K59" s="23" t="inlineStr">
+        <is>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="60" ht="18" customHeight="1">
       <c r="A60" s="20" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B60" s="20" t="n">
@@ -2882,7 +2880,7 @@
       </c>
       <c r="C60" s="21" t="inlineStr">
         <is>
-          <t>LG전자</t>
+          <t>TSMC</t>
         </is>
       </c>
       <c r="D60" s="20" t="n">
@@ -2897,18 +2895,18 @@
       <c r="G60" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H60" s="22" t="n">
-        <v>3.14</v>
-      </c>
-      <c r="I60" s="23" t="n">
-        <v>-15.07</v>
-      </c>
-      <c r="J60" s="24" t="inlineStr">
-        <is>
-          <t>네이버뉴스 기사 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K60" s="24" t="inlineStr">
+      <c r="H60" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I60" s="20" t="n">
+        <v/>
+      </c>
+      <c r="J60" s="23" t="inlineStr">
+        <is>
+          <t>네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K60" s="23" t="inlineStr">
         <is>
           <t>네이버</t>
         </is>
@@ -2917,7 +2915,7 @@
     <row r="61" ht="18" customHeight="1">
       <c r="A61" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B61" s="25" t="n">
@@ -2948,7 +2946,7 @@
       </c>
       <c r="J61" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +1724%</t>
+          <t>네이버 검색 당일 +2034%</t>
         </is>
       </c>
       <c r="K61" s="28" t="inlineStr">
@@ -2960,7 +2958,7 @@
     <row r="62" ht="18" customHeight="1">
       <c r="A62" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B62" s="25" t="n">
@@ -2991,7 +2989,7 @@
       </c>
       <c r="J62" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +814%</t>
+          <t>네이버 검색 당일 +1069%</t>
         </is>
       </c>
       <c r="K62" s="28" t="inlineStr">
@@ -3003,7 +3001,7 @@
     <row r="63" ht="18" customHeight="1">
       <c r="A63" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B63" s="25" t="n">
@@ -3011,7 +3009,7 @@
       </c>
       <c r="C63" s="26" t="inlineStr">
         <is>
-          <t>금호전기</t>
+          <t>에스엠벡셀</t>
         </is>
       </c>
       <c r="D63" s="25" t="n">
@@ -3026,15 +3024,15 @@
       <c r="G63" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H63" s="27" t="n">
-        <v>11.46</v>
+      <c r="H63" s="29" t="n">
+        <v>-0.16</v>
       </c>
       <c r="I63" s="27" t="n">
-        <v>12.25</v>
+        <v>38.77</v>
       </c>
       <c r="J63" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +410%</t>
+          <t>네이버 검색 당일 +525%</t>
         </is>
       </c>
       <c r="K63" s="28" t="inlineStr">
@@ -3136,22 +3134,22 @@
         <v>1</v>
       </c>
       <c r="C3" s="25" t="n">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="D3" s="25" t="n">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="E3" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F3" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="G3" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="H3" s="25" t="n"/>
@@ -3177,12 +3175,12 @@
       </c>
       <c r="F4" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="G4" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="H4" s="25" t="n"/>
@@ -3198,22 +3196,22 @@
         <v>1</v>
       </c>
       <c r="C5" s="25" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D5" s="25" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E5" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F5" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="G5" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="H5" s="27" t="n">
@@ -3243,12 +3241,12 @@
       </c>
       <c r="F6" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="G6" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="H6" s="29" t="n">
@@ -3261,38 +3259,42 @@
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="26" t="inlineStr">
         <is>
-          <t>인공지능</t>
+          <t>SK하이닉스</t>
         </is>
       </c>
       <c r="B7" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="25" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D7" s="25" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E7" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F7" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="G7" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="H7" s="25" t="n"/>
-      <c r="I7" s="25" t="n"/>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="H7" s="27" t="n">
+        <v>2.18</v>
+      </c>
+      <c r="I7" s="29" t="n">
+        <v>-24.97</v>
+      </c>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="26" t="inlineStr">
         <is>
-          <t>방산</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="B8" s="25" t="n">
@@ -3309,12 +3311,12 @@
       </c>
       <c r="F8" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="G8" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="H8" s="25" t="n"/>
@@ -3330,22 +3332,22 @@
         <v>1</v>
       </c>
       <c r="C9" s="25" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D9" s="25" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E9" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F9" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="G9" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="H9" s="29" t="n">
@@ -3358,64 +3360,60 @@
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="26" t="inlineStr">
         <is>
-          <t>삼성전기</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="B10" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C10" s="25" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D10" s="25" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E10" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F10" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="G10" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="H10" s="27" t="n">
-        <v>5.53</v>
-      </c>
-      <c r="I10" s="29" t="n">
-        <v>-24.05</v>
-      </c>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="H10" s="25" t="n"/>
+      <c r="I10" s="25" t="n"/>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="26" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>방산</t>
         </is>
       </c>
       <c r="B11" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="25" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D11" s="25" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E11" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F11" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="G11" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="H11" s="25" t="n"/>
@@ -3424,29 +3422,29 @@
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="26" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="B12" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C12" s="25" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D12" s="25" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E12" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F12" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="G12" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="H12" s="25" t="n"/>
@@ -3455,112 +3453,108 @@
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>삼성바이오로직스</t>
+          <t>모아라이프플러스</t>
         </is>
       </c>
       <c r="B13" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C13" s="25" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D13" s="25" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E13" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F13" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="G13" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="H13" s="27" t="n">
-        <v>4.03</v>
+        <v>8.33</v>
       </c>
       <c r="I13" s="27" t="n">
-        <v>5.82</v>
+        <v>0.78</v>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>SK하이닉스</t>
+          <t>엔터</t>
         </is>
       </c>
       <c r="B14" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C14" s="25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D14" s="25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E14" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F14" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="G14" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="H14" s="27" t="n">
-        <v>2.18</v>
-      </c>
-      <c r="I14" s="29" t="n">
-        <v>-24.97</v>
-      </c>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="H14" s="25" t="n"/>
+      <c r="I14" s="25" t="n"/>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>넥사다이내믹스</t>
+          <t>우진엔텍</t>
         </is>
       </c>
       <c r="B15" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C15" s="25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D15" s="25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E15" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F15" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="G15" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="H15" s="27" t="n">
-        <v>2.78</v>
-      </c>
-      <c r="I15" s="27" t="n">
-        <v>12.15</v>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="H15" s="29" t="n">
+        <v>-19.25</v>
+      </c>
+      <c r="I15" s="29" t="n">
+        <v>-19.25</v>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>엔터</t>
+          <t>카카오</t>
         </is>
       </c>
       <c r="B16" s="25" t="n">
@@ -3577,16 +3571,20 @@
       </c>
       <c r="F16" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="G16" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="H16" s="25" t="n"/>
-      <c r="I16" s="25" t="n"/>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="H16" s="27" t="n">
+        <v>2.76</v>
+      </c>
+      <c r="I16" s="29" t="n">
+        <v>-2.16</v>
+      </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
@@ -3608,12 +3606,12 @@
       </c>
       <c r="F17" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="G17" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="H17" s="27" t="n">
@@ -3643,12 +3641,12 @@
       </c>
       <c r="F18" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="G18" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="H18" s="27" t="n">
@@ -3661,7 +3659,7 @@
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>삼성SDI</t>
+          <t>피에스케이</t>
         </is>
       </c>
       <c r="B19" s="25" t="n">
@@ -3678,25 +3676,25 @@
       </c>
       <c r="F19" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="G19" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="H19" s="27" t="n">
-        <v>0.95</v>
+        <v>12.72</v>
       </c>
       <c r="I19" s="29" t="n">
-        <v>-6.53</v>
+        <v>-10.82</v>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="26" t="inlineStr">
         <is>
-          <t>삼성물산</t>
+          <t>피에스케이홀딩스</t>
         </is>
       </c>
       <c r="B20" s="25" t="n">
@@ -3713,25 +3711,25 @@
       </c>
       <c r="F20" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="G20" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="H20" s="27" t="n">
-        <v>7.78</v>
+        <v>10.96</v>
       </c>
       <c r="I20" s="29" t="n">
-        <v>-11.25</v>
+        <v>-4.82</v>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="26" t="inlineStr">
         <is>
-          <t>삼성전자우</t>
+          <t>한화솔루션</t>
         </is>
       </c>
       <c r="B21" s="25" t="n">
@@ -3748,231 +3746,231 @@
       </c>
       <c r="F21" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="G21" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="H21" s="27" t="n">
-        <v>8.539999999999999</v>
+        <v>6.08</v>
       </c>
       <c r="I21" s="29" t="n">
-        <v>-13.11</v>
+        <v>-12.04</v>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="26" t="inlineStr">
         <is>
-          <t>삼성중공업</t>
+          <t>네이버</t>
         </is>
       </c>
       <c r="B22" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C22" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D22" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E22" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F22" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="G22" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="H22" s="27" t="n">
-        <v>2.73</v>
-      </c>
-      <c r="I22" s="29" t="n">
-        <v>-2.49</v>
-      </c>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="H22" s="25" t="n"/>
+      <c r="I22" s="25" t="n"/>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="26" t="inlineStr">
         <is>
-          <t>철강</t>
+          <t>넥사다이내믹스</t>
         </is>
       </c>
       <c r="B23" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C23" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D23" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E23" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F23" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="G23" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="H23" s="25" t="n"/>
-      <c r="I23" s="25" t="n"/>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="H23" s="27" t="n">
+        <v>2.78</v>
+      </c>
+      <c r="I23" s="27" t="n">
+        <v>12.15</v>
+      </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="26" t="inlineStr">
         <is>
-          <t>피에스케이</t>
+          <t>동국제약</t>
         </is>
       </c>
       <c r="B24" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C24" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D24" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E24" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F24" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="G24" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="H24" s="27" t="n">
-        <v>12.72</v>
-      </c>
-      <c r="I24" s="29" t="n">
-        <v>-10.82</v>
+        <v>4.34</v>
+      </c>
+      <c r="I24" s="27" t="n">
+        <v>12.98</v>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="26" t="inlineStr">
         <is>
-          <t>피에스케이홀딩스</t>
+          <t>두산에너빌리티</t>
         </is>
       </c>
       <c r="B25" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C25" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D25" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E25" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F25" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="G25" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="H25" s="27" t="n">
-        <v>10.96</v>
+        <v>4.89</v>
       </c>
       <c r="I25" s="29" t="n">
-        <v>-4.82</v>
+        <v>-16.04</v>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="26" t="inlineStr">
         <is>
-          <t>한화솔루션</t>
+          <t>본느</t>
         </is>
       </c>
       <c r="B26" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C26" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D26" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E26" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F26" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="G26" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="H26" s="27" t="n">
-        <v>6.08</v>
+        <v>6.93</v>
       </c>
       <c r="I26" s="29" t="n">
-        <v>-12.04</v>
+        <v>-17.93</v>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="26" t="inlineStr">
         <is>
-          <t>한화시스템</t>
+          <t>삼성전기</t>
         </is>
       </c>
       <c r="B27" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C27" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D27" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E27" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F27" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="G27" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="H27" s="27" t="n">
-        <v>9.08</v>
-      </c>
-      <c r="I27" s="27" t="n">
-        <v>4.95</v>
+        <v>5.53</v>
+      </c>
+      <c r="I27" s="29" t="n">
+        <v>-24.05</v>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="26" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>에코프로비엠</t>
         </is>
       </c>
       <c r="B28" s="25" t="n">
@@ -3989,21 +3987,25 @@
       </c>
       <c r="F28" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="G28" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="H28" s="25" t="n"/>
-      <c r="I28" s="25" t="n"/>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="H28" s="27" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="I28" s="29" t="n">
+        <v>-15.81</v>
+      </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="26" t="inlineStr">
         <is>
-          <t>모아라이프플러스</t>
+          <t>엘앤씨바이오</t>
         </is>
       </c>
       <c r="B29" s="25" t="n">
@@ -4020,25 +4022,25 @@
       </c>
       <c r="F29" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="G29" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="H29" s="27" t="n">
-        <v>8.33</v>
+        <v>22.98</v>
       </c>
       <c r="I29" s="27" t="n">
-        <v>0.78</v>
+        <v>22.76</v>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="26" t="inlineStr">
         <is>
-          <t>본느</t>
+          <t>우리로</t>
         </is>
       </c>
       <c r="B30" s="25" t="n">
@@ -4055,25 +4057,25 @@
       </c>
       <c r="F30" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="G30" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="H30" s="27" t="n">
-        <v>6.93</v>
-      </c>
-      <c r="I30" s="29" t="n">
-        <v>-17.93</v>
+        <v>18.59</v>
+      </c>
+      <c r="I30" s="27" t="n">
+        <v>7.33</v>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="26" t="inlineStr">
         <is>
-          <t>삼성E&amp;A</t>
+          <t>카카오뱅크</t>
         </is>
       </c>
       <c r="B31" s="25" t="n">
@@ -4090,25 +4092,25 @@
       </c>
       <c r="F31" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="G31" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="H31" s="27" t="n">
-        <v>4.43</v>
-      </c>
-      <c r="I31" s="29" t="n">
-        <v>-8.98</v>
+        <v>1.8</v>
+      </c>
+      <c r="I31" s="27" t="n">
+        <v>4.25</v>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="26" t="inlineStr">
         <is>
-          <t>삼성생명</t>
+          <t>하이트진로</t>
         </is>
       </c>
       <c r="B32" s="25" t="n">
@@ -4125,161 +4127,161 @@
       </c>
       <c r="F32" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="G32" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="H32" s="27" t="n">
-        <v>5.78</v>
-      </c>
-      <c r="I32" s="29" t="n">
-        <v>-11.85</v>
+        <v>1.43</v>
+      </c>
+      <c r="I32" s="27" t="n">
+        <v>5.76</v>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="26" t="inlineStr">
         <is>
-          <t>삼성증권</t>
+          <t>HMM</t>
         </is>
       </c>
       <c r="B33" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C33" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D33" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E33" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F33" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="G33" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="H33" s="27" t="n">
-        <v>3.95</v>
-      </c>
-      <c r="I33" s="29" t="n">
-        <v>-8.029999999999999</v>
+        <v>1.51</v>
+      </c>
+      <c r="I33" s="27" t="n">
+        <v>13.19</v>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="26" t="inlineStr">
         <is>
-          <t>엘앤씨바이오</t>
+          <t>TSMC</t>
         </is>
       </c>
       <c r="B34" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C34" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D34" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E34" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F34" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="G34" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="H34" s="27" t="n">
-        <v>22.98</v>
-      </c>
-      <c r="I34" s="27" t="n">
-        <v>22.76</v>
-      </c>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="H34" s="25" t="n"/>
+      <c r="I34" s="25" t="n"/>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="26" t="inlineStr">
         <is>
-          <t>태양광</t>
+          <t>금호건설</t>
         </is>
       </c>
       <c r="B35" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C35" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D35" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E35" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F35" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="G35" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="H35" s="25" t="n"/>
-      <c r="I35" s="25" t="n"/>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="H35" s="27" t="n">
+        <v>5.12</v>
+      </c>
+      <c r="I35" s="29" t="n">
+        <v>-6.89</v>
+      </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="26" t="inlineStr">
         <is>
-          <t>하이트진로</t>
+          <t>뉴인텍</t>
         </is>
       </c>
       <c r="B36" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C36" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D36" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E36" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F36" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="G36" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="H36" s="27" t="n">
-        <v>1.43</v>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="H36" s="29" t="n">
+        <v>-13.33</v>
       </c>
       <c r="I36" s="27" t="n">
-        <v>5.76</v>
+        <v>39.09</v>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="26" t="inlineStr">
         <is>
-          <t>HMM</t>
+          <t>뉴파워프라즈마</t>
         </is>
       </c>
       <c r="B37" s="25" t="n">
@@ -4296,25 +4298,25 @@
       </c>
       <c r="F37" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="G37" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="H37" s="27" t="n">
-        <v>1.51</v>
-      </c>
-      <c r="I37" s="27" t="n">
-        <v>13.19</v>
+        <v>12.84</v>
+      </c>
+      <c r="I37" s="29" t="n">
+        <v>-15.86</v>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="26" t="inlineStr">
         <is>
-          <t>LG전자</t>
+          <t>대우건설</t>
         </is>
       </c>
       <c r="B38" s="25" t="n">
@@ -4331,25 +4333,25 @@
       </c>
       <c r="F38" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="G38" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="H38" s="27" t="n">
-        <v>3.14</v>
+        <v>3.57</v>
       </c>
       <c r="I38" s="29" t="n">
-        <v>-15.07</v>
+        <v>-10.9</v>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="26" t="inlineStr">
         <is>
-          <t>TS트릴리온</t>
+          <t>대한항공</t>
         </is>
       </c>
       <c r="B39" s="25" t="n">
@@ -4366,25 +4368,25 @@
       </c>
       <c r="F39" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="G39" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="H39" s="27" t="n">
-        <v>21.72</v>
-      </c>
-      <c r="I39" s="27" t="n">
-        <v>29.47</v>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="H39" s="29" t="n">
+        <v>-9.25</v>
+      </c>
+      <c r="I39" s="29" t="n">
+        <v>-13.11</v>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="26" t="inlineStr">
         <is>
-          <t>금호건설</t>
+          <t>롯데손해보험</t>
         </is>
       </c>
       <c r="B40" s="25" t="n">
@@ -4401,25 +4403,25 @@
       </c>
       <c r="F40" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="G40" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="H40" s="27" t="n">
-        <v>5.12</v>
-      </c>
-      <c r="I40" s="29" t="n">
-        <v>-6.89</v>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="H40" s="29" t="n">
+        <v>-0.59</v>
+      </c>
+      <c r="I40" s="27" t="n">
+        <v>10.24</v>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="26" t="inlineStr">
         <is>
-          <t>뉴인텍</t>
+          <t>삼성증권</t>
         </is>
       </c>
       <c r="B41" s="25" t="n">
@@ -4436,25 +4438,25 @@
       </c>
       <c r="F41" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="G41" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="H41" s="29" t="n">
-        <v>-13.33</v>
-      </c>
-      <c r="I41" s="27" t="n">
-        <v>39.09</v>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="H41" s="27" t="n">
+        <v>3.95</v>
+      </c>
+      <c r="I41" s="29" t="n">
+        <v>-8.029999999999999</v>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="26" t="inlineStr">
         <is>
-          <t>대한항공</t>
+          <t>에이엔피</t>
         </is>
       </c>
       <c r="B42" s="25" t="n">
@@ -4471,25 +4473,25 @@
       </c>
       <c r="F42" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="G42" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="H42" s="29" t="n">
-        <v>-9.25</v>
-      </c>
-      <c r="I42" s="29" t="n">
-        <v>-13.11</v>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="H42" s="27" t="n">
+        <v>12.93</v>
+      </c>
+      <c r="I42" s="27" t="n">
+        <v>71.89</v>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="26" t="inlineStr">
         <is>
-          <t>두산에너빌리티</t>
+          <t>클라우드</t>
         </is>
       </c>
       <c r="B43" s="25" t="n">
@@ -4506,25 +4508,21 @@
       </c>
       <c r="F43" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="G43" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="H43" s="27" t="n">
-        <v>4.89</v>
-      </c>
-      <c r="I43" s="29" t="n">
-        <v>-16.04</v>
-      </c>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="H43" s="25" t="n"/>
+      <c r="I43" s="25" t="n"/>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="26" t="inlineStr">
         <is>
-          <t>롯데손해보험</t>
+          <t>태영건설</t>
         </is>
       </c>
       <c r="B44" s="25" t="n">
@@ -4541,25 +4539,25 @@
       </c>
       <c r="F44" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="G44" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="H44" s="29" t="n">
-        <v>-0.59</v>
-      </c>
-      <c r="I44" s="27" t="n">
-        <v>10.24</v>
+        <v>-1.32</v>
+      </c>
+      <c r="I44" s="29" t="n">
+        <v>-3.81</v>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="26" t="inlineStr">
         <is>
-          <t>우리로</t>
+          <t>테라뷰</t>
         </is>
       </c>
       <c r="B45" s="25" t="n">
@@ -4576,25 +4574,25 @@
       </c>
       <c r="F45" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="G45" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="H45" s="27" t="n">
-        <v>18.59</v>
-      </c>
-      <c r="I45" s="27" t="n">
-        <v>7.33</v>
+        <v>4.5</v>
+      </c>
+      <c r="I45" s="29" t="n">
+        <v>-17.4</v>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="26" t="inlineStr">
         <is>
-          <t>우진엔텍</t>
+          <t>하이브</t>
         </is>
       </c>
       <c r="B46" s="25" t="n">
@@ -4611,25 +4609,25 @@
       </c>
       <c r="F46" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="G46" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="H46" s="29" t="n">
-        <v>-19.25</v>
-      </c>
-      <c r="I46" s="29" t="n">
-        <v>-19.25</v>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="H46" s="27" t="n">
+        <v>8.23</v>
+      </c>
+      <c r="I46" s="27" t="n">
+        <v>8.23</v>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="26" t="inlineStr">
         <is>
-          <t>테라뷰</t>
+          <t>하이퍼코퍼레이션</t>
         </is>
       </c>
       <c r="B47" s="25" t="n">
@@ -4646,25 +4644,25 @@
       </c>
       <c r="F47" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="G47" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="H47" s="27" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="I47" s="29" t="n">
-        <v>-17.4</v>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="H47" s="29" t="n">
+        <v>-24.66</v>
+      </c>
+      <c r="I47" s="27" t="n">
+        <v>73.84999999999999</v>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="26" t="inlineStr">
         <is>
-          <t>하이퍼코퍼레이션</t>
+          <t>한화시스템</t>
         </is>
       </c>
       <c r="B48" s="25" t="n">
@@ -4681,19 +4679,19 @@
       </c>
       <c r="F48" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="G48" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="H48" s="29" t="n">
-        <v>-24.66</v>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="H48" s="27" t="n">
+        <v>9.08</v>
       </c>
       <c r="I48" s="27" t="n">
-        <v>73.84999999999999</v>
+        <v>4.95</v>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
@@ -4716,12 +4714,12 @@
       </c>
       <c r="F49" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="G49" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="H49" s="29" t="n">
@@ -4751,12 +4749,12 @@
       </c>
       <c r="F50" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="G50" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="H50" s="27" t="n">
@@ -4769,7 +4767,7 @@
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="26" t="inlineStr">
         <is>
-          <t>금호전기</t>
+          <t>멜콘</t>
         </is>
       </c>
       <c r="B51" s="25" t="n">
@@ -4786,25 +4784,25 @@
       </c>
       <c r="F51" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="G51" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="H51" s="27" t="n">
-        <v>11.46</v>
-      </c>
-      <c r="I51" s="27" t="n">
-        <v>12.25</v>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="H51" s="29" t="n">
+        <v>-13.49</v>
+      </c>
+      <c r="I51" s="29" t="n">
+        <v>-13.49</v>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="26" t="inlineStr">
         <is>
-          <t>멜콘</t>
+          <t>에스엠벡셀</t>
         </is>
       </c>
       <c r="B52" s="25" t="n">
@@ -4821,19 +4819,19 @@
       </c>
       <c r="F52" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="G52" s="25" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="H52" s="29" t="n">
-        <v>-13.49</v>
-      </c>
-      <c r="I52" s="29" t="n">
-        <v>-13.49</v>
+        <v>-0.16</v>
+      </c>
+      <c r="I52" s="27" t="n">
+        <v>38.77</v>
       </c>
     </row>
   </sheetData>
@@ -4917,19 +4915,19 @@
         <v>1</v>
       </c>
       <c r="C3" s="36" t="n">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="D3" s="36" t="n">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="E3" s="36" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="F3" s="37" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="G3" s="37" t="inlineStr">
@@ -4955,12 +4953,12 @@
       </c>
       <c r="E4" s="36" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="F4" s="37" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="G4" s="37" t="inlineStr">
@@ -4979,19 +4977,19 @@
         <v>1</v>
       </c>
       <c r="C5" s="36" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D5" s="36" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E5" s="36" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="F5" s="37" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="G5" s="37" t="inlineStr">
@@ -5010,19 +5008,19 @@
         <v>1</v>
       </c>
       <c r="C6" s="36" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D6" s="36" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E6" s="36" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="F6" s="37" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="G6" s="37" t="inlineStr">
@@ -5034,26 +5032,26 @@
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="35" t="inlineStr">
         <is>
-          <t>태양광</t>
+          <t>엔터</t>
         </is>
       </c>
       <c r="B7" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="36" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D7" s="36" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E7" s="36" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="F7" s="37" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="G7" s="37" t="inlineStr">
@@ -5065,26 +5063,26 @@
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="35" t="inlineStr">
         <is>
-          <t>엔터</t>
+          <t>클라우드</t>
         </is>
       </c>
       <c r="B8" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="36" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D8" s="36" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E8" s="36" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="F8" s="37" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="G8" s="37" t="inlineStr">
@@ -5096,26 +5094,26 @@
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="35" t="inlineStr">
         <is>
-          <t>철강</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="B9" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="36" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D9" s="36" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E9" s="36" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="F9" s="37" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="G9" s="37" t="inlineStr">
@@ -5127,26 +5125,26 @@
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="35" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="B10" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C10" s="36" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D10" s="36" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E10" s="36" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="F10" s="37" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="G10" s="37" t="inlineStr">
@@ -5156,40 +5154,36 @@
       </c>
     </row>
     <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="35" t="inlineStr">
-        <is>
-          <t>인공지능</t>
-        </is>
-      </c>
-      <c r="B11" s="36" t="n">
-        <v>1</v>
-      </c>
-      <c r="C11" s="36" t="n">
-        <v>14</v>
-      </c>
-      <c r="D11" s="36" t="n">
-        <v>14</v>
-      </c>
-      <c r="E11" s="36" t="inlineStr">
-        <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="F11" s="37" t="inlineStr">
-        <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="G11" s="37" t="inlineStr">
-        <is>
-          <t>⚡ 관심</t>
-        </is>
-      </c>
+      <c r="A11" s="26" t="inlineStr">
+        <is>
+          <t>이차전지</t>
+        </is>
+      </c>
+      <c r="B11" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F11" s="28" t="inlineStr">
+        <is>
+          <t>감지 없음</t>
+        </is>
+      </c>
+      <c r="G11" s="28" t="inlineStr"/>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="26" t="inlineStr">
         <is>
-          <t>이차전지</t>
+          <t>AI반도체</t>
         </is>
       </c>
       <c r="B12" s="25" t="n">
@@ -5216,7 +5210,7 @@
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>AI반도체</t>
+          <t>전기차</t>
         </is>
       </c>
       <c r="B13" s="25" t="n">
@@ -5243,7 +5237,7 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>전기차</t>
+          <t>원전</t>
         </is>
       </c>
       <c r="B14" s="25" t="n">
@@ -5270,7 +5264,7 @@
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>원전</t>
+          <t>수소</t>
         </is>
       </c>
       <c r="B15" s="25" t="n">
@@ -5297,7 +5291,7 @@
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>수소</t>
+          <t>태양광</t>
         </is>
       </c>
       <c r="B16" s="25" t="n">
@@ -5378,7 +5372,7 @@
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>클라우드</t>
+          <t>조선</t>
         </is>
       </c>
       <c r="B19" s="25" t="n">
@@ -5405,7 +5399,7 @@
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="26" t="inlineStr">
         <is>
-          <t>조선</t>
+          <t>철강</t>
         </is>
       </c>
       <c r="B20" s="25" t="n">

</xml_diff>

<commit_message>
auto: 2026-10-20 06:54 자동 백업
</commit_message>
<xml_diff>
--- a/trend/stock_trend_history.xlsx
+++ b/trend/stock_trend_history.xlsx
@@ -57,13 +57,13 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="002563EB"/>
+      <color rgb="00E53935"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00E53935"/>
+      <color rgb="002563EB"/>
       <sz val="10"/>
     </font>
     <font>
@@ -258,14 +258,14 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -694,7 +694,7 @@
     <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-10-19 06:54</t>
+          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-10-20 06:54</t>
         </is>
       </c>
     </row>
@@ -708,7 +708,7 @@
       </c>
       <c r="E3" s="3" t="n"/>
       <c r="G3" s="5" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="H3" s="3" t="n"/>
       <c r="J3" s="6" t="n">
@@ -787,21 +787,21 @@
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-10-19) 상위: 반도체  점수 49.0점</t>
+          <t>⚡ 최신(2026-10-20) 상위: 반도체  점수 68.0점</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-10-19) 상위: LG  점수 20.0점</t>
+          <t>⚡ 최신(2026-10-20) 상위: LG  점수 22.0점</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-10-19) 상위: 바이오  점수 17.0점</t>
+          <t>⚡ 최신(2026-10-20) 상위: 방산  점수 20.0점</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="15" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B14" s="15" t="n">
@@ -928,10 +928,10 @@
         </is>
       </c>
       <c r="D14" s="15" t="n">
-        <v>49</v>
+        <v>68</v>
       </c>
       <c r="E14" s="15" t="n">
-        <v>49</v>
+        <v>68</v>
       </c>
       <c r="F14" s="15" t="n">
         <v>0</v>
@@ -947,19 +947,19 @@
       </c>
       <c r="J14" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급</t>
+          <t>Google 급상승 검색어 등장 (KR) / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급</t>
         </is>
       </c>
       <c r="K14" s="17" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>네이버, Google</t>
         </is>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="15" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B15" s="15" t="n">
@@ -971,10 +971,10 @@
         </is>
       </c>
       <c r="D15" s="15" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E15" s="15" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="F15" s="15" t="n">
         <v>0</v>
@@ -983,24 +983,26 @@
         <v>0</v>
       </c>
       <c r="H15" s="18" t="n">
-        <v>-1.16</v>
-      </c>
-      <c r="I15" s="18" t="n">
-        <v>-3.66</v>
+        <v>1.66</v>
+      </c>
+      <c r="I15" s="19" t="n">
+        <v>-2.07</v>
       </c>
       <c r="J15" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K15" s="17" t="n">
-        <v/>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 한국경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K15" s="17" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="15" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B16" s="15" t="n">
@@ -1008,14 +1010,14 @@
       </c>
       <c r="C16" s="16" t="inlineStr">
         <is>
-          <t>바이오</t>
+          <t>방산</t>
         </is>
       </c>
       <c r="D16" s="15" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E16" s="15" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="F16" s="15" t="n">
         <v>0</v>
@@ -1031,7 +1033,7 @@
       </c>
       <c r="J16" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
+          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K16" s="17" t="inlineStr">
@@ -1043,7 +1045,7 @@
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B17" s="15" t="n">
@@ -1051,14 +1053,14 @@
       </c>
       <c r="C17" s="16" t="inlineStr">
         <is>
-          <t>인공지능</t>
+          <t>바이오</t>
         </is>
       </c>
       <c r="D17" s="15" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E17" s="15" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F17" s="15" t="n">
         <v>0</v>
@@ -1074,7 +1076,7 @@
       </c>
       <c r="J17" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K17" s="17" t="inlineStr">
@@ -1086,7 +1088,7 @@
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B18" s="15" t="n">
@@ -1094,14 +1096,14 @@
       </c>
       <c r="C18" s="16" t="inlineStr">
         <is>
-          <t>방산</t>
+          <t>SK하이닉스</t>
         </is>
       </c>
       <c r="D18" s="15" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E18" s="15" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F18" s="15" t="n">
         <v>0</v>
@@ -1109,25 +1111,27 @@
       <c r="G18" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H18" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I18" s="15" t="n">
-        <v/>
+      <c r="H18" s="18" t="n">
+        <v>3.08</v>
+      </c>
+      <c r="I18" s="19" t="n">
+        <v>-18.75</v>
       </c>
       <c r="J18" s="17" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K18" s="17" t="n">
-        <v/>
+          <t>네이버 검색 당일 +152% / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K18" s="17" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B19" s="15" t="n">
@@ -1135,14 +1139,14 @@
       </c>
       <c r="C19" s="16" t="inlineStr">
         <is>
-          <t>LG전자</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="D19" s="15" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E19" s="15" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F19" s="15" t="n">
         <v>0</v>
@@ -1150,25 +1154,27 @@
       <c r="G19" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H19" s="19" t="n">
-        <v>3.14</v>
-      </c>
-      <c r="I19" s="18" t="n">
-        <v>-7.88</v>
+      <c r="H19" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I19" s="15" t="n">
+        <v/>
       </c>
       <c r="J19" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K19" s="17" t="n">
-        <v/>
+          <t>네이버뉴스 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K19" s="17" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B20" s="15" t="n">
@@ -1176,42 +1182,42 @@
       </c>
       <c r="C20" s="16" t="inlineStr">
         <is>
-          <t>삼성전자</t>
+          <t>현대로템</t>
         </is>
       </c>
       <c r="D20" s="15" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E20" s="15" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F20" s="15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G20" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H20" s="19" t="n">
-        <v>4.58</v>
-      </c>
-      <c r="I20" s="18" t="n">
-        <v>-13.55</v>
+      <c r="H20" s="18" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="I20" s="19" t="n">
+        <v>-0.2</v>
       </c>
       <c r="J20" s="17" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +93% / 중요공시 1건 / 네이버뉴스 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+          <t>중요공시 4건 / 중요공시 3일 +300% / 매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K20" s="17" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="15" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B21" s="15" t="n">
@@ -1242,7 +1248,7 @@
       </c>
       <c r="J21" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K21" s="17" t="inlineStr">
@@ -1254,7 +1260,7 @@
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="15" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B22" s="15" t="n">
@@ -1262,42 +1268,42 @@
       </c>
       <c r="C22" s="16" t="inlineStr">
         <is>
-          <t>모아데이타</t>
+          <t>전기차</t>
         </is>
       </c>
       <c r="D22" s="15" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E22" s="15" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="F22" s="15" t="n">
         <v>0</v>
       </c>
       <c r="G22" s="15" t="n">
-        <v>3</v>
-      </c>
-      <c r="H22" s="18" t="n">
-        <v>-14.95</v>
-      </c>
-      <c r="I22" s="19" t="n">
-        <v>8.140000000000001</v>
+        <v>0</v>
+      </c>
+      <c r="H22" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I22" s="15" t="n">
+        <v/>
       </c>
       <c r="J22" s="17" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +125% / 중요공시 6건 / 중요공시 7일 +200%</t>
+          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K22" s="17" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="15" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B23" s="15" t="n">
@@ -1305,42 +1311,42 @@
       </c>
       <c r="C23" s="16" t="inlineStr">
         <is>
-          <t>모아라이프플러스</t>
+          <t>HD현대중공업</t>
         </is>
       </c>
       <c r="D23" s="15" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E23" s="15" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F23" s="15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G23" s="15" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H23" s="19" t="n">
-        <v>8.33</v>
+        <v>-1.14</v>
       </c>
       <c r="I23" s="19" t="n">
-        <v>7.22</v>
+        <v>-3.47</v>
       </c>
       <c r="J23" s="17" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +105% / 중요공시 7건 / 중요공시 7일 +600%</t>
+          <t>중요공시 3건 / 중요공시 3일 +50% / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K23" s="17" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="15" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B24" s="15" t="n">
@@ -1348,14 +1354,14 @@
       </c>
       <c r="C24" s="16" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>삼성전기</t>
         </is>
       </c>
       <c r="D24" s="15" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E24" s="15" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F24" s="15" t="n">
         <v>0</v>
@@ -1363,25 +1369,27 @@
       <c r="G24" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H24" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I24" s="15" t="n">
-        <v/>
+      <c r="H24" s="18" t="n">
+        <v>3.04</v>
+      </c>
+      <c r="I24" s="19" t="n">
+        <v>-18.29</v>
       </c>
       <c r="J24" s="17" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K24" s="17" t="n">
-        <v/>
+          <t>중요공시 1건 / 매일경제 기사 언급 / 네이버뉴스 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K24" s="17" t="inlineStr">
+        <is>
+          <t>네이버, 공시</t>
+        </is>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="15" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B25" s="15" t="n">
@@ -1393,10 +1401,10 @@
         </is>
       </c>
       <c r="D25" s="15" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E25" s="15" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F25" s="15" t="n">
         <v>0</v>
@@ -1404,15 +1412,15 @@
       <c r="G25" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H25" s="19" t="n">
-        <v>8.460000000000001</v>
+      <c r="H25" s="18" t="n">
+        <v>3.34</v>
       </c>
       <c r="I25" s="18" t="n">
-        <v>-1.41</v>
+        <v>1.88</v>
       </c>
       <c r="J25" s="17" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K25" s="17" t="inlineStr">
@@ -1424,7 +1432,7 @@
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="15" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B26" s="15" t="n">
@@ -1432,42 +1440,42 @@
       </c>
       <c r="C26" s="16" t="inlineStr">
         <is>
-          <t>CS</t>
+          <t>모아데이타</t>
         </is>
       </c>
       <c r="D26" s="15" t="n">
         <v>9</v>
       </c>
       <c r="E26" s="15" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="F26" s="15" t="n">
         <v>0</v>
       </c>
       <c r="G26" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H26" s="18" t="n">
-        <v>-0.68</v>
-      </c>
-      <c r="I26" s="18" t="n">
-        <v>-1.67</v>
+        <v>3</v>
+      </c>
+      <c r="H26" s="19" t="n">
+        <v>-14.64</v>
+      </c>
+      <c r="I26" s="19" t="n">
+        <v>-7.69</v>
       </c>
       <c r="J26" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급</t>
+          <t>네이버 검색 당일 +131% / 중요공시 7건 / 중요공시 7일 +250%</t>
         </is>
       </c>
       <c r="K26" s="17" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="15" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B27" s="15" t="n">
@@ -1475,42 +1483,42 @@
       </c>
       <c r="C27" s="16" t="inlineStr">
         <is>
-          <t>HD현대중공업</t>
+          <t>모아라이프플러스</t>
         </is>
       </c>
       <c r="D27" s="15" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E27" s="15" t="n">
         <v>6</v>
       </c>
       <c r="F27" s="15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G27" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H27" s="19" t="n">
-        <v>1.01</v>
+        <v>3</v>
+      </c>
+      <c r="H27" s="18" t="n">
+        <v>12.31</v>
       </c>
       <c r="I27" s="18" t="n">
-        <v>-2.36</v>
+        <v>20.41</v>
       </c>
       <c r="J27" s="17" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 3일 +100% / Google 급상승 검색어 등장 (KR)</t>
+          <t>네이버 검색 당일 +110% / 중요공시 6건 / 중요공시 7일 +500%</t>
         </is>
       </c>
       <c r="K27" s="17" t="inlineStr">
         <is>
-          <t>Google, 공시</t>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="15" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B28" s="15" t="n">
@@ -1518,40 +1526,42 @@
       </c>
       <c r="C28" s="16" t="inlineStr">
         <is>
-          <t>조선</t>
+          <t>빅텍</t>
         </is>
       </c>
       <c r="D28" s="15" t="n">
         <v>8</v>
       </c>
       <c r="E28" s="15" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="F28" s="15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G28" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H28" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I28" s="15" t="n">
-        <v/>
+        <v>3</v>
+      </c>
+      <c r="H28" s="18" t="n">
+        <v>3.29</v>
+      </c>
+      <c r="I28" s="18" t="n">
+        <v>2.93</v>
       </c>
       <c r="J28" s="17" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K28" s="17" t="n">
-        <v/>
+          <t>중요공시 3건 / 중요공시 3일 +200% / 중요공시 7일 +200%</t>
+        </is>
+      </c>
+      <c r="K28" s="17" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="15" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B29" s="15" t="n">
@@ -1559,14 +1569,14 @@
       </c>
       <c r="C29" s="16" t="inlineStr">
         <is>
-          <t>우진엔텍</t>
+          <t>한미반도체</t>
         </is>
       </c>
       <c r="D29" s="15" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E29" s="15" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F29" s="15" t="n">
         <v>0</v>
@@ -1575,26 +1585,26 @@
         <v>0</v>
       </c>
       <c r="H29" s="18" t="n">
-        <v>-19.25</v>
-      </c>
-      <c r="I29" s="18" t="n">
-        <v>-19.25</v>
+        <v>2.85</v>
+      </c>
+      <c r="I29" s="19" t="n">
+        <v>-12.7</v>
       </c>
       <c r="J29" s="17" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +191% / 중요공시 1건 / 매일경제 헤드라인 언급</t>
+          <t>Google 급상승 검색어 등장 (KR) / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K29" s="17" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>Google</t>
         </is>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="15" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B30" s="15" t="n">
@@ -1602,14 +1612,14 @@
       </c>
       <c r="C30" s="16" t="inlineStr">
         <is>
-          <t>엔터</t>
+          <t>삼성SDI</t>
         </is>
       </c>
       <c r="D30" s="15" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E30" s="15" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F30" s="15" t="n">
         <v>0</v>
@@ -1617,27 +1627,27 @@
       <c r="G30" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H30" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I30" s="15" t="n">
-        <v/>
+      <c r="H30" s="18" t="n">
+        <v>11.51</v>
+      </c>
+      <c r="I30" s="18" t="n">
+        <v>5.35</v>
       </c>
       <c r="J30" s="17" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 네이버뉴스 기사 언급</t>
+          <t>Google 급상승 검색어 등장 (KR) / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K30" s="17" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>Google</t>
         </is>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="15" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B31" s="15" t="n">
@@ -1645,42 +1655,42 @@
       </c>
       <c r="C31" s="16" t="inlineStr">
         <is>
-          <t>전기차</t>
+          <t>LG디스플레이</t>
         </is>
       </c>
       <c r="D31" s="15" t="n">
         <v>7</v>
       </c>
       <c r="E31" s="15" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F31" s="15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G31" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H31" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I31" s="15" t="n">
-        <v/>
+      <c r="H31" s="18" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="I31" s="19" t="n">
+        <v>-3.09</v>
       </c>
       <c r="J31" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 기사 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>중요공시 2건 / 중요공시 3일 +100% / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K31" s="17" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="15" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B32" s="15" t="n">
@@ -1688,7 +1698,7 @@
       </c>
       <c r="C32" s="16" t="inlineStr">
         <is>
-          <t>게임</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="D32" s="15" t="n">
@@ -1711,7 +1721,7 @@
       </c>
       <c r="J32" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K32" s="17" t="n">
@@ -1719,43 +1729,43 @@
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
-      <c r="A33" s="20" t="inlineStr">
-        <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="B33" s="20" t="n">
+      <c r="A33" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B33" s="15" t="n">
         <v>20</v>
       </c>
-      <c r="C33" s="21" t="inlineStr">
-        <is>
-          <t>SK하이닉스</t>
-        </is>
-      </c>
-      <c r="D33" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="E33" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="F33" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G33" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H33" s="22" t="n">
-        <v>2.18</v>
-      </c>
-      <c r="I33" s="23" t="n">
-        <v>-21.18</v>
-      </c>
-      <c r="J33" s="24" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +146% / 매일경제 기사 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K33" s="24" t="inlineStr">
+      <c r="C33" s="16" t="inlineStr">
+        <is>
+          <t>하이브</t>
+        </is>
+      </c>
+      <c r="D33" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="E33" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="F33" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H33" s="18" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="I33" s="18" t="n">
+        <v>19.28</v>
+      </c>
+      <c r="J33" s="17" t="inlineStr">
+        <is>
+          <t>매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급</t>
+        </is>
+      </c>
+      <c r="K33" s="17" t="inlineStr">
         <is>
           <t>네이버</t>
         </is>
@@ -1764,7 +1774,7 @@
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="20" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B34" s="20" t="n">
@@ -1772,33 +1782,33 @@
       </c>
       <c r="C34" s="21" t="inlineStr">
         <is>
-          <t>다보링크</t>
+          <t>한화시스템</t>
         </is>
       </c>
       <c r="D34" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E34" s="20" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F34" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G34" s="20" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H34" s="22" t="n">
-        <v>9.51</v>
+        <v>1.24</v>
       </c>
       <c r="I34" s="22" t="n">
-        <v>11.42</v>
-      </c>
-      <c r="J34" s="24" t="inlineStr">
-        <is>
-          <t>중요공시 3건 / 중요공시 7일 +50%</t>
-        </is>
-      </c>
-      <c r="K34" s="24" t="inlineStr">
+        <v>9.4</v>
+      </c>
+      <c r="J34" s="23" t="inlineStr">
+        <is>
+          <t>중요공시 1건 / 매일경제 기사 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K34" s="23" t="inlineStr">
         <is>
           <t>공시</t>
         </is>
@@ -1807,7 +1817,7 @@
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="20" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B35" s="20" t="n">
@@ -1815,42 +1825,42 @@
       </c>
       <c r="C35" s="21" t="inlineStr">
         <is>
-          <t>현대제철</t>
+          <t>LG에너지솔루션</t>
         </is>
       </c>
       <c r="D35" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E35" s="20" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F35" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G35" s="20" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H35" s="22" t="n">
-        <v>4.82</v>
+        <v>6.2</v>
       </c>
       <c r="I35" s="22" t="n">
-        <v>3.1</v>
-      </c>
-      <c r="J35" s="24" t="inlineStr">
-        <is>
-          <t>Google 급상승 검색어 등장 (KR) / 네이버뉴스 기사 언급</t>
-        </is>
-      </c>
-      <c r="K35" s="24" t="inlineStr">
-        <is>
-          <t>Google, 네이버</t>
+        <v>8.07</v>
+      </c>
+      <c r="J35" s="23" t="inlineStr">
+        <is>
+          <t>중요공시 2건 / 중요공시 3일 +100% / 중요공시 7일 +100%</t>
+        </is>
+      </c>
+      <c r="K35" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="20" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B36" s="20" t="n">
@@ -1858,40 +1868,42 @@
       </c>
       <c r="C36" s="21" t="inlineStr">
         <is>
-          <t>LG유플러스</t>
+          <t>알테오젠</t>
         </is>
       </c>
       <c r="D36" s="20" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E36" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F36" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G36" s="20" t="n">
         <v>0</v>
       </c>
       <c r="H36" s="22" t="n">
-        <v>3.06</v>
+        <v>2.35</v>
       </c>
       <c r="I36" s="22" t="n">
-        <v>7.19</v>
-      </c>
-      <c r="J36" s="24" t="inlineStr">
-        <is>
-          <t>한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K36" s="24" t="n">
-        <v/>
+        <v>4.81</v>
+      </c>
+      <c r="J36" s="23" t="inlineStr">
+        <is>
+          <t>중요공시 2건 / 중요공시 3일 +100% / 네이버뉴스 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K36" s="23" t="inlineStr">
+        <is>
+          <t>네이버, 공시</t>
+        </is>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="20" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B37" s="20" t="n">
@@ -1899,42 +1911,42 @@
       </c>
       <c r="C37" s="21" t="inlineStr">
         <is>
-          <t>엘앤씨바이오</t>
+          <t>삼성전자</t>
         </is>
       </c>
       <c r="D37" s="20" t="n">
         <v>5</v>
       </c>
       <c r="E37" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="F37" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H37" s="22" t="n">
         <v>3</v>
       </c>
-      <c r="F37" s="20" t="n">
-        <v>2</v>
-      </c>
-      <c r="G37" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H37" s="22" t="n">
-        <v>22.98</v>
-      </c>
-      <c r="I37" s="22" t="n">
-        <v>5.87</v>
-      </c>
-      <c r="J37" s="24" t="inlineStr">
-        <is>
-          <t>중요공시 3건 / 중요공시 3일 +50%</t>
-        </is>
-      </c>
-      <c r="K37" s="24" t="inlineStr">
-        <is>
-          <t>공시</t>
+      <c r="I37" s="24" t="n">
+        <v>-10.96</v>
+      </c>
+      <c r="J37" s="23" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +98% / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K37" s="23" t="inlineStr">
+        <is>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="20" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B38" s="20" t="n">
@@ -1942,42 +1954,40 @@
       </c>
       <c r="C38" s="21" t="inlineStr">
         <is>
-          <t>에코프로비엠</t>
+          <t>SG</t>
         </is>
       </c>
       <c r="D38" s="20" t="n">
         <v>5</v>
       </c>
       <c r="E38" s="20" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F38" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G38" s="20" t="n">
         <v>0</v>
       </c>
       <c r="H38" s="22" t="n">
-        <v>3.7</v>
-      </c>
-      <c r="I38" s="23" t="n">
-        <v>-8.029999999999999</v>
-      </c>
-      <c r="J38" s="24" t="inlineStr">
-        <is>
-          <t>중요공시 3건 / 중요공시 3일 +50%</t>
-        </is>
-      </c>
-      <c r="K38" s="24" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+        <v>6.22</v>
+      </c>
+      <c r="I38" s="24" t="n">
+        <v>-1.63</v>
+      </c>
+      <c r="J38" s="23" t="inlineStr">
+        <is>
+          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K38" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="20" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B39" s="20" t="n">
@@ -1985,42 +1995,42 @@
       </c>
       <c r="C39" s="21" t="inlineStr">
         <is>
-          <t>본느</t>
+          <t>SFA반도체</t>
         </is>
       </c>
       <c r="D39" s="20" t="n">
         <v>5</v>
       </c>
       <c r="E39" s="20" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F39" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G39" s="20" t="n">
         <v>0</v>
       </c>
       <c r="H39" s="22" t="n">
-        <v>6.93</v>
-      </c>
-      <c r="I39" s="23" t="n">
-        <v>-13.6</v>
-      </c>
-      <c r="J39" s="24" t="inlineStr">
-        <is>
-          <t>중요공시 3건 / 중요공시 3일 +200%</t>
-        </is>
-      </c>
-      <c r="K39" s="24" t="inlineStr">
-        <is>
-          <t>공시</t>
+        <v>0.32</v>
+      </c>
+      <c r="I39" s="24" t="n">
+        <v>-12.78</v>
+      </c>
+      <c r="J39" s="23" t="inlineStr">
+        <is>
+          <t>Google 급상승 검색어 등장 (KR)</t>
+        </is>
+      </c>
+      <c r="K39" s="23" t="inlineStr">
+        <is>
+          <t>Google</t>
         </is>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="20" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B40" s="20" t="n">
@@ -2028,40 +2038,42 @@
       </c>
       <c r="C40" s="21" t="inlineStr">
         <is>
-          <t>기아</t>
+          <t>에코프로</t>
         </is>
       </c>
       <c r="D40" s="20" t="n">
         <v>5</v>
       </c>
       <c r="E40" s="20" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F40" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G40" s="20" t="n">
         <v>0</v>
       </c>
       <c r="H40" s="22" t="n">
-        <v>5.42</v>
+        <v>10.55</v>
       </c>
       <c r="I40" s="22" t="n">
-        <v>3.16</v>
-      </c>
-      <c r="J40" s="24" t="inlineStr">
-        <is>
-          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K40" s="24" t="n">
-        <v/>
+        <v>7.39</v>
+      </c>
+      <c r="J40" s="23" t="inlineStr">
+        <is>
+          <t>중요공시 3건 / 중요공시 3일 +50%</t>
+        </is>
+      </c>
+      <c r="K40" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="20" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B41" s="20" t="n">
@@ -2069,42 +2081,42 @@
       </c>
       <c r="C41" s="21" t="inlineStr">
         <is>
-          <t>하이퍼코퍼레이션</t>
+          <t>스피어</t>
         </is>
       </c>
       <c r="D41" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E41" s="20" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F41" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G41" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H41" s="23" t="n">
-        <v>-24.66</v>
-      </c>
-      <c r="I41" s="22" t="n">
-        <v>52.51</v>
-      </c>
-      <c r="J41" s="24" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +966% / 중요공시 1건</t>
-        </is>
-      </c>
-      <c r="K41" s="24" t="inlineStr">
-        <is>
-          <t>공시, 네이버</t>
+      <c r="H41" s="22" t="n">
+        <v>3.04</v>
+      </c>
+      <c r="I41" s="24" t="n">
+        <v>-4.76</v>
+      </c>
+      <c r="J41" s="23" t="inlineStr">
+        <is>
+          <t>중요공시 3건 / 중요공시 3일 +50%</t>
+        </is>
+      </c>
+      <c r="K41" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="20" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B42" s="20" t="n">
@@ -2112,14 +2124,14 @@
       </c>
       <c r="C42" s="21" t="inlineStr">
         <is>
-          <t>HMM</t>
+          <t>제주반도체</t>
         </is>
       </c>
       <c r="D42" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E42" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F42" s="20" t="n">
         <v>0</v>
@@ -2128,26 +2140,26 @@
         <v>0</v>
       </c>
       <c r="H42" s="22" t="n">
-        <v>1.51</v>
-      </c>
-      <c r="I42" s="22" t="n">
-        <v>8.01</v>
-      </c>
-      <c r="J42" s="24" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +232% / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K42" s="24" t="inlineStr">
-        <is>
-          <t>네이버</t>
+        <v>2.9</v>
+      </c>
+      <c r="I42" s="24" t="n">
+        <v>-11.93</v>
+      </c>
+      <c r="J42" s="23" t="inlineStr">
+        <is>
+          <t>Google 급상승 검색어 등장 (KR)</t>
+        </is>
+      </c>
+      <c r="K42" s="23" t="inlineStr">
+        <is>
+          <t>Google</t>
         </is>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="20" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B43" s="20" t="n">
@@ -2155,14 +2167,14 @@
       </c>
       <c r="C43" s="21" t="inlineStr">
         <is>
-          <t>금호건설</t>
+          <t>AI반도체</t>
         </is>
       </c>
       <c r="D43" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E43" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F43" s="20" t="n">
         <v>0</v>
@@ -2170,27 +2182,27 @@
       <c r="G43" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H43" s="22" t="n">
-        <v>5.12</v>
-      </c>
-      <c r="I43" s="23" t="n">
-        <v>-25.36</v>
-      </c>
-      <c r="J43" s="24" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +223% / 중요공시 1건</t>
-        </is>
-      </c>
-      <c r="K43" s="24" t="inlineStr">
-        <is>
-          <t>공시, 네이버</t>
+      <c r="H43" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I43" s="20" t="n">
+        <v/>
+      </c>
+      <c r="J43" s="23" t="inlineStr">
+        <is>
+          <t>Google 급상승 검색어 등장 (KR)</t>
+        </is>
+      </c>
+      <c r="K43" s="23" t="inlineStr">
+        <is>
+          <t>Google</t>
         </is>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="20" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B44" s="20" t="n">
@@ -2198,14 +2210,14 @@
       </c>
       <c r="C44" s="21" t="inlineStr">
         <is>
-          <t>형지글로벌</t>
+          <t>클라우드</t>
         </is>
       </c>
       <c r="D44" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E44" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F44" s="20" t="n">
         <v>0</v>
@@ -2213,27 +2225,27 @@
       <c r="G44" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H44" s="23" t="n">
-        <v>-18.32</v>
-      </c>
-      <c r="I44" s="23" t="n">
-        <v>-24.46</v>
-      </c>
-      <c r="J44" s="24" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +197% / 중요공시 1건</t>
-        </is>
-      </c>
-      <c r="K44" s="24" t="inlineStr">
-        <is>
-          <t>공시, 네이버</t>
+      <c r="H44" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I44" s="20" t="n">
+        <v/>
+      </c>
+      <c r="J44" s="23" t="inlineStr">
+        <is>
+          <t>매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
+        </is>
+      </c>
+      <c r="K44" s="23" t="inlineStr">
+        <is>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="20" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B45" s="20" t="n">
@@ -2241,7 +2253,7 @@
       </c>
       <c r="C45" s="21" t="inlineStr">
         <is>
-          <t>뉴인텍</t>
+          <t>바이오인프라</t>
         </is>
       </c>
       <c r="D45" s="20" t="n">
@@ -2256,27 +2268,27 @@
       <c r="G45" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H45" s="23" t="n">
-        <v>-13.33</v>
+      <c r="H45" s="20" t="n">
+        <v>0</v>
       </c>
       <c r="I45" s="22" t="n">
-        <v>89.89</v>
-      </c>
-      <c r="J45" s="24" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +194% / 중요공시 1건</t>
-        </is>
-      </c>
-      <c r="K45" s="24" t="inlineStr">
-        <is>
-          <t>공시, 네이버</t>
+        <v>119.52</v>
+      </c>
+      <c r="J45" s="23" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +242% / 중요공시 1건</t>
+        </is>
+      </c>
+      <c r="K45" s="23" t="inlineStr">
+        <is>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="20" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B46" s="20" t="n">
@@ -2284,7 +2296,7 @@
       </c>
       <c r="C46" s="21" t="inlineStr">
         <is>
-          <t>롯데손해보험</t>
+          <t>형지글로벌</t>
         </is>
       </c>
       <c r="D46" s="20" t="n">
@@ -2299,27 +2311,27 @@
       <c r="G46" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H46" s="23" t="n">
-        <v>-0.59</v>
-      </c>
-      <c r="I46" s="22" t="n">
-        <v>7.66</v>
-      </c>
-      <c r="J46" s="24" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +167% / 중요공시 1건</t>
-        </is>
-      </c>
-      <c r="K46" s="24" t="inlineStr">
-        <is>
-          <t>공시, 네이버</t>
+      <c r="H46" s="24" t="n">
+        <v>-5.45</v>
+      </c>
+      <c r="I46" s="24" t="n">
+        <v>-28.57</v>
+      </c>
+      <c r="J46" s="23" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +206% / 중요공시 1건</t>
+        </is>
+      </c>
+      <c r="K46" s="23" t="inlineStr">
+        <is>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="20" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B47" s="20" t="n">
@@ -2327,7 +2339,7 @@
       </c>
       <c r="C47" s="21" t="inlineStr">
         <is>
-          <t>에이엔피</t>
+          <t>뉴인텍</t>
         </is>
       </c>
       <c r="D47" s="20" t="n">
@@ -2343,26 +2355,26 @@
         <v>0</v>
       </c>
       <c r="H47" s="22" t="n">
-        <v>12.93</v>
+        <v>29.88</v>
       </c>
       <c r="I47" s="22" t="n">
-        <v>117.26</v>
-      </c>
-      <c r="J47" s="24" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +145% / 중요공시 1건</t>
-        </is>
-      </c>
-      <c r="K47" s="24" t="inlineStr">
-        <is>
-          <t>공시, 네이버</t>
+        <v>146.63</v>
+      </c>
+      <c r="J47" s="23" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +205% / 중요공시 1건</t>
+        </is>
+      </c>
+      <c r="K47" s="23" t="inlineStr">
+        <is>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="20" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B48" s="20" t="n">
@@ -2370,42 +2382,42 @@
       </c>
       <c r="C48" s="21" t="inlineStr">
         <is>
-          <t>LG디스플레이</t>
+          <t>롯데손해보험</t>
         </is>
       </c>
       <c r="D48" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E48" s="20" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F48" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G48" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H48" s="22" t="n">
-        <v>2.46</v>
-      </c>
-      <c r="I48" s="23" t="n">
-        <v>-3.35</v>
-      </c>
-      <c r="J48" s="24" t="inlineStr">
-        <is>
-          <t>중요공시 2건 / 중요공시 3일 +100%</t>
-        </is>
-      </c>
-      <c r="K48" s="24" t="inlineStr">
-        <is>
-          <t>공시</t>
+      <c r="H48" s="24" t="n">
+        <v>-1.98</v>
+      </c>
+      <c r="I48" s="22" t="n">
+        <v>5.53</v>
+      </c>
+      <c r="J48" s="23" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +175% / 중요공시 1건</t>
+        </is>
+      </c>
+      <c r="K48" s="23" t="inlineStr">
+        <is>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="20" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B49" s="20" t="n">
@@ -2413,42 +2425,42 @@
       </c>
       <c r="C49" s="21" t="inlineStr">
         <is>
-          <t>대우건설</t>
+          <t>에이엔피</t>
         </is>
       </c>
       <c r="D49" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E49" s="20" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F49" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G49" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H49" s="22" t="n">
-        <v>3.57</v>
-      </c>
-      <c r="I49" s="23" t="n">
-        <v>-7.04</v>
-      </c>
-      <c r="J49" s="24" t="inlineStr">
-        <is>
-          <t>중요공시 2건 / 중요공시 3일 +100%</t>
-        </is>
-      </c>
-      <c r="K49" s="24" t="inlineStr">
-        <is>
-          <t>공시</t>
+      <c r="H49" s="24" t="n">
+        <v>-29.91</v>
+      </c>
+      <c r="I49" s="22" t="n">
+        <v>52.28</v>
+      </c>
+      <c r="J49" s="23" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +158% / 중요공시 1건</t>
+        </is>
+      </c>
+      <c r="K49" s="23" t="inlineStr">
+        <is>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="20" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B50" s="20" t="n">
@@ -2456,33 +2468,33 @@
       </c>
       <c r="C50" s="21" t="inlineStr">
         <is>
-          <t>LG에너지솔루션</t>
+          <t>대우건설</t>
         </is>
       </c>
       <c r="D50" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E50" s="20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F50" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G50" s="20" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H50" s="22" t="n">
-        <v>2.67</v>
-      </c>
-      <c r="I50" s="22" t="n">
-        <v>1.77</v>
-      </c>
-      <c r="J50" s="24" t="inlineStr">
-        <is>
-          <t>중요공시 2건 / 중요공시 7일 +100%</t>
-        </is>
-      </c>
-      <c r="K50" s="24" t="inlineStr">
+        <v>1.62</v>
+      </c>
+      <c r="I50" s="24" t="n">
+        <v>-5.53</v>
+      </c>
+      <c r="J50" s="23" t="inlineStr">
+        <is>
+          <t>중요공시 2건 / 중요공시 3일 +100%</t>
+        </is>
+      </c>
+      <c r="K50" s="23" t="inlineStr">
         <is>
           <t>공시</t>
         </is>
@@ -2491,7 +2503,7 @@
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="20" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B51" s="20" t="n">
@@ -2499,42 +2511,42 @@
       </c>
       <c r="C51" s="21" t="inlineStr">
         <is>
-          <t>테라뷰</t>
+          <t>지투지바이오</t>
         </is>
       </c>
       <c r="D51" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E51" s="20" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F51" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G51" s="20" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H51" s="22" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="I51" s="23" t="n">
-        <v>-15.33</v>
-      </c>
-      <c r="J51" s="24" t="inlineStr">
-        <is>
-          <t>중요공시 2건 / 중요공시 7일 +100%</t>
-        </is>
-      </c>
-      <c r="K51" s="24" t="inlineStr">
-        <is>
-          <t>공시</t>
+        <v>24.64</v>
+      </c>
+      <c r="I51" s="22" t="n">
+        <v>5.56</v>
+      </c>
+      <c r="J51" s="23" t="inlineStr">
+        <is>
+          <t>중요공시 1건 / 네이버뉴스 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K51" s="23" t="inlineStr">
+        <is>
+          <t>네이버, 공시</t>
         </is>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="20" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B52" s="20" t="n">
@@ -2542,165 +2554,171 @@
       </c>
       <c r="C52" s="21" t="inlineStr">
         <is>
-          <t>삼성바이오로직스</t>
+          <t>철강</t>
         </is>
       </c>
       <c r="D52" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E52" s="20" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F52" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G52" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H52" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I52" s="20" t="n">
+        <v/>
+      </c>
+      <c r="J52" s="23" t="inlineStr">
+        <is>
+          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급</t>
+        </is>
+      </c>
+      <c r="K52" s="23" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="18" customHeight="1">
+      <c r="A53" s="25" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B53" s="25" t="n">
+        <v>40</v>
+      </c>
+      <c r="C53" s="26" t="inlineStr">
+        <is>
+          <t>멜콘</t>
+        </is>
+      </c>
+      <c r="D53" s="25" t="n">
         <v>3</v>
       </c>
-      <c r="H52" s="22" t="n">
-        <v>4.03</v>
-      </c>
-      <c r="I52" s="22" t="n">
-        <v>7.94</v>
-      </c>
-      <c r="J52" s="24" t="inlineStr">
-        <is>
-          <t>중요공시 2건 / 중요공시 7일 +100%</t>
-        </is>
-      </c>
-      <c r="K52" s="24" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="18" customHeight="1">
-      <c r="A53" s="20" t="inlineStr">
-        <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="B53" s="20" t="n">
-        <v>40</v>
-      </c>
-      <c r="C53" s="21" t="inlineStr">
-        <is>
-          <t>삼성전기</t>
-        </is>
-      </c>
-      <c r="D53" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E53" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F53" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G53" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H53" s="22" t="n">
-        <v>5.53</v>
-      </c>
-      <c r="I53" s="23" t="n">
-        <v>-20.7</v>
-      </c>
-      <c r="J53" s="24" t="inlineStr">
-        <is>
-          <t>한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K53" s="24" t="n">
-        <v/>
+      <c r="E53" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F53" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G53" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H53" s="27" t="n">
+        <v>-0.34</v>
+      </c>
+      <c r="I53" s="27" t="n">
+        <v>-13.79</v>
+      </c>
+      <c r="J53" s="28" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +1122%</t>
+        </is>
+      </c>
+      <c r="K53" s="28" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="54" ht="18" customHeight="1">
-      <c r="A54" s="20" t="inlineStr">
-        <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="B54" s="20" t="n">
+      <c r="A54" s="25" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B54" s="25" t="n">
         <v>41</v>
       </c>
-      <c r="C54" s="21" t="inlineStr">
-        <is>
-          <t>진에어</t>
-        </is>
-      </c>
-      <c r="D54" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E54" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F54" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G54" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H54" s="23" t="n">
-        <v>-2.45</v>
-      </c>
-      <c r="I54" s="22" t="n">
-        <v>4.93</v>
-      </c>
-      <c r="J54" s="24" t="inlineStr">
-        <is>
-          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K54" s="24" t="n">
-        <v/>
+      <c r="C54" s="26" t="inlineStr">
+        <is>
+          <t>에스엠벡셀</t>
+        </is>
+      </c>
+      <c r="D54" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E54" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F54" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G54" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H54" s="29" t="n">
+        <v>28.25</v>
+      </c>
+      <c r="I54" s="29" t="n">
+        <v>91.02</v>
+      </c>
+      <c r="J54" s="28" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +582%</t>
+        </is>
+      </c>
+      <c r="K54" s="28" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="55" ht="18" customHeight="1">
-      <c r="A55" s="20" t="inlineStr">
-        <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="B55" s="20" t="n">
+      <c r="A55" s="25" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B55" s="25" t="n">
         <v>42</v>
       </c>
-      <c r="C55" s="21" t="inlineStr">
-        <is>
-          <t>한국콜마</t>
-        </is>
-      </c>
-      <c r="D55" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E55" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F55" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G55" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H55" s="22" t="n">
-        <v>8.06</v>
-      </c>
-      <c r="I55" s="23" t="n">
-        <v>-0.84</v>
-      </c>
-      <c r="J55" s="24" t="inlineStr">
-        <is>
-          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K55" s="24" t="n">
-        <v/>
+      <c r="C55" s="26" t="inlineStr">
+        <is>
+          <t>금호전기</t>
+        </is>
+      </c>
+      <c r="D55" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E55" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F55" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G55" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H55" s="27" t="n">
+        <v>-1.47</v>
+      </c>
+      <c r="I55" s="27" t="n">
+        <v>-15.18</v>
+      </c>
+      <c r="J55" s="28" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +510%</t>
+        </is>
+      </c>
+      <c r="K55" s="28" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
     <row r="56" ht="18" customHeight="1">
       <c r="A56" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B56" s="25" t="n">
@@ -2708,7 +2726,7 @@
       </c>
       <c r="C56" s="26" t="inlineStr">
         <is>
-          <t>HC보광산업</t>
+          <t>HT로보틱스</t>
         </is>
       </c>
       <c r="D56" s="25" t="n">
@@ -2723,15 +2741,15 @@
       <c r="G56" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H56" s="27" t="n">
-        <v>14.17</v>
-      </c>
-      <c r="I56" s="27" t="n">
-        <v>13.24</v>
+      <c r="H56" s="29" t="n">
+        <v>3.51</v>
+      </c>
+      <c r="I56" s="29" t="n">
+        <v>49.59</v>
       </c>
       <c r="J56" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +2101%</t>
+          <t>네이버 검색 당일 +503%</t>
         </is>
       </c>
       <c r="K56" s="28" t="inlineStr">
@@ -2743,7 +2761,7 @@
     <row r="57" ht="18" customHeight="1">
       <c r="A57" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B57" s="25" t="n">
@@ -2751,7 +2769,7 @@
       </c>
       <c r="C57" s="26" t="inlineStr">
         <is>
-          <t>멜콘</t>
+          <t>TS트릴리온</t>
         </is>
       </c>
       <c r="D57" s="25" t="n">
@@ -2766,15 +2784,15 @@
       <c r="G57" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H57" s="29" t="n">
-        <v>-13.49</v>
+      <c r="H57" s="27" t="n">
+        <v>-7.14</v>
       </c>
       <c r="I57" s="29" t="n">
-        <v>-13.49</v>
+        <v>22.23</v>
       </c>
       <c r="J57" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +1100%</t>
+          <t>네이버 검색 당일 +375%</t>
         </is>
       </c>
       <c r="K57" s="28" t="inlineStr">
@@ -2786,7 +2804,7 @@
     <row r="58" ht="18" customHeight="1">
       <c r="A58" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B58" s="25" t="n">
@@ -2794,7 +2812,7 @@
       </c>
       <c r="C58" s="26" t="inlineStr">
         <is>
-          <t>에스엠벡셀</t>
+          <t>한화갤러리아우</t>
         </is>
       </c>
       <c r="D58" s="25" t="n">
@@ -2810,14 +2828,14 @@
         <v>0</v>
       </c>
       <c r="H58" s="29" t="n">
-        <v>-0.16</v>
-      </c>
-      <c r="I58" s="27" t="n">
-        <v>48.94</v>
+        <v>10.96</v>
+      </c>
+      <c r="I58" s="29" t="n">
+        <v>35.45</v>
       </c>
       <c r="J58" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +553%</t>
+          <t>네이버 검색 당일 +342%</t>
         </is>
       </c>
       <c r="K58" s="28" t="inlineStr">
@@ -2829,7 +2847,7 @@
     <row r="59" ht="18" customHeight="1">
       <c r="A59" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B59" s="25" t="n">
@@ -2837,7 +2855,7 @@
       </c>
       <c r="C59" s="26" t="inlineStr">
         <is>
-          <t>금호전기</t>
+          <t>화성밸브</t>
         </is>
       </c>
       <c r="D59" s="25" t="n">
@@ -2852,15 +2870,15 @@
       <c r="G59" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H59" s="27" t="n">
-        <v>11.46</v>
+      <c r="H59" s="29" t="n">
+        <v>9.67</v>
       </c>
       <c r="I59" s="29" t="n">
-        <v>-13.91</v>
+        <v>33.94</v>
       </c>
       <c r="J59" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +502%</t>
+          <t>네이버 검색 당일 +307%</t>
         </is>
       </c>
       <c r="K59" s="28" t="inlineStr">
@@ -2872,7 +2890,7 @@
     <row r="60" ht="18" customHeight="1">
       <c r="A60" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B60" s="25" t="n">
@@ -2880,7 +2898,7 @@
       </c>
       <c r="C60" s="26" t="inlineStr">
         <is>
-          <t>HT로보틱스</t>
+          <t>HMM</t>
         </is>
       </c>
       <c r="D60" s="25" t="n">
@@ -2895,15 +2913,15 @@
       <c r="G60" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H60" s="27" t="n">
-        <v>23.5</v>
-      </c>
-      <c r="I60" s="27" t="n">
-        <v>44.52</v>
+      <c r="H60" s="29" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="I60" s="29" t="n">
+        <v>9.380000000000001</v>
       </c>
       <c r="J60" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +466%</t>
+          <t>네이버 검색 당일 +242%</t>
         </is>
       </c>
       <c r="K60" s="28" t="inlineStr">
@@ -2915,7 +2933,7 @@
     <row r="61" ht="18" customHeight="1">
       <c r="A61" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B61" s="25" t="n">
@@ -2923,7 +2941,7 @@
       </c>
       <c r="C61" s="26" t="inlineStr">
         <is>
-          <t>듀켐바이오</t>
+          <t>팬오션</t>
         </is>
       </c>
       <c r="D61" s="25" t="n">
@@ -2939,14 +2957,14 @@
         <v>0</v>
       </c>
       <c r="H61" s="29" t="n">
-        <v>-2.9</v>
-      </c>
-      <c r="I61" s="27" t="n">
-        <v>25.14</v>
+        <v>1.05</v>
+      </c>
+      <c r="I61" s="29" t="n">
+        <v>3.06</v>
       </c>
       <c r="J61" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +462%</t>
+          <t>네이버 검색 당일 +240%</t>
         </is>
       </c>
       <c r="K61" s="28" t="inlineStr">
@@ -2958,7 +2976,7 @@
     <row r="62" ht="18" customHeight="1">
       <c r="A62" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B62" s="25" t="n">
@@ -2966,7 +2984,7 @@
       </c>
       <c r="C62" s="26" t="inlineStr">
         <is>
-          <t>TS트릴리온</t>
+          <t>한선엔지니어링</t>
         </is>
       </c>
       <c r="D62" s="25" t="n">
@@ -2981,15 +2999,15 @@
       <c r="G62" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H62" s="27" t="n">
-        <v>21.72</v>
-      </c>
-      <c r="I62" s="27" t="n">
-        <v>31.63</v>
+      <c r="H62" s="29" t="n">
+        <v>3.07</v>
+      </c>
+      <c r="I62" s="29" t="n">
+        <v>31.24</v>
       </c>
       <c r="J62" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +314%</t>
+          <t>네이버 검색 당일 +238%</t>
         </is>
       </c>
       <c r="K62" s="28" t="inlineStr">
@@ -3001,7 +3019,7 @@
     <row r="63" ht="18" customHeight="1">
       <c r="A63" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B63" s="25" t="n">
@@ -3009,7 +3027,7 @@
       </c>
       <c r="C63" s="26" t="inlineStr">
         <is>
-          <t>화성밸브</t>
+          <t>서산</t>
         </is>
       </c>
       <c r="D63" s="25" t="n">
@@ -3024,15 +3042,15 @@
       <c r="G63" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H63" s="27" t="n">
-        <v>10.71</v>
-      </c>
-      <c r="I63" s="27" t="n">
-        <v>22.13</v>
+      <c r="H63" s="29" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="I63" s="29" t="n">
+        <v>20.27</v>
       </c>
       <c r="J63" s="28" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +291%</t>
+          <t>네이버 검색 당일 +206%</t>
         </is>
       </c>
       <c r="K63" s="28" t="inlineStr">
@@ -3134,22 +3152,22 @@
         <v>1</v>
       </c>
       <c r="C3" s="25" t="n">
-        <v>49</v>
+        <v>68</v>
       </c>
       <c r="D3" s="25" t="n">
-        <v>49</v>
+        <v>68</v>
       </c>
       <c r="E3" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F3" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="G3" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="H3" s="25" t="n"/>
@@ -3165,57 +3183,57 @@
         <v>1</v>
       </c>
       <c r="C4" s="25" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D4" s="25" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E4" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F4" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="G4" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="H4" s="29" t="n">
-        <v>-1.16</v>
-      </c>
-      <c r="I4" s="29" t="n">
-        <v>-3.66</v>
+        <v>1.66</v>
+      </c>
+      <c r="I4" s="27" t="n">
+        <v>-2.07</v>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="26" t="inlineStr">
         <is>
-          <t>바이오</t>
+          <t>방산</t>
         </is>
       </c>
       <c r="B5" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="25" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D5" s="25" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E5" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F5" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="G5" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="H5" s="25" t="n"/>
@@ -3224,29 +3242,29 @@
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="26" t="inlineStr">
         <is>
-          <t>인공지능</t>
+          <t>바이오</t>
         </is>
       </c>
       <c r="B6" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="25" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D6" s="25" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E6" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F6" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="G6" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="H6" s="25" t="n"/>
@@ -3255,64 +3273,64 @@
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="26" t="inlineStr">
         <is>
-          <t>LG전자</t>
+          <t>SK하이닉스</t>
         </is>
       </c>
       <c r="B7" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="25" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D7" s="25" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E7" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F7" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="G7" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="H7" s="27" t="n">
-        <v>3.14</v>
-      </c>
-      <c r="I7" s="29" t="n">
-        <v>-7.88</v>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="H7" s="29" t="n">
+        <v>3.08</v>
+      </c>
+      <c r="I7" s="27" t="n">
+        <v>-18.75</v>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="26" t="inlineStr">
         <is>
-          <t>방산</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="B8" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="25" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D8" s="25" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E8" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F8" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="G8" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="H8" s="25" t="n"/>
@@ -3321,42 +3339,42 @@
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="26" t="inlineStr">
         <is>
-          <t>삼성전자</t>
+          <t>현대로템</t>
         </is>
       </c>
       <c r="B9" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="25" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D9" s="25" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E9" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F9" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="G9" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="H9" s="27" t="n">
-        <v>4.58</v>
-      </c>
-      <c r="I9" s="29" t="n">
-        <v>-13.55</v>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="H9" s="29" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="I9" s="27" t="n">
+        <v>-0.2</v>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="26" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>전기차</t>
         </is>
       </c>
       <c r="B10" s="25" t="n">
@@ -3373,12 +3391,12 @@
       </c>
       <c r="F10" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="G10" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="H10" s="25" t="n"/>
@@ -3387,143 +3405,143 @@
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="26" t="inlineStr">
         <is>
-          <t>CS</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="B11" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="25" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D11" s="25" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E11" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F11" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="G11" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="H11" s="29" t="n">
-        <v>-0.68</v>
-      </c>
-      <c r="I11" s="29" t="n">
-        <v>-1.67</v>
-      </c>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="H11" s="25" t="n"/>
+      <c r="I11" s="25" t="n"/>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="26" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>HD현대중공업</t>
         </is>
       </c>
       <c r="B12" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C12" s="25" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D12" s="25" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E12" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F12" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="G12" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="H12" s="25" t="n"/>
-      <c r="I12" s="25" t="n"/>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="H12" s="27" t="n">
+        <v>-1.14</v>
+      </c>
+      <c r="I12" s="27" t="n">
+        <v>-3.47</v>
+      </c>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>모아데이타</t>
+          <t>삼성전기</t>
         </is>
       </c>
       <c r="B13" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C13" s="25" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D13" s="25" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E13" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F13" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="G13" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="H13" s="29" t="n">
-        <v>-14.95</v>
+        <v>3.04</v>
       </c>
       <c r="I13" s="27" t="n">
-        <v>8.140000000000001</v>
+        <v>-18.29</v>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>모아라이프플러스</t>
+          <t>현대차</t>
         </is>
       </c>
       <c r="B14" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C14" s="25" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D14" s="25" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E14" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F14" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="G14" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="H14" s="27" t="n">
-        <v>8.33</v>
-      </c>
-      <c r="I14" s="27" t="n">
-        <v>7.22</v>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="H14" s="29" t="n">
+        <v>3.34</v>
+      </c>
+      <c r="I14" s="29" t="n">
+        <v>1.88</v>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>현대차</t>
+          <t>모아데이타</t>
         </is>
       </c>
       <c r="B15" s="25" t="n">
@@ -3540,60 +3558,60 @@
       </c>
       <c r="F15" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="G15" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="H15" s="27" t="n">
-        <v>8.460000000000001</v>
-      </c>
-      <c r="I15" s="29" t="n">
-        <v>-1.41</v>
+        <v>-14.64</v>
+      </c>
+      <c r="I15" s="27" t="n">
+        <v>-7.69</v>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>HD현대중공업</t>
+          <t>모아라이프플러스</t>
         </is>
       </c>
       <c r="B16" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C16" s="25" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D16" s="25" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E16" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F16" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="G16" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="H16" s="27" t="n">
-        <v>1.01</v>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="H16" s="29" t="n">
+        <v>12.31</v>
       </c>
       <c r="I16" s="29" t="n">
-        <v>-2.36</v>
+        <v>20.41</v>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>조선</t>
+          <t>빅텍</t>
         </is>
       </c>
       <c r="B17" s="25" t="n">
@@ -3610,83 +3628,95 @@
       </c>
       <c r="F17" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="G17" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="H17" s="25" t="n"/>
-      <c r="I17" s="25" t="n"/>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="H17" s="29" t="n">
+        <v>3.29</v>
+      </c>
+      <c r="I17" s="29" t="n">
+        <v>2.93</v>
+      </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="26" t="inlineStr">
         <is>
-          <t>게임</t>
+          <t>삼성SDI</t>
         </is>
       </c>
       <c r="B18" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C18" s="25" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D18" s="25" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E18" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F18" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="G18" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="H18" s="25" t="n"/>
-      <c r="I18" s="25" t="n"/>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="H18" s="29" t="n">
+        <v>11.51</v>
+      </c>
+      <c r="I18" s="29" t="n">
+        <v>5.35</v>
+      </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>엔터</t>
+          <t>한미반도체</t>
         </is>
       </c>
       <c r="B19" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C19" s="25" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D19" s="25" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E19" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F19" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="G19" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="H19" s="25" t="n"/>
-      <c r="I19" s="25" t="n"/>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="H19" s="29" t="n">
+        <v>2.85</v>
+      </c>
+      <c r="I19" s="27" t="n">
+        <v>-12.7</v>
+      </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="26" t="inlineStr">
         <is>
-          <t>우진엔텍</t>
+          <t>LG디스플레이</t>
         </is>
       </c>
       <c r="B20" s="25" t="n">
@@ -3703,25 +3733,25 @@
       </c>
       <c r="F20" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="G20" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="H20" s="29" t="n">
-        <v>-19.25</v>
-      </c>
-      <c r="I20" s="29" t="n">
-        <v>-19.25</v>
+        <v>0.27</v>
+      </c>
+      <c r="I20" s="27" t="n">
+        <v>-3.09</v>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="26" t="inlineStr">
         <is>
-          <t>전기차</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="B21" s="25" t="n">
@@ -3738,12 +3768,12 @@
       </c>
       <c r="F21" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="G21" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="H21" s="25" t="n"/>
@@ -3752,42 +3782,42 @@
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="26" t="inlineStr">
         <is>
-          <t>SK하이닉스</t>
+          <t>하이브</t>
         </is>
       </c>
       <c r="B22" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C22" s="25" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D22" s="25" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E22" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F22" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="G22" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="H22" s="27" t="n">
-        <v>2.18</v>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="H22" s="29" t="n">
+        <v>4.9</v>
       </c>
       <c r="I22" s="29" t="n">
-        <v>-21.18</v>
+        <v>19.28</v>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="26" t="inlineStr">
         <is>
-          <t>다보링크</t>
+          <t>LG에너지솔루션</t>
         </is>
       </c>
       <c r="B23" s="25" t="n">
@@ -3804,25 +3834,25 @@
       </c>
       <c r="F23" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="G23" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="H23" s="27" t="n">
-        <v>9.51</v>
-      </c>
-      <c r="I23" s="27" t="n">
-        <v>11.42</v>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="H23" s="29" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="I23" s="29" t="n">
+        <v>8.07</v>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="26" t="inlineStr">
         <is>
-          <t>현대제철</t>
+          <t>알테오젠</t>
         </is>
       </c>
       <c r="B24" s="25" t="n">
@@ -3839,60 +3869,60 @@
       </c>
       <c r="F24" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="G24" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="H24" s="27" t="n">
-        <v>4.82</v>
-      </c>
-      <c r="I24" s="27" t="n">
-        <v>3.1</v>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="H24" s="29" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="I24" s="29" t="n">
+        <v>4.81</v>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="26" t="inlineStr">
         <is>
-          <t>LG유플러스</t>
+          <t>한화시스템</t>
         </is>
       </c>
       <c r="B25" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C25" s="25" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D25" s="25" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E25" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F25" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="G25" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="H25" s="27" t="n">
-        <v>3.06</v>
-      </c>
-      <c r="I25" s="27" t="n">
-        <v>7.19</v>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="H25" s="29" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="I25" s="29" t="n">
+        <v>9.4</v>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="26" t="inlineStr">
         <is>
-          <t>기아</t>
+          <t>AI반도체</t>
         </is>
       </c>
       <c r="B26" s="25" t="n">
@@ -3909,25 +3939,21 @@
       </c>
       <c r="F26" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="G26" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="H26" s="27" t="n">
-        <v>5.42</v>
-      </c>
-      <c r="I26" s="27" t="n">
-        <v>3.16</v>
-      </c>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="H26" s="25" t="n"/>
+      <c r="I26" s="25" t="n"/>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="26" t="inlineStr">
         <is>
-          <t>본느</t>
+          <t>SFA반도체</t>
         </is>
       </c>
       <c r="B27" s="25" t="n">
@@ -3944,25 +3970,25 @@
       </c>
       <c r="F27" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="G27" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="H27" s="27" t="n">
-        <v>6.93</v>
-      </c>
-      <c r="I27" s="29" t="n">
-        <v>-13.6</v>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="H27" s="29" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="I27" s="27" t="n">
+        <v>-12.78</v>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="26" t="inlineStr">
         <is>
-          <t>에코프로비엠</t>
+          <t>SG</t>
         </is>
       </c>
       <c r="B28" s="25" t="n">
@@ -3979,25 +4005,25 @@
       </c>
       <c r="F28" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="G28" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="H28" s="27" t="n">
-        <v>3.7</v>
-      </c>
-      <c r="I28" s="29" t="n">
-        <v>-8.029999999999999</v>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="H28" s="29" t="n">
+        <v>6.22</v>
+      </c>
+      <c r="I28" s="27" t="n">
+        <v>-1.63</v>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="26" t="inlineStr">
         <is>
-          <t>엘앤씨바이오</t>
+          <t>삼성전자</t>
         </is>
       </c>
       <c r="B29" s="25" t="n">
@@ -4014,160 +4040,156 @@
       </c>
       <c r="F29" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="G29" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="H29" s="27" t="n">
-        <v>22.98</v>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="H29" s="29" t="n">
+        <v>3</v>
       </c>
       <c r="I29" s="27" t="n">
-        <v>5.87</v>
+        <v>-10.96</v>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="26" t="inlineStr">
         <is>
-          <t>HMM</t>
+          <t>스피어</t>
         </is>
       </c>
       <c r="B30" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C30" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D30" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E30" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F30" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="G30" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="H30" s="27" t="n">
-        <v>1.51</v>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="H30" s="29" t="n">
+        <v>3.04</v>
       </c>
       <c r="I30" s="27" t="n">
-        <v>8.01</v>
+        <v>-4.76</v>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="26" t="inlineStr">
         <is>
-          <t>LG디스플레이</t>
+          <t>에코프로</t>
         </is>
       </c>
       <c r="B31" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C31" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D31" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E31" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F31" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="G31" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="H31" s="27" t="n">
-        <v>2.46</v>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="H31" s="29" t="n">
+        <v>10.55</v>
       </c>
       <c r="I31" s="29" t="n">
-        <v>-3.35</v>
+        <v>7.39</v>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="26" t="inlineStr">
         <is>
-          <t>LG에너지솔루션</t>
+          <t>제주반도체</t>
         </is>
       </c>
       <c r="B32" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C32" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D32" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E32" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F32" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="G32" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="H32" s="27" t="n">
-        <v>2.67</v>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="H32" s="29" t="n">
+        <v>2.9</v>
       </c>
       <c r="I32" s="27" t="n">
-        <v>1.77</v>
+        <v>-11.93</v>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="26" t="inlineStr">
         <is>
-          <t>금호건설</t>
+          <t>클라우드</t>
         </is>
       </c>
       <c r="B33" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C33" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D33" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E33" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F33" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="G33" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="H33" s="27" t="n">
-        <v>5.12</v>
-      </c>
-      <c r="I33" s="29" t="n">
-        <v>-25.36</v>
-      </c>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="H33" s="25" t="n"/>
+      <c r="I33" s="25" t="n"/>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="26" t="inlineStr">
@@ -4189,19 +4211,19 @@
       </c>
       <c r="F34" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="G34" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="H34" s="29" t="n">
-        <v>-13.33</v>
-      </c>
-      <c r="I34" s="27" t="n">
-        <v>89.89</v>
+        <v>29.88</v>
+      </c>
+      <c r="I34" s="29" t="n">
+        <v>146.63</v>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
@@ -4224,19 +4246,19 @@
       </c>
       <c r="F35" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="G35" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="H35" s="27" t="n">
-        <v>3.57</v>
-      </c>
-      <c r="I35" s="29" t="n">
-        <v>-7.04</v>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="H35" s="29" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="I35" s="27" t="n">
+        <v>-5.53</v>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
@@ -4259,25 +4281,25 @@
       </c>
       <c r="F36" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="G36" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="H36" s="29" t="n">
-        <v>-0.59</v>
-      </c>
-      <c r="I36" s="27" t="n">
-        <v>7.66</v>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="H36" s="27" t="n">
+        <v>-1.98</v>
+      </c>
+      <c r="I36" s="29" t="n">
+        <v>5.53</v>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="26" t="inlineStr">
         <is>
-          <t>삼성바이오로직스</t>
+          <t>바이오인프라</t>
         </is>
       </c>
       <c r="B37" s="25" t="n">
@@ -4294,25 +4316,25 @@
       </c>
       <c r="F37" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="G37" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="H37" s="27" t="n">
-        <v>4.03</v>
-      </c>
-      <c r="I37" s="27" t="n">
-        <v>7.94</v>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="H37" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="I37" s="29" t="n">
+        <v>119.52</v>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="26" t="inlineStr">
         <is>
-          <t>삼성전기</t>
+          <t>에이엔피</t>
         </is>
       </c>
       <c r="B38" s="25" t="n">
@@ -4329,25 +4351,25 @@
       </c>
       <c r="F38" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="G38" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="H38" s="27" t="n">
-        <v>5.53</v>
+        <v>-29.91</v>
       </c>
       <c r="I38" s="29" t="n">
-        <v>-20.7</v>
+        <v>52.28</v>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="26" t="inlineStr">
         <is>
-          <t>에이엔피</t>
+          <t>지투지바이오</t>
         </is>
       </c>
       <c r="B39" s="25" t="n">
@@ -4364,25 +4386,25 @@
       </c>
       <c r="F39" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="G39" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="H39" s="27" t="n">
-        <v>12.93</v>
-      </c>
-      <c r="I39" s="27" t="n">
-        <v>117.26</v>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="H39" s="29" t="n">
+        <v>24.64</v>
+      </c>
+      <c r="I39" s="29" t="n">
+        <v>5.56</v>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="26" t="inlineStr">
         <is>
-          <t>진에어</t>
+          <t>철강</t>
         </is>
       </c>
       <c r="B40" s="25" t="n">
@@ -4399,25 +4421,21 @@
       </c>
       <c r="F40" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="G40" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="H40" s="29" t="n">
-        <v>-2.45</v>
-      </c>
-      <c r="I40" s="27" t="n">
-        <v>4.93</v>
-      </c>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="H40" s="25" t="n"/>
+      <c r="I40" s="25" t="n"/>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="26" t="inlineStr">
         <is>
-          <t>테라뷰</t>
+          <t>형지글로벌</t>
         </is>
       </c>
       <c r="B41" s="25" t="n">
@@ -4434,130 +4452,130 @@
       </c>
       <c r="F41" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="G41" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="H41" s="27" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="I41" s="29" t="n">
-        <v>-15.33</v>
+        <v>-5.45</v>
+      </c>
+      <c r="I41" s="27" t="n">
+        <v>-28.57</v>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="26" t="inlineStr">
         <is>
-          <t>하이퍼코퍼레이션</t>
+          <t>HMM</t>
         </is>
       </c>
       <c r="B42" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C42" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D42" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E42" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F42" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="G42" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="H42" s="29" t="n">
-        <v>-24.66</v>
-      </c>
-      <c r="I42" s="27" t="n">
-        <v>52.51</v>
+        <v>1.27</v>
+      </c>
+      <c r="I42" s="29" t="n">
+        <v>9.380000000000001</v>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="26" t="inlineStr">
         <is>
-          <t>한국콜마</t>
+          <t>HT로보틱스</t>
         </is>
       </c>
       <c r="B43" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C43" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D43" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E43" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F43" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="G43" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="H43" s="27" t="n">
-        <v>8.06</v>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="H43" s="29" t="n">
+        <v>3.51</v>
       </c>
       <c r="I43" s="29" t="n">
-        <v>-0.84</v>
+        <v>49.59</v>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="26" t="inlineStr">
         <is>
-          <t>형지글로벌</t>
+          <t>TS트릴리온</t>
         </is>
       </c>
       <c r="B44" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C44" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D44" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E44" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F44" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="G44" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="H44" s="29" t="n">
-        <v>-18.32</v>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="H44" s="27" t="n">
+        <v>-7.14</v>
       </c>
       <c r="I44" s="29" t="n">
-        <v>-24.46</v>
+        <v>22.23</v>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="26" t="inlineStr">
         <is>
-          <t>HC보광산업</t>
+          <t>금호전기</t>
         </is>
       </c>
       <c r="B45" s="25" t="n">
@@ -4574,25 +4592,25 @@
       </c>
       <c r="F45" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="G45" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="H45" s="27" t="n">
-        <v>14.17</v>
+        <v>-1.47</v>
       </c>
       <c r="I45" s="27" t="n">
-        <v>13.24</v>
+        <v>-15.18</v>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="26" t="inlineStr">
         <is>
-          <t>HT로보틱스</t>
+          <t>멜콘</t>
         </is>
       </c>
       <c r="B46" s="25" t="n">
@@ -4609,25 +4627,25 @@
       </c>
       <c r="F46" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="G46" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="H46" s="27" t="n">
-        <v>23.5</v>
+        <v>-0.34</v>
       </c>
       <c r="I46" s="27" t="n">
-        <v>44.52</v>
+        <v>-13.79</v>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="26" t="inlineStr">
         <is>
-          <t>TS트릴리온</t>
+          <t>서산</t>
         </is>
       </c>
       <c r="B47" s="25" t="n">
@@ -4644,25 +4662,25 @@
       </c>
       <c r="F47" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="G47" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="H47" s="27" t="n">
-        <v>21.72</v>
-      </c>
-      <c r="I47" s="27" t="n">
-        <v>31.63</v>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="H47" s="29" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="I47" s="29" t="n">
+        <v>20.27</v>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="26" t="inlineStr">
         <is>
-          <t>금호전기</t>
+          <t>에스엠벡셀</t>
         </is>
       </c>
       <c r="B48" s="25" t="n">
@@ -4679,25 +4697,25 @@
       </c>
       <c r="F48" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="G48" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="H48" s="27" t="n">
-        <v>11.46</v>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="H48" s="29" t="n">
+        <v>28.25</v>
       </c>
       <c r="I48" s="29" t="n">
-        <v>-13.91</v>
+        <v>91.02</v>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="26" t="inlineStr">
         <is>
-          <t>듀켐바이오</t>
+          <t>팬오션</t>
         </is>
       </c>
       <c r="B49" s="25" t="n">
@@ -4714,25 +4732,25 @@
       </c>
       <c r="F49" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="G49" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="H49" s="29" t="n">
-        <v>-2.9</v>
-      </c>
-      <c r="I49" s="27" t="n">
-        <v>25.14</v>
+        <v>1.05</v>
+      </c>
+      <c r="I49" s="29" t="n">
+        <v>3.06</v>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="26" t="inlineStr">
         <is>
-          <t>멜콘</t>
+          <t>한선엔지니어링</t>
         </is>
       </c>
       <c r="B50" s="25" t="n">
@@ -4749,25 +4767,25 @@
       </c>
       <c r="F50" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="G50" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="H50" s="29" t="n">
-        <v>-13.49</v>
+        <v>3.07</v>
       </c>
       <c r="I50" s="29" t="n">
-        <v>-13.49</v>
+        <v>31.24</v>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="26" t="inlineStr">
         <is>
-          <t>에스엠벡셀</t>
+          <t>한화갤러리아우</t>
         </is>
       </c>
       <c r="B51" s="25" t="n">
@@ -4784,19 +4802,19 @@
       </c>
       <c r="F51" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="G51" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="H51" s="29" t="n">
-        <v>-0.16</v>
-      </c>
-      <c r="I51" s="27" t="n">
-        <v>48.94</v>
+        <v>10.96</v>
+      </c>
+      <c r="I51" s="29" t="n">
+        <v>35.45</v>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
@@ -4819,19 +4837,19 @@
       </c>
       <c r="F52" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="G52" s="25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="H52" s="27" t="n">
-        <v>10.71</v>
-      </c>
-      <c r="I52" s="27" t="n">
-        <v>22.13</v>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="H52" s="29" t="n">
+        <v>9.67</v>
+      </c>
+      <c r="I52" s="29" t="n">
+        <v>33.94</v>
       </c>
     </row>
   </sheetData>
@@ -4915,19 +4933,19 @@
         <v>1</v>
       </c>
       <c r="C3" s="36" t="n">
-        <v>49</v>
+        <v>68</v>
       </c>
       <c r="D3" s="36" t="n">
-        <v>49</v>
+        <v>68</v>
       </c>
       <c r="E3" s="36" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="F3" s="37" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="G3" s="37" t="inlineStr">
@@ -4946,19 +4964,19 @@
         <v>1</v>
       </c>
       <c r="C4" s="36" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D4" s="36" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E4" s="36" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="F4" s="37" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="G4" s="37" t="inlineStr">
@@ -4970,26 +4988,26 @@
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="35" t="inlineStr">
         <is>
-          <t>전기차</t>
+          <t>AI반도체</t>
         </is>
       </c>
       <c r="B5" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="36" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D5" s="36" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E5" s="36" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="F5" s="37" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="G5" s="37" t="inlineStr">
@@ -5001,26 +5019,26 @@
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="35" t="inlineStr">
         <is>
-          <t>방산</t>
+          <t>전기차</t>
         </is>
       </c>
       <c r="B6" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="36" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D6" s="36" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E6" s="36" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="F6" s="37" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="G6" s="37" t="inlineStr">
@@ -5032,26 +5050,26 @@
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="35" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>방산</t>
         </is>
       </c>
       <c r="B7" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="36" t="n">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="D7" s="36" t="n">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="E7" s="36" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="F7" s="37" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="G7" s="37" t="inlineStr">
@@ -5063,7 +5081,7 @@
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="35" t="inlineStr">
         <is>
-          <t>게임</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="B8" s="36" t="n">
@@ -5077,12 +5095,12 @@
       </c>
       <c r="E8" s="36" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="F8" s="37" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="G8" s="37" t="inlineStr">
@@ -5094,26 +5112,26 @@
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="35" t="inlineStr">
         <is>
-          <t>엔터</t>
+          <t>클라우드</t>
         </is>
       </c>
       <c r="B9" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="36" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D9" s="36" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E9" s="36" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="F9" s="37" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="G9" s="37" t="inlineStr">
@@ -5125,26 +5143,26 @@
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="35" t="inlineStr">
         <is>
-          <t>조선</t>
+          <t>철강</t>
         </is>
       </c>
       <c r="B10" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C10" s="36" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D10" s="36" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="E10" s="36" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="F10" s="37" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="G10" s="37" t="inlineStr">
@@ -5170,12 +5188,12 @@
       </c>
       <c r="E11" s="36" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="F11" s="37" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="G11" s="37" t="inlineStr">
@@ -5194,19 +5212,19 @@
         <v>1</v>
       </c>
       <c r="C12" s="36" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D12" s="36" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="E12" s="36" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="F12" s="37" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="G12" s="37" t="inlineStr">
@@ -5245,7 +5263,7 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>AI반도체</t>
+          <t>원전</t>
         </is>
       </c>
       <c r="B14" s="25" t="n">
@@ -5272,7 +5290,7 @@
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>원전</t>
+          <t>수소</t>
         </is>
       </c>
       <c r="B15" s="25" t="n">
@@ -5299,7 +5317,7 @@
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>수소</t>
+          <t>태양광</t>
         </is>
       </c>
       <c r="B16" s="25" t="n">
@@ -5326,7 +5344,7 @@
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>태양광</t>
+          <t>게임</t>
         </is>
       </c>
       <c r="B17" s="25" t="n">
@@ -5353,7 +5371,7 @@
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="26" t="inlineStr">
         <is>
-          <t>핀테크</t>
+          <t>엔터</t>
         </is>
       </c>
       <c r="B18" s="25" t="n">
@@ -5380,7 +5398,7 @@
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>클라우드</t>
+          <t>핀테크</t>
         </is>
       </c>
       <c r="B19" s="25" t="n">
@@ -5407,7 +5425,7 @@
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="26" t="inlineStr">
         <is>
-          <t>철강</t>
+          <t>조선</t>
         </is>
       </c>
       <c r="B20" s="25" t="n">

</xml_diff>

<commit_message>
auto: 2026-10-25 07:05 자동 백업
</commit_message>
<xml_diff>
--- a/trend/stock_trend_history.xlsx
+++ b/trend/stock_trend_history.xlsx
@@ -694,7 +694,7 @@
     <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-10-24 06:54</t>
+          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-10-25 06:54</t>
         </is>
       </c>
     </row>
@@ -708,7 +708,7 @@
       </c>
       <c r="E3" s="3" t="n"/>
       <c r="G3" s="5" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="H3" s="3" t="n"/>
       <c r="J3" s="6" t="n">
@@ -787,21 +787,21 @@
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-10-24) 상위: 반도체  점수 44.0점</t>
+          <t>⚡ 최신(2026-10-25) 상위: 반도체  점수 65.0점</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-10-24) 상위: SK하이닉스  점수 39.0점</t>
+          <t>⚡ 최신(2026-10-25) 상위: SK하이닉스  점수 50.0점</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-10-24) 상위: 삼성E&amp;A  점수 18.0점</t>
+          <t>⚡ 최신(2026-10-25) 상위: 인공지능  점수 20.0점</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="15" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B14" s="15" t="n">
@@ -928,10 +928,10 @@
         </is>
       </c>
       <c r="D14" s="15" t="n">
-        <v>44</v>
+        <v>65</v>
       </c>
       <c r="E14" s="15" t="n">
-        <v>44</v>
+        <v>65</v>
       </c>
       <c r="F14" s="15" t="n">
         <v>0</v>
@@ -947,7 +947,7 @@
       </c>
       <c r="J14" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
+          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급</t>
         </is>
       </c>
       <c r="K14" s="17" t="inlineStr">
@@ -959,7 +959,7 @@
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="15" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B15" s="15" t="n">
@@ -971,10 +971,10 @@
         </is>
       </c>
       <c r="D15" s="15" t="n">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="E15" s="15" t="n">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="F15" s="15" t="n">
         <v>0</v>
@@ -990,7 +990,7 @@
       </c>
       <c r="J15" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 기사 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>매일경제 기사 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K15" s="17" t="inlineStr">
@@ -1002,7 +1002,7 @@
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="15" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B16" s="15" t="n">
@@ -1010,14 +1010,14 @@
       </c>
       <c r="C16" s="16" t="inlineStr">
         <is>
-          <t>삼성E&amp;A</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="D16" s="15" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="E16" s="15" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="F16" s="15" t="n">
         <v>0</v>
@@ -1025,27 +1025,27 @@
       <c r="G16" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H16" s="18" t="n">
-        <v>5.35</v>
-      </c>
-      <c r="I16" s="18" t="n">
-        <v>35.55</v>
+      <c r="H16" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I16" s="15" t="n">
+        <v/>
       </c>
       <c r="J16" s="17" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +80% / 중요공시 2건 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+          <t>매일경제 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K16" s="17" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B17" s="15" t="n">
@@ -1053,7 +1053,7 @@
       </c>
       <c r="C17" s="16" t="inlineStr">
         <is>
-          <t>인공지능</t>
+          <t>삼성전자</t>
         </is>
       </c>
       <c r="D17" s="15" t="n">
@@ -1068,27 +1068,27 @@
       <c r="G17" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H17" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I17" s="15" t="n">
-        <v/>
+      <c r="H17" s="19" t="n">
+        <v>-0.47</v>
+      </c>
+      <c r="I17" s="19" t="n">
+        <v>-1.61</v>
       </c>
       <c r="J17" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
+          <t>Google 급상승 검색어 등장 (KR) / 매일경제 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K17" s="17" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>네이버, Google</t>
         </is>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B18" s="15" t="n">
@@ -1131,7 +1131,7 @@
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B19" s="15" t="n">
@@ -1139,42 +1139,42 @@
       </c>
       <c r="C19" s="16" t="inlineStr">
         <is>
-          <t>셀트리온</t>
+          <t>조선</t>
         </is>
       </c>
       <c r="D19" s="15" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E19" s="15" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="F19" s="15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G19" s="15" t="n">
-        <v>3</v>
-      </c>
-      <c r="H19" s="19" t="n">
-        <v>-0.47</v>
-      </c>
-      <c r="I19" s="19" t="n">
-        <v>-0.67</v>
+        <v>0</v>
+      </c>
+      <c r="H19" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I19" s="15" t="n">
+        <v/>
       </c>
       <c r="J19" s="17" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 중요공시 3일 +100% / 중요공시 7일 +100% / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K19" s="17" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B20" s="15" t="n">
@@ -1182,14 +1182,14 @@
       </c>
       <c r="C20" s="16" t="inlineStr">
         <is>
-          <t>조선</t>
+          <t>삼성E&amp;A</t>
         </is>
       </c>
       <c r="D20" s="15" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E20" s="15" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F20" s="15" t="n">
         <v>0</v>
@@ -1197,25 +1197,27 @@
       <c r="G20" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H20" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I20" s="15" t="n">
-        <v/>
+      <c r="H20" s="18" t="n">
+        <v>5.35</v>
+      </c>
+      <c r="I20" s="18" t="n">
+        <v>35.55</v>
       </c>
       <c r="J20" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K20" s="17" t="n">
-        <v/>
+          <t>네이버 검색 당일 +200% / 중요공시 2건 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K20" s="17" t="inlineStr">
+        <is>
+          <t>공시, 네이버</t>
+        </is>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="15" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B21" s="15" t="n">
@@ -1223,14 +1225,14 @@
       </c>
       <c r="C21" s="16" t="inlineStr">
         <is>
-          <t>바이오</t>
+          <t>전기차</t>
         </is>
       </c>
       <c r="D21" s="15" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E21" s="15" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="F21" s="15" t="n">
         <v>0</v>
@@ -1246,7 +1248,7 @@
       </c>
       <c r="J21" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K21" s="17" t="inlineStr">
@@ -1258,7 +1260,7 @@
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="15" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B22" s="15" t="n">
@@ -1266,14 +1268,14 @@
       </c>
       <c r="C22" s="16" t="inlineStr">
         <is>
-          <t>삼성전자</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="D22" s="15" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E22" s="15" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F22" s="15" t="n">
         <v>0</v>
@@ -1281,27 +1283,25 @@
       <c r="G22" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H22" s="19" t="n">
-        <v>-0.47</v>
-      </c>
-      <c r="I22" s="19" t="n">
-        <v>-1.61</v>
+      <c r="H22" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I22" s="15" t="n">
+        <v/>
       </c>
       <c r="J22" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K22" s="17" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K22" s="17" t="n">
+        <v/>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="15" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B23" s="15" t="n">
@@ -1309,40 +1309,42 @@
       </c>
       <c r="C23" s="16" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>신한지주</t>
         </is>
       </c>
       <c r="D23" s="15" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E23" s="15" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="F23" s="15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G23" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H23" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I23" s="15" t="n">
-        <v/>
+        <v>3</v>
+      </c>
+      <c r="H23" s="19" t="n">
+        <v>-2.22</v>
+      </c>
+      <c r="I23" s="19" t="n">
+        <v>-6.18</v>
       </c>
       <c r="J23" s="17" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K23" s="17" t="n">
-        <v/>
+          <t>중요공시 3건 / 중요공시 3일 +200% / 중요공시 7일 +200%</t>
+        </is>
+      </c>
+      <c r="K23" s="17" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="15" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B24" s="15" t="n">
@@ -1350,14 +1352,14 @@
       </c>
       <c r="C24" s="16" t="inlineStr">
         <is>
-          <t>폴라리스AI</t>
+          <t>우리금융지주</t>
         </is>
       </c>
       <c r="D24" s="15" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E24" s="15" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="F24" s="15" t="n">
         <v>0</v>
@@ -1365,27 +1367,27 @@
       <c r="G24" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H24" s="18" t="n">
-        <v>4.15</v>
-      </c>
-      <c r="I24" s="18" t="n">
-        <v>25.31</v>
+      <c r="H24" s="19" t="n">
+        <v>-2.88</v>
+      </c>
+      <c r="I24" s="19" t="n">
+        <v>-4.11</v>
       </c>
       <c r="J24" s="17" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +134% / 중요공시 1건 / Google 급상승 검색어 등장 (KR)</t>
+          <t>중요공시 3건 / 매일경제 기사 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K24" s="17" t="inlineStr">
         <is>
-          <t>공시, 네이버, Google</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="15" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B25" s="15" t="n">
@@ -1393,14 +1395,14 @@
       </c>
       <c r="C25" s="16" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>하나금융지주</t>
         </is>
       </c>
       <c r="D25" s="15" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E25" s="15" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="F25" s="15" t="n">
         <v>0</v>
@@ -1408,27 +1410,27 @@
       <c r="G25" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H25" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I25" s="15" t="n">
-        <v/>
+      <c r="H25" s="19" t="n">
+        <v>-2.5</v>
+      </c>
+      <c r="I25" s="19" t="n">
+        <v>-4.65</v>
       </c>
       <c r="J25" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급</t>
+          <t>중요공시 6건 / 매일경제 기사 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K25" s="17" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="15" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B26" s="15" t="n">
@@ -1436,14 +1438,14 @@
       </c>
       <c r="C26" s="16" t="inlineStr">
         <is>
-          <t>SKAI</t>
+          <t>셀트리온</t>
         </is>
       </c>
       <c r="D26" s="15" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E26" s="15" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F26" s="15" t="n">
         <v>0</v>
@@ -1452,26 +1454,26 @@
         <v>0</v>
       </c>
       <c r="H26" s="19" t="n">
-        <v>-8.970000000000001</v>
-      </c>
-      <c r="I26" s="18" t="n">
-        <v>9.27</v>
+        <v>-0.47</v>
+      </c>
+      <c r="I26" s="19" t="n">
+        <v>-0.67</v>
       </c>
       <c r="J26" s="17" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +105% / Google 급상승 검색어 등장 (KR)</t>
+          <t>중요공시 2건 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K26" s="17" t="inlineStr">
         <is>
-          <t>네이버, Google</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="15" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B27" s="15" t="n">
@@ -1479,42 +1481,42 @@
       </c>
       <c r="C27" s="16" t="inlineStr">
         <is>
-          <t>신한지주</t>
+          <t>현대차</t>
         </is>
       </c>
       <c r="D27" s="15" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E27" s="15" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="F27" s="15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G27" s="15" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H27" s="19" t="n">
-        <v>-2.22</v>
+        <v>-2.5</v>
       </c>
       <c r="I27" s="19" t="n">
-        <v>-6.18</v>
+        <v>-6.69</v>
       </c>
       <c r="J27" s="17" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 3일 +200% / 중요공시 7일 +200%</t>
+          <t>네이버뉴스 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K27" s="17" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="15" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B28" s="15" t="n">
@@ -1522,253 +1524,253 @@
       </c>
       <c r="C28" s="16" t="inlineStr">
         <is>
-          <t>빅텍</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="D28" s="15" t="n">
         <v>7</v>
       </c>
       <c r="E28" s="15" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="F28" s="15" t="n">
         <v>0</v>
       </c>
       <c r="G28" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I28" s="15" t="n">
+        <v/>
+      </c>
+      <c r="J28" s="17" t="inlineStr">
+        <is>
+          <t>네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
+        </is>
+      </c>
+      <c r="K28" s="17" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="18" customHeight="1">
+      <c r="A29" s="20" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B29" s="20" t="n">
+        <v>16</v>
+      </c>
+      <c r="C29" s="21" t="inlineStr">
+        <is>
+          <t>카카오게임즈</t>
+        </is>
+      </c>
+      <c r="D29" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="E29" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="F29" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" s="22" t="n">
+        <v>6.51</v>
+      </c>
+      <c r="I29" s="22" t="n">
+        <v>13.27</v>
+      </c>
+      <c r="J29" s="23" t="inlineStr">
+        <is>
+          <t>한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K29" s="23" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="30" ht="18" customHeight="1">
+      <c r="A30" s="20" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B30" s="20" t="n">
+        <v>17</v>
+      </c>
+      <c r="C30" s="21" t="inlineStr">
+        <is>
+          <t>두산에너빌리티</t>
+        </is>
+      </c>
+      <c r="D30" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="E30" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="F30" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" s="24" t="n">
+        <v>-3.92</v>
+      </c>
+      <c r="I30" s="24" t="n">
+        <v>-8.539999999999999</v>
+      </c>
+      <c r="J30" s="23" t="inlineStr">
+        <is>
+          <t>네이버뉴스 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K30" s="23" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="18" customHeight="1">
+      <c r="A31" s="20" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B31" s="20" t="n">
+        <v>18</v>
+      </c>
+      <c r="C31" s="21" t="inlineStr">
+        <is>
+          <t>카카오</t>
+        </is>
+      </c>
+      <c r="D31" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="E31" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="F31" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" s="24" t="n">
+        <v>-1.32</v>
+      </c>
+      <c r="I31" s="24" t="n">
+        <v>-5.99</v>
+      </c>
+      <c r="J31" s="23" t="inlineStr">
+        <is>
+          <t>한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K31" s="23" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="32" ht="18" customHeight="1">
+      <c r="A32" s="20" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B32" s="20" t="n">
+        <v>19</v>
+      </c>
+      <c r="C32" s="21" t="inlineStr">
+        <is>
+          <t>현대로템</t>
+        </is>
+      </c>
+      <c r="D32" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="E32" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="H28" s="19" t="n">
-        <v>-3.32</v>
-      </c>
-      <c r="I28" s="18" t="n">
-        <v>25.78</v>
-      </c>
-      <c r="J28" s="17" t="inlineStr">
-        <is>
-          <t>네이버 검색 당일 +504% / 중요공시 2건 / 중요공시 7일 +100%</t>
-        </is>
-      </c>
-      <c r="K28" s="17" t="inlineStr">
-        <is>
-          <t>공시, 네이버</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="18" customHeight="1">
-      <c r="A29" s="15" t="inlineStr">
-        <is>
-          <t>2026-10-24</t>
-        </is>
-      </c>
-      <c r="B29" s="15" t="n">
-        <v>16</v>
-      </c>
-      <c r="C29" s="16" t="inlineStr">
-        <is>
-          <t>우리금융지주</t>
-        </is>
-      </c>
-      <c r="D29" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="E29" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="F29" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="G29" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H29" s="19" t="n">
-        <v>-2.88</v>
-      </c>
-      <c r="I29" s="19" t="n">
-        <v>-4.11</v>
-      </c>
-      <c r="J29" s="17" t="inlineStr">
-        <is>
-          <t>중요공시 3건 / 매일경제 기사 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K29" s="17" t="inlineStr">
+      <c r="F32" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="H32" s="24" t="n">
+        <v>-3.77</v>
+      </c>
+      <c r="I32" s="24" t="n">
+        <v>-16.31</v>
+      </c>
+      <c r="J32" s="23" t="inlineStr">
+        <is>
+          <t>중요공시 4건 / 중요공시 7일 +300%</t>
+        </is>
+      </c>
+      <c r="K32" s="23" t="inlineStr">
         <is>
           <t>공시</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="18" customHeight="1">
-      <c r="A30" s="15" t="inlineStr">
-        <is>
-          <t>2026-10-24</t>
-        </is>
-      </c>
-      <c r="B30" s="15" t="n">
-        <v>17</v>
-      </c>
-      <c r="C30" s="16" t="inlineStr">
-        <is>
-          <t>대한항공</t>
-        </is>
-      </c>
-      <c r="D30" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="E30" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="F30" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="G30" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H30" s="19" t="n">
-        <v>-2.27</v>
-      </c>
-      <c r="I30" s="19" t="n">
-        <v>-2.45</v>
-      </c>
-      <c r="J30" s="17" t="inlineStr">
-        <is>
-          <t>한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K30" s="17" t="n">
-        <v/>
-      </c>
-    </row>
-    <row r="31" ht="18" customHeight="1">
-      <c r="A31" s="15" t="inlineStr">
-        <is>
-          <t>2026-10-24</t>
-        </is>
-      </c>
-      <c r="B31" s="15" t="n">
-        <v>18</v>
-      </c>
-      <c r="C31" s="16" t="inlineStr">
-        <is>
-          <t>하나금융지주</t>
-        </is>
-      </c>
-      <c r="D31" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="E31" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="F31" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="G31" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H31" s="19" t="n">
-        <v>-2.5</v>
-      </c>
-      <c r="I31" s="19" t="n">
-        <v>-4.65</v>
-      </c>
-      <c r="J31" s="17" t="inlineStr">
-        <is>
-          <t>중요공시 6건 / 매일경제 기사 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K31" s="17" t="inlineStr">
+    <row r="33" ht="18" customHeight="1">
+      <c r="A33" s="20" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B33" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="C33" s="21" t="inlineStr">
+        <is>
+          <t>한솔아이원스</t>
+        </is>
+      </c>
+      <c r="D33" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="E33" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="F33" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H33" s="24" t="n">
+        <v>-2.12</v>
+      </c>
+      <c r="I33" s="24" t="n">
+        <v>-10.61</v>
+      </c>
+      <c r="J33" s="23" t="inlineStr">
+        <is>
+          <t>중요공시 3건 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K33" s="23" t="inlineStr">
         <is>
           <t>공시</t>
         </is>
-      </c>
-    </row>
-    <row r="32" ht="18" customHeight="1">
-      <c r="A32" s="15" t="inlineStr">
-        <is>
-          <t>2026-10-24</t>
-        </is>
-      </c>
-      <c r="B32" s="15" t="n">
-        <v>19</v>
-      </c>
-      <c r="C32" s="16" t="inlineStr">
-        <is>
-          <t>HD현대중공업</t>
-        </is>
-      </c>
-      <c r="D32" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="E32" s="15" t="n">
-        <v>4</v>
-      </c>
-      <c r="F32" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="G32" s="15" t="n">
-        <v>3</v>
-      </c>
-      <c r="H32" s="19" t="n">
-        <v>-0.49</v>
-      </c>
-      <c r="I32" s="19" t="n">
-        <v>-13.51</v>
-      </c>
-      <c r="J32" s="17" t="inlineStr">
-        <is>
-          <t>중요공시 2건 / 중요공시 7일 +100% / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K32" s="17" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="18" customHeight="1">
-      <c r="A33" s="15" t="inlineStr">
-        <is>
-          <t>2026-10-24</t>
-        </is>
-      </c>
-      <c r="B33" s="15" t="n">
-        <v>20</v>
-      </c>
-      <c r="C33" s="16" t="inlineStr">
-        <is>
-          <t>현대차</t>
-        </is>
-      </c>
-      <c r="D33" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="E33" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="F33" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="G33" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H33" s="19" t="n">
-        <v>-2.5</v>
-      </c>
-      <c r="I33" s="19" t="n">
-        <v>-6.69</v>
-      </c>
-      <c r="J33" s="17" t="inlineStr">
-        <is>
-          <t>한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K33" s="17" t="n">
-        <v/>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="20" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B34" s="20" t="n">
@@ -1776,7 +1778,7 @@
       </c>
       <c r="C34" s="21" t="inlineStr">
         <is>
-          <t>카카오게임즈</t>
+          <t>네이버</t>
         </is>
       </c>
       <c r="D34" s="20" t="n">
@@ -1791,15 +1793,15 @@
       <c r="G34" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H34" s="22" t="n">
-        <v>6.51</v>
-      </c>
-      <c r="I34" s="22" t="n">
-        <v>13.27</v>
+      <c r="H34" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I34" s="20" t="n">
+        <v/>
       </c>
       <c r="J34" s="23" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K34" s="23" t="n">
@@ -1809,7 +1811,7 @@
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="20" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B35" s="20" t="n">
@@ -1817,7 +1819,7 @@
       </c>
       <c r="C35" s="21" t="inlineStr">
         <is>
-          <t>카카오</t>
+          <t>게임</t>
         </is>
       </c>
       <c r="D35" s="20" t="n">
@@ -1832,11 +1834,11 @@
       <c r="G35" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H35" s="24" t="n">
-        <v>-1.32</v>
-      </c>
-      <c r="I35" s="24" t="n">
-        <v>-5.99</v>
+      <c r="H35" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I35" s="20" t="n">
+        <v/>
       </c>
       <c r="J35" s="23" t="inlineStr">
         <is>
@@ -1850,7 +1852,7 @@
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="20" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B36" s="20" t="n">
@@ -1858,42 +1860,42 @@
       </c>
       <c r="C36" s="21" t="inlineStr">
         <is>
-          <t>삼성물산</t>
+          <t>원전</t>
         </is>
       </c>
       <c r="D36" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E36" s="20" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F36" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G36" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H36" s="24" t="n">
-        <v>-0.52</v>
-      </c>
-      <c r="I36" s="22" t="n">
-        <v>0.7</v>
+      <c r="H36" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I36" s="20" t="n">
+        <v/>
       </c>
       <c r="J36" s="23" t="inlineStr">
         <is>
-          <t>중요공시 4건 / 중요공시 3일 +100% / 매일경제 기사 언급</t>
+          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K36" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="20" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B37" s="20" t="n">
@@ -1901,14 +1903,14 @@
       </c>
       <c r="C37" s="21" t="inlineStr">
         <is>
-          <t>한솔아이원스</t>
+          <t>삼성전자우</t>
         </is>
       </c>
       <c r="D37" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E37" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F37" s="20" t="n">
         <v>0</v>
@@ -1917,26 +1919,26 @@
         <v>0</v>
       </c>
       <c r="H37" s="24" t="n">
-        <v>-2.12</v>
+        <v>-0.24</v>
       </c>
       <c r="I37" s="24" t="n">
-        <v>-10.61</v>
+        <v>-1.66</v>
       </c>
       <c r="J37" s="23" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 매일경제 헤드라인 언급</t>
+          <t>Google 급상승 검색어 등장 (KR)</t>
         </is>
       </c>
       <c r="K37" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>Google</t>
         </is>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="20" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B38" s="20" t="n">
@@ -1944,42 +1946,42 @@
       </c>
       <c r="C38" s="21" t="inlineStr">
         <is>
-          <t>에이전트AI</t>
+          <t>비나텍</t>
         </is>
       </c>
       <c r="D38" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E38" s="20" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F38" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G38" s="20" t="n">
         <v>0</v>
       </c>
       <c r="H38" s="22" t="n">
-        <v>29.91</v>
+        <v>8.1</v>
       </c>
       <c r="I38" s="22" t="n">
-        <v>61.16</v>
+        <v>47.06</v>
       </c>
       <c r="J38" s="23" t="inlineStr">
         <is>
-          <t>중요공시 1건 / Google 급상승 검색어 등장 (KR)</t>
+          <t>중요공시 6건 / 중요공시 3일 +100%</t>
         </is>
       </c>
       <c r="K38" s="23" t="inlineStr">
         <is>
-          <t>공시, Google</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="20" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B39" s="20" t="n">
@@ -1987,14 +1989,14 @@
       </c>
       <c r="C39" s="21" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>Apple</t>
         </is>
       </c>
       <c r="D39" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E39" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F39" s="20" t="n">
         <v>0</v>
@@ -2010,17 +2012,19 @@
       </c>
       <c r="J39" s="23" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K39" s="23" t="n">
-        <v/>
+          <t>Google 급상승 검색어 등장 (US)</t>
+        </is>
+      </c>
+      <c r="K39" s="23" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="20" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B40" s="20" t="n">
@@ -2028,14 +2032,14 @@
       </c>
       <c r="C40" s="21" t="inlineStr">
         <is>
-          <t>KT&amp;G</t>
+          <t>빅텍</t>
         </is>
       </c>
       <c r="D40" s="20" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E40" s="20" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F40" s="20" t="n">
         <v>0</v>
@@ -2044,24 +2048,26 @@
         <v>0</v>
       </c>
       <c r="H40" s="24" t="n">
-        <v>-2.17</v>
-      </c>
-      <c r="I40" s="24" t="n">
-        <v>-1.04</v>
+        <v>-3.32</v>
+      </c>
+      <c r="I40" s="22" t="n">
+        <v>25.78</v>
       </c>
       <c r="J40" s="23" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K40" s="23" t="n">
-        <v/>
+          <t>네이버 검색 당일 +805% / 중요공시 2건</t>
+        </is>
+      </c>
+      <c r="K40" s="23" t="inlineStr">
+        <is>
+          <t>공시, 네이버</t>
+        </is>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="20" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B41" s="20" t="n">
@@ -2069,14 +2075,14 @@
       </c>
       <c r="C41" s="21" t="inlineStr">
         <is>
-          <t>KT</t>
+          <t>지투지바이오</t>
         </is>
       </c>
       <c r="D41" s="20" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E41" s="20" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F41" s="20" t="n">
         <v>0</v>
@@ -2084,25 +2090,27 @@
       <c r="G41" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H41" s="24" t="n">
-        <v>-1.68</v>
-      </c>
-      <c r="I41" s="24" t="n">
-        <v>-7.34</v>
+      <c r="H41" s="22" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="I41" s="22" t="n">
+        <v>58.72</v>
       </c>
       <c r="J41" s="23" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K41" s="23" t="n">
-        <v/>
+          <t>네이버 검색 당일 +263% / 중요공시 1건</t>
+        </is>
+      </c>
+      <c r="K41" s="23" t="inlineStr">
+        <is>
+          <t>공시, 네이버</t>
+        </is>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="20" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B42" s="20" t="n">
@@ -2110,14 +2118,14 @@
       </c>
       <c r="C42" s="21" t="inlineStr">
         <is>
-          <t>게임</t>
+          <t>폴라리스AI</t>
         </is>
       </c>
       <c r="D42" s="20" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E42" s="20" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F42" s="20" t="n">
         <v>0</v>
@@ -2125,25 +2133,27 @@
       <c r="G42" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H42" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I42" s="20" t="n">
-        <v/>
+      <c r="H42" s="22" t="n">
+        <v>4.15</v>
+      </c>
+      <c r="I42" s="22" t="n">
+        <v>25.31</v>
       </c>
       <c r="J42" s="23" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K42" s="23" t="n">
-        <v/>
+          <t>네이버 검색 당일 +258% / 중요공시 1건</t>
+        </is>
+      </c>
+      <c r="K42" s="23" t="inlineStr">
+        <is>
+          <t>공시, 네이버</t>
+        </is>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="20" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B43" s="20" t="n">
@@ -2151,14 +2161,14 @@
       </c>
       <c r="C43" s="21" t="inlineStr">
         <is>
-          <t>전기차</t>
+          <t>혜인</t>
         </is>
       </c>
       <c r="D43" s="20" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E43" s="20" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F43" s="20" t="n">
         <v>0</v>
@@ -2166,25 +2176,27 @@
       <c r="G43" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H43" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I43" s="20" t="n">
-        <v/>
+      <c r="H43" s="24" t="n">
+        <v>-9.17</v>
+      </c>
+      <c r="I43" s="22" t="n">
+        <v>33.65</v>
       </c>
       <c r="J43" s="23" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K43" s="23" t="n">
-        <v/>
+          <t>네이버 검색 당일 +209% / 중요공시 1건</t>
+        </is>
+      </c>
+      <c r="K43" s="23" t="inlineStr">
+        <is>
+          <t>공시, 네이버</t>
+        </is>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="20" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B44" s="20" t="n">
@@ -2192,42 +2204,40 @@
       </c>
       <c r="C44" s="21" t="inlineStr">
         <is>
-          <t>금호건설</t>
+          <t>디티에스</t>
         </is>
       </c>
       <c r="D44" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E44" s="20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F44" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G44" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H44" s="24" t="n">
-        <v>-3.58</v>
-      </c>
-      <c r="I44" s="24" t="n">
-        <v>-8.08</v>
+      <c r="H44" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I44" s="20" t="n">
+        <v/>
       </c>
       <c r="J44" s="23" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 3일 +50%</t>
-        </is>
-      </c>
-      <c r="K44" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K44" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="20" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B45" s="20" t="n">
@@ -2235,14 +2245,14 @@
       </c>
       <c r="C45" s="21" t="inlineStr">
         <is>
-          <t>AI반도체</t>
+          <t>LG디스플레이</t>
         </is>
       </c>
       <c r="D45" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E45" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F45" s="20" t="n">
         <v>0</v>
@@ -2250,27 +2260,27 @@
       <c r="G45" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H45" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I45" s="20" t="n">
-        <v/>
+      <c r="H45" s="24" t="n">
+        <v>-1.66</v>
+      </c>
+      <c r="I45" s="24" t="n">
+        <v>-5.33</v>
       </c>
       <c r="J45" s="23" t="inlineStr">
         <is>
-          <t>Google 급상승 검색어 등장 (KR)</t>
+          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K45" s="23" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="20" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B46" s="20" t="n">
@@ -2278,14 +2288,14 @@
       </c>
       <c r="C46" s="21" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>삼성물산</t>
         </is>
       </c>
       <c r="D46" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E46" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F46" s="20" t="n">
         <v>0</v>
@@ -2293,27 +2303,27 @@
       <c r="G46" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H46" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I46" s="20" t="n">
-        <v/>
+      <c r="H46" s="24" t="n">
+        <v>-0.52</v>
+      </c>
+      <c r="I46" s="22" t="n">
+        <v>0.7</v>
       </c>
       <c r="J46" s="23" t="inlineStr">
         <is>
-          <t>Google 급상승 검색어 등장 (KR)</t>
+          <t>중요공시 4건 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K46" s="23" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="20" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B47" s="20" t="n">
@@ -2321,42 +2331,42 @@
       </c>
       <c r="C47" s="21" t="inlineStr">
         <is>
-          <t>AI chip</t>
+          <t>현대건설</t>
         </is>
       </c>
       <c r="D47" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E47" s="20" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F47" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G47" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H47" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I47" s="20" t="n">
-        <v/>
+        <v>3</v>
+      </c>
+      <c r="H47" s="24" t="n">
+        <v>-2.15</v>
+      </c>
+      <c r="I47" s="24" t="n">
+        <v>-2.47</v>
       </c>
       <c r="J47" s="23" t="inlineStr">
         <is>
-          <t>Google 급상승 검색어 등장 (KR)</t>
+          <t>중요공시 2건 / 중요공시 7일 +100%</t>
         </is>
       </c>
       <c r="K47" s="23" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="20" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B48" s="20" t="n">
@@ -2364,42 +2374,42 @@
       </c>
       <c r="C48" s="21" t="inlineStr">
         <is>
-          <t>지투지바이오</t>
+          <t>HD현대중공업</t>
         </is>
       </c>
       <c r="D48" s="20" t="n">
         <v>4</v>
       </c>
       <c r="E48" s="20" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F48" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G48" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H48" s="22" t="n">
-        <v>18.8</v>
-      </c>
-      <c r="I48" s="22" t="n">
-        <v>58.72</v>
+        <v>3</v>
+      </c>
+      <c r="H48" s="24" t="n">
+        <v>-0.49</v>
+      </c>
+      <c r="I48" s="24" t="n">
+        <v>-13.51</v>
       </c>
       <c r="J48" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +163% / 중요공시 1건</t>
+          <t>중요공시 2건 / 중요공시 7일 +100%</t>
         </is>
       </c>
       <c r="K48" s="23" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="20" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B49" s="20" t="n">
@@ -2407,7 +2417,7 @@
       </c>
       <c r="C49" s="21" t="inlineStr">
         <is>
-          <t>혜인</t>
+          <t>국전</t>
         </is>
       </c>
       <c r="D49" s="20" t="n">
@@ -2423,26 +2433,26 @@
         <v>0</v>
       </c>
       <c r="H49" s="24" t="n">
-        <v>-9.17</v>
-      </c>
-      <c r="I49" s="22" t="n">
-        <v>33.65</v>
+        <v>-4.97</v>
+      </c>
+      <c r="I49" s="24" t="n">
+        <v>-12.4</v>
       </c>
       <c r="J49" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +159% / 중요공시 1건</t>
+          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K49" s="23" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="20" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B50" s="20" t="n">
@@ -2450,7 +2460,7 @@
       </c>
       <c r="C50" s="21" t="inlineStr">
         <is>
-          <t>LG디스플레이</t>
+          <t>노을</t>
         </is>
       </c>
       <c r="D50" s="20" t="n">
@@ -2465,11 +2475,11 @@
       <c r="G50" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H50" s="24" t="n">
-        <v>-1.66</v>
-      </c>
-      <c r="I50" s="24" t="n">
-        <v>-5.33</v>
+      <c r="H50" s="22" t="n">
+        <v>29.96</v>
+      </c>
+      <c r="I50" s="22" t="n">
+        <v>16.7</v>
       </c>
       <c r="J50" s="23" t="inlineStr">
         <is>
@@ -2485,7 +2495,7 @@
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="20" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B51" s="20" t="n">
@@ -2493,7 +2503,7 @@
       </c>
       <c r="C51" s="21" t="inlineStr">
         <is>
-          <t>국전</t>
+          <t>KT</t>
         </is>
       </c>
       <c r="D51" s="20" t="n">
@@ -2509,26 +2519,26 @@
         <v>0</v>
       </c>
       <c r="H51" s="24" t="n">
-        <v>-4.97</v>
+        <v>-1.68</v>
       </c>
       <c r="I51" s="24" t="n">
-        <v>-12.4</v>
+        <v>-7.34</v>
       </c>
       <c r="J51" s="23" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
+          <t>한국경제 헤드라인 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K51" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="20" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B52" s="20" t="n">
@@ -2536,7 +2546,7 @@
       </c>
       <c r="C52" s="21" t="inlineStr">
         <is>
-          <t>노을</t>
+          <t>클라우드</t>
         </is>
       </c>
       <c r="D52" s="20" t="n">
@@ -2551,27 +2561,27 @@
       <c r="G52" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H52" s="22" t="n">
-        <v>29.96</v>
-      </c>
-      <c r="I52" s="22" t="n">
-        <v>16.7</v>
+      <c r="H52" s="20" t="n">
+        <v/>
+      </c>
+      <c r="I52" s="20" t="n">
+        <v/>
       </c>
       <c r="J52" s="23" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
+          <t>네이버뉴스 기사 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K52" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="53" ht="18" customHeight="1">
       <c r="A53" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B53" s="25" t="n">
@@ -2602,7 +2612,7 @@
       </c>
       <c r="J53" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +6376%</t>
+          <t>네이버 검색 당일 +7205%</t>
         </is>
       </c>
       <c r="K53" s="29" t="inlineStr">
@@ -2614,7 +2624,7 @@
     <row r="54" ht="18" customHeight="1">
       <c r="A54" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B54" s="25" t="n">
@@ -2645,7 +2655,7 @@
       </c>
       <c r="J54" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +1265%</t>
+          <t>네이버 검색 당일 +1451%</t>
         </is>
       </c>
       <c r="K54" s="29" t="inlineStr">
@@ -2657,7 +2667,7 @@
     <row r="55" ht="18" customHeight="1">
       <c r="A55" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B55" s="25" t="n">
@@ -2688,7 +2698,7 @@
       </c>
       <c r="J55" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +784%</t>
+          <t>네이버 검색 당일 +869%</t>
         </is>
       </c>
       <c r="K55" s="29" t="inlineStr">
@@ -2700,7 +2710,7 @@
     <row r="56" ht="18" customHeight="1">
       <c r="A56" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B56" s="25" t="n">
@@ -2708,7 +2718,7 @@
       </c>
       <c r="C56" s="26" t="inlineStr">
         <is>
-          <t>앤로보틱스</t>
+          <t>스페코</t>
         </is>
       </c>
       <c r="D56" s="25" t="n">
@@ -2724,14 +2734,14 @@
         <v>0</v>
       </c>
       <c r="H56" s="28" t="n">
-        <v>20.12</v>
+        <v>27.09</v>
       </c>
       <c r="I56" s="28" t="n">
-        <v>49.58</v>
+        <v>41.72</v>
       </c>
       <c r="J56" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +281%</t>
+          <t>네이버 검색 당일 +668%</t>
         </is>
       </c>
       <c r="K56" s="29" t="inlineStr">
@@ -2743,7 +2753,7 @@
     <row r="57" ht="18" customHeight="1">
       <c r="A57" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B57" s="25" t="n">
@@ -2751,7 +2761,7 @@
       </c>
       <c r="C57" s="26" t="inlineStr">
         <is>
-          <t>휴니드</t>
+          <t>진양홀딩스</t>
         </is>
       </c>
       <c r="D57" s="25" t="n">
@@ -2766,15 +2776,15 @@
       <c r="G57" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H57" s="27" t="n">
-        <v>-0.92</v>
+      <c r="H57" s="28" t="n">
+        <v>4.12</v>
       </c>
       <c r="I57" s="28" t="n">
-        <v>16.53</v>
+        <v>4.29</v>
       </c>
       <c r="J57" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +246%</t>
+          <t>네이버 검색 당일 +546%</t>
         </is>
       </c>
       <c r="K57" s="29" t="inlineStr">
@@ -2786,7 +2796,7 @@
     <row r="58" ht="18" customHeight="1">
       <c r="A58" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B58" s="25" t="n">
@@ -2794,7 +2804,7 @@
       </c>
       <c r="C58" s="26" t="inlineStr">
         <is>
-          <t>형지엘리트</t>
+          <t>앤로보틱스</t>
         </is>
       </c>
       <c r="D58" s="25" t="n">
@@ -2809,15 +2819,15 @@
       <c r="G58" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H58" s="27" t="n">
-        <v>-14.87</v>
+      <c r="H58" s="28" t="n">
+        <v>20.12</v>
       </c>
       <c r="I58" s="28" t="n">
-        <v>19.93</v>
+        <v>49.58</v>
       </c>
       <c r="J58" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +237%</t>
+          <t>네이버 검색 당일 +455%</t>
         </is>
       </c>
       <c r="K58" s="29" t="inlineStr">
@@ -2829,7 +2839,7 @@
     <row r="59" ht="18" customHeight="1">
       <c r="A59" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B59" s="25" t="n">
@@ -2837,7 +2847,7 @@
       </c>
       <c r="C59" s="26" t="inlineStr">
         <is>
-          <t>스페코</t>
+          <t>진양산업</t>
         </is>
       </c>
       <c r="D59" s="25" t="n">
@@ -2853,14 +2863,14 @@
         <v>0</v>
       </c>
       <c r="H59" s="28" t="n">
-        <v>27.09</v>
+        <v>27.82</v>
       </c>
       <c r="I59" s="28" t="n">
-        <v>41.72</v>
+        <v>29.02</v>
       </c>
       <c r="J59" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +211%</t>
+          <t>네이버 검색 당일 +370%</t>
         </is>
       </c>
       <c r="K59" s="29" t="inlineStr">
@@ -2872,7 +2882,7 @@
     <row r="60" ht="18" customHeight="1">
       <c r="A60" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B60" s="25" t="n">
@@ -2880,7 +2890,7 @@
       </c>
       <c r="C60" s="26" t="inlineStr">
         <is>
-          <t>유니테크노</t>
+          <t>휴니드</t>
         </is>
       </c>
       <c r="D60" s="25" t="n">
@@ -2895,15 +2905,15 @@
       <c r="G60" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H60" s="28" t="n">
-        <v>10.56</v>
+      <c r="H60" s="27" t="n">
+        <v>-0.92</v>
       </c>
       <c r="I60" s="28" t="n">
-        <v>11.67</v>
+        <v>16.53</v>
       </c>
       <c r="J60" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +210%</t>
+          <t>네이버 검색 당일 +346%</t>
         </is>
       </c>
       <c r="K60" s="29" t="inlineStr">
@@ -2915,7 +2925,7 @@
     <row r="61" ht="18" customHeight="1">
       <c r="A61" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B61" s="25" t="n">
@@ -2946,7 +2956,7 @@
       </c>
       <c r="J61" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +155%</t>
+          <t>네이버 검색 당일 +328%</t>
         </is>
       </c>
       <c r="K61" s="29" t="inlineStr">
@@ -2958,7 +2968,7 @@
     <row r="62" ht="18" customHeight="1">
       <c r="A62" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B62" s="25" t="n">
@@ -2966,7 +2976,7 @@
       </c>
       <c r="C62" s="26" t="inlineStr">
         <is>
-          <t>자이언트스텝</t>
+          <t>진양화학</t>
         </is>
       </c>
       <c r="D62" s="25" t="n">
@@ -2982,14 +2992,14 @@
         <v>0</v>
       </c>
       <c r="H62" s="28" t="n">
-        <v>0.74</v>
+        <v>31.11</v>
       </c>
       <c r="I62" s="28" t="n">
-        <v>47.31</v>
+        <v>35.87</v>
       </c>
       <c r="J62" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +107%</t>
+          <t>네이버 검색 당일 +310%</t>
         </is>
       </c>
       <c r="K62" s="29" t="inlineStr">
@@ -3001,7 +3011,7 @@
     <row r="63" ht="18" customHeight="1">
       <c r="A63" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B63" s="25" t="n">
@@ -3009,7 +3019,7 @@
       </c>
       <c r="C63" s="26" t="inlineStr">
         <is>
-          <t>두산에너빌리티</t>
+          <t>형지엘리트</t>
         </is>
       </c>
       <c r="D63" s="25" t="n">
@@ -3025,18 +3035,20 @@
         <v>0</v>
       </c>
       <c r="H63" s="27" t="n">
-        <v>-3.92</v>
-      </c>
-      <c r="I63" s="27" t="n">
-        <v>-8.539999999999999</v>
+        <v>-14.87</v>
+      </c>
+      <c r="I63" s="28" t="n">
+        <v>19.93</v>
       </c>
       <c r="J63" s="29" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K63" s="29" t="n">
-        <v/>
+          <t>네이버 검색 당일 +308%</t>
+        </is>
+      </c>
+      <c r="K63" s="29" t="inlineStr">
+        <is>
+          <t>네이버</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -3132,22 +3144,22 @@
         <v>1</v>
       </c>
       <c r="C3" s="25" t="n">
-        <v>44</v>
+        <v>65</v>
       </c>
       <c r="D3" s="25" t="n">
-        <v>44</v>
+        <v>65</v>
       </c>
       <c r="E3" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F3" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="G3" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="H3" s="25" t="n"/>
@@ -3163,22 +3175,22 @@
         <v>1</v>
       </c>
       <c r="C4" s="25" t="n">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="D4" s="25" t="n">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="E4" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F4" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="G4" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="H4" s="28" t="n">
@@ -3191,42 +3203,38 @@
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="26" t="inlineStr">
         <is>
-          <t>삼성E&amp;A</t>
+          <t>인공지능</t>
         </is>
       </c>
       <c r="B5" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="25" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D5" s="25" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="E5" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F5" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="G5" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
-        </is>
-      </c>
-      <c r="H5" s="28" t="n">
-        <v>5.35</v>
-      </c>
-      <c r="I5" s="28" t="n">
-        <v>35.55</v>
-      </c>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="H5" s="25" t="n"/>
+      <c r="I5" s="25" t="n"/>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="26" t="inlineStr">
         <is>
-          <t>인공지능</t>
+          <t>삼성전자</t>
         </is>
       </c>
       <c r="B6" s="25" t="n">
@@ -3243,16 +3251,20 @@
       </c>
       <c r="F6" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="G6" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
-        </is>
-      </c>
-      <c r="H6" s="25" t="n"/>
-      <c r="I6" s="25" t="n"/>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="H6" s="27" t="n">
+        <v>-0.47</v>
+      </c>
+      <c r="I6" s="27" t="n">
+        <v>-1.61</v>
+      </c>
     </row>
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="26" t="inlineStr">
@@ -3274,12 +3286,12 @@
       </c>
       <c r="F7" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="G7" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="H7" s="27" t="n">
@@ -3292,95 +3304,95 @@
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="26" t="inlineStr">
         <is>
-          <t>셀트리온</t>
+          <t>조선</t>
         </is>
       </c>
       <c r="B8" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="25" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D8" s="25" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E8" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F8" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="G8" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
-        </is>
-      </c>
-      <c r="H8" s="27" t="n">
-        <v>-0.47</v>
-      </c>
-      <c r="I8" s="27" t="n">
-        <v>-0.67</v>
-      </c>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="H8" s="25" t="n"/>
+      <c r="I8" s="25" t="n"/>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="26" t="inlineStr">
         <is>
-          <t>조선</t>
+          <t>삼성E&amp;A</t>
         </is>
       </c>
       <c r="B9" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="25" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D9" s="25" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E9" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F9" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="G9" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
-        </is>
-      </c>
-      <c r="H9" s="25" t="n"/>
-      <c r="I9" s="25" t="n"/>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="H9" s="28" t="n">
+        <v>5.35</v>
+      </c>
+      <c r="I9" s="28" t="n">
+        <v>35.55</v>
+      </c>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="26" t="inlineStr">
         <is>
-          <t>바이오</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="B10" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C10" s="25" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="D10" s="25" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E10" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F10" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="G10" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="H10" s="25" t="n"/>
@@ -3389,29 +3401,29 @@
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="26" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>전기차</t>
         </is>
       </c>
       <c r="B11" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="25" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D11" s="25" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E11" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F11" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="G11" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="H11" s="25" t="n"/>
@@ -3420,178 +3432,178 @@
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="26" t="inlineStr">
         <is>
-          <t>삼성전자</t>
+          <t>신한지주</t>
         </is>
       </c>
       <c r="B12" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C12" s="25" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D12" s="25" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E12" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F12" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="G12" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="H12" s="27" t="n">
-        <v>-0.47</v>
+        <v>-2.22</v>
       </c>
       <c r="I12" s="27" t="n">
-        <v>-1.61</v>
+        <v>-6.18</v>
       </c>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>셀트리온</t>
         </is>
       </c>
       <c r="B13" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C13" s="25" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D13" s="25" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E13" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F13" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="G13" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
-        </is>
-      </c>
-      <c r="H13" s="25" t="n"/>
-      <c r="I13" s="25" t="n"/>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="H13" s="27" t="n">
+        <v>-0.47</v>
+      </c>
+      <c r="I13" s="27" t="n">
+        <v>-0.67</v>
+      </c>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>폴라리스AI</t>
+          <t>우리금융지주</t>
         </is>
       </c>
       <c r="B14" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C14" s="25" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D14" s="25" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E14" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F14" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="G14" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
-        </is>
-      </c>
-      <c r="H14" s="28" t="n">
-        <v>4.15</v>
-      </c>
-      <c r="I14" s="28" t="n">
-        <v>25.31</v>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="H14" s="27" t="n">
+        <v>-2.88</v>
+      </c>
+      <c r="I14" s="27" t="n">
+        <v>-4.11</v>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>SKAI</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="B15" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C15" s="25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D15" s="25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E15" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F15" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="G15" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
-        </is>
-      </c>
-      <c r="H15" s="27" t="n">
-        <v>-8.970000000000001</v>
-      </c>
-      <c r="I15" s="28" t="n">
-        <v>9.27</v>
-      </c>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="H15" s="25" t="n"/>
+      <c r="I15" s="25" t="n"/>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>신한지주</t>
+          <t>하나금융지주</t>
         </is>
       </c>
       <c r="B16" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C16" s="25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D16" s="25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E16" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F16" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="G16" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="H16" s="27" t="n">
-        <v>-2.22</v>
+        <v>-2.5</v>
       </c>
       <c r="I16" s="27" t="n">
-        <v>-6.18</v>
+        <v>-4.65</v>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>HD현대중공업</t>
+          <t>현대차</t>
         </is>
       </c>
       <c r="B17" s="25" t="n">
@@ -3608,200 +3620,188 @@
       </c>
       <c r="F17" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="G17" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="H17" s="27" t="n">
-        <v>-0.49</v>
+        <v>-2.5</v>
       </c>
       <c r="I17" s="27" t="n">
-        <v>-13.51</v>
+        <v>-6.69</v>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="26" t="inlineStr">
         <is>
-          <t>대한항공</t>
+          <t>게임</t>
         </is>
       </c>
       <c r="B18" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C18" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D18" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E18" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F18" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="G18" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
-        </is>
-      </c>
-      <c r="H18" s="27" t="n">
-        <v>-2.27</v>
-      </c>
-      <c r="I18" s="27" t="n">
-        <v>-2.45</v>
-      </c>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="H18" s="25" t="n"/>
+      <c r="I18" s="25" t="n"/>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>빅텍</t>
+          <t>네이버</t>
         </is>
       </c>
       <c r="B19" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C19" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D19" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E19" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F19" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="G19" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
-        </is>
-      </c>
-      <c r="H19" s="27" t="n">
-        <v>-3.32</v>
-      </c>
-      <c r="I19" s="28" t="n">
-        <v>25.78</v>
-      </c>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="H19" s="25" t="n"/>
+      <c r="I19" s="25" t="n"/>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="26" t="inlineStr">
         <is>
-          <t>우리금융지주</t>
+          <t>두산에너빌리티</t>
         </is>
       </c>
       <c r="B20" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C20" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D20" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E20" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F20" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="G20" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="H20" s="27" t="n">
-        <v>-2.88</v>
+        <v>-3.92</v>
       </c>
       <c r="I20" s="27" t="n">
-        <v>-4.11</v>
+        <v>-8.539999999999999</v>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="26" t="inlineStr">
         <is>
-          <t>하나금융지주</t>
+          <t>원전</t>
         </is>
       </c>
       <c r="B21" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C21" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D21" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E21" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F21" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="G21" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
-        </is>
-      </c>
-      <c r="H21" s="27" t="n">
-        <v>-2.5</v>
-      </c>
-      <c r="I21" s="27" t="n">
-        <v>-4.65</v>
-      </c>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="H21" s="25" t="n"/>
+      <c r="I21" s="25" t="n"/>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="26" t="inlineStr">
         <is>
-          <t>현대차</t>
+          <t>카카오</t>
         </is>
       </c>
       <c r="B22" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C22" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D22" s="25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E22" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F22" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="G22" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="H22" s="27" t="n">
-        <v>-2.5</v>
+        <v>-1.32</v>
       </c>
       <c r="I22" s="27" t="n">
-        <v>-6.69</v>
+        <v>-5.99</v>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="26" t="inlineStr">
         <is>
-          <t>KT</t>
+          <t>카카오게임즈</t>
         </is>
       </c>
       <c r="B23" s="25" t="n">
@@ -3818,25 +3818,25 @@
       </c>
       <c r="F23" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="G23" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
-        </is>
-      </c>
-      <c r="H23" s="27" t="n">
-        <v>-1.68</v>
-      </c>
-      <c r="I23" s="27" t="n">
-        <v>-7.34</v>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="H23" s="28" t="n">
+        <v>6.51</v>
+      </c>
+      <c r="I23" s="28" t="n">
+        <v>13.27</v>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="26" t="inlineStr">
         <is>
-          <t>KT&amp;G</t>
+          <t>한솔아이원스</t>
         </is>
       </c>
       <c r="B24" s="25" t="n">
@@ -3853,25 +3853,25 @@
       </c>
       <c r="F24" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="G24" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="H24" s="27" t="n">
-        <v>-2.17</v>
+        <v>-2.12</v>
       </c>
       <c r="I24" s="27" t="n">
-        <v>-1.04</v>
+        <v>-10.61</v>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="26" t="inlineStr">
         <is>
-          <t>게임</t>
+          <t>현대로템</t>
         </is>
       </c>
       <c r="B25" s="25" t="n">
@@ -3888,43 +3888,47 @@
       </c>
       <c r="F25" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="G25" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
-        </is>
-      </c>
-      <c r="H25" s="25" t="n"/>
-      <c r="I25" s="25" t="n"/>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="H25" s="27" t="n">
+        <v>-3.77</v>
+      </c>
+      <c r="I25" s="27" t="n">
+        <v>-16.31</v>
+      </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="26" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>Apple</t>
         </is>
       </c>
       <c r="B26" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C26" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D26" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E26" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F26" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="G26" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="H26" s="25" t="n"/>
@@ -3933,266 +3937,274 @@
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="26" t="inlineStr">
         <is>
-          <t>삼성물산</t>
+          <t>비나텍</t>
         </is>
       </c>
       <c r="B27" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C27" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D27" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E27" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F27" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="G27" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
-        </is>
-      </c>
-      <c r="H27" s="27" t="n">
-        <v>-0.52</v>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="H27" s="28" t="n">
+        <v>8.1</v>
       </c>
       <c r="I27" s="28" t="n">
-        <v>0.7</v>
+        <v>47.06</v>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="26" t="inlineStr">
         <is>
-          <t>에이전트AI</t>
+          <t>삼성전자우</t>
         </is>
       </c>
       <c r="B28" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C28" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D28" s="25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E28" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F28" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="G28" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
-        </is>
-      </c>
-      <c r="H28" s="28" t="n">
-        <v>29.91</v>
-      </c>
-      <c r="I28" s="28" t="n">
-        <v>61.16</v>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="H28" s="27" t="n">
+        <v>-0.24</v>
+      </c>
+      <c r="I28" s="27" t="n">
+        <v>-1.66</v>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="26" t="inlineStr">
         <is>
-          <t>전기차</t>
+          <t>HD현대중공업</t>
         </is>
       </c>
       <c r="B29" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C29" s="25" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D29" s="25" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E29" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F29" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="G29" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
-        </is>
-      </c>
-      <c r="H29" s="25" t="n"/>
-      <c r="I29" s="25" t="n"/>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="H29" s="27" t="n">
+        <v>-0.49</v>
+      </c>
+      <c r="I29" s="27" t="n">
+        <v>-13.51</v>
+      </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="26" t="inlineStr">
         <is>
-          <t>카카오</t>
+          <t>KT</t>
         </is>
       </c>
       <c r="B30" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C30" s="25" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D30" s="25" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E30" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F30" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="G30" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="H30" s="27" t="n">
-        <v>-1.32</v>
+        <v>-1.68</v>
       </c>
       <c r="I30" s="27" t="n">
-        <v>-5.99</v>
+        <v>-7.34</v>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="26" t="inlineStr">
         <is>
-          <t>카카오게임즈</t>
+          <t>LG디스플레이</t>
         </is>
       </c>
       <c r="B31" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C31" s="25" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D31" s="25" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E31" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F31" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="G31" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
-        </is>
-      </c>
-      <c r="H31" s="28" t="n">
-        <v>6.51</v>
-      </c>
-      <c r="I31" s="28" t="n">
-        <v>13.27</v>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="H31" s="27" t="n">
+        <v>-1.66</v>
+      </c>
+      <c r="I31" s="27" t="n">
+        <v>-5.33</v>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="26" t="inlineStr">
         <is>
-          <t>한솔아이원스</t>
+          <t>국전</t>
         </is>
       </c>
       <c r="B32" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C32" s="25" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D32" s="25" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E32" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F32" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="G32" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="H32" s="27" t="n">
-        <v>-2.12</v>
+        <v>-4.97</v>
       </c>
       <c r="I32" s="27" t="n">
-        <v>-10.61</v>
+        <v>-12.4</v>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="26" t="inlineStr">
         <is>
-          <t>AI chip</t>
+          <t>노을</t>
         </is>
       </c>
       <c r="B33" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C33" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D33" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E33" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F33" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="G33" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
-        </is>
-      </c>
-      <c r="H33" s="25" t="n"/>
-      <c r="I33" s="25" t="n"/>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="H33" s="28" t="n">
+        <v>29.96</v>
+      </c>
+      <c r="I33" s="28" t="n">
+        <v>16.7</v>
+      </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="26" t="inlineStr">
         <is>
-          <t>AI반도체</t>
+          <t>디티에스</t>
         </is>
       </c>
       <c r="B34" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C34" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D34" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E34" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F34" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="G34" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="H34" s="25" t="n"/>
@@ -4201,73 +4213,77 @@
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="26" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>빅텍</t>
         </is>
       </c>
       <c r="B35" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C35" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D35" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E35" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F35" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="G35" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
-        </is>
-      </c>
-      <c r="H35" s="25" t="n"/>
-      <c r="I35" s="25" t="n"/>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="H35" s="27" t="n">
+        <v>-3.32</v>
+      </c>
+      <c r="I35" s="28" t="n">
+        <v>25.78</v>
+      </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="26" t="inlineStr">
         <is>
-          <t>금호건설</t>
+          <t>삼성물산</t>
         </is>
       </c>
       <c r="B36" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C36" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D36" s="25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E36" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F36" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="G36" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="H36" s="27" t="n">
-        <v>-3.58</v>
-      </c>
-      <c r="I36" s="27" t="n">
-        <v>-8.08</v>
+        <v>-0.52</v>
+      </c>
+      <c r="I36" s="28" t="n">
+        <v>0.7</v>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="26" t="inlineStr">
         <is>
-          <t>LG디스플레이</t>
+          <t>지투지바이오</t>
         </is>
       </c>
       <c r="B37" s="25" t="n">
@@ -4284,25 +4300,25 @@
       </c>
       <c r="F37" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="G37" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
-        </is>
-      </c>
-      <c r="H37" s="27" t="n">
-        <v>-1.66</v>
-      </c>
-      <c r="I37" s="27" t="n">
-        <v>-5.33</v>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="H37" s="28" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="I37" s="28" t="n">
+        <v>58.72</v>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="26" t="inlineStr">
         <is>
-          <t>국전</t>
+          <t>클라우드</t>
         </is>
       </c>
       <c r="B38" s="25" t="n">
@@ -4319,25 +4335,21 @@
       </c>
       <c r="F38" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="G38" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
-        </is>
-      </c>
-      <c r="H38" s="27" t="n">
-        <v>-4.97</v>
-      </c>
-      <c r="I38" s="27" t="n">
-        <v>-12.4</v>
-      </c>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="H38" s="25" t="n"/>
+      <c r="I38" s="25" t="n"/>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="26" t="inlineStr">
         <is>
-          <t>노을</t>
+          <t>폴라리스AI</t>
         </is>
       </c>
       <c r="B39" s="25" t="n">
@@ -4354,25 +4366,25 @@
       </c>
       <c r="F39" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="G39" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="H39" s="28" t="n">
-        <v>29.96</v>
+        <v>4.15</v>
       </c>
       <c r="I39" s="28" t="n">
-        <v>16.7</v>
+        <v>25.31</v>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="26" t="inlineStr">
         <is>
-          <t>지투지바이오</t>
+          <t>현대건설</t>
         </is>
       </c>
       <c r="B40" s="25" t="n">
@@ -4389,19 +4401,19 @@
       </c>
       <c r="F40" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="G40" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
-        </is>
-      </c>
-      <c r="H40" s="28" t="n">
-        <v>18.8</v>
-      </c>
-      <c r="I40" s="28" t="n">
-        <v>58.72</v>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="H40" s="27" t="n">
+        <v>-2.15</v>
+      </c>
+      <c r="I40" s="27" t="n">
+        <v>-2.47</v>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
@@ -4424,12 +4436,12 @@
       </c>
       <c r="F41" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="G41" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="H41" s="27" t="n">
@@ -4459,12 +4471,12 @@
       </c>
       <c r="F42" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="G42" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="H42" s="27" t="n">
@@ -4477,7 +4489,7 @@
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="26" t="inlineStr">
         <is>
-          <t>두산에너빌리티</t>
+          <t>스페코</t>
         </is>
       </c>
       <c r="B43" s="25" t="n">
@@ -4494,25 +4506,25 @@
       </c>
       <c r="F43" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="G43" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
-        </is>
-      </c>
-      <c r="H43" s="27" t="n">
-        <v>-3.92</v>
-      </c>
-      <c r="I43" s="27" t="n">
-        <v>-8.539999999999999</v>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="H43" s="28" t="n">
+        <v>27.09</v>
+      </c>
+      <c r="I43" s="28" t="n">
+        <v>41.72</v>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="26" t="inlineStr">
         <is>
-          <t>스페코</t>
+          <t>앤로보틱스</t>
         </is>
       </c>
       <c r="B44" s="25" t="n">
@@ -4529,25 +4541,25 @@
       </c>
       <c r="F44" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="G44" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="H44" s="28" t="n">
-        <v>27.09</v>
+        <v>20.12</v>
       </c>
       <c r="I44" s="28" t="n">
-        <v>41.72</v>
+        <v>49.58</v>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="26" t="inlineStr">
         <is>
-          <t>앤로보틱스</t>
+          <t>엘리스</t>
         </is>
       </c>
       <c r="B45" s="25" t="n">
@@ -4564,25 +4576,25 @@
       </c>
       <c r="F45" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="G45" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
-        </is>
-      </c>
-      <c r="H45" s="28" t="n">
-        <v>20.12</v>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="H45" s="27" t="n">
+        <v>-3.5</v>
       </c>
       <c r="I45" s="28" t="n">
-        <v>49.58</v>
+        <v>47.73</v>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="26" t="inlineStr">
         <is>
-          <t>엘리스</t>
+          <t>진양산업</t>
         </is>
       </c>
       <c r="B46" s="25" t="n">
@@ -4599,25 +4611,25 @@
       </c>
       <c r="F46" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="G46" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
-        </is>
-      </c>
-      <c r="H46" s="27" t="n">
-        <v>-3.5</v>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="H46" s="28" t="n">
+        <v>27.82</v>
       </c>
       <c r="I46" s="28" t="n">
-        <v>47.73</v>
+        <v>29.02</v>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="26" t="inlineStr">
         <is>
-          <t>유니테크노</t>
+          <t>진양홀딩스</t>
         </is>
       </c>
       <c r="B47" s="25" t="n">
@@ -4634,25 +4646,25 @@
       </c>
       <c r="F47" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="G47" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="H47" s="28" t="n">
-        <v>10.56</v>
+        <v>4.12</v>
       </c>
       <c r="I47" s="28" t="n">
-        <v>11.67</v>
+        <v>4.29</v>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="26" t="inlineStr">
         <is>
-          <t>자이언트스텝</t>
+          <t>진양화학</t>
         </is>
       </c>
       <c r="B48" s="25" t="n">
@@ -4669,19 +4681,19 @@
       </c>
       <c r="F48" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="G48" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="H48" s="28" t="n">
-        <v>0.74</v>
+        <v>31.11</v>
       </c>
       <c r="I48" s="28" t="n">
-        <v>47.31</v>
+        <v>35.87</v>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
@@ -4704,12 +4716,12 @@
       </c>
       <c r="F49" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="G49" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="H49" s="27" t="n">
@@ -4739,12 +4751,12 @@
       </c>
       <c r="F50" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="G50" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="H50" s="27" t="n">
@@ -4774,12 +4786,12 @@
       </c>
       <c r="F51" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="G51" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="H51" s="27" t="n">
@@ -4809,12 +4821,12 @@
       </c>
       <c r="F52" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="G52" s="25" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="H52" s="27" t="n">
@@ -4905,19 +4917,19 @@
         <v>1</v>
       </c>
       <c r="C3" s="36" t="n">
-        <v>44</v>
+        <v>65</v>
       </c>
       <c r="D3" s="36" t="n">
-        <v>44</v>
+        <v>65</v>
       </c>
       <c r="E3" s="36" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F3" s="37" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="G3" s="37" t="inlineStr">
@@ -4929,26 +4941,26 @@
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="35" t="inlineStr">
         <is>
-          <t>바이오</t>
+          <t>전기차</t>
         </is>
       </c>
       <c r="B4" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C4" s="36" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="D4" s="36" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E4" s="36" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F4" s="37" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="G4" s="37" t="inlineStr">
@@ -4960,26 +4972,26 @@
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="35" t="inlineStr">
         <is>
-          <t>AI반도체</t>
+          <t>원전</t>
         </is>
       </c>
       <c r="B5" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="36" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D5" s="36" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E5" s="36" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F5" s="37" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="G5" s="37" t="inlineStr">
@@ -4991,26 +5003,26 @@
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="35" t="inlineStr">
         <is>
-          <t>전기차</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="B6" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="36" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D6" s="36" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E6" s="36" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F6" s="37" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="G6" s="37" t="inlineStr">
@@ -5022,26 +5034,26 @@
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="35" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>게임</t>
         </is>
       </c>
       <c r="B7" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="36" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D7" s="36" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E7" s="36" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F7" s="37" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="G7" s="37" t="inlineStr">
@@ -5053,26 +5065,26 @@
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="35" t="inlineStr">
         <is>
-          <t>게임</t>
+          <t>클라우드</t>
         </is>
       </c>
       <c r="B8" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="36" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D8" s="36" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E8" s="36" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F8" s="37" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="G8" s="37" t="inlineStr">
@@ -5091,19 +5103,19 @@
         <v>1</v>
       </c>
       <c r="C9" s="36" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D9" s="36" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E9" s="36" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F9" s="37" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="G9" s="37" t="inlineStr">
@@ -5122,19 +5134,19 @@
         <v>1</v>
       </c>
       <c r="C10" s="36" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D10" s="36" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E10" s="36" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F10" s="37" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="G10" s="37" t="inlineStr">
@@ -5153,19 +5165,19 @@
         <v>1</v>
       </c>
       <c r="C11" s="36" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D11" s="36" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E11" s="36" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F11" s="37" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="G11" s="37" t="inlineStr">
@@ -5204,7 +5216,7 @@
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>방산</t>
+          <t>바이오</t>
         </is>
       </c>
       <c r="B13" s="25" t="n">
@@ -5231,7 +5243,7 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>원전</t>
+          <t>AI반도체</t>
         </is>
       </c>
       <c r="B14" s="25" t="n">
@@ -5258,7 +5270,7 @@
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>수소</t>
+          <t>방산</t>
         </is>
       </c>
       <c r="B15" s="25" t="n">
@@ -5285,7 +5297,7 @@
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>태양광</t>
+          <t>수소</t>
         </is>
       </c>
       <c r="B16" s="25" t="n">
@@ -5312,7 +5324,7 @@
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>엔터</t>
+          <t>태양광</t>
         </is>
       </c>
       <c r="B17" s="25" t="n">
@@ -5339,7 +5351,7 @@
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="26" t="inlineStr">
         <is>
-          <t>핀테크</t>
+          <t>엔터</t>
         </is>
       </c>
       <c r="B18" s="25" t="n">
@@ -5366,7 +5378,7 @@
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>클라우드</t>
+          <t>핀테크</t>
         </is>
       </c>
       <c r="B19" s="25" t="n">

</xml_diff>

<commit_message>
auto: 2026-10-26 07:12 자동 백업
</commit_message>
<xml_diff>
--- a/trend/stock_trend_history.xlsx
+++ b/trend/stock_trend_history.xlsx
@@ -258,13 +258,13 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -694,7 +694,7 @@
     <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-10-25 06:54</t>
+          <t>📊 주식 트렌드 조기 감지 대시보드   |   최종 업데이트: 2026-10-26 06:54</t>
         </is>
       </c>
     </row>
@@ -787,21 +787,21 @@
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-10-25) 상위: 반도체  점수 65.0점</t>
+          <t>⚡ 최신(2026-10-26) 상위: 반도체  점수 67.0점</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-10-25) 상위: SK하이닉스  점수 50.0점</t>
+          <t>⚡ 최신(2026-10-26) 상위: SK하이닉스  점수 23.0점</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>⚡ 최신(2026-10-25) 상위: 인공지능  점수 20.0점</t>
+          <t>⚡ 최신(2026-10-26) 상위: 인공지능  점수 19.0점</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="15" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B14" s="15" t="n">
@@ -928,10 +928,10 @@
         </is>
       </c>
       <c r="D14" s="15" t="n">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="E14" s="15" t="n">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="F14" s="15" t="n">
         <v>0</v>
@@ -947,7 +947,7 @@
       </c>
       <c r="J14" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급</t>
+          <t>매일경제 기사 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K14" s="17" t="inlineStr">
@@ -959,7 +959,7 @@
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="15" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B15" s="15" t="n">
@@ -971,10 +971,10 @@
         </is>
       </c>
       <c r="D15" s="15" t="n">
-        <v>50</v>
+        <v>23</v>
       </c>
       <c r="E15" s="15" t="n">
-        <v>50</v>
+        <v>23</v>
       </c>
       <c r="F15" s="15" t="n">
         <v>0</v>
@@ -990,7 +990,7 @@
       </c>
       <c r="J15" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급</t>
+          <t>매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K15" s="17" t="inlineStr">
@@ -1002,7 +1002,7 @@
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="15" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B16" s="15" t="n">
@@ -1014,10 +1014,10 @@
         </is>
       </c>
       <c r="D16" s="15" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E16" s="15" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F16" s="15" t="n">
         <v>0</v>
@@ -1033,7 +1033,7 @@
       </c>
       <c r="J16" s="17" t="inlineStr">
         <is>
-          <t>매일경제 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급</t>
+          <t>매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K16" s="17" t="inlineStr">
@@ -1045,7 +1045,7 @@
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B17" s="15" t="n">
@@ -1057,10 +1057,10 @@
         </is>
       </c>
       <c r="D17" s="15" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E17" s="15" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F17" s="15" t="n">
         <v>0</v>
@@ -1076,19 +1076,19 @@
       </c>
       <c r="J17" s="17" t="inlineStr">
         <is>
-          <t>Google 급상승 검색어 등장 (KR) / 매일경제 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
+          <t>매일경제 기사 언급 / 매일경제 기사 언급 / 매일경제 기사 언급 / 네이버뉴스 기사 언급 / 매일경제 기사 언급</t>
         </is>
       </c>
       <c r="K17" s="17" t="inlineStr">
         <is>
-          <t>네이버, Google</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B18" s="15" t="n">
@@ -1096,14 +1096,14 @@
       </c>
       <c r="C18" s="16" t="inlineStr">
         <is>
-          <t>삼성전기</t>
+          <t>전기차</t>
         </is>
       </c>
       <c r="D18" s="15" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E18" s="15" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F18" s="15" t="n">
         <v>0</v>
@@ -1111,27 +1111,27 @@
       <c r="G18" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H18" s="19" t="n">
-        <v>-3.05</v>
-      </c>
-      <c r="I18" s="19" t="n">
-        <v>-6.17</v>
+      <c r="H18" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I18" s="15" t="n">
+        <v/>
       </c>
       <c r="J18" s="17" t="inlineStr">
         <is>
-          <t>중요공시 1건 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 기사 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K18" s="17" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B19" s="15" t="n">
@@ -1139,14 +1139,14 @@
       </c>
       <c r="C19" s="16" t="inlineStr">
         <is>
-          <t>조선</t>
+          <t>삼성E&amp;A</t>
         </is>
       </c>
       <c r="D19" s="15" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E19" s="15" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F19" s="15" t="n">
         <v>0</v>
@@ -1154,27 +1154,27 @@
       <c r="G19" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H19" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I19" s="15" t="n">
-        <v/>
+      <c r="H19" s="18" t="n">
+        <v>5.35</v>
+      </c>
+      <c r="I19" s="18" t="n">
+        <v>35.55</v>
       </c>
       <c r="J19" s="17" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>네이버 검색 당일 +220% / 중요공시 2건 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K19" s="17" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B20" s="15" t="n">
@@ -1182,14 +1182,14 @@
       </c>
       <c r="C20" s="16" t="inlineStr">
         <is>
-          <t>삼성E&amp;A</t>
+          <t>바이오</t>
         </is>
       </c>
       <c r="D20" s="15" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="E20" s="15" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F20" s="15" t="n">
         <v>0</v>
@@ -1197,27 +1197,27 @@
       <c r="G20" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H20" s="18" t="n">
-        <v>5.35</v>
-      </c>
-      <c r="I20" s="18" t="n">
-        <v>35.55</v>
+      <c r="H20" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I20" s="15" t="n">
+        <v/>
       </c>
       <c r="J20" s="17" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +200% / 중요공시 2건 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+          <t>한국경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K20" s="17" t="inlineStr">
         <is>
-          <t>공시, 네이버</t>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="15" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B21" s="15" t="n">
@@ -1225,7 +1225,7 @@
       </c>
       <c r="C21" s="16" t="inlineStr">
         <is>
-          <t>전기차</t>
+          <t>한솔아이원스</t>
         </is>
       </c>
       <c r="D21" s="15" t="n">
@@ -1240,27 +1240,27 @@
       <c r="G21" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H21" s="15" t="n">
-        <v/>
-      </c>
-      <c r="I21" s="15" t="n">
-        <v/>
+      <c r="H21" s="19" t="n">
+        <v>-2.12</v>
+      </c>
+      <c r="I21" s="19" t="n">
+        <v>-10.61</v>
       </c>
       <c r="J21" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>중요공시 3건 / 매일경제 헤드라인 언급 / 네이버뉴스 헤드라인 언급</t>
         </is>
       </c>
       <c r="K21" s="17" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="15" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B22" s="15" t="n">
@@ -1268,14 +1268,14 @@
       </c>
       <c r="C22" s="16" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>게임</t>
         </is>
       </c>
       <c r="D22" s="15" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E22" s="15" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F22" s="15" t="n">
         <v>0</v>
@@ -1291,7 +1291,7 @@
       </c>
       <c r="J22" s="17" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급 / 매일경제 기사 언급 / 한국경제 헤드라인 언급</t>
+          <t>한국경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K22" s="17" t="n">
@@ -1301,7 +1301,7 @@
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="15" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B23" s="15" t="n">
@@ -1309,42 +1309,40 @@
       </c>
       <c r="C23" s="16" t="inlineStr">
         <is>
-          <t>신한지주</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="D23" s="15" t="n">
         <v>8</v>
       </c>
       <c r="E23" s="15" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="F23" s="15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G23" s="15" t="n">
-        <v>3</v>
-      </c>
-      <c r="H23" s="19" t="n">
-        <v>-2.22</v>
-      </c>
-      <c r="I23" s="19" t="n">
-        <v>-6.18</v>
+        <v>0</v>
+      </c>
+      <c r="H23" s="15" t="n">
+        <v/>
+      </c>
+      <c r="I23" s="15" t="n">
+        <v/>
       </c>
       <c r="J23" s="17" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 중요공시 3일 +200% / 중요공시 7일 +200%</t>
-        </is>
-      </c>
-      <c r="K23" s="17" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>매일경제 헤드라인 언급 / 매일경제 기사 언급 / 한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K23" s="17" t="n">
+        <v/>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="15" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B24" s="15" t="n">
@@ -1352,42 +1350,42 @@
       </c>
       <c r="C24" s="16" t="inlineStr">
         <is>
-          <t>우리금융지주</t>
+          <t>빅텍</t>
         </is>
       </c>
       <c r="D24" s="15" t="n">
         <v>7</v>
       </c>
       <c r="E24" s="15" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="F24" s="15" t="n">
         <v>0</v>
       </c>
       <c r="G24" s="15" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H24" s="19" t="n">
-        <v>-2.88</v>
-      </c>
-      <c r="I24" s="19" t="n">
-        <v>-4.11</v>
+        <v>-3.32</v>
+      </c>
+      <c r="I24" s="18" t="n">
+        <v>25.78</v>
       </c>
       <c r="J24" s="17" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 매일경제 기사 언급 / 매일경제 헤드라인 언급</t>
+          <t>네이버 검색 당일 +903% / 중요공시 2건 / 중요공시 7일 +100%</t>
         </is>
       </c>
       <c r="K24" s="17" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>공시, 네이버</t>
         </is>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="15" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B25" s="15" t="n">
@@ -1395,7 +1393,7 @@
       </c>
       <c r="C25" s="16" t="inlineStr">
         <is>
-          <t>하나금융지주</t>
+          <t>우리금융지주</t>
         </is>
       </c>
       <c r="D25" s="15" t="n">
@@ -1411,14 +1409,14 @@
         <v>0</v>
       </c>
       <c r="H25" s="19" t="n">
-        <v>-2.5</v>
+        <v>-2.88</v>
       </c>
       <c r="I25" s="19" t="n">
-        <v>-4.65</v>
+        <v>-4.11</v>
       </c>
       <c r="J25" s="17" t="inlineStr">
         <is>
-          <t>중요공시 6건 / 매일경제 기사 언급 / 매일경제 헤드라인 언급</t>
+          <t>중요공시 3건 / 매일경제 기사 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K25" s="17" t="inlineStr">
@@ -1430,7 +1428,7 @@
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="15" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B26" s="15" t="n">
@@ -1438,7 +1436,7 @@
       </c>
       <c r="C26" s="16" t="inlineStr">
         <is>
-          <t>셀트리온</t>
+          <t>하나금융지주</t>
         </is>
       </c>
       <c r="D26" s="15" t="n">
@@ -1454,14 +1452,14 @@
         <v>0</v>
       </c>
       <c r="H26" s="19" t="n">
-        <v>-0.47</v>
+        <v>-2.5</v>
       </c>
       <c r="I26" s="19" t="n">
-        <v>-0.67</v>
+        <v>-4.65</v>
       </c>
       <c r="J26" s="17" t="inlineStr">
         <is>
-          <t>중요공시 2건 / 한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+          <t>중요공시 6건 / 매일경제 기사 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K26" s="17" t="inlineStr">
@@ -1473,7 +1471,7 @@
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="15" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B27" s="15" t="n">
@@ -1504,19 +1502,17 @@
       </c>
       <c r="J27" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K27" s="17" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K27" s="17" t="n">
+        <v/>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="15" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B28" s="15" t="n">
@@ -1547,7 +1543,7 @@
       </c>
       <c r="J28" s="17" t="inlineStr">
         <is>
-          <t>네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 헤드라인 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
+          <t>네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K28" s="17" t="inlineStr">
@@ -1559,7 +1555,7 @@
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="20" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B29" s="20" t="n">
@@ -1567,40 +1563,42 @@
       </c>
       <c r="C29" s="21" t="inlineStr">
         <is>
-          <t>카카오게임즈</t>
+          <t>현대로템</t>
         </is>
       </c>
       <c r="D29" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E29" s="20" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F29" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G29" s="20" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H29" s="22" t="n">
-        <v>6.51</v>
+        <v>-3.77</v>
       </c>
       <c r="I29" s="22" t="n">
-        <v>13.27</v>
+        <v>-16.31</v>
       </c>
       <c r="J29" s="23" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K29" s="23" t="n">
-        <v/>
+          <t>중요공시 4건 / 중요공시 7일 +300%</t>
+        </is>
+      </c>
+      <c r="K29" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="20" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B30" s="20" t="n">
@@ -1608,42 +1606,42 @@
       </c>
       <c r="C30" s="21" t="inlineStr">
         <is>
-          <t>두산에너빌리티</t>
+          <t>신한지주</t>
         </is>
       </c>
       <c r="D30" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E30" s="20" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F30" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G30" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H30" s="24" t="n">
-        <v>-3.92</v>
-      </c>
-      <c r="I30" s="24" t="n">
-        <v>-8.539999999999999</v>
+        <v>3</v>
+      </c>
+      <c r="H30" s="22" t="n">
+        <v>-2.22</v>
+      </c>
+      <c r="I30" s="22" t="n">
+        <v>-6.18</v>
       </c>
       <c r="J30" s="23" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 매일경제 기사 언급 / 매일경제 헤드라인 언급</t>
+          <t>중요공시 3건 / 중요공시 7일 +200%</t>
         </is>
       </c>
       <c r="K30" s="23" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>공시</t>
         </is>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="20" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B31" s="20" t="n">
@@ -1651,40 +1649,42 @@
       </c>
       <c r="C31" s="21" t="inlineStr">
         <is>
-          <t>카카오</t>
+          <t>금호건설</t>
         </is>
       </c>
       <c r="D31" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E31" s="20" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F31" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G31" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H31" s="24" t="n">
-        <v>-1.32</v>
-      </c>
-      <c r="I31" s="24" t="n">
-        <v>-5.99</v>
+        <v>3</v>
+      </c>
+      <c r="H31" s="22" t="n">
+        <v>-3.58</v>
+      </c>
+      <c r="I31" s="22" t="n">
+        <v>-8.08</v>
       </c>
       <c r="J31" s="23" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K31" s="23" t="n">
-        <v/>
+          <t>중요공시 3건 / 중요공시 7일 +200%</t>
+        </is>
+      </c>
+      <c r="K31" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="20" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B32" s="20" t="n">
@@ -1692,30 +1692,30 @@
       </c>
       <c r="C32" s="21" t="inlineStr">
         <is>
-          <t>현대로템</t>
+          <t>현대건설</t>
         </is>
       </c>
       <c r="D32" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E32" s="20" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F32" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G32" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="H32" s="24" t="n">
-        <v>-3.77</v>
-      </c>
-      <c r="I32" s="24" t="n">
-        <v>-16.31</v>
+      <c r="H32" s="22" t="n">
+        <v>-2.15</v>
+      </c>
+      <c r="I32" s="22" t="n">
+        <v>-2.47</v>
       </c>
       <c r="J32" s="23" t="inlineStr">
         <is>
-          <t>중요공시 4건 / 중요공시 7일 +300%</t>
+          <t>중요공시 2건 / 중요공시 3일 +100% / 중요공시 7일 +100%</t>
         </is>
       </c>
       <c r="K32" s="23" t="inlineStr">
@@ -1727,7 +1727,7 @@
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="20" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B33" s="20" t="n">
@@ -1735,7 +1735,7 @@
       </c>
       <c r="C33" s="21" t="inlineStr">
         <is>
-          <t>한솔아이원스</t>
+          <t>HD현대중공업</t>
         </is>
       </c>
       <c r="D33" s="20" t="n">
@@ -1750,27 +1750,27 @@
       <c r="G33" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H33" s="24" t="n">
-        <v>-2.12</v>
-      </c>
-      <c r="I33" s="24" t="n">
-        <v>-10.61</v>
+      <c r="H33" s="22" t="n">
+        <v>-0.49</v>
+      </c>
+      <c r="I33" s="22" t="n">
+        <v>-13.51</v>
       </c>
       <c r="J33" s="23" t="inlineStr">
         <is>
-          <t>중요공시 3건 / 매일경제 헤드라인 언급</t>
+          <t>중요공시 2건 / Google 급상승 검색어 등장 (KR)</t>
         </is>
       </c>
       <c r="K33" s="23" t="inlineStr">
         <is>
-          <t>공시</t>
+          <t>Google, 공시</t>
         </is>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="20" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B34" s="20" t="n">
@@ -1778,40 +1778,42 @@
       </c>
       <c r="C34" s="21" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>예스티</t>
         </is>
       </c>
       <c r="D34" s="20" t="n">
         <v>6</v>
       </c>
       <c r="E34" s="20" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F34" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G34" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H34" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I34" s="20" t="n">
-        <v/>
+      <c r="H34" s="22" t="n">
+        <v>-6.68</v>
+      </c>
+      <c r="I34" s="24" t="n">
+        <v>5.08</v>
       </c>
       <c r="J34" s="23" t="inlineStr">
         <is>
-          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K34" s="23" t="n">
-        <v/>
+          <t>중요공시 2건 / 중요공시 3일 +100% / 한국경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K34" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="20" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B35" s="20" t="n">
@@ -1819,7 +1821,7 @@
       </c>
       <c r="C35" s="21" t="inlineStr">
         <is>
-          <t>게임</t>
+          <t>GS</t>
         </is>
       </c>
       <c r="D35" s="20" t="n">
@@ -1834,15 +1836,15 @@
       <c r="G35" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H35" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I35" s="20" t="n">
-        <v/>
+      <c r="H35" s="22" t="n">
+        <v>-3.42</v>
+      </c>
+      <c r="I35" s="22" t="n">
+        <v>-8.43</v>
       </c>
       <c r="J35" s="23" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급 / 한국경제 헤드라인 언급</t>
+          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K35" s="23" t="n">
@@ -1852,7 +1854,7 @@
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="20" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B36" s="20" t="n">
@@ -1860,7 +1862,7 @@
       </c>
       <c r="C36" s="21" t="inlineStr">
         <is>
-          <t>원전</t>
+          <t>네이버</t>
         </is>
       </c>
       <c r="D36" s="20" t="n">
@@ -1883,19 +1885,17 @@
       </c>
       <c r="J36" s="23" t="inlineStr">
         <is>
-          <t>네이버뉴스 헤드라인 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K36" s="23" t="inlineStr">
-        <is>
-          <t>네이버</t>
-        </is>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K36" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="20" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B37" s="20" t="n">
@@ -1903,14 +1903,14 @@
       </c>
       <c r="C37" s="21" t="inlineStr">
         <is>
-          <t>삼성전자우</t>
+          <t>기아</t>
         </is>
       </c>
       <c r="D37" s="20" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E37" s="20" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F37" s="20" t="n">
         <v>0</v>
@@ -1918,27 +1918,25 @@
       <c r="G37" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H37" s="24" t="n">
-        <v>-0.24</v>
-      </c>
-      <c r="I37" s="24" t="n">
-        <v>-1.66</v>
+      <c r="H37" s="22" t="n">
+        <v>-1.57</v>
+      </c>
+      <c r="I37" s="22" t="n">
+        <v>-3.79</v>
       </c>
       <c r="J37" s="23" t="inlineStr">
         <is>
-          <t>Google 급상승 검색어 등장 (KR)</t>
-        </is>
-      </c>
-      <c r="K37" s="23" t="inlineStr">
-        <is>
-          <t>Google</t>
-        </is>
+          <t>한국경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K37" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="20" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B38" s="20" t="n">
@@ -1946,42 +1944,40 @@
       </c>
       <c r="C38" s="21" t="inlineStr">
         <is>
-          <t>비나텍</t>
+          <t>LG전자</t>
         </is>
       </c>
       <c r="D38" s="20" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E38" s="20" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F38" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G38" s="20" t="n">
         <v>0</v>
       </c>
       <c r="H38" s="22" t="n">
-        <v>8.1</v>
+        <v>-1.77</v>
       </c>
       <c r="I38" s="22" t="n">
-        <v>47.06</v>
+        <v>-8.789999999999999</v>
       </c>
       <c r="J38" s="23" t="inlineStr">
         <is>
-          <t>중요공시 6건 / 중요공시 3일 +100%</t>
-        </is>
-      </c>
-      <c r="K38" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
-        </is>
+          <t>매일경제 헤드라인 언급 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K38" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="20" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B39" s="20" t="n">
@@ -1989,14 +1985,14 @@
       </c>
       <c r="C39" s="21" t="inlineStr">
         <is>
-          <t>Apple</t>
+          <t>조선</t>
         </is>
       </c>
       <c r="D39" s="20" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E39" s="20" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F39" s="20" t="n">
         <v>0</v>
@@ -2012,19 +2008,17 @@
       </c>
       <c r="J39" s="23" t="inlineStr">
         <is>
-          <t>Google 급상승 검색어 등장 (US)</t>
-        </is>
-      </c>
-      <c r="K39" s="23" t="inlineStr">
-        <is>
-          <t>Google</t>
-        </is>
+          <t>매일경제 헤드라인 언급 / 한국경제 헤드라인 언급 / 매일경제 기사 언급</t>
+        </is>
+      </c>
+      <c r="K39" s="23" t="n">
+        <v/>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="20" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B40" s="20" t="n">
@@ -2032,14 +2026,14 @@
       </c>
       <c r="C40" s="21" t="inlineStr">
         <is>
-          <t>빅텍</t>
+          <t>혜인</t>
         </is>
       </c>
       <c r="D40" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E40" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F40" s="20" t="n">
         <v>0</v>
@@ -2047,15 +2041,15 @@
       <c r="G40" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H40" s="24" t="n">
-        <v>-3.32</v>
-      </c>
-      <c r="I40" s="22" t="n">
-        <v>25.78</v>
+      <c r="H40" s="22" t="n">
+        <v>-9.17</v>
+      </c>
+      <c r="I40" s="24" t="n">
+        <v>33.65</v>
       </c>
       <c r="J40" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +805% / 중요공시 2건</t>
+          <t>네이버 검색 당일 +224% / 중요공시 1건 / 네이버뉴스 기사 언급</t>
         </is>
       </c>
       <c r="K40" s="23" t="inlineStr">
@@ -2067,7 +2061,7 @@
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="20" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B41" s="20" t="n">
@@ -2090,15 +2084,15 @@
       <c r="G41" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H41" s="22" t="n">
+      <c r="H41" s="24" t="n">
         <v>18.8</v>
       </c>
-      <c r="I41" s="22" t="n">
+      <c r="I41" s="24" t="n">
         <v>58.72</v>
       </c>
       <c r="J41" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +263% / 중요공시 1건</t>
+          <t>네이버 검색 당일 +280% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K41" s="23" t="inlineStr">
@@ -2110,7 +2104,7 @@
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="20" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B42" s="20" t="n">
@@ -2133,15 +2127,15 @@
       <c r="G42" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H42" s="22" t="n">
+      <c r="H42" s="24" t="n">
         <v>4.15</v>
       </c>
-      <c r="I42" s="22" t="n">
+      <c r="I42" s="24" t="n">
         <v>25.31</v>
       </c>
       <c r="J42" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +258% / 중요공시 1건</t>
+          <t>네이버 검색 당일 +271% / 중요공시 1건</t>
         </is>
       </c>
       <c r="K42" s="23" t="inlineStr">
@@ -2153,7 +2147,7 @@
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="20" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B43" s="20" t="n">
@@ -2161,7 +2155,7 @@
       </c>
       <c r="C43" s="21" t="inlineStr">
         <is>
-          <t>혜인</t>
+          <t>삼성전기</t>
         </is>
       </c>
       <c r="D43" s="20" t="n">
@@ -2176,15 +2170,15 @@
       <c r="G43" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H43" s="24" t="n">
-        <v>-9.17</v>
+      <c r="H43" s="22" t="n">
+        <v>-3.05</v>
       </c>
       <c r="I43" s="22" t="n">
-        <v>33.65</v>
+        <v>-6.17</v>
       </c>
       <c r="J43" s="23" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +209% / 중요공시 1건</t>
+          <t>중요공시 1건 / 네이버뉴스 기사 언급 / 매일경제 헤드라인 언급</t>
         </is>
       </c>
       <c r="K43" s="23" t="inlineStr">
@@ -2196,7 +2190,7 @@
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="20" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B44" s="20" t="n">
@@ -2204,7 +2198,7 @@
       </c>
       <c r="C44" s="21" t="inlineStr">
         <is>
-          <t>디티에스</t>
+          <t>국전</t>
         </is>
       </c>
       <c r="D44" s="20" t="n">
@@ -2219,25 +2213,27 @@
       <c r="G44" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H44" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I44" s="20" t="n">
-        <v/>
+      <c r="H44" s="22" t="n">
+        <v>-4.97</v>
+      </c>
+      <c r="I44" s="22" t="n">
+        <v>-12.4</v>
       </c>
       <c r="J44" s="23" t="inlineStr">
         <is>
-          <t>한국경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K44" s="23" t="n">
-        <v/>
+          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
+        </is>
+      </c>
+      <c r="K44" s="23" t="inlineStr">
+        <is>
+          <t>공시</t>
+        </is>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="20" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B45" s="20" t="n">
@@ -2245,7 +2241,7 @@
       </c>
       <c r="C45" s="21" t="inlineStr">
         <is>
-          <t>LG디스플레이</t>
+          <t>노을</t>
         </is>
       </c>
       <c r="D45" s="20" t="n">
@@ -2261,10 +2257,10 @@
         <v>0</v>
       </c>
       <c r="H45" s="24" t="n">
-        <v>-1.66</v>
+        <v>29.96</v>
       </c>
       <c r="I45" s="24" t="n">
-        <v>-5.33</v>
+        <v>16.7</v>
       </c>
       <c r="J45" s="23" t="inlineStr">
         <is>
@@ -2278,301 +2274,301 @@
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
-      <c r="A46" s="20" t="inlineStr">
-        <is>
-          <t>2026-10-25</t>
-        </is>
-      </c>
-      <c r="B46" s="20" t="n">
+      <c r="A46" s="25" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B46" s="25" t="n">
         <v>33</v>
       </c>
-      <c r="C46" s="21" t="inlineStr">
-        <is>
-          <t>삼성물산</t>
-        </is>
-      </c>
-      <c r="D46" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E46" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F46" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G46" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H46" s="24" t="n">
-        <v>-0.52</v>
-      </c>
-      <c r="I46" s="22" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="J46" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 4건 / 매일경제 기사 언급</t>
-        </is>
-      </c>
-      <c r="K46" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
+      <c r="C46" s="26" t="inlineStr">
+        <is>
+          <t>엘리스</t>
+        </is>
+      </c>
+      <c r="D46" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E46" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F46" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G46" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H46" s="27" t="n">
+        <v>-3.5</v>
+      </c>
+      <c r="I46" s="28" t="n">
+        <v>47.73</v>
+      </c>
+      <c r="J46" s="29" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +7335%</t>
+        </is>
+      </c>
+      <c r="K46" s="29" t="inlineStr">
+        <is>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
-      <c r="A47" s="20" t="inlineStr">
-        <is>
-          <t>2026-10-25</t>
-        </is>
-      </c>
-      <c r="B47" s="20" t="n">
+      <c r="A47" s="25" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B47" s="25" t="n">
         <v>34</v>
       </c>
-      <c r="C47" s="21" t="inlineStr">
-        <is>
-          <t>현대건설</t>
-        </is>
-      </c>
-      <c r="D47" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E47" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="F47" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G47" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="H47" s="24" t="n">
-        <v>-2.15</v>
-      </c>
-      <c r="I47" s="24" t="n">
-        <v>-2.47</v>
-      </c>
-      <c r="J47" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 2건 / 중요공시 7일 +100%</t>
-        </is>
-      </c>
-      <c r="K47" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
+      <c r="C47" s="26" t="inlineStr">
+        <is>
+          <t>푸드나무</t>
+        </is>
+      </c>
+      <c r="D47" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E47" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F47" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H47" s="27" t="n">
+        <v>-14.29</v>
+      </c>
+      <c r="I47" s="27" t="n">
+        <v>-58.79</v>
+      </c>
+      <c r="J47" s="29" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +1488%</t>
+        </is>
+      </c>
+      <c r="K47" s="29" t="inlineStr">
+        <is>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
-      <c r="A48" s="20" t="inlineStr">
-        <is>
-          <t>2026-10-25</t>
-        </is>
-      </c>
-      <c r="B48" s="20" t="n">
+      <c r="A48" s="25" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B48" s="25" t="n">
         <v>35</v>
       </c>
-      <c r="C48" s="21" t="inlineStr">
-        <is>
-          <t>HD현대중공업</t>
-        </is>
-      </c>
-      <c r="D48" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E48" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="F48" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G48" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="H48" s="24" t="n">
-        <v>-0.49</v>
-      </c>
-      <c r="I48" s="24" t="n">
-        <v>-13.51</v>
-      </c>
-      <c r="J48" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 2건 / 중요공시 7일 +100%</t>
-        </is>
-      </c>
-      <c r="K48" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
+      <c r="C48" s="26" t="inlineStr">
+        <is>
+          <t>DGI</t>
+        </is>
+      </c>
+      <c r="D48" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E48" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F48" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G48" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H48" s="27" t="n">
+        <v>-13.26</v>
+      </c>
+      <c r="I48" s="27" t="n">
+        <v>-3.99</v>
+      </c>
+      <c r="J48" s="29" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +893%</t>
+        </is>
+      </c>
+      <c r="K48" s="29" t="inlineStr">
+        <is>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
-      <c r="A49" s="20" t="inlineStr">
-        <is>
-          <t>2026-10-25</t>
-        </is>
-      </c>
-      <c r="B49" s="20" t="n">
+      <c r="A49" s="25" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B49" s="25" t="n">
         <v>36</v>
       </c>
-      <c r="C49" s="21" t="inlineStr">
-        <is>
-          <t>국전</t>
-        </is>
-      </c>
-      <c r="D49" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E49" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F49" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G49" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H49" s="24" t="n">
-        <v>-4.97</v>
-      </c>
-      <c r="I49" s="24" t="n">
-        <v>-12.4</v>
-      </c>
-      <c r="J49" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K49" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
+      <c r="C49" s="26" t="inlineStr">
+        <is>
+          <t>스페코</t>
+        </is>
+      </c>
+      <c r="D49" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E49" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F49" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G49" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H49" s="28" t="n">
+        <v>27.09</v>
+      </c>
+      <c r="I49" s="28" t="n">
+        <v>41.72</v>
+      </c>
+      <c r="J49" s="29" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +890%</t>
+        </is>
+      </c>
+      <c r="K49" s="29" t="inlineStr">
+        <is>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
-      <c r="A50" s="20" t="inlineStr">
-        <is>
-          <t>2026-10-25</t>
-        </is>
-      </c>
-      <c r="B50" s="20" t="n">
+      <c r="A50" s="25" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B50" s="25" t="n">
         <v>37</v>
       </c>
-      <c r="C50" s="21" t="inlineStr">
-        <is>
-          <t>노을</t>
-        </is>
-      </c>
-      <c r="D50" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E50" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F50" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G50" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H50" s="22" t="n">
-        <v>29.96</v>
-      </c>
-      <c r="I50" s="22" t="n">
-        <v>16.7</v>
-      </c>
-      <c r="J50" s="23" t="inlineStr">
-        <is>
-          <t>중요공시 1건 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K50" s="23" t="inlineStr">
-        <is>
-          <t>공시</t>
+      <c r="C50" s="26" t="inlineStr">
+        <is>
+          <t>진양홀딩스</t>
+        </is>
+      </c>
+      <c r="D50" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E50" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F50" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G50" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H50" s="28" t="n">
+        <v>4.12</v>
+      </c>
+      <c r="I50" s="28" t="n">
+        <v>4.29</v>
+      </c>
+      <c r="J50" s="29" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +636%</t>
+        </is>
+      </c>
+      <c r="K50" s="29" t="inlineStr">
+        <is>
+          <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
-      <c r="A51" s="20" t="inlineStr">
-        <is>
-          <t>2026-10-25</t>
-        </is>
-      </c>
-      <c r="B51" s="20" t="n">
+      <c r="A51" s="25" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B51" s="25" t="n">
         <v>38</v>
       </c>
-      <c r="C51" s="21" t="inlineStr">
-        <is>
-          <t>KT</t>
-        </is>
-      </c>
-      <c r="D51" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E51" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F51" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G51" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H51" s="24" t="n">
-        <v>-1.68</v>
-      </c>
-      <c r="I51" s="24" t="n">
-        <v>-7.34</v>
-      </c>
-      <c r="J51" s="23" t="inlineStr">
-        <is>
-          <t>한국경제 헤드라인 언급 / 네이버뉴스 기사 언급</t>
-        </is>
-      </c>
-      <c r="K51" s="23" t="inlineStr">
+      <c r="C51" s="26" t="inlineStr">
+        <is>
+          <t>앤로보틱스</t>
+        </is>
+      </c>
+      <c r="D51" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E51" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F51" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G51" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H51" s="28" t="n">
+        <v>20.12</v>
+      </c>
+      <c r="I51" s="28" t="n">
+        <v>49.58</v>
+      </c>
+      <c r="J51" s="29" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +493%</t>
+        </is>
+      </c>
+      <c r="K51" s="29" t="inlineStr">
         <is>
           <t>네이버</t>
         </is>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
-      <c r="A52" s="20" t="inlineStr">
-        <is>
-          <t>2026-10-25</t>
-        </is>
-      </c>
-      <c r="B52" s="20" t="n">
+      <c r="A52" s="25" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B52" s="25" t="n">
         <v>39</v>
       </c>
-      <c r="C52" s="21" t="inlineStr">
-        <is>
-          <t>클라우드</t>
-        </is>
-      </c>
-      <c r="D52" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E52" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F52" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G52" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H52" s="20" t="n">
-        <v/>
-      </c>
-      <c r="I52" s="20" t="n">
-        <v/>
-      </c>
-      <c r="J52" s="23" t="inlineStr">
-        <is>
-          <t>네이버뉴스 기사 언급 / 매일경제 헤드라인 언급</t>
-        </is>
-      </c>
-      <c r="K52" s="23" t="inlineStr">
+      <c r="C52" s="26" t="inlineStr">
+        <is>
+          <t>진양산업</t>
+        </is>
+      </c>
+      <c r="D52" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E52" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F52" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G52" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H52" s="28" t="n">
+        <v>27.82</v>
+      </c>
+      <c r="I52" s="28" t="n">
+        <v>29.02</v>
+      </c>
+      <c r="J52" s="29" t="inlineStr">
+        <is>
+          <t>네이버 검색 당일 +423%</t>
+        </is>
+      </c>
+      <c r="K52" s="29" t="inlineStr">
         <is>
           <t>네이버</t>
         </is>
@@ -2581,7 +2577,7 @@
     <row r="53" ht="18" customHeight="1">
       <c r="A53" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B53" s="25" t="n">
@@ -2589,7 +2585,7 @@
       </c>
       <c r="C53" s="26" t="inlineStr">
         <is>
-          <t>엘리스</t>
+          <t>한일단조</t>
         </is>
       </c>
       <c r="D53" s="25" t="n">
@@ -2605,14 +2601,14 @@
         <v>0</v>
       </c>
       <c r="H53" s="27" t="n">
-        <v>-3.5</v>
+        <v>-1.49</v>
       </c>
       <c r="I53" s="28" t="n">
-        <v>47.73</v>
+        <v>9.48</v>
       </c>
       <c r="J53" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +7205%</t>
+          <t>네이버 검색 당일 +367%</t>
         </is>
       </c>
       <c r="K53" s="29" t="inlineStr">
@@ -2624,7 +2620,7 @@
     <row r="54" ht="18" customHeight="1">
       <c r="A54" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B54" s="25" t="n">
@@ -2632,7 +2628,7 @@
       </c>
       <c r="C54" s="26" t="inlineStr">
         <is>
-          <t>푸드나무</t>
+          <t>휴니드</t>
         </is>
       </c>
       <c r="D54" s="25" t="n">
@@ -2648,14 +2644,14 @@
         <v>0</v>
       </c>
       <c r="H54" s="27" t="n">
-        <v>-14.29</v>
-      </c>
-      <c r="I54" s="27" t="n">
-        <v>-58.79</v>
+        <v>-0.92</v>
+      </c>
+      <c r="I54" s="28" t="n">
+        <v>16.53</v>
       </c>
       <c r="J54" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +1451%</t>
+          <t>네이버 검색 당일 +359%</t>
         </is>
       </c>
       <c r="K54" s="29" t="inlineStr">
@@ -2667,7 +2663,7 @@
     <row r="55" ht="18" customHeight="1">
       <c r="A55" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B55" s="25" t="n">
@@ -2675,7 +2671,7 @@
       </c>
       <c r="C55" s="26" t="inlineStr">
         <is>
-          <t>DGI</t>
+          <t>진양화학</t>
         </is>
       </c>
       <c r="D55" s="25" t="n">
@@ -2690,15 +2686,15 @@
       <c r="G55" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H55" s="27" t="n">
-        <v>-13.26</v>
-      </c>
-      <c r="I55" s="27" t="n">
-        <v>-3.99</v>
+      <c r="H55" s="28" t="n">
+        <v>31.11</v>
+      </c>
+      <c r="I55" s="28" t="n">
+        <v>35.87</v>
       </c>
       <c r="J55" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +869%</t>
+          <t>네이버 검색 당일 +349%</t>
         </is>
       </c>
       <c r="K55" s="29" t="inlineStr">
@@ -2710,7 +2706,7 @@
     <row r="56" ht="18" customHeight="1">
       <c r="A56" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B56" s="25" t="n">
@@ -2718,7 +2714,7 @@
       </c>
       <c r="C56" s="26" t="inlineStr">
         <is>
-          <t>스페코</t>
+          <t>형지엘리트</t>
         </is>
       </c>
       <c r="D56" s="25" t="n">
@@ -2733,15 +2729,15 @@
       <c r="G56" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H56" s="28" t="n">
-        <v>27.09</v>
+      <c r="H56" s="27" t="n">
+        <v>-14.87</v>
       </c>
       <c r="I56" s="28" t="n">
-        <v>41.72</v>
+        <v>19.93</v>
       </c>
       <c r="J56" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +668%</t>
+          <t>네이버 검색 당일 +322%</t>
         </is>
       </c>
       <c r="K56" s="29" t="inlineStr">
@@ -2753,7 +2749,7 @@
     <row r="57" ht="18" customHeight="1">
       <c r="A57" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B57" s="25" t="n">
@@ -2761,7 +2757,7 @@
       </c>
       <c r="C57" s="26" t="inlineStr">
         <is>
-          <t>진양홀딩스</t>
+          <t>유니테크노</t>
         </is>
       </c>
       <c r="D57" s="25" t="n">
@@ -2777,14 +2773,14 @@
         <v>0</v>
       </c>
       <c r="H57" s="28" t="n">
-        <v>4.12</v>
+        <v>10.56</v>
       </c>
       <c r="I57" s="28" t="n">
-        <v>4.29</v>
+        <v>11.67</v>
       </c>
       <c r="J57" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +546%</t>
+          <t>네이버 검색 당일 +294%</t>
         </is>
       </c>
       <c r="K57" s="29" t="inlineStr">
@@ -2796,7 +2792,7 @@
     <row r="58" ht="18" customHeight="1">
       <c r="A58" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B58" s="25" t="n">
@@ -2804,7 +2800,7 @@
       </c>
       <c r="C58" s="26" t="inlineStr">
         <is>
-          <t>앤로보틱스</t>
+          <t>진양폴리</t>
         </is>
       </c>
       <c r="D58" s="25" t="n">
@@ -2820,14 +2816,14 @@
         <v>0</v>
       </c>
       <c r="H58" s="28" t="n">
-        <v>20.12</v>
+        <v>29.5</v>
       </c>
       <c r="I58" s="28" t="n">
-        <v>49.58</v>
+        <v>29.19</v>
       </c>
       <c r="J58" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +455%</t>
+          <t>네이버 검색 당일 +225%</t>
         </is>
       </c>
       <c r="K58" s="29" t="inlineStr">
@@ -2839,7 +2835,7 @@
     <row r="59" ht="18" customHeight="1">
       <c r="A59" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B59" s="25" t="n">
@@ -2847,7 +2843,7 @@
       </c>
       <c r="C59" s="26" t="inlineStr">
         <is>
-          <t>진양산업</t>
+          <t>SKAI</t>
         </is>
       </c>
       <c r="D59" s="25" t="n">
@@ -2862,15 +2858,15 @@
       <c r="G59" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H59" s="28" t="n">
-        <v>27.82</v>
+      <c r="H59" s="27" t="n">
+        <v>-8.970000000000001</v>
       </c>
       <c r="I59" s="28" t="n">
-        <v>29.02</v>
+        <v>9.27</v>
       </c>
       <c r="J59" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +370%</t>
+          <t>네이버 검색 당일 +209%</t>
         </is>
       </c>
       <c r="K59" s="29" t="inlineStr">
@@ -2882,7 +2878,7 @@
     <row r="60" ht="18" customHeight="1">
       <c r="A60" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B60" s="25" t="n">
@@ -2890,7 +2886,7 @@
       </c>
       <c r="C60" s="26" t="inlineStr">
         <is>
-          <t>휴니드</t>
+          <t>대모</t>
         </is>
       </c>
       <c r="D60" s="25" t="n">
@@ -2905,15 +2901,15 @@
       <c r="G60" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H60" s="27" t="n">
-        <v>-0.92</v>
+      <c r="H60" s="28" t="n">
+        <v>6.23</v>
       </c>
       <c r="I60" s="28" t="n">
-        <v>16.53</v>
+        <v>16.67</v>
       </c>
       <c r="J60" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +346%</t>
+          <t>네이버 검색 당일 +182%</t>
         </is>
       </c>
       <c r="K60" s="29" t="inlineStr">
@@ -2925,7 +2921,7 @@
     <row r="61" ht="18" customHeight="1">
       <c r="A61" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B61" s="25" t="n">
@@ -2933,7 +2929,7 @@
       </c>
       <c r="C61" s="26" t="inlineStr">
         <is>
-          <t>한일단조</t>
+          <t>자이언트스텝</t>
         </is>
       </c>
       <c r="D61" s="25" t="n">
@@ -2948,15 +2944,15 @@
       <c r="G61" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H61" s="27" t="n">
-        <v>-1.49</v>
+      <c r="H61" s="28" t="n">
+        <v>0.74</v>
       </c>
       <c r="I61" s="28" t="n">
-        <v>9.48</v>
+        <v>47.31</v>
       </c>
       <c r="J61" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +328%</t>
+          <t>네이버 검색 당일 +170%</t>
         </is>
       </c>
       <c r="K61" s="29" t="inlineStr">
@@ -2968,7 +2964,7 @@
     <row r="62" ht="18" customHeight="1">
       <c r="A62" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B62" s="25" t="n">
@@ -2976,7 +2972,7 @@
       </c>
       <c r="C62" s="26" t="inlineStr">
         <is>
-          <t>진양화학</t>
+          <t>모니터랩</t>
         </is>
       </c>
       <c r="D62" s="25" t="n">
@@ -2992,14 +2988,14 @@
         <v>0</v>
       </c>
       <c r="H62" s="28" t="n">
-        <v>31.11</v>
+        <v>9.27</v>
       </c>
       <c r="I62" s="28" t="n">
-        <v>35.87</v>
+        <v>11.09</v>
       </c>
       <c r="J62" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +310%</t>
+          <t>네이버 검색 당일 +162%</t>
         </is>
       </c>
       <c r="K62" s="29" t="inlineStr">
@@ -3011,7 +3007,7 @@
     <row r="63" ht="18" customHeight="1">
       <c r="A63" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B63" s="25" t="n">
@@ -3019,7 +3015,7 @@
       </c>
       <c r="C63" s="26" t="inlineStr">
         <is>
-          <t>형지엘리트</t>
+          <t>KBI동양철관</t>
         </is>
       </c>
       <c r="D63" s="25" t="n">
@@ -3035,14 +3031,14 @@
         <v>0</v>
       </c>
       <c r="H63" s="27" t="n">
-        <v>-14.87</v>
-      </c>
-      <c r="I63" s="28" t="n">
-        <v>19.93</v>
+        <v>-6.91</v>
+      </c>
+      <c r="I63" s="27" t="n">
+        <v>-0.45</v>
       </c>
       <c r="J63" s="29" t="inlineStr">
         <is>
-          <t>네이버 검색 당일 +308%</t>
+          <t>네이버 검색 당일 +118%</t>
         </is>
       </c>
       <c r="K63" s="29" t="inlineStr">
@@ -3144,22 +3140,22 @@
         <v>1</v>
       </c>
       <c r="C3" s="25" t="n">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D3" s="25" t="n">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="E3" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F3" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="G3" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="H3" s="25" t="n"/>
@@ -3175,22 +3171,22 @@
         <v>1</v>
       </c>
       <c r="C4" s="25" t="n">
-        <v>50</v>
+        <v>23</v>
       </c>
       <c r="D4" s="25" t="n">
-        <v>50</v>
+        <v>23</v>
       </c>
       <c r="E4" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F4" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="G4" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="H4" s="28" t="n">
@@ -3210,22 +3206,22 @@
         <v>1</v>
       </c>
       <c r="C5" s="25" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D5" s="25" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E5" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F5" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="G5" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="H5" s="25" t="n"/>
@@ -3241,22 +3237,22 @@
         <v>1</v>
       </c>
       <c r="C6" s="25" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D6" s="25" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E6" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F6" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="G6" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="H6" s="27" t="n">
@@ -3269,64 +3265,60 @@
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="26" t="inlineStr">
         <is>
-          <t>삼성전기</t>
+          <t>전기차</t>
         </is>
       </c>
       <c r="B7" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="25" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D7" s="25" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E7" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F7" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="G7" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
-        </is>
-      </c>
-      <c r="H7" s="27" t="n">
-        <v>-3.05</v>
-      </c>
-      <c r="I7" s="27" t="n">
-        <v>-6.17</v>
-      </c>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="H7" s="25" t="n"/>
+      <c r="I7" s="25" t="n"/>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="26" t="inlineStr">
         <is>
-          <t>조선</t>
+          <t>바이오</t>
         </is>
       </c>
       <c r="B8" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="25" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="D8" s="25" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E8" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F8" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="G8" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="H8" s="25" t="n"/>
@@ -3342,22 +3334,22 @@
         <v>1</v>
       </c>
       <c r="C9" s="25" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="D9" s="25" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="E9" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F9" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="G9" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="H9" s="28" t="n">
@@ -3370,7 +3362,7 @@
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="26" t="inlineStr">
         <is>
-          <t>로봇</t>
+          <t>한솔아이원스</t>
         </is>
       </c>
       <c r="B10" s="25" t="n">
@@ -3387,43 +3379,47 @@
       </c>
       <c r="F10" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="G10" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
-        </is>
-      </c>
-      <c r="H10" s="25" t="n"/>
-      <c r="I10" s="25" t="n"/>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="H10" s="27" t="n">
+        <v>-2.12</v>
+      </c>
+      <c r="I10" s="27" t="n">
+        <v>-10.61</v>
+      </c>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="26" t="inlineStr">
         <is>
-          <t>전기차</t>
+          <t>게임</t>
         </is>
       </c>
       <c r="B11" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="25" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D11" s="25" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E11" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F11" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="G11" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="H11" s="25" t="n"/>
@@ -3432,7 +3428,7 @@
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="26" t="inlineStr">
         <is>
-          <t>신한지주</t>
+          <t>로봇</t>
         </is>
       </c>
       <c r="B12" s="25" t="n">
@@ -3449,25 +3445,21 @@
       </c>
       <c r="F12" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="G12" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
-        </is>
-      </c>
-      <c r="H12" s="27" t="n">
-        <v>-2.22</v>
-      </c>
-      <c r="I12" s="27" t="n">
-        <v>-6.18</v>
-      </c>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="H12" s="25" t="n"/>
+      <c r="I12" s="25" t="n"/>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>셀트리온</t>
+          <t>빅텍</t>
         </is>
       </c>
       <c r="B13" s="25" t="n">
@@ -3484,19 +3476,19 @@
       </c>
       <c r="F13" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="G13" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="H13" s="27" t="n">
-        <v>-0.47</v>
-      </c>
-      <c r="I13" s="27" t="n">
-        <v>-0.67</v>
+        <v>-3.32</v>
+      </c>
+      <c r="I13" s="28" t="n">
+        <v>25.78</v>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
@@ -3519,12 +3511,12 @@
       </c>
       <c r="F14" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="G14" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="H14" s="27" t="n">
@@ -3554,12 +3546,12 @@
       </c>
       <c r="F15" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="G15" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="H15" s="25" t="n"/>
@@ -3585,12 +3577,12 @@
       </c>
       <c r="F16" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="G16" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="H16" s="27" t="n">
@@ -3620,12 +3612,12 @@
       </c>
       <c r="F17" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="G17" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="H17" s="27" t="n">
@@ -3638,7 +3630,7 @@
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="26" t="inlineStr">
         <is>
-          <t>게임</t>
+          <t>GS</t>
         </is>
       </c>
       <c r="B18" s="25" t="n">
@@ -3655,21 +3647,25 @@
       </c>
       <c r="F18" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="G18" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
-        </is>
-      </c>
-      <c r="H18" s="25" t="n"/>
-      <c r="I18" s="25" t="n"/>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="H18" s="27" t="n">
+        <v>-3.42</v>
+      </c>
+      <c r="I18" s="27" t="n">
+        <v>-8.43</v>
+      </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>HD현대중공업</t>
         </is>
       </c>
       <c r="B19" s="25" t="n">
@@ -3686,21 +3682,25 @@
       </c>
       <c r="F19" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="G19" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
-        </is>
-      </c>
-      <c r="H19" s="25" t="n"/>
-      <c r="I19" s="25" t="n"/>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="H19" s="27" t="n">
+        <v>-0.49</v>
+      </c>
+      <c r="I19" s="27" t="n">
+        <v>-13.51</v>
+      </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="26" t="inlineStr">
         <is>
-          <t>두산에너빌리티</t>
+          <t>LG전자</t>
         </is>
       </c>
       <c r="B20" s="25" t="n">
@@ -3717,25 +3717,25 @@
       </c>
       <c r="F20" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="G20" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="H20" s="27" t="n">
-        <v>-3.92</v>
+        <v>-1.77</v>
       </c>
       <c r="I20" s="27" t="n">
-        <v>-8.539999999999999</v>
+        <v>-8.789999999999999</v>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="26" t="inlineStr">
         <is>
-          <t>원전</t>
+          <t>금호건설</t>
         </is>
       </c>
       <c r="B21" s="25" t="n">
@@ -3752,21 +3752,25 @@
       </c>
       <c r="F21" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="G21" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
-        </is>
-      </c>
-      <c r="H21" s="25" t="n"/>
-      <c r="I21" s="25" t="n"/>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="H21" s="27" t="n">
+        <v>-3.58</v>
+      </c>
+      <c r="I21" s="27" t="n">
+        <v>-8.08</v>
+      </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="26" t="inlineStr">
         <is>
-          <t>카카오</t>
+          <t>기아</t>
         </is>
       </c>
       <c r="B22" s="25" t="n">
@@ -3783,25 +3787,25 @@
       </c>
       <c r="F22" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="G22" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="H22" s="27" t="n">
-        <v>-1.32</v>
+        <v>-1.57</v>
       </c>
       <c r="I22" s="27" t="n">
-        <v>-5.99</v>
+        <v>-3.79</v>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="26" t="inlineStr">
         <is>
-          <t>카카오게임즈</t>
+          <t>네이버</t>
         </is>
       </c>
       <c r="B23" s="25" t="n">
@@ -3818,25 +3822,21 @@
       </c>
       <c r="F23" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="G23" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
-        </is>
-      </c>
-      <c r="H23" s="28" t="n">
-        <v>6.51</v>
-      </c>
-      <c r="I23" s="28" t="n">
-        <v>13.27</v>
-      </c>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="H23" s="25" t="n"/>
+      <c r="I23" s="25" t="n"/>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="26" t="inlineStr">
         <is>
-          <t>한솔아이원스</t>
+          <t>신한지주</t>
         </is>
       </c>
       <c r="B24" s="25" t="n">
@@ -3853,25 +3853,25 @@
       </c>
       <c r="F24" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="G24" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="H24" s="27" t="n">
-        <v>-2.12</v>
+        <v>-2.22</v>
       </c>
       <c r="I24" s="27" t="n">
-        <v>-10.61</v>
+        <v>-6.18</v>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="26" t="inlineStr">
         <is>
-          <t>현대로템</t>
+          <t>예스티</t>
         </is>
       </c>
       <c r="B25" s="25" t="n">
@@ -3888,47 +3888,47 @@
       </c>
       <c r="F25" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="G25" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="H25" s="27" t="n">
-        <v>-3.77</v>
-      </c>
-      <c r="I25" s="27" t="n">
-        <v>-16.31</v>
+        <v>-6.68</v>
+      </c>
+      <c r="I25" s="28" t="n">
+        <v>5.08</v>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="26" t="inlineStr">
         <is>
-          <t>Apple</t>
+          <t>조선</t>
         </is>
       </c>
       <c r="B26" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C26" s="25" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D26" s="25" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E26" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F26" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="G26" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="H26" s="25" t="n"/>
@@ -3937,112 +3937,112 @@
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="26" t="inlineStr">
         <is>
-          <t>비나텍</t>
+          <t>현대건설</t>
         </is>
       </c>
       <c r="B27" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C27" s="25" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D27" s="25" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E27" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F27" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="G27" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
-        </is>
-      </c>
-      <c r="H27" s="28" t="n">
-        <v>8.1</v>
-      </c>
-      <c r="I27" s="28" t="n">
-        <v>47.06</v>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="H27" s="27" t="n">
+        <v>-2.15</v>
+      </c>
+      <c r="I27" s="27" t="n">
+        <v>-2.47</v>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="26" t="inlineStr">
         <is>
-          <t>삼성전자우</t>
+          <t>현대로템</t>
         </is>
       </c>
       <c r="B28" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C28" s="25" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D28" s="25" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E28" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F28" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="G28" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="H28" s="27" t="n">
-        <v>-0.24</v>
+        <v>-3.77</v>
       </c>
       <c r="I28" s="27" t="n">
-        <v>-1.66</v>
+        <v>-16.31</v>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="26" t="inlineStr">
         <is>
-          <t>HD현대중공업</t>
+          <t>혜인</t>
         </is>
       </c>
       <c r="B29" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C29" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D29" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E29" s="32" t="n">
         <v>1</v>
       </c>
       <c r="F29" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="G29" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="H29" s="27" t="n">
-        <v>-0.49</v>
-      </c>
-      <c r="I29" s="27" t="n">
-        <v>-13.51</v>
+        <v>-9.17</v>
+      </c>
+      <c r="I29" s="28" t="n">
+        <v>33.65</v>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="26" t="inlineStr">
         <is>
-          <t>KT</t>
+          <t>국전</t>
         </is>
       </c>
       <c r="B30" s="25" t="n">
@@ -4059,25 +4059,25 @@
       </c>
       <c r="F30" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="G30" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="H30" s="27" t="n">
-        <v>-1.68</v>
+        <v>-4.97</v>
       </c>
       <c r="I30" s="27" t="n">
-        <v>-7.34</v>
+        <v>-12.4</v>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="26" t="inlineStr">
         <is>
-          <t>LG디스플레이</t>
+          <t>노을</t>
         </is>
       </c>
       <c r="B31" s="25" t="n">
@@ -4094,25 +4094,25 @@
       </c>
       <c r="F31" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="G31" s="25" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
-        </is>
-      </c>
-      <c r="H31